<commit_message>
Scan: 2026-09-14 08:38 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD7"/>
+  <dimension ref="A1:AD13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1052,7 +1052,7 @@
         <v>0.415</v>
       </c>
       <c r="P6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="n">
         <v>6.357</v>
@@ -1229,6 +1229,747 @@
         </is>
       </c>
       <c r="AD7" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-14T08:36:18+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>4369.7998</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4379.2998</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4348</v>
+      </c>
+      <c r="H8" t="n">
+        <v>4353</v>
+      </c>
+      <c r="I8" t="n">
+        <v>14789</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" t="n">
+        <v>39</v>
+      </c>
+      <c r="L8" t="n">
+        <v>-0.102</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="N8" t="n">
+        <v>40</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>-0.666</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Founders Metals (TSXV:FDR) Falls 5.65% as Profit-Taking Tests Strong Antino Gold Momentum - kalkine.ca</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQWjZmSkNZV2p0c3pfYWd1Y2U0NnVtdlNaTGdEU3dDbEZ1QTV2WVZCUXp2bmZFVE5ETHByVmc4R1lBUFlDU2JsejNyNkNCcEk3R2lUQUpPbnl5ZS1aeWZGN0lISTVocl9leXVOdTBrN2dKdGJyVl85N0pUQlFtaEZvTXF3V2MzU0xNcTFydU5fNWZsamhnNDVqSThhVEVuaHYweTI5c1g3ZDlDOWplQl8zVGJqa3JnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-14T08:36:18+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>102.68</v>
+      </c>
+      <c r="F9" t="n">
+        <v>103.64</v>
+      </c>
+      <c r="G9" t="n">
+        <v>101.94</v>
+      </c>
+      <c r="H9" t="n">
+        <v>103.53</v>
+      </c>
+      <c r="I9" t="n">
+        <v>29973</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" t="n">
+        <v>40</v>
+      </c>
+      <c r="L9" t="n">
+        <v>-0.015</v>
+      </c>
+      <c r="M9" t="n">
+        <v>-0.248</v>
+      </c>
+      <c r="N9" t="n">
+        <v>40</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="P9" t="n">
+        <v>-0.119</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>3.965</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Current price of oil as of July 30, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9odGxncTZBdXJrcnd4Zm1GSENJSFpJQUJxbGphdTV2dTRfQTVmMzVFQ21PTGhzY19DSGVFUWpoeEtGMDZhNzRveUNoaDBlcDVLSmRpaFh6ZnA1emJSVllSYTNR?oc=5</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Oil prices surge 15% as Strait of Hormuz disruptions tighten supply - Offshore Technology</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPdndjemtyTkduUUpSVnR6aXJUNXBBR0JNd1FaaURNWmtvWm9WTkZUME50Qk1NVDUtdEtqcWE2R0xvUGRKNHBWZDMtblpaY1h1TE5zcmgycU5kS29mYU02N1BOdThBMUhUMDM0T1FScDZRY0JzYlRXTTJVajFYbkh3Rmp0MDFDeVZQcFhKSjhpaklySjZrVWJCZVoyWkw?oc=5</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Oil's roundtrip back to $100. Why China could determine what happens next - cnbc.com</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOa0xDNl91YjR4WVVvTXU5UlVvMnVQWUs0SDVCRFZFV0VxWVJzLVdsTWZuN1RiSjkxamJwdUkyVUdzZndiTXlITFdQWEVrSzJmSjN1bkczVjhhRktQSHR1UlMzMUtRalJZbmtLbDAtX0FJb1Ntb213dXFxeHMtVXh0NG5sd2ctUVdMWUJDQmF4R1U4V0hQZXQ0WVJDbVBWZDItbXAwbGxiWVFFSGs?oc=5</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>Dow Jones Futures Rise, Oil Prices Fall, Oracle Jumps; CPI Inflation Data To Inform Fed - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPZGdpMlBVbExibHozSndzcGVmRE9SOVdnMnJDbmFSX2NSbjRQamJhd3R6dEkxX2tlaTkwdWRjVlplWkpsQTJoamljRzhQcXZkUmhDTmgtRWY0U1RwRUlEYUdoRmVmVkktM3FDNWpyVXRFNkpEWGl5ZlhHaGNadmVKTUx5NlhlQXE1ejdTUlowM0dGM1lPRkdTb2xRV2pKczR6aWtoLXRMWG11RDlUaXRuZDc3eUh1SDBmQ2NZQ2laTzBXMGtVQ0NpVjNhU2FvZ1ItWDhQWV9n?oc=5</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - cnbc.com</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>VIX Breaks Out Before CPI: S&amp;P 500 Clinging to Support as Oil Gets Rejected at $104 - YouTube</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiQkFVX3lxTE5OVDlua2JHTEZ1Y25SWWtneWdRazB4R0cwWEY1dWFRWnU0SktHYjRzc2dYOGVYZWJ4NlJxeTBYMUg4Zw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-14T08:36:18+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>DX=F</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>37</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="N10" t="n">
+        <v>38</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="P10" t="n">
+        <v>-0.119</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>5.496</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>US Dollar outlook: Hawkish Fed repricing strengthens the bull case - stonex.com</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNRlJTZ3dmU0NMcWtjQU9uU1pXSDQ1Uk5YOGFCVTQwSlExOFZtcjBGT1VZdXppTkpqYkdoaUtTTWw0aVJxclFIaWFnWXItUzBDTkNNSGg1b0t3dVhvREJSQjJRYUFEMGpMa0pNTVpMUzdpT0YwRngyZi1nMlRCdHJlVjVkc0tvU3RqV2pPNzhtYUNhVXlWVXpPRlpiLXBFTE1KNjZoU2lZLXpUaE9CM0hTLTVRSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Dovish Fed Bets Pummel Dollar, Boost Gold Ahead of NFP - Investing.com</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPZDNJaUJnTUhOckR3ODFMRjN3M3QtZ1NzUmtvYnRUOVlyWEo2Nzg4d3l5Tkl4SFNRMVJCUnlNeGxUYm5NQkxpNmxEdzVpU3ZHTkhRUXh0bEdhNld2WHFBVmNCRTBEY2dsUkxqVlYtYTUwX21GR1JZNnZjazk2OXBjNW80dWo3Nmx5TXZYLUY0WkZLei14eWV4dDlkRGVheWM?oc=5</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>Q&amp;A on the Dollar Meltdown - Robin J Brooks | Substack</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE1iTlBuOHZORHl4Y0YtclRnalp6NW9kOVhMVVNHX3h5cVM5WjBJdk5vZTd4STQwaHNUNmw5aVE3b1ZWUW0zS19oYnFfMXRCQWhtZjZVbUo2X0cwSVBCcTd3bzJZU0ppOHhnZmJUQXJmUThCRzZV?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-14T08:36:18+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>7620.25</v>
+      </c>
+      <c r="F11" t="n">
+        <v>7624.75</v>
+      </c>
+      <c r="G11" t="n">
+        <v>7604</v>
+      </c>
+      <c r="H11" t="n">
+        <v>7606.5</v>
+      </c>
+      <c r="I11" t="n">
+        <v>44502</v>
+      </c>
+      <c r="J11" t="n">
+        <v>4</v>
+      </c>
+      <c r="K11" t="n">
+        <v>38</v>
+      </c>
+      <c r="L11" t="n">
+        <v>-0.132</v>
+      </c>
+      <c r="M11" t="n">
+        <v>-0.004</v>
+      </c>
+      <c r="N11" t="n">
+        <v>40</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="P11" t="n">
+        <v>-0.08500000000000001</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>-0.076</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Bitmine Surges 8% on Ethereum Strength After Cantor Fitzgerald Doubles Its Target, SharpLink Advances 9%, Strategy Gains 4% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPemN4ODV3YldjcDUxb1FRWXc1OWV4bXZwVEhOWTMtbDJaNG92V0xpd0V6OTBxM3lRN0RZUEtWQkRWQW9Kb0hNUF8zS2FBOU5BUlpFTmpvNFBiYnpSVEhHMmtCU2JMdzNjRlNXRWtwaUM1eUxrVjRWQ3VQT2Q4MVJHaHBfdHBRUFpETTVnT012dEJQQV9mcHNOOHUwQnlVU2ZibW51TTBzMHdvTXhsQnlMMzJjT0lhcTNvVktGLTVfN1o3ZXlkLV9JNWRZVVFvakVaaDdIMGxWdFJXUVMxT19rREpueFJibmw0WllRUDk1ckgwUHB1?oc=5</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>'Titanic' has a happy ending: Robust rally caps Wall Street's week of red - TradingView</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSG12a01IVVJtakhLMFlscGk0SXRsa0M2UUwtakVNd041MUV0RVdjanozTGlFdWFpZ2dCai10NlYtbW42d3pnQ1lseGdvMGR5VV9USlk0T09WNW93TVhPMVUyUHpQT1ZDLWRBRWdBcHIzbTN4T0VhVVBZb0pzeHlqTEJNS0ZnTXlXUDlTYmRFbHYxYVJWSDQ1THZBSXhIckdURjdPY25wcWc3SXJ2R2pFX1lIVFVoem51RmZDTHhOWkVIRVIwWWdlZE1odzFGTG9DeFo5NHUycw?oc=5</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 11: HPE Surges on AI Infrastructure Demand and Recently Raised Guidance - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxQWHZrbGtuQ2NuRE92NG4temVfd3BnRnJ3ZDJQYlUzZGpBSnFIYWlLQ0VfVks2enFoZGdGamlac3MwdUFCb2JtTmlpV2NhaFFqUzZNQkhPS01ZVGNGTzNHZ05FbVFrWDVHN3F1Mjk1YU1uekRmRWktenpIX1dVQzd5RTJsZ3l2alRmNmxLUWNsY09xQTVJbnc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>Barclays lifts S&amp;P 500 index's year-end target to 7,950 on strong earnings - reuters.com</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQdEpJSkhqQ0dZZjZvbFZ3MU9EbGZpa0l4ZjJNazczLTZQTVVfZHlJVmxRVEx3ZFRpLWRwdEhycTRXbGtFdnplbnAwOEgzWG5VQXlYNEdkWE9pVTV0aGl0ZkdsSTBNb1M4U21LWkxPeUVBYWZLTDFZem81OWEtenIwa2E5bjlsdU1Bcmh2SzROZTR2RGFpOVQ4YTRTT21QWXpBX2k2dHV0S3hROHNkYmhR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Airbus stock rebounds after breaking its 196 € support level - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQTXFjUFRkaWo0Uy1RWThWLU14eFJ3VzF4Z1hyT3ZxMmgzUHdaSWRWSEpCZW1NaXpVU2pQRWxRUVRJT2ExS1FGSHB6VWVOR2pUXzlQUnNhcUxBSjRacjc2bmFHcWNtdmxIWXZHdi1vUjBfeTExYUNHVjROanlpRU5UOGJKeFE3VTY2M2ZzYmNaQVZ1d0xYdlhXVmN1S3BlZUdnRjM1U1FCU0hfUFdsWGIyV0Q0X0tJeDBxTWZwRGZ3?oc=5</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-14T08:36:18+00:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>29015</v>
+      </c>
+      <c r="F12" t="n">
+        <v>29037.5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>28900</v>
+      </c>
+      <c r="H12" t="n">
+        <v>28903</v>
+      </c>
+      <c r="I12" t="n">
+        <v>19345</v>
+      </c>
+      <c r="J12" t="n">
+        <v>4</v>
+      </c>
+      <c r="K12" t="n">
+        <v>40</v>
+      </c>
+      <c r="L12" t="n">
+        <v>-0.135</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="N12" t="n">
+        <v>36</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.416</v>
+      </c>
+      <c r="P12" t="n">
+        <v>-0.054</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>6.796</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 ends higher as strong inflation data cements rate-hike bets - reuters.com</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQOTZpMXRyVmxGMjJTRmVVOV91TnZIWlJsZS1BNlE3bENxRlRlVnh2RFZKQmdwUVNydUJQd1RvZlZLam1KbnR2ZS1Vd2VNaWhrN3lNZ3hETUtvcTVxYTFEOENQQ292eWk0YXJYYjBrekoycE5sU0FqdloxRXNZcTcyd1dnYkFEdGpmMV9Pd0lwemdYWmd0aHZaYmpkWmlLOFgxdnc?oc=5</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>The S&amp;P 500 is back at a record high and the Dow just hit 54,000 - CNN</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE9sNTR6eTFUS1JYX1lnaWVIZGxJeVhmbENJMHN3SUc4TTlSaHpweUdwNUNLejJtSmIwb0x0SEQxalc2OVN1X2s1WFhPSWt2X2VrcFFVeXhVVVpxYVVnaUFjRDR3SUFxbzA?oc=5</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>Dow Drops 628, Nasdaq Falls 86, S&amp;P 500 Loses 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOdElkenZMSDNpN1JfQ3VrQVBPYjBzTVgyOVNrRFVCX2JBWXk3WFRtb3hrLTFUbUlpTHNwbWsyX0tjY0RFMmFwOFNPTk42OEtzbWZPTkh0TXBGR2RRdHU1c3Zkd2g5Z2p5ckdqMVVMUElCeWstcEd4X3IxWWFUbGlPQVlnV3lYeWdneVZja05ueW8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>Katie Stockton: Bracing for volatility after Nasdaq broke below recent support - cnbc.com</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLWhuVXhhdF9LbEhfSTV2RlNTZ0IyVjBlcUxGS0RQLXA5S0xjUWFZa3c3Nm1OZmxSRU5mVmVLZzRkbEFKYWd1YWFoVHdadUpRRXlMc1BSVi1BY2Q5RlVLRzVoa2xuRkxZdThVS0VVTzRYY256MHZha1l6RDlrU0NaVXZGZW1qZFRWbTBOUFBTRGxUck9ZWk9tWlY4bl9LcU1BVG5Ka0RVVURXallmZGhqT1BacEpBYnFTUzBIRQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-14T08:36:18+00:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>77646.46090000001</v>
+      </c>
+      <c r="F13" t="n">
+        <v>77916.75</v>
+      </c>
+      <c r="G13" t="n">
+        <v>77338.50780000001</v>
+      </c>
+      <c r="H13" t="n">
+        <v>77703.47659999999</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2311450624</v>
+      </c>
+      <c r="J13" t="n">
+        <v>4</v>
+      </c>
+      <c r="K13" t="n">
+        <v>38</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="N13" t="n">
+        <v>38</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="P13" t="n">
+        <v>-0.091</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>5.801</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - cnbc.com</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Bitmine Surges 8% on Ethereum Strength After Cantor Fitzgerald Doubles Its Target, SharpLink Advances 9%, Strategy Gains 4% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPemN4ODV3YldjcDUxb1FRWXc1OWV4bXZwVEhOWTMtbDJaNG92V0xpd0V6OTBxM3lRN0RZUEtWQkRWQW9Kb0hNUF8zS2FBOU5BUlpFTmpvNFBiYnpSVEhHMmtCU2JMdzNjRlNXRWtwaUM1eUxrVjRWQ3VQT2Q4MVJHaHBfdHBRUFpETTVnT012dEJQQV9mcHNOOHUwQnlVU2ZibW51TTBzMHdvTXhsQnlMMzJjT0lhcTNvVktGLTVfN1o3ZXlkLV9JNWRZVVFvakVaaDdIMGxWdFJXUVMxT19rREpueFJibmw0WllRUDk1ckgwUHB1?oc=5</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>Strategy's $200M Bitcoin sale didn't drop prices, signaling strong market demand. - Pluang</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQZ2stY3N4T3I2NU50Q3d2cUVaSUJYWUg5aGc4cnlmZmgtMi16cGVISVZaaWNqTmhLRnhqSkU4bVlkeGpZMmtlMVRUQ1FjV0FhX044amFzR3NhYWY2TW5NU0VqLVdvclo5d3d3Rm43YnZfR1kwQXgycU92ZWpSbDQyMFZIT1lhdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Current price of Bitcoin for September 11, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTFBzdXZINHB2Z3h2a3pmd3JQUFY5TlRvZk8zcnhBdGxUQ2FDb3BiZWNiREprRGRscFViVUhhNTI0VXE5NWxDandwN1JOazJLeWt0YWVpTmJCRkdHRUdtQVVMNTQ4RWhuQVU?oc=5</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-14 08:54 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD13"/>
+  <dimension ref="A1:AD19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1970,6 +1970,762 @@
         </is>
       </c>
       <c r="AD13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-14T08:52:00+00:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>4369.7998</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4379.2998</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4348</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4353</v>
+      </c>
+      <c r="I14" t="n">
+        <v>15716</v>
+      </c>
+      <c r="J14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K14" t="n">
+        <v>39</v>
+      </c>
+      <c r="L14" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="N14" t="n">
+        <v>40</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>-1.304</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>Founders Metals (TSXV:FDR) Falls 5.65% as Profit-Taking Tests Strong Antino Gold Momentum - kalkine.ca</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQWjZmSkNZV2p0c3pfYWd1Y2U0NnVtdlNaTGdEU3dDbEZ1QTV2WVZCUXp2bmZFVE5ETHByVmc4R1lBUFlDU2JsejNyNkNCcEk3R2lUQUpPbnl5ZS1aeWZGN0lISTVocl9leXVOdTBrN2dKdGJyVl85N0pUQlFtaEZvTXF3V2MzU0xNcTFydU5fNWZsamhnNDVqSThhVEVuaHYweTI5c1g3ZDlDOWplQl8zVGJqa3JnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-14T08:52:00+00:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>102.68</v>
+      </c>
+      <c r="F15" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="G15" t="n">
+        <v>101.94</v>
+      </c>
+      <c r="H15" t="n">
+        <v>103.13</v>
+      </c>
+      <c r="I15" t="n">
+        <v>34787</v>
+      </c>
+      <c r="J15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K15" t="n">
+        <v>40</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M15" t="n">
+        <v>-0.267</v>
+      </c>
+      <c r="N15" t="n">
+        <v>40</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.257</v>
+      </c>
+      <c r="P15" t="n">
+        <v>-0.167</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>5.597</v>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Current price of oil as of July 30, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9odGxncTZBdXJrcnd4Zm1GSENJSFpJQUJxbGphdTV2dTRfQTVmMzVFQ21PTGhzY19DSGVFUWpoeEtGMDZhNzRveUNoaDBlcDVLSmRpaFh6ZnA1emJSVllSYTNR?oc=5</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>London Gas Oil breaks resistance at $1,273: Live levels By Investing.com - Investing.com India</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQOFJZcEZXSVpGOEZvTVR0SGRqYmZ4WF9SZ3RKajNUVWZDM2t3U3BOa3lQWk1oMUpnOF9UTTk0eFpwdzR0TEVzbHlHelFkb0xxZ3lFX08tR0gyblJWX20xenlXMi0xNVFfSlJ4UDdVUWtZcW5hV19VRHZIS0taRmRDRzlOek1wb2hmR3lpMGhGS0ZwbVVVZ0p4NFhibHBOTkdrd0JpWnVpSDl1dw?oc=5</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Oil's roundtrip back to $100. Why China could determine what happens next - CNBC</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOa0xDNl91YjR4WVVvTXU5UlVvMnVQWUs0SDVCRFZFV0VxWVJzLVdsTWZuN1RiSjkxamJwdUkyVUdzZndiTXlITFdQWEVrSzJmSjN1bkczVjhhRktQSHR1UlMzMUtRalJZbmtLbDAtX0FJb1Ntb213dXFxeHMtVXh0NG5sd2ctUVdMWUJDQmF4R1U4V0hQZXQ0WVJDbVBWZDItbXAwbGxiWVFFSGs?oc=5</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>OPEC oil output falls in August, Reuters survey shows - Reuters</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcGZWQVVsSEY1MDZDLXRVM2g2N0t1bHJ1VXpWX3pScTFZak53OGQ5VVNxemw0Mjdrd1paNjRYb1YtdFlYN3RIOURKM00xZmc4eFRlTHk2cTNhODJKWW5TOS1BMEE1cVF2NTN5YjJaeHRRNFlBVHUwUU9CN0pyOEdRMHE0c2VtcGNvamRPVFd3OVVlTnFmV3Fobks2WlZJU21oRW44?oc=5</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>Dow Jones Futures Rise, Oil Prices Fall, Oracle Jumps; CPI Inflation Data To Inform Fed - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPZGdpMlBVbExibHozSndzcGVmRE9SOVdnMnJDbmFSX2NSbjRQamJhd3R6dEkxX2tlaTkwdWRjVlplWkpsQTJoamljRzhQcXZkUmhDTmgtRWY0U1RwRUlEYUdoRmVmVkktM3FDNWpyVXRFNkpEWGl5ZlhHaGNadmVKTUx5NlhlQXE1ejdTUlowM0dGM1lPRkdTb2xRV2pKczR6aWtoLXRMWG11RDlUaXRuZDc3eUh1SDBmQ2NZQ2laTzBXMGtVQ0NpVjNhU2FvZ1ItWDhQWV9n?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-14T08:52:00+00:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>99.343</v>
+      </c>
+      <c r="F16" t="n">
+        <v>99.59</v>
+      </c>
+      <c r="G16" t="n">
+        <v>99.307</v>
+      </c>
+      <c r="H16" t="n">
+        <v>99.571</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>4</v>
+      </c>
+      <c r="K16" t="n">
+        <v>37</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="N16" t="n">
+        <v>38</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="P16" t="n">
+        <v>-0.116</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>3.831</v>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>US Dollar outlook: Hawkish Fed repricing strengthens the bull case - stonex.com</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNRlJTZ3dmU0NMcWtjQU9uU1pXSDQ1Uk5YOGFCVTQwSlExOFZtcjBGT1VZdXppTkpqYkdoaUtTTWw0aVJxclFIaWFnWXItUzBDTkNNSGg1b0t3dVhvREJSQjJRYUFEMGpMa0pNTVpMUzdpT0YwRngyZi1nMlRCdHJlVjVkc0tvU3RqV2pPNzhtYUNhVXlWVXpPRlpiLXBFTE1KNjZoU2lZLXpUaE9CM0hTLTVRSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>Dovish Fed Bets Pummel Dollar, Boost Gold Ahead of NFP - Investing.com</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPZDNJaUJnTUhOckR3ODFMRjN3M3QtZ1NzUmtvYnRUOVlyWEo2Nzg4d3l5Tkl4SFNRMVJCUnlNeGxUYm5NQkxpNmxEdzVpU3ZHTkhRUXh0bEdhNld2WHFBVmNCRTBEY2dsUkxqVlYtYTUwX21GR1JZNnZjazk2OXBjNW80dWo3Nmx5TXZYLUY0WkZLei14eWV4dDlkRGVheWM?oc=5</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>Q&amp;A on the Dollar Meltdown - Robin J Brooks | Substack</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE1iTlBuOHZORHl4Y0YtclRnalp6NW9kOVhMVVNHX3h5cVM5WjBJdk5vZTd4STQwaHNUNmw5aVE3b1ZWUW0zS19oYnFfMXRCQWhtZjZVbUo2X0cwSVBCcTd3bzJZU0ppOHhnZmJUQXJmUThCRzZV?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-14T08:52:00+00:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>7620.25</v>
+      </c>
+      <c r="F17" t="n">
+        <v>7624.75</v>
+      </c>
+      <c r="G17" t="n">
+        <v>7603.5</v>
+      </c>
+      <c r="H17" t="n">
+        <v>7609.5</v>
+      </c>
+      <c r="I17" t="n">
+        <v>50717</v>
+      </c>
+      <c r="J17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" t="n">
+        <v>38</v>
+      </c>
+      <c r="L17" t="n">
+        <v>-0.152</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-0.004</v>
+      </c>
+      <c r="N17" t="n">
+        <v>40</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="P17" t="n">
+        <v>-0.059</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.9340000000000001</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Bitmine Surges 8% on Ethereum Strength After Cantor Fitzgerald Doubles Its Target, SharpLink Advances 9%, Strategy Gains 4% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPemN4ODV3YldjcDUxb1FRWXc1OWV4bXZwVEhOWTMtbDJaNG92V0xpd0V6OTBxM3lRN0RZUEtWQkRWQW9Kb0hNUF8zS2FBOU5BUlpFTmpvNFBiYnpSVEhHMmtCU2JMdzNjRlNXRWtwaUM1eUxrVjRWQ3VQT2Q4MVJHaHBfdHBRUFpETTVnT012dEJQQV9mcHNOOHUwQnlVU2ZibW51TTBzMHdvTXhsQnlMMzJjT0lhcTNvVktGLTVfN1o3ZXlkLV9JNWRZVVFvakVaaDdIMGxWdFJXUVMxT19rREpueFJibmw0WllRUDk1ckgwUHB1?oc=5</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>'Titanic' has a happy ending: Robust rally caps Wall Street's week of red - TradingView</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSG12a01IVVJtakhLMFlscGk0SXRsa0M2UUwtakVNd041MUV0RVdjanozTGlFdWFpZ2dCai10NlYtbW42d3pnQ1lseGdvMGR5VV9USlk0T09WNW93TVhPMVUyUHpQT1ZDLWRBRWdBcHIzbTN4T0VhVVBZb0pzeHlqTEJNS0ZnTXlXUDlTYmRFbHYxYVJWSDQ1THZBSXhIckdURjdPY25wcWc3SXJ2R2pFX1lIVFVoem51RmZDTHhOWkVIRVIwWWdlZE1odzFGTG9DeFo5NHUycw?oc=5</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 11: HPE Surges on AI Infrastructure Demand and Recently Raised Guidance - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxQWHZrbGtuQ2NuRE92NG4temVfd3BnRnJ3ZDJQYlUzZGpBSnFIYWlLQ0VfVks2enFoZGdGamlac3MwdUFCb2JtTmlpV2NhaFFqUzZNQkhPS01ZVGNGTzNHZ05FbVFrWDVHN3F1Mjk1YU1uekRmRWktenpIX1dVQzd5RTJsZ3l2alRmNmxLUWNsY09xQTVJbnc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>Barclays lifts S&amp;P 500 index's year-end target to 7,950 on strong earnings - Reuters</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQdEpJSkhqQ0dZZjZvbFZ3MU9EbGZpa0l4ZjJNazczLTZQTVVfZHlJVmxRVEx3ZFRpLWRwdEhycTRXbGtFdnplbnAwOEgzWG5VQXlYNEdkWE9pVTV0aGl0ZkdsSTBNb1M4U21LWkxPeUVBYWZLTDFZem81OWEtenIwa2E5bjlsdU1Bcmh2SzROZTR2RGFpOVQ4YTRTT21QWXpBX2k2dHV0S3hROHNkYmhR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>Airbus stock rebounds after breaking its 196 € support level - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQTXFjUFRkaWo0Uy1RWThWLU14eFJ3VzF4Z1hyT3ZxMmgzUHdaSWRWSEpCZW1NaXpVU2pQRWxRUVRJT2ExS1FGSHB6VWVOR2pUXzlQUnNhcUxBSjRacjc2bmFHcWNtdmxIWXZHdi1vUjBfeTExYUNHVjROanlpRU5UOGJKeFE3VTY2M2ZzYmNaQVZ1d0xYdlhXVmN1S3BlZUdnRjM1U1FCU0hfUFdsWGIyV0Q0X0tJeDBxTWZwRGZ3?oc=5</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-14T08:52:00+00:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>29015</v>
+      </c>
+      <c r="F18" t="n">
+        <v>29037.5</v>
+      </c>
+      <c r="G18" t="n">
+        <v>28872.5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>28902.5</v>
+      </c>
+      <c r="I18" t="n">
+        <v>21681</v>
+      </c>
+      <c r="J18" t="n">
+        <v>4</v>
+      </c>
+      <c r="K18" t="n">
+        <v>40</v>
+      </c>
+      <c r="L18" t="n">
+        <v>-0.136</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="N18" t="n">
+        <v>36</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.408</v>
+      </c>
+      <c r="P18" t="n">
+        <v>-0.054</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>6.614</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>The S&amp;P 500 is back at a record high and the Dow just hit 54,000 | CNN Business - CNN</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE9sNTR6eTFUS1JYX1lnaWVIZGxJeVhmbENJMHN3SUc4TTlSaHpweUdwNUNLejJtSmIwb0x0SEQxalc2OVN1X2s1WFhPSWt2X2VrcFFVeXhVVVpxYVVnaUFjRDR3SUFxbzA?oc=5</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 ends higher as strong inflation data cements rate-hike bets - Reuters</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQOTZpMXRyVmxGMjJTRmVVOV91TnZIWlJsZS1BNlE3bENxRlRlVnh2RFZKQmdwUVNydUJQd1RvZlZLam1KbnR2ZS1Vd2VNaWhrN3lNZ3hETUtvcTVxYTFEOENQQ292eWk0YXJYYjBrekoycE5sU0FqdloxRXNZcTcyd1dnYkFEdGpmMV9Pd0lwemdYWmd0aHZaYmpkWmlLOFgxdnc?oc=5</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>SpaceX Stock Breaks Out 7% as Charter Mobile Talks and $4.3B Nasdaq-100 Buying Fuel Rally - tradingkey.com</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNazNUbDNRRjJfNjIzeDZfMkQxS1NzdlJ3VEpRZFVLQjdLZC1fWFBheUpjbF9xNGtpQTdEbE9JX0VFNVByelBKdW82R0ZyVDJGcVRsTlJocmxIZVdUelYycUVGQTFRb3FOQ0FEWG5nU3IyMmJUWWNqVkY2MXFjd0pFM0otUFFPWG4tZGE0SXhZb0Myb21ldkE1Q1Zsd2JaNmNqWHRlYUZueTV3ZmEzQXpMdzR3RlVRNEhsUFBtaTdR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>Dow Drops 628, Nasdaq Falls 86, S&amp;P 500 Loses 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOdElkenZMSDNpN1JfQ3VrQVBPYjBzTVgyOVNrRFVCX2JBWXk3WFRtb3hrLTFUbUlpTHNwbWsyX0tjY0RFMmFwOFNPTk42OEtzbWZPTkh0TXBGR2RRdHU1c3Zkd2g5Z2p5ckdqMVVMUElCeWstcEd4X3IxWWFUbGlPQVlnV3lYeWdneVZja05ueW8?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-14T08:52:00+00:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>77646.46090000001</v>
+      </c>
+      <c r="F19" t="n">
+        <v>77916.75</v>
+      </c>
+      <c r="G19" t="n">
+        <v>77338.50780000001</v>
+      </c>
+      <c r="H19" t="n">
+        <v>77652.21090000001</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2394064896</v>
+      </c>
+      <c r="J19" t="n">
+        <v>4</v>
+      </c>
+      <c r="K19" t="n">
+        <v>38</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="N19" t="n">
+        <v>38</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="P19" t="n">
+        <v>-0.091</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Bitmine Surges 8% on Ethereum Strength After Cantor Fitzgerald Doubles Its Target, SharpLink Advances 9%, Strategy Gains 4% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPemN4ODV3YldjcDUxb1FRWXc1OWV4bXZwVEhOWTMtbDJaNG92V0xpd0V6OTBxM3lRN0RZUEtWQkRWQW9Kb0hNUF8zS2FBOU5BUlpFTmpvNFBiYnpSVEhHMmtCU2JMdzNjRlNXRWtwaUM1eUxrVjRWQ3VQT2Q4MVJHaHBfdHBRUFpETTVnT012dEJQQV9mcHNOOHUwQnlVU2ZibW51TTBzMHdvTXhsQnlMMzJjT0lhcTNvVktGLTVfN1o3ZXlkLV9JNWRZVVFvakVaaDdIMGxWdFJXUVMxT19rREpueFJibmw0WllRUDk1ckgwUHB1?oc=5</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>Strategy's $200M Bitcoin sale didn't drop prices, signaling strong market demand. - Pluang</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQZ2stY3N4T3I2NU50Q3d2cUVaSUJYWUg5aGc4cnlmZmgtMi16cGVISVZaaWNqTmhLRnhqSkU4bVlkeGpZMmtlMVRUQ1FjV0FhX044amFzR3NhYWY2TW5NU0VqLVdvclo5d3d3Rm43YnZfR1kwQXgycU92ZWpSbDQyMFZIT1lhdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Current price of Bitcoin for September 11, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTFBzdXZINHB2Z3h2a3pmd3JQUFY5TlRvZk8zcnhBdGxUQ2FDb3BiZWNiREprRGRscFViVUhhNTI0VXE5NWxDandwN1JOazJLeWt0YWVpTmJCRkdHRUdtQVVMNTQ4RWhuQVU?oc=5</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-14 09:41 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD19"/>
+  <dimension ref="A1:AD25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2726,6 +2726,762 @@
         </is>
       </c>
       <c r="AD19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-14T09:39:43+00:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>4377.8999</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4379.2998</v>
+      </c>
+      <c r="G20" t="n">
+        <v>4320.1001</v>
+      </c>
+      <c r="H20" t="n">
+        <v>4326.8999</v>
+      </c>
+      <c r="I20" t="n">
+        <v>20800</v>
+      </c>
+      <c r="J20" t="n">
+        <v>4</v>
+      </c>
+      <c r="K20" t="n">
+        <v>39</v>
+      </c>
+      <c r="L20" t="n">
+        <v>-0.104</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="N20" t="n">
+        <v>40</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>Founders Metals (TSXV:FDR) Falls 5.65% as Profit-Taking Tests Strong Antino Gold Momentum - kalkine.ca</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQWjZmSkNZV2p0c3pfYWd1Y2U0NnVtdlNaTGdEU3dDbEZ1QTV2WVZCUXp2bmZFVE5ETHByVmc4R1lBUFlDU2JsejNyNkNCcEk3R2lUQUpPbnl5ZS1aeWZGN0lISTVocl9leXVOdTBrN2dKdGJyVl85N0pUQlFtaEZvTXF3V2MzU0xNcTFydU5fNWZsamhnNDVqSThhVEVuaHYweTI5c1g3ZDlDOWplQl8zVGJqa3JnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-14T09:39:43+00:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>102.22</v>
+      </c>
+      <c r="F21" t="n">
+        <v>103.83</v>
+      </c>
+      <c r="G21" t="n">
+        <v>101.94</v>
+      </c>
+      <c r="H21" t="n">
+        <v>102.83</v>
+      </c>
+      <c r="I21" t="n">
+        <v>38334</v>
+      </c>
+      <c r="J21" t="n">
+        <v>4</v>
+      </c>
+      <c r="K21" t="n">
+        <v>40</v>
+      </c>
+      <c r="L21" t="n">
+        <v>-0.007</v>
+      </c>
+      <c r="M21" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="N21" t="n">
+        <v>40</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="P21" t="n">
+        <v>-0.158</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>4.834</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>US Dollar Gains as Oil Rally and AI Concerns Hit Risk Appetite - Investing.com</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNYnpIU2MtQ09aemlJcXpnMlNqNURRVFU3R2xmekhQcE9CODZEOE9wWFN5MlpDNmtjYVVpSjJ5N2pCZFllb0pkbVlQamw2Z1pGNHhpRENHVGpUelBCa1pZS0xrVXJLdnJkOUk2a2JKTHdPSC0ydVpkOVFZeDAxcndKM2lNWTJqYnhjYXZkMHR3bHRBZWlOWjJYcnNnVDNaeXNGckJ4ejhGRUlqRjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Current price of oil as of July 30, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9odGxncTZBdXJrcnd4Zm1GSENJSFpJQUJxbGphdTV2dTRfQTVmMzVFQ21PTGhzY19DSGVFUWpoeEtGMDZhNzRveUNoaDBlcDVLSmRpaFh6ZnA1emJSVllSYTNR?oc=5</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Oil's roundtrip back to $100. Why China could determine what happens next - CNBC</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOa0xDNl91YjR4WVVvTXU5UlVvMnVQWUs0SDVCRFZFV0VxWVJzLVdsTWZuN1RiSjkxamJwdUkyVUdzZndiTXlITFdQWEVrSzJmSjN1bkczVjhhRktQSHR1UlMzMUtRalJZbmtLbDAtX0FJb1Ntb213dXFxeHMtVXh0NG5sd2ctUVdMWUJDQmF4R1U4V0hQZXQ0WVJDbVBWZDItbXAwbGxiWVFFSGs?oc=5</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>OPEC oil output falls in August, Reuters survey shows - Reuters</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcGZWQVVsSEY1MDZDLXRVM2g2N0t1bHJ1VXpWX3pScTFZak53OGQ5VVNxemw0Mjdrd1paNjRYb1YtdFlYN3RIOURKM00xZmc4eFRlTHk2cTNhODJKWW5TOS1BMEE1cVF2NTN5YjJaeHRRNFlBVHUwUU9CN0pyOEdRMHE0c2VtcGNvamRPVFd3OVVlTnFmV3Fobks2WlZJU21oRW44?oc=5</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>Organization of the Petroleum Exporting Countries - opec.org</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE5TYnpCM2R2ZEh2OGpWR1o3VXRJZjJTQWZMRWMyOGQtUG9JdUxwelZUUjNyWjJteWE5Qmlod3l0dFAtNDBvZVprVGVyRzhZeU9CNndJU041eUtXMzNPdHU1bl8tZS1XVHU0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-14T09:39:43+00:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>99.31399999999999</v>
+      </c>
+      <c r="F22" t="n">
+        <v>99.602</v>
+      </c>
+      <c r="G22" t="n">
+        <v>99.309</v>
+      </c>
+      <c r="H22" t="n">
+        <v>99.53100000000001</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>4</v>
+      </c>
+      <c r="K22" t="n">
+        <v>37</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="N22" t="n">
+        <v>39</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="P22" t="n">
+        <v>-0.118</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>4.825</v>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>US Dollar outlook: Hawkish Fed repricing strengthens the bull case - stonex.com</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNRlJTZ3dmU0NMcWtjQU9uU1pXSDQ1Uk5YOGFCVTQwSlExOFZtcjBGT1VZdXppTkpqYkdoaUtTTWw0aVJxclFIaWFnWXItUzBDTkNNSGg1b0t3dVhvREJSQjJRYUFEMGpMa0pNTVpMUzdpT0YwRngyZi1nMlRCdHJlVjVkc0tvU3RqV2pPNzhtYUNhVXlWVXpPRlpiLXBFTE1KNjZoU2lZLXpUaE9CM0hTLTVRSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>Dovish Fed Bets Pummel Dollar, Boost Gold Ahead of NFP - Investing.com</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPZDNJaUJnTUhOckR3ODFMRjN3M3QtZ1NzUmtvYnRUOVlyWEo2Nzg4d3l5Tkl4SFNRMVJCUnlNeGxUYm5NQkxpNmxEdzVpU3ZHTkhRUXh0bEdhNld2WHFBVmNCRTBEY2dsUkxqVlYtYTUwX21GR1JZNnZjazk2OXBjNW80dWo3Nmx5TXZYLUY0WkZLei14eWV4dDlkRGVheWM?oc=5</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>Q&amp;A on the Dollar Meltdown - Robin J Brooks | Substack</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE1iTlBuOHZORHl4Y0YtclRnalp6NW9kOVhMVVNHX3h5cVM5WjBJdk5vZTd4STQwaHNUNmw5aVE3b1ZWUW0zS19oYnFfMXRCQWhtZjZVbUo2X0cwSVBCcTd3bzJZU0ppOHhnZmJUQXJmUThCRzZV?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-14T09:39:43+00:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>7620</v>
+      </c>
+      <c r="F23" t="n">
+        <v>7624.75</v>
+      </c>
+      <c r="G23" t="n">
+        <v>7593.75</v>
+      </c>
+      <c r="H23" t="n">
+        <v>7601</v>
+      </c>
+      <c r="I23" t="n">
+        <v>64216</v>
+      </c>
+      <c r="J23" t="n">
+        <v>4</v>
+      </c>
+      <c r="K23" t="n">
+        <v>38</v>
+      </c>
+      <c r="L23" t="n">
+        <v>-0.174</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="N23" t="n">
+        <v>40</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.233</v>
+      </c>
+      <c r="P23" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.341</v>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Bitmine Surges 8% on Ethereum Strength After Cantor Fitzgerald Doubles Its Target, SharpLink Advances 9%, Strategy Gains 4% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPemN4ODV3YldjcDUxb1FRWXc1OWV4bXZwVEhOWTMtbDJaNG92V0xpd0V6OTBxM3lRN0RZUEtWQkRWQW9Kb0hNUF8zS2FBOU5BUlpFTmpvNFBiYnpSVEhHMmtCU2JMdzNjRlNXRWtwaUM1eUxrVjRWQ3VQT2Q4MVJHaHBfdHBRUFpETTVnT012dEJQQV9mcHNOOHUwQnlVU2ZibW51TTBzMHdvTXhsQnlMMzJjT0lhcTNvVktGLTVfN1o3ZXlkLV9JNWRZVVFvakVaaDdIMGxWdFJXUVMxT19rREpueFJibmw0WllRUDk1ckgwUHB1?oc=5</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>'Titanic' has a happy ending: Robust rally caps Wall Street's week of red - TradingView</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSG12a01IVVJtakhLMFlscGk0SXRsa0M2UUwtakVNd041MUV0RVdjanozTGlFdWFpZ2dCai10NlYtbW42d3pnQ1lseGdvMGR5VV9USlk0T09WNW93TVhPMVUyUHpQT1ZDLWRBRWdBcHIzbTN4T0VhVVBZb0pzeHlqTEJNS0ZnTXlXUDlTYmRFbHYxYVJWSDQ1THZBSXhIckdURjdPY25wcWc3SXJ2R2pFX1lIVFVoem51RmZDTHhOWkVIRVIwWWdlZE1odzFGTG9DeFo5NHUycw?oc=5</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 11: HPE Surges on AI Infrastructure Demand and Recently Raised Guidance - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxQWHZrbGtuQ2NuRE92NG4temVfd3BnRnJ3ZDJQYlUzZGpBSnFIYWlLQ0VfVks2enFoZGdGamlac3MwdUFCb2JtTmlpV2NhaFFqUzZNQkhPS01ZVGNGTzNHZ05FbVFrWDVHN3F1Mjk1YU1uekRmRWktenpIX1dVQzd5RTJsZ3l2alRmNmxLUWNsY09xQTVJbnc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>Barclays lifts S&amp;P 500 index's year-end target to 7,950 on strong earnings - Reuters</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQdEpJSkhqQ0dZZjZvbFZ3MU9EbGZpa0l4ZjJNazczLTZQTVVfZHlJVmxRVEx3ZFRpLWRwdEhycTRXbGtFdnplbnAwOEgzWG5VQXlYNEdkWE9pVTV0aGl0ZkdsSTBNb1M4U21LWkxPeUVBYWZLTDFZem81OWEtenIwa2E5bjlsdU1Bcmh2SzROZTR2RGFpOVQ4YTRTT21QWXpBX2k2dHV0S3hROHNkYmhR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>Airbus stock rebounds after breaking its 196 € support level - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQTXFjUFRkaWo0Uy1RWThWLU14eFJ3VzF4Z1hyT3ZxMmgzUHdaSWRWSEpCZW1NaXpVU2pQRWxRUVRJT2ExS1FGSHB6VWVOR2pUXzlQUnNhcUxBSjRacjc2bmFHcWNtdmxIWXZHdi1vUjBfeTExYUNHVjROanlpRU5UOGJKeFE3VTY2M2ZzYmNaQVZ1d0xYdlhXVmN1S3BlZUdnRjM1U1FCU0hfUFdsWGIyV0Q0X0tJeDBxTWZwRGZ3?oc=5</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-14T09:39:43+00:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>29014.5</v>
+      </c>
+      <c r="F24" t="n">
+        <v>29037.5</v>
+      </c>
+      <c r="G24" t="n">
+        <v>28816.25</v>
+      </c>
+      <c r="H24" t="n">
+        <v>28856.25</v>
+      </c>
+      <c r="I24" t="n">
+        <v>26957</v>
+      </c>
+      <c r="J24" t="n">
+        <v>4</v>
+      </c>
+      <c r="K24" t="n">
+        <v>40</v>
+      </c>
+      <c r="L24" t="n">
+        <v>-0.197</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="N24" t="n">
+        <v>36</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="P24" t="n">
+        <v>-0.041</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>5.969</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>The S&amp;P 500 is back at a record high and the Dow just hit 54,000 | CNN Business - CNN</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE9sNTR6eTFUS1JYX1lnaWVIZGxJeVhmbENJMHN3SUc4TTlSaHpweUdwNUNLejJtSmIwb0x0SEQxalc2OVN1X2s1WFhPSWt2X2VrcFFVeXhVVVpxYVVnaUFjRDR3SUFxbzA?oc=5</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 ends higher as strong inflation data cements rate-hike bets - Reuters</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQOTZpMXRyVmxGMjJTRmVVOV91TnZIWlJsZS1BNlE3bENxRlRlVnh2RFZKQmdwUVNydUJQd1RvZlZLam1KbnR2ZS1Vd2VNaWhrN3lNZ3hETUtvcTVxYTFEOENQQ292eWk0YXJYYjBrekoycE5sU0FqdloxRXNZcTcyd1dnYkFEdGpmMV9Pd0lwemdYWmd0aHZaYmpkWmlLOFgxdnc?oc=5</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>SpaceX Stock Breaks Out 7% as Charter Mobile Talks and $4.3B Nasdaq-100 Buying Fuel Rally - tradingkey.com</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNazNUbDNRRjJfNjIzeDZfMkQxS1NzdlJ3VEpRZFVLQjdLZC1fWFBheUpjbF9xNGtpQTdEbE9JX0VFNVByelBKdW82R0ZyVDJGcVRsTlJocmxIZVdUelYycUVGQTFRb3FOQ0FEWG5nU3IyMmJUWWNqVkY2MXFjd0pFM0otUFFPWG4tZGE0SXhZb0Myb21ldkE1Q1Zsd2JaNmNqWHRlYUZueTV3ZmEzQXpMdzR3RlVRNEhsUFBtaTdR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>Dow Drops 628, Nasdaq Falls 86, S&amp;P 500 Loses 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOdElkenZMSDNpN1JfQ3VrQVBPYjBzTVgyOVNrRFVCX2JBWXk3WFRtb3hrLTFUbUlpTHNwbWsyX0tjY0RFMmFwOFNPTk42OEtzbWZPTkh0TXBGR2RRdHU1c3Zkd2g5Z2p5ckdqMVVMUElCeWstcEd4X3IxWWFUbGlPQVlnV3lYeWdneVZja05ueW8?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-14T09:39:43+00:00</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>77583.99219999999</v>
+      </c>
+      <c r="F25" t="n">
+        <v>77936.86719999999</v>
+      </c>
+      <c r="G25" t="n">
+        <v>77337.96090000001</v>
+      </c>
+      <c r="H25" t="n">
+        <v>77840.63280000001</v>
+      </c>
+      <c r="I25" t="n">
+        <v>2090127360</v>
+      </c>
+      <c r="J25" t="n">
+        <v>4</v>
+      </c>
+      <c r="K25" t="n">
+        <v>39</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="N25" t="n">
+        <v>38</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.262</v>
+      </c>
+      <c r="P25" t="n">
+        <v>-0.08799999999999999</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>6.573</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - cnbc.com</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>Bitmine Surges 8% on Ethereum Strength After Cantor Fitzgerald Doubles Its Target, SharpLink Advances 9%, Strategy Gains 4% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPemN4ODV3YldjcDUxb1FRWXc1OWV4bXZwVEhOWTMtbDJaNG92V0xpd0V6OTBxM3lRN0RZUEtWQkRWQW9Kb0hNUF8zS2FBOU5BUlpFTmpvNFBiYnpSVEhHMmtCU2JMdzNjRlNXRWtwaUM1eUxrVjRWQ3VQT2Q4MVJHaHBfdHBRUFpETTVnT012dEJQQV9mcHNOOHUwQnlVU2ZibW51TTBzMHdvTXhsQnlMMzJjT0lhcTNvVktGLTVfN1o3ZXlkLV9JNWRZVVFvakVaaDdIMGxWdFJXUVMxT19rREpueFJibmw0WllRUDk1ckgwUHB1?oc=5</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>Strategy's $200M Bitcoin sale didn't drop prices, signaling strong market demand. - Pluang</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQZ2stY3N4T3I2NU50Q3d2cUVaSUJYWUg5aGc4cnlmZmgtMi16cGVISVZaaWNqTmhLRnhqSkU4bVlkeGpZMmtlMVRUQ1FjV0FhX044amFzR3NhYWY2TW5NU0VqLVdvclo5d3d3Rm43YnZfR1kwQXgycU92ZWpSbDQyMFZIT1lhdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Current price of Bitcoin for September 11, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTFBzdXZINHB2Z3h2a3pmd3JQUFY5TlRvZk8zcnhBdGxUQ2FDb3BiZWNiREprRGRscFViVUhhNTI0VXE5NWxDandwN1JOazJLeWt0YWVpTmJCRkdHRUdtQVVMNTQ4RWhuQVU?oc=5</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-14 17:54 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD25"/>
+  <dimension ref="A1:AD31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3484,6 +3484,762 @@
       <c r="AD25" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-14T17:52:18+00:00</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>4312.1001</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4358.8999</v>
+      </c>
+      <c r="G26" t="n">
+        <v>4303.7002</v>
+      </c>
+      <c r="H26" t="n">
+        <v>4351.1001</v>
+      </c>
+      <c r="I26" t="n">
+        <v>46637</v>
+      </c>
+      <c r="J26" t="n">
+        <v>4</v>
+      </c>
+      <c r="K26" t="n">
+        <v>39</v>
+      </c>
+      <c r="L26" t="n">
+        <v>-0.044</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="N26" t="n">
+        <v>40</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.351</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>Wall Street turns bullish on gold price ahead of the Fed, Main Street clings to slim bullish majority despite weekly slide - KITCO</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQM0hVdUNrZEZxdm8xb0RMbzVWdm5wTjkxYW1UR2FjSE42Si1XTEk0Q3Q1eU1BeW00NlF5aWVZc3Zsclk2OWY2V2dlUHNzeC05UWZZTldXdEhHNjN0Y0V6d2RKMUR2elNab0F6WWhFbzNPZGotQk4xeGhOeHJhcU84Z2dnc1BNUVZZY1dQWHBpOU1EeS00ZHZTTFZxMWxfbktzZjliSTRlbm1LQlVDT3dvLUJYMXg4SHc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>Gold and Silver Price Forecast: Will CPI Trigger a Breakdown? - FXEmpire</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQX0xZUzFaNWYtaS1XU244eFRjTkUxSGlqTHh4aWVXSkRBWU4yOERmd3k3OGN4eUVnUGRLVUFzX1JNTk51WlZfZzFBWnphRHpWNm1wSlBLS0RSZmlLUzFoVUhZcjdGTXpWMlBjbHlGYkJTM0xZMFRhTEp0YWRsRFUxZ0FxNkdKVkt4TXJEcERKUTI5WVJIVmp4bW5iUDVpRm1TeFh6eHc5ZFFJTU1hNEtV?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-14T17:52:18+00:00</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="F27" t="n">
+        <v>104.51</v>
+      </c>
+      <c r="G27" t="n">
+        <v>100.79</v>
+      </c>
+      <c r="H27" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="I27" t="n">
+        <v>147584</v>
+      </c>
+      <c r="J27" t="n">
+        <v>4</v>
+      </c>
+      <c r="K27" t="n">
+        <v>40</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="M27" t="n">
+        <v>-0.257</v>
+      </c>
+      <c r="N27" t="n">
+        <v>40</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0.143</v>
+      </c>
+      <c r="P27" t="n">
+        <v>-0.157</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>3.242</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>US Dollar Gains as Oil Rally and AI Concerns Hit Risk Appetite - Investing.com</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNYnpIU2MtQ09aemlJcXpnMlNqNURRVFU3R2xmekhQcE9CODZEOE9wWFN5MlpDNmtjYVVpSjJ5N2pCZFllb0pkbVlQamw2Z1pGNHhpRENHVGpUelBCa1pZS0xrVXJLdnJkOUk2a2JKTHdPSC0ydVpkOVFZeDAxcndKM2lNWTJqYnhjYXZkMHR3bHRBZWlOWjJYcnNnVDNaeXNGckJ4ejhGRUlqRjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>London Gas Oil breaks resistance at $1,273: Live levels By Investing.com - Investing.com India</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQOFJZcEZXSVpGOEZvTVR0SGRqYmZ4WF9SZ3RKajNUVWZDM2t3U3BOa3lQWk1oMUpnOF9UTTk0eFpwdzR0TEVzbHlHelFkb0xxZ3lFX08tR0gyblJWX20xenlXMi0xNVFfSlJ4UDdVUWtZcW5hV19VRHZIS0taRmRDRzlOek1wb2hmR3lpMGhGS0ZwbVVVZ0p4NFhibHBOTkdrd0JpWnVpSDl1dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>Gold Falls Rs 500 On Crude Surge, Strong Dollar - Deccan Chronicle</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQRHE1SGJkVHZuWUdXNThqeG1mNl9VaGRpZTJmMHJCX09hYnF0UkZwcXgtWUowdzFDYkxTb3VUSmdUSVdpRW4xMzNwTkVTZFVzUDdLcE9oWVJrUlc5RE1oa0VyY0ZCUkcyV2ZSREVJNkNXM2xsVk9lY2lCeFFDOFcyYW5ieGt4N0hqU293OFV3T01lVXpIWVU3eHdYR0c1cGdORU1JOWFzcmrSAa4BQVVfeXFMUFRZQXR2RU5ybDg3YUd0eVVsekgtMnZkYTBKRlZRdVRIWXZJajdQVmoxajBoX3J2d1pibHZpaVBvbFJ0ZDFwX2toR0k0ajEtTFpFU01RNEhqMDlNMk1iUkdDbVU1OHlzR193MVJiSl9ZLVZ0dkFJNkk1NE92MTVLOHZ4aVkzaDNCdlFtcUlBYm1FYlNmRUpjLU0zanlCVWNHWVlXVzJnX0NfbVZxdEdB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>OPEC oil output falls in August, Reuters survey shows - Reuters</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcGZWQVVsSEY1MDZDLXRVM2g2N0t1bHJ1VXpWX3pScTFZak53OGQ5VVNxemw0Mjdrd1paNjRYb1YtdFlYN3RIOURKM00xZmc4eFRlTHk2cTNhODJKWW5TOS1BMEE1cVF2NTN5YjJaeHRRNFlBVHUwUU9CN0pyOEdRMHE0c2VtcGNvamRPVFd3OVVlTnFmV3Fobks2WlZJU21oRW44?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-14T17:52:18+00:00</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>99.717</v>
+      </c>
+      <c r="F28" t="n">
+        <v>99.72799999999999</v>
+      </c>
+      <c r="G28" t="n">
+        <v>99.374</v>
+      </c>
+      <c r="H28" t="n">
+        <v>99.44</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>4</v>
+      </c>
+      <c r="K28" t="n">
+        <v>38</v>
+      </c>
+      <c r="L28" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="N28" t="n">
+        <v>39</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="P28" t="n">
+        <v>-0.116</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>2.653</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>US Dollar outlook: Hawkish Fed repricing strengthens the bull case - stonex.com</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNRlJTZ3dmU0NMcWtjQU9uU1pXSDQ1Uk5YOGFCVTQwSlExOFZtcjBGT1VZdXppTkpqYkdoaUtTTWw0aVJxclFIaWFnWXItUzBDTkNNSGg1b0t3dVhvREJSQjJRYUFEMGpMa0pNTVpMUzdpT0YwRngyZi1nMlRCdHJlVjVkc0tvU3RqV2pPNzhtYUNhVXlWVXpPRlpiLXBFTE1KNjZoU2lZLXpUaE9CM0hTLTVRSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>Million dollar winning scratch-off sold at Lackawanna County retailer - WNEP</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxPcXdKdTBCNFlfRzZyX1dDbllTXzQzQk9xMktmTVRlSFF2Q3RmOXV0V3A3Tlh2dzY1X09pdm9TSjRjYzNPZXYwTl95U3NRdl9qNUVUM29DZ0RqSmlqeHdsbWlwV25vVmpxWGZTd3VZX0FwUjhmaUVGSDhBZ2pVMGtycEoxNkNBeFhIMFFVN0hBbUg4Q0tQeVM0ZVU5WkxoNUoyZXh6LTJXRHNEaUZZbzRLMnF6YlFBbHFCR3pDUXA1RDMyeWUwbl9fYTdNNEc2M3U5NDZ3cUZSb1BXWmdrOVN6dVU1WlAxS2N6YUI3RjAtdjJuYjNRVzFPdHh5TmQyeXdWMUxZ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>Dovish Fed Bets Pummel Dollar, Boost Gold Ahead of NFP - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPZDNJaUJnTUhOckR3ODFMRjN3M3QtZ1NzUmtvYnRUOVlyWEo2Nzg4d3l5Tkl4SFNRMVJCUnlNeGxUYm5NQkxpNmxEdzVpU3ZHTkhRUXh0bEdhNld2WHFBVmNCRTBEY2dsUkxqVlYtYTUwX21GR1JZNnZjazk2OXBjNW80dWo3Nmx5TXZYLUY0WkZLei14eWV4dDlkRGVheWM?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-14T17:52:18+00:00</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>7615.75</v>
+      </c>
+      <c r="F29" t="n">
+        <v>7719.75</v>
+      </c>
+      <c r="G29" t="n">
+        <v>7595.25</v>
+      </c>
+      <c r="H29" t="n">
+        <v>7710.5</v>
+      </c>
+      <c r="I29" t="n">
+        <v>997518</v>
+      </c>
+      <c r="J29" t="n">
+        <v>4</v>
+      </c>
+      <c r="K29" t="n">
+        <v>38</v>
+      </c>
+      <c r="L29" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="N29" t="n">
+        <v>39</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0.136</v>
+      </c>
+      <c r="P29" t="n">
+        <v>-0.059</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>-1.651</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Tax revenue surges amid boom in stock market - Taipei Times</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBVYTNZQ2Q4RFRxNEVSUnVLLTZRQUkyVjF1dEtOZ0hiZ1NreVV3NUx1b1RXdWNoRXZIWlB6MnhXakR3SFdvTGt5SG1NZWFLVjZrUGd4MXk0dVEzRkY5NGJkTUtWSmtwalA5RWlLXzQyVGMwN2pjcEE?oc=5</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>C3.ai Jumps 7% as Software Rally Lifts Beaten-Down AI Names; UiPath Climbs 8%, SoundHound AI Gains 5% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNZVhGa3hKakF5UFBTNTRkLUNCcGF6WXZiaF84aUNHbUhWeHlLbUR4NEhpU2FKZGZOTXFpZUpLZjd1aHQ2V3doTk5pWE9yNjB2VmdvcEc1SllGQm9JMk1sWkFhSXBFeTZZUFpyT1lyTTdNZllaVXdBalRSeW54MzM1WnB4YzUtXzh3aGwybWR6V1B1b2pJWFlNWmp3ZTdWYUM2OElIdFljRDhVV21LQnAxcGxZbnZob2FEbWtMMWdXeEU5WGQydHpLZEJ4U1dWR2o4QmJkVnRkbw?oc=5</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>'Titanic' has a happy ending: Robust rally caps Wall Street's week of red - TradingView</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSG12a01IVVJtakhLMFlscGk0SXRsa0M2UUwtakVNd041MUV0RVdjanozTGlFdWFpZ2dCai10NlYtbW42d3pnQ1lseGdvMGR5VV9USlk0T09WNW93TVhPMVUyUHpQT1ZDLWRBRWdBcHIzbTN4T0VhVVBZb0pzeHlqTEJNS0ZnTXlXUDlTYmRFbHYxYVJWSDQ1THZBSXhIckdURjdPY25wcWc3SXJ2R2pFX1lIVFVoem51RmZDTHhOWkVIRVIwWWdlZE1odzFGTG9DeFo5NHUycw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>Barclays lifts S&amp;P 500 index's year-end target to 7,950 on strong earnings - Reuters</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQdEpJSkhqQ0dZZjZvbFZ3MU9EbGZpa0l4ZjJNazczLTZQTVVfZHlJVmxRVEx3ZFRpLWRwdEhycTRXbGtFdnplbnAwOEgzWG5VQXlYNEdkWE9pVTV0aGl0ZkdsSTBNb1M4U21LWkxPeUVBYWZLTDFZem81OWEtenIwa2E5bjlsdU1Bcmh2SzROZTR2RGFpOVQ4YTRTT21QWXpBX2k2dHV0S3hROHNkYmhR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Airbus stock rebounds after breaking its 196 € support level - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQTXFjUFRkaWo0Uy1RWThWLU14eFJ3VzF4Z1hyT3ZxMmgzUHdaSWRWSEpCZW1NaXpVU2pQRWxRUVRJT2ExS1FGSHB6VWVOR2pUXzlQUnNhcUxBSjRacjc2bmFHcWNtdmxIWXZHdi1vUjBfeTExYUNHVjROanlpRU5UOGJKeFE3VTY2M2ZzYmNaQVZ1d0xYdlhXVmN1S3BlZUdnRjM1U1FCU0hfUFdsWGIyV0Q0X0tJeDBxTWZwRGZ3?oc=5</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-14T17:52:18+00:00</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>29003.5</v>
+      </c>
+      <c r="F30" t="n">
+        <v>29585.75</v>
+      </c>
+      <c r="G30" t="n">
+        <v>28955.75</v>
+      </c>
+      <c r="H30" t="n">
+        <v>29584</v>
+      </c>
+      <c r="I30" t="n">
+        <v>230252</v>
+      </c>
+      <c r="J30" t="n">
+        <v>4</v>
+      </c>
+      <c r="K30" t="n">
+        <v>40</v>
+      </c>
+      <c r="L30" t="n">
+        <v>-0.178</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="N30" t="n">
+        <v>34</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="P30" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>S&amp;P and Nasdaq hit record highs, continuing remarkable recovery from war shock - CNN</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBFM0dLbkRoQTEzbmVyNGdlZERORGZXdEJrOVh3U0FZVnJsNk0zQjFWVVF6a0NhQThTbS0zMUJTdmdHWm1JYVF3LW5VUWVJWFk1MUd6WlVNWU9aa0dENG9rbkYzRDFpcmhSQ1BJ?oc=5</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Cybersecurity is one corner of the tech market that's getting a boost from AI doomsday fears - Business Insider</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOUkdOM3BPSE8xMS0yWndCcE1aSzd0a3FXOUxIa0tGU3hZMDZ0WGtUODdqVEIwSWkyMnU4d3hIN0ZtZ0NiVmhFc25DM3lkS2kyMXMtUHNwOUdsRll1LUg0VWU5NWFsekZsOXF5M2hBdVhBOTJnYXpnd21Ga1JpUG83RmZfcWNHLWFwQUk2NGd0WjhxMDRrUnhmVkZYSXlmbEsyTkxMV3NwR1MydXkx?oc=5</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>The S&amp;P 500 is back at a record high and the Dow just hit 54,000 | CNN Business - CNN</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE9sNTR6eTFUS1JYX1lnaWVIZGxJeVhmbENJMHN3SUc4TTlSaHpweUdwNUNLejJtSmIwb0x0SEQxalc2OVN1X2s1WFhPSWt2X2VrcFFVeXhVVVpxYVVnaUFjRDR3SUFxbzA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>Wall St falls as AI anxiety batters Nvidia, chipmakers - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPLUFFaDBPNXQyQ3J4aUp3M3NsenNDMWU2SFRVQUhseDZTcHdMVTZSLVZ1dFBXZUNDcnROWHdxM2c0N0N5QW9xbVVWUWZ4ZnV0R1hVWmhWd0xyMWpWRUxpWHVYR093bVRERmlIb2pFYWJ5NzNxcU1kNzVReDFiOWZWcnVad01fS0xMSlZWRWhkVm1MUmR0Uk5VUHRQOGw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>Wall St falls as AI anxiety batters Nvidia, chipmakers - Reuters</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQYVB5TUc4VTc5MGdNMjVWcVYxUUszYjdXU3hrVnZXbVRCRm40Z3JBX3BhTElKaXVFQmU4SW82WWRwLVdxcGFTVVhPclllM25kSzR0MWdqUmU5YjQydl9MZDhLZ1MzQmF0b01UY3MxaWx0VkxOMjJUQzhmbHJPQjQzdXJMWkJ2OGs5R0ZQc2FjeVpEdjZkM2VqMC1aeGhXSm8?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-14T17:52:18+00:00</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>78145.9531</v>
+      </c>
+      <c r="F31" t="n">
+        <v>78992.3594</v>
+      </c>
+      <c r="G31" t="n">
+        <v>78145.9531</v>
+      </c>
+      <c r="H31" t="n">
+        <v>78977.8594</v>
+      </c>
+      <c r="I31" t="n">
+        <v>4754268160</v>
+      </c>
+      <c r="J31" t="n">
+        <v>4</v>
+      </c>
+      <c r="K31" t="n">
+        <v>39</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0.08799999999999999</v>
+      </c>
+      <c r="N31" t="n">
+        <v>37</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="P31" t="n">
+        <v>-0.177</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>6.851</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>Bitmine Surges 8% on Ethereum Strength After Cantor Fitzgerald Doubles Its Target, SharpLink Advances 9%, Strategy Gains 4% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPemN4ODV3YldjcDUxb1FRWXc1OWV4bXZwVEhOWTMtbDJaNG92V0xpd0V6OTBxM3lRN0RZUEtWQkRWQW9Kb0hNUF8zS2FBOU5BUlpFTmpvNFBiYnpSVEhHMmtCU2JMdzNjRlNXRWtwaUM1eUxrVjRWQ3VQT2Q4MVJHaHBfdHBRUFpETTVnT012dEJQQV9mcHNOOHUwQnlVU2ZibW51TTBzMHdvTXhsQnlMMzJjT0lhcTNvVktGLTVfN1o3ZXlkLV9JNWRZVVFvakVaaDdIMGxWdFJXUVMxT19rREpueFJibmw0WllRUDk1ckgwUHB1?oc=5</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Seven assets enter Kraken liquidation window after withdrawals close Monday - CryptoSlate</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxORVd0T3hNS0lyVG54R1kzcXpndG5yQ0N0bHNFODlZQXBwZ0NlUy13cmFwWlN4QzlZU3pFMlZwZzUtMHBsQnZXT2NXZlhodmI0VmpRczdRajRkbjU5VEVmWWlWeEpzTUVvcUtOTTdraXFadkhuaFNLbXZlSlcxeTlrYnhleE1mWUhQVUZUS0lJYzRJdEhNeUhVRUg4VHBidVN6Mnc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>Short squeeze sends Bitcoin to $72,000 and erases $1.6 billion - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQZW1XSk9xaTJRRmdNUnJoV3NXZ2t3RnZYdHg5NUVnc0U5Zk8wQmFtYWhvSVVScVFSRFlGbXl6dWh6Y19tN1pFZ3RwY0NseFhQYWF5S0ljNlB2c2wyZDRqNGlFLTFod1dtTzJYeFdNaEZuNEJCaVZJMW1sdW9ZUXJhcVFXa1hmcUJlWDgyQUdLWlJRX25mNkprSGFFQQ?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-14 23:02 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD31"/>
+  <dimension ref="A1:AD37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4238,6 +4238,762 @@
         </is>
       </c>
       <c r="AD31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQZW1XSk9xaTJRRmdNUnJoV3NXZ2t3RnZYdHg5NUVnc0U5Zk8wQmFtYWhvSVVScVFSRFlGbXl6dWh6Y19tN1pFZ3RwY0NseFhQYWF5S0ljNlB2c2wyZDRqNGlFLTFod1dtTzJYeFdNaEZuNEJCaVZJMW1sdW9ZUXJhcVFXa1hmcUJlWDgyQUdLWlJRX25mNkprSGFFQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:00:40+00:00</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>4351.7002</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4356.7002</v>
+      </c>
+      <c r="G32" t="n">
+        <v>4322.7998</v>
+      </c>
+      <c r="H32" t="n">
+        <v>4336.7998</v>
+      </c>
+      <c r="I32" t="n">
+        <v>17262</v>
+      </c>
+      <c r="J32" t="n">
+        <v>4</v>
+      </c>
+      <c r="K32" t="n">
+        <v>39</v>
+      </c>
+      <c r="L32" t="n">
+        <v>-0.092</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="N32" t="n">
+        <v>40</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0.491</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>Founders Metals (TSXV:FDR) Falls 5.65% as Profit-Taking Tests Strong Antino Gold Momentum - kalkine.ca</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQWjZmSkNZV2p0c3pfYWd1Y2U0NnVtdlNaTGdEU3dDbEZ1QTV2WVZCUXp2bmZFVE5ETHByVmc4R1lBUFlDU2JsejNyNkNCcEk3R2lUQUpPbnl5ZS1aeWZGN0lISTVocl9leXVOdTBrN2dKdGJyVl85N0pUQlFtaEZvTXF3V2MzU0xNcTFydU5fNWZsamhnNDVqSThhVEVuaHYweTI5c1g3ZDlDOWplQl8zVGJqa3JnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - fxstreet.com</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:00:40+00:00</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>101.71</v>
+      </c>
+      <c r="F33" t="n">
+        <v>102.08</v>
+      </c>
+      <c r="G33" t="n">
+        <v>100.53</v>
+      </c>
+      <c r="H33" t="n">
+        <v>101.94</v>
+      </c>
+      <c r="I33" t="n">
+        <v>60770</v>
+      </c>
+      <c r="J33" t="n">
+        <v>4</v>
+      </c>
+      <c r="K33" t="n">
+        <v>40</v>
+      </c>
+      <c r="L33" t="n">
+        <v>-0.055</v>
+      </c>
+      <c r="M33" t="n">
+        <v>-0.283</v>
+      </c>
+      <c r="N33" t="n">
+        <v>40</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.156</v>
+      </c>
+      <c r="P33" t="n">
+        <v>-0.114</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>2.038</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>US Dollar Gains as Oil Rally and AI Concerns Hit Risk Appetite - Investing.com</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNYnpIU2MtQ09aemlJcXpnMlNqNURRVFU3R2xmekhQcE9CODZEOE9wWFN5MlpDNmtjYVVpSjJ5N2pCZFllb0pkbVlQamw2Z1pGNHhpRENHVGpUelBCa1pZS0xrVXJLdnJkOUk2a2JKTHdPSC0ydVpkOVFZeDAxcndKM2lNWTJqYnhjYXZkMHR3bHRBZWlOWjJYcnNnVDNaeXNGckJ4ejhGRUlqRjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>Oil's roundtrip back to $100. Why China could determine what happens next - CNBC</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOa0xDNl91YjR4WVVvTXU5UlVvMnVQWUs0SDVCRFZFV0VxWVJzLVdsTWZuN1RiSjkxamJwdUkyVUdzZndiTXlITFdQWEVrSzJmSjN1bkczVjhhRktQSHR1UlMzMUtRalJZbmtLbDAtX0FJb1Ntb213dXFxeHMtVXh0NG5sd2ctUVdMWUJDQmF4R1U4V0hQZXQ0WVJDbVBWZDItbXAwbGxiWVFFSGs?oc=5</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>Gold Falls Rs 500 On Crude Surge, Strong Dollar - Deccan Chronicle</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQRHE1SGJkVHZuWUdXNThqeG1mNl9VaGRpZTJmMHJCX09hYnF0UkZwcXgtWUowdzFDYkxTb3VUSmdUSVdpRW4xMzNwTkVTZFVzUDdLcE9oWVJrUlc5RE1oa0VyY0ZCUkcyV2ZSREVJNkNXM2xsVk9lY2lCeFFDOFcyYW5ieGt4N0hqU293OFV3T01lVXpIWVU3eHdYR0c1cGdORU1JOWFzcmrSAa4BQVVfeXFMUFRZQXR2RU5ybDg3YUd0eVVsekgtMnZkYTBKRlZRdVRIWXZJajdQVmoxajBoX3J2d1pibHZpaVBvbFJ0ZDFwX2toR0k0ajEtTFpFU01RNEhqMDlNMk1iUkdDbVU1OHlzR193MVJiSl9ZLVZ0dkFJNkk1NE92MTVLOHZ4aVkzaDNCdlFtcUlBYm1FYlNmRUpjLU0zanlCVWNHWVlXVzJnX0NfbVZxdEdB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>OPEC oil output falls in August, Reuters survey shows - Reuters</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcGZWQVVsSEY1MDZDLXRVM2g2N0t1bHJ1VXpWX3pScTFZak53OGQ5VVNxemw0Mjdrd1paNjRYb1YtdFlYN3RIOURKM00xZmc4eFRlTHk2cTNhODJKWW5TOS1BMEE1cVF2NTN5YjJaeHRRNFlBVHUwUU9CN0pyOEdRMHE0c2VtcGNvamRPVFd3OVVlTnFmV3Fobks2WlZJU21oRW44?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:00:40+00:00</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>99.39100000000001</v>
+      </c>
+      <c r="F34" t="n">
+        <v>99.517</v>
+      </c>
+      <c r="G34" t="n">
+        <v>99.39100000000001</v>
+      </c>
+      <c r="H34" t="n">
+        <v>99.467</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>4</v>
+      </c>
+      <c r="K34" t="n">
+        <v>38</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="N34" t="n">
+        <v>40</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="P34" t="n">
+        <v>-0.114</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>3.573</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - moomoo.com</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>US Dollar outlook: Hawkish Fed repricing strengthens the bull case - stonex.com</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNRlJTZ3dmU0NMcWtjQU9uU1pXSDQ1Uk5YOGFCVTQwSlExOFZtcjBGT1VZdXppTkpqYkdoaUtTTWw0aVJxclFIaWFnWXItUzBDTkNNSGg1b0t3dVhvREJSQjJRYUFEMGpMa0pNTVpMUzdpT0YwRngyZi1nMlRCdHJlVjVkc0tvU3RqV2pPNzhtYUNhVXlWVXpPRlpiLXBFTE1KNjZoU2lZLXpUaE9CM0hTLTVRSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - fxstreet.com</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - mufgresearch.com</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>Million dollar winning scratch-off sold at Lackawanna County retailer - WNEP</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxPcXdKdTBCNFlfRzZyX1dDbllTXzQzQk9xMktmTVRlSFF2Q3RmOXV0V3A3Tlh2dzY1X09pdm9TSjRjYzNPZXYwTl95U3NRdl9qNUVUM29DZ0RqSmlqeHdsbWlwV25vVmpxWGZTd3VZX0FwUjhmaUVGSDhBZ2pVMGtycEoxNkNBeFhIMFFVN0hBbUg4Q0tQeVM0ZVU5WkxoNUoyZXh6LTJXRHNEaUZZbzRLMnF6YlFBbHFCR3pDUXA1RDMyeWUwbl9fYTdNNEc2M3U5NDZ3cUZSb1BXWmdrOVN6dVU1WlAxS2N6YUI3RjAtdjJuYjNRVzFPdHh5TmQyeXdWMUxZ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:00:40+00:00</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>7707.5</v>
+      </c>
+      <c r="F35" t="n">
+        <v>7712.25</v>
+      </c>
+      <c r="G35" t="n">
+        <v>7689.5</v>
+      </c>
+      <c r="H35" t="n">
+        <v>7698.25</v>
+      </c>
+      <c r="I35" t="n">
+        <v>424336</v>
+      </c>
+      <c r="J35" t="n">
+        <v>4</v>
+      </c>
+      <c r="K35" t="n">
+        <v>38</v>
+      </c>
+      <c r="L35" t="n">
+        <v>-0.409</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="N35" t="n">
+        <v>38</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="P35" t="n">
+        <v>-0.08599999999999999</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>-5.733</v>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Tax revenue surges amid boom in stock market - Taipei Times</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBVYTNZQ2Q4RFRxNEVSUnVLLTZRQUkyVjF1dEtOZ0hiZ1NreVV3NUx1b1RXdWNoRXZIWlB6MnhXakR3SFdvTGt5SG1NZWFLVjZrUGd4MXk0dVEzRkY5NGJkTUtWSmtwalA5RWlLXzQyVGMwN2pjcEE?oc=5</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Wall Street hits record as S&amp;P 500 continues 2-week rally, boosted by hopes for Iran war's end - PBS</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQS3kycm9PYWZzVnJiVllILUtRZlFlN19waWNzNG9hNXNReGNLRkJSdnpfNmdjaTZhTk1CdGM2THJIVlJ1RmZTc0VNS2ZvT2Rmc3JndlZWS1ItMWM0RG93X3ZjdUQ4anZJMENjXzhjaWtpVzdNTTBXbHlXd2RTR1M2WF96ZlFscVRoSXBxcjlVdE9OSFRTaDk4NmJFTGItZnJ6Y3JiVHhZMEw4NXVYZ3ZNb1V5OTFmdDhTVHNheXZ0RE9Lb1ZZRHd30gHMAUFVX3lxTE5od2ZpbkRoY2pjaG1DcVRKTVlRaUZBY0p5a2hpUDMtTFhab0ZzWG5teFZIQUNldDNoWHV0T0dsOHhFMjZGckxEMW5kZUpULXQwMFY2OFJwX2RmUFZTeVRPcW5DYmxYcFUtdXpRNlJCLWR4cDB0N2VvUDlFSUJjYXlxME9tT01sNmxDZ3JDanlOc2QySllnU3FPNmEwakJnOWFxVVhGYVNJMl9nUVk0a1B1N3N3TTBSNVo4MmhkZGFCNEloa3NkczBlS05aNA?oc=5</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>Illumina Stock Analysis: Bullish Trend Holds, Momentum in Focus - The Cryptonomist</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQaUstS2lxb25wVWhUUm9ZZjM4WUpYekk3Mk1VVjdHYWdaZUE2alhkXzVKMXlOOHZ0ekVOSE5EWXYtS1o2QjFyVGVockpyVWZPVXdhUTNsSFcyMEE5aFZqb0l4M045T3Z4cnNuU2t4ckpBYTNmZEhGZWstVlV2YlkzQW0zSkpNYUtzeTRYZ2NrMG9nWDhwQ0x2QTZsNVg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>Barclays lifts S&amp;P 500 index's year-end target to 7,950 on strong earnings - Reuters</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQdEpJSkhqQ0dZZjZvbFZ3MU9EbGZpa0l4ZjJNazczLTZQTVVfZHlJVmxRVEx3ZFRpLWRwdEhycTRXbGtFdnplbnAwOEgzWG5VQXlYNEdkWE9pVTV0aGl0ZkdsSTBNb1M4U21LWkxPeUVBYWZLTDFZem81OWEtenIwa2E5bjlsdU1Bcmh2SzROZTR2RGFpOVQ4YTRTT21QWXpBX2k2dHV0S3hROHNkYmhR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>Cramer: This market has eerie parallels with 2018. Here's what investors should do - CNBC</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQODBLSzhYc0tERGFFMFpBa2lJU0IzX0JTM3d3amdHTFhRTVktNHhPeXhOOXJqeHRNOVpYNHpmTnhlTy00T29uYTBneXN4MjBvY2h0dm01VDVnOTJTOEV3Zk41Z1gwMDNKZXJDV19FY05sSWlOTk1iZV9mSEREczZrcjBnVWkzUnp6RFZtMGRKVGtTTERVRU9IR095TEhtZDZh0gGmAUFVX3lxTE5GTlVOU0NqMXdnUTVkcmpNTnEweUNWNS1tRjVjUjFZNzlEcHB0X0RSa3lDNXpRbTNYbFV1VmpFTXdSdEdQOE11cEpTVFVtUENfT21mcjhpTmpOamNmbFN2YlUzby1jeUhrM2hTNE5WX0xnTG0wU1JHcVRjRjRLTnJaaTh6M0Q5aFhkbDZXOXZXLUVhcWpIZ2pKX1JCNGM1ZUhRQjc0N1E?oc=5</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>Airbus stock rebounds after breaking its 196 € support level - ideal-investisseur.fr</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQTXFjUFRkaWo0Uy1RWThWLU14eFJ3VzF4Z1hyT3ZxMmgzUHdaSWRWSEpCZW1NaXpVU2pQRWxRUVRJT2ExS1FGSHB6VWVOR2pUXzlQUnNhcUxBSjRacjc2bmFHcWNtdmxIWXZHdi1vUjBfeTExYUNHVjROanlpRU5UOGJKeFE3VTY2M2ZzYmNaQVZ1d0xYdlhXVmN1S3BlZUdnRjM1U1FCU0hfUFdsWGIyV0Q0X0tJeDBxTWZwRGZ3?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:00:40+00:00</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>29582</v>
+      </c>
+      <c r="F36" t="n">
+        <v>29601.25</v>
+      </c>
+      <c r="G36" t="n">
+        <v>29444.5</v>
+      </c>
+      <c r="H36" t="n">
+        <v>29470</v>
+      </c>
+      <c r="I36" t="n">
+        <v>91472</v>
+      </c>
+      <c r="J36" t="n">
+        <v>4</v>
+      </c>
+      <c r="K36" t="n">
+        <v>40</v>
+      </c>
+      <c r="L36" t="n">
+        <v>-0.276</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="N36" t="n">
+        <v>34</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0.321</v>
+      </c>
+      <c r="P36" t="n">
+        <v>-0.053</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>2.936</v>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>S&amp;P and Nasdaq hit record highs, continuing remarkable recovery from war shock - CNN</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBFM0dLbkRoQTEzbmVyNGdlZERORGZXdEJrOVh3U0FZVnJsNk0zQjFWVVF6a0NhQThTbS0zMUJTdmdHWm1JYVF3LW5VUWVJWFk1MUd6WlVNWU9aa0dENG9rbkYzRDFpcmhSQ1BJ?oc=5</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Cybersecurity is one corner of the tech market that's getting a boost from AI doomsday fears - Business Insider</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOUkdOM3BPSE8xMS0yWndCcE1aSzd0a3FXOUxIa0tGU3hZMDZ0WGtUODdqVEIwSWkyMnU4d3hIN0ZtZ0NiVmhFc25DM3lkS2kyMXMtUHNwOUdsRll1LUg0VWU5NWFsekZsOXF5M2hBdVhBOTJnYXpnd21Ga1JpUG83RmZfcWNHLWFwQUk2NGd0WjhxMDRrUnhmVkZYSXlmbEsyTkxMV3NwR1MydXkx?oc=5</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>Hong Kong Stocks Rise on Monday on Tech, Biotech Gains; Trigiant Jumps 47% - marketscreener.com</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQVkwyeVQyZXlfYlFKTVBlMHRUSjdxVWo5czVkRjRZRk9jQkFQWE5EX1hSQ2RFamFpV0RBdk55c3ZuOUdRNk5CdE1rU3RodExUOXZESmo1LU1rU2hyTlg0R2dYLUM3NGdIQkpiRGlQVHpMcHlrQlRpbzc2QzdTTVZtLXdPT3Z3Z2RVYU9KSnVNc0RBMDRVYUt3X2ROYUhocHZuWVdmRDJCYlVvNHk2S1QwczZCTmgzMHlKM0NxS1hvVHJwdw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>Nasdaq Recovers 296 Points as Monday’s AI Selloff Narrows - TechStock²</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNdFcwaXJ4WGZ3VlAzWXRIVnNLUVRwTVZxYndxVm5KVEl6dHlBdURIajlkNUxCVzY3dlg0amFQelI5Sm9Fb1IxTnV0dDdxLUxtWUdYVmpMWmdjNDdieGtGczBqdTg4QzVkamNfSEx0QjlpZUJ5bTVjcVhrSS1vVnV4NDlCRQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>The Stock Market’s Breaking Point May Be Near - seekingalpha.com</t>
+        </is>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQMnJCdzF3WTYtVU5CdU9qbllzMjk5c0FPbUxSei0wc2VuaGV1TmNTeDJwX3lDT0RtbVFVRjktUDBVbWxIRGo1TlNIUEU3cGplWkluQjEtZkV4QUhWV1NzOUsxcjBvemROMnptSnpuNGI2dk4yb1FaVWJldGNkZjhyYkt6cUtnMkxkZEtmVTVR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:00:40+00:00</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>78985</v>
+      </c>
+      <c r="F37" t="n">
+        <v>79583.10159999999</v>
+      </c>
+      <c r="G37" t="n">
+        <v>78490.1406</v>
+      </c>
+      <c r="H37" t="n">
+        <v>78499.36719999999</v>
+      </c>
+      <c r="I37" t="n">
+        <v>2747867136</v>
+      </c>
+      <c r="J37" t="n">
+        <v>4</v>
+      </c>
+      <c r="K37" t="n">
+        <v>39</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="N37" t="n">
+        <v>37</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0.339</v>
+      </c>
+      <c r="P37" t="n">
+        <v>-0.166</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>8.154</v>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>Bitmine Surges 8% on Ethereum Strength After Cantor Fitzgerald Doubles Its Target, SharpLink Advances 9%, Strategy Gains 4% - 247wallst.com</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPemN4ODV3YldjcDUxb1FRWXc1OWV4bXZwVEhOWTMtbDJaNG92V0xpd0V6OTBxM3lRN0RZUEtWQkRWQW9Kb0hNUF8zS2FBOU5BUlpFTmpvNFBiYnpSVEhHMmtCU2JMdzNjRlNXRWtwaUM1eUxrVjRWQ3VQT2Q4MVJHaHBfdHBRUFpETTVnT012dEJQQV9mcHNOOHUwQnlVU2ZibW51TTBzMHdvTXhsQnlMMzJjT0lhcTNvVktGLTVfN1o3ZXlkLV9JNWRZVVFvakVaaDdIMGxWdFJXUVMxT19rREpueFJibmw0WllRUDk1ckgwUHB1?oc=5</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>Seven assets enter Kraken liquidation window after withdrawals close Monday - cryptoslate.com</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxORVd0T3hNS0lyVG54R1kzcXpndG5yQ0N0bHNFODlZQXBwZ0NlUy13cmFwWlN4QzlZU3pFMlZwZzUtMHBsQnZXT2NXZlhodmI0VmpRczdRajRkbjU5VEVmWWlWeEpzTUVvcUtOTTdraXFadkhuaFNLbXZlSlcxeTlrYnhleE1mWUhQVUZUS0lJYzRJdEhNeUhVRUg4VHBidVN6Mnc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>Short squeeze sends Bitcoin to $72,000 and erases $1.6 billion - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="AD37" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQZW1XSk9xaTJRRmdNUnJoV3NXZ2t3RnZYdHg5NUVnc0U5Zk8wQmFtYWhvSVVScVFSRFlGbXl6dWh6Y19tN1pFZ3RwY0NseFhQYWF5S0ljNlB2c2wyZDRqNGlFLTFod1dtTzJYeFdNaEZuNEJCaVZJMW1sdW9ZUXJhcVFXa1hmcUJlWDgyQUdLWlJRX25mNkprSGFFQQ?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-15 03:51 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD37"/>
+  <dimension ref="A1:AD43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4997,6 +4997,762 @@
       <c r="AD37" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQZW1XSk9xaTJRRmdNUnJoV3NXZ2t3RnZYdHg5NUVnc0U5Zk8wQmFtYWhvSVVScVFSRFlGbXl6dWh6Y19tN1pFZ3RwY0NseFhQYWF5S0ljNlB2c2wyZDRqNGlFLTFod1dtTzJYeFdNaEZuNEJCaVZJMW1sdW9ZUXJhcVFXa1hmcUJlWDgyQUdLWlJRX25mNkprSGFFQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-15T03:48:36+00:00</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>4328.8999</v>
+      </c>
+      <c r="F38" t="n">
+        <v>4358.2002</v>
+      </c>
+      <c r="G38" t="n">
+        <v>4323.7998</v>
+      </c>
+      <c r="H38" t="n">
+        <v>4350.6001</v>
+      </c>
+      <c r="I38" t="n">
+        <v>17098</v>
+      </c>
+      <c r="J38" t="n">
+        <v>4</v>
+      </c>
+      <c r="K38" t="n">
+        <v>39</v>
+      </c>
+      <c r="L38" t="n">
+        <v>-0.038</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="N38" t="n">
+        <v>40</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>1.024</v>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>Founders Metals (TSXV:FDR) Falls 5.65% as Profit-Taking Tests Strong Antino Gold Momentum - kalkine.ca</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQWjZmSkNZV2p0c3pfYWd1Y2U0NnVtdlNaTGdEU3dDbEZ1QTV2WVZCUXp2bmZFVE5ETHByVmc4R1lBUFlDU2JsejNyNkNCcEk3R2lUQUpPbnl5ZS1aeWZGN0lISTVocl9leXVOdTBrN2dKdGJyVl85N0pUQlFtaEZvTXF3V2MzU0xNcTFydU5fNWZsamhnNDVqSThhVEVuaHYweTI5c1g3ZDlDOWplQl8zVGJqa3JnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-09-15T03:48:36+00:00</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>102.17</v>
+      </c>
+      <c r="F39" t="n">
+        <v>103.16</v>
+      </c>
+      <c r="G39" t="n">
+        <v>102.03</v>
+      </c>
+      <c r="H39" t="n">
+        <v>102.92</v>
+      </c>
+      <c r="I39" t="n">
+        <v>15112</v>
+      </c>
+      <c r="J39" t="n">
+        <v>4</v>
+      </c>
+      <c r="K39" t="n">
+        <v>40</v>
+      </c>
+      <c r="L39" t="n">
+        <v>-0.022</v>
+      </c>
+      <c r="M39" t="n">
+        <v>-0.256</v>
+      </c>
+      <c r="N39" t="n">
+        <v>40</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0.136</v>
+      </c>
+      <c r="P39" t="n">
+        <v>-0.095</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>2.295</v>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>US Dollar Gains as Oil Rally and AI Concerns Hit Risk Appetite - Investing.com</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNYnpIU2MtQ09aemlJcXpnMlNqNURRVFU3R2xmekhQcE9CODZEOE9wWFN5MlpDNmtjYVVpSjJ5N2pCZFllb0pkbVlQamw2Z1pGNHhpRENHVGpUelBCa1pZS0xrVXJLdnJkOUk2a2JKTHdPSC0ydVpkOVFZeDAxcndKM2lNWTJqYnhjYXZkMHR3bHRBZWlOWjJYcnNnVDNaeXNGckJ4ejhGRUlqRjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>Gold Falls Rs 500 On Crude Surge, Strong Dollar - Deccan Chronicle</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQRHE1SGJkVHZuWUdXNThqeG1mNl9VaGRpZTJmMHJCX09hYnF0UkZwcXgtWUowdzFDYkxTb3VUSmdUSVdpRW4xMzNwTkVTZFVzUDdLcE9oWVJrUlc5RE1oa0VyY0ZCUkcyV2ZSREVJNkNXM2xsVk9lY2lCeFFDOFcyYW5ieGt4N0hqU293OFV3T01lVXpIWVU3eHdYR0c1cGdORU1JOWFzcmrSAa4BQVVfeXFMUFRZQXR2RU5ybDg3YUd0eVVsekgtMnZkYTBKRlZRdVRIWXZJajdQVmoxajBoX3J2d1pibHZpaVBvbFJ0ZDFwX2toR0k0ajEtTFpFU01RNEhqMDlNMk1iUkdDbVU1OHlzR193MVJiSl9ZLVZ0dkFJNkk1NE92MTVLOHZ4aVkzaDNCdlFtcUlBYm1FYlNmRUpjLU0zanlCVWNHWVlXVzJnX0NfbVZxdEdB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-15T03:48:36+00:00</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>99.489</v>
+      </c>
+      <c r="F40" t="n">
+        <v>99.625</v>
+      </c>
+      <c r="G40" t="n">
+        <v>99.48699999999999</v>
+      </c>
+      <c r="H40" t="n">
+        <v>99.604</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" t="n">
+        <v>4</v>
+      </c>
+      <c r="K40" t="n">
+        <v>37</v>
+      </c>
+      <c r="L40" t="n">
+        <v>-0.064</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="N40" t="n">
+        <v>40</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="P40" t="n">
+        <v>-0.123</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>US Dollar outlook: Hawkish Fed repricing strengthens the bull case - stonex.com</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNRlJTZ3dmU0NMcWtjQU9uU1pXSDQ1Uk5YOGFCVTQwSlExOFZtcjBGT1VZdXppTkpqYkdoaUtTTWw0aVJxclFIaWFnWXItUzBDTkNNSGg1b0t3dVhvREJSQjJRYUFEMGpMa0pNTVpMUzdpT0YwRngyZi1nMlRCdHJlVjVkc0tvU3RqV2pPNzhtYUNhVXlWVXpPRlpiLXBFTE1KNjZoU2lZLXpUaE9CM0hTLTVRSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>Million dollar winning scratch-off sold at Lackawanna County retailer - WNEP</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxPcXdKdTBCNFlfRzZyX1dDbllTXzQzQk9xMktmTVRlSFF2Q3RmOXV0V3A3Tlh2dzY1X09pdm9TSjRjYzNPZXYwTl95U3NRdl9qNUVUM29DZ0RqSmlqeHdsbWlwV25vVmpxWGZTd3VZX0FwUjhmaUVGSDhBZ2pVMGtycEoxNkNBeFhIMFFVN0hBbUg4Q0tQeVM0ZVU5WkxoNUoyZXh6LTJXRHNEaUZZbzRLMnF6YlFBbHFCR3pDUXA1RDMyeWUwbl9fYTdNNEc2M3U5NDZ3cUZSb1BXWmdrOVN6dVU1WlAxS2N6YUI3RjAtdjJuYjNRVzFPdHh5TmQyeXdWMUxZ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>Dovish Fed Bets Pummel Dollar, Boost Gold Ahead of NFP - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPZDNJaUJnTUhOckR3ODFMRjN3M3QtZ1NzUmtvYnRUOVlyWEo2Nzg4d3l5Tkl4SFNRMVJCUnlNeGxUYm5NQkxpNmxEdzVpU3ZHTkhRUXh0bEdhNld2WHFBVmNCRTBEY2dsUkxqVlYtYTUwX21GR1JZNnZjazk2OXBjNW80dWo3Nmx5TXZYLUY0WkZLei14eWV4dDlkRGVheWM?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-15T03:48:36+00:00</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>7696</v>
+      </c>
+      <c r="F41" t="n">
+        <v>7701</v>
+      </c>
+      <c r="G41" t="n">
+        <v>7687</v>
+      </c>
+      <c r="H41" t="n">
+        <v>7687.5</v>
+      </c>
+      <c r="I41" t="n">
+        <v>26982</v>
+      </c>
+      <c r="J41" t="n">
+        <v>4</v>
+      </c>
+      <c r="K41" t="n">
+        <v>39</v>
+      </c>
+      <c r="L41" t="n">
+        <v>-0.409</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="N41" t="n">
+        <v>38</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0.126</v>
+      </c>
+      <c r="P41" t="n">
+        <v>-0.042</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>-5.068</v>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Tax revenue surges amid boom in stock market - Taipei Times</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBVYTNZQ2Q4RFRxNEVSUnVLLTZRQUkyVjF1dEtOZ0hiZ1NreVV3NUx1b1RXdWNoRXZIWlB6MnhXakR3SFdvTGt5SG1NZWFLVjZrUGd4MXk0dVEzRkY5NGJkTUtWSmtwalA5RWlLXzQyVGMwN2pjcEE?oc=5</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>C3.ai Jumps 7% as Software Rally Lifts Beaten-Down AI Names; UiPath Climbs 8%, SoundHound AI Gains 5% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNZVhGa3hKakF5UFBTNTRkLUNCcGF6WXZiaF84aUNHbUhWeHlLbUR4NEhpU2FKZGZOTXFpZUpLZjd1aHQ2V3doTk5pWE9yNjB2VmdvcEc1SllGQm9JMk1sWkFhSXBFeTZZUFpyT1lyTTdNZllaVXdBalRSeW54MzM1WnB4YzUtXzh3aGwybWR6V1B1b2pJWFlNWmp3ZTdWYUM2OElIdFljRDhVV21LQnAxcGxZbnZob2FEbWtMMWdXeEU5WGQydHpLZEJ4U1dWR2o4QmJkVnRkbw?oc=5</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>Wall Street hits record as S&amp;P 500 continues 2-week rally, boosted by hopes for Iran war's end - PBS</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQS3kycm9PYWZzVnJiVllILUtRZlFlN19waWNzNG9hNXNReGNLRkJSdnpfNmdjaTZhTk1CdGM2THJIVlJ1RmZTc0VNS2ZvT2Rmc3JndlZWS1ItMWM0RG93X3ZjdUQ4anZJMENjXzhjaWtpVzdNTTBXbHlXd2RTR1M2WF96ZlFscVRoSXBxcjlVdE9OSFRTaDk4NmJFTGItZnJ6Y3JiVHhZMEw4NXVYZ3ZNb1V5OTFmdDhTVHNheXZ0RE9Lb1ZZRHd30gHMAUFVX3lxTE5od2ZpbkRoY2pjaG1DcVRKTVlRaUZBY0p5a2hpUDMtTFhab0ZzWG5teFZIQUNldDNoWHV0T0dsOHhFMjZGckxEMW5kZUpULXQwMFY2OFJwX2RmUFZTeVRPcW5DYmxYcFUtdXpRNlJCLWR4cDB0N2VvUDlFSUJjYXlxME9tT01sNmxDZ3JDanlOc2QySllnU3FPNmEwakJnOWFxVVhGYVNJMl9nUVk0a1B1N3N3TTBSNVo4MmhkZGFCNEloa3NkczBlS05aNA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Barclays lifts S&amp;P 500 index's year-end target to 7,950 on strong earnings - Reuters</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQdEpJSkhqQ0dZZjZvbFZ3MU9EbGZpa0l4ZjJNazczLTZQTVVfZHlJVmxRVEx3ZFRpLWRwdEhycTRXbGtFdnplbnAwOEgzWG5VQXlYNEdkWE9pVTV0aGl0ZkdsSTBNb1M4U21LWkxPeUVBYWZLTDFZem81OWEtenIwa2E5bjlsdU1Bcmh2SzROZTR2RGFpOVQ4YTRTT21QWXpBX2k2dHV0S3hROHNkYmhR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>Airbus stock rebounds after breaking its 196 € support level - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQTXFjUFRkaWo0Uy1RWThWLU14eFJ3VzF4Z1hyT3ZxMmgzUHdaSWRWSEpCZW1NaXpVU2pQRWxRUVRJT2ExS1FGSHB6VWVOR2pUXzlQUnNhcUxBSjRacjc2bmFHcWNtdmxIWXZHdi1vUjBfeTExYUNHVjROanlpRU5UOGJKeFE3VTY2M2ZzYmNaQVZ1d0xYdlhXVmN1S3BlZUdnRjM1U1FCU0hfUFdsWGIyV0Q0X0tJeDBxTWZwRGZ3?oc=5</t>
+        </is>
+      </c>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-15T03:48:36+00:00</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>29457.25</v>
+      </c>
+      <c r="F42" t="n">
+        <v>29495.25</v>
+      </c>
+      <c r="G42" t="n">
+        <v>29426.75</v>
+      </c>
+      <c r="H42" t="n">
+        <v>29444.75</v>
+      </c>
+      <c r="I42" t="n">
+        <v>18927</v>
+      </c>
+      <c r="J42" t="n">
+        <v>4</v>
+      </c>
+      <c r="K42" t="n">
+        <v>40</v>
+      </c>
+      <c r="L42" t="n">
+        <v>-0.253</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="N42" t="n">
+        <v>33</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="P42" t="n">
+        <v>-0.058</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>2.411</v>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>S&amp;P and Nasdaq hit record highs, continuing remarkable recovery from war shock - CNN</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBFM0dLbkRoQTEzbmVyNGdlZERORGZXdEJrOVh3U0FZVnJsNk0zQjFWVVF6a0NhQThTbS0zMUJTdmdHWm1JYVF3LW5VUWVJWFk1MUd6WlVNWU9aa0dENG9rbkYzRDFpcmhSQ1BJ?oc=5</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Cybersecurity is one corner of the tech market that's getting a boost from AI doomsday fears - Business Insider</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOUkdOM3BPSE8xMS0yWndCcE1aSzd0a3FXOUxIa0tGU3hZMDZ0WGtUODdqVEIwSWkyMnU4d3hIN0ZtZ0NiVmhFc25DM3lkS2kyMXMtUHNwOUdsRll1LUg0VWU5NWFsekZsOXF5M2hBdVhBOTJnYXpnd21Ga1JpUG83RmZfcWNHLWFwQUk2NGd0WjhxMDRrUnhmVkZYSXlmbEsyTkxMV3NwR1MydXkx?oc=5</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>The S&amp;P 500 is back at a record high and the Dow just hit 54,000 | CNN Business - CNN</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE9sNTR6eTFUS1JYX1lnaWVIZGxJeVhmbENJMHN3SUc4TTlSaHpweUdwNUNLejJtSmIwb0x0SEQxalc2OVN1X2s1WFhPSWt2X2VrcFFVeXhVVVpxYVVnaUFjRDR3SUFxbzA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>QQQ: volume node tests, breaks and retests for NASDAQ:QQQ by AuctionFoundry - TradingView</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxORFVBaWZoUklsNVkxUDE0VnEtQUx5OEtMWlhHczdBVWl5TVhLNG5lTUp5cGxQUDdqSTVtWi1kdVFDZ296TG9LRGs0NUV1dTJYMkFNZ19jNWNicG9NbjM0UGlZUEEzTU1FeE1PQ3BMX0NyZElodmU4SHZQc3IzS3N0LTA3dUNsMFZ4a1M3Y19KZTNaQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>Nasdaq Breaks Support As Chip Sell-Off Deepens; Knight-Swift, Canadian Pacific, AbbVie In Focus - Video - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOa0VQNUt2ZDVDYmZpdDB6V3lwVVdxemtUWU5xU0wyTHVKdmtuNzJEU29WUGNSVkNtRjFXV0xIRnQ5N3RodFF3d2JyOFBBbkZQTDVrZWV3R2QzeWctZ1JCS09Bc2VOU2JqWnM4VnlMZjFQVUh2VHNqdzBocUJ3Zm5XSTQ2b19jU3pvZFhvYWNucF9ydU5uLVhqNWN0SDUxZ3BKMXdN?oc=5</t>
+        </is>
+      </c>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>Katie Stockton: Bracing for volatility after Nasdaq broke below recent support - CNBC</t>
+        </is>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLWhuVXhhdF9LbEhfSTV2RlNTZ0IyVjBlcUxGS0RQLXA5S0xjUWFZa3c3Nm1OZmxSRU5mVmVLZzRkbEFKYWd1YWFoVHdadUpRRXlMc1BSVi1BY2Q5RlVLRzVoa2xuRkxZdThVS0VVTzRYY256MHZha1l6RDlrU0NaVXZGZW1qZFRWbTBOUFBTRGxUck9ZWk9tWlY4bl9LcU1BVG5Ka0RVVURXallmZGhqT1BacEpBYnFTUzBIRQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-15T03:48:36+00:00</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>78170</v>
+      </c>
+      <c r="F43" t="n">
+        <v>78242.75</v>
+      </c>
+      <c r="G43" t="n">
+        <v>77681.22659999999</v>
+      </c>
+      <c r="H43" t="n">
+        <v>77714.46090000001</v>
+      </c>
+      <c r="I43" t="n">
+        <v>1119905792</v>
+      </c>
+      <c r="J43" t="n">
+        <v>4</v>
+      </c>
+      <c r="K43" t="n">
+        <v>39</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0.148</v>
+      </c>
+      <c r="N43" t="n">
+        <v>37</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="P43" t="n">
+        <v>-0.208</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>JUST (JST) Surges 3.16% on TRON MetaMask Integration - CoinMarketCap</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFBqUXhEMXI0X0J4MURYaWFlSnBmNWEwTk1tZUNxZVdPY2ZTQU43UTBRVklIdm8yMEZBTWRaUmExc29semtnOHVIdTdlcHRhQUROTWpZbGw3RzV0cVNEWXlHV3hRRENyMFZuRU1HTTVZVzQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Crashes $1,200 As Treasury’s Bond Rescue Backfires - Coinpedia</t>
+        </is>
+      </c>
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPb0ptV09MaS1jdnhORlVpcXVCU3VLSjhaamlhV09DVHNFZnpxbTkzb3VXeXVxZ2FiT3dkLXVGa29GQVd2cTNLM19rbW9GMDhWRGo5cWJOYVFfTmFaQVd4cF9WUHViOWxSSVg1UGVRRHpoc215ajNFQVNtNVI3YUcyQkZicjhJWXN1WFVjeV9LV1RzMl9fOG1pZ1U1eHEyLXl0VS1z0gGoAUFVX3lxTE5YV0swMElha1VQc3IwdVloNE5WelZOSEhlUGNMNWI1SGlqRmFoa1BDNWxra3dlUlhNOXl5SjZWR3RXbDVCWlJnTEpsMGxWaUpuVHZGSHctNWJOdkxEMlV1clhFR3pIWkRvWWFXYldwUk9kd1JOd3JDRW9QX2QzcXJvWkdwemgxRjNBdU9Va0FBNHBMX2ZBU0hGNHZTTl9na3JiSzdNcUtLMw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>How Low Can Bitcoin Go? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNQ0dNeTZHbVVDMUxaQjlRTkhhTGx6Q3U1d2pzREhfYllsMldmZkZpYkwxY3lwMVp0Rm5tbUI2dWpsWEFBWVR5WGd4ZnhuUWtuWUpZVVhLRjB6Z3NRcGMwRlg5UGZLbXJfdHJQeXZCb0UwUkZHdDB6X1prcTFYaERDT2x2UVY4Rk1i?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-15 09:19 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD43"/>
+  <dimension ref="A1:AD49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5751,6 +5751,762 @@
         </is>
       </c>
       <c r="AD43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNQ0dNeTZHbVVDMUxaQjlRTkhhTGx6Q3U1d2pzREhfYllsMldmZkZpYkwxY3lwMVp0Rm5tbUI2dWpsWEFBWVR5WGd4ZnhuUWtuWUpZVVhLRjB6Z3NRcGMwRlg5UGZLbXJfdHJQeXZCb0UwUkZHdDB6X1prcTFYaERDT2x2UVY4Rk1i?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-15T09:16:47+00:00</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>4331.1001</v>
+      </c>
+      <c r="F44" t="n">
+        <v>4335.7002</v>
+      </c>
+      <c r="G44" t="n">
+        <v>4301.7002</v>
+      </c>
+      <c r="H44" t="n">
+        <v>4305.3999</v>
+      </c>
+      <c r="I44" t="n">
+        <v>19935</v>
+      </c>
+      <c r="J44" t="n">
+        <v>4</v>
+      </c>
+      <c r="K44" t="n">
+        <v>39</v>
+      </c>
+      <c r="L44" t="n">
+        <v>-0.044</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="N44" t="n">
+        <v>40</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0.147</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>1.588</v>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Central Banks Go All In On Gold, Buying 27 Tons In A Single Month - Yellow.com</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOWHhCUFdxN2VMQUdfelRiYU8tV3BTcDl4SkwxUllLRmxxN2VtM0NyTWNWNmRPalRzeTNBbGZDWWdMaGE4ZUJ1Vlc2QUJDM3d6amwxd0VSa3RjVUVpNWJQUzkxREQzR0F3MV95RDRkUTM4NXBNZVRyaHlsdi0tcGpaU0pB?oc=5</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>China’s central bank buys 20.2 tonnes of gold in August, largest purchase since 2023 - KITCO</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWDFEUjBvUmhpWnhKb1dmOC1Kd1U3MjVCNG1WSUxXdFdydW1EekdVUDdDb1BDY3FBSVZEMzl0bV9UZGZJV1ZuSDFEb250emQzTm5PY3pfZFktZUdxOV9LNUxzNGFvNHVOcndfWENQVnpzVldMWHJHWHhxdHZHS0ZQYm1FaHFTaVhwRXRsb0hZMUs0WThnNkppalB3OHlOQUhZT1Awakl4dEdudW01aEtnTjFFOUdjZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>Founders Metals (TSXV:FDR) Falls 5.65% as Profit-Taking Tests Strong Antino Gold Momentum - kalkine.ca</t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQWjZmSkNZV2p0c3pfYWd1Y2U0NnVtdlNaTGdEU3dDbEZ1QTV2WVZCUXp2bmZFVE5ETHByVmc4R1lBUFlDU2JsejNyNkNCcEk3R2lUQUpPbnl5ZS1aeWZGN0lISTVocl9leXVOdTBrN2dKdGJyVl85N0pUQlFtaEZvTXF3V2MzU0xNcTFydU5fNWZsamhnNDVqSThhVEVuaHYweTI5c1g3ZDlDOWplQl8zVGJqa3JnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AB44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-15T09:16:47+00:00</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>103</v>
+      </c>
+      <c r="F45" t="n">
+        <v>103.96</v>
+      </c>
+      <c r="G45" t="n">
+        <v>102.92</v>
+      </c>
+      <c r="H45" t="n">
+        <v>103.36</v>
+      </c>
+      <c r="I45" t="n">
+        <v>25390</v>
+      </c>
+      <c r="J45" t="n">
+        <v>4</v>
+      </c>
+      <c r="K45" t="n">
+        <v>40</v>
+      </c>
+      <c r="L45" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="M45" t="n">
+        <v>-0.246</v>
+      </c>
+      <c r="N45" t="n">
+        <v>40</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0.136</v>
+      </c>
+      <c r="P45" t="n">
+        <v>-0.092</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>Sensex, Nifty Gain as IT Stocks Rally Despite Oil Surge - HDFC Sky</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOeVhSVVNsSDlpbXl4WEVWd0JDaFZfRExQUzlBQjJHT216al9BeGxJNlEtcGpqV01MaTE1S3pYZkRZa3pVbVdmdElkdWxYQ3p6THZrcWV3YUlaSm9fN3ZuVVRDSzJBWmJ6OTIzUi1ONF9YNjdtcU5XMUZQdjJ5djBrSXgzY1c3dURLczJMSWF0bGRzMkl2bFZ2NGFzMmxNcllJaXhlZkVVTy1EQmctdkJqZDlJRmpNa05wNDJZajJKajZBQlFKekE?oc=5</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>US Dollar Gains as Oil Rally and AI Concerns Hit Risk Appetite - Investing.com</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNYnpIU2MtQ09aemlJcXpnMlNqNURRVFU3R2xmekhQcE9CODZEOE9wWFN5MlpDNmtjYVVpSjJ5N2pCZFllb0pkbVlQamw2Z1pGNHhpRENHVGpUelBCa1pZS0xrVXJLdnJkOUk2a2JKTHdPSC0ydVpkOVFZeDAxcndKM2lNWTJqYnhjYXZkMHR3bHRBZWlOWjJYcnNnVDNaeXNGckJ4ejhGRUlqRjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>Dow Jones Futures Rise, Oil Prices Fall, Oracle Jumps; CPI Inflation Data To Inform Fed - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPZGdpMlBVbExibHozSndzcGVmRE9SOVdnMnJDbmFSX2NSbjRQamJhd3R6dEkxX2tlaTkwdWRjVlplWkpsQTJoamljRzhQcXZkUmhDTmgtRWY0U1RwRUlEYUdoRmVmVkktM3FDNWpyVXRFNkpEWGl5ZlhHaGNadmVKTUx5NlhlQXE1ejdTUlowM0dGM1lPRkdTb2xRV2pKczR6aWtoLXRMWG11RDlUaXRuZDc3eUh1SDBmQ2NZQ2laTzBXMGtVQ0NpVjNhU2FvZ1ItWDhQWV9n?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-15T09:16:47+00:00</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>99.624</v>
+      </c>
+      <c r="F46" t="n">
+        <v>99.687</v>
+      </c>
+      <c r="G46" t="n">
+        <v>99.583</v>
+      </c>
+      <c r="H46" t="n">
+        <v>99.639</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>4</v>
+      </c>
+      <c r="K46" t="n">
+        <v>38</v>
+      </c>
+      <c r="L46" t="n">
+        <v>-0.08400000000000001</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="N46" t="n">
+        <v>39</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="P46" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>1.218</v>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>US Dollar outlook: Hawkish Fed repricing strengthens the bull case - stonex.com</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNRlJTZ3dmU0NMcWtjQU9uU1pXSDQ1Uk5YOGFCVTQwSlExOFZtcjBGT1VZdXppTkpqYkdoaUtTTWw0aVJxclFIaWFnWXItUzBDTkNNSGg1b0t3dVhvREJSQjJRYUFEMGpMa0pNTVpMUzdpT0YwRngyZi1nMlRCdHJlVjVkc0tvU3RqV2pPNzhtYUNhVXlWVXpPRlpiLXBFTE1KNjZoU2lZLXpUaE9CM0hTLTVRSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>Dollar Rises as 10-Year Treasury Yield Hits Highest Since 2007 - Global Banking &amp; Finance Review</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxONmpEYnFtQ0xnTTNQZjhxQTJaUVhRUVhIbURwb1pZc2VEQVRDOFlIQWgzSnh1eGJPZDlWMjJ2YjZRVDlwN08tazFUc2RxRGF2V0trd0xraW5qX1E3OGplNTlpWVFjZUhZMzBJOWxTQWZIbUVmSUFIOEM1bWpOM2lBUklyWXVWaDhLZEMxN1RmbTcteENSWnBVUnBPYjc4cUE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - FXStreet</t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AB46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC46" t="inlineStr">
+        <is>
+          <t>Million dollar winning scratch-off sold at Lackawanna County retailer - WNEP</t>
+        </is>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxPcXdKdTBCNFlfRzZyX1dDbllTXzQzQk9xMktmTVRlSFF2Q3RmOXV0V3A3Tlh2dzY1X09pdm9TSjRjYzNPZXYwTl95U3NRdl9qNUVUM29DZ0RqSmlqeHdsbWlwV25vVmpxWGZTd3VZX0FwUjhmaUVGSDhBZ2pVMGtycEoxNkNBeFhIMFFVN0hBbUg4Q0tQeVM0ZVU5WkxoNUoyZXh6LTJXRHNEaUZZbzRLMnF6YlFBbHFCR3pDUXA1RDMyeWUwbl9fYTdNNEc2M3U5NDZ3cUZSb1BXWmdrOVN6dVU1WlAxS2N6YUI3RjAtdjJuYjNRVzFPdHh5TmQyeXdWMUxZ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-15T09:16:47+00:00</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>7675</v>
+      </c>
+      <c r="F47" t="n">
+        <v>7677.75</v>
+      </c>
+      <c r="G47" t="n">
+        <v>7645</v>
+      </c>
+      <c r="H47" t="n">
+        <v>7649.25</v>
+      </c>
+      <c r="I47" t="n">
+        <v>87397</v>
+      </c>
+      <c r="J47" t="n">
+        <v>4</v>
+      </c>
+      <c r="K47" t="n">
+        <v>39</v>
+      </c>
+      <c r="L47" t="n">
+        <v>-0.329</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="N47" t="n">
+        <v>39</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0.228</v>
+      </c>
+      <c r="P47" t="n">
+        <v>-0.067</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>-1.978</v>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Tax revenue surges amid boom in stock market - Taipei Times</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBVYTNZQ2Q4RFRxNEVSUnVLLTZRQUkyVjF1dEtOZ0hiZ1NreVV3NUx1b1RXdWNoRXZIWlB6MnhXakR3SFdvTGt5SG1NZWFLVjZrUGd4MXk0dVEzRkY5NGJkTUtWSmtwalA5RWlLXzQyVGMwN2pjcEE?oc=5</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>C3.ai Jumps 7% as Software Rally Lifts Beaten-Down AI Names; UiPath Climbs 8%, SoundHound AI Gains 5% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNZVhGa3hKakF5UFBTNTRkLUNCcGF6WXZiaF84aUNHbUhWeHlLbUR4NEhpU2FKZGZOTXFpZUpLZjd1aHQ2V3doTk5pWE9yNjB2VmdvcEc1SllGQm9JMk1sWkFhSXBFeTZZUFpyT1lyTTdNZllaVXdBalRSeW54MzM1WnB4YzUtXzh3aGwybWR6V1B1b2pJWFlNWmp3ZTdWYUM2OElIdFljRDhVV21LQnAxcGxZbnZob2FEbWtMMWdXeEU5WGQydHpLZEJ4U1dWR2o4QmJkVnRkbw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>Barclays lifts S&amp;P 500 index's year-end target to 7,950 on strong earnings - Reuters</t>
+        </is>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQdEpJSkhqQ0dZZjZvbFZ3MU9EbGZpa0l4ZjJNazczLTZQTVVfZHlJVmxRVEx3ZFRpLWRwdEhycTRXbGtFdnplbnAwOEgzWG5VQXlYNEdkWE9pVTV0aGl0ZkdsSTBNb1M4U21LWkxPeUVBYWZLTDFZem81OWEtenIwa2E5bjlsdU1Bcmh2SzROZTR2RGFpOVQ4YTRTT21QWXpBX2k2dHV0S3hROHNkYmhR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>Rexel stock breaks through its 35.40 € support and slides towards a floor - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB47" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxNYmJGM0Ria0tiUk8zcHJ6RExXSDFGSFVFY3Q4WXVfZldBM3NzYlNwaWxyaDhrNHhLREdNRXd2Z0R3cGpZekVJUl8tc3AweUx5Mm5uUWJ4dWh2cjhVTHFQbWQzYzFNZ2F1WEdrUTYtM2FRa1g4ckF3YTQ1RHRHQ3NxajJMbkZEWVZqZjlzaEpVbUs0UWkzb2l5R1htaG1CeXFOU1EySnJNcDNUWFd5LXVIdldidnhQTlltdFdRVUplZXFDZWt0R0FwXzlEVE1saWs?oc=5</t>
+        </is>
+      </c>
+      <c r="AC47" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-15T09:16:47+00:00</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>29378.25</v>
+      </c>
+      <c r="F48" t="n">
+        <v>29395.25</v>
+      </c>
+      <c r="G48" t="n">
+        <v>29231</v>
+      </c>
+      <c r="H48" t="n">
+        <v>29268.25</v>
+      </c>
+      <c r="I48" t="n">
+        <v>26030</v>
+      </c>
+      <c r="J48" t="n">
+        <v>4</v>
+      </c>
+      <c r="K48" t="n">
+        <v>40</v>
+      </c>
+      <c r="L48" t="n">
+        <v>-0.216</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="N48" t="n">
+        <v>35</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0.272</v>
+      </c>
+      <c r="P48" t="n">
+        <v>-0.08500000000000001</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>2.938</v>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>S&amp;P and Nasdaq hit record highs, continuing remarkable recovery from war shock - CNN</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBFM0dLbkRoQTEzbmVyNGdlZERORGZXdEJrOVh3U0FZVnJsNk0zQjFWVVF6a0NhQThTbS0zMUJTdmdHWm1JYVF3LW5VUWVJWFk1MUd6WlVNWU9aa0dENG9rbkYzRDFpcmhSQ1BJ?oc=5</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Cybersecurity is one corner of the tech market that's getting a boost from AI doomsday fears - Business Insider</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOUkdOM3BPSE8xMS0yWndCcE1aSzd0a3FXOUxIa0tGU3hZMDZ0WGtUODdqVEIwSWkyMnU4d3hIN0ZtZ0NiVmhFc25DM3lkS2kyMXMtUHNwOUdsRll1LUg0VWU5NWFsekZsOXF5M2hBdVhBOTJnYXpnd21Ga1JpUG83RmZfcWNHLWFwQUk2NGd0WjhxMDRrUnhmVkZYSXlmbEsyTkxMV3NwR1MydXkx?oc=5</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>The S&amp;P 500 is back at a record high and the Dow just hit 54,000 | CNN Business - CNN</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE9sNTR6eTFUS1JYX1lnaWVIZGxJeVhmbENJMHN3SUc4TTlSaHpweUdwNUNLejJtSmIwb0x0SEQxalc2OVN1X2s1WFhPSWt2X2VrcFFVeXhVVVpxYVVnaUFjRDR3SUFxbzA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>QQQ: volume node tests, breaks and retests for NASDAQ:QQQ by AuctionFoundry - TradingView</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxORFVBaWZoUklsNVkxUDE0VnEtQUx5OEtMWlhHczdBVWl5TVhLNG5lTUp5cGxQUDdqSTVtWi1kdVFDZ296TG9LRGs0NUV1dTJYMkFNZ19jNWNicG9NbjM0UGlZUEEzTU1FeE1PQ3BMX0NyZElodmU4SHZQc3IzS3N0LTA3dUNsMFZ4a1M3Y19KZTNaQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>Nasdaq Breaks Support As Chip Sell-Off Deepens; Knight-Swift, Canadian Pacific, AbbVie In Focus - Video - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOa0VQNUt2ZDVDYmZpdDB6V3lwVVdxemtUWU5xU0wyTHVKdmtuNzJEU29WUGNSVkNtRjFXV0xIRnQ5N3RodFF3d2JyOFBBbkZQTDVrZWV3R2QzeWctZ1JCS09Bc2VOU2JqWnM4VnlMZjFQVUh2VHNqdzBocUJ3Zm5XSTQ2b19jU3pvZFhvYWNucF9ydU5uLVhqNWN0SDUxZ3BKMXdN?oc=5</t>
+        </is>
+      </c>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>Nasdaq breaks a new record after Ceasefire extension – Dow Jones and US Stock Market Outlook - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNU21uTDlsYjhfQ0w2UEF5STJ4Qm5xajNPS1gxT3B5MFFPbmZMTDQxR0VKcXA1blY0S1kxLTFWT3FZcFczc1NZWWpCRGhqX0ZpblpDNFVJc3J0aExpYl9Eb2xycHpiY3o1NjRDTEhVdHMyZU9yZU9leXZDcllQbjFkcUhFVnp3NFdQNkdhMkZnRVRsZXZBNXl2Z1VhYjdDU29jbnR6WUFKMllmYWs?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-15T09:16:47+00:00</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>77620.8438</v>
+      </c>
+      <c r="F49" t="n">
+        <v>77711.5938</v>
+      </c>
+      <c r="G49" t="n">
+        <v>76650.89840000001</v>
+      </c>
+      <c r="H49" t="n">
+        <v>76873.71090000001</v>
+      </c>
+      <c r="I49" t="n">
+        <v>1724790784</v>
+      </c>
+      <c r="J49" t="n">
+        <v>4</v>
+      </c>
+      <c r="K49" t="n">
+        <v>39</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="N49" t="n">
+        <v>37</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0.283</v>
+      </c>
+      <c r="P49" t="n">
+        <v>-0.197</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>6.298</v>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>Bitmine Surges 8% on Ethereum Strength After Cantor Fitzgerald Doubles Its Target, SharpLink Advances 9%, Strategy Gains 4% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPemN4ODV3YldjcDUxb1FRWXc1OWV4bXZwVEhOWTMtbDJaNG92V0xpd0V6OTBxM3lRN0RZUEtWQkRWQW9Kb0hNUF8zS2FBOU5BUlpFTmpvNFBiYnpSVEhHMmtCU2JMdzNjRlNXRWtwaUM1eUxrVjRWQ3VQT2Q4MVJHaHBfdHBRUFpETTVnT012dEJQQV9mcHNOOHUwQnlVU2ZibW51TTBzMHdvTXhsQnlMMzJjT0lhcTNvVktGLTVfN1o3ZXlkLV9JNWRZVVFvakVaaDdIMGxWdFJXUVMxT19rREpueFJibmw0WllRUDk1ckgwUHB1?oc=5</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Crashes $1,200 As Treasury’s Bond Rescue Backfires - Coinpedia</t>
+        </is>
+      </c>
+      <c r="AB49" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPb0ptV09MaS1jdnhORlVpcXVCU3VLSjhaamlhV09DVHNFZnpxbTkzb3VXeXVxZ2FiT3dkLXVGa29GQVd2cTNLM19rbW9GMDhWRGo5cWJOYVFfTmFaQVd4cF9WUHViOWxSSVg1UGVRRHpoc215ajNFQVNtNVI3YUcyQkZicjhJWXN1WFVjeV9LV1RzMl9fOG1pZ1U1eHEyLXl0VS1z0gGoAUFVX3lxTE5YV0swMElha1VQc3IwdVloNE5WelZOSEhlUGNMNWI1SGlqRmFoa1BDNWxra3dlUlhNOXl5SjZWR3RXbDVCWlJnTEpsMGxWaUpuVHZGSHctNWJOdkxEMlV1clhFR3pIWkRvWWFXYldwUk9kd1JOd3JDRW9QX2QzcXJvWkdwemgxRjNBdU9Va0FBNHBMX2ZBU0hGNHZTTl9na3JiSzdNcUtLMw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>How Low Can Bitcoin Go? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AD49" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNQ0dNeTZHbVVDMUxaQjlRTkhhTGx6Q3U1d2pzREhfYllsMldmZkZpYkwxY3lwMVp0Rm5tbUI2dWpsWEFBWVR5WGd4ZnhuUWtuWUpZVVhLRjB6Z3NRcGMwRlg5UGZLbXJfdHJQeXZCb0UwUkZHdDB6X1prcTFYaERDT2x2UVY4Rk1i?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-15 16:31 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD49"/>
+  <dimension ref="A1:AD55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6509,6 +6509,762 @@
       <c r="AD49" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNQ0dNeTZHbVVDMUxaQjlRTkhhTGx6Q3U1d2pzREhfYllsMldmZkZpYkwxY3lwMVp0Rm5tbUI2dWpsWEFBWVR5WGd4ZnhuUWtuWUpZVVhLRjB6Z3NRcGMwRlg5UGZLbXJfdHJQeXZCb0UwUkZHdDB6X1prcTFYaERDT2x2UVY4Rk1i?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-15T16:28:40+00:00</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>4330.2002</v>
+      </c>
+      <c r="F50" t="n">
+        <v>4340.7002</v>
+      </c>
+      <c r="G50" t="n">
+        <v>4313</v>
+      </c>
+      <c r="H50" t="n">
+        <v>4327.7998</v>
+      </c>
+      <c r="I50" t="n">
+        <v>34822</v>
+      </c>
+      <c r="J50" t="n">
+        <v>4</v>
+      </c>
+      <c r="K50" t="n">
+        <v>40</v>
+      </c>
+      <c r="L50" t="n">
+        <v>-0.121</v>
+      </c>
+      <c r="M50" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="N50" t="n">
+        <v>40</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="P50" t="n">
+        <v>-0.008999999999999999</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>0.763</v>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>Founders Metals (TSXV:FDR) Falls 5.65% as Profit-Taking Tests Strong Antino Gold Momentum - kalkine.ca</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQWjZmSkNZV2p0c3pfYWd1Y2U0NnVtdlNaTGdEU3dDbEZ1QTV2WVZCUXp2bmZFVE5ETHByVmc4R1lBUFlDU2JsejNyNkNCcEk3R2lUQUpPbnl5ZS1aeWZGN0lISTVocl9leXVOdTBrN2dKdGJyVl85N0pUQlFtaEZvTXF3V2MzU0xNcTFydU5fNWZsamhnNDVqSThhVEVuaHYweTI5c1g3ZDlDOWplQl8zVGJqa3JnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AB50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - fxstreet.com</t>
+        </is>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-15T16:28:40+00:00</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="F51" t="n">
+        <v>105.65</v>
+      </c>
+      <c r="G51" t="n">
+        <v>101.28</v>
+      </c>
+      <c r="H51" t="n">
+        <v>105.54</v>
+      </c>
+      <c r="I51" t="n">
+        <v>138118</v>
+      </c>
+      <c r="J51" t="n">
+        <v>4</v>
+      </c>
+      <c r="K51" t="n">
+        <v>40</v>
+      </c>
+      <c r="L51" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="M51" t="n">
+        <v>-0.277</v>
+      </c>
+      <c r="N51" t="n">
+        <v>40</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="P51" t="n">
+        <v>-0.019</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>1.102</v>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Antioxidants for Crude Oil Market to Accelerate by 2035, Driven by Rising Heavy Sour Crude Processing - IndexBox</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQWTVSYlo2TlZ4emlNR3VPWGJPa015SW9SRWtGM1ZVZExqY0Z1S2hhUWp5UXM2a013ZW5zcm9jUXcyc0FHU0Y1RTlGSDh2Tklrc3JrLU04ZXBuQjJ5U1VnLS1Fc0Fab2RvSGx0T3N0TmVRTDBZQi1QRGxXcDBCZHBGLWYxdVc0S1VUZzlIaVB5SjF2cElDcnR3QWVSYUE0TFNUWi04T0RBVE5GSlhlQ1Utd19CSzNoMUZvOUlpYUZ3OW9xbmZsbExGSGFn?oc=5</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>Organization of the Petroleum Exporting Countries - opec.org</t>
+        </is>
+      </c>
+      <c r="AB51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE5TYnpCM2R2ZEh2OGpWR1o3VXRJZjJTQWZMRWMyOGQtUG9JdUxwelZUUjNyWjJteWE5Qmlod3l0dFAtNDBvZVprVGVyRzhZeU9CNndJU041eUtXMzNPdHU1bl8tZS1XVHU0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC51" t="inlineStr">
+        <is>
+          <t>Dow Jones Futures Rise, Oil Prices Fall, Oracle Jumps; CPI Inflation Data To Inform Fed - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPZGdpMlBVbExibHozSndzcGVmRE9SOVdnMnJDbmFSX2NSbjRQamJhd3R6dEkxX2tlaTkwdWRjVlplWkpsQTJoamljRzhQcXZkUmhDTmgtRWY0U1RwRUlEYUdoRmVmVkktM3FDNWpyVXRFNkpEWGl5ZlhHaGNadmVKTUx5NlhlQXE1ejdTUlowM0dGM1lPRkdTb2xRV2pKczR6aWtoLXRMWG11RDlUaXRuZDc3eUh1SDBmQ2NZQ2laTzBXMGtVQ0NpVjNhU2FvZ1ItWDhQWV9n?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-15T16:28:40+00:00</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>99.587</v>
+      </c>
+      <c r="F52" t="n">
+        <v>99.652</v>
+      </c>
+      <c r="G52" t="n">
+        <v>99.53</v>
+      </c>
+      <c r="H52" t="n">
+        <v>99.652</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="n">
+        <v>4</v>
+      </c>
+      <c r="K52" t="n">
+        <v>39</v>
+      </c>
+      <c r="L52" t="n">
+        <v>-0.115</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0.194</v>
+      </c>
+      <c r="N52" t="n">
+        <v>39</v>
+      </c>
+      <c r="O52" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="P52" t="n">
+        <v>-0.077</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>US Dollar outlook: Hawkish Fed repricing strengthens the bull case - stonex.com</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNRlJTZ3dmU0NMcWtjQU9uU1pXSDQ1Uk5YOGFCVTQwSlExOFZtcjBGT1VZdXppTkpqYkdoaUtTTWw0aVJxclFIaWFnWXItUzBDTkNNSGg1b0t3dVhvREJSQjJRYUFEMGpMa0pNTVpMUzdpT0YwRngyZi1nMlRCdHJlVjVkc0tvU3RqV2pPNzhtYUNhVXlWVXpPRlpiLXBFTE1KNjZoU2lZLXpUaE9CM0hTLTVRSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>Dovish Fed Bets Pummel Dollar, Boost Gold Ahead of NFP - Investing.com</t>
+        </is>
+      </c>
+      <c r="AB52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPZDNJaUJnTUhOckR3ODFMRjN3M3QtZ1NzUmtvYnRUOVlyWEo2Nzg4d3l5Tkl4SFNRMVJCUnlNeGxUYm5NQkxpNmxEdzVpU3ZHTkhRUXh0bEdhNld2WHFBVmNCRTBEY2dsUkxqVlYtYTUwX21GR1JZNnZjazk2OXBjNW80dWo3Nmx5TXZYLUY0WkZLei14eWV4dDlkRGVheWM?oc=5</t>
+        </is>
+      </c>
+      <c r="AC52" t="inlineStr">
+        <is>
+          <t>The Dollar Index falls through a war and a hawkish repricing - fxstreet.com</t>
+        </is>
+      </c>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNVFRZaFp1RzRGblVrRGFlYlUteDBWNE5PRmNKSlZ1VmU0Y09naUFPWmw3U0tiZmY5VGJ1Wkp6N1pROGhtQVItYkczcGFvTmE2TGVYSG9MRGIwbXJNeWkySmI3ZkNBUU1LaU5TQ0E4UFR2N1JyMEZVZ2Jxd1NxTXZ1YV9qZ2NMck8xNFJfUXRKVnhBWVNJZUlia1ZHMFFyTkMtT3BhYXpn?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-15T16:28:40+00:00</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>7689</v>
+      </c>
+      <c r="F53" t="n">
+        <v>7693.5</v>
+      </c>
+      <c r="G53" t="n">
+        <v>7643.5</v>
+      </c>
+      <c r="H53" t="n">
+        <v>7653.75</v>
+      </c>
+      <c r="I53" t="n">
+        <v>777524</v>
+      </c>
+      <c r="J53" t="n">
+        <v>4</v>
+      </c>
+      <c r="K53" t="n">
+        <v>38</v>
+      </c>
+      <c r="L53" t="n">
+        <v>-0.174</v>
+      </c>
+      <c r="M53" t="n">
+        <v>-0.011</v>
+      </c>
+      <c r="N53" t="n">
+        <v>39</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="P53" t="n">
+        <v>-0.076</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Tax revenue surges amid boom in stock market - Taipei Times</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBVYTNZQ2Q4RFRxNEVSUnVLLTZRQUkyVjF1dEtOZ0hiZ1NreVV3NUx1b1RXdWNoRXZIWlB6MnhXakR3SFdvTGt5SG1NZWFLVjZrUGd4MXk0dVEzRkY5NGJkTUtWSmtwalA5RWlLXzQyVGMwN2pjcEE?oc=5</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>Illumina Stock Analysis: Bullish Trend Holds, Momentum in Focus - The Cryptonomist</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQaUstS2lxb25wVWhUUm9ZZjM4WUpYekk3Mk1VVjdHYWdaZUE2alhkXzVKMXlOOHZ0ekVOSE5EWXYtS1o2QjFyVGVockpyVWZPVXdhUTNsSFcyMEE5aFZqb0l4M045T3Z4cnNuU2t4ckpBYTNmZEhGZWstVlV2YlkzQW0zSkpNYUtzeTRYZ2NrMG9nWDhwQ0x2QTZsNVg?oc=5</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 11: HPE Surges on AI Infrastructure Demand and Recently Raised Guidance - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxQWHZrbGtuQ2NuRE92NG4temVfd3BnRnJ3ZDJQYlUzZGpBSnFIYWlLQ0VfVks2enFoZGdGamlac3MwdUFCb2JtTmlpV2NhaFFqUzZNQkhPS01ZVGNGTzNHZ05FbVFrWDVHN3F1Mjk1YU1uekRmRWktenpIX1dVQzd5RTJsZ3l2alRmNmxLUWNsY09xQTVJbnc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>Barclays lifts S&amp;P 500 index's year-end target to 7,950 on strong earnings - Reuters</t>
+        </is>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQdEpJSkhqQ0dZZjZvbFZ3MU9EbGZpa0l4ZjJNazczLTZQTVVfZHlJVmxRVEx3ZFRpLWRwdEhycTRXbGtFdnplbnAwOEgzWG5VQXlYNEdkWE9pVTV0aGl0ZkdsSTBNb1M4U21LWkxPeUVBYWZLTDFZem81OWEtenIwa2E5bjlsdU1Bcmh2SzROZTR2RGFpOVQ4YTRTT21QWXpBX2k2dHV0S3hROHNkYmhR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>Rexel stock breaks through its 35.40 € support and slides towards a floor - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxNYmJGM0Ria0tiUk8zcHJ6RExXSDFGSFVFY3Q4WXVfZldBM3NzYlNwaWxyaDhrNHhLREdNRXd2Z0R3cGpZekVJUl8tc3AweUx5Mm5uUWJ4dWh2cjhVTHFQbWQzYzFNZ2F1WEdrUTYtM2FRa1g4ckF3YTQ1RHRHQ3NxajJMbkZEWVZqZjlzaEpVbUs0UWkzb2l5R1htaG1CeXFOU1EySnJNcDNUWFd5LXVIdldidnhQTlltdFdRVUplZXFDZWt0R0FwXzlEVE1saWs?oc=5</t>
+        </is>
+      </c>
+      <c r="AC53" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-15T16:28:40+00:00</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>29433.75</v>
+      </c>
+      <c r="F54" t="n">
+        <v>29453.5</v>
+      </c>
+      <c r="G54" t="n">
+        <v>29215.75</v>
+      </c>
+      <c r="H54" t="n">
+        <v>29271</v>
+      </c>
+      <c r="I54" t="n">
+        <v>220942</v>
+      </c>
+      <c r="J54" t="n">
+        <v>4</v>
+      </c>
+      <c r="K54" t="n">
+        <v>39</v>
+      </c>
+      <c r="L54" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="N54" t="n">
+        <v>36</v>
+      </c>
+      <c r="O54" t="n">
+        <v>0.332</v>
+      </c>
+      <c r="P54" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>1.419</v>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Amplitude: The Rebound Rally Is Here, Fueled By Impressive Backlog Growth (NASDAQ:AMPL) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPVFNMdU5VS0tzT25fVGpuY1ZnaTkwcTNzZGdxQldPREF0VUtGeW1JSG4yRUVZMGNYZzJiTTI0MTgzclpBU0FqNGdTTXRwLUxtdjFCUC1SRWVJNmNWQTJtcTQxWlFXRDJFRUpyaGwwQjJhcWdKUTlPUmNveDB3SjRSV0xRZHROQldCX1hxVFdEU2Rvc2tfVy1nT1ZRdlotOHZFN1pSOGg0RXk4THR1NlRSdEFB?oc=5</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>S&amp;P and Nasdaq hit record highs, continuing remarkable recovery from war shock - CNN</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBFM0dLbkRoQTEzbmVyNGdlZERORGZXdEJrOVh3U0FZVnJsNk0zQjFWVVF6a0NhQThTbS0zMUJTdmdHWm1JYVF3LW5VUWVJWFk1MUd6WlVNWU9aa0dENG9rbkYzRDFpcmhSQ1BJ?oc=5</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>Cybersecurity is one corner of the tech market that's getting a boost from AI doomsday fears - Business Insider</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOUkdOM3BPSE8xMS0yWndCcE1aSzd0a3FXOUxIa0tGU3hZMDZ0WGtUODdqVEIwSWkyMnU4d3hIN0ZtZ0NiVmhFc25DM3lkS2kyMXMtUHNwOUdsRll1LUg0VWU5NWFsekZsOXF5M2hBdVhBOTJnYXpnd21Ga1JpUG83RmZfcWNHLWFwQUk2NGd0WjhxMDRrUnhmVkZYSXlmbEsyTkxMV3NwR1MydXkx?oc=5</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>QQQ: volume node tests, breaks and retests for NASDAQ:QQQ by AuctionFoundry - tradingview.com</t>
+        </is>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxORFVBaWZoUklsNVkxUDE0VnEtQUx5OEtMWlhHczdBVWl5TVhLNG5lTUp5cGxQUDdqSTVtWi1kdVFDZ296TG9LRGs0NUV1dTJYMkFNZ19jNWNicG9NbjM0UGlZUEEzTU1FeE1PQ3BMX0NyZElodmU4SHZQc3IzS3N0LTA3dUNsMFZ4a1M3Y19KZTNaQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>Fortune Tech: AI stocks fall, Mustafa Suleyman speaks, OpenAI’s California compliance - Fortune</t>
+        </is>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPV09SLWgzYTBFb2tRN0NNaVFqRGNnLXVSeFdZcC16M0g5YVA5RjJWNmw3RFAtckh2cXpSdWFNQWhZM3o0emtnMnNmVjFSYUE3T3M5bVo1ZmlCQ2tSMmZWN0F6Sm93Mm4zMFZtNlU3MERrR1Z1Q1hjOTE3dW5uR2Vib2xtUHljQjBmemd6WDN0RUhoaUY0d0VYcDhn?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-15T16:28:40+00:00</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>76916.25</v>
+      </c>
+      <c r="F55" t="n">
+        <v>77094.0469</v>
+      </c>
+      <c r="G55" t="n">
+        <v>75545.2188</v>
+      </c>
+      <c r="H55" t="n">
+        <v>76390.85159999999</v>
+      </c>
+      <c r="I55" t="n">
+        <v>6006796288</v>
+      </c>
+      <c r="J55" t="n">
+        <v>4</v>
+      </c>
+      <c r="K55" t="n">
+        <v>39</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0.124</v>
+      </c>
+      <c r="N55" t="n">
+        <v>37</v>
+      </c>
+      <c r="O55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="P55" t="n">
+        <v>-0.093</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>8.052</v>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - cnbc.com</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>Bitmine Surges 8% on Ethereum Strength After Cantor Fitzgerald Doubles Its Target, SharpLink Advances 9%, Strategy Gains 4% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPemN4ODV3YldjcDUxb1FRWXc1OWV4bXZwVEhOWTMtbDJaNG92V0xpd0V6OTBxM3lRN0RZUEtWQkRWQW9Kb0hNUF8zS2FBOU5BUlpFTmpvNFBiYnpSVEhHMmtCU2JMdzNjRlNXRWtwaUM1eUxrVjRWQ3VQT2Q4MVJHaHBfdHBRUFpETTVnT012dEJQQV9mcHNOOHUwQnlVU2ZibW51TTBzMHdvTXhsQnlMMzJjT0lhcTNvVktGLTVfN1o3ZXlkLV9JNWRZVVFvakVaaDdIMGxWdFJXUVMxT19rREpueFJibmw0WllRUDk1ckgwUHB1?oc=5</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="Z55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>Bitcoin and gold touted as hedges against currency debasement as US debt tops $40 trillion - tradingview.com</t>
+        </is>
+      </c>
+      <c r="AB55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxPMFFOejYzSnZwaUdrNmdPWnEtR2V5WmVaTndxaHg3Qlk1V1Nqa1NZZ0xUaTlDbzNaTU1IaTRqc3lxY2F3eUJYV3VaVE9uWnhyTC1BVHdza3B4SW51UDcxeU5nQm9ueVdlVC11d0ExeDNVdTJtWjZNVGFnUHQxdVFtTnVaVmxvZ29ZbnJmeVVqYjBGZ2hXRF9QQ0F5UmtuQW9TUHUtMWNSTmNXRDlyYmlqZHVXaHdjT3IwcTZGdDhTcVJnWkozOWxXWkdxdS1hamdHbDNyWHdvUEZ2OXVqaTE5ZGZiaUFocDdUb0E?oc=5</t>
+        </is>
+      </c>
+      <c r="AC55" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Crashes $1,200 As Treasury’s Bond Rescue Backfires - coinpedia.org</t>
+        </is>
+      </c>
+      <c r="AD55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPb0ptV09MaS1jdnhORlVpcXVCU3VLSjhaamlhV09DVHNFZnpxbTkzb3VXeXVxZ2FiT3dkLXVGa29GQVd2cTNLM19rbW9GMDhWRGo5cWJOYVFfTmFaQVd4cF9WUHViOWxSSVg1UGVRRHpoc215ajNFQVNtNVI3YUcyQkZicjhJWXN1WFVjeV9LV1RzMl9fOG1pZ1U1eHEyLXl0VS1z0gGoAUFVX3lxTE5YV0swMElha1VQc3IwdVloNE5WelZOSEhlUGNMNWI1SGlqRmFoa1BDNWxra3dlUlhNOXl5SjZWR3RXbDVCWlJnTEpsMGxWaUpuVHZGSHctNWJOdkxEMlV1clhFR3pIWkRvWWFXYldwUk9kd1JOd3JDRW9QX2QzcXJvWkdwemgxRjNBdU9Va0FBNHBMX2ZBU0hGNHZTTl9na3JiSzdNcUtLMw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-15 22:48 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD55"/>
+  <dimension ref="A1:AD61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7265,6 +7265,762 @@
       <c r="AD55" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPb0ptV09MaS1jdnhORlVpcXVCU3VLSjhaamlhV09DVHNFZnpxbTkzb3VXeXVxZ2FiT3dkLXVGa29GQVd2cTNLM19rbW9GMDhWRGo5cWJOYVFfTmFaQVd4cF9WUHViOWxSSVg1UGVRRHpoc215ajNFQVNtNVI3YUcyQkZicjhJWXN1WFVjeV9LV1RzMl9fOG1pZ1U1eHEyLXl0VS1z0gGoAUFVX3lxTE5YV0swMElha1VQc3IwdVloNE5WelZOSEhlUGNMNWI1SGlqRmFoa1BDNWxra3dlUlhNOXl5SjZWR3RXbDVCWlJnTEpsMGxWaUpuVHZGSHctNWJOdkxEMlV1clhFR3pIWkRvWWFXYldwUk9kd1JOd3JDRW9QX2QzcXJvWkdwemgxRjNBdU9Va0FBNHBMX2ZBU0hGNHZTTl9na3JiSzdNcUtLMw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-15T22:46:15+00:00</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>4335.5</v>
+      </c>
+      <c r="F56" t="n">
+        <v>4350.7998</v>
+      </c>
+      <c r="G56" t="n">
+        <v>4330.8999</v>
+      </c>
+      <c r="H56" t="n">
+        <v>4337.6001</v>
+      </c>
+      <c r="I56" t="n">
+        <v>16697</v>
+      </c>
+      <c r="J56" t="n">
+        <v>4</v>
+      </c>
+      <c r="K56" t="n">
+        <v>40</v>
+      </c>
+      <c r="L56" t="n">
+        <v>-0.098</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="N56" t="n">
+        <v>40</v>
+      </c>
+      <c r="O56" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="P56" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>0.367</v>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>Founders Metals (TSXV:FDR) Falls 5.65% as Profit-Taking Tests Strong Antino Gold Momentum - kalkine.ca</t>
+        </is>
+      </c>
+      <c r="Z56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQWjZmSkNZV2p0c3pfYWd1Y2U0NnVtdlNaTGdEU3dDbEZ1QTV2WVZCUXp2bmZFVE5ETHByVmc4R1lBUFlDU2JsejNyNkNCcEk3R2lUQUpPbnl5ZS1aeWZGN0lISTVocl9leXVOdTBrN2dKdGJyVl85N0pUQlFtaEZvTXF3V2MzU0xNcTFydU5fNWZsamhnNDVqSThhVEVuaHYweTI5c1g3ZDlDOWplQl8zVGJqa3JnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA56" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AB56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC56" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AD56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-15T22:46:15+00:00</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>106.46</v>
+      </c>
+      <c r="F57" t="n">
+        <v>106.54</v>
+      </c>
+      <c r="G57" t="n">
+        <v>105.24</v>
+      </c>
+      <c r="H57" t="n">
+        <v>105.28</v>
+      </c>
+      <c r="I57" t="n">
+        <v>45485</v>
+      </c>
+      <c r="J57" t="n">
+        <v>4</v>
+      </c>
+      <c r="K57" t="n">
+        <v>40</v>
+      </c>
+      <c r="L57" t="n">
+        <v>-0.023</v>
+      </c>
+      <c r="M57" t="n">
+        <v>-0.286</v>
+      </c>
+      <c r="N57" t="n">
+        <v>40</v>
+      </c>
+      <c r="O57" t="n">
+        <v>0.132</v>
+      </c>
+      <c r="P57" t="n">
+        <v>-0.07199999999999999</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>2.179</v>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>Antioxidants for Crude Oil Market to Accelerate by 2035, Driven by Rising Heavy Sour Crude Processing - IndexBox</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQWTVSYlo2TlZ4emlNR3VPWGJPa015SW9SRWtGM1ZVZExqY0Z1S2hhUWp5UXM2a013ZW5zcm9jUXcyc0FHU0Y1RTlGSDh2Tklrc3JrLU04ZXBuQjJ5U1VnLS1Fc0Fab2RvSGx0T3N0TmVRTDBZQi1QRGxXcDBCZHBGLWYxdVc0S1VUZzlIaVB5SjF2cElDcnR3QWVSYUE0TFNUWi04T0RBVE5GSlhlQ1Utd19CSzNoMUZvOUlpYUZ3OW9xbmZsbExGSGFn?oc=5</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>London Gas Oil breaks resistance at $1,273: Live levels By Investing.com - Investing.com India</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQOFJZcEZXSVpGOEZvTVR0SGRqYmZ4WF9SZ3RKajNUVWZDM2t3U3BOa3lQWk1oMUpnOF9UTTk0eFpwdzR0TEVzbHlHelFkb0xxZ3lFX08tR0gyblJWX20xenlXMi0xNVFfSlJ4UDdVUWtZcW5hV19VRHZIS0taRmRDRzlOek1wb2hmR3lpMGhGS0ZwbVVVZ0p4NFhibHBOTkdrd0JpWnVpSDl1dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>Venezuela's withdrawal from OPEC gains traction in the oil - Inspenet</t>
+        </is>
+      </c>
+      <c r="Z57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE5Ic05DVGZPeUJyQU9nNzlrVFgzQWdFNTdVZFdEb0pRMGFYN0lRUHcwWW13ZlNUQnUtamVwdGUtT3p1X2h0SnRMbzVGLVY3dzlqS09hSF9BRFpyOWZ4Q0dvRExCT0poVTZKTWlqUjRZQW1GZ00?oc=5</t>
+        </is>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC57" t="inlineStr">
+        <is>
+          <t>VIX Breaks Out Before CPI: S&amp;P 500 Clinging to Support as Oil Gets Rejected at $104 - youtu.be</t>
+        </is>
+      </c>
+      <c r="AD57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiQkFVX3lxTE5OVDlua2JHTEZ1Y25SWWtneWdRazB4R0cwWEY1dWFRWnU0SktHYjRzc2dYOGVYZWJ4NlJxeTBYMUg4Zw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-15T22:46:15+00:00</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>99.616</v>
+      </c>
+      <c r="F58" t="n">
+        <v>99.65900000000001</v>
+      </c>
+      <c r="G58" t="n">
+        <v>99.607</v>
+      </c>
+      <c r="H58" t="n">
+        <v>99.61199999999999</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" t="n">
+        <v>4</v>
+      </c>
+      <c r="K58" t="n">
+        <v>38</v>
+      </c>
+      <c r="L58" t="n">
+        <v>-0.118</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N58" t="n">
+        <v>40</v>
+      </c>
+      <c r="O58" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="P58" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>-0.459</v>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>US Dollar outlook: Hawkish Fed repricing strengthens the bull case - stonex.com</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNRlJTZ3dmU0NMcWtjQU9uU1pXSDQ1Uk5YOGFCVTQwSlExOFZtcjBGT1VZdXppTkpqYkdoaUtTTWw0aVJxclFIaWFnWXItUzBDTkNNSGg1b0t3dVhvREJSQjJRYUFEMGpMa0pNTVpMUzdpT0YwRngyZi1nMlRCdHJlVjVkc0tvU3RqV2pPNzhtYUNhVXlWVXpPRlpiLXBFTE1KNjZoU2lZLXpUaE9CM0hTLTVRSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC58" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-15T22:46:15+00:00</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>7655.5</v>
+      </c>
+      <c r="F59" t="n">
+        <v>7666</v>
+      </c>
+      <c r="G59" t="n">
+        <v>7648</v>
+      </c>
+      <c r="H59" t="n">
+        <v>7665.5</v>
+      </c>
+      <c r="I59" t="n">
+        <v>379661</v>
+      </c>
+      <c r="J59" t="n">
+        <v>4</v>
+      </c>
+      <c r="K59" t="n">
+        <v>38</v>
+      </c>
+      <c r="L59" t="n">
+        <v>-0.237</v>
+      </c>
+      <c r="M59" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="N59" t="n">
+        <v>39</v>
+      </c>
+      <c r="O59" t="n">
+        <v>0.309</v>
+      </c>
+      <c r="P59" t="n">
+        <v>-0.078</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>1.029</v>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>Tax revenue surges amid boom in stock market - Taipei Times</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBVYTNZQ2Q4RFRxNEVSUnVLLTZRQUkyVjF1dEtOZ0hiZ1NreVV3NUx1b1RXdWNoRXZIWlB6MnhXakR3SFdvTGt5SG1NZWFLVjZrUGd4MXk0dVEzRkY5NGJkTUtWSmtwalA5RWlLXzQyVGMwN2pjcEE?oc=5</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>Illumina Stock Analysis: Bullish Trend Holds, Momentum in Focus - The Cryptonomist</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQaUstS2lxb25wVWhUUm9ZZjM4WUpYekk3Mk1VVjdHYWdaZUE2alhkXzVKMXlOOHZ0ekVOSE5EWXYtS1o2QjFyVGVockpyVWZPVXdhUTNsSFcyMEE5aFZqb0l4M045T3Z4cnNuU2t4ckpBYTNmZEhGZWstVlV2YlkzQW0zSkpNYUtzeTRYZ2NrMG9nWDhwQ0x2QTZsNVg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>Rexel stock breaks through its 35.40 € support and slides towards a floor - ideal-investisseur.fr</t>
+        </is>
+      </c>
+      <c r="AB59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxNYmJGM0Ria0tiUk8zcHJ6RExXSDFGSFVFY3Q4WXVfZldBM3NzYlNwaWxyaDhrNHhLREdNRXd2Z0R3cGpZekVJUl8tc3AweUx5Mm5uUWJ4dWh2cjhVTHFQbWQzYzFNZ2F1WEdrUTYtM2FRa1g4ckF3YTQ1RHRHQ3NxajJMbkZEWVZqZjlzaEpVbUs0UWkzb2l5R1htaG1CeXFOU1EySnJNcDNUWFd5LXVIdldidnhQTlltdFdRVUplZXFDZWt0R0FwXzlEVE1saWs?oc=5</t>
+        </is>
+      </c>
+      <c r="AC59" t="inlineStr">
+        <is>
+          <t>Stock Market Today: S&amp;P 500, Dow and Nasdaq Futures Fall as Brent Hovers Near $107 and FOMC Commences Two - benzinga.com</t>
+        </is>
+      </c>
+      <c r="AD59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingJBVV95cUxPUGk4NExHaEY5b3ZTZDk3eUpEa2hHMjA3Yjh6Szd6Z2xKSFZrQnkzcFR2QmsyWUhBSlI5d0NYRUx5amZZZEUzTVYtVEpDQkZPRlM4c1JZXzFHNVZYaWwzQXRfSFdVSUlGNEJTb2dodGpxdnBzX3FGejh4aGtIZlVFQ0RVYUZEYU9SNFMwR25wZFd2WWFpTGpyOWMxSkFxWG0tZDRoMzdhMGduWHJTdnFJdkZ5YzY1TTVGOXJtM1M1OGRUa1c0WkhNTUdlaGFIUGxVZmhELWtpX0dhV2VFalJBZXpCeFUzQjVvMUZwb2ZLRWpSS0ZvYVVlT1ZITEZTMFk3SUx4S3ZhR3lMcExSLVJtRmMyX0pjaS1Vdm5PdzB3?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-15T22:46:15+00:00</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>29263.5</v>
+      </c>
+      <c r="F60" t="n">
+        <v>29291</v>
+      </c>
+      <c r="G60" t="n">
+        <v>29207.5</v>
+      </c>
+      <c r="H60" t="n">
+        <v>29284.25</v>
+      </c>
+      <c r="I60" t="n">
+        <v>96888</v>
+      </c>
+      <c r="J60" t="n">
+        <v>4</v>
+      </c>
+      <c r="K60" t="n">
+        <v>40</v>
+      </c>
+      <c r="L60" t="n">
+        <v>-0.348</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N60" t="n">
+        <v>36</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0.264</v>
+      </c>
+      <c r="P60" t="n">
+        <v>-0.019</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>-0.215</v>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Amplitude: The Rebound Rally Is Here, Fueled By Impressive Backlog Growth (NASDAQ:AMPL) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPVFNMdU5VS0tzT25fVGpuY1ZnaTkwcTNzZGdxQldPREF0VUtGeW1JSG4yRUVZMGNYZzJiTTI0MTgzclpBU0FqNGdTTXRwLUxtdjFCUC1SRWVJNmNWQTJtcTQxWlFXRDJFRUpyaGwwQjJhcWdKUTlPUmNveDB3SjRSV0xRZHROQldCX1hxVFdEU2Rvc2tfVy1nT1ZRdlotOHZFN1pSOGg0RXk4THR1NlRSdEFB?oc=5</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Qualys gains another 7%, extends previous day's rally (QLYS:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQd2UxRm5EenY5VmZnZzh1Vy1OTmxTX2dNQmRyZzd2d3NwdW93S3lENEYxVEVPVDJWZVNwQWJzM3ltQnpxM1RuNnVGYUI5cVlEU0h5OTJqTzRUZUlJaEl5cjlMeDU2VzVfWHRHUUNBQTVSdDRyZWNmSml2ZVQzR01pcDFLa0puRWNUT1NnV2Q0bHZyUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>S&amp;P and Nasdaq hit record highs, continuing remarkable recovery from war shock - CNN</t>
+        </is>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBFM0dLbkRoQTEzbmVyNGdlZERORGZXdEJrOVh3U0FZVnJsNk0zQjFWVVF6a0NhQThTbS0zMUJTdmdHWm1JYVF3LW5VUWVJWFk1MUd6WlVNWU9aa0dENG9rbkYzRDFpcmhSQ1BJ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>QQQ: volume node tests, breaks and retests for NASDAQ:QQQ by AuctionFoundry - tradingview.com</t>
+        </is>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxORFVBaWZoUklsNVkxUDE0VnEtQUx5OEtMWlhHczdBVWl5TVhLNG5lTUp5cGxQUDdqSTVtWi1kdVFDZ296TG9LRGs0NUV1dTJYMkFNZ19jNWNicG9NbjM0UGlZUEEzTU1FeE1PQ3BMX0NyZElodmU4SHZQc3IzS3N0LTA3dUNsMFZ4a1M3Y19KZTNaQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>Dow Jones Futures: S&amp;P 500, Nasdaq Break Support; How Will Bonds React To Fed Rate Hike, Outlook? - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNcDY5cGk1b1piYWlVVV9zbXlFVjRZRjNGSDZOWUU1emRTYWd2dExlYS1wcFBPRTBTcTNQNkdLWUhrUnRtdDNjLXgzM05NblpsZjUybUlDbFdUT2JicmhzenFNUjFqa0h1Y0VLdXpvWTM1S2RyWjNaaUxzcG84ckhTNzlxM285OGdiQ3R4UVpwTEhsYTlacmc2Q09tS2VxNk15VkluVWlveUFLalNOZjVPUW9KRmFyc1BCbXRDSERmNU1EZEJGTXc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC60" t="inlineStr">
+        <is>
+          <t>Katie Stockton: Bracing for volatility after Nasdaq broke below recent support - CNBC</t>
+        </is>
+      </c>
+      <c r="AD60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLWhuVXhhdF9LbEhfSTV2RlNTZ0IyVjBlcUxGS0RQLXA5S0xjUWFZa3c3Nm1OZmxSRU5mVmVLZzRkbEFKYWd1YWFoVHdadUpRRXlMc1BSVi1BY2Q5RlVLRzVoa2xuRkxZdThVS0VVTzRYY256MHZha1l6RDlrU0NaVXZGZW1qZFRWbTBOUFBTRGxUck9ZWk9tWlY4bl9LcU1BVG5Ka0RVVURXallmZGhqT1BacEpBYnFTUzBIRQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-15T22:46:15+00:00</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>75936.78909999999</v>
+      </c>
+      <c r="F61" t="n">
+        <v>76245.52340000001</v>
+      </c>
+      <c r="G61" t="n">
+        <v>75110.0312</v>
+      </c>
+      <c r="H61" t="n">
+        <v>75633.6094</v>
+      </c>
+      <c r="I61" t="n">
+        <v>2446082048</v>
+      </c>
+      <c r="J61" t="n">
+        <v>4</v>
+      </c>
+      <c r="K61" t="n">
+        <v>39</v>
+      </c>
+      <c r="L61" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="M61" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="N61" t="n">
+        <v>36</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0.229</v>
+      </c>
+      <c r="P61" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>10.913</v>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>Bitcoin price extends gains, briefly tops $81,000 as crypto rally gathers pace - CNBC</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQdlVlbW1UcGhZSVR6dW9SVTIxX2xrREJYT2VrTnBCRENqeVp4ZUdpUERjemp6QmNLY1h0cUlVYm91OVBublNPOXh0aVdHWHdaU0JyX2gwanhxM0FuYmhfbUNOQjF4UVZPenhjd2tBaDBzbF9DbnMySkotcUpoLVVtekJld2QzcjJaUDNfWFF0cnRRY3NvUk5SMVB6MjLSAaIBQVVfeXFMUE5UVkdmUVAwazBVMTE3Rk5qNUIyTmtPZFhtUzdOVmhSQV9fUUVlT3VpUmZnQnJ5WlR5WWxsTk5ycEpwV0xOMmlkR05NQWNLVzA3R0JYSk5YUFh6NE9CTGtzVXpfeVNLb2l6TFVQUWxKOWthZGlwdHZEMlQwT0JWOEdWVXQwdlViNW9uZG5SQmZKQUhLSTdrOVpuRHBrNUV6a19B?oc=5</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - Pulse 2.0</t>
+        </is>
+      </c>
+      <c r="Z61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="AB61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC61" t="inlineStr">
+        <is>
+          <t>Bitcoin and gold touted as hedges against currency debasement as US debt tops $40 trillion - tradingview.com</t>
+        </is>
+      </c>
+      <c r="AD61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxPMFFOejYzSnZwaUdrNmdPWnEtR2V5WmVaTndxaHg3Qlk1V1Nqa1NZZ0xUaTlDbzNaTU1IaTRqc3lxY2F3eUJYV3VaVE9uWnhyTC1BVHdza3B4SW51UDcxeU5nQm9ueVdlVC11d0ExeDNVdTJtWjZNVGFnUHQxdVFtTnVaVmxvZ29ZbnJmeVVqYjBGZ2hXRF9QQ0F5UmtuQW9TUHUtMWNSTmNXRDlyYmlqZHVXaHdjT3IwcTZGdDhTcVJnWkozOWxXWkdxdS1hamdHbDNyWHdvUEZ2OXVqaTE5ZGZiaUFocDdUb0E?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-16 03:47 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD61"/>
+  <dimension ref="A1:AD67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8019,6 +8019,762 @@
         </is>
       </c>
       <c r="AD61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxPMFFOejYzSnZwaUdrNmdPWnEtR2V5WmVaTndxaHg3Qlk1V1Nqa1NZZ0xUaTlDbzNaTU1IaTRqc3lxY2F3eUJYV3VaVE9uWnhyTC1BVHdza3B4SW51UDcxeU5nQm9ueVdlVC11d0ExeDNVdTJtWjZNVGFnUHQxdVFtTnVaVmxvZ29ZbnJmeVVqYjBGZ2hXRF9QQ0F5UmtuQW9TUHUtMWNSTmNXRDlyYmlqZHVXaHdjT3IwcTZGdDhTcVJnWkozOWxXWkdxdS1hamdHbDNyWHdvUEZ2OXVqaTE5ZGZiaUFocDdUb0E?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-16T03:45:03+00:00</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>4323.8999</v>
+      </c>
+      <c r="F62" t="n">
+        <v>4381.8999</v>
+      </c>
+      <c r="G62" t="n">
+        <v>4315.2002</v>
+      </c>
+      <c r="H62" t="n">
+        <v>4370.2002</v>
+      </c>
+      <c r="I62" t="n">
+        <v>28841</v>
+      </c>
+      <c r="J62" t="n">
+        <v>4</v>
+      </c>
+      <c r="K62" t="n">
+        <v>39</v>
+      </c>
+      <c r="L62" t="n">
+        <v>-0.121</v>
+      </c>
+      <c r="M62" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="N62" t="n">
+        <v>40</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="P62" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>0.227</v>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="Z62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - fxstreet.com</t>
+        </is>
+      </c>
+      <c r="AB62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC62" t="inlineStr">
+        <is>
+          <t>Gold is the 'North Star' in a world drowning in debt - Sprott’s Ryan McIntyre - kitco.com</t>
+        </is>
+      </c>
+      <c r="AD62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxQVDhrNkQxYVJCd2x0TWx0UU5KRWNDdjYzeVY5MTJjdDA3bUs3d1hiZjNzWF9qbGRBOFZrZGlxaVQ1b2Y2RUw4RmNYM3FsU3ZDMWI0RGg5aDl4NkluMTV3SjFNNF9DSjBMRzFwZnMxcHN4VElrVlI4OXZfclY1UFlHRkF1STg4Um91MExqbFZzV3BRYk5ET3FYN2VfT29YMjlOcmg5dmp3?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-16T03:45:03+00:00</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>105.36</v>
+      </c>
+      <c r="F63" t="n">
+        <v>105.42</v>
+      </c>
+      <c r="G63" t="n">
+        <v>104.23</v>
+      </c>
+      <c r="H63" t="n">
+        <v>104.73</v>
+      </c>
+      <c r="I63" t="n">
+        <v>14061</v>
+      </c>
+      <c r="J63" t="n">
+        <v>4</v>
+      </c>
+      <c r="K63" t="n">
+        <v>40</v>
+      </c>
+      <c r="L63" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="M63" t="n">
+        <v>-0.264</v>
+      </c>
+      <c r="N63" t="n">
+        <v>40</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="P63" t="n">
+        <v>-0.08699999999999999</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Antioxidants for Crude Oil Market to Accelerate by 2035, Driven by Rising Heavy Sour Crude Processing - IndexBox</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQWTVSYlo2TlZ4emlNR3VPWGJPa015SW9SRWtGM1ZVZExqY0Z1S2hhUWp5UXM2a013ZW5zcm9jUXcyc0FHU0Y1RTlGSDh2Tklrc3JrLU04ZXBuQjJ5U1VnLS1Fc0Fab2RvSGx0T3N0TmVRTDBZQi1QRGxXcDBCZHBGLWYxdVc0S1VUZzlIaVB5SjF2cElDcnR3QWVSYUE0TFNUWi04T0RBVE5GSlhlQ1Utd19CSzNoMUZvOUlpYUZ3OW9xbmZsbExGSGFn?oc=5</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>Oil's roundtrip back to $100. Why China could determine what happens next - CNBC</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOa0xDNl91YjR4WVVvTXU5UlVvMnVQWUs0SDVCRFZFV0VxWVJzLVdsTWZuN1RiSjkxamJwdUkyVUdzZndiTXlITFdQWEVrSzJmSjN1bkczVjhhRktQSHR1UlMzMUtRalJZbmtLbDAtX0FJb1Ntb213dXFxeHMtVXh0NG5sd2ctUVdMWUJDQmF4R1U4V0hQZXQ0WVJDbVBWZDItbXAwbGxiWVFFSGs?oc=5</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AB63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC63" t="inlineStr">
+        <is>
+          <t>VIX Breaks Out Before CPI: S&amp;P 500 Clinging to Support as Oil Gets Rejected at $104 - YouTube</t>
+        </is>
+      </c>
+      <c r="AD63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiQkFVX3lxTE5OVDlua2JHTEZ1Y25SWWtneWdRazB4R0cwWEY1dWFRWnU0SktHYjRzc2dYOGVYZWJ4NlJxeTBYMUg4Zw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-16T03:45:03+00:00</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>99.681</v>
+      </c>
+      <c r="F64" t="n">
+        <v>99.735</v>
+      </c>
+      <c r="G64" t="n">
+        <v>99.63500000000001</v>
+      </c>
+      <c r="H64" t="n">
+        <v>99.658</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" t="n">
+        <v>4</v>
+      </c>
+      <c r="K64" t="n">
+        <v>39</v>
+      </c>
+      <c r="L64" t="n">
+        <v>-0.052</v>
+      </c>
+      <c r="M64" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="N64" t="n">
+        <v>40</v>
+      </c>
+      <c r="O64" t="n">
+        <v>0.231</v>
+      </c>
+      <c r="P64" t="n">
+        <v>-0.023</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>3.107</v>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>US Dollar outlook: Hawkish Fed repricing strengthens the bull case - stonex.com</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNRlJTZ3dmU0NMcWtjQU9uU1pXSDQ1Uk5YOGFCVTQwSlExOFZtcjBGT1VZdXppTkpqYkdoaUtTTWw0aVJxclFIaWFnWXItUzBDTkNNSGg1b0t3dVhvREJSQjJRYUFEMGpMa0pNTVpMUzdpT0YwRngyZi1nMlRCdHJlVjVkc0tvU3RqV2pPNzhtYUNhVXlWVXpPRlpiLXBFTE1KNjZoU2lZLXpUaE9CM0hTLTVRSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - fxstreet.com</t>
+        </is>
+      </c>
+      <c r="AB64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC64" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-16T03:45:03+00:00</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>7665.5</v>
+      </c>
+      <c r="F65" t="n">
+        <v>7678</v>
+      </c>
+      <c r="G65" t="n">
+        <v>7658.75</v>
+      </c>
+      <c r="H65" t="n">
+        <v>7671.5</v>
+      </c>
+      <c r="I65" t="n">
+        <v>30666</v>
+      </c>
+      <c r="J65" t="n">
+        <v>4</v>
+      </c>
+      <c r="K65" t="n">
+        <v>38</v>
+      </c>
+      <c r="L65" t="n">
+        <v>-0.08799999999999999</v>
+      </c>
+      <c r="M65" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="N65" t="n">
+        <v>38</v>
+      </c>
+      <c r="O65" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="P65" t="n">
+        <v>-0.061</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>5.446</v>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Tax revenue surges amid boom in stock market - Taipei Times</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBVYTNZQ2Q4RFRxNEVSUnVLLTZRQUkyVjF1dEtOZ0hiZ1NreVV3NUx1b1RXdWNoRXZIWlB6MnhXakR3SFdvTGt5SG1NZWFLVjZrUGd4MXk0dVEzRkY5NGJkTUtWSmtwalA5RWlLXzQyVGMwN2pjcEE?oc=5</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Illumina Stock Analysis: Bullish Trend Holds, Momentum in Focus - The Cryptonomist</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQaUstS2lxb25wVWhUUm9ZZjM4WUpYekk3Mk1VVjdHYWdaZUE2alhkXzVKMXlOOHZ0ekVOSE5EWXYtS1o2QjFyVGVockpyVWZPVXdhUTNsSFcyMEE5aFZqb0l4M045T3Z4cnNuU2t4ckpBYTNmZEhGZWstVlV2YlkzQW0zSkpNYUtzeTRYZ2NrMG9nWDhwQ0x2QTZsNVg?oc=5</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 11: HPE Surges on AI Infrastructure Demand and Recently Raised Guidance - The Globe and Mail</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxOYXB1N0ZORG4ycmM4b2wtdEFqWFRRQVluWkNOYV81RUhYVU9RQ1QyZnoxTlZuNldUYWZXUzAwVmdITHNhS1VOa252ZDdPUTVFdDZlSjl3R2N1MURkQzF6dU5sdHkyU05Nd0hfckJRTFhSTW1STEdsbE96MW9rMDZNM2xMUXpodDJyR2tCR2JhWTZRbXFmQkNPU3pSTTVad0Ywd0loVkZhWnNpaXo1OXZrOWp0ZkJUQVR3SVJXVVlBc1NNMC1NenRiQVBBRHhPNUtiVDBhRGFiVFBiRG5JRVNNU1d3WTNyblE1TFp2OWZpUHQ4Q2hQSEV4T2FoM2VKREVnOW9OTF9tb250anc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>The Fed has to walk a fine line Wednesday. How the stock market may react, according to JPMorgan - CNBC</t>
+        </is>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxOTzM4VU4tbFZGTzNNVklGTGdqcVA5d0NfbXRlc3pKSWZHZVdfa3dGdzhKazQxNFBIRjhVN2RWMm13UV9za1NCVkpIbUtSRW1KMUlydmZENS14NW1PczBib1BiUmtUT2NxQm41SThmVUl6b24yVDNtbXdKeFhSTEpHS1F6aEg0dHJkNmE0MWg5czU4OFpwV1ZUeTVXd3RnR2NTQ3EyUXI0aW1PSEFVM0NjNWZR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB65" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC65" t="inlineStr">
+        <is>
+          <t>Stock Market Today: S&amp;P 500, Dow and Nasdaq Futures Fall as Brent Hovers Near $107 and FOMC Commences Two - Benzinga</t>
+        </is>
+      </c>
+      <c r="AD65" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingJBVV95cUxPUGk4NExHaEY5b3ZTZDk3eUpEa2hHMjA3Yjh6Szd6Z2xKSFZrQnkzcFR2QmsyWUhBSlI5d0NYRUx5amZZZEUzTVYtVEpDQkZPRlM4c1JZXzFHNVZYaWwzQXRfSFdVSUlGNEJTb2dodGpxdnBzX3FGejh4aGtIZlVFQ0RVYUZEYU9SNFMwR25wZFd2WWFpTGpyOWMxSkFxWG0tZDRoMzdhMGduWHJTdnFJdkZ5YzY1TTVGOXJtM1M1OGRUa1c0WkhNTUdlaGFIUGxVZmhELWtpX0dhV2VFalJBZXpCeFUzQjVvMUZwb2ZLRWpSS0ZvYVVlT1ZITEZTMFk3SUx4S3ZhR3lMcExSLVJtRmMyX0pjaS1Vdm5PdzB3?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-09-16T03:45:03+00:00</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>29277.5</v>
+      </c>
+      <c r="F66" t="n">
+        <v>29358.5</v>
+      </c>
+      <c r="G66" t="n">
+        <v>29226</v>
+      </c>
+      <c r="H66" t="n">
+        <v>29305.25</v>
+      </c>
+      <c r="I66" t="n">
+        <v>22646</v>
+      </c>
+      <c r="J66" t="n">
+        <v>4</v>
+      </c>
+      <c r="K66" t="n">
+        <v>40</v>
+      </c>
+      <c r="L66" t="n">
+        <v>-0.322</v>
+      </c>
+      <c r="M66" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="N66" t="n">
+        <v>35</v>
+      </c>
+      <c r="O66" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="P66" t="n">
+        <v>-0.047</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>1.692</v>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Amplitude: The Rebound Rally Is Here, Fueled By Impressive Backlog Growth (NASDAQ:AMPL) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPVFNMdU5VS0tzT25fVGpuY1ZnaTkwcTNzZGdxQldPREF0VUtGeW1JSG4yRUVZMGNYZzJiTTI0MTgzclpBU0FqNGdTTXRwLUxtdjFCUC1SRWVJNmNWQTJtcTQxWlFXRDJFRUpyaGwwQjJhcWdKUTlPUmNveDB3SjRSV0xRZHROQldCX1hxVFdEU2Rvc2tfVy1nT1ZRdlotOHZFN1pSOGg0RXk4THR1NlRSdEFB?oc=5</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>Qualys gains another 7%, extends previous day's rally (QLYS:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQd2UxRm5EenY5VmZnZzh1Vy1OTmxTX2dNQmRyZzd2d3NwdW93S3lENEYxVEVPVDJWZVNwQWJzM3ltQnpxM1RuNnVGYUI5cVlEU0h5OTJqTzRUZUlJaEl5cjlMeDU2VzVfWHRHUUNBQTVSdDRyZWNmSml2ZVQzR01pcDFLa0puRWNUT1NnV2Q0bHZyUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>CrowdStrike jumps 14% amid cybersecurity sector rally (CRWD:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQMlJKdG1qdU5YMnRHRE1GaEIxbHpRNTFYSldxMnZzSmVEQ3dDTmVfMXJ1XzZJTGdGbzhsZXdwQ3l2NVBEU3YtQ3V1U3RGQWNISTBIcmxRQk40dFpMNm41SlZaVktvMkp0NDZuTjVGZ1dSNlU3NEpLaGxHamlzTjk4OFdiYXZ5Z1Jmd1Uwc3RYMGEtMl9IZHJVRkl4LWt3YjA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>QQQ: volume node tests, breaks and retests for NASDAQ:QQQ by AuctionFoundry - TradingView</t>
+        </is>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxORFVBaWZoUklsNVkxUDE0VnEtQUx5OEtMWlhHczdBVWl5TVhLNG5lTUp5cGxQUDdqSTVtWi1kdVFDZ296TG9LRGs0NUV1dTJYMkFNZ19jNWNicG9NbjM0UGlZUEEzTU1FeE1PQ3BMX0NyZElodmU4SHZQc3IzS3N0LTA3dUNsMFZ4a1M3Y19KZTNaQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>BREAKING 🚨 Nasdaq tumbles 2.4%, Bitcoin tests key $60K support - XTB.com</t>
+        </is>
+      </c>
+      <c r="AB66" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNckVRZWlwM05WMndXTGljRENoYlNnZkZ0S1hEQ2VDcFhWVTVKd2ktT0M2bEF3TmNTR2tiLTlpcEZ3VE90dWFMTFFsdVozVnRyNXB6Y0kycS00VHRIei0tWnRSRHdnLXJTeEZBVWxFN1Y3UWlIcVNyNjRTc3B0dW1VNHBmbTJmeUdZWERpaXIteU5QdDl1RERZbW9NNndnTzlIRkVWUGlLLXJKVkZrazZmUUVRcnA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC66" t="inlineStr">
+        <is>
+          <t>Katie Stockton: Bracing for volatility after Nasdaq broke below recent support - CNBC</t>
+        </is>
+      </c>
+      <c r="AD66" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLWhuVXhhdF9LbEhfSTV2RlNTZ0IyVjBlcUxGS0RQLXA5S0xjUWFZa3c3Nm1OZmxSRU5mVmVLZzRkbEFKYWd1YWFoVHdadUpRRXlMc1BSVi1BY2Q5RlVLRzVoa2xuRkxZdThVS0VVTzRYY256MHZha1l6RDlrU0NaVXZGZW1qZFRWbTBOUFBTRGxUck9ZWk9tWlY4bl9LcU1BVG5Ka0RVVURXallmZGhqT1BacEpBYnFTUzBIRQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-09-16T03:45:03+00:00</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>75594.4531</v>
+      </c>
+      <c r="F67" t="n">
+        <v>76030.24219999999</v>
+      </c>
+      <c r="G67" t="n">
+        <v>75403.00780000001</v>
+      </c>
+      <c r="H67" t="n">
+        <v>75743.32030000001</v>
+      </c>
+      <c r="I67" t="n">
+        <v>6206447616</v>
+      </c>
+      <c r="J67" t="n">
+        <v>4</v>
+      </c>
+      <c r="K67" t="n">
+        <v>39</v>
+      </c>
+      <c r="L67" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="M67" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="N67" t="n">
+        <v>36</v>
+      </c>
+      <c r="O67" t="n">
+        <v>0.284</v>
+      </c>
+      <c r="P67" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>13.197</v>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>Bitmine Surges 8% on Ethereum Strength After Cantor Fitzgerald Doubles Its Target, SharpLink Advances 9%, Strategy Gains 4% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPemN4ODV3YldjcDUxb1FRWXc1OWV4bXZwVEhOWTMtbDJaNG92V0xpd0V6OTBxM3lRN0RZUEtWQkRWQW9Kb0hNUF8zS2FBOU5BUlpFTmpvNFBiYnpSVEhHMmtCU2JMdzNjRlNXRWtwaUM1eUxrVjRWQ3VQT2Q4MVJHaHBfdHBRUFpETTVnT012dEJQQV9mcHNOOHUwQnlVU2ZibW51TTBzMHdvTXhsQnlMMzJjT0lhcTNvVktGLTVfN1o3ZXlkLV9JNWRZVVFvakVaaDdIMGxWdFJXUVMxT19rREpueFJibmw0WllRUDk1ckgwUHB1?oc=5</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - Pulse 2.0</t>
+        </is>
+      </c>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>Bernstein Is Calling $150,000 Bitcoin by December, But Prediction Markets Are Pricing $75,000 - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB67" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxNZXl2aFYzMEJFVHg0UTQwbDJBb3lXeWx0ZDFmVVU5dG1heTFSSGNCZmgtMnRFcTZocHQyeDY2YVk2WHR6ckVsU0pJS01vTFd4SUZqRGoxMHl5QmZxQmhIWU9Xd1Y4cEtCd3gtdHc0aFBuX0puLWVzSzM0eE15Q2dWaWRjNk5MZUVKUkpXYkVZVUJPTUFrbzVobml2OGJkS29qWlItRUVvQUdtc25UX0YwbGlBeW5pTWZnX3QydUVTRDRjdVJtUFRqbzdJZ2x3cVNQazdPRTg1eTVPUXp3bXRCRQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC67" t="inlineStr">
+        <is>
+          <t>Bitcoin and gold touted as hedges against currency debasement as US debt tops $40 trillion - TradingView</t>
+        </is>
+      </c>
+      <c r="AD67" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxPMFFOejYzSnZwaUdrNmdPWnEtR2V5WmVaTndxaHg3Qlk1V1Nqa1NZZ0xUaTlDbzNaTU1IaTRqc3lxY2F3eUJYV3VaVE9uWnhyTC1BVHdza3B4SW51UDcxeU5nQm9ueVdlVC11d0ExeDNVdTJtWjZNVGFnUHQxdVFtTnVaVmxvZ29ZbnJmeVVqYjBGZ2hXRF9QQ0F5UmtuQW9TUHUtMWNSTmNXRDlyYmlqZHVXaHdjT3IwcTZGdDhTcVJnWkozOWxXWkdxdS1hamdHbDNyWHdvUEZ2OXVqaTE5ZGZiaUFocDdUb0E?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-16 09:11 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD67"/>
+  <dimension ref="A1:AD73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8775,6 +8775,762 @@
         </is>
       </c>
       <c r="AD67" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxPMFFOejYzSnZwaUdrNmdPWnEtR2V5WmVaTndxaHg3Qlk1V1Nqa1NZZ0xUaTlDbzNaTU1IaTRqc3lxY2F3eUJYV3VaVE9uWnhyTC1BVHdza3B4SW51UDcxeU5nQm9ueVdlVC11d0ExeDNVdTJtWjZNVGFnUHQxdVFtTnVaVmxvZ29ZbnJmeVVqYjBGZ2hXRF9QQ0F5UmtuQW9TUHUtMWNSTmNXRDlyYmlqZHVXaHdjT3IwcTZGdDhTcVJnWkozOWxXWkdxdS1hamdHbDNyWHdvUEZ2OXVqaTE5ZGZiaUFocDdUb0E?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-16T09:09:43+00:00</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>4366.8999</v>
+      </c>
+      <c r="F68" t="n">
+        <v>4379.1001</v>
+      </c>
+      <c r="G68" t="n">
+        <v>4361.7002</v>
+      </c>
+      <c r="H68" t="n">
+        <v>4371.2002</v>
+      </c>
+      <c r="I68" t="n">
+        <v>16438</v>
+      </c>
+      <c r="J68" t="n">
+        <v>4</v>
+      </c>
+      <c r="K68" t="n">
+        <v>39</v>
+      </c>
+      <c r="L68" t="n">
+        <v>-0.138</v>
+      </c>
+      <c r="M68" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="N68" t="n">
+        <v>40</v>
+      </c>
+      <c r="O68" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="P68" t="n">
+        <v>-0.028</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>-0.803</v>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>Gold hits record high as investors seek safety - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVWt1Y1hBWG5uZFNjRUFtZHlqRUhfZGV6VzAtQ0tBT2VlVDVEZEJ2WHN0YndCcXRzSjNtVnFhUFZZZ2F4RFRxYkdsSF91eDk2MFl5R3JNWk1HREJjSVdhUE1uTTU1N1Z6Y2xfZzZCSDZ4YnhaT1czcWdXeHE3SjJBR2FqUm43Z0paUG5OVEdsWVdYYnZBWVHSAZsBQVVfeXFMTWh6VXlqZGZVbUl3SHVfQ195WFFveEVkLU9TU1RXMTZBdVhodU16UWxLLWVScDNsc2VGMThyT0RTTHB4SVNRYU1KWmRycHhnTEc0NTJ1RWgzdGc2Y0VkanR4QUtlUWFBSnB2cElORUltQk9XdWRLNXhKbU5jRUFqQVd6bG5YbURJakxhNTl3UEk4RzBaQzVJaVdRdFk?oc=5</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="Z68" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE1RUlV0Nm0zNm5aN2V4SzY0SXRSa25YSGlDNHhWeG0zS0lWYUI5U08weWF0Q25FTVZLRzJiRXE3VnZxSUFQVUp5ZW9hSFJuRGljUU9XT0F6aDNqa0d4XzFmaEJ0R0EwZGZiX1JTZlJhZUo2aExX?oc=5</t>
+        </is>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB68" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC68" t="inlineStr">
+        <is>
+          <t>Gold is the 'North Star' in a world drowning in debt - Sprott’s Ryan McIntyre - KITCO</t>
+        </is>
+      </c>
+      <c r="AD68" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxQVDhrNkQxYVJCd2x0TWx0UU5KRWNDdjYzeVY5MTJjdDA3bUs3d1hiZjNzWF9qbGRBOFZrZGlxaVQ1b2Y2RUw4RmNYM3FsU3ZDMWI0RGg5aDl4NkluMTV3SjFNNF9DSjBMRzFwZnMxcHN4VElrVlI4OXZfclY1UFlHRkF1STg4Um91MExqbFZzV3BRYk5ET3FYN2VfT29YMjlOcmg5dmp3?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-16T09:09:43+00:00</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>104.83</v>
+      </c>
+      <c r="F69" t="n">
+        <v>104.89</v>
+      </c>
+      <c r="G69" t="n">
+        <v>103.76</v>
+      </c>
+      <c r="H69" t="n">
+        <v>104.49</v>
+      </c>
+      <c r="I69" t="n">
+        <v>23700</v>
+      </c>
+      <c r="J69" t="n">
+        <v>4</v>
+      </c>
+      <c r="K69" t="n">
+        <v>40</v>
+      </c>
+      <c r="L69" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M69" t="n">
+        <v>-0.301</v>
+      </c>
+      <c r="N69" t="n">
+        <v>40</v>
+      </c>
+      <c r="O69" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="P69" t="n">
+        <v>-0.136</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>0.658</v>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>Antioxidants for Crude Oil Market to Accelerate by 2035, Driven by Rising Heavy Sour Crude Processing - IndexBox</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQWTVSYlo2TlZ4emlNR3VPWGJPa015SW9SRWtGM1ZVZExqY0Z1S2hhUWp5UXM2a013ZW5zcm9jUXcyc0FHU0Y1RTlGSDh2Tklrc3JrLU04ZXBuQjJ5U1VnLS1Fc0Fab2RvSGx0T3N0TmVRTDBZQi1QRGxXcDBCZHBGLWYxdVc0S1VUZzlIaVB5SjF2cElDcnR3QWVSYUE0TFNUWi04T0RBVE5GSlhlQ1Utd19CSzNoMUZvOUlpYUZ3OW9xbmZsbExGSGFn?oc=5</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>Japan imports surge 28% in August as energy costs widen trade gap - Sharjah24</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE0tRXZ6Q0VFOEMyVU9ya2JWdlZCa2l3c2tkaGdZYVdpeV9maVRZRVZuV3k3UkxGcTBMN2YyZEMtbEtiaWNGRkNUYTBiRUJTbzhCdkNtYlZ6emxHTWc?oc=5</t>
+        </is>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>Venezuela's withdrawal from OPEC gains traction in the oil - Inspenet</t>
+        </is>
+      </c>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE5Ic05DVGZPeUJyQU9nNzlrVFgzQWdFNTdVZFdEb0pRMGFYN0lRUHcwWW13ZlNUQnUtamVwdGUtT3p1X2h0SnRMbzVGLVY3dzlqS09hSF9BRFpyOWZ4Q0dvRExCT0poVTZKTWlqUjRZQW1GZ00?oc=5</t>
+        </is>
+      </c>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB69" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC69" t="inlineStr">
+        <is>
+          <t>OPEC oil output falls in August, Reuters survey shows - Reuters</t>
+        </is>
+      </c>
+      <c r="AD69" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcGZWQVVsSEY1MDZDLXRVM2g2N0t1bHJ1VXpWX3pScTFZak53OGQ5VVNxemw0Mjdrd1paNjRYb1YtdFlYN3RIOURKM00xZmc4eFRlTHk2cTNhODJKWW5TOS1BMEE1cVF2NTN5YjJaeHRRNFlBVHUwUU9CN0pyOEdRMHE0c2VtcGNvamRPVFd3OVVlTnFmV3Fobks2WlZJU21oRW44?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-16T09:09:43+00:00</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>99.57899999999999</v>
+      </c>
+      <c r="F70" t="n">
+        <v>99.66</v>
+      </c>
+      <c r="G70" t="n">
+        <v>99.53700000000001</v>
+      </c>
+      <c r="H70" t="n">
+        <v>99.654</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" t="n">
+        <v>4</v>
+      </c>
+      <c r="K70" t="n">
+        <v>39</v>
+      </c>
+      <c r="L70" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="M70" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="N70" t="n">
+        <v>39</v>
+      </c>
+      <c r="O70" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="P70" t="n">
+        <v>-0.047</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>1.806</v>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Major Banks' Dollar Insurance Sales Triple Amid Won Strength - 조선일보</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPampQV05WMEh5VXhCSGt0a2FGLWtUVFFLcXh0dUV4TTJkZHNHNGV1aHB0S0ViSmx4NnZ2dTdraTZWWDZXOXJ2MndUU3p0ZzdsRGJvdXJBQzlrb0RHYUhWMFNGOC13X1ZRaVY3aExvVzZxcFhSTVhad01aSm5OOHFwTUNwdHZ4T0ZKZFQ4d2FR?oc=5</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>US Dollar outlook: Hawkish Fed repricing strengthens the bull case - stonex.com</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNRlJTZ3dmU0NMcWtjQU9uU1pXSDQ1Uk5YOGFCVTQwSlExOFZtcjBGT1VZdXppTkpqYkdoaUtTTWw0aVJxclFIaWFnWXItUzBDTkNNSGg1b0t3dVhvREJSQjJRYUFEMGpMa0pNTVpMUzdpT0YwRngyZi1nMlRCdHJlVjVkc0tvU3RqV2pPNzhtYUNhVXlWVXpPRlpiLXBFTE1KNjZoU2lZLXpUaE9CM0hTLTVRSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z70" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB70" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC70" t="inlineStr">
+        <is>
+          <t>Indonesian Rupiah gains as US Dollar weakens ahead of Fed rate decision - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD70" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOc09LZlhsd3FaTkpSdlVWb0pfR0l6c0VCWFlmcmh2bWN0VTQwRjFwTThtS0o3VEY5cVBBck9FWExBY3pCWS0tNnh3S0dmWmpuWFdubGtUQ1ZvZnkydkExNU03OXlhMGhDd3BiMmRwTG9LeFZxOGJnVy1JS1dreTVwLVdicTU4OVNxVW1aN3pHWFpZeHdWUTVvNVRVUXNJUlhCUTVqaWd6NHdxaG8tak9iU0dpTUg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-16T09:09:43+00:00</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>7670.5</v>
+      </c>
+      <c r="F71" t="n">
+        <v>7678</v>
+      </c>
+      <c r="G71" t="n">
+        <v>7663.5</v>
+      </c>
+      <c r="H71" t="n">
+        <v>7672</v>
+      </c>
+      <c r="I71" t="n">
+        <v>47910</v>
+      </c>
+      <c r="J71" t="n">
+        <v>4</v>
+      </c>
+      <c r="K71" t="n">
+        <v>39</v>
+      </c>
+      <c r="L71" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="N71" t="n">
+        <v>39</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0.398</v>
+      </c>
+      <c r="P71" t="n">
+        <v>-0.079</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>7.269</v>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>Tax revenue surges amid boom in stock market - Taipei Times</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBVYTNZQ2Q4RFRxNEVSUnVLLTZRQUkyVjF1dEtOZ0hiZ1NreVV3NUx1b1RXdWNoRXZIWlB6MnhXakR3SFdvTGt5SG1NZWFLVjZrUGd4MXk0dVEzRkY5NGJkTUtWSmtwalA5RWlLXzQyVGMwN2pjcEE?oc=5</t>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>Illumina Stock Analysis: Bullish Trend Holds, Momentum in Focus - The Cryptonomist</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQaUstS2lxb25wVWhUUm9ZZjM4WUpYekk3Mk1VVjdHYWdaZUE2alhkXzVKMXlOOHZ0ekVOSE5EWXYtS1o2QjFyVGVockpyVWZPVXdhUTNsSFcyMEE5aFZqb0l4M045T3Z4cnNuU2t4ckpBYTNmZEhGZWstVlV2YlkzQW0zSkpNYUtzeTRYZ2NrMG9nWDhwQ0x2QTZsNVg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>The Fed has to walk a fine line Wednesday. How the stock market may react, according to JPMorgan - CNBC</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxOTzM4VU4tbFZGTzNNVklGTGdqcVA5d0NfbXRlc3pKSWZHZVdfa3dGdzhKazQxNFBIRjhVN2RWMm13UV9za1NCVkpIbUtSRW1KMUlydmZENS14NW1PczBib1BiUmtUT2NxQm41SThmVUl6b24yVDNtbXdKeFhSTEpHS1F6aEg0dHJkNmE0MWg5czU4OFpwV1ZUeTVXd3RnR2NTQ3EyUXI0aW1PSEFVM0NjNWZR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>Rexel stock breaks through its 35.40 € support and slides towards a floor - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB71" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxNYmJGM0Ria0tiUk8zcHJ6RExXSDFGSFVFY3Q4WXVfZldBM3NzYlNwaWxyaDhrNHhLREdNRXd2Z0R3cGpZekVJUl8tc3AweUx5Mm5uUWJ4dWh2cjhVTHFQbWQzYzFNZ2F1WEdrUTYtM2FRa1g4ckF3YTQ1RHRHQ3NxajJMbkZEWVZqZjlzaEpVbUs0UWkzb2l5R1htaG1CeXFOU1EySnJNcDNUWFd5LXVIdldidnhQTlltdFdRVUplZXFDZWt0R0FwXzlEVE1saWs?oc=5</t>
+        </is>
+      </c>
+      <c r="AC71" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD71" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-16T09:09:43+00:00</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>29334</v>
+      </c>
+      <c r="F72" t="n">
+        <v>29398</v>
+      </c>
+      <c r="G72" t="n">
+        <v>29326</v>
+      </c>
+      <c r="H72" t="n">
+        <v>29369.5</v>
+      </c>
+      <c r="I72" t="n">
+        <v>23359</v>
+      </c>
+      <c r="J72" t="n">
+        <v>4</v>
+      </c>
+      <c r="K72" t="n">
+        <v>40</v>
+      </c>
+      <c r="L72" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="M72" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="N72" t="n">
+        <v>35</v>
+      </c>
+      <c r="O72" t="n">
+        <v>0.224</v>
+      </c>
+      <c r="P72" t="n">
+        <v>-0.059</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>-0.5649999999999999</v>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Amplitude: The Rebound Rally Is Here, Fueled By Impressive Backlog Growth (NASDAQ:AMPL) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPVFNMdU5VS0tzT25fVGpuY1ZnaTkwcTNzZGdxQldPREF0VUtGeW1JSG4yRUVZMGNYZzJiTTI0MTgzclpBU0FqNGdTTXRwLUxtdjFCUC1SRWVJNmNWQTJtcTQxWlFXRDJFRUpyaGwwQjJhcWdKUTlPUmNveDB3SjRSV0xRZHROQldCX1hxVFdEU2Rvc2tfVy1nT1ZRdlotOHZFN1pSOGg0RXk4THR1NlRSdEFB?oc=5</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>Qualys gains another 7%, extends previous day's rally (QLYS:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQd2UxRm5EenY5VmZnZzh1Vy1OTmxTX2dNQmRyZzd2d3NwdW93S3lENEYxVEVPVDJWZVNwQWJzM3ltQnpxM1RuNnVGYUI5cVlEU0h5OTJqTzRUZUlJaEl5cjlMeDU2VzVfWHRHUUNBQTVSdDRyZWNmSml2ZVQzR01pcDFLa0puRWNUT1NnV2Q0bHZyUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>S&amp;P and Nasdaq hit record highs, continuing remarkable recovery from war shock - CNN</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBFM0dLbkRoQTEzbmVyNGdlZERORGZXdEJrOVh3U0FZVnJsNk0zQjFWVVF6a0NhQThTbS0zMUJTdmdHWm1JYVF3LW5VUWVJWFk1MUd6WlVNWU9aa0dENG9rbkYzRDFpcmhSQ1BJ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>QQQ: volume node tests, breaks and retests for NASDAQ:QQQ by AuctionFoundry - TradingView</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxORFVBaWZoUklsNVkxUDE0VnEtQUx5OEtMWlhHczdBVWl5TVhLNG5lTUp5cGxQUDdqSTVtWi1kdVFDZ296TG9LRGs0NUV1dTJYMkFNZ19jNWNicG9NbjM0UGlZUEEzTU1FeE1PQ3BMX0NyZElodmU4SHZQc3IzS3N0LTA3dUNsMFZ4a1M3Y19KZTNaQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t>BREAKING 🚨 Nasdaq tumbles 2.4%, Bitcoin tests key $60K support - XTB.com</t>
+        </is>
+      </c>
+      <c r="AB72" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNckVRZWlwM05WMndXTGljRENoYlNnZkZ0S1hEQ2VDcFhWVTVKd2ktT0M2bEF3TmNTR2tiLTlpcEZ3VE90dWFMTFFsdVozVnRyNXB6Y0kycS00VHRIei0tWnRSRHdnLXJTeEZBVWxFN1Y3UWlIcVNyNjRTc3B0dW1VNHBmbTJmeUdZWERpaXIteU5QdDl1RERZbW9NNndnTzlIRkVWUGlLLXJKVkZrazZmUUVRcnA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC72" t="inlineStr">
+        <is>
+          <t>Katie Stockton: Bracing for volatility after Nasdaq broke below recent support - CNBC</t>
+        </is>
+      </c>
+      <c r="AD72" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLWhuVXhhdF9LbEhfSTV2RlNTZ0IyVjBlcUxGS0RQLXA5S0xjUWFZa3c3Nm1OZmxSRU5mVmVLZzRkbEFKYWd1YWFoVHdadUpRRXlMc1BSVi1BY2Q5RlVLRzVoa2xuRkxZdThVS0VVTzRYY256MHZha1l6RDlrU0NaVXZGZW1qZFRWbTBOUFBTRGxUck9ZWk9tWlY4bl9LcU1BVG5Ka0RVVURXallmZGhqT1BacEpBYnFTUzBIRQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-09-16T09:09:43+00:00</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>75929.1562</v>
+      </c>
+      <c r="F73" t="n">
+        <v>76025.1562</v>
+      </c>
+      <c r="G73" t="n">
+        <v>75284.36719999999</v>
+      </c>
+      <c r="H73" t="n">
+        <v>75775.1875</v>
+      </c>
+      <c r="I73" t="n">
+        <v>4259074048</v>
+      </c>
+      <c r="J73" t="n">
+        <v>4</v>
+      </c>
+      <c r="K73" t="n">
+        <v>37</v>
+      </c>
+      <c r="L73" t="n">
+        <v>0.222</v>
+      </c>
+      <c r="M73" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="N73" t="n">
+        <v>34</v>
+      </c>
+      <c r="O73" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P73" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>12.414</v>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>Bitmine Surges 8% on Ethereum Strength After Cantor Fitzgerald Doubles Its Target, SharpLink Advances 9%, Strategy Gains 4% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPemN4ODV3YldjcDUxb1FRWXc1OWV4bXZwVEhOWTMtbDJaNG92V0xpd0V6OTBxM3lRN0RZUEtWQkRWQW9Kb0hNUF8zS2FBOU5BUlpFTmpvNFBiYnpSVEhHMmtCU2JMdzNjRlNXRWtwaUM1eUxrVjRWQ3VQT2Q4MVJHaHBfdHBRUFpETTVnT012dEJQQV9mcHNOOHUwQnlVU2ZibW51TTBzMHdvTXhsQnlMMzJjT0lhcTNvVktGLTVfN1o3ZXlkLV9JNWRZVVFvakVaaDdIMGxWdFJXUVMxT19rREpueFJibmw0WllRUDk1ckgwUHB1?oc=5</t>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - pulse2.com</t>
+        </is>
+      </c>
+      <c r="Z73" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA73" t="inlineStr">
+        <is>
+          <t>Bernstein Is Calling $150,000 Bitcoin by December, But Prediction Markets Are Pricing $75,000 - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB73" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxNZXl2aFYzMEJFVHg0UTQwbDJBb3lXeWx0ZDFmVVU5dG1heTFSSGNCZmgtMnRFcTZocHQyeDY2YVk2WHR6ckVsU0pJS01vTFd4SUZqRGoxMHl5QmZxQmhIWU9Xd1Y4cEtCd3gtdHc0aFBuX0puLWVzSzM0eE15Q2dWaWRjNk5MZUVKUkpXYkVZVUJPTUFrbzVobml2OGJkS29qWlItRUVvQUdtc25UX0YwbGlBeW5pTWZnX3QydUVTRDRjdVJtUFRqbzdJZ2x3cVNQazdPRTg1eTVPUXp3bXRCRQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC73" t="inlineStr">
+        <is>
+          <t>Bitcoin and gold touted as hedges against currency debasement as US debt tops $40 trillion - TradingView</t>
+        </is>
+      </c>
+      <c r="AD73" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxPMFFOejYzSnZwaUdrNmdPWnEtR2V5WmVaTndxaHg3Qlk1V1Nqa1NZZ0xUaTlDbzNaTU1IaTRqc3lxY2F3eUJYV3VaVE9uWnhyTC1BVHdza3B4SW51UDcxeU5nQm9ueVdlVC11d0ExeDNVdTJtWjZNVGFnUHQxdVFtTnVaVmxvZ29ZbnJmeVVqYjBGZ2hXRF9QQ0F5UmtuQW9TUHUtMWNSTmNXRDlyYmlqZHVXaHdjT3IwcTZGdDhTcVJnWkozOWxXWkdxdS1hamdHbDNyWHdvUEZ2OXVqaTE5ZGZiaUFocDdUb0E?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-16 16:21 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD73"/>
+  <dimension ref="A1:AD79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9533,6 +9533,762 @@
       <c r="AD73" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxPMFFOejYzSnZwaUdrNmdPWnEtR2V5WmVaTndxaHg3Qlk1V1Nqa1NZZ0xUaTlDbzNaTU1IaTRqc3lxY2F3eUJYV3VaVE9uWnhyTC1BVHdza3B4SW51UDcxeU5nQm9ueVdlVC11d0ExeDNVdTJtWjZNVGFnUHQxdVFtTnVaVmxvZ29ZbnJmeVVqYjBGZ2hXRF9QQ0F5UmtuQW9TUHUtMWNSTmNXRDlyYmlqZHVXaHdjT3IwcTZGdDhTcVJnWkozOWxXWkdxdS1hamdHbDNyWHdvUEZ2OXVqaTE5ZGZiaUFocDdUb0E?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-09-16T16:19:24+00:00</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>4388.5</v>
+      </c>
+      <c r="F74" t="n">
+        <v>4405.2002</v>
+      </c>
+      <c r="G74" t="n">
+        <v>4364.5</v>
+      </c>
+      <c r="H74" t="n">
+        <v>4391.2998</v>
+      </c>
+      <c r="I74" t="n">
+        <v>44629</v>
+      </c>
+      <c r="J74" t="n">
+        <v>4</v>
+      </c>
+      <c r="K74" t="n">
+        <v>39</v>
+      </c>
+      <c r="L74" t="n">
+        <v>-0.194</v>
+      </c>
+      <c r="M74" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="N74" t="n">
+        <v>40</v>
+      </c>
+      <c r="O74" t="n">
+        <v>-0.017</v>
+      </c>
+      <c r="P74" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>-4.619</v>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Spark Starts Tungsten Exploration at Seridó as Global Demand Surges - TMX Newsfile</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOaUUzcW0td2tKUk9KSk15VTRtbXFHazdHRl9oeWh4VzM0M2Y4VUthT0NVWnVuZE9BZ2t6ZUxDdmhCcUo4T3pteDVyTk1UT09SbU5uSHJHU204TFI0UE5TeUozc1ZkUGowUmg2ckZWRDkxVU1OOEJOSkdVQUJsZkRqTnZTTHBjMUNYLVhxU2pfanFCODRPSV92ZVQ2eWpDN0xZQ2VHek9hVU1EMFQ1QWYw?oc=5</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z74" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA74" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AB74" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC74" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD74" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-09-16T16:19:24+00:00</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="F75" t="n">
+        <v>104.12</v>
+      </c>
+      <c r="G75" t="n">
+        <v>100.97</v>
+      </c>
+      <c r="H75" t="n">
+        <v>102.31</v>
+      </c>
+      <c r="I75" t="n">
+        <v>111747</v>
+      </c>
+      <c r="J75" t="n">
+        <v>4</v>
+      </c>
+      <c r="K75" t="n">
+        <v>40</v>
+      </c>
+      <c r="L75" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="M75" t="n">
+        <v>-0.239</v>
+      </c>
+      <c r="N75" t="n">
+        <v>40</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="P75" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>1.808</v>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>Venezuela's withdrawal from OPEC gains traction in the oil - Inspenet</t>
+        </is>
+      </c>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE5Ic05DVGZPeUJyQU9nNzlrVFgzQWdFNTdVZFdEb0pRMGFYN0lRUHcwWW13ZlNUQnUtamVwdGUtT3p1X2h0SnRMbzVGLVY3dzlqS09hSF9BRFpyOWZ4Q0dvRExCT0poVTZKTWlqUjRZQW1GZ00?oc=5</t>
+        </is>
+      </c>
+      <c r="AA75" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB75" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC75" t="inlineStr">
+        <is>
+          <t>OPEC oil output falls in August, Reuters survey shows - Reuters</t>
+        </is>
+      </c>
+      <c r="AD75" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcGZWQVVsSEY1MDZDLXRVM2g2N0t1bHJ1VXpWX3pScTFZak53OGQ5VVNxemw0Mjdrd1paNjRYb1YtdFlYN3RIOURKM00xZmc4eFRlTHk2cTNhODJKWW5TOS1BMEE1cVF2NTN5YjJaeHRRNFlBVHUwUU9CN0pyOEdRMHE0c2VtcGNvamRPVFd3OVVlTnFmV3Fobks2WlZJU21oRW44?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-09-16T16:19:24+00:00</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>99.702</v>
+      </c>
+      <c r="F76" t="n">
+        <v>99.748</v>
+      </c>
+      <c r="G76" t="n">
+        <v>99.64</v>
+      </c>
+      <c r="H76" t="n">
+        <v>99.70999999999999</v>
+      </c>
+      <c r="I76" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" t="n">
+        <v>4</v>
+      </c>
+      <c r="K76" t="n">
+        <v>39</v>
+      </c>
+      <c r="L76" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="M76" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="N76" t="n">
+        <v>39</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0.173</v>
+      </c>
+      <c r="P76" t="n">
+        <v>-0.079</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>3.482</v>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>US Dollar outlook: Hawkish Fed repricing strengthens the bull case - stonex.com</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNRlJTZ3dmU0NMcWtjQU9uU1pXSDQ1Uk5YOGFCVTQwSlExOFZtcjBGT1VZdXppTkpqYkdoaUtTTWw0aVJxclFIaWFnWXItUzBDTkNNSGg1b0t3dVhvREJSQjJRYUFEMGpMa0pNTVpMUzdpT0YwRngyZi1nMlRCdHJlVjVkc0tvU3RqV2pPNzhtYUNhVXlWVXpPRlpiLXBFTE1KNjZoU2lZLXpUaE9CM0hTLTVRSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>US Dollar Price Forecast: DXY Eyes 99.58 as Jobs Week Tests Hawkish Fed; Eyes on EUR/USD and GBP/USD - sg.finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxPWEFMSHF3NGEtMWlQQndSN0ZSSnlpU2ZTTkhkcTVFb3JVZWZUMnVqVEpjVjAyXzZ3Z0tSbUhSRFJFa20ta3c0dXpSc1lrTm4xVGRJeTJpRWVHQzhYVU1LM1kyYmNxX0liVnA1M1RLOVhxV3hBZU5xNWM3UlB2cTJrMlFYNA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>Indonesian Rupiah gains as US Dollar weakens ahead of Fed rate decision - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB76" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOc09LZlhsd3FaTkpSdlVWb0pfR0l6c0VCWFlmcmh2bWN0VTQwRjFwTThtS0o3VEY5cVBBck9FWExBY3pCWS0tNnh3S0dmWmpuWFdubGtUQ1ZvZnkydkExNU03OXlhMGhDd3BiMmRwTG9LeFZxOGJnVy1JS1dreTVwLVdicTU4OVNxVW1aN3pHWFpZeHdWUTVvNVRVUXNJUlhCUTVqaWd6NHdxaG8tak9iU0dpTUg?oc=5</t>
+        </is>
+      </c>
+      <c r="AC76" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD76" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-09-16T16:19:24+00:00</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>7679.75</v>
+      </c>
+      <c r="F77" t="n">
+        <v>7699</v>
+      </c>
+      <c r="G77" t="n">
+        <v>7669</v>
+      </c>
+      <c r="H77" t="n">
+        <v>7686</v>
+      </c>
+      <c r="I77" t="n">
+        <v>502574</v>
+      </c>
+      <c r="J77" t="n">
+        <v>4</v>
+      </c>
+      <c r="K77" t="n">
+        <v>38</v>
+      </c>
+      <c r="L77" t="n">
+        <v>-0.135</v>
+      </c>
+      <c r="M77" t="n">
+        <v>-0.003</v>
+      </c>
+      <c r="N77" t="n">
+        <v>39</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="P77" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>1.976</v>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>Tax revenue surges amid boom in stock market - Taipei Times</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBVYTNZQ2Q4RFRxNEVSUnVLLTZRQUkyVjF1dEtOZ0hiZ1NreVV3NUx1b1RXdWNoRXZIWlB6MnhXakR3SFdvTGt5SG1NZWFLVjZrUGd4MXk0dVEzRkY5NGJkTUtWSmtwalA5RWlLXzQyVGMwN2pjcEE?oc=5</t>
+        </is>
+      </c>
+      <c r="W77" t="inlineStr">
+        <is>
+          <t>Illumina Stock Analysis: Bullish Trend Holds, Momentum in Focus - The Cryptonomist</t>
+        </is>
+      </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQaUstS2lxb25wVWhUUm9ZZjM4WUpYekk3Mk1VVjdHYWdaZUE2alhkXzVKMXlOOHZ0ekVOSE5EWXYtS1o2QjFyVGVockpyVWZPVXdhUTNsSFcyMEE5aFZqb0l4M045T3Z4cnNuU2t4ckpBYTNmZEhGZWstVlV2YlkzQW0zSkpNYUtzeTRYZ2NrMG9nWDhwQ0x2QTZsNVg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>The Fed has to walk a fine line Wednesday. How the stock market may react, according to JPMorgan - CNBC</t>
+        </is>
+      </c>
+      <c r="Z77" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxOTzM4VU4tbFZGTzNNVklGTGdqcVA5d0NfbXRlc3pKSWZHZVdfa3dGdzhKazQxNFBIRjhVN2RWMm13UV9za1NCVkpIbUtSRW1KMUlydmZENS14NW1PczBib1BiUmtUT2NxQm41SThmVUl6b24yVDNtbXdKeFhSTEpHS1F6aEg0dHJkNmE0MWg5czU4OFpwV1ZUeTVXd3RnR2NTQ3EyUXI0aW1PSEFVM0NjNWZR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA77" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB77" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC77" t="inlineStr">
+        <is>
+          <t>Trigano stock breaks through its 146.20 € support level and erases its rebound - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AD77" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxQdUJZN3VGa3JYcVA3S0g3MGNMTWxQNFpib2FVb1RhWWdRM3VjVzg5VnNFT2pTbGZrUVpjYWNnbldBTzg5TEdYcno5V0tJXy1UeUJEMlRFanlhZUhVSlpjSXg2aHZCb2R4R0x5Ti1oNlNQbTlUckhlcjByMVFWUTJrNWZQZHhBZE9IUHgtdWNUX3pXTFVRRmdrN3J2SzNtc0lQbVNFZXRFY3FDWlJIYzN2SExXOHN1c3NHS0VlemVwMDdFYUc3LWtWaEl5WmlwSkRYQjFnS1N3?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-09-16T16:19:24+00:00</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>29401.25</v>
+      </c>
+      <c r="F78" t="n">
+        <v>29549.75</v>
+      </c>
+      <c r="G78" t="n">
+        <v>29363.75</v>
+      </c>
+      <c r="H78" t="n">
+        <v>29479.25</v>
+      </c>
+      <c r="I78" t="n">
+        <v>189389</v>
+      </c>
+      <c r="J78" t="n">
+        <v>4</v>
+      </c>
+      <c r="K78" t="n">
+        <v>40</v>
+      </c>
+      <c r="L78" t="n">
+        <v>-0.176</v>
+      </c>
+      <c r="M78" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="N78" t="n">
+        <v>36</v>
+      </c>
+      <c r="O78" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="P78" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>Qualys gains another 7%, extends previous day's rally (QLYS:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQd2UxRm5EenY5VmZnZzh1Vy1OTmxTX2dNQmRyZzd2d3NwdW93S3lENEYxVEVPVDJWZVNwQWJzM3ltQnpxM1RuNnVGYUI5cVlEU0h5OTJqTzRUZUlJaEl5cjlMeDU2VzVfWHRHUUNBQTVSdDRyZWNmSml2ZVQzR01pcDFLa0puRWNUT1NnV2Q0bHZyUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high on strong Big Tech Q1 2026 earnings - equiti.com</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOOVE5Q1lMRW84cG9XUDFEWm1odC1hTTNvbm1CajdWR1Y4V2hleEFWSjVhNVpYS2VVRGFGcURJMGVoNGwwbXhDeDZTcHN1V0VWT1RFVFVEaExMMGx3YTZfTnphNkJNZnA3S0J1NmFFRWY3ZHYxcFhiUzI5RTc3SGdWbWk3Q1NsSlBLR3l5akg3Z0hSM1lmWGZtY09DbVEySDlmRUJDV0JiTjRqZ3gz?oc=5</t>
+        </is>
+      </c>
+      <c r="W78" t="inlineStr">
+        <is>
+          <t>AI Safety Warning Roils US Stocks: Cybersecurity Shares Surge as Software-Chip Divergence Hits Record - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE1YcW5WbEhROGJoRmt2ZXJrS0FkS2F3WU90a3NCM3JYRlJrd2tUQncyVXF5Y2lZekNpS1k0UEo2MFFRSmtKMVE2ZTBBMElZN1RKU1ZQOGc3d1ZkdHZCRWJkREZhT3JlS1YtUkw1dzRianEzemhFU3c?oc=5</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>QQQ: volume node tests, breaks and retests for NASDAQ:QQQ by AuctionFoundry - TradingView</t>
+        </is>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxORFVBaWZoUklsNVkxUDE0VnEtQUx5OEtMWlhHczdBVWl5TVhLNG5lTUp5cGxQUDdqSTVtWi1kdVFDZ296TG9LRGs0NUV1dTJYMkFNZ19jNWNicG9NbjM0UGlZUEEzTU1FeE1PQ3BMX0NyZElodmU4SHZQc3IzS3N0LTA3dUNsMFZ4a1M3Y19KZTNaQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA78" t="inlineStr">
+        <is>
+          <t>Nasdaq breaks a new record after Ceasefire extension – Dow Jones and US Stock Market Outlook - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="AB78" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNU21uTDlsYjhfQ0w2UEF5STJ4Qm5xajNPS1gxT3B5MFFPbmZMTDQxR0VKcXA1blY0S1kxLTFWT3FZcFczc1NZWWpCRGhqX0ZpblpDNFVJc3J0aExpYl9Eb2xycHpiY3o1NjRDTEhVdHMyZU9yZU9leXZDcllQbjFkcUhFVnp3NFdQNkdhMkZnRVRsZXZBNXl2Z1VhYjdDU29jbnR6WUFKMllmYWs?oc=5</t>
+        </is>
+      </c>
+      <c r="AC78" t="inlineStr">
+        <is>
+          <t>Katie Stockton: Bracing for volatility after Nasdaq broke below recent support - CNBC</t>
+        </is>
+      </c>
+      <c r="AD78" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLWhuVXhhdF9LbEhfSTV2RlNTZ0IyVjBlcUxGS0RQLXA5S0xjUWFZa3c3Nm1OZmxSRU5mVmVLZzRkbEFKYWd1YWFoVHdadUpRRXlMc1BSVi1BY2Q5RlVLRzVoa2xuRkxZdThVS0VVTzRYY256MHZha1l6RDlrU0NaVXZGZW1qZFRWbTBOUFBTRGxUck9ZWk9tWlY4bl9LcU1BVG5Ka0RVVURXallmZGhqT1BacEpBYnFTUzBIRQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-09-16T16:19:24+00:00</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>75890.4062</v>
+      </c>
+      <c r="F79" t="n">
+        <v>75895.1094</v>
+      </c>
+      <c r="G79" t="n">
+        <v>75351.57030000001</v>
+      </c>
+      <c r="H79" t="n">
+        <v>75788.67969999999</v>
+      </c>
+      <c r="I79" t="n">
+        <v>3199692800</v>
+      </c>
+      <c r="J79" t="n">
+        <v>4</v>
+      </c>
+      <c r="K79" t="n">
+        <v>38</v>
+      </c>
+      <c r="L79" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="M79" t="n">
+        <v>0.089</v>
+      </c>
+      <c r="N79" t="n">
+        <v>34</v>
+      </c>
+      <c r="O79" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="P79" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>8.991</v>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W79" t="inlineStr">
+        <is>
+          <t>Bitcoin price extends gains, briefly tops $81,000 as crypto rally gathers pace - CNBC</t>
+        </is>
+      </c>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQdlVlbW1UcGhZSVR6dW9SVTIxX2xrREJYT2VrTnBCRENqeVp4ZUdpUERjemp6QmNLY1h0cUlVYm91OVBublNPOXh0aVdHWHdaU0JyX2gwanhxM0FuYmhfbUNOQjF4UVZPenhjd2tBaDBzbF9DbnMySkotcUpoLVVtekJld2QzcjJaUDNfWFF0cnRRY3NvUk5SMVB6MjLSAaIBQVVfeXFMUE5UVkdmUVAwazBVMTE3Rk5qNUIyTmtPZFhtUzdOVmhSQV9fUUVlT3VpUmZnQnJ5WlR5WWxsTk5ycEpwV0xOMmlkR05NQWNLVzA3R0JYSk5YUFh6NE9CTGtzVXpfeVNLb2l6TFVQUWxKOWthZGlwdHZEMlQwT0JWOEdWVXQwdlViNW9uZG5SQmZKQUhLSTdrOVpuRHBrNUV6a19B?oc=5</t>
+        </is>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - Pulse 2.0</t>
+        </is>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA79" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="AB79" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC79" t="inlineStr">
+        <is>
+          <t>Bitcoin holds above key moving averages despite CLARITY Act sell-off - coinjournal.net</t>
+        </is>
+      </c>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNZXktaUlVZWpGb0JBUEpiTk50am9GV0VaaG1TRzhsNENZaG1JZ0JTUTZMZ1pWbjZ2WWJKOUpObXBPMjlvZXZIV092ODFXT3p3YXc3dnFxSnRUODM3Rmt2RGNCbUZvNTk2X0NKQUE4ODFtamhRNXp4WDZRSUNCMktZaXZxMkcxS3YyTTBYNmFBM1B4eVNyeXViVy1BVG9nTU0?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-16 22:44 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD79"/>
+  <dimension ref="A1:AD85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10289,6 +10289,762 @@
       <c r="AD79" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNZXktaUlVZWpGb0JBUEpiTk50am9GV0VaaG1TRzhsNENZaG1JZ0JTUTZMZ1pWbjZ2WWJKOUpObXBPMjlvZXZIV092ODFXT3p3YXc3dnFxSnRUODM3Rmt2RGNCbUZvNTk2X0NKQUE4ODFtamhRNXp4WDZRSUNCMktZaXZxMkcxS3YyTTBYNmFBM1B4eVNyeXViVy1BVG9nTU0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-09-16T22:42:21+00:00</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>GCJ27.CMX</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>4461.2998</v>
+      </c>
+      <c r="F80" t="n">
+        <v>4469.8999</v>
+      </c>
+      <c r="G80" t="n">
+        <v>4350</v>
+      </c>
+      <c r="H80" t="n">
+        <v>4383.6001</v>
+      </c>
+      <c r="I80" t="n">
+        <v>935</v>
+      </c>
+      <c r="J80" t="n">
+        <v>4</v>
+      </c>
+      <c r="K80" t="n">
+        <v>39</v>
+      </c>
+      <c r="L80" t="n">
+        <v>-0.229</v>
+      </c>
+      <c r="M80" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="N80" t="n">
+        <v>40</v>
+      </c>
+      <c r="O80" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="P80" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>Spark Starts Tungsten Exploration at Seridó as Global Demand Surges - TMX Newsfile</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOaUUzcW0td2tKUk9KSk15VTRtbXFHazdHRl9oeWh4VzM0M2Y4VUthT0NVWnVuZE9BZ2t6ZUxDdmhCcUo4T3pteDVyTk1UT09SbU5uSHJHU204TFI0UE5TeUozc1ZkUGowUmg2ckZWRDkxVU1OOEJOSkdVQUJsZkRqTnZTTHBjMUNYLVhxU2pfanFCODRPSV92ZVQ2eWpDN0xZQ2VHek9hVU1EMFQ1QWYw?oc=5</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>Founders Metals (TSXV:FDR) Falls 5.65% as Profit-Taking Tests Strong Antino Gold Momentum - kalkine.ca</t>
+        </is>
+      </c>
+      <c r="Z80" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQWjZmSkNZV2p0c3pfYWd1Y2U0NnVtdlNaTGdEU3dDbEZ1QTV2WVZCUXp2bmZFVE5ETHByVmc4R1lBUFlDU2JsejNyNkNCcEk3R2lUQUpPbnl5ZS1aeWZGN0lISTVocl9leXVOdTBrN2dKdGJyVl85N0pUQlFtaEZvTXF3V2MzU0xNcTFydU5fNWZsamhnNDVqSThhVEVuaHYweTI5c1g3ZDlDOWplQl8zVGJqa3JnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA80" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="AB80" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AC80" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AD80" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-09-16T22:42:21+00:00</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>102.29</v>
+      </c>
+      <c r="F81" t="n">
+        <v>102.87</v>
+      </c>
+      <c r="G81" t="n">
+        <v>101.72</v>
+      </c>
+      <c r="H81" t="n">
+        <v>101.92</v>
+      </c>
+      <c r="I81" t="n">
+        <v>39236</v>
+      </c>
+      <c r="J81" t="n">
+        <v>4</v>
+      </c>
+      <c r="K81" t="n">
+        <v>40</v>
+      </c>
+      <c r="L81" t="n">
+        <v>-0.055</v>
+      </c>
+      <c r="M81" t="n">
+        <v>-0.219</v>
+      </c>
+      <c r="N81" t="n">
+        <v>40</v>
+      </c>
+      <c r="O81" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="P81" t="n">
+        <v>-0.082</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>0.508</v>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>Oil's roundtrip back to $100. Why China could determine what happens next - CNBC</t>
+        </is>
+      </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOa0xDNl91YjR4WVVvTXU5UlVvMnVQWUs0SDVCRFZFV0VxWVJzLVdsTWZuN1RiSjkxamJwdUkyVUdzZndiTXlITFdQWEVrSzJmSjN1bkczVjhhRktQSHR1UlMzMUtRalJZbmtLbDAtX0FJb1Ntb213dXFxeHMtVXh0NG5sd2ctUVdMWUJDQmF4R1U4V0hQZXQ0WVJDbVBWZDItbXAwbGxiWVFFSGs?oc=5</t>
+        </is>
+      </c>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z81" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA81" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AB81" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC81" t="inlineStr">
+        <is>
+          <t>VIX Breaks Out Before CPI: S&amp;P 500 Clinging to Support as Oil Gets Rejected at $104 - YouTube</t>
+        </is>
+      </c>
+      <c r="AD81" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiQkFVX3lxTE5OVDlua2JHTEZ1Y25SWWtneWdRazB4R0cwWEY1dWFRWnU0SktHYjRzc2dYOGVYZWJ4NlJxeTBYMUg4Zw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-09-16T22:42:21+00:00</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>100.251</v>
+      </c>
+      <c r="F82" t="n">
+        <v>100.354</v>
+      </c>
+      <c r="G82" t="n">
+        <v>100.15</v>
+      </c>
+      <c r="H82" t="n">
+        <v>100.34</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" t="n">
+        <v>4</v>
+      </c>
+      <c r="K82" t="n">
+        <v>38</v>
+      </c>
+      <c r="L82" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="M82" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="N82" t="n">
+        <v>40</v>
+      </c>
+      <c r="O82" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="P82" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>2</v>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>Dollar holds firm as angst over Iran-U.S. stand-off drives safe-haven demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPYjVva2k0WFlQTjA2T1hrRzhuaENsdEJaMW4zaVJLSHZRbVBIMENzRlc2Qzl0NGJNVm54RGlBckI4WGpuV05Md3puR1Q2cDBOaDBGbkpvWTVDWDF6aFFOMU5ZN1l3WjFoaG01VjFQU0Jfai1WX3pyVHlSbGQ5cks5OHlET3N5T1BHX2Z0UkJlT0t4MWhkWEZQMVJfZmhUa0Nv0gGmAUFVX3lxTFA1RUg3R3RlUmFOYXo0Z25OTVdzOWJkM0dER0tPMVJFWjdRZVhBa1dBa1FyTXZ1aldVOXUwcllYaHJtaDVNYTZuNTNyMnRPRGRmTUlxQXBKdHp2c0o5d2VwLWN3WVRReVBIX1ZZTm1mcHhvZnVxS09NYk1GTDhBYkpzbHJaMmlNNFprSlE5NEdtT09tdk81MlZabmNDLUNNSF9idklOX0E?oc=5</t>
+        </is>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - FXStreet</t>
+        </is>
+      </c>
+      <c r="Z82" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA82" t="inlineStr">
+        <is>
+          <t>US stocks rebound as dovish Fed and weak ADP cool yields, dent dollar and lift gold - VT Markets</t>
+        </is>
+      </c>
+      <c r="AB82" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQUW1QcWR4RlJfWFVoVENIX05tcjJSR3dkbm9rMzVnNFZvaDUzbHlfSU41LTNHTFctZ3NLRFVtVjUyaEdtUnpvdGtoZHdLbjFRdndoZWxCRUxIc2d3NEFrVmNKUGFNbzF0Y1FBYXRIRHktamFaRkc0bnlYV2Nya21WU1g0Rlgxa2ZGaFF3QktZNEtJWlFsRkI3VjFxNWxfaHlVamtFaU1DeUtrdVdnMnppV2pfMWhzQV81UDZ6TXVYX1lUZjhZMUpR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC82" t="inlineStr">
+        <is>
+          <t>Indonesian Rupiah gains as US Dollar weakens ahead of Fed rate decision - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD82" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOc09LZlhsd3FaTkpSdlVWb0pfR0l6c0VCWFlmcmh2bWN0VTQwRjFwTThtS0o3VEY5cVBBck9FWExBY3pCWS0tNnh3S0dmWmpuWFdubGtUQ1ZvZnkydkExNU03OXlhMGhDd3BiMmRwTG9LeFZxOGJnVy1JS1dreTVwLVdicTU4OVNxVW1aN3pHWFpZeHdWUTVvNVRVUXNJUlhCUTVqaWd6NHdxaG8tak9iU0dpTUg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-09-16T22:42:21+00:00</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>7684.5</v>
+      </c>
+      <c r="F83" t="n">
+        <v>7694.25</v>
+      </c>
+      <c r="G83" t="n">
+        <v>7575</v>
+      </c>
+      <c r="H83" t="n">
+        <v>7634.25</v>
+      </c>
+      <c r="I83" t="n">
+        <v>882276</v>
+      </c>
+      <c r="J83" t="n">
+        <v>4</v>
+      </c>
+      <c r="K83" t="n">
+        <v>38</v>
+      </c>
+      <c r="L83" t="n">
+        <v>-0.276</v>
+      </c>
+      <c r="M83" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="N83" t="n">
+        <v>39</v>
+      </c>
+      <c r="O83" t="n">
+        <v>0.266</v>
+      </c>
+      <c r="P83" t="n">
+        <v>-0.016</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>-0.549</v>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>Tax revenue surges amid boom in stock market - Taipei Times</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBVYTNZQ2Q4RFRxNEVSUnVLLTZRQUkyVjF1dEtOZ0hiZ1NreVV3NUx1b1RXdWNoRXZIWlB6MnhXakR3SFdvTGt5SG1NZWFLVjZrUGd4MXk0dVEzRkY5NGJkTUtWSmtwalA5RWlLXzQyVGMwN2pjcEE?oc=5</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>'Titanic' has a happy ending: Robust rally caps Wall Street's week of red - TradingView</t>
+        </is>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSG12a01IVVJtakhLMFlscGk0SXRsa0M2UUwtakVNd041MUV0RVdjanozTGlFdWFpZ2dCai10NlYtbW42d3pnQ1lseGdvMGR5VV9USlk0T09WNW93TVhPMVUyUHpQT1ZDLWRBRWdBcHIzbTN4T0VhVVBZb0pzeHlqTEJNS0ZnTXlXUDlTYmRFbHYxYVJWSDQ1THZBSXhIckdURjdPY25wcWc3SXJ2R2pFX1lIVFVoem51RmZDTHhOWkVIRVIwWWdlZE1odzFGTG9DeFo5NHUycw?oc=5</t>
+        </is>
+      </c>
+      <c r="W83" t="inlineStr">
+        <is>
+          <t>Almirall stock gains after breaking key resistance on Madrid exchange - ad-hoc-news.de</t>
+        </is>
+      </c>
+      <c r="X83" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxPOWR3MHhPVmk4SHVHd0FlYTlCYkdicEdoOUZXcC1ybVRoVmFOa25oOWJUa3V6cmRtMVN5WGQyQ3RYVU93Mno2dVdaRnV0TUxNLTBfR0pPdUsyWVlMaXFqNXpTYnBrWFpHX3RuVXVFSEtkeHN4Um1LUWc2N1NUZnp3ZURYQU1FN3NqWDR1QW9leUlnQ0NtbER4WHdGMWJ1djlGcTRtSXpTcE1mMDd2azlHSjJPRXVlR1o1Ujh4ZGpaUFhKZ0E1Zk1vbG1lNGk?oc=5</t>
+        </is>
+      </c>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>The Fed has to walk a fine line Wednesday. How the stock market may react, according to JPMorgan - CNBC</t>
+        </is>
+      </c>
+      <c r="Z83" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxOTzM4VU4tbFZGTzNNVklGTGdqcVA5d0NfbXRlc3pKSWZHZVdfa3dGdzhKazQxNFBIRjhVN2RWMm13UV9za1NCVkpIbUtSRW1KMUlydmZENS14NW1PczBib1BiUmtUT2NxQm41SThmVUl6b24yVDNtbXdKeFhSTEpHS1F6aEg0dHJkNmE0MWg5czU4OFpwV1ZUeTVXd3RnR2NTQ3EyUXI0aW1PSEFVM0NjNWZR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA83" t="inlineStr">
+        <is>
+          <t>Trigano stock breaks through its 146.20 € support level and erases its rebound - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB83" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxQdUJZN3VGa3JYcVA3S0g3MGNMTWxQNFpib2FVb1RhWWdRM3VjVzg5VnNFT2pTbGZrUVpjYWNnbldBTzg5TEdYcno5V0tJXy1UeUJEMlRFanlhZUhVSlpjSXg2aHZCb2R4R0x5Ti1oNlNQbTlUckhlcjByMVFWUTJrNWZQZHhBZE9IUHgtdWNUX3pXTFVRRmdrN3J2SzNtc0lQbVNFZXRFY3FDWlJIYzN2SExXOHN1c3NHS0VlemVwMDdFYUc3LWtWaEl5WmlwSkRYQjFnS1N3?oc=5</t>
+        </is>
+      </c>
+      <c r="AC83" t="inlineStr">
+        <is>
+          <t>Dow Drops 631, Nasdaq Slips 3, S&amp;P 500 Falls 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD83" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQVFVRNlU5aU5HaTYzZ2tnN1Nabng2cWNEd2VPQzdxcU96aHRDOFgyTUR0S3hQNXQ3MVVXQ2xDRGZKWkxNQVgyQl83eW1VQU8yX2hZVS0yR25COHJyTndBcG5xZUd2dFVvOUNPOE5BSkhnaVN4dGVQVFNreWQ0SmFFcTZwdFdmUlZqcTFsekRMcw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-09-16T22:42:21+00:00</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>29478.75</v>
+      </c>
+      <c r="F84" t="n">
+        <v>29539</v>
+      </c>
+      <c r="G84" t="n">
+        <v>29053</v>
+      </c>
+      <c r="H84" t="n">
+        <v>29333.25</v>
+      </c>
+      <c r="I84" t="n">
+        <v>264627</v>
+      </c>
+      <c r="J84" t="n">
+        <v>4</v>
+      </c>
+      <c r="K84" t="n">
+        <v>40</v>
+      </c>
+      <c r="L84" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="M84" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="N84" t="n">
+        <v>36</v>
+      </c>
+      <c r="O84" t="n">
+        <v>0.238</v>
+      </c>
+      <c r="P84" t="n">
+        <v>-0.07099999999999999</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>0.484</v>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>S&amp;P and Nasdaq hit record highs, continuing remarkable recovery from war shock - CNN</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBFM0dLbkRoQTEzbmVyNGdlZERORGZXdEJrOVh3U0FZVnJsNk0zQjFWVVF6a0NhQThTbS0zMUJTdmdHWm1JYVF3LW5VUWVJWFk1MUd6WlVNWU9aa0dENG9rbkYzRDFpcmhSQ1BJ?oc=5</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>Lumentum Holdings rises 10% amid optical networking rally (LITE:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOOEE3X3dfVkk2Z19nNG5LRGxXblNEakFtdDZ2bDByUWdPeS1QYl9MYkpkVDRmX3g0SGg1SjhnVHRqMVc4R1RxMTN0UHo0OUtUdDlaaUVPM0pjd09NV2xjZGdoaTVHTEZILVlNNWlvSnNSd1lfRUlBeF8xLWxpQUVMWEUtU1RBZExfMDBJWXZ6Z2xtNjJFbGNsM3pR?oc=5</t>
+        </is>
+      </c>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>AI Safety Warning Roils US Stocks: Cybersecurity Shares Surge as Software-Chip Divergence Hits Record - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE1YcW5WbEhROGJoRmt2ZXJrS0FkS2F3WU90a3NCM3JYRlJrd2tUQncyVXF5Y2lZekNpS1k0UEo2MFFRSmtKMVE2ZTBBMElZN1RKU1ZQOGc3d1ZkdHZCRWJkREZhT3JlS1YtUkw1dzRianEzemhFU3c?oc=5</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>QQQ: volume node tests, breaks and retests for NASDAQ:QQQ by AuctionFoundry - TradingView</t>
+        </is>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxORFVBaWZoUklsNVkxUDE0VnEtQUx5OEtMWlhHczdBVWl5TVhLNG5lTUp5cGxQUDdqSTVtWi1kdVFDZ296TG9LRGs0NUV1dTJYMkFNZ19jNWNicG9NbjM0UGlZUEEzTU1FeE1PQ3BMX0NyZElodmU4SHZQc3IzS3N0LTA3dUNsMFZ4a1M3Y19KZTNaQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>Dow Drops 631, Nasdaq Slips 3, S&amp;P 500 Falls 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB84" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQVFVRNlU5aU5HaTYzZ2tnN1Nabng2cWNEd2VPQzdxcU96aHRDOFgyTUR0S3hQNXQ3MVVXQ2xDRGZKWkxNQVgyQl83eW1VQU8yX2hZVS0yR25COHJyTndBcG5xZUd2dFVvOUNPOE5BSkhnaVN4dGVQVFNreWQ0SmFFcTZwdFdmUlZqcTFsekRMcw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC84" t="inlineStr">
+        <is>
+          <t>Katie Stockton: Bracing for volatility after Nasdaq broke below recent support - CNBC</t>
+        </is>
+      </c>
+      <c r="AD84" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLWhuVXhhdF9LbEhfSTV2RlNTZ0IyVjBlcUxGS0RQLXA5S0xjUWFZa3c3Nm1OZmxSRU5mVmVLZzRkbEFKYWd1YWFoVHdadUpRRXlMc1BSVi1BY2Q5RlVLRzVoa2xuRkxZdThVS0VVTzRYY256MHZha1l6RDlrU0NaVXZGZW1qZFRWbTBOUFBTRGxUck9ZWk9tWlY4bl9LcU1BVG5Ka0RVVURXallmZGhqT1BacEpBYnFTUzBIRQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-09-16T22:42:21+00:00</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>75596.47659999999</v>
+      </c>
+      <c r="F85" t="n">
+        <v>76330.22659999999</v>
+      </c>
+      <c r="G85" t="n">
+        <v>75172.14840000001</v>
+      </c>
+      <c r="H85" t="n">
+        <v>75745.61719999999</v>
+      </c>
+      <c r="I85" t="n">
+        <v>2576197632</v>
+      </c>
+      <c r="J85" t="n">
+        <v>4</v>
+      </c>
+      <c r="K85" t="n">
+        <v>38</v>
+      </c>
+      <c r="L85" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="M85" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="N85" t="n">
+        <v>34</v>
+      </c>
+      <c r="O85" t="n">
+        <v>0.348</v>
+      </c>
+      <c r="P85" t="n">
+        <v>-0.034</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>10.163</v>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W85" t="inlineStr">
+        <is>
+          <t>Crypto extends gains after biggest 3-day rally since 2023 - CNBC</t>
+        </is>
+      </c>
+      <c r="X85" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOU2taT3BZSUl5LTZSSVJ5ZEtlSjR1N1NsdmRldjNBaWhfeWtBSVBqR0xFR0pKVjZLUW50RkF6VnVBMVJLWjZrYVhUZEpXakg2Q29jQXA3R3BQQ2hla1ZWZ0VHd05Jc1ptdmZhWTZxazFJRWZPME1lVTZfQzNoV1c2OFNjcGVTaFBnQ3dOVFVSWEV4RXhTNEh1YzVB0gGfAUFVX3lxTFA0RUhQT3dVbUo4OTA3azBmRHFRV1lCYXhlb2pJQzRDV2o5N2lpSWlwamoyeGRLclFReHJMZ1V5NldQUTNvQWhpc1dCLTAwNVFMUkpvRmhyVG1qbjVYZGxpdjExdHh6SndiU2dBNzNIMm1lS1VRYnV2QXc4cmo3RW9IdjdRS0dhdjRRbjBxRElaamV5clp2eEpTSVJWNU40OA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - Pulse 2.0</t>
+        </is>
+      </c>
+      <c r="Z85" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA85" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="AB85" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC85" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - Crypto News</t>
+        </is>
+      </c>
+      <c r="AD85" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-17 03:52 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD85"/>
+  <dimension ref="A1:AD91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11045,6 +11045,762 @@
       <c r="AD85" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-09-17T03:50:29+00:00</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>4309.7998</v>
+      </c>
+      <c r="F86" t="n">
+        <v>4356.2002</v>
+      </c>
+      <c r="G86" t="n">
+        <v>4304.3999</v>
+      </c>
+      <c r="H86" t="n">
+        <v>4330.2998</v>
+      </c>
+      <c r="I86" t="n">
+        <v>27166</v>
+      </c>
+      <c r="J86" t="n">
+        <v>4</v>
+      </c>
+      <c r="K86" t="n">
+        <v>39</v>
+      </c>
+      <c r="L86" t="n">
+        <v>-0.223</v>
+      </c>
+      <c r="M86" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="N86" t="n">
+        <v>40</v>
+      </c>
+      <c r="O86" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="P86" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>-2.625</v>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>Spark Starts Tungsten Exploration at Seridó as Global Demand Surges - TMX Newsfile</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOaUUzcW0td2tKUk9KSk15VTRtbXFHazdHRl9oeWh4VzM0M2Y4VUthT0NVWnVuZE9BZ2t6ZUxDdmhCcUo4T3pteDVyTk1UT09SbU5uSHJHU204TFI0UE5TeUozc1ZkUGowUmg2ckZWRDkxVU1OOEJOSkdVQUJsZkRqTnZTTHBjMUNYLVhxU2pfanFCODRPSV92ZVQ2eWpDN0xZQ2VHek9hVU1EMFQ1QWYw?oc=5</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="W86" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X86" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>Founders Metals (TSXV:FDR) Falls 5.65% as Profit-Taking Tests Strong Antino Gold Momentum - kalkine.ca</t>
+        </is>
+      </c>
+      <c r="Z86" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQWjZmSkNZV2p0c3pfYWd1Y2U0NnVtdlNaTGdEU3dDbEZ1QTV2WVZCUXp2bmZFVE5ETHByVmc4R1lBUFlDU2JsejNyNkNCcEk3R2lUQUpPbnl5ZS1aeWZGN0lISTVocl9leXVOdTBrN2dKdGJyVl85N0pUQlFtaEZvTXF3V2MzU0xNcTFydU5fNWZsamhnNDVqSThhVEVuaHYweTI5c1g3ZDlDOWplQl8zVGJqa3JnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA86" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AB86" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC86" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - gold.org</t>
+        </is>
+      </c>
+      <c r="AD86" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-09-17T03:50:29+00:00</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>101.76</v>
+      </c>
+      <c r="F87" t="n">
+        <v>102.46</v>
+      </c>
+      <c r="G87" t="n">
+        <v>101.07</v>
+      </c>
+      <c r="H87" t="n">
+        <v>102.02</v>
+      </c>
+      <c r="I87" t="n">
+        <v>11436</v>
+      </c>
+      <c r="J87" t="n">
+        <v>4</v>
+      </c>
+      <c r="K87" t="n">
+        <v>40</v>
+      </c>
+      <c r="L87" t="n">
+        <v>-0.008999999999999999</v>
+      </c>
+      <c r="M87" t="n">
+        <v>-0.218</v>
+      </c>
+      <c r="N87" t="n">
+        <v>40</v>
+      </c>
+      <c r="O87" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="P87" t="n">
+        <v>-0.115</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>1.678</v>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>Oil Recovery Emulsifier Market to Accelerate by 2035, Driven by Electronics and Semiconductor Cleaning Demand - IndexBox</t>
+        </is>
+      </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxNXzZWY252MUpwZm9lekhaU29tTlJCTng3ZXpOaXowSE16TExxQkVPTWFPSEF5TW9Fci14Q21RdWdRSllTQUFXY25RTXZ3YWdZMXhldEc5b0NBMFVRZ2lzM0M3clhOeEdKSTI3RnQ1NVdNOTRYdjVvdlNoWW5JWjF3Z1B0YWhYdXRITmV4MWNkUC1KYU9rN3JIdm5hY3FnOXhheEVhaTdKRVF6RHZFbjBWbEZuWkVMaWRPXzFCT2lMbFNXMTR2OFRDeTBTWUdCZk95RkhTdA?oc=5</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="W87" t="inlineStr">
+        <is>
+          <t>Current price of oil as of July 30, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9odGxncTZBdXJrcnd4Zm1GSENJSFpJQUJxbGphdTV2dTRfQTVmMzVFQ21PTGhzY19DSGVFUWpoeEtGMDZhNzRveUNoaDBlcDVLSmRpaFh6ZnA1emJSVllSYTNR?oc=5</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z87" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA87" t="inlineStr">
+        <is>
+          <t>OPEC oil output falls in August, Reuters survey shows - Reuters</t>
+        </is>
+      </c>
+      <c r="AB87" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcGZWQVVsSEY1MDZDLXRVM2g2N0t1bHJ1VXpWX3pScTFZak53OGQ5VVNxemw0Mjdrd1paNjRYb1YtdFlYN3RIOURKM00xZmc4eFRlTHk2cTNhODJKWW5TOS1BMEE1cVF2NTN5YjJaeHRRNFlBVHUwUU9CN0pyOEdRMHE0c2VtcGNvamRPVFd3OVVlTnFmV3Fobks2WlZJU21oRW44?oc=5</t>
+        </is>
+      </c>
+      <c r="AC87" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD87" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-09-17T03:50:29+00:00</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>100.266</v>
+      </c>
+      <c r="F88" t="n">
+        <v>100.367</v>
+      </c>
+      <c r="G88" t="n">
+        <v>100.224</v>
+      </c>
+      <c r="H88" t="n">
+        <v>100.321</v>
+      </c>
+      <c r="I88" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" t="n">
+        <v>4</v>
+      </c>
+      <c r="K88" t="n">
+        <v>39</v>
+      </c>
+      <c r="L88" t="n">
+        <v>-0.028</v>
+      </c>
+      <c r="M88" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="N88" t="n">
+        <v>40</v>
+      </c>
+      <c r="O88" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="P88" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>0.856</v>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>Dollar holds firm as angst over Iran-U.S. stand-off drives safe-haven demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPYjVva2k0WFlQTjA2T1hrRzhuaENsdEJaMW4zaVJLSHZRbVBIMENzRlc2Qzl0NGJNVm54RGlBckI4WGpuV05Md3puR1Q2cDBOaDBGbkpvWTVDWDF6aFFOMU5ZN1l3WjFoaG01VjFQU0Jfai1WX3pyVHlSbGQ5cks5OHlET3N5T1BHX2Z0UkJlT0t4MWhkWEZQMVJfZmhUa0Nv0gGmAUFVX3lxTFA1RUg3R3RlUmFOYXo0Z25OTVdzOWJkM0dER0tPMVJFWjdRZVhBa1dBa1FyTXZ1aldVOXUwcllYaHJtaDVNYTZuNTNyMnRPRGRmTUlxQXBKdHp2c0o5d2VwLWN3WVRReVBIX1ZZTm1mcHhvZnVxS09NYk1GTDhBYkpzbHJaMmlNNFprSlE5NEdtT09tdk81MlZabmNDLUNNSF9idklOX0E?oc=5</t>
+        </is>
+      </c>
+      <c r="W88" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z88" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA88" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB88" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC88" t="inlineStr">
+        <is>
+          <t>Indonesian Rupiah gains as US Dollar weakens ahead of Fed rate decision - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD88" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOc09LZlhsd3FaTkpSdlVWb0pfR0l6c0VCWFlmcmh2bWN0VTQwRjFwTThtS0o3VEY5cVBBck9FWExBY3pCWS0tNnh3S0dmWmpuWFdubGtUQ1ZvZnkydkExNU03OXlhMGhDd3BiMmRwTG9LeFZxOGJnVy1JS1dreTVwLVdicTU4OVNxVW1aN3pHWFpZeHdWUTVvNVRVUXNJUlhCUTVqaWd6NHdxaG8tak9iU0dpTUg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-09-17T03:50:29+00:00</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>7657.5</v>
+      </c>
+      <c r="F89" t="n">
+        <v>7669.75</v>
+      </c>
+      <c r="G89" t="n">
+        <v>7654</v>
+      </c>
+      <c r="H89" t="n">
+        <v>7669.75</v>
+      </c>
+      <c r="I89" t="n">
+        <v>49630</v>
+      </c>
+      <c r="J89" t="n">
+        <v>4</v>
+      </c>
+      <c r="K89" t="n">
+        <v>38</v>
+      </c>
+      <c r="L89" t="n">
+        <v>-0.281</v>
+      </c>
+      <c r="M89" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="N89" t="n">
+        <v>39</v>
+      </c>
+      <c r="O89" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="P89" t="n">
+        <v>-0.026</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>-0.667</v>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>Tax revenue surges amid boom in stock market - Taipei Times</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBVYTNZQ2Q4RFRxNEVSUnVLLTZRQUkyVjF1dEtOZ0hiZ1NreVV3NUx1b1RXdWNoRXZIWlB6MnhXakR3SFdvTGt5SG1NZWFLVjZrUGd4MXk0dVEzRkY5NGJkTUtWSmtwalA5RWlLXzQyVGMwN2pjcEE?oc=5</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 11: HPE Surges on AI Infrastructure Demand and Recently Raised Guidance - The Globe and Mail</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxQWjNhWk9lUkVTV185bEdldml2Mk16MTFRLWtFd1lKUXlMMlJRNC02dXpRVkFrUjYzNlNhRENiUnIySEE2MUdMRmFvV3pfaVM3NE5HSEZ6ZU9qNU82bnFnS1FBVGNmTVdad3FXc2M4NDljeHc5SjZDcjVlQ2M2SWt0YXJpeXZPUVhxNFFGZFhycUhYd3FnR3BlWGdoYlh0b0Uxdm9VZkRseG1odFpKVDFXdWlmQlkzR0dwOVl6aTVkTEQybVZWWnRVUTB5akN0YzFZRXFWUUtNSXJIRlVIQzEzWkRlSUZ2MDdxMmUxcFdMc2FmdFdmMFJKc29Yc3Vqb2JIaTlFb0pXVmM5bGs?oc=5</t>
+        </is>
+      </c>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>'Titanic' has a happy ending: Robust rally caps Wall Street's week of red - TradingView</t>
+        </is>
+      </c>
+      <c r="X89" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSG12a01IVVJtakhLMFlscGk0SXRsa0M2UUwtakVNd041MUV0RVdjanozTGlFdWFpZ2dCai10NlYtbW42d3pnQ1lseGdvMGR5VV9USlk0T09WNW93TVhPMVUyUHpQT1ZDLWRBRWdBcHIzbTN4T0VhVVBZb0pzeHlqTEJNS0ZnTXlXUDlTYmRFbHYxYVJWSDQ1THZBSXhIckdURjdPY25wcWc3SXJ2R2pFX1lIVFVoem51RmZDTHhOWkVIRVIwWWdlZE1odzFGTG9DeFo5NHUycw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y89" t="inlineStr">
+        <is>
+          <t>Trigano stock breaks through its 146.20 € support level and erases its rebound - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="Z89" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxQdUJZN3VGa3JYcVA3S0g3MGNMTWxQNFpib2FVb1RhWWdRM3VjVzg5VnNFT2pTbGZrUVpjYWNnbldBTzg5TEdYcno5V0tJXy1UeUJEMlRFanlhZUhVSlpjSXg2aHZCb2R4R0x5Ti1oNlNQbTlUckhlcjByMVFWUTJrNWZQZHhBZE9IUHgtdWNUX3pXTFVRRmdrN3J2SzNtc0lQbVNFZXRFY3FDWlJIYzN2SExXOHN1c3NHS0VlemVwMDdFYUc3LWtWaEl5WmlwSkRYQjFnS1N3?oc=5</t>
+        </is>
+      </c>
+      <c r="AA89" t="inlineStr">
+        <is>
+          <t>If a Market Crash Is Coming, Here’s a Piece of Warren Buffett Wisdom That You Should Follow - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="AB89" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxNeG5qQTVNSG4xQzNUNEJBSGtqbVowRVVNUnRlM0dMQzA3Y1pjU1JtUHc4ZVFfbnpZbnd2dklraURfZVpiTEJpOFhHbGE2RmFxcXVKUDB4OWhXMmFzaGxuN0dPVWNJSHdtT3lRWFdkNDdyRjQwRy1jejAwZ3M3QXczM1RKbDdFSUNhRXdHZm42Ukx4dEpJbUcyVG51aExfbWRIZFgyVE5Ra2ZkZVo3dEtHQm1ORVhrYVJRWkFnWnpBcVJJV3FRZWU1TXRhWkZFZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC89" t="inlineStr">
+        <is>
+          <t>Dow Drops 631, Nasdaq Slips 3, S&amp;P 500 Falls 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD89" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQVFVRNlU5aU5HaTYzZ2tnN1Nabng2cWNEd2VPQzdxcU96aHRDOFgyTUR0S3hQNXQ3MVVXQ2xDRGZKWkxNQVgyQl83eW1VQU8yX2hZVS0yR25COHJyTndBcG5xZUd2dFVvOUNPOE5BSkhnaVN4dGVQVFNreWQ0SmFFcTZwdFdmUlZqcTFsekRMcw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-09-17T03:50:29+00:00</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>29451.5</v>
+      </c>
+      <c r="F90" t="n">
+        <v>29478</v>
+      </c>
+      <c r="G90" t="n">
+        <v>29406.25</v>
+      </c>
+      <c r="H90" t="n">
+        <v>29461.5</v>
+      </c>
+      <c r="I90" t="n">
+        <v>25974</v>
+      </c>
+      <c r="J90" t="n">
+        <v>4</v>
+      </c>
+      <c r="K90" t="n">
+        <v>40</v>
+      </c>
+      <c r="L90" t="n">
+        <v>-0.231</v>
+      </c>
+      <c r="M90" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="N90" t="n">
+        <v>37</v>
+      </c>
+      <c r="O90" t="n">
+        <v>0.177</v>
+      </c>
+      <c r="P90" t="n">
+        <v>-0.018</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>0.151</v>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>Qualys gains another 7%, extends previous day's rally (QLYS:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQd2UxRm5EenY5VmZnZzh1Vy1OTmxTX2dNQmRyZzd2d3NwdW93S3lENEYxVEVPVDJWZVNwQWJzM3ltQnpxM1RuNnVGYUI5cVlEU0h5OTJqTzRUZUlJaEl5cjlMeDU2VzVfWHRHUUNBQTVSdDRyZWNmSml2ZVQzR01pcDFLa0puRWNUT1NnV2Q0bHZyUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high on strong Big Tech Q1 2026 earnings - equiti.com</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOOVE5Q1lMRW84cG9XUDFEWm1odC1hTTNvbm1CajdWR1Y4V2hleEFWSjVhNVpYS2VVRGFGcURJMGVoNGwwbXhDeDZTcHN1V0VWT1RFVFVEaExMMGx3YTZfTnphNkJNZnA3S0J1NmFFRWY3ZHYxcFhiUzI5RTc3SGdWbWk3Q1NsSlBLR3l5akg3Z0hSM1lmWGZtY09DbVEySDlmRUJDV0JiTjRqZ3gz?oc=5</t>
+        </is>
+      </c>
+      <c r="W90" t="inlineStr">
+        <is>
+          <t>AI Safety Warning Roils US Stocks: Cybersecurity Shares Surge as Software-Chip Divergence Hits Record - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE1YcW5WbEhROGJoRmt2ZXJrS0FkS2F3WU90a3NCM3JYRlJrd2tUQncyVXF5Y2lZekNpS1k0UEo2MFFRSmtKMVE2ZTBBMElZN1RKU1ZQOGc3d1ZkdHZCRWJkREZhT3JlS1YtUkw1dzRianEzemhFU3c?oc=5</t>
+        </is>
+      </c>
+      <c r="Y90" t="inlineStr">
+        <is>
+          <t>QQQ: volume node tests, breaks and retests for NASDAQ:QQQ by AuctionFoundry - TradingView</t>
+        </is>
+      </c>
+      <c r="Z90" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxORFVBaWZoUklsNVkxUDE0VnEtQUx5OEtMWlhHczdBVWl5TVhLNG5lTUp5cGxQUDdqSTVtWi1kdVFDZ296TG9LRGs0NUV1dTJYMkFNZ19jNWNicG9NbjM0UGlZUEEzTU1FeE1PQ3BMX0NyZElodmU4SHZQc3IzS3N0LTA3dUNsMFZ4a1M3Y19KZTNaQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA90" t="inlineStr">
+        <is>
+          <t>Dow Drops 631, Nasdaq Slips 3, S&amp;P 500 Falls 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB90" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQVFVRNlU5aU5HaTYzZ2tnN1Nabng2cWNEd2VPQzdxcU96aHRDOFgyTUR0S3hQNXQ3MVVXQ2xDRGZKWkxNQVgyQl83eW1VQU8yX2hZVS0yR25COHJyTndBcG5xZUd2dFVvOUNPOE5BSkhnaVN4dGVQVFNreWQ0SmFFcTZwdFdmUlZqcTFsekRMcw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC90" t="inlineStr">
+        <is>
+          <t>Katie Stockton: Bracing for volatility after Nasdaq broke below recent support - CNBC</t>
+        </is>
+      </c>
+      <c r="AD90" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLWhuVXhhdF9LbEhfSTV2RlNTZ0IyVjBlcUxGS0RQLXA5S0xjUWFZa3c3Nm1OZmxSRU5mVmVLZzRkbEFKYWd1YWFoVHdadUpRRXlMc1BSVi1BY2Q5RlVLRzVoa2xuRkxZdThVS0VVTzRYY256MHZha1l6RDlrU0NaVXZGZW1qZFRWbTBOUFBTRGxUck9ZWk9tWlY4bl9LcU1BVG5Ka0RVVURXallmZGhqT1BacEpBYnFTUzBIRQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-09-17T03:50:29+00:00</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>76146.57030000001</v>
+      </c>
+      <c r="F91" t="n">
+        <v>76704.60159999999</v>
+      </c>
+      <c r="G91" t="n">
+        <v>76008.3125</v>
+      </c>
+      <c r="H91" t="n">
+        <v>76369.3125</v>
+      </c>
+      <c r="I91" t="n">
+        <v>4821362688</v>
+      </c>
+      <c r="J91" t="n">
+        <v>4</v>
+      </c>
+      <c r="K91" t="n">
+        <v>38</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="M91" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="N91" t="n">
+        <v>34</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="P91" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>12.812</v>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>Crypto Trading Volume Surges as September Tests Strength of August Demand - CryptoRank</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNbDVSTFEtRFUxcVAzSFROUVpiN2x1RXhSWUxheU1Fa0FnY2JLbWpCcnhQYmJ2Rkh1YkN2UUFHZ28zdXV3d1hZaVktQ2FydHJKY291VEhpT0pYOXlQeU54aXlEMVpvd0ZRc0dJcnJQcFZQOHZoNk9RM20xOTdnWFUyS0RVTXMzQUlnXzQ2Wi1kaGc0Ry1kWDlRdHp2alBwRWJBTlNFa0hyNGctYkdFd2tHaQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W91" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - Pulse 2.0</t>
+        </is>
+      </c>
+      <c r="Z91" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA91" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - Crypto News</t>
+        </is>
+      </c>
+      <c r="AB91" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC91" t="inlineStr">
+        <is>
+          <t>Crypto’s Latest Rebound is Fueled By More Liquidations - bloomberg.com</t>
+        </is>
+      </c>
+      <c r="AD91" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcTZKMERXNUtEc1UtZTlmNy1RS21TYTV1ZXJuUzF3Rjkza1Zwbk4yWW5aRmxQSDRoWW4wU0ZadTVydVdiS01pNGlnYjZ3R0loMmp4YzNQT0N4TjVsNERrLWhzRm5QWEJFNFVFZ2lxZzNtRkM0c3Q5RkV6YzlubW9RSFZ6SFF0OHJXdHlONS1TS2Itd0JSaG5IVHJmdzNOY3l1RjNsNHFsckU?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-17 09:19 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD91"/>
+  <dimension ref="A1:AD97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11801,6 +11801,762 @@
       <c r="AD91" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcTZKMERXNUtEc1UtZTlmNy1RS21TYTV1ZXJuUzF3Rjkza1Zwbk4yWW5aRmxQSDRoWW4wU0ZadTVydVdiS01pNGlnYjZ3R0loMmp4YzNQT0N4TjVsNERrLWhzRm5QWEJFNFVFZ2lxZzNtRkM0c3Q5RkV6YzlubW9RSFZ6SFF0OHJXdHlONS1TS2Itd0JSaG5IVHJmdzNOY3l1RjNsNHFsckU?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-09-17T09:17:25+00:00</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>4342.5</v>
+      </c>
+      <c r="F92" t="n">
+        <v>4374.3999</v>
+      </c>
+      <c r="G92" t="n">
+        <v>4342.2998</v>
+      </c>
+      <c r="H92" t="n">
+        <v>4355.2002</v>
+      </c>
+      <c r="I92" t="n">
+        <v>20678</v>
+      </c>
+      <c r="J92" t="n">
+        <v>4</v>
+      </c>
+      <c r="K92" t="n">
+        <v>39</v>
+      </c>
+      <c r="L92" t="n">
+        <v>-0.172</v>
+      </c>
+      <c r="M92" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="N92" t="n">
+        <v>40</v>
+      </c>
+      <c r="O92" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="P92" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>-3.54</v>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>Spark Starts Tungsten Exploration at Seridó as Global Demand Surges - TMX Newsfile</t>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOaUUzcW0td2tKUk9KSk15VTRtbXFHazdHRl9oeWh4VzM0M2Y4VUthT0NVWnVuZE9BZ2t6ZUxDdmhCcUo4T3pteDVyTk1UT09SbU5uSHJHU204TFI0UE5TeUozc1ZkUGowUmg2ckZWRDkxVU1OOEJOSkdVQUJsZkRqTnZTTHBjMUNYLVhxU2pfanFCODRPSV92ZVQ2eWpDN0xZQ2VHek9hVU1EMFQ1QWYw?oc=5</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="W92" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X92" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y92" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z92" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA92" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AB92" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC92" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AD92" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-09-17T09:17:25+00:00</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>101.43</v>
+      </c>
+      <c r="F93" t="n">
+        <v>101.98</v>
+      </c>
+      <c r="G93" t="n">
+        <v>100.39</v>
+      </c>
+      <c r="H93" t="n">
+        <v>101.49</v>
+      </c>
+      <c r="I93" t="n">
+        <v>27565</v>
+      </c>
+      <c r="J93" t="n">
+        <v>4</v>
+      </c>
+      <c r="K93" t="n">
+        <v>40</v>
+      </c>
+      <c r="L93" t="n">
+        <v>-0.018</v>
+      </c>
+      <c r="M93" t="n">
+        <v>-0.196</v>
+      </c>
+      <c r="N93" t="n">
+        <v>40</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0.187</v>
+      </c>
+      <c r="P93" t="n">
+        <v>-0.151</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>3.393</v>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="W93" t="inlineStr">
+        <is>
+          <t>Current price of oil as of July 30, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9odGxncTZBdXJrcnd4Zm1GSENJSFpJQUJxbGphdTV2dTRfQTVmMzVFQ21PTGhzY19DSGVFUWpoeEtGMDZhNzRveUNoaDBlcDVLSmRpaFh6ZnA1emJSVllSYTNR?oc=5</t>
+        </is>
+      </c>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z93" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA93" t="inlineStr">
+        <is>
+          <t>OPEC oil output falls in August, Reuters survey shows - Reuters</t>
+        </is>
+      </c>
+      <c r="AB93" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcGZWQVVsSEY1MDZDLXRVM2g2N0t1bHJ1VXpWX3pScTFZak53OGQ5VVNxemw0Mjdrd1paNjRYb1YtdFlYN3RIOURKM00xZmc4eFRlTHk2cTNhODJKWW5TOS1BMEE1cVF2NTN5YjJaeHRRNFlBVHUwUU9CN0pyOEdRMHE0c2VtcGNvamRPVFd3OVVlTnFmV3Fobks2WlZJU21oRW44?oc=5</t>
+        </is>
+      </c>
+      <c r="AC93" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD93" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-09-17T09:17:25+00:00</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>100.244</v>
+      </c>
+      <c r="F94" t="n">
+        <v>100.254</v>
+      </c>
+      <c r="G94" t="n">
+        <v>100.101</v>
+      </c>
+      <c r="H94" t="n">
+        <v>100.177</v>
+      </c>
+      <c r="I94" t="n">
+        <v>0</v>
+      </c>
+      <c r="J94" t="n">
+        <v>4</v>
+      </c>
+      <c r="K94" t="n">
+        <v>39</v>
+      </c>
+      <c r="L94" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="M94" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="N94" t="n">
+        <v>40</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="P94" t="n">
+        <v>-0.007</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>1.367</v>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>Dollar holds firm as angst over Iran-U.S. stand-off drives safe-haven demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPYjVva2k0WFlQTjA2T1hrRzhuaENsdEJaMW4zaVJLSHZRbVBIMENzRlc2Qzl0NGJNVm54RGlBckI4WGpuV05Md3puR1Q2cDBOaDBGbkpvWTVDWDF6aFFOMU5ZN1l3WjFoaG01VjFQU0Jfai1WX3pyVHlSbGQ5cks5OHlET3N5T1BHX2Z0UkJlT0t4MWhkWEZQMVJfZmhUa0Nv0gGmAUFVX3lxTFA1RUg3R3RlUmFOYXo0Z25OTVdzOWJkM0dER0tPMVJFWjdRZVhBa1dBa1FyTXZ1aldVOXUwcllYaHJtaDVNYTZuNTNyMnRPRGRmTUlxQXBKdHp2c0o5d2VwLWN3WVRReVBIX1ZZTm1mcHhvZnVxS09NYk1GTDhBYkpzbHJaMmlNNFprSlE5NEdtT09tdk81MlZabmNDLUNNSF9idklOX0E?oc=5</t>
+        </is>
+      </c>
+      <c r="W94" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z94" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA94" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - fxstreet.com</t>
+        </is>
+      </c>
+      <c r="AB94" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC94" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD94" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-09-17T09:17:25+00:00</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>7657</v>
+      </c>
+      <c r="F95" t="n">
+        <v>7689.25</v>
+      </c>
+      <c r="G95" t="n">
+        <v>7656.75</v>
+      </c>
+      <c r="H95" t="n">
+        <v>7686.5</v>
+      </c>
+      <c r="I95" t="n">
+        <v>69386</v>
+      </c>
+      <c r="J95" t="n">
+        <v>4</v>
+      </c>
+      <c r="K95" t="n">
+        <v>38</v>
+      </c>
+      <c r="L95" t="n">
+        <v>-0.305</v>
+      </c>
+      <c r="M95" t="n">
+        <v>-0.026</v>
+      </c>
+      <c r="N95" t="n">
+        <v>39</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0.355</v>
+      </c>
+      <c r="P95" t="n">
+        <v>-0.051</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>0.635</v>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>Tax revenue surges amid boom in stock market - Taipei Times</t>
+        </is>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBVYTNZQ2Q4RFRxNEVSUnVLLTZRQUkyVjF1dEtOZ0hiZ1NreVV3NUx1b1RXdWNoRXZIWlB6MnhXakR3SFdvTGt5SG1NZWFLVjZrUGd4MXk0dVEzRkY5NGJkTUtWSmtwalA5RWlLXzQyVGMwN2pjcEE?oc=5</t>
+        </is>
+      </c>
+      <c r="W95" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 2: Dell Surges 16% on Soaring AI Backlog - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQWTRuSVIyTFR2RTZveHRTN3hEWnBwSDl4T2J4ZHZPT01OdEYzWUk3MXZJZjNIc0tTMGYtYmFIYnkxd1dfVVVKTks0MmhzTlc5Z014VHVMMHJVMmZkWWlYVXdHWlczYWRQNzRyYk5leV9ncFBQVE1CbVdTbGNxclNhTy1JNEQwSlVmNjhjOGZrQXBLZlFG?oc=5</t>
+        </is>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>Wall Street Drops as Fed Chair Kevin Warsh Delivers Hawkish Remarks - news.sbs.co.kr</t>
+        </is>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE1LOHlueWljVGhtM3ZlS0JMQlNaMWFmMGp0bFZFVkZZbXZNb0Nsb1RFYy1RVzJieHFJZ2xia0ZUTHRZMnJOcUhMMEg0UkE5N2xCM2haM05RT3ZncjA1NVNMU3dHS3ZjamFnYnhKVUNR0gFmQVVfeXFMUFhmOVBrU1hyR1ktdXJxWDBBLU9iQURxVEZLN1NoVGVwUmV1eGpKMGs0ZjBhcUdSaFFnZVJVS2ltNGE3SmNmNFB6N1RONDVGYURnQXdvMnNNTEVTQ2huenBLc1V1YnFB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>Dow Drops 631, Nasdaq Slips 3, S&amp;P 500 Falls 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB95" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQVFVRNlU5aU5HaTYzZ2tnN1Nabng2cWNEd2VPQzdxcU96aHRDOFgyTUR0S3hQNXQ3MVVXQ2xDRGZKWkxNQVgyQl83eW1VQU8yX2hZVS0yR25COHJyTndBcG5xZUd2dFVvOUNPOE5BSkhnaVN4dGVQVFNreWQ0SmFFcTZwdFdmUlZqcTFsekRMcw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC95" t="inlineStr">
+        <is>
+          <t>Dow Drops 328, Nasdaq Falls 205, S&amp;P 500 Slips 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD95" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNd1haNmttZldnUzZjUGF2U2p6WmEtWXpoTVZjTFAyc3EzcUhWaHdoY2tnalNGc1ZYcVlMUXFicWlxTUE3TUowaVVfbFlIMWgyeGdNcDBNNVE3Z1J6S1lHa0p3TnBQbDRDVThGR3RMSXBlbS1MbHFVX3EwemVxRlZ6RzVEVVdvT2hiSVRydlNtalVnQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-09-17T09:17:25+00:00</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>29372.5</v>
+      </c>
+      <c r="F96" t="n">
+        <v>29584</v>
+      </c>
+      <c r="G96" t="n">
+        <v>29368.75</v>
+      </c>
+      <c r="H96" t="n">
+        <v>29578.25</v>
+      </c>
+      <c r="I96" t="n">
+        <v>29413</v>
+      </c>
+      <c r="J96" t="n">
+        <v>4</v>
+      </c>
+      <c r="K96" t="n">
+        <v>40</v>
+      </c>
+      <c r="L96" t="n">
+        <v>-0.231</v>
+      </c>
+      <c r="M96" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="N96" t="n">
+        <v>36</v>
+      </c>
+      <c r="O96" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="P96" t="n">
+        <v>-0.014</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>Qualys gains another 7%, extends previous day's rally (QLYS:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQd2UxRm5EenY5VmZnZzh1Vy1OTmxTX2dNQmRyZzd2d3NwdW93S3lENEYxVEVPVDJWZVNwQWJzM3ltQnpxM1RuNnVGYUI5cVlEU0h5OTJqTzRUZUlJaEl5cjlMeDU2VzVfWHRHUUNBQTVSdDRyZWNmSml2ZVQzR01pcDFLa0puRWNUT1NnV2Q0bHZyUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>Lumentum Holdings rises 10% amid optical networking rally (LITE:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOOEE3X3dfVkk2Z19nNG5LRGxXblNEakFtdDZ2bDByUWdPeS1QYl9MYkpkVDRmX3g0SGg1SjhnVHRqMVc4R1RxMTN0UHo0OUtUdDlaaUVPM0pjd09NV2xjZGdoaTVHTEZILVlNNWlvSnNSd1lfRUlBeF8xLWxpQUVMWEUtU1RBZExfMDBJWXZ6Z2xtNjJFbGNsM3pR?oc=5</t>
+        </is>
+      </c>
+      <c r="W96" t="inlineStr">
+        <is>
+          <t>Cybersecurity is one corner of the tech market that's getting a boost from AI doomsday fears - Business Insider</t>
+        </is>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOUkdOM3BPSE8xMS0yWndCcE1aSzd0a3FXOUxIa0tGU3hZMDZ0WGtUODdqVEIwSWkyMnU4d3hIN0ZtZ0NiVmhFc25DM3lkS2kyMXMtUHNwOUdsRll1LUg0VWU5NWFsekZsOXF5M2hBdVhBOTJnYXpnd21Ga1JpUG83RmZfcWNHLWFwQUk2NGd0WjhxMDRrUnhmVkZYSXlmbEsyTkxMV3NwR1MydXkx?oc=5</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>Dow Drops 631, Nasdaq Slips 3, S&amp;P 500 Falls 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQVFVRNlU5aU5HaTYzZ2tnN1Nabng2cWNEd2VPQzdxcU96aHRDOFgyTUR0S3hQNXQ3MVVXQ2xDRGZKWkxNQVgyQl83eW1VQU8yX2hZVS0yR25COHJyTndBcG5xZUd2dFVvOUNPOE5BSkhnaVN4dGVQVFNreWQ0SmFFcTZwdFdmUlZqcTFsekRMcw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>Katie Stockton: Bracing for volatility after Nasdaq broke below recent support - CNBC</t>
+        </is>
+      </c>
+      <c r="AB96" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLWhuVXhhdF9LbEhfSTV2RlNTZ0IyVjBlcUxGS0RQLXA5S0xjUWFZa3c3Nm1OZmxSRU5mVmVLZzRkbEFKYWd1YWFoVHdadUpRRXlMc1BSVi1BY2Q5RlVLRzVoa2xuRkxZdThVS0VVTzRYY256MHZha1l6RDlrU0NaVXZGZW1qZFRWbTBOUFBTRGxUck9ZWk9tWlY4bl9LcU1BVG5Ka0RVVURXallmZGhqT1BacEpBYnFTUzBIRQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC96" t="inlineStr">
+        <is>
+          <t>Dow Drops 328, Nasdaq Falls 205, S&amp;P 500 Slips 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD96" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNd1haNmttZldnUzZjUGF2U2p6WmEtWXpoTVZjTFAyc3EzcUhWaHdoY2tnalNGc1ZYcVlMUXFicWlxTUE3TUowaVVfbFlIMWgyeGdNcDBNNVE3Z1J6S1lHa0p3TnBQbDRDVThGR3RMSXBlbS1MbHFVX3EwemVxRlZ6RzVEVVdvT2hiSVRydlNtalVnQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-09-17T09:17:25+00:00</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>76244.7812</v>
+      </c>
+      <c r="F97" t="n">
+        <v>76658.4375</v>
+      </c>
+      <c r="G97" t="n">
+        <v>76222.2969</v>
+      </c>
+      <c r="H97" t="n">
+        <v>76609.8125</v>
+      </c>
+      <c r="I97" t="n">
+        <v>1533702144</v>
+      </c>
+      <c r="J97" t="n">
+        <v>4</v>
+      </c>
+      <c r="K97" t="n">
+        <v>39</v>
+      </c>
+      <c r="L97" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="M97" t="n">
+        <v>-0.019</v>
+      </c>
+      <c r="N97" t="n">
+        <v>33</v>
+      </c>
+      <c r="O97" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="P97" t="n">
+        <v>-0.018</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>14.38</v>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>Crypto Trading Volume Surges as September Tests Strength of August Demand - CryptoRank</t>
+        </is>
+      </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNbDVSTFEtRFUxcVAzSFROUVpiN2x1RXhSWUxheU1Fa0FnY2JLbWpCcnhQYmJ2Rkh1YkN2UUFHZ28zdXV3d1hZaVktQ2FydHJKY291VEhpT0pYOXlQeU54aXlEMVpvd0ZRc0dJcnJQcFZQOHZoNk9RM20xOTdnWFUyS0RVTXMzQUlnXzQ2Wi1kaGc0Ry1kWDlRdHp2alBwRWJBTlNFa0hyNGctYkdFd2tHaQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W97" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - foxbusiness.com</t>
+        </is>
+      </c>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y97" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - Pulse 2.0</t>
+        </is>
+      </c>
+      <c r="Z97" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA97" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - Crypto News</t>
+        </is>
+      </c>
+      <c r="AB97" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC97" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - global.morningstar.com</t>
+        </is>
+      </c>
+      <c r="AD97" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-17 16:28 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD97"/>
+  <dimension ref="A1:AD103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12557,6 +12557,762 @@
       <c r="AD97" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-09-17T16:26:43+00:00</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>4413.7998</v>
+      </c>
+      <c r="F98" t="n">
+        <v>4420.8999</v>
+      </c>
+      <c r="G98" t="n">
+        <v>4391.7998</v>
+      </c>
+      <c r="H98" t="n">
+        <v>4407.2998</v>
+      </c>
+      <c r="I98" t="n">
+        <v>38436</v>
+      </c>
+      <c r="J98" t="n">
+        <v>4</v>
+      </c>
+      <c r="K98" t="n">
+        <v>39</v>
+      </c>
+      <c r="L98" t="n">
+        <v>-0.124</v>
+      </c>
+      <c r="M98" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="N98" t="n">
+        <v>40</v>
+      </c>
+      <c r="O98" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P98" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>Copper Miners Capitalize on Tight Supply &amp; Growing Demand - ETF Trends</t>
+        </is>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQTHJDUGNNT3BEei1wbGJCVnd4X2JuX2Jsb1JtSGpLbHBFQnphd1JQSWR1MUxJdm1hMlprT19qc1o5WnVTeGg4WWlCaUg0X3BHVDlvUW9xamx3N3lJNmJKam8ya3hwQ25wbmlXcHJQT0lRRkxjakZYMVZUU1hKZUV3U0tqWlBKODlOYnBibUxtalpjd0FzWFJnME56azZLanR4ZkpOdWc5RWNhbjBaQ0pLS1Bndw?oc=5</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>Gold gains over 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W98" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="Z98" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA98" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AB98" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC98" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD98" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-09-17T16:26:43+00:00</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>99.97</v>
+      </c>
+      <c r="F99" t="n">
+        <v>101.29</v>
+      </c>
+      <c r="G99" t="n">
+        <v>99.59</v>
+      </c>
+      <c r="H99" t="n">
+        <v>101.19</v>
+      </c>
+      <c r="I99" t="n">
+        <v>67350</v>
+      </c>
+      <c r="J99" t="n">
+        <v>4</v>
+      </c>
+      <c r="K99" t="n">
+        <v>40</v>
+      </c>
+      <c r="L99" t="n">
+        <v>-0.063</v>
+      </c>
+      <c r="M99" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="N99" t="n">
+        <v>40</v>
+      </c>
+      <c r="O99" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="P99" t="n">
+        <v>-0.104</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>1.935</v>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>Gold gains over 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA99" t="inlineStr">
+        <is>
+          <t>OPEC oil output falls in August, Reuters survey shows - Reuters</t>
+        </is>
+      </c>
+      <c r="AB99" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcGZWQVVsSEY1MDZDLXRVM2g2N0t1bHJ1VXpWX3pScTFZak53OGQ5VVNxemw0Mjdrd1paNjRYb1YtdFlYN3RIOURKM00xZmc4eFRlTHk2cTNhODJKWW5TOS1BMEE1cVF2NTN5YjJaeHRRNFlBVHUwUU9CN0pyOEdRMHE0c2VtcGNvamRPVFd3OVVlTnFmV3Fobks2WlZJU21oRW44?oc=5</t>
+        </is>
+      </c>
+      <c r="AC99" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD99" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-09-17T16:26:43+00:00</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>100.077</v>
+      </c>
+      <c r="F100" t="n">
+        <v>100.25</v>
+      </c>
+      <c r="G100" t="n">
+        <v>100.036</v>
+      </c>
+      <c r="H100" t="n">
+        <v>100.23</v>
+      </c>
+      <c r="I100" t="n">
+        <v>0</v>
+      </c>
+      <c r="J100" t="n">
+        <v>4</v>
+      </c>
+      <c r="K100" t="n">
+        <v>39</v>
+      </c>
+      <c r="L100" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="M100" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="N100" t="n">
+        <v>39</v>
+      </c>
+      <c r="O100" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="P100" t="n">
+        <v>-0.036</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>0.538</v>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>Dollar holds firm as angst over Iran-U.S. stand-off drives safe-haven demand - CNBC</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPYjVva2k0WFlQTjA2T1hrRzhuaENsdEJaMW4zaVJLSHZRbVBIMENzRlc2Qzl0NGJNVm54RGlBckI4WGpuV05Md3puR1Q2cDBOaDBGbkpvWTVDWDF6aFFOMU5ZN1l3WjFoaG01VjFQU0Jfai1WX3pyVHlSbGQ5cks5OHlET3N5T1BHX2Z0UkJlT0t4MWhkWEZQMVJfZmhUa0Nv0gGmAUFVX3lxTFA1RUg3R3RlUmFOYXo0Z25OTVdzOWJkM0dER0tPMVJFWjdRZVhBa1dBa1FyTXZ1aldVOXUwcllYaHJtaDVNYTZuNTNyMnRPRGRmTUlxQXBKdHp2c0o5d2VwLWN3WVRReVBIX1ZZTm1mcHhvZnVxS09NYk1GTDhBYkpzbHJaMmlNNFprSlE5NEdtT09tdk81MlZabmNDLUNNSF9idklOX0E?oc=5</t>
+        </is>
+      </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W100" t="inlineStr">
+        <is>
+          <t>Gold rebounds above $4,300 after Fed hike as dollar eases - Investing.com</t>
+        </is>
+      </c>
+      <c r="X100" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQMmUxMzhHWWZ1aTVBY21hU3RQVFlxcVhUdENoSE04MkFiQ3FZZVAxVjZ1d1VQVVJpVXkzc2dpVDU1MUo1aF9GWTFsNjB6SzhiTjRjZUVQempuczM4aXllX0tCaS1xU1d2dkEwZkhBTVFLMWtzeEhUSllsTUU4WEtiS0d0WVRpU0JKejVDa1pzbERTQXBrZmlJV25lQnlXamw3OGRyYnBaeGFCd0d0TVF6TUZvSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y100" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z100" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA100" t="inlineStr">
+        <is>
+          <t>Gold climbs over 2% as US Dollar trims post-Fed gains - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB100" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPRG5KNUhGZkw4cUIzSmtOLV92bmhnbWE0a1NZMGJSNHdnUnluM05tT2hKSk44cFZFME52LWxETTlvUllCX2VkdHVNLTVlaXdaTURfWHBXY3J2U01BVXl1TDE0dWQyT1ZVV1VwR0RyZ2p0MTdUbmExY1dlNHJPS3EzaVN1MWpwSzVGR1dIYW56aTk1SnlLMnpFcFNpeW4xNVVZT19lcmZhV2JldHJwcTJn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC100" t="inlineStr">
+        <is>
+          <t>FX Daily: Fed hold can hit the dollar today - think.ing.com</t>
+        </is>
+      </c>
+      <c r="AD100" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE91QWFPVUVXdGYyVGFxekZhSXBLNzFWN2xfWkJVRXNud05nSzJPQXpwN1hjbzJxZ0ZWLWdmTWhXbzI4NFRXdnpobUc2MllDT1VFQWtFbzhiZ1kzX0Z2c3FGal9nZF91Y19ISENwR1RVdnBRVVVhc0EtY3BmOEZKU1k?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-09-17T16:26:43+00:00</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>7717.75</v>
+      </c>
+      <c r="F101" t="n">
+        <v>7722</v>
+      </c>
+      <c r="G101" t="n">
+        <v>7680.5</v>
+      </c>
+      <c r="H101" t="n">
+        <v>7704.5</v>
+      </c>
+      <c r="I101" t="n">
+        <v>551704</v>
+      </c>
+      <c r="J101" t="n">
+        <v>4</v>
+      </c>
+      <c r="K101" t="n">
+        <v>39</v>
+      </c>
+      <c r="L101" t="n">
+        <v>-0.192</v>
+      </c>
+      <c r="M101" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="N101" t="n">
+        <v>40</v>
+      </c>
+      <c r="O101" t="n">
+        <v>0.312</v>
+      </c>
+      <c r="P101" t="n">
+        <v>-0.003</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>2.005</v>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>Revvity Inc. stock extends rally after 52-week high and strong S&amp;P 500 outperformance - ad-hoc-news.de</t>
+        </is>
+      </c>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQQjZaU0U2bnZyaFFXRW1GdkpiaUdUTzg3VFNrbUE0QndoNjFLcE53Qlg4Tnd5M2lsdGNzVkJjNF9NeWw0UmhCZk83VkM2dWNhNVRVRlF5bUEtOGZWb2hGQ29tN3dHdjMtSnpFZnlBZ194VndfNmxVdVdPWjFuU1RjZW5RUUdiSi1SRFBZdjAySS1hNHpIbWxNaFQ4R1VoSTZMc3YtdHZKR08zalk3bVdES2p3RkpJVnZiUDUxY0JkV3VaQ0lGai1MWTRZczd3NTE2VVE?oc=5</t>
+        </is>
+      </c>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 2: Dell Surges 16% on Soaring AI Backlog - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X101" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQWTRuSVIyTFR2RTZveHRTN3hEWnBwSDl4T2J4ZHZPT01OdEYzWUk3MXZJZjNIc0tTMGYtYmFIYnkxd1dfVVVKTks0MmhzTlc5Z014VHVMMHJVMmZkWWlYVXdHWlczYWRQNzRyYk5leV9ncFBQVE1CbVdTbGNxclNhTy1JNEQwSlVmNjhjOGZrQXBLZlFG?oc=5</t>
+        </is>
+      </c>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t>Wall Street Drops as Fed Chair Kevin Warsh Delivers Hawkish Remarks - news.sbs.co.kr</t>
+        </is>
+      </c>
+      <c r="Z101" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE1LOHlueWljVGhtM3ZlS0JMQlNaMWFmMGp0bFZFVkZZbXZNb0Nsb1RFYy1RVzJieHFJZ2xia0ZUTHRZMnJOcUhMMEg0UkE5N2xCM2haM05RT3ZncjA1NVNMU3dHS3ZjamFnYnhKVUNR0gFmQVVfeXFMUFhmOVBrU1hyR1ktdXJxWDBBLU9iQURxVEZLN1NoVGVwUmV1eGpKMGs0ZjBhcUdSaFFnZVJVS2ltNGE3SmNmNFB6N1RONDVGYURnQXdvMnNNTEVTQ2huenBLc1V1YnFB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA101" t="inlineStr">
+        <is>
+          <t>Dow Drops 631, Nasdaq Slips 3, S&amp;P 500 Falls 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB101" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQVFVRNlU5aU5HaTYzZ2tnN1Nabng2cWNEd2VPQzdxcU96aHRDOFgyTUR0S3hQNXQ3MVVXQ2xDRGZKWkxNQVgyQl83eW1VQU8yX2hZVS0yR25COHJyTndBcG5xZUd2dFVvOUNPOE5BSkhnaVN4dGVQVFNreWQ0SmFFcTZwdFdmUlZqcTFsekRMcw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC101" t="inlineStr">
+        <is>
+          <t>Dow Drops 328, Nasdaq Falls 205, S&amp;P 500 Slips 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD101" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNd1haNmttZldnUzZjUGF2U2p6WmEtWXpoTVZjTFAyc3EzcUhWaHdoY2tnalNGc1ZYcVlMUXFicWlxTUE3TUowaVVfbFlIMWgyeGdNcDBNNVE3Z1J6S1lHa0p3TnBQbDRDVThGR3RMSXBlbS1MbHFVX3EwemVxRlZ6RzVEVVdvT2hiSVRydlNtalVnQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-09-17T16:26:43+00:00</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>29724.25</v>
+      </c>
+      <c r="F102" t="n">
+        <v>29750</v>
+      </c>
+      <c r="G102" t="n">
+        <v>29605.75</v>
+      </c>
+      <c r="H102" t="n">
+        <v>29737.25</v>
+      </c>
+      <c r="I102" t="n">
+        <v>216537</v>
+      </c>
+      <c r="J102" t="n">
+        <v>4</v>
+      </c>
+      <c r="K102" t="n">
+        <v>40</v>
+      </c>
+      <c r="L102" t="n">
+        <v>-0.345</v>
+      </c>
+      <c r="M102" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="N102" t="n">
+        <v>37</v>
+      </c>
+      <c r="O102" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P102" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>-2.621</v>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>Lumentum Holdings rises 10% amid optical networking rally (LITE:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOOEE3X3dfVkk2Z19nNG5LRGxXblNEakFtdDZ2bDByUWdPeS1QYl9MYkpkVDRmX3g0SGg1SjhnVHRqMVc4R1RxMTN0UHo0OUtUdDlaaUVPM0pjd09NV2xjZGdoaTVHTEZILVlNNWlvSnNSd1lfRUlBeF8xLWxpQUVMWEUtU1RBZExfMDBJWXZ6Z2xtNjJFbGNsM3pR?oc=5</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>Cybersecurity is one corner of the tech market that's getting a boost from AI doomsday fears - Business Insider</t>
+        </is>
+      </c>
+      <c r="V102" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOUkdOM3BPSE8xMS0yWndCcE1aSzd0a3FXOUxIa0tGU3hZMDZ0WGtUODdqVEIwSWkyMnU4d3hIN0ZtZ0NiVmhFc25DM3lkS2kyMXMtUHNwOUdsRll1LUg0VWU5NWFsekZsOXF5M2hBdVhBOTJnYXpnd21Ga1JpUG83RmZfcWNHLWFwQUk2NGd0WjhxMDRrUnhmVkZYSXlmbEsyTkxMV3NwR1MydXkx?oc=5</t>
+        </is>
+      </c>
+      <c r="W102" t="inlineStr">
+        <is>
+          <t>European stocks rise on tech gains ahead of Fed decision - Anadolu Ajansı</t>
+        </is>
+      </c>
+      <c r="X102" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNM2V1cUpxYmtQVy1jWUQ3c2dxOVEwd1Q1NDNoVGhaYzh4QkFTbVZDYkZxUnVSb09hejE4RTFKM2lVekNLTEt5U0g4TjJXSkcyc2Y5T3R1M0QwNTdsa01OLVItMGhpdHJpOVRfc3RrVzBwVlo0WmRCdUlscjVjaENUeklXMTBUOW13cmZTYTFndkdqT0k0MF9QOQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y102" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA102" t="inlineStr">
+        <is>
+          <t>Nasdaq rises as markets recover from Fed-driven selloff - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AB102" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOWS0zdTlhbWQ3LWdDYWVPN0tiY0lUMlJET2JuaXdYRy1IWlpRQXRJTVdtTHRGUkJpbVpoUkRvUm5lTkgtLUxTZzUyOVZVb3NtWXJCN29nV3hVQ3ZyN1l1cHotVEhnN1FlLTdzOGVnZ2l2OFRQSFJiMXNKak9EUlBIMEFUSTkzVzd5U3hacHVCVy1leXFvVjRDYjhLY1pFSm1pdnp2NTJablBWbGVWYm1qamJZUWlzUl9hS3VEamo1dmtvdkQ0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC102" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="AD102" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-09-17T16:26:43+00:00</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>76646.71090000001</v>
+      </c>
+      <c r="F103" t="n">
+        <v>76966.75</v>
+      </c>
+      <c r="G103" t="n">
+        <v>75937.10159999999</v>
+      </c>
+      <c r="H103" t="n">
+        <v>76620.32030000001</v>
+      </c>
+      <c r="I103" t="n">
+        <v>965734400</v>
+      </c>
+      <c r="J103" t="n">
+        <v>4</v>
+      </c>
+      <c r="K103" t="n">
+        <v>38</v>
+      </c>
+      <c r="L103" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="M103" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="N103" t="n">
+        <v>34</v>
+      </c>
+      <c r="O103" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="P103" t="n">
+        <v>-0.057</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>9.154</v>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>Crypto Market Breadth Surges to 89 Advancers in QC 100, Bitcoin Trails Behind - KuCoin</t>
+        </is>
+      </c>
+      <c r="V103" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOOHE3cXV2S0FIWmRkZllNcFFSd0ttQXp2UVltTWhJUUZta2NETEZ4TWp1clhnbXF4bnNlVjhKdGNVUnNDeHl0endMbUZyTTRPN29qWFR6Qjk1SFR5a0I5c1NLbGVyRWZLZW80RlNZNEVDY1lLbm9mYktBMHV0UFEzVjByM1RFeG5IcGp6U2FMMlhDWWUyMnlOYk1MZVU4Z3EtN0pQLTZEYTBfZldlVjdj?oc=5</t>
+        </is>
+      </c>
+      <c r="W103" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="Z103" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA103" t="inlineStr">
+        <is>
+          <t>Zcash jumps 17% amid $345M liquidations after F... - Pluang</t>
+        </is>
+      </c>
+      <c r="AB103" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxPNTZnb05wT2NfdkRGTmxpYjloR2xRRFNVQm1BLVdqdlFaVjNad0d1c3dELTVGLThEMllvV0FDa0FTUUZEekxYc2VPRzYta29nbkV4MF9FemVicmNzNG1DLTJZTnI4MUtnSngwN3hXdlJUMGpkSUt5T016dE9kaDRGaXlVR01XWUJLT0h6Yw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC103" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - Crypto News</t>
+        </is>
+      </c>
+      <c r="AD103" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-17 22:46 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD103"/>
+  <dimension ref="A1:AD109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13313,6 +13313,762 @@
       <c r="AD103" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-09-17T22:44:35+00:00</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>4401.2002</v>
+      </c>
+      <c r="F104" t="n">
+        <v>4405.6001</v>
+      </c>
+      <c r="G104" t="n">
+        <v>4380.2998</v>
+      </c>
+      <c r="H104" t="n">
+        <v>4385.7998</v>
+      </c>
+      <c r="I104" t="n">
+        <v>12548</v>
+      </c>
+      <c r="J104" t="n">
+        <v>4</v>
+      </c>
+      <c r="K104" t="n">
+        <v>40</v>
+      </c>
+      <c r="L104" t="n">
+        <v>-0.08799999999999999</v>
+      </c>
+      <c r="M104" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="N104" t="n">
+        <v>40</v>
+      </c>
+      <c r="O104" t="n">
+        <v>0.191</v>
+      </c>
+      <c r="P104" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>2.066</v>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>Copper Miners Capitalize on Tight Supply &amp; Growing Demand - ETF Trends</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQTHJDUGNNT3BEei1wbGJCVnd4X2JuX2Jsb1JtSGpLbHBFQnphd1JQSWR1MUxJdm1hMlprT19qc1o5WnVTeGg4WWlCaUg0X3BHVDlvUW9xamx3N3lJNmJKam8ya3hwQ25wbmlXcHJQT0lRRkxjakZYMVZUU1hKZUV3U0tqWlBKODlOYnBibUxtalpjd0FzWFJnME56azZLanR4ZkpOdWc5RWNhbjBaQ0pLS1Bndw?oc=5</t>
+        </is>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>Gold gains over 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="V104" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W104" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="X104" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="Z104" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA104" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB104" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC104" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD104" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-09-17T22:44:35+00:00</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>101.98</v>
+      </c>
+      <c r="F105" t="n">
+        <v>102.15</v>
+      </c>
+      <c r="G105" t="n">
+        <v>100.88</v>
+      </c>
+      <c r="H105" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="I105" t="n">
+        <v>27959</v>
+      </c>
+      <c r="J105" t="n">
+        <v>4</v>
+      </c>
+      <c r="K105" t="n">
+        <v>40</v>
+      </c>
+      <c r="L105" t="n">
+        <v>-0.114</v>
+      </c>
+      <c r="M105" t="n">
+        <v>-0.252</v>
+      </c>
+      <c r="N105" t="n">
+        <v>40</v>
+      </c>
+      <c r="O105" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="P105" t="n">
+        <v>-0.138</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>2.868</v>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>Gold gains over 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="V105" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W105" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y105" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 14, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z105" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE4tdE1rdjRWWXpiWnJuWTNleXhKNGN1ZW9Qb3h1Ujh6cU91RFhOUXBDWXNaTXI4UVpVQnpPbEU3OTM5aUpWdTYxTGk0Um51cTY1X3psSF9MVXdoZHJpbWJXUkpn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA105" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB105" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC105" t="inlineStr">
+        <is>
+          <t>OPEC oil output falls in August, Reuters survey shows - Reuters</t>
+        </is>
+      </c>
+      <c r="AD105" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcGZWQVVsSEY1MDZDLXRVM2g2N0t1bHJ1VXpWX3pScTFZak53OGQ5VVNxemw0Mjdrd1paNjRYb1YtdFlYN3RIOURKM00xZmc4eFRlTHk2cTNhODJKWW5TOS1BMEE1cVF2NTN5YjJaeHRRNFlBVHUwUU9CN0pyOEdRMHE0c2VtcGNvamRPVFd3OVVlTnFmV3Fobks2WlZJU21oRW44?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-09-17T22:44:35+00:00</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>100.248</v>
+      </c>
+      <c r="F106" t="n">
+        <v>100.253</v>
+      </c>
+      <c r="G106" t="n">
+        <v>100.196</v>
+      </c>
+      <c r="H106" t="n">
+        <v>100.236</v>
+      </c>
+      <c r="I106" t="n">
+        <v>0</v>
+      </c>
+      <c r="J106" t="n">
+        <v>4</v>
+      </c>
+      <c r="K106" t="n">
+        <v>39</v>
+      </c>
+      <c r="L106" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="M106" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="N106" t="n">
+        <v>39</v>
+      </c>
+      <c r="O106" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="P106" t="n">
+        <v>-0.066</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>1.888</v>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>US dollar index hits its highest since May as war-driven oil rally boosts safe-haven demand - aa.com.tr</t>
+        </is>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxOWkZKOWhZTF80bEh1ODhHd2s4dDM1Zm9sNTB6a25FME9HYy1UYkV5RllBdmJwTVJKUzMyMWRxVnJhRUt1eW9KSnQtNnR1SFUySEQ3eGtWaER0ZEtaVk84ZGM5REZmWmVrNklENFpKWldMNEtEN2JkbFpOSFZwb082NWxIWFgtTUNfdVg4RnZOMzVFd3F1VmFscUtleEg0MmN3RmcweldUOGpsRUxzMENSMVpOM1NUTGZkMTNHRm12UDRuRXdwcmdSeXQ1bGc?oc=5</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>Dollar holds firm as angst over Iran-U.S. stand-off drives safe-haven demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V106" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPYjVva2k0WFlQTjA2T1hrRzhuaENsdEJaMW4zaVJLSHZRbVBIMENzRlc2Qzl0NGJNVm54RGlBckI4WGpuV05Md3puR1Q2cDBOaDBGbkpvWTVDWDF6aFFOMU5ZN1l3WjFoaG01VjFQU0Jfai1WX3pyVHlSbGQ5cks5OHlET3N5T1BHX2Z0UkJlT0t4MWhkWEZQMVJfZmhUa0Nv0gGmAUFVX3lxTFA1RUg3R3RlUmFOYXo0Z25OTVdzOWJkM0dER0tPMVJFWjdRZVhBa1dBa1FyTXZ1aldVOXUwcllYaHJtaDVNYTZuNTNyMnRPRGRmTUlxQXBKdHp2c0o5d2VwLWN3WVRReVBIX1ZZTm1mcHhvZnVxS09NYk1GTDhBYkpzbHJaMmlNNFprSlE5NEdtT09tdk81MlZabmNDLUNNSF9idklOX0E?oc=5</t>
+        </is>
+      </c>
+      <c r="W106" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X106" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y106" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - FXStreet</t>
+        </is>
+      </c>
+      <c r="Z106" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA106" t="inlineStr">
+        <is>
+          <t>US stocks rebound as dovish Fed and weak ADP cool yields, dent dollar and lift gold - VT Markets</t>
+        </is>
+      </c>
+      <c r="AB106" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQUW1QcWR4RlJfWFVoVENIX05tcjJSR3dkbm9rMzVnNFZvaDUzbHlfSU41LTNHTFctZ3NLRFVtVjUyaEdtUnpvdGtoZHdLbjFRdndoZWxCRUxIc2d3NEFrVmNKUGFNbzF0Y1FBYXRIRHktamFaRkc0bnlYV2Nya21WU1g0Rlgxa2ZGaFF3QktZNEtJWlFsRkI3VjFxNWxfaHlVamtFaU1DeUtrdVdnMnppV2pfMWhzQV81UDZ6TXVYX1lUZjhZMUpR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC106" t="inlineStr">
+        <is>
+          <t>Gold climbs over 2% as US Dollar trims post-Fed gains - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD106" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPRG5KNUhGZkw4cUIzSmtOLV92bmhnbWE0a1NZMGJSNHdnUnluM05tT2hKSk44cFZFME52LWxETTlvUllCX2VkdHVNLTVlaXdaTURfWHBXY3J2U01BVXl1TDE0dWQyT1ZVV1VwR0RyZ2p0MTdUbmExY1dlNHJPS3EzaVN1MWpwSzVGR1dIYW56aTk1SnlLMnpFcFNpeW4xNVVZT19lcmZhV2JldHJwcTJn?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-09-17T22:44:35+00:00</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>7707.75</v>
+      </c>
+      <c r="F107" t="n">
+        <v>7715.5</v>
+      </c>
+      <c r="G107" t="n">
+        <v>7697.5</v>
+      </c>
+      <c r="H107" t="n">
+        <v>7698</v>
+      </c>
+      <c r="I107" t="n">
+        <v>337651</v>
+      </c>
+      <c r="J107" t="n">
+        <v>4</v>
+      </c>
+      <c r="K107" t="n">
+        <v>40</v>
+      </c>
+      <c r="L107" t="n">
+        <v>-0.281</v>
+      </c>
+      <c r="M107" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="N107" t="n">
+        <v>40</v>
+      </c>
+      <c r="O107" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="P107" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>1.676</v>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 2: Dell Surges 16% on Soaring AI Backlog - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQWTRuSVIyTFR2RTZveHRTN3hEWnBwSDl4T2J4ZHZPT01OdEYzWUk3MXZJZjNIc0tTMGYtYmFIYnkxd1dfVVVKTks0MmhzTlc5Z014VHVMMHJVMmZkWWlYVXdHWlczYWRQNzRyYk5leV9ncFBQVE1CbVdTbGNxclNhTy1JNEQwSlVmNjhjOGZrQXBLZlFG?oc=5</t>
+        </is>
+      </c>
+      <c r="W107" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 11: HPE Surges on AI Infrastructure Demand and Recently Raised Guidance - The Globe and Mail</t>
+        </is>
+      </c>
+      <c r="X107" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxOYXB1N0ZORG4ycmM4b2wtdEFqWFRRQVluWkNOYV81RUhYVU9RQ1QyZnoxTlZuNldUYWZXUzAwVmdITHNhS1VOa252ZDdPUTVFdDZlSjl3R2N1MURkQzF6dU5sdHkyU05Nd0hfckJRTFhSTW1STEdsbE96MW9rMDZNM2xMUXpodDJyR2tCR2JhWTZRbXFmQkNPU3pSTTVad0Ywd0loVkZhWnNpaXo1OXZrOWp0ZkJUQVR3SVJXVVlBc1NNMC1NenRiQVBBRHhPNUtiVDBhRGFiVFBiRG5JRVNNU1d3WTNyblE1TFp2OWZpUHQ4Q2hQSEV4T2FoM2VKREVnOW9OTF9tb250anc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="Z107" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA107" t="inlineStr">
+        <is>
+          <t>SPIE stock breaks through its support at €43.10 and falls 2.5% - ideal-investisseur.fr</t>
+        </is>
+      </c>
+      <c r="AB107" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQRVVnaWZ4MlBIbFVrUmo3Z0pCb0VMOTB5LWlYQ25zLU54UmVjMFJEUWptX1FyOEZsbGY5Z1dNSUxqbUxVMFAxcjRZSDMzek5WcjctempiZThIdEtmTm8waVN0bFZuVlVUS044MUhPNXp6b1pBcTlqM1QtQThGMVJLUGYtVGpmdmdKeDNDQWFTenJXeng1OUxCVy1nODRCM0drWkpiaXNZZzRFYjBza2RxMkFJUlZ0U2F0dlVZTEVXQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC107" t="inlineStr">
+        <is>
+          <t>Wall Street Drops as Fed Chair Kevin Warsh Delivers Hawkish Remarks - news.sbs.co.kr</t>
+        </is>
+      </c>
+      <c r="AD107" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE1LOHlueWljVGhtM3ZlS0JMQlNaMWFmMGp0bFZFVkZZbXZNb0Nsb1RFYy1RVzJieHFJZ2xia0ZUTHRZMnJOcUhMMEg0UkE5N2xCM2haM05RT3ZncjA1NVNMU3dHS3ZjamFnYnhKVUNR0gFmQVVfeXFMUFhmOVBrU1hyR1ktdXJxWDBBLU9iQURxVEZLN1NoVGVwUmV1eGpKMGs0ZjBhcUdSaFFnZVJVS2ltNGE3SmNmNFB6N1RONDVGYURnQXdvMnNNTEVTQ2huenBLc1V1YnFB?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-09-17T22:44:35+00:00</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>29742.5</v>
+      </c>
+      <c r="F108" t="n">
+        <v>29793.25</v>
+      </c>
+      <c r="G108" t="n">
+        <v>29674.5</v>
+      </c>
+      <c r="H108" t="n">
+        <v>29679.75</v>
+      </c>
+      <c r="I108" t="n">
+        <v>107991</v>
+      </c>
+      <c r="J108" t="n">
+        <v>4</v>
+      </c>
+      <c r="K108" t="n">
+        <v>38</v>
+      </c>
+      <c r="L108" t="n">
+        <v>-0.355</v>
+      </c>
+      <c r="M108" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="N108" t="n">
+        <v>37</v>
+      </c>
+      <c r="O108" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="P108" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>-4.201</v>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>US Stocks Rise as Fed Rate Hike Materializes, Nasdaq Gains 1.7%; Tech and Memory Stocks Lead AI-Related Gains; Micron Up 5% - TradingKey</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQaHR2eEdSdEhkb1hPYmNDOG5jOTJmWjBGeFRzZE1nOUFDVXBlX05iOVJ5VjJIS2lBbzJ3VzdaYi05Q3JXQXhBQ2NrTXhWazFaY1RKSHFzdVFrNnJxbkJjd0RjYTdLcDFTT2FxYWd1aUc2eFlfcVEzbWZ0NExpM3V1RU93ZDl3WlZ4eVYzQ3lraXhaX05rTFh3NWxuVVpGVTQySndBUnh2WDlmMDRQMnFiQldfZmNHMXJVSHlTN29BREo2THNPUmRpNlQtc2s4bG1ic2o0Rg?oc=5</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>S&amp;P and Nasdaq hit record highs, continuing remarkable recovery from war shock - CNN</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBFM0dLbkRoQTEzbmVyNGdlZERORGZXdEJrOVh3U0FZVnJsNk0zQjFWVVF6a0NhQThTbS0zMUJTdmdHWm1JYVF3LW5VUWVJWFk1MUd6WlVNWU9aa0dENG9rbkYzRDFpcmhSQ1BJ?oc=5</t>
+        </is>
+      </c>
+      <c r="W108" t="inlineStr">
+        <is>
+          <t>European stocks rise on tech gains ahead of Fed decision - aa.com.tr</t>
+        </is>
+      </c>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNM2V1cUpxYmtQVy1jWUQ3c2dxOVEwd1Q1NDNoVGhaYzh4QkFTbVZDYkZxUnVSb09hejE4RTFKM2lVekNLTEt5U0g4TjJXSkcyc2Y5T3R1M0QwNTdsa01OLVItMGhpdHJpOVRfc3RrVzBwVlo0WmRCdUlscjVjaENUeklXMTBUOW13cmZTYTFndkdqT0k0MF9QOQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z108" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA108" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 17: CoreWeave Falls on Convertible Debt and Share Sale Announcement - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="AB108" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxOZFBscEwwWGdXV1dvNTRVYWZabHNZdzJYM2ZYLWRHT25IMWREb0w2TEFBSjVrRG9jTnR3a2ZjWHI2UElPWS1XMEhqNFRGbGhRNG1uejNnWWtkRURZQTROUXk1TDVVS3hGTFgybEJlWkszaFpmWjlaRFBwLTVheGVWbmRhUXdVcjFwamI3Ui0zRFl1azZEeENvSU96cFFlVU1tSE5wYU1uR1g1cXEtV3FQMkhWS1l0S0lzLVFaMnNuZnhSZ1JLdGx5NmFvLXcwcVlsQTRtODNkNldIVk5sV3RRTWlZWWE3QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC108" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD108" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-09-17T22:44:35+00:00</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>76506.39840000001</v>
+      </c>
+      <c r="F109" t="n">
+        <v>76672.49219999999</v>
+      </c>
+      <c r="G109" t="n">
+        <v>76186.88280000001</v>
+      </c>
+      <c r="H109" t="n">
+        <v>76352</v>
+      </c>
+      <c r="I109" t="n">
+        <v>436015104</v>
+      </c>
+      <c r="J109" t="n">
+        <v>4</v>
+      </c>
+      <c r="K109" t="n">
+        <v>36</v>
+      </c>
+      <c r="L109" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M109" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="N109" t="n">
+        <v>35</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="P109" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>7.657</v>
+      </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - Fox Business</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="V109" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W109" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X109" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y109" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - Pulse 2.0</t>
+        </is>
+      </c>
+      <c r="Z109" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA109" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="AB109" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC109" t="inlineStr">
+        <is>
+          <t>Zcash jumps 17% amid $345M liquidations after F... - Pluang</t>
+        </is>
+      </c>
+      <c r="AD109" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxPNTZnb05wT2NfdkRGTmxpYjloR2xRRFNVQm1BLVdqdlFaVjNad0d1c3dELTVGLThEMllvV0FDa0FTUUZEekxYc2VPRzYta29nbkV4MF9FemVicmNzNG1DLTJZTnI4MUtnSngwN3hXdlJUMGpkSUt5T016dE9kaDRGaXlVR01XWUJLT0h6Yw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-18 03:38 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AD115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14067,6 +14067,762 @@
         </is>
       </c>
       <c r="AD109" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxPNTZnb05wT2NfdkRGTmxpYjloR2xRRFNVQm1BLVdqdlFaVjNad0d1c3dELTVGLThEMllvV0FDa0FTUUZEekxYc2VPRzYta29nbkV4MF9FemVicmNzNG1DLTJZTnI4MUtnSngwN3hXdlJUMGpkSUt5T016dE9kaDRGaXlVR01XWUJLT0h6Yw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:36:48+00:00</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>4384.3999</v>
+      </c>
+      <c r="F110" t="n">
+        <v>4404.6001</v>
+      </c>
+      <c r="G110" t="n">
+        <v>4372.2002</v>
+      </c>
+      <c r="H110" t="n">
+        <v>4377</v>
+      </c>
+      <c r="I110" t="n">
+        <v>15822</v>
+      </c>
+      <c r="J110" t="n">
+        <v>4</v>
+      </c>
+      <c r="K110" t="n">
+        <v>40</v>
+      </c>
+      <c r="L110" t="n">
+        <v>-0.118</v>
+      </c>
+      <c r="M110" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="N110" t="n">
+        <v>40</v>
+      </c>
+      <c r="O110" t="n">
+        <v>0.183</v>
+      </c>
+      <c r="P110" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>1.293</v>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>Copper Miners Capitalize on Tight Supply &amp; Growing Demand - ETF Trends</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQTHJDUGNNT3BEei1wbGJCVnd4X2JuX2Jsb1JtSGpLbHBFQnphd1JQSWR1MUxJdm1hMlprT19qc1o5WnVTeGg4WWlCaUg0X3BHVDlvUW9xamx3N3lJNmJKam8ya3hwQ25wbmlXcHJQT0lRRkxjakZYMVZUU1hKZUV3U0tqWlBKODlOYnBibUxtalpjd0FzWFJnME56azZLanR4ZkpOdWc5RWNhbjBaQ0pLS1Bndw?oc=5</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="V110" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W110" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="X110" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y110" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="Z110" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA110" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB110" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+      <c r="AC110" t="inlineStr">
+        <is>
+          <t>Gold ETFs Shine in H1 2026 with Unprecedented Liquidity - Investing News Network</t>
+        </is>
+      </c>
+      <c r="AD110" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE1JaGRkaHpGODN4bGpQdFl6S3VyUjZKYzRvWUxjUjhyQ0lVXzZMZEltdGkwMEo2d0lhVWVmMDVUYUJfRXF4emdyX0ZTd0N6SVgwN3kxMFVXTkt5WXZJbE8ybVNRLUJYTVZy?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:36:48+00:00</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>101.08</v>
+      </c>
+      <c r="F111" t="n">
+        <v>101.57</v>
+      </c>
+      <c r="G111" t="n">
+        <v>100.76</v>
+      </c>
+      <c r="H111" t="n">
+        <v>101.24</v>
+      </c>
+      <c r="I111" t="n">
+        <v>3714</v>
+      </c>
+      <c r="J111" t="n">
+        <v>4</v>
+      </c>
+      <c r="K111" t="n">
+        <v>40</v>
+      </c>
+      <c r="L111" t="n">
+        <v>-0.051</v>
+      </c>
+      <c r="M111" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="N111" t="n">
+        <v>40</v>
+      </c>
+      <c r="O111" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="P111" t="n">
+        <v>-0.094</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>1.234</v>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="V111" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W111" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X111" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y111" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z111" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE00VzJTYmxIdkNabVVzbnY3V2lyT0tMYkxJOTBOVEUxN0oydU5BYlB3T1FiUFd6MUdLcXpqb0l0WDdKRXZLbmdydlRwWERJbVV6RkdqNVQ0RDZqUHJoZEtia3lB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA111" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB111" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC111" t="inlineStr">
+        <is>
+          <t>OPEC oil output falls in August, Reuters survey shows - Reuters</t>
+        </is>
+      </c>
+      <c r="AD111" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcGZWQVVsSEY1MDZDLXRVM2g2N0t1bHJ1VXpWX3pScTFZak53OGQ5VVNxemw0Mjdrd1paNjRYb1YtdFlYN3RIOURKM00xZmc4eFRlTHk2cTNhODJKWW5TOS1BMEE1cVF2NTN5YjJaeHRRNFlBVHUwUU9CN0pyOEdRMHE0c2VtcGNvamRPVFd3OVVlTnFmV3Fobks2WlZJU21oRW44?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:36:48+00:00</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>100.255</v>
+      </c>
+      <c r="F112" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="G112" t="n">
+        <v>100.206</v>
+      </c>
+      <c r="H112" t="n">
+        <v>100.27</v>
+      </c>
+      <c r="I112" t="n">
+        <v>0</v>
+      </c>
+      <c r="J112" t="n">
+        <v>4</v>
+      </c>
+      <c r="K112" t="n">
+        <v>39</v>
+      </c>
+      <c r="L112" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="M112" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="N112" t="n">
+        <v>39</v>
+      </c>
+      <c r="O112" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="P112" t="n">
+        <v>-0.058</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>2.947</v>
+      </c>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>US dollar index hits its highest since May as war-driven oil rally boosts safe-haven demand - Anadolu Ajansı</t>
+        </is>
+      </c>
+      <c r="V112" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxOWkZKOWhZTF80bEh1ODhHd2s4dDM1Zm9sNTB6a25FME9HYy1UYkV5RllBdmJwTVJKUzMyMWRxVnJhRUt1eW9KSnQtNnR1SFUySEQ3eGtWaER0ZEtaVk84ZGM5REZmWmVrNklENFpKWldMNEtEN2JkbFpOSFZwb082NWxIWFgtTUNfdVg4RnZOMzVFd3F1VmFscUtleEg0MmN3RmcweldUOGpsRUxzMENSMVpOM1NUTGZkMTNHRm12UDRuRXdwcmdSeXQ1bGc?oc=5</t>
+        </is>
+      </c>
+      <c r="W112" t="inlineStr">
+        <is>
+          <t>United States Dollar Index rises as strong NFP revives Fed hike bets - Mitrade</t>
+        </is>
+      </c>
+      <c r="X112" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxOWnp0dmNKOUxXeUJubHNPYmNTUHdEOExRSy1rbzAzUHZiQ0RJSVZSbGZNWkh4ck9jSnVCU181cmVQQVFSUDRNeGJ3Z1NYenZrWHFFVE0wZDZpZmlIQlR3Y1hVNkRFS2EwVmVseGZyYnV5TkpvbnNZeXJ4T0g3OWlyY3Vjbw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y112" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z112" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA112" t="inlineStr">
+        <is>
+          <t>Gold climbs over 2% as US Dollar trims post-Fed gains - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB112" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPRG5KNUhGZkw4cUIzSmtOLV92bmhnbWE0a1NZMGJSNHdnUnluM05tT2hKSk44cFZFME52LWxETTlvUllCX2VkdHVNLTVlaXdaTURfWHBXY3J2U01BVXl1TDE0dWQyT1ZVV1VwR0RyZ2p0MTdUbmExY1dlNHJPS3EzaVN1MWpwSzVGR1dIYW56aTk1SnlLMnpFcFNpeW4xNVVZT19lcmZhV2JldHJwcTJn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC112" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD112" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:36:48+00:00</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>7700.75</v>
+      </c>
+      <c r="F113" t="n">
+        <v>7709.75</v>
+      </c>
+      <c r="G113" t="n">
+        <v>7696</v>
+      </c>
+      <c r="H113" t="n">
+        <v>7709.5</v>
+      </c>
+      <c r="I113" t="n">
+        <v>24565</v>
+      </c>
+      <c r="J113" t="n">
+        <v>4</v>
+      </c>
+      <c r="K113" t="n">
+        <v>40</v>
+      </c>
+      <c r="L113" t="n">
+        <v>-0.284</v>
+      </c>
+      <c r="M113" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="N113" t="n">
+        <v>40</v>
+      </c>
+      <c r="O113" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="P113" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 2: Dell Surges 16% on Soaring AI Backlog - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQWTRuSVIyTFR2RTZveHRTN3hEWnBwSDl4T2J4ZHZPT01OdEYzWUk3MXZJZjNIc0tTMGYtYmFIYnkxd1dfVVVKTks0MmhzTlc5Z014VHVMMHJVMmZkWWlYVXdHWlczYWRQNzRyYk5leV9ncFBQVE1CbVdTbGNxclNhTy1JNEQwSlVmNjhjOGZrQXBLZlFG?oc=5</t>
+        </is>
+      </c>
+      <c r="W113" t="inlineStr">
+        <is>
+          <t>SNDK Stock Breaks Resistance as NAND Demand Strengthens SanDisk but Memory Risks Remain - FXLeaders</t>
+        </is>
+      </c>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPVXFEeDQxXy1zUk5CSzNOMzNlLWx2QkRBYUhxUV9ObV9naWxTdS1GZXNmSXNaRG1XUmFZbldRMWliWVpQNmtjV2ZaTXJ0VlpGZDhlQTU0M1F1RUtmMEFwQ3pkNXRxYkJ6UjZVNE0tYWtLMlh4bkpqVWxMUXRveE82c1VyR3FXUlZ5SWZRQVc5YUN6SWhteGtNUjBPdUx1NG0tUUFIN0RMcHFRSUVsMHVxUnVFRS1CWVlBVEx3cUVhcDRqaTB3SkZBdC1B?oc=5</t>
+        </is>
+      </c>
+      <c r="Y113" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - proactiveinvestors.com</t>
+        </is>
+      </c>
+      <c r="Z113" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA113" t="inlineStr">
+        <is>
+          <t>SPIE stock breaks through its support at €43.10 and falls 2.5% - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB113" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQRVVnaWZ4MlBIbFVrUmo3Z0pCb0VMOTB5LWlYQ25zLU54UmVjMFJEUWptX1FyOEZsbGY5Z1dNSUxqbUxVMFAxcjRZSDMzek5WcjctempiZThIdEtmTm8waVN0bFZuVlVUS044MUhPNXp6b1pBcTlqM1QtQThGMVJLUGYtVGpmdmdKeDNDQWFTenJXeng1OUxCVy1nODRCM0drWkpiaXNZZzRFYjBza2RxMkFJUlZ0U2F0dlVZTEVXQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC113" t="inlineStr">
+        <is>
+          <t>Wall Street Drops as Fed Chair Kevin Warsh Delivers Hawkish Remarks - news.sbs.co.kr</t>
+        </is>
+      </c>
+      <c r="AD113" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE1LOHlueWljVGhtM3ZlS0JMQlNaMWFmMGp0bFZFVkZZbXZNb0Nsb1RFYy1RVzJieHFJZ2xia0ZUTHRZMnJOcUhMMEg0UkE5N2xCM2haM05RT3ZncjA1NVNMU3dHS3ZjamFnYnhKVUNR0gFmQVVfeXFMUFhmOVBrU1hyR1ktdXJxWDBBLU9iQURxVEZLN1NoVGVwUmV1eGpKMGs0ZjBhcUdSaFFnZVJVS2ltNGE3SmNmNFB6N1RONDVGYURnQXdvMnNNTEVTQ2huenBLc1V1YnFB?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:36:48+00:00</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>29697.25</v>
+      </c>
+      <c r="F114" t="n">
+        <v>29738.5</v>
+      </c>
+      <c r="G114" t="n">
+        <v>29648</v>
+      </c>
+      <c r="H114" t="n">
+        <v>29736.5</v>
+      </c>
+      <c r="I114" t="n">
+        <v>20749</v>
+      </c>
+      <c r="J114" t="n">
+        <v>4</v>
+      </c>
+      <c r="K114" t="n">
+        <v>37</v>
+      </c>
+      <c r="L114" t="n">
+        <v>-0.394</v>
+      </c>
+      <c r="M114" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="N114" t="n">
+        <v>37</v>
+      </c>
+      <c r="O114" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="P114" t="n">
+        <v>-0.011</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>-5.06</v>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>Samsung Electronics, SK hynix surge as U.S. tech stocks rally - 매일경제</t>
+        </is>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE1iMG1NRW5Wa0RYWEU1Y19TOGhPck9LTHozNTdYM043RHFYWlJsZzEtQVAzYTNkbHNhRE1rNEVIMUx5N29idV93bkc3cEo4ZExsLVE?oc=5</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>US Stocks Rise as Fed Rate Hike Materializes, Nasdaq Gains 1.7%; Tech and Memory Stocks Lead AI-Related Gains; Micron Up 5% - TradingKey</t>
+        </is>
+      </c>
+      <c r="V114" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQaHR2eEdSdEhkb1hPYmNDOG5jOTJmWjBGeFRzZE1nOUFDVXBlX05iOVJ5VjJIS2lBbzJ3VzdaYi05Q3JXQXhBQ2NrTXhWazFaY1RKSHFzdVFrNnJxbkJjd0RjYTdLcDFTT2FxYWd1aUc2eFlfcVEzbWZ0NExpM3V1RU93ZDl3WlZ4eVYzQ3lraXhaX05rTFh3NWxuVVpGVTQySndBUnh2WDlmMDRQMnFiQldfZmNHMXJVSHlTN29BREo2THNPUmRpNlQtc2s4bG1ic2o0Rg?oc=5</t>
+        </is>
+      </c>
+      <c r="W114" t="inlineStr">
+        <is>
+          <t>S&amp;P and Nasdaq hit record highs, continuing remarkable recovery from war shock - CNN</t>
+        </is>
+      </c>
+      <c r="X114" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBFM0dLbkRoQTEzbmVyNGdlZERORGZXdEJrOVh3U0FZVnJsNk0zQjFWVVF6a0NhQThTbS0zMUJTdmdHWm1JYVF3LW5VUWVJWFk1MUd6WlVNWU9aa0dENG9rbkYzRDFpcmhSQ1BJ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y114" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z114" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA114" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 17: CoreWeave Falls on Convertible Debt and Share Sale Announcement - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="AB114" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxOZFBscEwwWGdXV1dvNTRVYWZabHNZdzJYM2ZYLWRHT25IMWREb0w2TEFBSjVrRG9jTnR3a2ZjWHI2UElPWS1XMEhqNFRGbGhRNG1uejNnWWtkRURZQTROUXk1TDVVS3hGTFgybEJlWkszaFpmWjlaRFBwLTVheGVWbmRhUXdVcjFwamI3Ui0zRFl1azZEeENvSU96cFFlVU1tSE5wYU1uR1g1cXEtV3FQMkhWS1l0S0lzLVFaMnNuZnhSZ1JLdGx5NmFvLXcwcVlsQTRtODNkNldIVk5sV3RRTWlZWWE3QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC114" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - proactiveinvestors.com</t>
+        </is>
+      </c>
+      <c r="AD114" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:36:48+00:00</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>76342.5</v>
+      </c>
+      <c r="F115" t="n">
+        <v>77516.72659999999</v>
+      </c>
+      <c r="G115" t="n">
+        <v>76217.1094</v>
+      </c>
+      <c r="H115" t="n">
+        <v>77298.22659999999</v>
+      </c>
+      <c r="I115" t="n">
+        <v>2060034048</v>
+      </c>
+      <c r="J115" t="n">
+        <v>4</v>
+      </c>
+      <c r="K115" t="n">
+        <v>37</v>
+      </c>
+      <c r="L115" t="n">
+        <v>-0.017</v>
+      </c>
+      <c r="M115" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="N115" t="n">
+        <v>35</v>
+      </c>
+      <c r="O115" t="n">
+        <v>0.404</v>
+      </c>
+      <c r="P115" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>7.752</v>
+      </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to three-month high as momentum builds - foxbusiness.com</t>
+        </is>
+      </c>
+      <c r="V115" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9GWnpPTVdhalZlX29PZmhxWWFzRlEwbGQ2Q2VuUm1ISTRKY2EwOUdEb3drMU9LdE16NXhRdGwyakxPOWdSR2ZKS0NoWUJzNGZZVVA5dnRlb01WRHM?oc=5</t>
+        </is>
+      </c>
+      <c r="W115" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X115" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y115" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - Pulse 2.0</t>
+        </is>
+      </c>
+      <c r="Z115" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA115" t="inlineStr">
+        <is>
+          <t>Bitcoin, Ether rebound as short liquidations hit $427 million - qz.com</t>
+        </is>
+      </c>
+      <c r="AB115" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBwS21sQ0RlNWhYREVhTjVEdGhnekF0SVVIZ3V3VUxoSXMtS0t6dUlDMGVYenpPeTZEM1ItdDhNZGdNLWlQa2pvQXhYcXVfNjRPOFNLYXFiYS1PY2ZreHVMajRQUHhSNlJ2UUVIcmktOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC115" t="inlineStr">
+        <is>
+          <t>Zcash jumps 17% amid $345M liquidations after F... - Pluang</t>
+        </is>
+      </c>
+      <c r="AD115" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxPNTZnb05wT2NfdkRGTmxpYjloR2xRRFNVQm1BLVdqdlFaVjNad0d1c3dELTVGLThEMllvV0FDa0FTUUZEekxYc2VPRzYta29nbkV4MF9FemVicmNzNG1DLTJZTnI4MUtnSngwN3hXdlJUMGpkSUt5T016dE9kaDRGaXlVR01XWUJLT0h6Yw?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-18 09:00 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD115"/>
+  <dimension ref="A1:AD121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14827,6 +14827,474 @@
           <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxPNTZnb05wT2NfdkRGTmxpYjloR2xRRFNVQm1BLVdqdlFaVjNad0d1c3dELTVGLThEMllvV0FDa0FTUUZEekxYc2VPRzYta29nbkV4MF9FemVicmNzNG1DLTJZTnI4MUtnSngwN3hXdlJUMGpkSUt5T016dE9kaDRGaXlVR01XWUJLT0h6Yw?oc=5</t>
         </is>
       </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-09-18T08:52:29+00:00</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>4406.7002</v>
+      </c>
+      <c r="F116" t="n">
+        <v>4439.7998</v>
+      </c>
+      <c r="G116" t="n">
+        <v>4399.7998</v>
+      </c>
+      <c r="H116" t="n">
+        <v>4425.1001</v>
+      </c>
+      <c r="I116" t="n">
+        <v>22836</v>
+      </c>
+      <c r="J116" t="n">
+        <v>4</v>
+      </c>
+      <c r="K116" t="n">
+        <v>0</v>
+      </c>
+      <c r="L116" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" t="n">
+        <v>0</v>
+      </c>
+      <c r="N116" t="n">
+        <v>0</v>
+      </c>
+      <c r="O116" t="n">
+        <v>0</v>
+      </c>
+      <c r="P116" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q116" t="n">
+        <v>0</v>
+      </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S116" t="inlineStr"/>
+      <c r="T116" t="inlineStr"/>
+      <c r="U116" t="inlineStr"/>
+      <c r="V116" t="inlineStr"/>
+      <c r="W116" t="inlineStr"/>
+      <c r="X116" t="inlineStr"/>
+      <c r="Y116" t="inlineStr"/>
+      <c r="Z116" t="inlineStr"/>
+      <c r="AA116" t="inlineStr"/>
+      <c r="AB116" t="inlineStr"/>
+      <c r="AC116" t="inlineStr"/>
+      <c r="AD116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-09-18T08:52:29+00:00</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>101</v>
+      </c>
+      <c r="F117" t="n">
+        <v>101.18</v>
+      </c>
+      <c r="G117" t="n">
+        <v>94.83</v>
+      </c>
+      <c r="H117" t="n">
+        <v>95.58</v>
+      </c>
+      <c r="I117" t="n">
+        <v>46272</v>
+      </c>
+      <c r="J117" t="n">
+        <v>4</v>
+      </c>
+      <c r="K117" t="n">
+        <v>0</v>
+      </c>
+      <c r="L117" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" t="n">
+        <v>0</v>
+      </c>
+      <c r="N117" t="n">
+        <v>0</v>
+      </c>
+      <c r="O117" t="n">
+        <v>0</v>
+      </c>
+      <c r="P117" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>0</v>
+      </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S117" t="inlineStr"/>
+      <c r="T117" t="inlineStr"/>
+      <c r="U117" t="inlineStr"/>
+      <c r="V117" t="inlineStr"/>
+      <c r="W117" t="inlineStr"/>
+      <c r="X117" t="inlineStr"/>
+      <c r="Y117" t="inlineStr"/>
+      <c r="Z117" t="inlineStr"/>
+      <c r="AA117" t="inlineStr"/>
+      <c r="AB117" t="inlineStr"/>
+      <c r="AC117" t="inlineStr"/>
+      <c r="AD117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-09-18T08:52:29+00:00</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>100.248</v>
+      </c>
+      <c r="F118" t="n">
+        <v>100.382</v>
+      </c>
+      <c r="G118" t="n">
+        <v>100.217</v>
+      </c>
+      <c r="H118" t="n">
+        <v>100.376</v>
+      </c>
+      <c r="I118" t="n">
+        <v>0</v>
+      </c>
+      <c r="J118" t="n">
+        <v>4</v>
+      </c>
+      <c r="K118" t="n">
+        <v>0</v>
+      </c>
+      <c r="L118" t="n">
+        <v>0</v>
+      </c>
+      <c r="M118" t="n">
+        <v>0</v>
+      </c>
+      <c r="N118" t="n">
+        <v>0</v>
+      </c>
+      <c r="O118" t="n">
+        <v>0</v>
+      </c>
+      <c r="P118" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q118" t="n">
+        <v>0</v>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S118" t="inlineStr"/>
+      <c r="T118" t="inlineStr"/>
+      <c r="U118" t="inlineStr"/>
+      <c r="V118" t="inlineStr"/>
+      <c r="W118" t="inlineStr"/>
+      <c r="X118" t="inlineStr"/>
+      <c r="Y118" t="inlineStr"/>
+      <c r="Z118" t="inlineStr"/>
+      <c r="AA118" t="inlineStr"/>
+      <c r="AB118" t="inlineStr"/>
+      <c r="AC118" t="inlineStr"/>
+      <c r="AD118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-09-18T08:52:29+00:00</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>7721.5</v>
+      </c>
+      <c r="F119" t="n">
+        <v>7739.25</v>
+      </c>
+      <c r="G119" t="n">
+        <v>7721.25</v>
+      </c>
+      <c r="H119" t="n">
+        <v>7728.75</v>
+      </c>
+      <c r="I119" t="n">
+        <v>52790</v>
+      </c>
+      <c r="J119" t="n">
+        <v>4</v>
+      </c>
+      <c r="K119" t="n">
+        <v>0</v>
+      </c>
+      <c r="L119" t="n">
+        <v>0</v>
+      </c>
+      <c r="M119" t="n">
+        <v>0</v>
+      </c>
+      <c r="N119" t="n">
+        <v>0</v>
+      </c>
+      <c r="O119" t="n">
+        <v>0</v>
+      </c>
+      <c r="P119" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q119" t="n">
+        <v>0</v>
+      </c>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S119" t="inlineStr"/>
+      <c r="T119" t="inlineStr"/>
+      <c r="U119" t="inlineStr"/>
+      <c r="V119" t="inlineStr"/>
+      <c r="W119" t="inlineStr"/>
+      <c r="X119" t="inlineStr"/>
+      <c r="Y119" t="inlineStr"/>
+      <c r="Z119" t="inlineStr"/>
+      <c r="AA119" t="inlineStr"/>
+      <c r="AB119" t="inlineStr"/>
+      <c r="AC119" t="inlineStr"/>
+      <c r="AD119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-09-18T08:52:29+00:00</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>29810.25</v>
+      </c>
+      <c r="F120" t="n">
+        <v>29966.75</v>
+      </c>
+      <c r="G120" t="n">
+        <v>29803</v>
+      </c>
+      <c r="H120" t="n">
+        <v>29911.5</v>
+      </c>
+      <c r="I120" t="n">
+        <v>36051</v>
+      </c>
+      <c r="J120" t="n">
+        <v>4</v>
+      </c>
+      <c r="K120" t="n">
+        <v>0</v>
+      </c>
+      <c r="L120" t="n">
+        <v>0</v>
+      </c>
+      <c r="M120" t="n">
+        <v>0</v>
+      </c>
+      <c r="N120" t="n">
+        <v>0</v>
+      </c>
+      <c r="O120" t="n">
+        <v>0</v>
+      </c>
+      <c r="P120" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>0</v>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr"/>
+      <c r="T120" t="inlineStr"/>
+      <c r="U120" t="inlineStr"/>
+      <c r="V120" t="inlineStr"/>
+      <c r="W120" t="inlineStr"/>
+      <c r="X120" t="inlineStr"/>
+      <c r="Y120" t="inlineStr"/>
+      <c r="Z120" t="inlineStr"/>
+      <c r="AA120" t="inlineStr"/>
+      <c r="AB120" t="inlineStr"/>
+      <c r="AC120" t="inlineStr"/>
+      <c r="AD120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-09-18T08:52:29+00:00</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>77433.9688</v>
+      </c>
+      <c r="F121" t="n">
+        <v>78200</v>
+      </c>
+      <c r="G121" t="n">
+        <v>77332.07030000001</v>
+      </c>
+      <c r="H121" t="n">
+        <v>78178.3125</v>
+      </c>
+      <c r="I121" t="n">
+        <v>3334350848</v>
+      </c>
+      <c r="J121" t="n">
+        <v>4</v>
+      </c>
+      <c r="K121" t="n">
+        <v>0</v>
+      </c>
+      <c r="L121" t="n">
+        <v>0</v>
+      </c>
+      <c r="M121" t="n">
+        <v>0</v>
+      </c>
+      <c r="N121" t="n">
+        <v>0</v>
+      </c>
+      <c r="O121" t="n">
+        <v>0</v>
+      </c>
+      <c r="P121" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q121" t="n">
+        <v>0</v>
+      </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr"/>
+      <c r="T121" t="inlineStr"/>
+      <c r="U121" t="inlineStr"/>
+      <c r="V121" t="inlineStr"/>
+      <c r="W121" t="inlineStr"/>
+      <c r="X121" t="inlineStr"/>
+      <c r="Y121" t="inlineStr"/>
+      <c r="Z121" t="inlineStr"/>
+      <c r="AA121" t="inlineStr"/>
+      <c r="AB121" t="inlineStr"/>
+      <c r="AC121" t="inlineStr"/>
+      <c r="AD121" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Scan: 2026-09-18 16:01 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD121"/>
+  <dimension ref="A1:AD127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14893,18 +14893,6 @@
           <t>finbert</t>
         </is>
       </c>
-      <c r="S116" t="inlineStr"/>
-      <c r="T116" t="inlineStr"/>
-      <c r="U116" t="inlineStr"/>
-      <c r="V116" t="inlineStr"/>
-      <c r="W116" t="inlineStr"/>
-      <c r="X116" t="inlineStr"/>
-      <c r="Y116" t="inlineStr"/>
-      <c r="Z116" t="inlineStr"/>
-      <c r="AA116" t="inlineStr"/>
-      <c r="AB116" t="inlineStr"/>
-      <c r="AC116" t="inlineStr"/>
-      <c r="AD116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -14971,18 +14959,6 @@
           <t>finbert</t>
         </is>
       </c>
-      <c r="S117" t="inlineStr"/>
-      <c r="T117" t="inlineStr"/>
-      <c r="U117" t="inlineStr"/>
-      <c r="V117" t="inlineStr"/>
-      <c r="W117" t="inlineStr"/>
-      <c r="X117" t="inlineStr"/>
-      <c r="Y117" t="inlineStr"/>
-      <c r="Z117" t="inlineStr"/>
-      <c r="AA117" t="inlineStr"/>
-      <c r="AB117" t="inlineStr"/>
-      <c r="AC117" t="inlineStr"/>
-      <c r="AD117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -15049,18 +15025,6 @@
           <t>finbert</t>
         </is>
       </c>
-      <c r="S118" t="inlineStr"/>
-      <c r="T118" t="inlineStr"/>
-      <c r="U118" t="inlineStr"/>
-      <c r="V118" t="inlineStr"/>
-      <c r="W118" t="inlineStr"/>
-      <c r="X118" t="inlineStr"/>
-      <c r="Y118" t="inlineStr"/>
-      <c r="Z118" t="inlineStr"/>
-      <c r="AA118" t="inlineStr"/>
-      <c r="AB118" t="inlineStr"/>
-      <c r="AC118" t="inlineStr"/>
-      <c r="AD118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -15127,18 +15091,6 @@
           <t>finbert</t>
         </is>
       </c>
-      <c r="S119" t="inlineStr"/>
-      <c r="T119" t="inlineStr"/>
-      <c r="U119" t="inlineStr"/>
-      <c r="V119" t="inlineStr"/>
-      <c r="W119" t="inlineStr"/>
-      <c r="X119" t="inlineStr"/>
-      <c r="Y119" t="inlineStr"/>
-      <c r="Z119" t="inlineStr"/>
-      <c r="AA119" t="inlineStr"/>
-      <c r="AB119" t="inlineStr"/>
-      <c r="AC119" t="inlineStr"/>
-      <c r="AD119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -15205,18 +15157,6 @@
           <t>finbert</t>
         </is>
       </c>
-      <c r="S120" t="inlineStr"/>
-      <c r="T120" t="inlineStr"/>
-      <c r="U120" t="inlineStr"/>
-      <c r="V120" t="inlineStr"/>
-      <c r="W120" t="inlineStr"/>
-      <c r="X120" t="inlineStr"/>
-      <c r="Y120" t="inlineStr"/>
-      <c r="Z120" t="inlineStr"/>
-      <c r="AA120" t="inlineStr"/>
-      <c r="AB120" t="inlineStr"/>
-      <c r="AC120" t="inlineStr"/>
-      <c r="AD120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -15283,18 +15223,762 @@
           <t>finbert</t>
         </is>
       </c>
-      <c r="S121" t="inlineStr"/>
-      <c r="T121" t="inlineStr"/>
-      <c r="U121" t="inlineStr"/>
-      <c r="V121" t="inlineStr"/>
-      <c r="W121" t="inlineStr"/>
-      <c r="X121" t="inlineStr"/>
-      <c r="Y121" t="inlineStr"/>
-      <c r="Z121" t="inlineStr"/>
-      <c r="AA121" t="inlineStr"/>
-      <c r="AB121" t="inlineStr"/>
-      <c r="AC121" t="inlineStr"/>
-      <c r="AD121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-09-18T16:00:11+00:00</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>4420.8999</v>
+      </c>
+      <c r="F122" t="n">
+        <v>4421.8999</v>
+      </c>
+      <c r="G122" t="n">
+        <v>4381</v>
+      </c>
+      <c r="H122" t="n">
+        <v>4393.7002</v>
+      </c>
+      <c r="I122" t="n">
+        <v>41030</v>
+      </c>
+      <c r="J122" t="n">
+        <v>4</v>
+      </c>
+      <c r="K122" t="n">
+        <v>40</v>
+      </c>
+      <c r="L122" t="n">
+        <v>-0.161</v>
+      </c>
+      <c r="M122" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="N122" t="n">
+        <v>40</v>
+      </c>
+      <c r="O122" t="n">
+        <v>0.151</v>
+      </c>
+      <c r="P122" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="Q122" t="n">
+        <v>-0.197</v>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>Have Fed Rate Hike Headwinds Been Priced In? Gold Rebounds Strongly Toward $4,400, Poised for a New Rally - TradingKey</t>
+        </is>
+      </c>
+      <c r="V122" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxQaXdWX09aV29LZzBDaVo5dTNDbG8wbGR6bGZnMk05cGp6SGdEVTZOazc4d0gtYUU5WXZnaGIzV3MwMFNnbm1sTEswRnBNRzQwWk1MZi1ob0pRYXY1MEJBMGdVQ0NKYTFXSkJqamZDRjhtLVRTQ2ZmalJKckQyX3pGWGhDVzRlcWpiQjkxTDBXYlZheGdRT2JMb2ZUX1ZVNW5Oakhhd2N0Znc3ZDcxOVJVSlY5cFI1UGt5VF9FZ3FhLUlSUFFP?oc=5</t>
+        </is>
+      </c>
+      <c r="W122" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="X122" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="Y122" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="Z122" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA122" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB122" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC122" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD122" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-09-18T16:00:11+00:00</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>96.22</v>
+      </c>
+      <c r="F123" t="n">
+        <v>98.01000000000001</v>
+      </c>
+      <c r="G123" t="n">
+        <v>95.65000000000001</v>
+      </c>
+      <c r="H123" t="n">
+        <v>97.06999999999999</v>
+      </c>
+      <c r="I123" t="n">
+        <v>108346</v>
+      </c>
+      <c r="J123" t="n">
+        <v>4</v>
+      </c>
+      <c r="K123" t="n">
+        <v>39</v>
+      </c>
+      <c r="L123" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="M123" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="N123" t="n">
+        <v>40</v>
+      </c>
+      <c r="O123" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="P123" t="n">
+        <v>-0.08400000000000001</v>
+      </c>
+      <c r="Q123" t="n">
+        <v>3.409</v>
+      </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="V123" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="W123" t="inlineStr">
+        <is>
+          <t>Crude Oil &amp; Gold Forecast: Key Levels to Watch - FOREX.com</t>
+        </is>
+      </c>
+      <c r="X123" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPWTB1cHRpdk5MalktTnBqZV91SUZjNDZDRV9Fc0tLZ2ZCUFVqSmk0d21BYTk3SnBHVVJsQ0tyVGwyQnVhd1lrNFEzV2M3Vk5jbC15aVlVM1Zyd0QtVWlCR2ktZ19UNDdRSDFwQlNtdV9PTk5sa1pfTzFhSTJQZ1pXVVFud3VrcVhGR2JWLURfZ19VS3NFQ1RVTlFR?oc=5</t>
+        </is>
+      </c>
+      <c r="Y123" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z123" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA123" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB123" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC123" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD123" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-09-18T16:00:11+00:00</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>100.505</v>
+      </c>
+      <c r="F124" t="n">
+        <v>100.564</v>
+      </c>
+      <c r="G124" t="n">
+        <v>100.248</v>
+      </c>
+      <c r="H124" t="n">
+        <v>100.397</v>
+      </c>
+      <c r="I124" t="n">
+        <v>0</v>
+      </c>
+      <c r="J124" t="n">
+        <v>4</v>
+      </c>
+      <c r="K124" t="n">
+        <v>39</v>
+      </c>
+      <c r="L124" t="n">
+        <v>0.149</v>
+      </c>
+      <c r="M124" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="N124" t="n">
+        <v>39</v>
+      </c>
+      <c r="O124" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="P124" t="n">
+        <v>-0.064</v>
+      </c>
+      <c r="Q124" t="n">
+        <v>4.811</v>
+      </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>US dollar index hits its highest since May as war-driven oil rally boosts safe-haven demand - Anadolu Ajansı</t>
+        </is>
+      </c>
+      <c r="V124" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxOWkZKOWhZTF80bEh1ODhHd2s4dDM1Zm9sNTB6a25FME9HYy1UYkV5RllBdmJwTVJKUzMyMWRxVnJhRUt1eW9KSnQtNnR1SFUySEQ3eGtWaER0ZEtaVk84ZGM5REZmWmVrNklENFpKWldMNEtEN2JkbFpOSFZwb082NWxIWFgtTUNfdVg4RnZOMzVFd3F1VmFscUtleEg0MmN3RmcweldUOGpsRUxzMENSMVpOM1NUTGZkMTNHRm12UDRuRXdwcmdSeXQ1bGc?oc=5</t>
+        </is>
+      </c>
+      <c r="W124" t="inlineStr">
+        <is>
+          <t>United States Dollar Index rises as strong NFP revives Fed hike bets - Mitrade</t>
+        </is>
+      </c>
+      <c r="X124" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxOWnp0dmNKOUxXeUJubHNPYmNTUHdEOExRSy1rbzAzUHZiQ0RJSVZSbGZNWkh4ck9jSnVCU181cmVQQVFSUDRNeGJ3Z1NYenZrWHFFVE0wZDZpZmlIQlR3Y1hVNkRFS2EwVmVseGZyYnV5TkpvbnNZeXJ4T0g3OWlyY3Vjbw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y124" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z124" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA124" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AB124" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC124" t="inlineStr">
+        <is>
+          <t>Dollar rebounds from losses sparked by Treasury buyback plan - Reuters</t>
+        </is>
+      </c>
+      <c r="AD124" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPamFxZlBhRm1DcmRBZF9VSDd4aXllSmNTWEttZ2dLUkprSnJ5c2xBNXRKT1lQTDdrbXlUUjBnTXdWdVRrWENPYkRkal9pbm9UVDNueFd0am56Z3JCakxsZ2ZHclBRMHpyUUMzeVJHV1FPcVp1dXBYNUtMNk81Z3k1QkRmV1RnRHdPVjhDU3hNYS1xaWxYOU4wMUQwWk5nTDJPWG9kblZIQV9xOG11QTJR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-09-18T16:00:11+00:00</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>7712.25</v>
+      </c>
+      <c r="F125" t="n">
+        <v>7715</v>
+      </c>
+      <c r="G125" t="n">
+        <v>7683.25</v>
+      </c>
+      <c r="H125" t="n">
+        <v>7688.25</v>
+      </c>
+      <c r="I125" t="n">
+        <v>524314</v>
+      </c>
+      <c r="J125" t="n">
+        <v>4</v>
+      </c>
+      <c r="K125" t="n">
+        <v>40</v>
+      </c>
+      <c r="L125" t="n">
+        <v>-0.143</v>
+      </c>
+      <c r="M125" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="N125" t="n">
+        <v>40</v>
+      </c>
+      <c r="O125" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="P125" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="Q125" t="n">
+        <v>3.898</v>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 2: Dell Surges 16% on Soaring AI Backlog - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="V125" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQWTRuSVIyTFR2RTZveHRTN3hEWnBwSDl4T2J4ZHZPT01OdEYzWUk3MXZJZjNIc0tTMGYtYmFIYnkxd1dfVVVKTks0MmhzTlc5Z014VHVMMHJVMmZkWWlYVXdHWlczYWRQNzRyYk5leV9ncFBQVE1CbVdTbGNxclNhTy1JNEQwSlVmNjhjOGZrQXBLZlFG?oc=5</t>
+        </is>
+      </c>
+      <c r="W125" t="inlineStr">
+        <is>
+          <t>OSR Holdings (OSRH) Surges 15%: Small-Cap Stock Breaks Resistance, Eyes $0.50 Level - Dividend ETF - CarePlus VietNam</t>
+        </is>
+      </c>
+      <c r="X125" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPeU1GWGNLRllfbnJweWwzWDBwZnZTOGphUXlMOVFLMFcwc0RqUGJXVGFxcmx1Mkdwa25XanZ5ZGVRbDczQkd2bzZRX3k3UXRuZlFkYWp0dzVacWkzbzQtaG9adEhDWi00cGx0eXlGc2Z4Q0I4UUZqR1czN2ltaHc3MkdsRnBuY1pLRXR6UjlaMHRpSHctSXVtVDJxZkVwekxNbUhKd3lIaVpmeUNxU3NLRnYwM0pJdE9BU2cxdmxB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y125" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="Z125" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA125" t="inlineStr">
+        <is>
+          <t>LVMH stock breaks through 406 € support and falls 20% over three months - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB125" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOZ0owTDAydXBkUDIwMkFqd3ZrRVBqYVhRR21nWUxtXzg5OXVFZUt6WkRPdWdmak4tZE02WGxvdGR3MjdodnhHU2xiZXVqcmxiMndSbkUwSFdfZnFKcHBFVHZicDdSVHBDcTQ3c2trOE8xRlBfbklBZHlHa1F4dTJFWEdtYzQwQVloRGNPa1lFZ3kybS1UX1VFdnoteE11eUJkcjc1LWpCYmV4LTk4Z29XaWFLRHdobFg4UUNxMmg3bkptaUZJYUd4X25YQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC125" t="inlineStr">
+        <is>
+          <t>Wall Street Drops as Fed Chair Kevin Warsh Delivers Hawkish Remarks - news.sbs.co.kr</t>
+        </is>
+      </c>
+      <c r="AD125" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE1LOHlueWljVGhtM3ZlS0JMQlNaMWFmMGp0bFZFVkZZbXZNb0Nsb1RFYy1RVzJieHFJZ2xia0ZUTHRZMnJOcUhMMEg0UkE5N2xCM2haM05RT3ZncjA1NVNMU3dHS3ZjamFnYnhKVUNR0gFmQVVfeXFMUFhmOVBrU1hyR1ktdXJxWDBBLU9iQURxVEZLN1NoVGVwUmV1eGpKMGs0ZjBhcUdSaFFnZVJVS2ltNGE3SmNmNFB6N1RONDVGYURnQXdvMnNNTEVTQ2huenBLc1V1YnFB?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-09-18T16:00:11+00:00</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>29839.75</v>
+      </c>
+      <c r="F126" t="n">
+        <v>29853.5</v>
+      </c>
+      <c r="G126" t="n">
+        <v>29692.75</v>
+      </c>
+      <c r="H126" t="n">
+        <v>29723.5</v>
+      </c>
+      <c r="I126" t="n">
+        <v>205649</v>
+      </c>
+      <c r="J126" t="n">
+        <v>4</v>
+      </c>
+      <c r="K126" t="n">
+        <v>38</v>
+      </c>
+      <c r="L126" t="n">
+        <v>-0.313</v>
+      </c>
+      <c r="M126" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="N126" t="n">
+        <v>38</v>
+      </c>
+      <c r="O126" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="P126" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="Q126" t="n">
+        <v>-2.052</v>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>German Medical Cannabis Sales Boost High Tide To Record Performance (NASDAQ:HITI) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPWk4xOHF4YTkxMlliTXAyRDl4bERlWU1ZcFR5ZDYyR1BvYnZUdXNrNXNxX0lVMVBPR0JVbk4wVUhLUDNzbDlrdndfRzRLUlZrWUY4aVVlZ0tneUtFRjF3M2ZnME96RVc3b3VrLWdKQWpDNFp6RmQtSHZLOXlNZzNqTHpQWDByV2JRM3JQcXI4QVBIdVA3enRnMWkzMUtfR29rZUNpcGRsXzZzXzZY?oc=5</t>
+        </is>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>Samsung Electronics, SK hynix surge as U.S. tech stocks rally - 매일경제</t>
+        </is>
+      </c>
+      <c r="V126" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE55T0VWYmJHT1k0U1U3bldzSXpxTFNoNUVobHNVSHpjVmFhTGQzQUR3b0VDWkpvYlpHR0tFOWM2WXREa2U5NzQwbzE5TVFYT1BrSERZRjFhQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W126" t="inlineStr">
+        <is>
+          <t>US Stocks Rise as Fed Rate Hike Materializes, Nasdaq Gains 1.7%; Tech and Memory Stocks Lead AI-Related Gains; Micron Up 5% - TradingKey</t>
+        </is>
+      </c>
+      <c r="X126" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQaHR2eEdSdEhkb1hPYmNDOG5jOTJmWjBGeFRzZE1nOUFDVXBlX05iOVJ5VjJIS2lBbzJ3VzdaYi05Q3JXQXhBQ2NrTXhWazFaY1RKSHFzdVFrNnJxbkJjd0RjYTdLcDFTT2FxYWd1aUc2eFlfcVEzbWZ0NExpM3V1RU93ZDl3WlZ4eVYzQ3lraXhaX05rTFh3NWxuVVpGVTQySndBUnh2WDlmMDRQMnFiQldfZmNHMXJVSHlTN29BREo2THNPUmRpNlQtc2s4bG1ic2o0Rg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y126" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z126" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA126" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="AB126" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC126" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 17: CoreWeave Falls on Convertible Debt and Share Sale Announcement - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="AD126" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxOZFBscEwwWGdXV1dvNTRVYWZabHNZdzJYM2ZYLWRHT25IMWREb0w2TEFBSjVrRG9jTnR3a2ZjWHI2UElPWS1XMEhqNFRGbGhRNG1uejNnWWtkRURZQTROUXk1TDVVS3hGTFgybEJlWkszaFpmWjlaRFBwLTVheGVWbmRhUXdVcjFwamI3Ui0zRFl1azZEeENvSU96cFFlVU1tSE5wYU1uR1g1cXEtV3FQMkhWS1l0S0lzLVFaMnNuZnhSZ1JLdGx5NmFvLXcwcVlsQTRtODNkNldIVk5sV3RRTWlZWWE3QQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-09-18T16:00:11+00:00</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>77966.9688</v>
+      </c>
+      <c r="F127" t="n">
+        <v>81096.49219999999</v>
+      </c>
+      <c r="G127" t="n">
+        <v>77900.78909999999</v>
+      </c>
+      <c r="H127" t="n">
+        <v>80686.10159999999</v>
+      </c>
+      <c r="I127" t="n">
+        <v>10273374208</v>
+      </c>
+      <c r="J127" t="n">
+        <v>4</v>
+      </c>
+      <c r="K127" t="n">
+        <v>35</v>
+      </c>
+      <c r="L127" t="n">
+        <v>-0.073</v>
+      </c>
+      <c r="M127" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="N127" t="n">
+        <v>33</v>
+      </c>
+      <c r="O127" t="n">
+        <v>0.303</v>
+      </c>
+      <c r="P127" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="Q127" t="n">
+        <v>4.721</v>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Signal Upside as Rally Meets Fed Risk - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdnRMeHk0bG9HRHBNaXlkMFBXRlVja3hLN3dvN2RMUUlWQlo1NzROQW5Da1pnU1h1dmFhUTdwUHdvdXlxZG1Ob2xrZU14RmR4dGtYa3ZzcFBSTnhNSDI3NFRvTDhsODljMUF3VW03UnZTTXkwdm80Um5IaVdzY25Zb0lrRUQ3WGZuVkFZNEdEV1JTVXBmc1dCcmF1ejI5V1U?oc=5</t>
+        </is>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>NEAR Protocol Price Rally Gains Momentum as Hyperliquid Perps Launch Adds Fresh Catalyst - Coinpedia</t>
+        </is>
+      </c>
+      <c r="V127" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOdXo2RDdjZDEzZGdSU3FWV2FQM1Q1QmpHa01YalB0UGRlZmFRWTQzRy1oeUhvb1ljTlJmNVFMSzBYWnJiOTVRX3FVcjdteFRlakRTMTJINy1TYkE0dDhKNF9oOWNrV19neS10ZHY4V25xeDZWYmxmOExnM250eVNWeDNGYnhUdVF5ZW9sY2VDczV6aDNseEZnbE5JdTJrbi1FdG9hX3VoZkpwR1hRTVpqaTRxaFFyVjhUdkJHZS0xZmZabUhtRTlvZ25B0gHKAUFVX3lxTE51ejZEN2NkMTNkZ1JTcVZXYVAzVDVCakdrTVhqUHRQZGVmYVFZNDNHLWh5SG9vWWNOUmY1UUxLMFhacmI5NVFfcVVyN214VGVqRFMxMkg3LVNiQTR0OEo0X2g5Y2tXX2d5LXRkdjhXbnF4NlZibGY4TGczbnR5U1Z4M0ZieFR1UXllb2xjZUNzNXpoM2x4RmdsTkl1MmtuLUV0b2FfdWhmSnBHWFFNWmppNHFoUXJWOFR2QkdlLTFmZlptSG1FOW9nbkE?oc=5</t>
+        </is>
+      </c>
+      <c r="W127" t="inlineStr">
+        <is>
+          <t>Stellar (XLM) Surges 5% on Protocol 28 Upgrade and Altcoin Rally - CoinMarketCap</t>
+        </is>
+      </c>
+      <c r="X127" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFByVlVxX2JTVE9LdTZBZzNjOUp1VnJ2OTlwWHNvRmk5SGVOWDdjbmRrMzR2UXJJWEVHd0dmNTZYTkJlaUNTSXkzMzRKOTFrOXN5RzVYSjkxdHpRbFdKODZ3aV9Zb2JYbndoTmw0ZFRjbnY?oc=5</t>
+        </is>
+      </c>
+      <c r="Y127" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - Pulse 2.0</t>
+        </is>
+      </c>
+      <c r="Z127" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA127" t="inlineStr">
+        <is>
+          <t>Analyst: Bitcoin Rebounds to $77,400 as Short Liquidations Push Buyers Temporarily Ahead - 深潮TechFlow</t>
+        </is>
+      </c>
+      <c r="AB127" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5DUG1VT3dlckQ0T2ZvM2lCZGpFMlA0WTJoUkp6OTBlSkdHVFJURWV1NS0zSWJ0TEJPYloxenp4T1pLOXpBbVQ1XzFlQ0hHUVNkWlFJTkVaVE1JeVVuOG50Z3Bn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC127" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="AD127" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Scan: 2026-09-18 18:58 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD127"/>
+  <dimension ref="A1:AD133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15977,6 +15977,762 @@
       <c r="AD127" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-09-18T18:56:39+00:00</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>4391.2002</v>
+      </c>
+      <c r="F128" t="n">
+        <v>4435.2002</v>
+      </c>
+      <c r="G128" t="n">
+        <v>4386.1001</v>
+      </c>
+      <c r="H128" t="n">
+        <v>4420.5</v>
+      </c>
+      <c r="I128" t="n">
+        <v>29110</v>
+      </c>
+      <c r="J128" t="n">
+        <v>4</v>
+      </c>
+      <c r="K128" t="n">
+        <v>39</v>
+      </c>
+      <c r="L128" t="n">
+        <v>-0.169</v>
+      </c>
+      <c r="M128" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="N128" t="n">
+        <v>40</v>
+      </c>
+      <c r="O128" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="P128" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="Q128" t="n">
+        <v>-2.523</v>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="V128" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="W128" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="X128" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y128" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z128" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA128" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="AB128" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC128" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD128" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-09-18T18:56:39+00:00</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>97.06</v>
+      </c>
+      <c r="F129" t="n">
+        <v>97.36</v>
+      </c>
+      <c r="G129" t="n">
+        <v>95.54000000000001</v>
+      </c>
+      <c r="H129" t="n">
+        <v>95.63</v>
+      </c>
+      <c r="I129" t="n">
+        <v>101542</v>
+      </c>
+      <c r="J129" t="n">
+        <v>4</v>
+      </c>
+      <c r="K129" t="n">
+        <v>39</v>
+      </c>
+      <c r="L129" t="n">
+        <v>-0.067</v>
+      </c>
+      <c r="M129" t="n">
+        <v>-0.205</v>
+      </c>
+      <c r="N129" t="n">
+        <v>40</v>
+      </c>
+      <c r="O129" t="n">
+        <v>0.126</v>
+      </c>
+      <c r="P129" t="n">
+        <v>-0.081</v>
+      </c>
+      <c r="Q129" t="n">
+        <v>0.713</v>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="V129" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="W129" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X129" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y129" t="inlineStr">
+        <is>
+          <t>Oil prices hover near pre-conflict levels as OPEC+ boosts output again - Fox Business</t>
+        </is>
+      </c>
+      <c r="Z129" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOMkNoTG5aUlhwNXRMdk1hN3dUZV9RRkhCWFA0Ul9oMTRiZUlfWGNNQlV4VjkzamwxMXQ0VnJ0dlVXZGVYendtNTN5SDNvdGNKX2hHSlhsQTBBMzRJMDQtUm9xRDFicEU5THVmdV9rd2kxSW8wMndST2MzV2l3ZmVpYUdpZHdZQ0dNMFhSRE1EbVpEOUFhV29iRm9NbmRaZU41Wk130gGoAUFVX3lxTE5WSVpvZE9sRFp1VVVoTTVvZzlLaF9XRE8zM0FZS05JMm9NQUhuRTZQQXcxaURUQlJOd0ZDSlJvM1dRSmFacVNqMnJsTG1zeUpBYzdVeEhZb0NKUkYxM0VOX2tDa1FzQnIydDhkYW5PZThrU3F2YmNFekxqQkF3NnRhaVJ5UlZSbGJ5THVhTUZJMWltUmZ5aGpQMWxZOEhEZjZuLU05VW9LQw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA129" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AB129" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC129" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD129" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-09-18T18:56:39+00:00</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>100.454</v>
+      </c>
+      <c r="F130" t="n">
+        <v>100.468</v>
+      </c>
+      <c r="G130" t="n">
+        <v>100.206</v>
+      </c>
+      <c r="H130" t="n">
+        <v>100.234</v>
+      </c>
+      <c r="I130" t="n">
+        <v>0</v>
+      </c>
+      <c r="J130" t="n">
+        <v>4</v>
+      </c>
+      <c r="K130" t="n">
+        <v>39</v>
+      </c>
+      <c r="L130" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="M130" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="N130" t="n">
+        <v>39</v>
+      </c>
+      <c r="O130" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="P130" t="n">
+        <v>-0.036</v>
+      </c>
+      <c r="Q130" t="n">
+        <v>4.562</v>
+      </c>
+      <c r="R130" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S130" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U130" t="inlineStr">
+        <is>
+          <t>United States Dollar Index rises as strong NFP revives Fed hike bets - Mitrade</t>
+        </is>
+      </c>
+      <c r="V130" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxOWnp0dmNKOUxXeUJubHNPYmNTUHdEOExRSy1rbzAzUHZiQ0RJSVZSbGZNWkh4ck9jSnVCU181cmVQQVFSUDRNeGJ3Z1NYenZrWHFFVE0wZDZpZmlIQlR3Y1hVNkRFS2EwVmVseGZyYnV5TkpvbnNZeXJ4T0g3OWlyY3Vjbw?oc=5</t>
+        </is>
+      </c>
+      <c r="W130" t="inlineStr">
+        <is>
+          <t>FOMC minutes dent DXY rally - FXStreet</t>
+        </is>
+      </c>
+      <c r="X130" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE8zeUZ4XzVZN0t1NUxzdkYxa3lKZVF1b2lvbXhZOHFvSGVNRWJXdlc4QzZyOW9paG9ySExidGE4WDZtaG5tZE1WY3k4UHVNY054NGthZ0dPU29LQ0RfamxVQmxKZ0ZVMWNEWE1ISFltMnZyMmRfM2pGT01qZDVfNDg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y130" t="inlineStr">
+        <is>
+          <t>Gold climbs over 2% as US Dollar trims post-Fed gains - FXStreet</t>
+        </is>
+      </c>
+      <c r="Z130" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPRG5KNUhGZkw4cUIzSmtOLV92bmhnbWE0a1NZMGJSNHdnUnluM05tT2hKSk44cFZFME52LWxETTlvUllCX2VkdHVNLTVlaXdaTURfWHBXY3J2U01BVXl1TDE0dWQyT1ZVV1VwR0RyZ2p0MTdUbmExY1dlNHJPS3EzaVN1MWpwSzVGR1dIYW56aTk1SnlLMnpFcFNpeW4xNVVZT19lcmZhV2JldHJwcTJn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA130" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AB130" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC130" t="inlineStr">
+        <is>
+          <t>Japanese Yen slides as markets look beyond BoJ rate hike - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD130" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOdmVjTXhZSVBDdFJRQ3lBNEZQbEFmdlFwM0VCdXF1RkRWSFRUaVhMdHVvUnd5ZUczc29NYVBPcVVjMzhVV2U1dnJVLWx2YldCZjIzdmUydHUxTTFzeTBWbnBweXMyLUgzV2pKREpsQS1zOE5YcVhXeWVQSWZYY2tBMzhENkh6SVdiemtnRGV4VEgzWkJaemxwdHhudU5fdlNibmpoQjR5S1pRZw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-09-18T18:56:39+00:00</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>7695</v>
+      </c>
+      <c r="F131" t="n">
+        <v>7712.25</v>
+      </c>
+      <c r="G131" t="n">
+        <v>7675</v>
+      </c>
+      <c r="H131" t="n">
+        <v>7711.25</v>
+      </c>
+      <c r="I131" t="n">
+        <v>378874</v>
+      </c>
+      <c r="J131" t="n">
+        <v>4</v>
+      </c>
+      <c r="K131" t="n">
+        <v>40</v>
+      </c>
+      <c r="L131" t="n">
+        <v>-0.054</v>
+      </c>
+      <c r="M131" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="N131" t="n">
+        <v>40</v>
+      </c>
+      <c r="O131" t="n">
+        <v>0.353</v>
+      </c>
+      <c r="P131" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="Q131" t="n">
+        <v>5.997</v>
+      </c>
+      <c r="R131" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S131" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T131" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U131" t="inlineStr">
+        <is>
+          <t>OSR Holdings (OSRH) Surges 15%: Small-Cap Stock Breaks Resistance, Eyes $0.50 Level - Dividend ETF - CarePlus VietNam</t>
+        </is>
+      </c>
+      <c r="V131" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPeU1GWGNLRllfbnJweWwzWDBwZnZTOGphUXlMOVFLMFcwc0RqUGJXVGFxcmx1Mkdwa25XanZ5ZGVRbDczQkd2bzZRX3k3UXRuZlFkYWp0dzVacWkzbzQtaG9adEhDWi00cGx0eXlGc2Z4Q0I4UUZqR1czN2ltaHc3MkdsRnBuY1pLRXR6UjlaMHRpSHctSXVtVDJxZkVwekxNbUhKd3lIaVpmeUNxU3NLRnYwM0pJdE9BU2cxdmxB?oc=5</t>
+        </is>
+      </c>
+      <c r="W131" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="X131" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y131" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="Z131" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA131" t="inlineStr">
+        <is>
+          <t>LVMH stock breaks through 406 € support and falls 20% over three months - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB131" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOZ0owTDAydXBkUDIwMkFqd3ZrRVBqYVhRR21nWUxtXzg5OXVFZUt6WkRPdWdmak4tZE02WGxvdGR3MjdodnhHU2xiZXVqcmxiMndSbkUwSFdfZnFKcHBFVHZicDdSVHBDcTQ3c2trOE8xRlBfbklBZHlHa1F4dTJFWEdtYzQwQVloRGNPa1lFZ3kybS1UX1VFdnoteE11eUJkcjc1LWpCYmV4LTk4Z29XaWFLRHdobFg4UUNxMmg3bkptaUZJYUd4X25YQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC131" t="inlineStr">
+        <is>
+          <t>Organon (OGN) Stock Forecast: When Will $13.68 Resistance Break? 2026-09-17 - Bull Flag - CarePlus VietNam</t>
+        </is>
+      </c>
+      <c r="AD131" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPeEUtMzJ4SzBpempVRlQxVXhLWmZiam0xVnI0b3JILUhLcjJwdVVXcHp4dGhKMUhJNTFXbGVoMmpCRWZmYm52N0tVeW1QWEFQaGZzV0NLQnhFUHg0Y2d3UllBMDhxUDdiM3FLbWRrdDMtUk9aV29BaU9vdEp1bEpOclZfeFNtU1dsaEdYUmJvSy01d242djFXcWZWQTFybGdNRzBfYlZhOU1SYW9LWDRDRU9B?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-09-18T18:56:39+00:00</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>29758.25</v>
+      </c>
+      <c r="F132" t="n">
+        <v>29824.5</v>
+      </c>
+      <c r="G132" t="n">
+        <v>29659.25</v>
+      </c>
+      <c r="H132" t="n">
+        <v>29818.25</v>
+      </c>
+      <c r="I132" t="n">
+        <v>132259</v>
+      </c>
+      <c r="J132" t="n">
+        <v>4</v>
+      </c>
+      <c r="K132" t="n">
+        <v>38</v>
+      </c>
+      <c r="L132" t="n">
+        <v>-0.284</v>
+      </c>
+      <c r="M132" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="N132" t="n">
+        <v>38</v>
+      </c>
+      <c r="O132" t="n">
+        <v>0.201</v>
+      </c>
+      <c r="P132" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="Q132" t="n">
+        <v>-1.566</v>
+      </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>German Medical Cannabis Sales Boost High Tide To Record Performance (NASDAQ:HITI) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPWk4xOHF4YTkxMlliTXAyRDl4bERlWU1ZcFR5ZDYyR1BvYnZUdXNrNXNxX0lVMVBPR0JVbk4wVUhLUDNzbDlrdndfRzRLUlZrWUY4aVVlZ0tneUtFRjF3M2ZnME96RVc3b3VrLWdKQWpDNFp6RmQtSHZLOXlNZzNqTHpQWDByV2JRM3JQcXI4QVBIdVA3enRnMWkzMUtfR29rZUNpcGRsXzZzXzZY?oc=5</t>
+        </is>
+      </c>
+      <c r="U132" t="inlineStr">
+        <is>
+          <t>Samsung Electronics, SK hynix surge as U.S. tech stocks rally - 매일경제</t>
+        </is>
+      </c>
+      <c r="V132" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE55T0VWYmJHT1k0U1U3bldzSXpxTFNoNUVobHNVSHpjVmFhTGQzQUR3b0VDWkpvYlpHR0tFOWM2WXREa2U5NzQwbzE5TVFYT1BrSERZRjFhQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W132" t="inlineStr">
+        <is>
+          <t>US Stocks Rise as Fed Rate Hike Materializes, Nasdaq Gains 1.7%; Tech and Memory Stocks Lead AI-Related Gains; Micron Up 5% - TradingKey</t>
+        </is>
+      </c>
+      <c r="X132" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQaHR2eEdSdEhkb1hPYmNDOG5jOTJmWjBGeFRzZE1nOUFDVXBlX05iOVJ5VjJIS2lBbzJ3VzdaYi05Q3JXQXhBQ2NrTXhWazFaY1RKSHFzdVFrNnJxbkJjd0RjYTdLcDFTT2FxYWd1aUc2eFlfcVEzbWZ0NExpM3V1RU93ZDl3WlZ4eVYzQ3lraXhaX05rTFh3NWxuVVpGVTQySndBUnh2WDlmMDRQMnFiQldfZmNHMXJVSHlTN29BREo2THNPUmRpNlQtc2s4bG1ic2o0Rg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y132" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - forex.com</t>
+        </is>
+      </c>
+      <c r="Z132" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA132" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 17: CoreWeave Falls on Convertible Debt and Share Sale Announcement - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="AB132" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxOZFBscEwwWGdXV1dvNTRVYWZabHNZdzJYM2ZYLWRHT25IMWREb0w2TEFBSjVrRG9jTnR3a2ZjWHI2UElPWS1XMEhqNFRGbGhRNG1uejNnWWtkRURZQTROUXk1TDVVS3hGTFgybEJlWkszaFpmWjlaRFBwLTVheGVWbmRhUXdVcjFwamI3Ui0zRFl1azZEeENvSU96cFFlVU1tSE5wYU1uR1g1cXEtV3FQMkhWS1l0S0lzLVFaMnNuZnhSZ1JLdGx5NmFvLXcwcVlsQTRtODNkNldIVk5sV3RRTWlZWWE3QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC132" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD132" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-09-18T18:56:39+00:00</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>80904.99219999999</v>
+      </c>
+      <c r="F133" t="n">
+        <v>81236.72659999999</v>
+      </c>
+      <c r="G133" t="n">
+        <v>80504.14840000001</v>
+      </c>
+      <c r="H133" t="n">
+        <v>80946.07030000001</v>
+      </c>
+      <c r="I133" t="n">
+        <v>5146540032</v>
+      </c>
+      <c r="J133" t="n">
+        <v>4</v>
+      </c>
+      <c r="K133" t="n">
+        <v>39</v>
+      </c>
+      <c r="L133" t="n">
+        <v>-0.004</v>
+      </c>
+      <c r="M133" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="N133" t="n">
+        <v>32</v>
+      </c>
+      <c r="O133" t="n">
+        <v>0.312</v>
+      </c>
+      <c r="P133" t="n">
+        <v>-0.005</v>
+      </c>
+      <c r="Q133" t="n">
+        <v>8.416</v>
+      </c>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S133" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Signal Upside as Rally Meets Fed Risk - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T133" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdnRMeHk0bG9HRHBNaXlkMFBXRlVja3hLN3dvN2RMUUlWQlo1NzROQW5Da1pnU1h1dmFhUTdwUHdvdXlxZG1Ob2xrZU14RmR4dGtYa3ZzcFBSTnhNSDI3NFRvTDhsODljMUF3VW03UnZTTXkwdm80Um5IaVdzY25Zb0lrRUQ3WGZuVkFZNEdEV1JTVXBmc1dCcmF1ejI5V1U?oc=5</t>
+        </is>
+      </c>
+      <c r="U133" t="inlineStr">
+        <is>
+          <t>NEAR Protocol Price Rally Gains Momentum as Hyperliquid Perps Launch Adds Fresh Catalyst - Coinpedia</t>
+        </is>
+      </c>
+      <c r="V133" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOdXo2RDdjZDEzZGdSU3FWV2FQM1Q1QmpHa01YalB0UGRlZmFRWTQzRy1oeUhvb1ljTlJmNVFMSzBYWnJiOTVRX3FVcjdteFRlakRTMTJINy1TYkE0dDhKNF9oOWNrV19neS10ZHY4V25xeDZWYmxmOExnM250eVNWeDNGYnhUdVF5ZW9sY2VDczV6aDNseEZnbE5JdTJrbi1FdG9hX3VoZkpwR1hRTVpqaTRxaFFyVjhUdkJHZS0xZmZabUhtRTlvZ25B0gHKAUFVX3lxTE51ejZEN2NkMTNkZ1JTcVZXYVAzVDVCakdrTVhqUHRQZGVmYVFZNDNHLWh5SG9vWWNOUmY1UUxLMFhacmI5NVFfcVVyN214VGVqRFMxMkg3LVNiQTR0OEo0X2g5Y2tXX2d5LXRkdjhXbnF4NlZibGY4TGczbnR5U1Z4M0ZieFR1UXllb2xjZUNzNXpoM2x4RmdsTkl1MmtuLUV0b2FfdWhmSnBHWFFNWmppNHFoUXJWOFR2QkdlLTFmZlptSG1FOW9nbkE?oc=5</t>
+        </is>
+      </c>
+      <c r="W133" t="inlineStr">
+        <is>
+          <t>Stacks (STX) Surges 10% on Bitcoin DeFi Launch - CoinMarketCap</t>
+        </is>
+      </c>
+      <c r="X133" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE0zRi1rQi1vR2N6d1F1TTdqTDVIdjA0NkU1dTRXQ2t2YnF6OEpCWElpTXdMSFp5OXZ1SHhTemwzTmppSHF5MzNsbVBvazItTGwzOHMxUS0xdXB6djFPMHJtWHYxTEIyc0ktX2tTbm9xRHo?oc=5</t>
+        </is>
+      </c>
+      <c r="Y133" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - Pulse 2.0</t>
+        </is>
+      </c>
+      <c r="Z133" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA133" t="inlineStr">
+        <is>
+          <t>Analyst: Bitcoin Rebounds to $77,400 as Short Liquidations Push Buyers Temporarily Ahead - 深潮TechFlow</t>
+        </is>
+      </c>
+      <c r="AB133" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5DUG1VT3dlckQ0T2ZvM2lCZGpFMlA0WTJoUkp6OTBlSkdHVFJURWV1NS0zSWJ0TEJPYloxenp4T1pLOXpBbVQ1XzFlQ0hHUVNkWlFJTkVaVE1JeVVuOG50Z3Bn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC133" t="inlineStr">
+        <is>
+          <t>Bitcoin Jumps Above $81,000 as Crypto Liquidations Hit $300M in Four Hours - coingape.com</t>
+        </is>
+      </c>
+      <c r="AD133" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOcDg2RTB3OENSVFNIQmtDSWRGLWtydEpHMkxYa0pnMmJwTEliMDFvMzZ6cUp4aGJyZnBxU1dXeU52eEJNbW85OW1QUmRGRkllanJQczZwdjNyeG9uNEpEck94SmtGcWYyRjBDMl9tREJBZWxqOW90NzZJQ28zenFzUEpsRDNRT2xkeENIeG5OT3MzcFg0TmYydw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-18 22:25 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD133"/>
+  <dimension ref="A1:AD139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16731,6 +16731,762 @@
         </is>
       </c>
       <c r="AD133" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOcDg2RTB3OENSVFNIQmtDSWRGLWtydEpHMkxYa0pnMmJwTEliMDFvMzZ6cUp4aGJyZnBxU1dXeU52eEJNbW85OW1QUmRGRkllanJQczZwdjNyeG9uNEpEck94SmtGcWYyRjBDMl9tREJBZWxqOW90NzZJQ28zenFzUEpsRDNRT2xkeENIeG5OT3MzcFg0TmYydw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:23:10+00:00</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>4421.2002</v>
+      </c>
+      <c r="F134" t="n">
+        <v>4435.2002</v>
+      </c>
+      <c r="G134" t="n">
+        <v>4413.5</v>
+      </c>
+      <c r="H134" t="n">
+        <v>4415.8999</v>
+      </c>
+      <c r="I134" t="n">
+        <v>20009</v>
+      </c>
+      <c r="J134" t="n">
+        <v>4</v>
+      </c>
+      <c r="K134" t="n">
+        <v>39</v>
+      </c>
+      <c r="L134" t="n">
+        <v>-0.233</v>
+      </c>
+      <c r="M134" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="N134" t="n">
+        <v>32</v>
+      </c>
+      <c r="O134" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="P134" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="Q134" t="n">
+        <v>1.552</v>
+      </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S134" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T134" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U134" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V134" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W134" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - azernews.az</t>
+        </is>
+      </c>
+      <c r="X134" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y134" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z134" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA134" t="inlineStr">
+        <is>
+          <t>Gold prices rebound after initial drop, supported by 50-week EMA near $4,300 level. - Pluang</t>
+        </is>
+      </c>
+      <c r="AB134" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQc0d1ZHF1bnVtNk13MzFqR0pNMmV3eWw3TGJLQU9xaHVUZElVSmR6VVotNnp6SEMzZ29IT2V2N0lTS2xXSEZ0RlBPNG9PYkFBVmhrN1ZvX0I4QnpzOEZzbFI5dTFKZDBJZVZiaFpKUlRCQ1h4b3NuaTNUamlMZHZYSy1RQjdjRlZCYzgwNTZZTjVKVWRDelpQY1NIdUM?oc=5</t>
+        </is>
+      </c>
+      <c r="AC134" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD134" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:23:10+00:00</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>95.98999999999999</v>
+      </c>
+      <c r="F135" t="n">
+        <v>96.17</v>
+      </c>
+      <c r="G135" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="H135" t="n">
+        <v>95.47</v>
+      </c>
+      <c r="I135" t="n">
+        <v>66441</v>
+      </c>
+      <c r="J135" t="n">
+        <v>4</v>
+      </c>
+      <c r="K135" t="n">
+        <v>39</v>
+      </c>
+      <c r="L135" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="M135" t="n">
+        <v>-0.159</v>
+      </c>
+      <c r="N135" t="n">
+        <v>40</v>
+      </c>
+      <c r="O135" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="P135" t="n">
+        <v>-0.096</v>
+      </c>
+      <c r="Q135" t="n">
+        <v>2.784</v>
+      </c>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S135" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="U135" t="inlineStr">
+        <is>
+          <t>Maine heating oil prices surge 74% as Assistance Agencies face historic demand ahead of Winter - WABI</t>
+        </is>
+      </c>
+      <c r="V135" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPMTR5amJveF9SdzYtR1E1WmEtN0xuaUNINHNLU3pGU0xPS0Z4R1NXRVJDWkFyUGRHUGhVdDBQWGZHUzB0Z1JaYkNyaFRIZFRKQXZuLTZIUFVkSl8zRFFKaW9IV1JEX0hVdzN1UDdESWgwWGgzRnloTTdqZGdNNFlsdFZlaXlqMGdOTXRsRjRCN2t3dGppS3FmTGE4d2dXZGFOcmtPdzdqQVNENnRFZU02c1kwR0dabDVfT3g00gHPAUFVX3lxTFAwc3ZIazdfU3ZjVXRJcDN4VTBZQjRCRHBGeVdhRkpuenY0Z0Yxb3VEejFheUlHZ1lOanFMRDZ4WUU5ZEE4M2p4MmdaWWxJbXBGM2dWb0ZsbHpHWlNldG9zbEtTMmQxOEtjeEN5MDBIbFBKYnRsRkhnRlFUbnRKSEZRZnhFbmpyTVUxNEJCRFFvQW1oVmkxamllM1I5MUc4TGlqZTBGN1d1VlFGdm55ejhFdTRPcHdfQjF6ejRhazd5cUN6NWQ0TlV6WlhzOXd5Yw?oc=5</t>
+        </is>
+      </c>
+      <c r="W135" t="inlineStr">
+        <is>
+          <t>Crude Oil &amp; Gold Forecast: Key Levels to Watch - FOREX.com</t>
+        </is>
+      </c>
+      <c r="X135" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPWTB1cHRpdk5MalktTnBqZV91SUZjNDZDRV9Fc0tLZ2ZCUFVqSmk0d21BYTk3SnBHVVJsQ0tyVGwyQnVhd1lrNFEzV2M3Vk5jbC15aVlVM1Zyd0QtVWlCR2ktZ19UNDdRSDFwQlNtdV9PTk5sa1pfTzFhSTJQZ1pXVVFud3VrcVhGR2JWLURfZ19VS3NFQ1RVTlFR?oc=5</t>
+        </is>
+      </c>
+      <c r="Y135" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z135" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA135" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB135" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC135" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD135" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:23:10+00:00</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="F136" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="G136" t="n">
+        <v>100.165</v>
+      </c>
+      <c r="H136" t="n">
+        <v>100.215</v>
+      </c>
+      <c r="I136" t="n">
+        <v>0</v>
+      </c>
+      <c r="J136" t="n">
+        <v>4</v>
+      </c>
+      <c r="K136" t="n">
+        <v>39</v>
+      </c>
+      <c r="L136" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="M136" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="N136" t="n">
+        <v>39</v>
+      </c>
+      <c r="O136" t="n">
+        <v>0.124</v>
+      </c>
+      <c r="P136" t="n">
+        <v>-0.028</v>
+      </c>
+      <c r="Q136" t="n">
+        <v>5.271</v>
+      </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>United States Dollar Index rises as strong NFP revives Fed hike bets - Mitrade</t>
+        </is>
+      </c>
+      <c r="V136" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxOWnp0dmNKOUxXeUJubHNPYmNTUHdEOExRSy1rbzAzUHZiQ0RJSVZSbGZNWkh4ck9jSnVCU181cmVQQVFSUDRNeGJ3Z1NYenZrWHFFVE0wZDZpZmlIQlR3Y1hVNkRFS2EwVmVseGZyYnV5TkpvbnNZeXJ4T0g3OWlyY3Vjbw?oc=5</t>
+        </is>
+      </c>
+      <c r="W136" t="inlineStr">
+        <is>
+          <t>FOMC minutes dent DXY rally - FXStreet</t>
+        </is>
+      </c>
+      <c r="X136" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE8zeUZ4XzVZN0t1NUxzdkYxa3lKZVF1b2lvbXhZOHFvSGVNRWJXdlc4QzZyOW9paG9ySExidGE4WDZtaG5tZE1WY3k4UHVNY054NGthZ0dPU29LQ0RfamxVQmxKZ0ZVMWNEWE1ISFltMnZyMmRfM2pGT01qZDVfNDg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y136" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z136" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA136" t="inlineStr">
+        <is>
+          <t>Gold climbs over 2% as US Dollar trims post-Fed gains - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB136" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPRG5KNUhGZkw4cUIzSmtOLV92bmhnbWE0a1NZMGJSNHdnUnluM05tT2hKSk44cFZFME52LWxETTlvUllCX2VkdHVNLTVlaXdaTURfWHBXY3J2U01BVXl1TDE0dWQyT1ZVV1VwR0RyZ2p0MTdUbmExY1dlNHJPS3EzaVN1MWpwSzVGR1dIYW56aTk1SnlLMnpFcFNpeW4xNVVZT19lcmZhV2JldHJwcTJn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC136" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - mufgresearch.com</t>
+        </is>
+      </c>
+      <c r="AD136" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:23:10+00:00</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>7690</v>
+      </c>
+      <c r="F137" t="n">
+        <v>7729.25</v>
+      </c>
+      <c r="G137" t="n">
+        <v>7686.25</v>
+      </c>
+      <c r="H137" t="n">
+        <v>7725</v>
+      </c>
+      <c r="I137" t="n">
+        <v>474169</v>
+      </c>
+      <c r="J137" t="n">
+        <v>4</v>
+      </c>
+      <c r="K137" t="n">
+        <v>40</v>
+      </c>
+      <c r="L137" t="n">
+        <v>-0.096</v>
+      </c>
+      <c r="M137" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="N137" t="n">
+        <v>40</v>
+      </c>
+      <c r="O137" t="n">
+        <v>0.413</v>
+      </c>
+      <c r="P137" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="Q137" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U137" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="V137" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="W137" t="inlineStr">
+        <is>
+          <t>SanDisk SNDK Stock Breaks Resistance as NAND Demand Strengthens but Memory Risks Remain - FXLeaders</t>
+        </is>
+      </c>
+      <c r="X137" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPSENjb3VhWEFEQTd5a0xIM0hGQWFUcTJfU1QyZXZ1VTluMndraDNNSnh2Y25xS0RkWjZJR2JsNDlnRk1KOGFwM0c1NlE3RGN1ZkFhVjA0SXBDNVhISXp1YUxkVnhpUzJGeHVOVHMxVExMTHhmZ0pVMExkSnNNV3BwV2MxMlBYZ1NTMlhmQmpxajdLaUtKNTFKSXllNGc1RUgydm5kZ1RXd1c4VmRBSlA1RUFvMm96QTN3QzdfZWh4MTJ0amY3bk16MDR3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y137" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="Z137" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA137" t="inlineStr">
+        <is>
+          <t>Weekly Market Update: Stocks Flat as Healthcare Rises, Utilities Fall - Morningstar</t>
+        </is>
+      </c>
+      <c r="AB137" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPWW44Z2Jhck5VdTFkTFpKNXhBMjJ3QjJreGFLVzJZcnpIOHZEeVhHS3RRSDFkM0l3b2xucC0xOXlOQlB6MHN6RnFXVTZNV2lHSy1QdGdSN2NqZUx6Q0NzTVpyVFNjU21yWnRQdGhDVy1tYlRiRTJYSDBXeUxRVkxISVFia25rNEkxcVlQbDgyY2hPa3RMOHZLdks3ZGZSSXFlTlE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC137" t="inlineStr">
+        <is>
+          <t>LVMH stock breaks through 406 € support and falls 20% over three months - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AD137" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOZ0owTDAydXBkUDIwMkFqd3ZrRVBqYVhRR21nWUxtXzg5OXVFZUt6WkRPdWdmak4tZE02WGxvdGR3MjdodnhHU2xiZXVqcmxiMndSbkUwSFdfZnFKcHBFVHZicDdSVHBDcTQ3c2trOE8xRlBfbklBZHlHa1F4dTJFWEdtYzQwQVloRGNPa1lFZ3kybS1UX1VFdnoteE11eUJkcjc1LWpCYmV4LTk4Z29XaWFLRHdobFg4UUNxMmg3bkptaUZJYUd4X25YQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:23:10+00:00</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>29728</v>
+      </c>
+      <c r="F138" t="n">
+        <v>29993.25</v>
+      </c>
+      <c r="G138" t="n">
+        <v>29719.75</v>
+      </c>
+      <c r="H138" t="n">
+        <v>29955</v>
+      </c>
+      <c r="I138" t="n">
+        <v>144899</v>
+      </c>
+      <c r="J138" t="n">
+        <v>4</v>
+      </c>
+      <c r="K138" t="n">
+        <v>38</v>
+      </c>
+      <c r="L138" t="n">
+        <v>-0.356</v>
+      </c>
+      <c r="M138" t="n">
+        <v>0.138</v>
+      </c>
+      <c r="N138" t="n">
+        <v>38</v>
+      </c>
+      <c r="O138" t="n">
+        <v>0.212</v>
+      </c>
+      <c r="P138" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="Q138" t="n">
+        <v>-2.732</v>
+      </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>German Medical Cannabis Sales Boost High Tide To Record Performance (NASDAQ:HITI) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPWk4xOHF4YTkxMlliTXAyRDl4bERlWU1ZcFR5ZDYyR1BvYnZUdXNrNXNxX0lVMVBPR0JVbk4wVUhLUDNzbDlrdndfRzRLUlZrWUY4aVVlZ0tneUtFRjF3M2ZnME96RVc3b3VrLWdKQWpDNFp6RmQtSHZLOXlNZzNqTHpQWDByV2JRM3JQcXI4QVBIdVA3enRnMWkzMUtfR29rZUNpcGRsXzZzXzZY?oc=5</t>
+        </is>
+      </c>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>Samsung Electronics, SK hynix surge as U.S. tech stocks rally - 매일경제</t>
+        </is>
+      </c>
+      <c r="V138" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE55T0VWYmJHT1k0U1U3bldzSXpxTFNoNUVobHNVSHpjVmFhTGQzQUR3b0VDWkpvYlpHR0tFOWM2WXREa2U5NzQwbzE5TVFYT1BrSERZRjFhQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W138" t="inlineStr">
+        <is>
+          <t>European stocks rise on tech gains ahead of Fed decision - Anadolu Ajansı</t>
+        </is>
+      </c>
+      <c r="X138" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOOEowelRuazlxN3Y4ZTR4V3A4NUlERk9DYlE1QWh6dXhxQTM2bXVBLUp1NFZfU2NOb2lWcGd1SEN2SGgtR0c5c0p4a2FOdHo0bTZNemMxVUlRVTFHNHFHVFBWRUtzb1hpa2pXRUNqVVNTQVFyRVBwUk92YktXYktBLTJiRF8wSVk4bXRDMXpIWHQ4ODlxenNzcndUN29FZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y138" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z138" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA138" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AB138" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+      <c r="AC138" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - tradingview.com</t>
+        </is>
+      </c>
+      <c r="AD138" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:23:10+00:00</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>80929.60159999999</v>
+      </c>
+      <c r="F139" t="n">
+        <v>81372.42969999999</v>
+      </c>
+      <c r="G139" t="n">
+        <v>80888.5938</v>
+      </c>
+      <c r="H139" t="n">
+        <v>81249.8281</v>
+      </c>
+      <c r="I139" t="n">
+        <v>2780684288</v>
+      </c>
+      <c r="J139" t="n">
+        <v>4</v>
+      </c>
+      <c r="K139" t="n">
+        <v>40</v>
+      </c>
+      <c r="L139" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="M139" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="N139" t="n">
+        <v>35</v>
+      </c>
+      <c r="O139" t="n">
+        <v>0.339</v>
+      </c>
+      <c r="P139" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="Q139" t="n">
+        <v>6.232</v>
+      </c>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Signal Upside as Rally Meets Fed Risk - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdnRMeHk0bG9HRHBNaXlkMFBXRlVja3hLN3dvN2RMUUlWQlo1NzROQW5Da1pnU1h1dmFhUTdwUHdvdXlxZG1Ob2xrZU14RmR4dGtYa3ZzcFBSTnhNSDI3NFRvTDhsODljMUF3VW03UnZTTXkwdm80Um5IaVdzY25Zb0lrRUQ3WGZuVkFZNEdEV1JTVXBmc1dCcmF1ejI5V1U?oc=5</t>
+        </is>
+      </c>
+      <c r="U139" t="inlineStr">
+        <is>
+          <t>Cryptocurrency prices rally with Bitcoin above $81,000 and notable gains across major coins. - Pluang</t>
+        </is>
+      </c>
+      <c r="V139" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE10SDlSX0gxRTdXX3Y4d1BucG9icDlxQVRXc2dpNng1eHFIRHRiRkxTTE5aQ3g0Z2hFZ3ZCUGVOQm1FUWJReURmNE1tQTVxMmdpS1B4U1U0SGgyQnU4MjFvMkRUNXNlakVkVE05cEdlRHp1bFRs?oc=5</t>
+        </is>
+      </c>
+      <c r="W139" t="inlineStr">
+        <is>
+          <t>XRP Surges 6.9% as Bitcoin Rebound Reopens Door to Golden Cross - Decrypt</t>
+        </is>
+      </c>
+      <c r="X139" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ucm9hYldRNWMyRDBjREdzNUthTTVMa3RZcEY5WUdWWjNmOUMya0JSemRqUXE4Q2dNd3JpcFB1ejViT3ZvUWVMUGt5MDlTaHVXd0NVbE9vb0tQYU9Qd3o3czJBRFhBWmI4NGJlaC1sWjQxM3haR3NBM1lWRmJpZ9IBhgFBVV95cUxOM1RxOHBBS0hRVXpGLTlUS3JzUjhIYmFjTG1vdFZiWDhRUE9PV2VlWnBGMmRFMmNpWFhIcjdoeG9SOWJaZ0hwT2N6NG9rbkJuS3g2R01aMlo0allaRDh2WFdxY05neGlaejlwSUtIVGlYRVA1MlZOTUxHR3g0b2UweV9oenZoZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y139" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - Pulse 2.0</t>
+        </is>
+      </c>
+      <c r="Z139" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA139" t="inlineStr">
+        <is>
+          <t>Analyst: Bitcoin Rebounds to $77,400 as Short Liquidations Push Buyers Temporarily Ahead - 深潮TechFlow</t>
+        </is>
+      </c>
+      <c r="AB139" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5DUG1VT3dlckQ0T2ZvM2lCZGpFMlA0WTJoUkp6OTBlSkdHVFJURWV1NS0zSWJ0TEJPYloxenp4T1pLOXpBbVQ1XzFlQ0hHUVNkWlFJTkVaVE1JeVVuOG50Z3Bn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC139" t="inlineStr">
+        <is>
+          <t>Bitcoin Jumps Above $81,000 as Crypto Liquidations Hit $300M in Four Hours - CoinGape</t>
+        </is>
+      </c>
+      <c r="AD139" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOcDg2RTB3OENSVFNIQmtDSWRGLWtydEpHMkxYa0pnMmJwTEliMDFvMzZ6cUp4aGJyZnBxU1dXeU52eEJNbW85OW1QUmRGRkllanJQczZwdjNyeG9uNEpEck94SmtGcWYyRjBDMl9tREJBZWxqOW90NzZJQ28zenFzUEpsRDNRT2xkeENIeG5OT3MzcFg0TmYydw?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-19 03:36 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD139"/>
+  <dimension ref="A1:AD145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17489,6 +17489,762 @@
       <c r="AD139" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOcDg2RTB3OENSVFNIQmtDSWRGLWtydEpHMkxYa0pnMmJwTEliMDFvMzZ6cUp4aGJyZnBxU1dXeU52eEJNbW85OW1QUmRGRkllanJQczZwdjNyeG9uNEpEck94SmtGcWYyRjBDMl9tREJBZWxqOW90NzZJQ28zenFzUEpsRDNRT2xkeENIeG5OT3MzcFg0TmYydw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-09-19T03:34:12+00:00</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>4421.2002</v>
+      </c>
+      <c r="F140" t="n">
+        <v>4435.2002</v>
+      </c>
+      <c r="G140" t="n">
+        <v>4413.5</v>
+      </c>
+      <c r="H140" t="n">
+        <v>4415.8999</v>
+      </c>
+      <c r="I140" t="n">
+        <v>20009</v>
+      </c>
+      <c r="J140" t="n">
+        <v>4</v>
+      </c>
+      <c r="K140" t="n">
+        <v>40</v>
+      </c>
+      <c r="L140" t="n">
+        <v>-0.075</v>
+      </c>
+      <c r="M140" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="N140" t="n">
+        <v>40</v>
+      </c>
+      <c r="O140" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="P140" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="Q140" t="n">
+        <v>-0.775</v>
+      </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U140" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V140" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W140" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X140" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y140" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z140" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA140" t="inlineStr">
+        <is>
+          <t>Gold prices rebound after initial drop, supported by 50-week EMA near $4,300 level. - Pluang</t>
+        </is>
+      </c>
+      <c r="AB140" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQc0d1ZHF1bnVtNk13MzFqR0pNMmV3eWw3TGJLQU9xaHVUZElVSmR6VVotNnp6SEMzZ29IT2V2N0lTS2xXSEZ0RlBPNG9PYkFBVmhrN1ZvX0I4QnpzOEZzbFI5dTFKZDBJZVZiaFpKUlRCQ1h4b3NuaTNUamlMZHZYSy1RQjdjRlZCYzgwNTZZTjVKVWRDelpQY1NIdUM?oc=5</t>
+        </is>
+      </c>
+      <c r="AC140" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="AD140" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-09-19T03:34:12+00:00</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>95.98999999999999</v>
+      </c>
+      <c r="F141" t="n">
+        <v>96.17</v>
+      </c>
+      <c r="G141" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="H141" t="n">
+        <v>95.47</v>
+      </c>
+      <c r="I141" t="n">
+        <v>66441</v>
+      </c>
+      <c r="J141" t="n">
+        <v>4</v>
+      </c>
+      <c r="K141" t="n">
+        <v>39</v>
+      </c>
+      <c r="L141" t="n">
+        <v>-0.051</v>
+      </c>
+      <c r="M141" t="n">
+        <v>-0.189</v>
+      </c>
+      <c r="N141" t="n">
+        <v>40</v>
+      </c>
+      <c r="O141" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="P141" t="n">
+        <v>-0.113</v>
+      </c>
+      <c r="Q141" t="n">
+        <v>-0.751</v>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="V141" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="W141" t="inlineStr">
+        <is>
+          <t>Maine heating oil prices surge 74% as Assistance Agencies face historic demand ahead of Winter - WABI</t>
+        </is>
+      </c>
+      <c r="X141" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPMTR5amJveF9SdzYtR1E1WmEtN0xuaUNINHNLU3pGU0xPS0Z4R1NXRVJDWkFyUGRHUGhVdDBQWGZHUzB0Z1JaYkNyaFRIZFRKQXZuLTZIUFVkSl8zRFFKaW9IV1JEX0hVdzN1UDdESWgwWGgzRnloTTdqZGdNNFlsdFZlaXlqMGdOTXRsRjRCN2t3dGppS3FmTGE4d2dXZGFOcmtPdzdqQVNENnRFZU02c1kwR0dabDVfT3g00gHPAUFVX3lxTFAwc3ZIazdfU3ZjVXRJcDN4VTBZQjRCRHBGeVdhRkpuenY0Z0Yxb3VEejFheUlHZ1lOanFMRDZ4WUU5ZEE4M2p4MmdaWWxJbXBGM2dWb0ZsbHpHWlNldG9zbEtTMmQxOEtjeEN5MDBIbFBKYnRsRkhnRlFUbnRKSEZRZnhFbmpyTVUxNEJCRFFvQW1oVmkxamllM1I5MUc4TGlqZTBGN1d1VlFGdm55ejhFdTRPcHdfQjF6ejRhazd5cUN6NWQ0TlV6WlhzOXd5Yw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y141" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z141" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA141" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB141" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC141" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD141" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-09-19T03:34:12+00:00</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="F142" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="G142" t="n">
+        <v>100.165</v>
+      </c>
+      <c r="H142" t="n">
+        <v>100.215</v>
+      </c>
+      <c r="I142" t="n">
+        <v>0</v>
+      </c>
+      <c r="J142" t="n">
+        <v>4</v>
+      </c>
+      <c r="K142" t="n">
+        <v>38</v>
+      </c>
+      <c r="L142" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="M142" t="n">
+        <v>0.176</v>
+      </c>
+      <c r="N142" t="n">
+        <v>39</v>
+      </c>
+      <c r="O142" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="P142" t="n">
+        <v>-0.07199999999999999</v>
+      </c>
+      <c r="Q142" t="n">
+        <v>2.021</v>
+      </c>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U142" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V142" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W142" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X142" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y142" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z142" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA142" t="inlineStr">
+        <is>
+          <t>Gold climbs over 2% as US Dollar trims post-Fed gains - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB142" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPRG5KNUhGZkw4cUIzSmtOLV92bmhnbWE0a1NZMGJSNHdnUnluM05tT2hKSk44cFZFME52LWxETTlvUllCX2VkdHVNLTVlaXdaTURfWHBXY3J2U01BVXl1TDE0dWQyT1ZVV1VwR0RyZ2p0MTdUbmExY1dlNHJPS3EzaVN1MWpwSzVGR1dIYW56aTk1SnlLMnpFcFNpeW4xNVVZT19lcmZhV2JldHJwcTJn?oc=5</t>
+        </is>
+      </c>
+      <c r="AC142" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD142" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-09-19T03:34:12+00:00</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>7690</v>
+      </c>
+      <c r="F143" t="n">
+        <v>7729.25</v>
+      </c>
+      <c r="G143" t="n">
+        <v>7686.25</v>
+      </c>
+      <c r="H143" t="n">
+        <v>7712.5</v>
+      </c>
+      <c r="I143" t="n">
+        <v>474169</v>
+      </c>
+      <c r="J143" t="n">
+        <v>4</v>
+      </c>
+      <c r="K143" t="n">
+        <v>40</v>
+      </c>
+      <c r="L143" t="n">
+        <v>-0.143</v>
+      </c>
+      <c r="M143" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="N143" t="n">
+        <v>40</v>
+      </c>
+      <c r="O143" t="n">
+        <v>0.373</v>
+      </c>
+      <c r="P143" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="Q143" t="n">
+        <v>4.605</v>
+      </c>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="U143" t="inlineStr">
+        <is>
+          <t>SanDisk SNDK Stock Breaks Resistance as NAND Demand Strengthens but Memory Risks Remain - FXLeaders</t>
+        </is>
+      </c>
+      <c r="V143" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPSENjb3VhWEFEQTd5a0xIM0hGQWFUcTJfU1QyZXZ1VTluMndraDNNSnh2Y25xS0RkWjZJR2JsNDlnRk1KOGFwM0c1NlE3RGN1ZkFhVjA0SXBDNVhISXp1YUxkVnhpUzJGeHVOVHMxVExMTHhmZ0pVMExkSnNNV3BwV2MxMlBYZ1NTMlhmQmpxajdLaUtKNTFKSXllNGc1RUgydm5kZ1RXd1c4VmRBSlA1RUFvMm96QTN3QzdfZWh4MTJ0amY3bk16MDR3?oc=5</t>
+        </is>
+      </c>
+      <c r="W143" t="inlineStr">
+        <is>
+          <t>Dow surges to record close after a fresh tech rally and a plunge in oil prices - Business Insider</t>
+        </is>
+      </c>
+      <c r="X143" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOS0hLS2NLYi1nYlZnTmRJNTRtQXAyZUh5MExFZUVXcEtOTEhzVF9zeHozLThnVHVETGtwMVBFZFBUb3dVaDJlMmtmTUd6Y2ZmUVhMZjRxck41ZEJDZFNqSG5PRm96VXR6bE9tLWlybXBqVWh4NjRUSUJIcFVjdE9xRml2YWJVYTZvMmM4aTQ5bw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y143" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="Z143" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA143" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - CarePlus VietNam</t>
+        </is>
+      </c>
+      <c r="AB143" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC143" t="inlineStr">
+        <is>
+          <t>LVMH stock breaks through 406 € support and falls 20% over three months - ideal-investisseur.fr</t>
+        </is>
+      </c>
+      <c r="AD143" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOZ0owTDAydXBkUDIwMkFqd3ZrRVBqYVhRR21nWUxtXzg5OXVFZUt6WkRPdWdmak4tZE02WGxvdGR3MjdodnhHU2xiZXVqcmxiMndSbkUwSFdfZnFKcHBFVHZicDdSVHBDcTQ3c2trOE8xRlBfbklBZHlHa1F4dTJFWEdtYzQwQVloRGNPa1lFZ3kybS1UX1VFdnoteE11eUJkcjc1LWpCYmV4LTk4Z29XaWFLRHdobFg4UUNxMmg3bkptaUZJYUd4X25YQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-09-19T03:34:12+00:00</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>29728</v>
+      </c>
+      <c r="F144" t="n">
+        <v>29993.25</v>
+      </c>
+      <c r="G144" t="n">
+        <v>29719.75</v>
+      </c>
+      <c r="H144" t="n">
+        <v>29917.25</v>
+      </c>
+      <c r="I144" t="n">
+        <v>144899</v>
+      </c>
+      <c r="J144" t="n">
+        <v>4</v>
+      </c>
+      <c r="K144" t="n">
+        <v>38</v>
+      </c>
+      <c r="L144" t="n">
+        <v>-0.425</v>
+      </c>
+      <c r="M144" t="n">
+        <v>0.132</v>
+      </c>
+      <c r="N144" t="n">
+        <v>37</v>
+      </c>
+      <c r="O144" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="P144" t="n">
+        <v>-0.003</v>
+      </c>
+      <c r="Q144" t="n">
+        <v>-5.084</v>
+      </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>German Medical Cannabis Sales Boost High Tide To Record Performance (NASDAQ:HITI) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPWk4xOHF4YTkxMlliTXAyRDl4bERlWU1ZcFR5ZDYyR1BvYnZUdXNrNXNxX0lVMVBPR0JVbk4wVUhLUDNzbDlrdndfRzRLUlZrWUY4aVVlZ0tneUtFRjF3M2ZnME96RVc3b3VrLWdKQWpDNFp6RmQtSHZLOXlNZzNqTHpQWDByV2JRM3JQcXI4QVBIdVA3enRnMWkzMUtfR29rZUNpcGRsXzZzXzZY?oc=5</t>
+        </is>
+      </c>
+      <c r="U144" t="inlineStr">
+        <is>
+          <t>European stocks rise on tech gains ahead of Fed decision - Anadolu Ajansı</t>
+        </is>
+      </c>
+      <c r="V144" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOOEowelRuazlxN3Y4ZTR4V3A4NUlERk9DYlE1QWh6dXhxQTM2bXVBLUp1NFZfU2NOb2lWcGd1SEN2SGgtR0c5c0p4a2FOdHo0bTZNemMxVUlRVTFHNHFHVFBWRUtzb1hpa2pXRUNqVVNTQVFyRVBwUk92YktXYktBLTJiRF8wSVk4bXRDMXpIWHQ4ODlxenNzcndUN29FZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W144" t="inlineStr">
+        <is>
+          <t>AI Server Stocks Rally as the Hardware Bid Broadens: Hewlett Packard Enterprise Jumps 9%, Super Micro Climbs 6%, Dell Rises 3% - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X144" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNbUk4OGEtN1VjNjBIT1NxMGlpa2tEVC1sTExGOXpKUUpyc1VBX254dVlrTDEtSXN6VkxYM004OFY5eWlObFAwRV84NEVXSlh4WVhtRzFhTXV2eExDcjMxc2JDY1g3TW1DYldOanJmRFJ5eFozYzVLOXVyUExuRDMyak42MnlIcUNJaXRoWGQzbFhGNXNvekxWajhDZGs?oc=5</t>
+        </is>
+      </c>
+      <c r="Y144" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z144" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA144" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB144" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC144" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD144" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-09-19T03:34:12+00:00</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>80880.61719999999</v>
+      </c>
+      <c r="F145" t="n">
+        <v>81704.8594</v>
+      </c>
+      <c r="G145" t="n">
+        <v>80827.57030000001</v>
+      </c>
+      <c r="H145" t="n">
+        <v>81104.14840000001</v>
+      </c>
+      <c r="I145" t="n">
+        <v>2574458880</v>
+      </c>
+      <c r="J145" t="n">
+        <v>4</v>
+      </c>
+      <c r="K145" t="n">
+        <v>40</v>
+      </c>
+      <c r="L145" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="M145" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="N145" t="n">
+        <v>35</v>
+      </c>
+      <c r="O145" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="P145" t="n">
+        <v>-0.041</v>
+      </c>
+      <c r="Q145" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Signal Upside as Rally Meets Fed Risk - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdnRMeHk0bG9HRHBNaXlkMFBXRlVja3hLN3dvN2RMUUlWQlo1NzROQW5Da1pnU1h1dmFhUTdwUHdvdXlxZG1Ob2xrZU14RmR4dGtYa3ZzcFBSTnhNSDI3NFRvTDhsODljMUF3VW03UnZTTXkwdm80Um5IaVdzY25Zb0lrRUQ3WGZuVkFZNEdEV1JTVXBmc1dCcmF1ejI5V1U?oc=5</t>
+        </is>
+      </c>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>Chainlink Surges 4% on Market Rally and Adoption News - CoinMarketCap</t>
+        </is>
+      </c>
+      <c r="V145" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFBvRUpqRDRKOUxtNjV3VXJwVHVFWnhGTDdraVFnQmg1Mk1GLXBkVlo1bkdHelI2Slc3OWk1SGlzdDJKWHE1NU1wVUhyeUZjVVJJbDc0SnM5NVFWa0R3bjZoSXNwU2FYVUVncTloRlRHb18?oc=5</t>
+        </is>
+      </c>
+      <c r="W145" t="inlineStr">
+        <is>
+          <t>Cryptocurrency prices rally with Bitcoin above $81,000 and notable gains across major coins. - Pluang</t>
+        </is>
+      </c>
+      <c r="X145" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE10SDlSX0gxRTdXX3Y4d1BucG9icDlxQVRXc2dpNng1eHFIRHRiRkxTTE5aQ3g0Z2hFZ3ZCUGVOQm1FUWJReURmNE1tQTVxMmdpS1B4U1U0SGgyQnU4MjFvMkRUNXNlakVkVE05cEdlRHp1bFRs?oc=5</t>
+        </is>
+      </c>
+      <c r="Y145" t="inlineStr">
+        <is>
+          <t>CoinShares Posts $21.6 Million Segment EBITDA And Positive Inflows Despite Sharp Crypto Market Decline - Pulse 2.0</t>
+        </is>
+      </c>
+      <c r="Z145" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQLWZDMlFYQUR6TmF3eWtYWFNjMnFqUW44eGVrbTMtcUwxVGg3V2lyRVMxTW1lWFAzWTVKenVYVXJWZW5lcE1LWjRPeTYzV0tYSndiNmdXN0dPWURxS3ltYkJkcVYzZkRmTWV6VHR1VWs2MXhiQjdhNFlwTHFKOXgxYl9veWxKdUpKRjVidDBuanprMERQbGdXZ2lxbG1uRDkteVhWRVhUdTZ3dXlIM1dKWDdHNl9JOFFvYlQyX2dn0gHDAUFVX3lxTFBhOVBDQmRCeDNpM0dmNEptWUtIdHRjemIzaXFhQXdjbGdGUUswRTg5TzhGOUhlcEJUVlZaQ1lYTnFwWk91czV1X3hGelRUUkZQNE1uaUJQZUVuSV80QW9nSkdOR2xZQ1pqLXl5d255QkkyeGpDNEpCZjhIOWhBWkZwNVlkeHJjT1RaSGdFMHhLRVlZNTFmZnhDdW9pVW95ZmlWQllWVk8xSlkzVWZsbVRoeFlaSENWdlJPbmNlS1RtVmRNSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA145" t="inlineStr">
+        <is>
+          <t>Bitcoin Jumps Above $81,000 as Crypto Liquidations Hit $300M in Four Hours - CoinGape</t>
+        </is>
+      </c>
+      <c r="AB145" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOcDg2RTB3OENSVFNIQmtDSWRGLWtydEpHMkxYa0pnMmJwTEliMDFvMzZ6cUp4aGJyZnBxU1dXeU52eEJNbW85OW1QUmRGRkllanJQczZwdjNyeG9uNEpEck94SmtGcWYyRjBDMl9tREJBZWxqOW90NzZJQ28zenFzUEpsRDNRT2xkeENIeG5OT3MzcFg0TmYydw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC145" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="AD145" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-19 08:40 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD145"/>
+  <dimension ref="A1:AD151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18245,6 +18245,762 @@
       <c r="AD145" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-09-19T08:38:27+00:00</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>4421.2002</v>
+      </c>
+      <c r="F146" t="n">
+        <v>4435.2002</v>
+      </c>
+      <c r="G146" t="n">
+        <v>4413.5</v>
+      </c>
+      <c r="H146" t="n">
+        <v>4424.8999</v>
+      </c>
+      <c r="I146" t="n">
+        <v>20009</v>
+      </c>
+      <c r="J146" t="n">
+        <v>4</v>
+      </c>
+      <c r="K146" t="n">
+        <v>40</v>
+      </c>
+      <c r="L146" t="n">
+        <v>-0.126</v>
+      </c>
+      <c r="M146" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="N146" t="n">
+        <v>40</v>
+      </c>
+      <c r="O146" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="P146" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="Q146" t="n">
+        <v>0.654</v>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="V146" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="W146" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="X146" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y146" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="Z146" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA146" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB146" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC146" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD146" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-09-19T08:38:27+00:00</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>95.98999999999999</v>
+      </c>
+      <c r="F147" t="n">
+        <v>96.17</v>
+      </c>
+      <c r="G147" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="H147" t="n">
+        <v>96.08</v>
+      </c>
+      <c r="I147" t="n">
+        <v>66441</v>
+      </c>
+      <c r="J147" t="n">
+        <v>4</v>
+      </c>
+      <c r="K147" t="n">
+        <v>40</v>
+      </c>
+      <c r="L147" t="n">
+        <v>-0.177</v>
+      </c>
+      <c r="M147" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="N147" t="n">
+        <v>40</v>
+      </c>
+      <c r="O147" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="P147" t="n">
+        <v>-0.143</v>
+      </c>
+      <c r="Q147" t="n">
+        <v>-2.279</v>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - energynow.com</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="V147" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W147" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X147" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y147" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z147" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA147" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB147" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC147" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD147" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-09-19T08:38:27+00:00</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="F148" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="G148" t="n">
+        <v>100.165</v>
+      </c>
+      <c r="H148" t="n">
+        <v>100.215</v>
+      </c>
+      <c r="I148" t="n">
+        <v>0</v>
+      </c>
+      <c r="J148" t="n">
+        <v>4</v>
+      </c>
+      <c r="K148" t="n">
+        <v>39</v>
+      </c>
+      <c r="L148" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="M148" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="N148" t="n">
+        <v>39</v>
+      </c>
+      <c r="O148" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="P148" t="n">
+        <v>-0.07199999999999999</v>
+      </c>
+      <c r="Q148" t="n">
+        <v>4.021</v>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - moomoo.com</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V148" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W148" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X148" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y148" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z148" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA148" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AB148" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC148" t="inlineStr">
+        <is>
+          <t>Dovish Fed Bets Pummel Dollar, Boost Gold Ahead of NFP - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD148" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPZDNJaUJnTUhOckR3ODFMRjN3M3QtZ1NzUmtvYnRUOVlyWEo2Nzg4d3l5Tkl4SFNRMVJCUnlNeGxUYm5NQkxpNmxEdzVpU3ZHTkhRUXh0bEdhNld2WHFBVmNCRTBEY2dsUkxqVlYtYTUwX21GR1JZNnZjazk2OXBjNW80dWo3Nmx5TXZYLUY0WkZLei14eWV4dDlkRGVheWM?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-09-19T08:38:27+00:00</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>7690</v>
+      </c>
+      <c r="F149" t="n">
+        <v>7729.25</v>
+      </c>
+      <c r="G149" t="n">
+        <v>7686.25</v>
+      </c>
+      <c r="H149" t="n">
+        <v>7712.5</v>
+      </c>
+      <c r="I149" t="n">
+        <v>474169</v>
+      </c>
+      <c r="J149" t="n">
+        <v>4</v>
+      </c>
+      <c r="K149" t="n">
+        <v>40</v>
+      </c>
+      <c r="L149" t="n">
+        <v>-0.167</v>
+      </c>
+      <c r="M149" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="N149" t="n">
+        <v>40</v>
+      </c>
+      <c r="O149" t="n">
+        <v>0.323</v>
+      </c>
+      <c r="P149" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="Q149" t="n">
+        <v>3.127</v>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - reuters.com</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U149" t="inlineStr">
+        <is>
+          <t>SanDisk SNDK Stock Breaks Resistance as NAND Demand Strengthens but Memory Risks Remain - FXLeaders</t>
+        </is>
+      </c>
+      <c r="V149" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPSENjb3VhWEFEQTd5a0xIM0hGQWFUcTJfU1QyZXZ1VTluMndraDNNSnh2Y25xS0RkWjZJR2JsNDlnRk1KOGFwM0c1NlE3RGN1ZkFhVjA0SXBDNVhISXp1YUxkVnhpUzJGeHVOVHMxVExMTHhmZ0pVMExkSnNNV3BwV2MxMlBYZ1NTMlhmQmpxajdLaUtKNTFKSXllNGc1RUgydm5kZ1RXd1c4VmRBSlA1RUFvMm96QTN3QzdfZWh4MTJ0amY3bk16MDR3?oc=5</t>
+        </is>
+      </c>
+      <c r="W149" t="inlineStr">
+        <is>
+          <t>Dow surges to record close after a fresh tech rally and a plunge in oil prices - Business Insider</t>
+        </is>
+      </c>
+      <c r="X149" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOS0hLS2NLYi1nYlZnTmRJNTRtQXAyZUh5MExFZUVXcEtOTEhzVF9zeHozLThnVHVETGtwMVBFZFBUb3dVaDJlMmtmTUd6Y2ZmUVhMZjRxck41ZEJDZFNqSG5PRm96VXR6bE9tLWlybXBqVWh4NjRUSUJIcFVjdE9xRml2YWJVYTZvMmM4aTQ5bw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y149" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="Z149" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA149" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - CarePlus VietNam</t>
+        </is>
+      </c>
+      <c r="AB149" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC149" t="inlineStr">
+        <is>
+          <t>Weekly Market Update: Stocks Flat as Healthcare Rises, Utilities Fall - Morningstar</t>
+        </is>
+      </c>
+      <c r="AD149" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPWW44Z2Jhck5VdTFkTFpKNXhBMjJ3QjJreGFLVzJZcnpIOHZEeVhHS3RRSDFkM0l3b2xucC0xOXlOQlB6MHN6RnFXVTZNV2lHSy1QdGdSN2NqZUx6Q0NzTVpyVFNjU21yWnRQdGhDVy1tYlRiRTJYSDBXeUxRVkxISVFia25rNEkxcVlQbDgyY2hPa3RMOHZLdks3ZGZSSXFlTlE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-09-19T08:38:27+00:00</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>29728</v>
+      </c>
+      <c r="F150" t="n">
+        <v>29993.25</v>
+      </c>
+      <c r="G150" t="n">
+        <v>29719.75</v>
+      </c>
+      <c r="H150" t="n">
+        <v>29917.25</v>
+      </c>
+      <c r="I150" t="n">
+        <v>144899</v>
+      </c>
+      <c r="J150" t="n">
+        <v>4</v>
+      </c>
+      <c r="K150" t="n">
+        <v>40</v>
+      </c>
+      <c r="L150" t="n">
+        <v>-0.391</v>
+      </c>
+      <c r="M150" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="N150" t="n">
+        <v>37</v>
+      </c>
+      <c r="O150" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="P150" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="Q150" t="n">
+        <v>-5.025</v>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>German Medical Cannabis Sales Boost High Tide To Record Performance (NASDAQ:HITI) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPWk4xOHF4YTkxMlliTXAyRDl4bERlWU1ZcFR5ZDYyR1BvYnZUdXNrNXNxX0lVMVBPR0JVbk4wVUhLUDNzbDlrdndfRzRLUlZrWUY4aVVlZ0tneUtFRjF3M2ZnME96RVc3b3VrLWdKQWpDNFp6RmQtSHZLOXlNZzNqTHpQWDByV2JRM3JQcXI4QVBIdVA3enRnMWkzMUtfR29rZUNpcGRsXzZzXzZY?oc=5</t>
+        </is>
+      </c>
+      <c r="U150" t="inlineStr">
+        <is>
+          <t>Samsung Electronics, SK hynix surge as U.S. tech stocks rally - 매일경제</t>
+        </is>
+      </c>
+      <c r="V150" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE55T0VWYmJHT1k0U1U3bldzSXpxTFNoNUVobHNVSHpjVmFhTGQzQUR3b0VDWkpvYlpHR0tFOWM2WXREa2U5NzQwbzE5TVFYT1BrSERZRjFhQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W150" t="inlineStr">
+        <is>
+          <t>European stocks rise on tech gains ahead of Fed decision - Anadolu Ajansı</t>
+        </is>
+      </c>
+      <c r="X150" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOOEowelRuazlxN3Y4ZTR4V3A4NUlERk9DYlE1QWh6dXhxQTM2bXVBLUp1NFZfU2NOb2lWcGd1SEN2SGgtR0c5c0p4a2FOdHo0bTZNemMxVUlRVTFHNHFHVFBWRUtzb1hpa2pXRUNqVVNTQVFyRVBwUk92YktXYktBLTJiRF8wSVk4bXRDMXpIWHQ4ODlxenNzcndUN29FZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y150" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z150" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA150" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB150" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC150" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD150" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-09-19T08:38:27+00:00</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>80997.75</v>
+      </c>
+      <c r="F151" t="n">
+        <v>81374.9688</v>
+      </c>
+      <c r="G151" t="n">
+        <v>80900</v>
+      </c>
+      <c r="H151" t="n">
+        <v>81294.1562</v>
+      </c>
+      <c r="I151" t="n">
+        <v>0</v>
+      </c>
+      <c r="J151" t="n">
+        <v>4</v>
+      </c>
+      <c r="K151" t="n">
+        <v>39</v>
+      </c>
+      <c r="L151" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="M151" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N151" t="n">
+        <v>36</v>
+      </c>
+      <c r="O151" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="P151" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="Q151" t="n">
+        <v>12.048</v>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Signal Upside as Rally Meets Fed Risk - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdnRMeHk0bG9HRHBNaXlkMFBXRlVja3hLN3dvN2RMUUlWQlo1NzROQW5Da1pnU1h1dmFhUTdwUHdvdXlxZG1Ob2xrZU14RmR4dGtYa3ZzcFBSTnhNSDI3NFRvTDhsODljMUF3VW03UnZTTXkwdm80Um5IaVdzY25Zb0lrRUQ3WGZuVkFZNEdEV1JTVXBmc1dCcmF1ejI5V1U?oc=5</t>
+        </is>
+      </c>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>Cryptocurrency prices rally with Bitcoin above $81,000 and notable gains across major coins. - Pluang</t>
+        </is>
+      </c>
+      <c r="V151" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE10SDlSX0gxRTdXX3Y4d1BucG9icDlxQVRXc2dpNng1eHFIRHRiRkxTTE5aQ3g0Z2hFZ3ZCUGVOQm1FUWJReURmNE1tQTVxMmdpS1B4U1U0SGgyQnU4MjFvMkRUNXNlakVkVE05cEdlRHp1bFRs?oc=5</t>
+        </is>
+      </c>
+      <c r="W151" t="inlineStr">
+        <is>
+          <t>XRP Surges 6.9% as Bitcoin Rebound Reopens Door to Golden Cross - Decrypt</t>
+        </is>
+      </c>
+      <c r="X151" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ucm9hYldRNWMyRDBjREdzNUthTTVMa3RZcEY5WUdWWjNmOUMya0JSemRqUXE4Q2dNd3JpcFB1ejViT3ZvUWVMUGt5MDlTaHVXd0NVbE9vb0tQYU9Qd3o3czJBRFhBWmI4NGJlaC1sWjQxM3haR3NBM1lWRmJpZ9IBhgFBVV95cUxOM1RxOHBBS0hRVXpGLTlUS3JzUjhIYmFjTG1vdFZiWDhRUE9PV2VlWnBGMmRFMmNpWFhIcjdoeG9SOWJaZ0hwT2N6NG9rbkJuS3g2R01aMlo0allaRDh2WFdxY05neGlaejlwSUtIVGlYRVA1MlZOTUxHR3g0b2UweV9oenZoZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y151" t="inlineStr">
+        <is>
+          <t>Bitcoin Jumps Above $81,000 as Crypto Liquidations Hit $300M in Four Hours - CoinGape</t>
+        </is>
+      </c>
+      <c r="Z151" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOcDg2RTB3OENSVFNIQmtDSWRGLWtydEpHMkxYa0pnMmJwTEliMDFvMzZ6cUp4aGJyZnBxU1dXeU52eEJNbW85OW1QUmRGRkllanJQczZwdjNyeG9uNEpEck94SmtGcWYyRjBDMl9tREJBZWxqOW90NzZJQ28zenFzUEpsRDNRT2xkeENIeG5OT3MzcFg0TmYydw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA151" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="AB151" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC151" t="inlineStr">
+        <is>
+          <t>Bitcoin Jumps Above $81,000 as Crypto Liquidations Hit $300M in Four Hours - Cryptonews.net</t>
+        </is>
+      </c>
+      <c r="AD151" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiWEFVX3lxTFBOYmRKRTZZVGtfSkV2YlhlYW9JUzd6S2F4TnpOQ2NKT0ItUUhLbHo2TW44RzA5MmlYbEpjTi1aenh4QUZaV29FTGhmMWhLTmUtcXVmN0puZ1M?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-19 15:34 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD151"/>
+  <dimension ref="A1:AD157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19001,6 +19001,762 @@
       <c r="AD151" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiWEFVX3lxTFBOYmRKRTZZVGtfSkV2YlhlYW9JUzd6S2F4TnpOQ2NKT0ItUUhLbHo2TW44RzA5MmlYbEpjTi1aenh4QUZaV29FTGhmMWhLTmUtcXVmN0puZ1M?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-09-19T15:32:19+00:00</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>4421.2002</v>
+      </c>
+      <c r="F152" t="n">
+        <v>4435.2002</v>
+      </c>
+      <c r="G152" t="n">
+        <v>4413.5</v>
+      </c>
+      <c r="H152" t="n">
+        <v>4424.8999</v>
+      </c>
+      <c r="I152" t="n">
+        <v>20009</v>
+      </c>
+      <c r="J152" t="n">
+        <v>4</v>
+      </c>
+      <c r="K152" t="n">
+        <v>40</v>
+      </c>
+      <c r="L152" t="n">
+        <v>-0.011</v>
+      </c>
+      <c r="M152" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="N152" t="n">
+        <v>40</v>
+      </c>
+      <c r="O152" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="P152" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="Q152" t="n">
+        <v>1.981</v>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U152" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="V152" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="W152" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="X152" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y152" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z152" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA152" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="AB152" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC152" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD152" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-09-19T15:32:19+00:00</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>95.98999999999999</v>
+      </c>
+      <c r="F153" t="n">
+        <v>96.17</v>
+      </c>
+      <c r="G153" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="H153" t="n">
+        <v>96.08</v>
+      </c>
+      <c r="I153" t="n">
+        <v>66441</v>
+      </c>
+      <c r="J153" t="n">
+        <v>4</v>
+      </c>
+      <c r="K153" t="n">
+        <v>40</v>
+      </c>
+      <c r="L153" t="n">
+        <v>-0.114</v>
+      </c>
+      <c r="M153" t="n">
+        <v>-0.194</v>
+      </c>
+      <c r="N153" t="n">
+        <v>32</v>
+      </c>
+      <c r="O153" t="n">
+        <v>-0.08599999999999999</v>
+      </c>
+      <c r="P153" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="Q153" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U153" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="V153" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W153" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X153" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y153" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 17, 2026 - fortune.com</t>
+        </is>
+      </c>
+      <c r="Z153" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE00VzJTYmxIdkNabVVzbnY3V2lyT0tMYkxJOTBOVEUxN0oydU5BYlB3T1FiUFd6MUdLcXpqb0l0WDdKRXZLbmdydlRwWERJbVV6RkdqNVQ0RDZqUHJoZEtia3lB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA153" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB153" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC153" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD153" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-09-19T15:32:19+00:00</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="F154" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="G154" t="n">
+        <v>100.165</v>
+      </c>
+      <c r="H154" t="n">
+        <v>100.215</v>
+      </c>
+      <c r="I154" t="n">
+        <v>0</v>
+      </c>
+      <c r="J154" t="n">
+        <v>4</v>
+      </c>
+      <c r="K154" t="n">
+        <v>39</v>
+      </c>
+      <c r="L154" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="M154" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="N154" t="n">
+        <v>39</v>
+      </c>
+      <c r="O154" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="P154" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="Q154" t="n">
+        <v>6.969</v>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S154" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U154" t="inlineStr">
+        <is>
+          <t>FOMC minutes dent DXY rally - FXStreet</t>
+        </is>
+      </c>
+      <c r="V154" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE8zeUZ4XzVZN0t1NUxzdkYxa3lKZVF1b2lvbXhZOHFvSGVNRWJXdlc4QzZyOW9paG9ySExidGE4WDZtaG5tZE1WY3k4UHVNY054NGthZ0dPU29LQ0RfamxVQmxKZ0ZVMWNEWE1ISFltMnZyMmRfM2pGT01qZDVfNDg?oc=5</t>
+        </is>
+      </c>
+      <c r="W154" t="inlineStr">
+        <is>
+          <t>Dollar rises to session high after Warsh comments, set for weekly gain - CNBC</t>
+        </is>
+      </c>
+      <c r="X154" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOanlNNVpTVDdjS3h1VUtWVXNxZHF4Y2xPREllbVBhX3ZNQ1MwUlJaTGlWeVY3UTM4QmVMbW54a1BNand2eDViNV9JRnR4aVhOdDBpR2Z0Z01qY0EtRmFUWXZabEdONXZURGpUNGo2dWpHNnBLejhfMG5fRGZnRUp0aTBpVExJOGxlbE1KbThpNTJGU2tvZXgway1namdvVGVWcUHSAacBQVVfeXFMT1pORFNoRHVORVI4YTdOcVlXbS1GZ3I5MHNNZXNjbXRDaW5rQXBPbWRSbWNKcDlhSFg4UlpYSFA2Ul9RbVIwRGV5bjlpT1RXaTVMSFNYdElGZ24zUUhkQXhwVjV2NUxPNFZaT0hBWmxUMlNMakcwSlRpYXFqNGdvZ25EZ2JjcHFGaDRQYXIySUtwTkNsUWJnelVZNjBsN1ZSS1VPT1pZQkE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y154" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z154" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA154" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AB154" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC154" t="inlineStr">
+        <is>
+          <t>DXY Falls After Jobs Report - TradingView</t>
+        </is>
+      </c>
+      <c r="AD154" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNSEw2V2JQUlhSd1FvVjhhQlRoSGdrS1V2OUR6QnlSVUF0amg2dDNzWUd3cEh2Slg0ODBNNzVKejgzNGxPbFpZd3N2NG56eFhDYTBTLWpZSVd5WlY2RGQ2SnpKaTNoMkRUckNqQnl5MFZlUVlqWVpmcVBLWHgyLV9PcGhYdGY?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-09-19T15:32:19+00:00</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>7690</v>
+      </c>
+      <c r="F155" t="n">
+        <v>7729.25</v>
+      </c>
+      <c r="G155" t="n">
+        <v>7686.25</v>
+      </c>
+      <c r="H155" t="n">
+        <v>7712.5</v>
+      </c>
+      <c r="I155" t="n">
+        <v>474169</v>
+      </c>
+      <c r="J155" t="n">
+        <v>4</v>
+      </c>
+      <c r="K155" t="n">
+        <v>40</v>
+      </c>
+      <c r="L155" t="n">
+        <v>-0.207</v>
+      </c>
+      <c r="M155" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="N155" t="n">
+        <v>40</v>
+      </c>
+      <c r="O155" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="P155" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="Q155" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S155" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T155" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U155" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="V155" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="W155" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 11: HPE Surges on AI Infrastructure Demand and Recently Raised Guidance - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="X155" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxPMzNYVmJhWm9DS0NJazRybkMxdVQwR1hnMTNxUjVrb2JrN0FyMnZWcWo3UjJtMDFNNWhyQ1VRdWRmTl9nUlRsTXZSclJXSmNJWG5VTUpLcW5BS3U5aXgzTy1zS081OUxLZFlGQzByM2JYS21XQm13ekV0NXFXcHFUaWFyRjZOaHZDZ2NvVEFwS3ZyY1VxZzJOSThqR2hfZkFpQ2VfUGtTbEF1cVZKRG4tMHl1VnNVNkdjUUgxV3Y2WFFJSlAyNU91MnJfcGhJd1J0dlAzamUxS2ljVzNjeDdZLVJzN3VLaWtfd0pn?oc=5</t>
+        </is>
+      </c>
+      <c r="Y155" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="Z155" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA155" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - CarePlus VietNam</t>
+        </is>
+      </c>
+      <c r="AB155" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC155" t="inlineStr">
+        <is>
+          <t>Weekly Market Update: Stocks Flat as Healthcare Rises, Utilities Fall - Morningstar</t>
+        </is>
+      </c>
+      <c r="AD155" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPWW44Z2Jhck5VdTFkTFpKNXhBMjJ3QjJreGFLVzJZcnpIOHZEeVhHS3RRSDFkM0l3b2xucC0xOXlOQlB6MHN6RnFXVTZNV2lHSy1QdGdSN2NqZUx6Q0NzTVpyVFNjU21yWnRQdGhDVy1tYlRiRTJYSDBXeUxRVkxISVFia25rNEkxcVlQbDgyY2hPa3RMOHZLdks3ZGZSSXFlTlE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-09-19T15:32:19+00:00</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>29728</v>
+      </c>
+      <c r="F156" t="n">
+        <v>29993.25</v>
+      </c>
+      <c r="G156" t="n">
+        <v>29719.75</v>
+      </c>
+      <c r="H156" t="n">
+        <v>29917.25</v>
+      </c>
+      <c r="I156" t="n">
+        <v>144899</v>
+      </c>
+      <c r="J156" t="n">
+        <v>4</v>
+      </c>
+      <c r="K156" t="n">
+        <v>40</v>
+      </c>
+      <c r="L156" t="n">
+        <v>-0.221</v>
+      </c>
+      <c r="M156" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="N156" t="n">
+        <v>38</v>
+      </c>
+      <c r="O156" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="P156" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="Q156" t="n">
+        <v>-2.289</v>
+      </c>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>Samsung Electronics, SK hynix surge as U.S. tech stocks rally - 매일경제</t>
+        </is>
+      </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE55T0VWYmJHT1k0U1U3bldzSXpxTFNoNUVobHNVSHpjVmFhTGQzQUR3b0VDWkpvYlpHR0tFOWM2WXREa2U5NzQwbzE5TVFYT1BrSERZRjFhQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U156" t="inlineStr">
+        <is>
+          <t>European stocks rise on tech gains ahead of Fed decision - aa.com.tr</t>
+        </is>
+      </c>
+      <c r="V156" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOOEowelRuazlxN3Y4ZTR4V3A4NUlERk9DYlE1QWh6dXhxQTM2bXVBLUp1NFZfU2NOb2lWcGd1SEN2SGgtR0c5c0p4a2FOdHo0bTZNemMxVUlRVTFHNHFHVFBWRUtzb1hpa2pXRUNqVVNTQVFyRVBwUk92YktXYktBLTJiRF8wSVk4bXRDMXpIWHQ4ODlxenNzcndUN29FZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W156" t="inlineStr">
+        <is>
+          <t>AI Server Stocks Rally as the Hardware Bid Broadens: Hewlett Packard Enterprise Jumps 9%, Super Micro Climbs 6%, Dell Rises 3% - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X156" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNbUk4OGEtN1VjNjBIT1NxMGlpa2tEVC1sTExGOXpKUUpyc1VBX254dVlrTDEtSXN6VkxYM004OFY5eWlObFAwRV84NEVXSlh4WVhtRzFhTXV2eExDcjMxc2JDY1g3TW1DYldOanJmRFJ5eFozYzVLOXVyUExuRDMyak42MnlIcUNJaXRoWGQzbFhGNXNvekxWajhDZGs?oc=5</t>
+        </is>
+      </c>
+      <c r="Y156" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z156" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA156" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB156" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC156" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD156" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-09-19T15:32:19+00:00</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>81282.99219999999</v>
+      </c>
+      <c r="F157" t="n">
+        <v>81734.25</v>
+      </c>
+      <c r="G157" t="n">
+        <v>81148.42969999999</v>
+      </c>
+      <c r="H157" t="n">
+        <v>81619.03909999999</v>
+      </c>
+      <c r="I157" t="n">
+        <v>367648768</v>
+      </c>
+      <c r="J157" t="n">
+        <v>4</v>
+      </c>
+      <c r="K157" t="n">
+        <v>40</v>
+      </c>
+      <c r="L157" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="M157" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="N157" t="n">
+        <v>34</v>
+      </c>
+      <c r="O157" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="P157" t="n">
+        <v>-0.028</v>
+      </c>
+      <c r="Q157" t="n">
+        <v>13.342</v>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Signal Upside as Rally Meets Fed Risk - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdnRMeHk0bG9HRHBNaXlkMFBXRlVja3hLN3dvN2RMUUlWQlo1NzROQW5Da1pnU1h1dmFhUTdwUHdvdXlxZG1Ob2xrZU14RmR4dGtYa3ZzcFBSTnhNSDI3NFRvTDhsODljMUF3VW03UnZTTXkwdm80Um5IaVdzY25Zb0lrRUQ3WGZuVkFZNEdEV1JTVXBmc1dCcmF1ejI5V1U?oc=5</t>
+        </is>
+      </c>
+      <c r="U157" t="inlineStr">
+        <is>
+          <t>Chainlink Surges 4% on Market Rally and Adoption News - CoinMarketCap</t>
+        </is>
+      </c>
+      <c r="V157" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFBvRUpqRDRKOUxtNjV3VXJwVHVFWnhGTDdraVFnQmg1Mk1GLXBkVlo1bkdHelI2Slc3OWk1SGlzdDJKWHE1NU1wVUhyeUZjVVJJbDc0SnM5NVFWa0R3bjZoSXNwU2FYVUVncTloRlRHb18?oc=5</t>
+        </is>
+      </c>
+      <c r="W157" t="inlineStr">
+        <is>
+          <t>XRP Surges 6.9% as Bitcoin Rebound Reopens Door to Golden Cross - Decrypt</t>
+        </is>
+      </c>
+      <c r="X157" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ucm9hYldRNWMyRDBjREdzNUthTTVMa3RZcEY5WUdWWjNmOUMya0JSemRqUXE4Q2dNd3JpcFB1ejViT3ZvUWVMUGt5MDlTaHVXd0NVbE9vb0tQYU9Qd3o3czJBRFhBWmI4NGJlaC1sWjQxM3haR3NBM1lWRmJpZ9IBhgFBVV95cUxOM1RxOHBBS0hRVXpGLTlUS3JzUjhIYmFjTG1vdFZiWDhRUE9PV2VlWnBGMmRFMmNpWFhIcjdoeG9SOWJaZ0hwT2N6NG9rbkJuS3g2R01aMlo0allaRDh2WFdxY05neGlaejlwSUtIVGlYRVA1MlZOTUxHR3g0b2UweV9oenZoZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y157" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="Z157" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA157" t="inlineStr">
+        <is>
+          <t>Bitcoin Jumps Above $81,000 as Crypto Liquidations Hit $300M in Four Hours - Cryptonews.net</t>
+        </is>
+      </c>
+      <c r="AB157" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiWEFVX3lxTFBOYmRKRTZZVGtfSkV2YlhlYW9JUzd6S2F4TnpOQ2NKT0ItUUhLbHo2TW44RzA5MmlYbEpjTi1aenh4QUZaV29FTGhmMWhLTmUtcXVmN0puZ1M?oc=5</t>
+        </is>
+      </c>
+      <c r="AC157" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - crypto.news</t>
+        </is>
+      </c>
+      <c r="AD157" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-19 18:30 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD157"/>
+  <dimension ref="A1:AD163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19755,6 +19755,762 @@
         </is>
       </c>
       <c r="AD157" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-09-19T18:28:53+00:00</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>4421.2002</v>
+      </c>
+      <c r="F158" t="n">
+        <v>4435.2002</v>
+      </c>
+      <c r="G158" t="n">
+        <v>4413.5</v>
+      </c>
+      <c r="H158" t="n">
+        <v>4424.8999</v>
+      </c>
+      <c r="I158" t="n">
+        <v>20009</v>
+      </c>
+      <c r="J158" t="n">
+        <v>4</v>
+      </c>
+      <c r="K158" t="n">
+        <v>40</v>
+      </c>
+      <c r="L158" t="n">
+        <v>-0.015</v>
+      </c>
+      <c r="M158" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="N158" t="n">
+        <v>40</v>
+      </c>
+      <c r="O158" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="P158" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="Q158" t="n">
+        <v>1.717</v>
+      </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U158" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="V158" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="W158" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="X158" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y158" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z158" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA158" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="AB158" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC158" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD158" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-09-19T18:28:53+00:00</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>95.98999999999999</v>
+      </c>
+      <c r="F159" t="n">
+        <v>96.17</v>
+      </c>
+      <c r="G159" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="H159" t="n">
+        <v>96.08</v>
+      </c>
+      <c r="I159" t="n">
+        <v>66441</v>
+      </c>
+      <c r="J159" t="n">
+        <v>4</v>
+      </c>
+      <c r="K159" t="n">
+        <v>40</v>
+      </c>
+      <c r="L159" t="n">
+        <v>-0.187</v>
+      </c>
+      <c r="M159" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="N159" t="n">
+        <v>40</v>
+      </c>
+      <c r="O159" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="P159" t="n">
+        <v>-0.149</v>
+      </c>
+      <c r="Q159" t="n">
+        <v>-1.723</v>
+      </c>
+      <c r="R159" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S159" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T159" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U159" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="V159" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W159" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X159" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y159" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z159" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA159" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB159" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE00VzJTYmxIdkNabVVzbnY3V2lyT0tMYkxJOTBOVEUxN0oydU5BYlB3T1FiUFd6MUdLcXpqb0l0WDdKRXZLbmdydlRwWERJbVV6RkdqNVQ0RDZqUHJoZEtia3lB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC159" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD159" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-09-19T18:28:53+00:00</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="F160" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="G160" t="n">
+        <v>100.165</v>
+      </c>
+      <c r="H160" t="n">
+        <v>100.215</v>
+      </c>
+      <c r="I160" t="n">
+        <v>0</v>
+      </c>
+      <c r="J160" t="n">
+        <v>4</v>
+      </c>
+      <c r="K160" t="n">
+        <v>38</v>
+      </c>
+      <c r="L160" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="M160" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="N160" t="n">
+        <v>40</v>
+      </c>
+      <c r="O160" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="P160" t="n">
+        <v>-0.098</v>
+      </c>
+      <c r="Q160" t="n">
+        <v>4.997</v>
+      </c>
+      <c r="R160" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S160" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="T160" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U160" t="inlineStr">
+        <is>
+          <t>FOMC minutes dent DXY rally - FXStreet</t>
+        </is>
+      </c>
+      <c r="V160" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE8zeUZ4XzVZN0t1NUxzdkYxa3lKZVF1b2lvbXhZOHFvSGVNRWJXdlc4QzZyOW9paG9ySExidGE4WDZtaG5tZE1WY3k4UHVNY054NGthZ0dPU29LQ0RfamxVQmxKZ0ZVMWNEWE1ISFltMnZyMmRfM2pGT01qZDVfNDg?oc=5</t>
+        </is>
+      </c>
+      <c r="W160" t="inlineStr">
+        <is>
+          <t>Dollar rises to session high after Warsh comments, set for weekly gain - CNBC</t>
+        </is>
+      </c>
+      <c r="X160" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOanlNNVpTVDdjS3h1VUtWVXNxZHF4Y2xPREllbVBhX3ZNQ1MwUlJaTGlWeVY3UTM4QmVMbW54a1BNand2eDViNV9JRnR4aVhOdDBpR2Z0Z01qY0EtRmFUWXZabEdONXZURGpUNGo2dWpHNnBLejhfMG5fRGZnRUp0aTBpVExJOGxlbE1KbThpNTJGU2tvZXgway1namdvVGVWcUHSAacBQVVfeXFMT1pORFNoRHVORVI4YTdOcVlXbS1GZ3I5MHNNZXNjbXRDaW5rQXBPbWRSbWNKcDlhSFg4UlpYSFA2Ul9RbVIwRGV5bjlpT1RXaTVMSFNYdElGZ24zUUhkQXhwVjV2NUxPNFZaT0hBWmxUMlNMakcwSlRpYXFqNGdvZ25EZ2JjcHFGaDRQYXIySUtwTkNsUWJnelVZNjBsN1ZSS1VPT1pZQkE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y160" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z160" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA160" t="inlineStr">
+        <is>
+          <t>FX Daily: Fed hold can hit the dollar today - think.ing.com</t>
+        </is>
+      </c>
+      <c r="AB160" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE91QWFPVUVXdGYyVGFxekZhSXBLNzFWN2xfWkJVRXNud05nSzJPQXpwN1hjbzJxZ0ZWLWdmTWhXbzI4NFRXdnpobUc2MllDT1VFQWtFbzhiZ1kzX0Z2c3FGal9nZF91Y19ISENwR1RVdnBRVVVhc0EtY3BmOEZKU1k?oc=5</t>
+        </is>
+      </c>
+      <c r="AC160" t="inlineStr">
+        <is>
+          <t>Dovish Fed Bets Pummel Dollar, Boost Gold Ahead of NFP - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD160" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPZDNJaUJnTUhOckR3ODFMRjN3M3QtZ1NzUmtvYnRUOVlyWEo2Nzg4d3l5Tkl4SFNRMVJCUnlNeGxUYm5NQkxpNmxEdzVpU3ZHTkhRUXh0bEdhNld2WHFBVmNCRTBEY2dsUkxqVlYtYTUwX21GR1JZNnZjazk2OXBjNW80dWo3Nmx5TXZYLUY0WkZLei14eWV4dDlkRGVheWM?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-09-19T18:28:53+00:00</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>7690</v>
+      </c>
+      <c r="F161" t="n">
+        <v>7729.25</v>
+      </c>
+      <c r="G161" t="n">
+        <v>7686.25</v>
+      </c>
+      <c r="H161" t="n">
+        <v>7712.5</v>
+      </c>
+      <c r="I161" t="n">
+        <v>474169</v>
+      </c>
+      <c r="J161" t="n">
+        <v>4</v>
+      </c>
+      <c r="K161" t="n">
+        <v>40</v>
+      </c>
+      <c r="L161" t="n">
+        <v>-0.258</v>
+      </c>
+      <c r="M161" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="N161" t="n">
+        <v>40</v>
+      </c>
+      <c r="O161" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="P161" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="Q161" t="n">
+        <v>0.8080000000000001</v>
+      </c>
+      <c r="R161" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T161" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U161" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 2: Dell Surges 16% on Soaring AI Backlog - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="V161" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQWTRuSVIyTFR2RTZveHRTN3hEWnBwSDl4T2J4ZHZPT01OdEYzWUk3MXZJZjNIc0tTMGYtYmFIYnkxd1dfVVVKTks0MmhzTlc5Z014VHVMMHJVMmZkWWlYVXdHWlczYWRQNzRyYk5leV9ncFBQVE1CbVdTbGNxclNhTy1JNEQwSlVmNjhjOGZrQXBLZlFG?oc=5</t>
+        </is>
+      </c>
+      <c r="W161" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="X161" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y161" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="Z161" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA161" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - CarePlus VietNam</t>
+        </is>
+      </c>
+      <c r="AB161" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC161" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD161" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-09-19T18:28:53+00:00</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>29728</v>
+      </c>
+      <c r="F162" t="n">
+        <v>29993.25</v>
+      </c>
+      <c r="G162" t="n">
+        <v>29719.75</v>
+      </c>
+      <c r="H162" t="n">
+        <v>29917.25</v>
+      </c>
+      <c r="I162" t="n">
+        <v>144899</v>
+      </c>
+      <c r="J162" t="n">
+        <v>4</v>
+      </c>
+      <c r="K162" t="n">
+        <v>40</v>
+      </c>
+      <c r="L162" t="n">
+        <v>-0.247</v>
+      </c>
+      <c r="M162" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="N162" t="n">
+        <v>36</v>
+      </c>
+      <c r="O162" t="n">
+        <v>0.136</v>
+      </c>
+      <c r="P162" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="Q162" t="n">
+        <v>-0.496</v>
+      </c>
+      <c r="R162" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S162" t="inlineStr">
+        <is>
+          <t>Samsung Electronics, SK hynix surge as U.S. tech stocks rally - 매일경제</t>
+        </is>
+      </c>
+      <c r="T162" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE55T0VWYmJHT1k0U1U3bldzSXpxTFNoNUVobHNVSHpjVmFhTGQzQUR3b0VDWkpvYlpHR0tFOWM2WXREa2U5NzQwbzE5TVFYT1BrSERZRjFhQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U162" t="inlineStr">
+        <is>
+          <t>European stocks rise on tech gains ahead of Fed decision - Anadolu Ajansı</t>
+        </is>
+      </c>
+      <c r="V162" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOOEowelRuazlxN3Y4ZTR4V3A4NUlERk9DYlE1QWh6dXhxQTM2bXVBLUp1NFZfU2NOb2lWcGd1SEN2SGgtR0c5c0p4a2FOdHo0bTZNemMxVUlRVTFHNHFHVFBWRUtzb1hpa2pXRUNqVVNTQVFyRVBwUk92YktXYktBLTJiRF8wSVk4bXRDMXpIWHQ4ODlxenNzcndUN29FZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W162" t="inlineStr">
+        <is>
+          <t>AI Server Stocks Rally as the Hardware Bid Broadens: Hewlett Packard Enterprise Jumps 9%, Super Micro Climbs 6%, Dell Rises 3% - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X162" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNbUk4OGEtN1VjNjBIT1NxMGlpa2tEVC1sTExGOXpKUUpyc1VBX254dVlrTDEtSXN6VkxYM004OFY5eWlObFAwRV84NEVXSlh4WVhtRzFhTXV2eExDcjMxc2JDY1g3TW1DYldOanJmRFJ5eFozYzVLOXVyUExuRDMyak42MnlIcUNJaXRoWGQzbFhGNXNvekxWajhDZGs?oc=5</t>
+        </is>
+      </c>
+      <c r="Y162" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - forex.com</t>
+        </is>
+      </c>
+      <c r="Z162" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA162" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB162" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC162" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD162" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-09-19T18:28:53+00:00</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>81554.8906</v>
+      </c>
+      <c r="F163" t="n">
+        <v>81910.78909999999</v>
+      </c>
+      <c r="G163" t="n">
+        <v>81311.1562</v>
+      </c>
+      <c r="H163" t="n">
+        <v>81404.99219999999</v>
+      </c>
+      <c r="I163" t="n">
+        <v>885194752</v>
+      </c>
+      <c r="J163" t="n">
+        <v>4</v>
+      </c>
+      <c r="K163" t="n">
+        <v>38</v>
+      </c>
+      <c r="L163" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="M163" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="N163" t="n">
+        <v>34</v>
+      </c>
+      <c r="O163" t="n">
+        <v>0.408</v>
+      </c>
+      <c r="P163" t="n">
+        <v>-0.075</v>
+      </c>
+      <c r="Q163" t="n">
+        <v>11.074</v>
+      </c>
+      <c r="R163" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S163" t="inlineStr">
+        <is>
+          <t>XRP Surges 6.9% as Bitcoin Rebound Reopens Door to Golden Cross - Decrypt</t>
+        </is>
+      </c>
+      <c r="T163" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ucm9hYldRNWMyRDBjREdzNUthTTVMa3RZcEY5WUdWWjNmOUMya0JSemRqUXE4Q2dNd3JpcFB1ejViT3ZvUWVMUGt5MDlTaHVXd0NVbE9vb0tQYU9Qd3o3czJBRFhBWmI4NGJlaC1sWjQxM3haR3NBM1lWRmJpZ9IBhgFBVV95cUxOM1RxOHBBS0hRVXpGLTlUS3JzUjhIYmFjTG1vdFZiWDhRUE9PV2VlWnBGMmRFMmNpWFhIcjdoeG9SOWJaZ0hwT2N6NG9rbkJuS3g2R01aMlo0allaRDh2WFdxY05neGlaejlwSUtIVGlYRVA1MlZOTUxHR3g0b2UweV9oenZoZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U163" t="inlineStr">
+        <is>
+          <t>Stacks (STX) Surges 11.4% Amid Bitcoin Rally and DeFi Hype - CoinMarketCap</t>
+        </is>
+      </c>
+      <c r="V163" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFB3enFnM25xMGVjZnlXUmZCdVg4V0tjTC1FT3RSUlNpQmRQb2NWSzJ5ZlRyWXJhVzhybzFxa3JzbXA5ZWNiSzV6cVkwTG51aHEyNVBNY1czUF9xOFlmcE55MkM4TmxmS2dJZnNHbmxkamM?oc=5</t>
+        </is>
+      </c>
+      <c r="W163" t="inlineStr">
+        <is>
+          <t>BlackRock clients buy $108M Bitcoin via IBIT as institutional demand stays strong - Pluang</t>
+        </is>
+      </c>
+      <c r="X163" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQbHV3QW80d1E2TzFjbVQ0QkltRlg5dmJ5eHJOVTFpUEstdWNPMWtnNG9qUUxxazBBMV91bVVjNnRJczRzRnJGV2FrLVpwX0xmdUljVnVETE9BelVrcklzc2M4SnoySlFuOXpLWk13d25qRGZuTmtTMlJXenZHNGNpYmxRbjkwSFRTMXdtS3lPQkRSQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y163" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="Z163" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA163" t="inlineStr">
+        <is>
+          <t>Bitcoin Jumps Above $81,000 as Crypto Liquidations Hit $300M in Four Hours - Cryptonews.net</t>
+        </is>
+      </c>
+      <c r="AB163" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiWEFVX3lxTFBOYmRKRTZZVGtfSkV2YlhlYW9JUzd6S2F4TnpOQ2NKT0ItUUhLbHo2TW44RzA5MmlYbEpjTi1aenh4QUZaV29FTGhmMWhLTmUtcXVmN0puZ1M?oc=5</t>
+        </is>
+      </c>
+      <c r="AC163" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - Crypto News</t>
+        </is>
+      </c>
+      <c r="AD163" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-19 22:14 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD163"/>
+  <dimension ref="A1:AD169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20511,6 +20511,762 @@
         </is>
       </c>
       <c r="AD163" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-09-19T22:12:22+00:00</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>4421.2002</v>
+      </c>
+      <c r="F164" t="n">
+        <v>4435.2002</v>
+      </c>
+      <c r="G164" t="n">
+        <v>4413.5</v>
+      </c>
+      <c r="H164" t="n">
+        <v>4424.8999</v>
+      </c>
+      <c r="I164" t="n">
+        <v>20009</v>
+      </c>
+      <c r="J164" t="n">
+        <v>4</v>
+      </c>
+      <c r="K164" t="n">
+        <v>39</v>
+      </c>
+      <c r="L164" t="n">
+        <v>-0.059</v>
+      </c>
+      <c r="M164" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="N164" t="n">
+        <v>40</v>
+      </c>
+      <c r="O164" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="P164" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="Q164" t="n">
+        <v>0.642</v>
+      </c>
+      <c r="R164" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S164" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T164" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U164" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="V164" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="W164" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="X164" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y164" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z164" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA164" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="AB164" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC164" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD164" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-09-19T22:12:22+00:00</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>95.98999999999999</v>
+      </c>
+      <c r="F165" t="n">
+        <v>96.17</v>
+      </c>
+      <c r="G165" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="H165" t="n">
+        <v>96.08</v>
+      </c>
+      <c r="I165" t="n">
+        <v>66441</v>
+      </c>
+      <c r="J165" t="n">
+        <v>4</v>
+      </c>
+      <c r="K165" t="n">
+        <v>40</v>
+      </c>
+      <c r="L165" t="n">
+        <v>-0.142</v>
+      </c>
+      <c r="M165" t="n">
+        <v>-0.181</v>
+      </c>
+      <c r="N165" t="n">
+        <v>40</v>
+      </c>
+      <c r="O165" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="P165" t="n">
+        <v>-0.058</v>
+      </c>
+      <c r="Q165" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="R165" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S165" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T165" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U165" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="V165" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W165" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X165" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y165" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z165" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE00VzJTYmxIdkNabVVzbnY3V2lyT0tMYkxJOTBOVEUxN0oydU5BYlB3T1FiUFd6MUdLcXpqb0l0WDdKRXZLbmdydlRwWERJbVV6RkdqNVQ0RDZqUHJoZEtia3lB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA165" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB165" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC165" t="inlineStr">
+        <is>
+          <t>OPEC oil output falls in August, Reuters survey shows - Reuters</t>
+        </is>
+      </c>
+      <c r="AD165" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcGZWQVVsSEY1MDZDLXRVM2g2N0t1bHJ1VXpWX3pScTFZak53OGQ5VVNxemw0Mjdrd1paNjRYb1YtdFlYN3RIOURKM00xZmc4eFRlTHk2cTNhODJKWW5TOS1BMEE1cVF2NTN5YjJaeHRRNFlBVHUwUU9CN0pyOEdRMHE0c2VtcGNvamRPVFd3OVVlTnFmV3Fobks2WlZJU21oRW44?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-09-19T22:12:22+00:00</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="F166" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="G166" t="n">
+        <v>100.165</v>
+      </c>
+      <c r="H166" t="n">
+        <v>100.215</v>
+      </c>
+      <c r="I166" t="n">
+        <v>0</v>
+      </c>
+      <c r="J166" t="n">
+        <v>4</v>
+      </c>
+      <c r="K166" t="n">
+        <v>39</v>
+      </c>
+      <c r="L166" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="M166" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="N166" t="n">
+        <v>40</v>
+      </c>
+      <c r="O166" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="P166" t="n">
+        <v>-0.039</v>
+      </c>
+      <c r="Q166" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="R166" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S166" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="T166" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U166" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens as BOJ Dissent Clouds Rate-Hike Outlook - Global Banking &amp; Finance Review</t>
+        </is>
+      </c>
+      <c r="V166" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPcDhOdGkwRnVsTWlBeXRTNXRfTENuNjcwbFNGMFVXMllsWTJVTXRSVVA0UC1tSGQyR3ljb1FxRUdCaDlDam5Lc2RFSUZLMWhzOUhlRW9OeDJObWg1MDNReWVZUXl1UF9Dc1lZT1NkWDBqU3hPYjNMTXlKM21qUjE0UTQxZktkSzJHSXpfMWFTOEo?oc=5</t>
+        </is>
+      </c>
+      <c r="W166" t="inlineStr">
+        <is>
+          <t>Dollar rises to session high after Warsh comments, set for weekly gain - CNBC</t>
+        </is>
+      </c>
+      <c r="X166" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOanlNNVpTVDdjS3h1VUtWVXNxZHF4Y2xPREllbVBhX3ZNQ1MwUlJaTGlWeVY3UTM4QmVMbW54a1BNand2eDViNV9JRnR4aVhOdDBpR2Z0Z01qY0EtRmFUWXZabEdONXZURGpUNGo2dWpHNnBLejhfMG5fRGZnRUp0aTBpVExJOGxlbE1KbThpNTJGU2tvZXgway1namdvVGVWcUHSAacBQVVfeXFMT1pORFNoRHVORVI4YTdOcVlXbS1GZ3I5MHNNZXNjbXRDaW5rQXBPbWRSbWNKcDlhSFg4UlpYSFA2Ul9RbVIwRGV5bjlpT1RXaTVMSFNYdElGZ24zUUhkQXhwVjV2NUxPNFZaT0hBWmxUMlNMakcwSlRpYXFqNGdvZ25EZ2JjcHFGaDRQYXIySUtwTkNsUWJnelVZNjBsN1ZSS1VPT1pZQkE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y166" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z166" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA166" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB166" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC166" t="inlineStr">
+        <is>
+          <t>Fed Rate Hike Expectations Cool as Dollar Index Heads for 0.7% Weekly Drop; Yen Posts Strongest Week Since July - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="AD166" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE94WlM1ZkNvNFh0OHpwd2NJSERscXJnUlFBSnZfQkF1SnVOU0RRVExqU2V1VHhkSjFPb0RzNzBabjEyQ0RxVnpvdzY3ekF5eWdBM2JYNWJOZHVzV2hZSEpSYnowczBuNDJVOFZFcktSUTVsQnktZUE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-09-19T22:12:22+00:00</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>7690</v>
+      </c>
+      <c r="F167" t="n">
+        <v>7729.25</v>
+      </c>
+      <c r="G167" t="n">
+        <v>7686.25</v>
+      </c>
+      <c r="H167" t="n">
+        <v>7712.5</v>
+      </c>
+      <c r="I167" t="n">
+        <v>474169</v>
+      </c>
+      <c r="J167" t="n">
+        <v>4</v>
+      </c>
+      <c r="K167" t="n">
+        <v>40</v>
+      </c>
+      <c r="L167" t="n">
+        <v>-0.133</v>
+      </c>
+      <c r="M167" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="N167" t="n">
+        <v>40</v>
+      </c>
+      <c r="O167" t="n">
+        <v>0.314</v>
+      </c>
+      <c r="P167" t="n">
+        <v>-0.011</v>
+      </c>
+      <c r="Q167" t="n">
+        <v>3.621</v>
+      </c>
+      <c r="R167" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T167" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U167" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 2: Dell Surges 16% on Soaring AI Backlog - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="V167" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQWTRuSVIyTFR2RTZveHRTN3hEWnBwSDl4T2J4ZHZPT01OdEYzWUk3MXZJZjNIc0tTMGYtYmFIYnkxd1dfVVVKTks0MmhzTlc5Z014VHVMMHJVMmZkWWlYVXdHWlczYWRQNzRyYk5leV9ncFBQVE1CbVdTbGNxclNhTy1JNEQwSlVmNjhjOGZrQXBLZlFG?oc=5</t>
+        </is>
+      </c>
+      <c r="W167" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="X167" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y167" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="Z167" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA167" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - CarePlus VietNam</t>
+        </is>
+      </c>
+      <c r="AB167" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC167" t="inlineStr">
+        <is>
+          <t>Darden Stock Breaks $207.25 as Earnings Week Puts $202.75 Support in Focus - tradingkey.com</t>
+        </is>
+      </c>
+      <c r="AD167" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPcEZ2cWsxRG44VFRXZkw3dWstakNwczBXVEVEOFpPZHVnSm1XME1QV2I4RUxZckNWcGxITF9LX2pVazVVc0JuNXlfLVUzaHBwWHZoQm91d0tSZmxiY25aVVFCeHNlTXdvZ3JpNWpaeV9QTDA4YS1wdzBmQUxmVnBFZjNCQ3Z2ZXplUnR3RjBWX0VGeTd6alRyTkZsQ01rZ0VNdkRXN2VpdkpnWm1OVU9tbQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-09-19T22:12:22+00:00</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>29728</v>
+      </c>
+      <c r="F168" t="n">
+        <v>29993.25</v>
+      </c>
+      <c r="G168" t="n">
+        <v>29719.75</v>
+      </c>
+      <c r="H168" t="n">
+        <v>29917.25</v>
+      </c>
+      <c r="I168" t="n">
+        <v>144899</v>
+      </c>
+      <c r="J168" t="n">
+        <v>4</v>
+      </c>
+      <c r="K168" t="n">
+        <v>40</v>
+      </c>
+      <c r="L168" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="M168" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="N168" t="n">
+        <v>38</v>
+      </c>
+      <c r="O168" t="n">
+        <v>0.127</v>
+      </c>
+      <c r="P168" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="Q168" t="n">
+        <v>-1.794</v>
+      </c>
+      <c r="R168" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S168" t="inlineStr">
+        <is>
+          <t>US Stocks Rise as Fed Rate Hike Materializes, Nasdaq Gains 1.7%; Tech and Memory Stocks Lead AI-Related Gains; Micron Up 5% - tradingkey.com</t>
+        </is>
+      </c>
+      <c r="T168" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQaHR2eEdSdEhkb1hPYmNDOG5jOTJmWjBGeFRzZE1nOUFDVXBlX05iOVJ5VjJIS2lBbzJ3VzdaYi05Q3JXQXhBQ2NrTXhWazFaY1RKSHFzdVFrNnJxbkJjd0RjYTdLcDFTT2FxYWd1aUc2eFlfcVEzbWZ0NExpM3V1RU93ZDl3WlZ4eVYzQ3lraXhaX05rTFh3NWxuVVpGVTQySndBUnh2WDlmMDRQMnFiQldfZmNHMXJVSHlTN29BREo2THNPUmRpNlQtc2s4bG1ic2o0Rg?oc=5</t>
+        </is>
+      </c>
+      <c r="U168" t="inlineStr">
+        <is>
+          <t>AI Server Stocks Rally as the Hardware Bid Broadens: Hewlett Packard Enterprise Jumps 9%, Super Micro Climbs 6%, Dell Rises 3% - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="V168" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNbUk4OGEtN1VjNjBIT1NxMGlpa2tEVC1sTExGOXpKUUpyc1VBX254dVlrTDEtSXN6VkxYM004OFY5eWlObFAwRV84NEVXSlh4WVhtRzFhTXV2eExDcjMxc2JDY1g3TW1DYldOanJmRFJ5eFozYzVLOXVyUExuRDMyak42MnlIcUNJaXRoWGQzbFhGNXNvekxWajhDZGs?oc=5</t>
+        </is>
+      </c>
+      <c r="W168" t="inlineStr">
+        <is>
+          <t>Tesla Swing Trade for NASDAQ:TSLA by Vasileios_Kairaktidis - TradingView</t>
+        </is>
+      </c>
+      <c r="X168" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE5RRTFlWVkxVDdrUUhKSE1MY3I0QWUtdy00WmpqVi1SZkhybUhIRkcwWTRBd2RSNjZHSGF0Ujd5RTV3dGhWWUxYa05tMjdlT2NQNkRaTDV3MHZoeFNucTZ1ZUU0WnA1ajhmdGs2ZHVKaFVnczRw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y168" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z168" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA168" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB168" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC168" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD168" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-09-19T22:12:22+00:00</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>81427.32030000001</v>
+      </c>
+      <c r="F169" t="n">
+        <v>81445.3281</v>
+      </c>
+      <c r="G169" t="n">
+        <v>80869.60159999999</v>
+      </c>
+      <c r="H169" t="n">
+        <v>80982.0469</v>
+      </c>
+      <c r="I169" t="n">
+        <v>587524096</v>
+      </c>
+      <c r="J169" t="n">
+        <v>4</v>
+      </c>
+      <c r="K169" t="n">
+        <v>39</v>
+      </c>
+      <c r="L169" t="n">
+        <v>0.103</v>
+      </c>
+      <c r="M169" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="N169" t="n">
+        <v>34</v>
+      </c>
+      <c r="O169" t="n">
+        <v>0.353</v>
+      </c>
+      <c r="P169" t="n">
+        <v>-0.065</v>
+      </c>
+      <c r="Q169" t="n">
+        <v>10.509</v>
+      </c>
+      <c r="R169" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S169" t="inlineStr">
+        <is>
+          <t>XRP Surges 6.9% as Bitcoin Rebound Reopens Door to Golden Cross - Decrypt</t>
+        </is>
+      </c>
+      <c r="T169" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ucm9hYldRNWMyRDBjREdzNUthTTVMa3RZcEY5WUdWWjNmOUMya0JSemRqUXE4Q2dNd3JpcFB1ejViT3ZvUWVMUGt5MDlTaHVXd0NVbE9vb0tQYU9Qd3o3czJBRFhBWmI4NGJlaC1sWjQxM3haR3NBM1lWRmJpZ9IBhgFBVV95cUxOM1RxOHBBS0hRVXpGLTlUS3JzUjhIYmFjTG1vdFZiWDhRUE9PV2VlWnBGMmRFMmNpWFhIcjdoeG9SOWJaZ0hwT2N6NG9rbkJuS3g2R01aMlo0allaRDh2WFdxY05neGlaejlwSUtIVGlYRVA1MlZOTUxHR3g0b2UweV9oenZoZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U169" t="inlineStr">
+        <is>
+          <t>Stacks (STX) Surges 11.4% Amid Bitcoin Rally and DeFi Hype - CoinMarketCap</t>
+        </is>
+      </c>
+      <c r="V169" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFB3enFnM25xMGVjZnlXUmZCdVg4V0tjTC1FT3RSUlNpQmRQb2NWSzJ5ZlRyWXJhVzhybzFxa3JzbXA5ZWNiSzV6cVkwTG51aHEyNVBNY1czUF9xOFlmcE55MkM4TmxmS2dJZnNHbmxkamM?oc=5</t>
+        </is>
+      </c>
+      <c r="W169" t="inlineStr">
+        <is>
+          <t>BlackRock clients buy $108M Bitcoin via IBIT as institutional demand stays strong - pluang.com</t>
+        </is>
+      </c>
+      <c r="X169" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQbHV3QW80d1E2TzFjbVQ0QkltRlg5dmJ5eHJOVTFpUEstdWNPMWtnNG9qUUxxazBBMV91bVVjNnRJczRzRnJGV2FrLVpwX0xmdUljVnVETE9BelVrcklzc2M4SnoySlFuOXpLWk13d25qRGZuTmtTMlJXenZHNGNpYmxRbjkwSFRTMXdtS3lPQkRSQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y169" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="Z169" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA169" t="inlineStr">
+        <is>
+          <t>Bitcoin Jumps Above $81,000 as Crypto Liquidations Hit $300M in Four Hours - Cryptonews.net</t>
+        </is>
+      </c>
+      <c r="AB169" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiWEFVX3lxTFBOYmRKRTZZVGtfSkV2YlhlYW9JUzd6S2F4TnpOQ2NKT0ItUUhLbHo2TW44RzA5MmlYbEpjTi1aenh4QUZaV29FTGhmMWhLTmUtcXVmN0puZ1M?oc=5</t>
+        </is>
+      </c>
+      <c r="AC169" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - Crypto News</t>
+        </is>
+      </c>
+      <c r="AD169" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-20 03:51 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD169"/>
+  <dimension ref="A1:AD175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21267,6 +21267,762 @@
         </is>
       </c>
       <c r="AD169" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-09-20T03:49:59+00:00</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>4421.2002</v>
+      </c>
+      <c r="F170" t="n">
+        <v>4435.2002</v>
+      </c>
+      <c r="G170" t="n">
+        <v>4413.5</v>
+      </c>
+      <c r="H170" t="n">
+        <v>4424.8999</v>
+      </c>
+      <c r="I170" t="n">
+        <v>20009</v>
+      </c>
+      <c r="J170" t="n">
+        <v>4</v>
+      </c>
+      <c r="K170" t="n">
+        <v>39</v>
+      </c>
+      <c r="L170" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="M170" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="N170" t="n">
+        <v>40</v>
+      </c>
+      <c r="O170" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="P170" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="Q170" t="n">
+        <v>-0.183</v>
+      </c>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="T170" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="U170" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - cnbc.com</t>
+        </is>
+      </c>
+      <c r="V170" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W170" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="X170" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y170" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z170" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA170" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AB170" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC170" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AD170" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-09-20T03:49:59+00:00</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>95.98999999999999</v>
+      </c>
+      <c r="F171" t="n">
+        <v>96.17</v>
+      </c>
+      <c r="G171" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="H171" t="n">
+        <v>96.08</v>
+      </c>
+      <c r="I171" t="n">
+        <v>66441</v>
+      </c>
+      <c r="J171" t="n">
+        <v>4</v>
+      </c>
+      <c r="K171" t="n">
+        <v>40</v>
+      </c>
+      <c r="L171" t="n">
+        <v>-0.014</v>
+      </c>
+      <c r="M171" t="n">
+        <v>-0.148</v>
+      </c>
+      <c r="N171" t="n">
+        <v>40</v>
+      </c>
+      <c r="O171" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="P171" t="n">
+        <v>-0.122</v>
+      </c>
+      <c r="Q171" t="n">
+        <v>0.141</v>
+      </c>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - cnbc.com</t>
+        </is>
+      </c>
+      <c r="T171" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U171" t="inlineStr">
+        <is>
+          <t>Maine heating oil prices surge 74% as Assistance Agencies face historic demand ahead of Winter - WABI</t>
+        </is>
+      </c>
+      <c r="V171" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPMTR5amJveF9SdzYtR1E1WmEtN0xuaUNINHNLU3pGU0xPS0Z4R1NXRVJDWkFyUGRHUGhVdDBQWGZHUzB0Z1JaYkNyaFRIZFRKQXZuLTZIUFVkSl8zRFFKaW9IV1JEX0hVdzN1UDdESWgwWGgzRnloTTdqZGdNNFlsdFZlaXlqMGdOTXRsRjRCN2t3dGppS3FmTGE4d2dXZGFOcmtPdzdqQVNENnRFZU02c1kwR0dabDVfT3g00gHPAUFVX3lxTFAwc3ZIazdfU3ZjVXRJcDN4VTBZQjRCRHBGeVdhRkpuenY0Z0Yxb3VEejFheUlHZ1lOanFMRDZ4WUU5ZEE4M2p4MmdaWWxJbXBGM2dWb0ZsbHpHWlNldG9zbEtTMmQxOEtjeEN5MDBIbFBKYnRsRkhnRlFUbnRKSEZRZnhFbmpyTVUxNEJCRFFvQW1oVmkxamllM1I5MUc4TGlqZTBGN1d1VlFGdm55ejhFdTRPcHdfQjF6ejRhazd5cUN6NWQ0TlV6WlhzOXd5Yw?oc=5</t>
+        </is>
+      </c>
+      <c r="W171" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - cnbc.com</t>
+        </is>
+      </c>
+      <c r="X171" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y171" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z171" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA171" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB171" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE00VzJTYmxIdkNabVVzbnY3V2lyT0tMYkxJOTBOVEUxN0oydU5BYlB3T1FiUFd6MUdLcXpqb0l0WDdKRXZLbmdydlRwWERJbVV6RkdqNVQ0RDZqUHJoZEtia3lB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC171" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD171" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-09-20T03:49:59+00:00</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="F172" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="G172" t="n">
+        <v>100.165</v>
+      </c>
+      <c r="H172" t="n">
+        <v>100.215</v>
+      </c>
+      <c r="I172" t="n">
+        <v>0</v>
+      </c>
+      <c r="J172" t="n">
+        <v>4</v>
+      </c>
+      <c r="K172" t="n">
+        <v>39</v>
+      </c>
+      <c r="L172" t="n">
+        <v>0.211</v>
+      </c>
+      <c r="M172" t="n">
+        <v>0.151</v>
+      </c>
+      <c r="N172" t="n">
+        <v>40</v>
+      </c>
+      <c r="O172" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="P172" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="Q172" t="n">
+        <v>7.221</v>
+      </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T172" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U172" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="V172" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W172" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens as BOJ Dissent Clouds Rate-Hike Outlook - Global Banking &amp; Finance Review</t>
+        </is>
+      </c>
+      <c r="X172" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPcDhOdGkwRnVsTWlBeXRTNXRfTENuNjcwbFNGMFVXMllsWTJVTXRSVVA0UC1tSGQyR3ljb1FxRUdCaDlDam5Lc2RFSUZLMWhzOUhlRW9OeDJObWg1MDNReWVZUXl1UF9Dc1lZT1NkWDBqU3hPYjNMTXlKM21qUjE0UTQxZktkSzJHSXpfMWFTOEo?oc=5</t>
+        </is>
+      </c>
+      <c r="Y172" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z172" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA172" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB172" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC172" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD172" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-09-20T03:49:59+00:00</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>7690</v>
+      </c>
+      <c r="F173" t="n">
+        <v>7729.25</v>
+      </c>
+      <c r="G173" t="n">
+        <v>7686.25</v>
+      </c>
+      <c r="H173" t="n">
+        <v>7712.5</v>
+      </c>
+      <c r="I173" t="n">
+        <v>474169</v>
+      </c>
+      <c r="J173" t="n">
+        <v>4</v>
+      </c>
+      <c r="K173" t="n">
+        <v>40</v>
+      </c>
+      <c r="L173" t="n">
+        <v>-0.028</v>
+      </c>
+      <c r="M173" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="N173" t="n">
+        <v>40</v>
+      </c>
+      <c r="O173" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="P173" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="Q173" t="n">
+        <v>5.072</v>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 2: Dell Surges 16% on Soaring AI Backlog - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T173" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQWTRuSVIyTFR2RTZveHRTN3hEWnBwSDl4T2J4ZHZPT01OdEYzWUk3MXZJZjNIc0tTMGYtYmFIYnkxd1dfVVVKTks0MmhzTlc5Z014VHVMMHJVMmZkWWlYVXdHWlczYWRQNzRyYk5leV9ncFBQVE1CbVdTbGNxclNhTy1JNEQwSlVmNjhjOGZrQXBLZlFG?oc=5</t>
+        </is>
+      </c>
+      <c r="U173" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="V173" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="W173" t="inlineStr">
+        <is>
+          <t>SanDisk SNDK Stock Breaks Resistance as NAND Demand Strengthens but Memory Risks Remain - FXLeaders</t>
+        </is>
+      </c>
+      <c r="X173" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPSENjb3VhWEFEQTd5a0xIM0hGQWFUcTJfU1QyZXZ1VTluMndraDNNSnh2Y25xS0RkWjZJR2JsNDlnRk1KOGFwM0c1NlE3RGN1ZkFhVjA0SXBDNVhISXp1YUxkVnhpUzJGeHVOVHMxVExMTHhmZ0pVMExkSnNNV3BwV2MxMlBYZ1NTMlhmQmpxajdLaUtKNTFKSXllNGc1RUgydm5kZ1RXd1c4VmRBSlA1RUFvMm96QTN3QzdfZWh4MTJ0amY3bk16MDR3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y173" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z173" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA173" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="AB173" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC173" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD173" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-09-20T03:49:59+00:00</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>29728</v>
+      </c>
+      <c r="F174" t="n">
+        <v>29993.25</v>
+      </c>
+      <c r="G174" t="n">
+        <v>29719.75</v>
+      </c>
+      <c r="H174" t="n">
+        <v>29917.25</v>
+      </c>
+      <c r="I174" t="n">
+        <v>144899</v>
+      </c>
+      <c r="J174" t="n">
+        <v>4</v>
+      </c>
+      <c r="K174" t="n">
+        <v>40</v>
+      </c>
+      <c r="L174" t="n">
+        <v>-0.235</v>
+      </c>
+      <c r="M174" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="N174" t="n">
+        <v>38</v>
+      </c>
+      <c r="O174" t="n">
+        <v>0.214</v>
+      </c>
+      <c r="P174" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="Q174" t="n">
+        <v>0.366</v>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>German Medical Cannabis Sales Boost High Tide To Record Performance (NASDAQ:HITI) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T174" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPWk4xOHF4YTkxMlliTXAyRDl4bERlWU1ZcFR5ZDYyR1BvYnZUdXNrNXNxX0lVMVBPR0JVbk4wVUhLUDNzbDlrdndfRzRLUlZrWUY4aVVlZ0tneUtFRjF3M2ZnME96RVc3b3VrLWdKQWpDNFp6RmQtSHZLOXlNZzNqTHpQWDByV2JRM3JQcXI4QVBIdVA3enRnMWkzMUtfR29rZUNpcGRsXzZzXzZY?oc=5</t>
+        </is>
+      </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq End Higher As Chipmakers Rally, While Dow Posts Best First Half In Five Years — LUNR, AMZN, PLTR, XYZ, AVAV In Focus - Stocktwits</t>
+        </is>
+      </c>
+      <c r="V174" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAJBVV95cUxQUUF0MS1WaEhhRk9BTkk4LUJWMjNHN1lTZ2oxdFJvS1VPRWowTG1KZW8tWHItVnlQaThDZThxZXp1eTFULTFlU21ETTVxcVREMmZQNU9DZ21hTVhJZjBKd2dNUEp2c3dDUmluWlNjOXlldTZ3d1F2aUxrMHo2ejJMSTdmRTJRNlRGblVLS2w5REJhWXRMX19PRld5Z2xKcm1odFhvSGVfMUM2WGU1MndJelM5MFRKMjR0NXJubDlaSkUtMERuU1puRGxjekhsMEZrazVRUjdPWFRoTWpkZXltVWRVb1B6Q2JhdWNyMURDRDljdFo3b3lVMm1sVHY0N29jSlhaRER5T2VQVUt5Z0VObnZkOVZEMmN3VEVEaA?oc=5</t>
+        </is>
+      </c>
+      <c r="W174" t="inlineStr">
+        <is>
+          <t>European stocks rise on tech gains ahead of Fed decision - Anadolu Ajansı</t>
+        </is>
+      </c>
+      <c r="X174" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOOEowelRuazlxN3Y4ZTR4V3A4NUlERk9DYlE1QWh6dXhxQTM2bXVBLUp1NFZfU2NOb2lWcGd1SEN2SGgtR0c5c0p4a2FOdHo0bTZNemMxVUlRVTFHNHFHVFBWRUtzb1hpa2pXRUNqVVNTQVFyRVBwUk92YktXYktBLTJiRF8wSVk4bXRDMXpIWHQ4ODlxenNzcndUN29FZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y174" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z174" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA174" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB174" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC174" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD174" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-09-20T03:49:59+00:00</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>81235.5469</v>
+      </c>
+      <c r="F175" t="n">
+        <v>81302.35159999999</v>
+      </c>
+      <c r="G175" t="n">
+        <v>80091.0312</v>
+      </c>
+      <c r="H175" t="n">
+        <v>80443.82030000001</v>
+      </c>
+      <c r="I175" t="n">
+        <v>3526641664</v>
+      </c>
+      <c r="J175" t="n">
+        <v>4</v>
+      </c>
+      <c r="K175" t="n">
+        <v>38</v>
+      </c>
+      <c r="L175" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="M175" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="N175" t="n">
+        <v>35</v>
+      </c>
+      <c r="O175" t="n">
+        <v>0.414</v>
+      </c>
+      <c r="P175" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q175" t="n">
+        <v>8.269</v>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S175" t="inlineStr">
+        <is>
+          <t>Best Crypto Presale To Buy Now: Remittix Gains Momentum as Institutional Crypto Access Expands - techbullion.com</t>
+        </is>
+      </c>
+      <c r="T175" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPRXk2bEdHNHZEcVhCZXBLX3BnOHQ2SjZQdEhkNVJUZ3o3NW5wMDFNWVphXzVkUkVBcDBMMHAxWEc1cW1FMlEtUDFCY3BxTHAwcmZrOEhoQ1JBcU5tc1lMZlRUTjIxU1JUM2VuTXRIUUZPQW5VckhWWkJweHphWGxWaWZQLVI4bmtDMHpRZXZjNzUteG1WNWo2TzR2SWhkdWpkLWt3M3FpQlF6X0VHT2dvUllsdWVuYVRRMmc?oc=5</t>
+        </is>
+      </c>
+      <c r="U175" t="inlineStr">
+        <is>
+          <t>XRP Surges 6.9% as Bitcoin Rebound Reopens Door to Golden Cross - Decrypt</t>
+        </is>
+      </c>
+      <c r="V175" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ucm9hYldRNWMyRDBjREdzNUthTTVMa3RZcEY5WUdWWjNmOUMya0JSemRqUXE4Q2dNd3JpcFB1ejViT3ZvUWVMUGt5MDlTaHVXd0NVbE9vb0tQYU9Qd3o3czJBRFhBWmI4NGJlaC1sWjQxM3haR3NBM1lWRmJpZ9IBhgFBVV95cUxOM1RxOHBBS0hRVXpGLTlUS3JzUjhIYmFjTG1vdFZiWDhRUE9PV2VlWnBGMmRFMmNpWFhIcjdoeG9SOWJaZ0hwT2N6NG9rbkJuS3g2R01aMlo0allaRDh2WFdxY05neGlaejlwSUtIVGlYRVA1MlZOTUxHR3g0b2UweV9oenZoZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W175" t="inlineStr">
+        <is>
+          <t>BlackRock clients buy $108M Bitcoin via IBIT as institutional demand stays strong - Pluang</t>
+        </is>
+      </c>
+      <c r="X175" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQbHV3QW80d1E2TzFjbVQ0QkltRlg5dmJ5eHJOVTFpUEstdWNPMWtnNG9qUUxxazBBMV91bVVjNnRJczRzRnJGV2FrLVpwX0xmdUljVnVETE9BelVrcklzc2M4SnoySlFuOXpLWk13d25qRGZuTmtTMlJXenZHNGNpYmxRbjkwSFRTMXdtS3lPQkRSQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y175" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="Z175" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA175" t="inlineStr">
+        <is>
+          <t>Bitcoin Is 11 Days From Its First Winning Quarter in a Year. What Needs to Hold Until September 30? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB175" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQTU9EX0F6eUx0b0Q4cVhJMEtNLU92NXJPTmNvSGk2VVJmamw2dEhRdVN6Mi1xWThSbWY1MFRoVjlXWWVFUTdZcm1vajFTY3BXM0k0OHJYaFRZNmZ6dzZjRWFzUjFaeUstUlo5emkxNVhYay10WTJKT1JpbnZEM2xMUExDZ2YzM1dBWTYtbEpqS0pBUTRzUEFKeENRckJONVdnRTFGWm1mVUNOckc2dm4wSHRlQlhrcS1XUGlUQS10SjhlbGVxWFFxXy01VU1lMUNtMXdiX1U5OXBZUVhHRXN0V2lUZUJXYUhlSlFqUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC175" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - Crypto News</t>
+        </is>
+      </c>
+      <c r="AD175" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-20 09:11 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD175"/>
+  <dimension ref="A1:AD181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22023,6 +22023,762 @@
         </is>
       </c>
       <c r="AD175" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-09-20T09:09:20+00:00</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>4421.2002</v>
+      </c>
+      <c r="F176" t="n">
+        <v>4435.2002</v>
+      </c>
+      <c r="G176" t="n">
+        <v>4413.5</v>
+      </c>
+      <c r="H176" t="n">
+        <v>4424.8999</v>
+      </c>
+      <c r="I176" t="n">
+        <v>20009</v>
+      </c>
+      <c r="J176" t="n">
+        <v>4</v>
+      </c>
+      <c r="K176" t="n">
+        <v>39</v>
+      </c>
+      <c r="L176" t="n">
+        <v>-0.043</v>
+      </c>
+      <c r="M176" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="N176" t="n">
+        <v>40</v>
+      </c>
+      <c r="O176" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="P176" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="Q176" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S176" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T176" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U176" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V176" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W176" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X176" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y176" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="Z176" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA176" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB176" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC176" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD176" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-09-20T09:09:20+00:00</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>95.98999999999999</v>
+      </c>
+      <c r="F177" t="n">
+        <v>96.17</v>
+      </c>
+      <c r="G177" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="H177" t="n">
+        <v>96.08</v>
+      </c>
+      <c r="I177" t="n">
+        <v>66441</v>
+      </c>
+      <c r="J177" t="n">
+        <v>4</v>
+      </c>
+      <c r="K177" t="n">
+        <v>40</v>
+      </c>
+      <c r="L177" t="n">
+        <v>-0.168</v>
+      </c>
+      <c r="M177" t="n">
+        <v>-0.153</v>
+      </c>
+      <c r="N177" t="n">
+        <v>40</v>
+      </c>
+      <c r="O177" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="P177" t="n">
+        <v>-0.108</v>
+      </c>
+      <c r="Q177" t="n">
+        <v>-2.595</v>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S177" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T177" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U177" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="V177" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="W177" t="inlineStr">
+        <is>
+          <t>Maine heating oil prices surge 74% as Assistance Agencies face historic demand ahead of Winter - WABI</t>
+        </is>
+      </c>
+      <c r="X177" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPMTR5amJveF9SdzYtR1E1WmEtN0xuaUNINHNLU3pGU0xPS0Z4R1NXRVJDWkFyUGRHUGhVdDBQWGZHUzB0Z1JaYkNyaFRIZFRKQXZuLTZIUFVkSl8zRFFKaW9IV1JEX0hVdzN1UDdESWgwWGgzRnloTTdqZGdNNFlsdFZlaXlqMGdOTXRsRjRCN2t3dGppS3FmTGE4d2dXZGFOcmtPdzdqQVNENnRFZU02c1kwR0dabDVfT3g00gHPAUFVX3lxTFAwc3ZIazdfU3ZjVXRJcDN4VTBZQjRCRHBGeVdhRkpuenY0Z0Yxb3VEejFheUlHZ1lOanFMRDZ4WUU5ZEE4M2p4MmdaWWxJbXBGM2dWb0ZsbHpHWlNldG9zbEtTMmQxOEtjeEN5MDBIbFBKYnRsRkhnRlFUbnRKSEZRZnhFbmpyTVUxNEJCRFFvQW1oVmkxamllM1I5MUc4TGlqZTBGN1d1VlFGdm55ejhFdTRPcHdfQjF6ejRhazd5cUN6NWQ0TlV6WlhzOXd5Yw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y177" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z177" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA177" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB177" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE00VzJTYmxIdkNabVVzbnY3V2lyT0tMYkxJOTBOVEUxN0oydU5BYlB3T1FiUFd6MUdLcXpqb0l0WDdKRXZLbmdydlRwWERJbVV6RkdqNVQ0RDZqUHJoZEtia3lB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC177" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD177" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-09-20T09:09:20+00:00</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="F178" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="G178" t="n">
+        <v>100.165</v>
+      </c>
+      <c r="H178" t="n">
+        <v>100.215</v>
+      </c>
+      <c r="I178" t="n">
+        <v>0</v>
+      </c>
+      <c r="J178" t="n">
+        <v>4</v>
+      </c>
+      <c r="K178" t="n">
+        <v>39</v>
+      </c>
+      <c r="L178" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="M178" t="n">
+        <v>0.149</v>
+      </c>
+      <c r="N178" t="n">
+        <v>40</v>
+      </c>
+      <c r="O178" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="P178" t="n">
+        <v>-0.038</v>
+      </c>
+      <c r="Q178" t="n">
+        <v>5.858</v>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S178" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T178" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U178" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V178" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W178" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X178" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y178" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z178" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA178" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB178" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC178" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD178" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-09-20T09:09:20+00:00</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>7690</v>
+      </c>
+      <c r="F179" t="n">
+        <v>7729.25</v>
+      </c>
+      <c r="G179" t="n">
+        <v>7686.25</v>
+      </c>
+      <c r="H179" t="n">
+        <v>7712.5</v>
+      </c>
+      <c r="I179" t="n">
+        <v>474169</v>
+      </c>
+      <c r="J179" t="n">
+        <v>4</v>
+      </c>
+      <c r="K179" t="n">
+        <v>39</v>
+      </c>
+      <c r="L179" t="n">
+        <v>-0.112</v>
+      </c>
+      <c r="M179" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="N179" t="n">
+        <v>40</v>
+      </c>
+      <c r="O179" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="P179" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="Q179" t="n">
+        <v>2.489</v>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S179" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 2: Dell Surges 16% on Soaring AI Backlog - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T179" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQWTRuSVIyTFR2RTZveHRTN3hEWnBwSDl4T2J4ZHZPT01OdEYzWUk3MXZJZjNIc0tTMGYtYmFIYnkxd1dfVVVKTks0MmhzTlc5Z014VHVMMHJVMmZkWWlYVXdHWlczYWRQNzRyYk5leV9ncFBQVE1CbVdTbGNxclNhTy1JNEQwSlVmNjhjOGZrQXBLZlFG?oc=5</t>
+        </is>
+      </c>
+      <c r="U179" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="V179" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="W179" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq End Higher As Chipmakers Rally, While Dow Posts Best First Half In Five Years — LUNR, AMZN, PLTR, XYZ, AVAV In Focus - Stocktwits</t>
+        </is>
+      </c>
+      <c r="X179" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAJBVV95cUxQUUF0MS1WaEhhRk9BTkk4LUJWMjNHN1lTZ2oxdFJvS1VPRWowTG1KZW8tWHItVnlQaThDZThxZXp1eTFULTFlU21ETTVxcVREMmZQNU9DZ21hTVhJZjBKd2dNUEp2c3dDUmluWlNjOXlldTZ3d1F2aUxrMHo2ejJMSTdmRTJRNlRGblVLS2w5REJhWXRMX19PRld5Z2xKcm1odFhvSGVfMUM2WGU1MndJelM5MFRKMjR0NXJubDlaSkUtMERuU1puRGxjekhsMEZrazVRUjdPWFRoTWpkZXltVWRVb1B6Q2JhdWNyMURDRDljdFo3b3lVMm1sVHY0N29jSlhaRER5T2VQVUt5Z0VObnZkOVZEMmN3VEVEaA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y179" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="Z179" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA179" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - CarePlus VietNam</t>
+        </is>
+      </c>
+      <c r="AB179" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC179" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD179" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-09-20T09:09:20+00:00</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>29728</v>
+      </c>
+      <c r="F180" t="n">
+        <v>29993.25</v>
+      </c>
+      <c r="G180" t="n">
+        <v>29719.75</v>
+      </c>
+      <c r="H180" t="n">
+        <v>29917.25</v>
+      </c>
+      <c r="I180" t="n">
+        <v>144899</v>
+      </c>
+      <c r="J180" t="n">
+        <v>4</v>
+      </c>
+      <c r="K180" t="n">
+        <v>40</v>
+      </c>
+      <c r="L180" t="n">
+        <v>-0.291</v>
+      </c>
+      <c r="M180" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="N180" t="n">
+        <v>38</v>
+      </c>
+      <c r="O180" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="P180" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="Q180" t="n">
+        <v>-2.364</v>
+      </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S180" t="inlineStr">
+        <is>
+          <t>S&amp;P and Nasdaq hit record highs, continuing remarkable recovery from war shock - CNN</t>
+        </is>
+      </c>
+      <c r="T180" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBFM0dLbkRoQTEzbmVyNGdlZERORGZXdEJrOVh3U0FZVnJsNk0zQjFWVVF6a0NhQThTbS0zMUJTdmdHWm1JYVF3LW5VUWVJWFk1MUd6WlVNWU9aa0dENG9rbkYzRDFpcmhSQ1BJ?oc=5</t>
+        </is>
+      </c>
+      <c r="U180" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq End Higher As Chipmakers Rally, While Dow Posts Best First Half In Five Years — LUNR, AMZN, PLTR, XYZ, AVAV In Focus - Stocktwits</t>
+        </is>
+      </c>
+      <c r="V180" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAJBVV95cUxQUUF0MS1WaEhhRk9BTkk4LUJWMjNHN1lTZ2oxdFJvS1VPRWowTG1KZW8tWHItVnlQaThDZThxZXp1eTFULTFlU21ETTVxcVREMmZQNU9DZ21hTVhJZjBKd2dNUEp2c3dDUmluWlNjOXlldTZ3d1F2aUxrMHo2ejJMSTdmRTJRNlRGblVLS2w5REJhWXRMX19PRld5Z2xKcm1odFhvSGVfMUM2WGU1MndJelM5MFRKMjR0NXJubDlaSkUtMERuU1puRGxjekhsMEZrazVRUjdPWFRoTWpkZXltVWRVb1B6Q2JhdWNyMURDRDljdFo3b3lVMm1sVHY0N29jSlhaRER5T2VQVUt5Z0VObnZkOVZEMmN3VEVEaA?oc=5</t>
+        </is>
+      </c>
+      <c r="W180" t="inlineStr">
+        <is>
+          <t>European stocks rise on tech gains ahead of Fed decision - Anadolu Ajansı</t>
+        </is>
+      </c>
+      <c r="X180" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOOEowelRuazlxN3Y4ZTR4V3A4NUlERk9DYlE1QWh6dXhxQTM2bXVBLUp1NFZfU2NOb2lWcGd1SEN2SGgtR0c5c0p4a2FOdHo0bTZNemMxVUlRVTFHNHFHVFBWRUtzb1hpa2pXRUNqVVNTQVFyRVBwUk92YktXYktBLTJiRF8wSVk4bXRDMXpIWHQ4ODlxenNzcndUN29FZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y180" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z180" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA180" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB180" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC180" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD180" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-09-20T09:09:20+00:00</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>80456.00780000001</v>
+      </c>
+      <c r="F181" t="n">
+        <v>80573.6094</v>
+      </c>
+      <c r="G181" t="n">
+        <v>80139.6406</v>
+      </c>
+      <c r="H181" t="n">
+        <v>80244.00780000001</v>
+      </c>
+      <c r="I181" t="n">
+        <v>2468294656</v>
+      </c>
+      <c r="J181" t="n">
+        <v>4</v>
+      </c>
+      <c r="K181" t="n">
+        <v>37</v>
+      </c>
+      <c r="L181" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="M181" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="N181" t="n">
+        <v>36</v>
+      </c>
+      <c r="O181" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="P181" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="Q181" t="n">
+        <v>7.109</v>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S181" t="inlineStr">
+        <is>
+          <t>Best Crypto Presale To Buy Now: Remittix Gains Momentum as Institutional Crypto Access Expands - TechBullion</t>
+        </is>
+      </c>
+      <c r="T181" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPRXk2bEdHNHZEcVhCZXBLX3BnOHQ2SjZQdEhkNVJUZ3o3NW5wMDFNWVphXzVkUkVBcDBMMHAxWEc1cW1FMlEtUDFCY3BxTHAwcmZrOEhoQ1JBcU5tc1lMZlRUTjIxU1JUM2VuTXRIUUZPQW5VckhWWkJweHphWGxWaWZQLVI4bmtDMHpRZXZjNzUteG1WNWo2TzR2SWhkdWpkLWt3M3FpQlF6X0VHT2dvUllsdWVuYVRRMmc?oc=5</t>
+        </is>
+      </c>
+      <c r="U181" t="inlineStr">
+        <is>
+          <t>BlackRock clients buy $108M Bitcoin via IBIT as institutional demand stays strong - Pluang</t>
+        </is>
+      </c>
+      <c r="V181" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQbHV3QW80d1E2TzFjbVQ0QkltRlg5dmJ5eHJOVTFpUEstdWNPMWtnNG9qUUxxazBBMV91bVVjNnRJczRzRnJGV2FrLVpwX0xmdUljVnVETE9BelVrcklzc2M4SnoySlFuOXpLWk13d25qRGZuTmtTMlJXenZHNGNpYmxRbjkwSFRTMXdtS3lPQkRSQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W181" t="inlineStr">
+        <is>
+          <t>Bitcoin price extends gains, briefly tops $81,000 as crypto rally gathers pace - CNBC</t>
+        </is>
+      </c>
+      <c r="X181" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQdlVlbW1UcGhZSVR6dW9SVTIxX2xrREJYT2VrTnBCRENqeVp4ZUdpUERjemp6QmNLY1h0cUlVYm91OVBublNPOXh0aVdHWHdaU0JyX2gwanhxM0FuYmhfbUNOQjF4UVZPenhjd2tBaDBzbF9DbnMySkotcUpoLVVtekJld2QzcjJaUDNfWFF0cnRRY3NvUk5SMVB6MjLSAaIBQVVfeXFMUE5UVkdmUVAwazBVMTE3Rk5qNUIyTmtPZFhtUzdOVmhSQV9fUUVlT3VpUmZnQnJ5WlR5WWxsTk5ycEpwV0xOMmlkR05NQWNLVzA3R0JYSk5YUFh6NE9CTGtzVXpfeVNLb2l6TFVQUWxKOWthZGlwdHZEMlQwT0JWOEdWVXQwdlViNW9uZG5SQmZKQUhLSTdrOVpuRHBrNUV6a19B?oc=5</t>
+        </is>
+      </c>
+      <c r="Y181" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="Z181" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA181" t="inlineStr">
+        <is>
+          <t>Bitcoin Is 11 Days From Its First Winning Quarter in a Year. What Needs to Hold Until September 30? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB181" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQTU9EX0F6eUx0b0Q4cVhJMEtNLU92NXJPTmNvSGk2VVJmamw2dEhRdVN6Mi1xWThSbWY1MFRoVjlXWWVFUTdZcm1vajFTY3BXM0k0OHJYaFRZNmZ6dzZjRWFzUjFaeUstUlo5emkxNVhYay10WTJKT1JpbnZEM2xMUExDZ2YzM1dBWTYtbEpqS0pBUTRzUEFKeENRckJONVdnRTFGWm1mVUNOckc2dm4wSHRlQlhrcS1XUGlUQS10SjhlbGVxWFFxXy01VU1lMUNtMXdiX1U5OXBZUVhHRXN0V2lUZUJXYUhlSlFqUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC181" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - crypto.news</t>
+        </is>
+      </c>
+      <c r="AD181" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-20 15:39 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD181"/>
+  <dimension ref="A1:AD187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22779,6 +22779,762 @@
         </is>
       </c>
       <c r="AD181" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-09-20T15:37:05+00:00</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>4421.2002</v>
+      </c>
+      <c r="F182" t="n">
+        <v>4435.2002</v>
+      </c>
+      <c r="G182" t="n">
+        <v>4413.5</v>
+      </c>
+      <c r="H182" t="n">
+        <v>4424.8999</v>
+      </c>
+      <c r="I182" t="n">
+        <v>20009</v>
+      </c>
+      <c r="J182" t="n">
+        <v>4</v>
+      </c>
+      <c r="K182" t="n">
+        <v>40</v>
+      </c>
+      <c r="L182" t="n">
+        <v>-0.041</v>
+      </c>
+      <c r="M182" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="N182" t="n">
+        <v>40</v>
+      </c>
+      <c r="O182" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="P182" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="Q182" t="n">
+        <v>2.554</v>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S182" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T182" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U182" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V182" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W182" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X182" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y182" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z182" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA182" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AB182" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC182" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="AD182" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-09-20T15:37:05+00:00</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>95.98999999999999</v>
+      </c>
+      <c r="F183" t="n">
+        <v>96.17</v>
+      </c>
+      <c r="G183" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="H183" t="n">
+        <v>96.08</v>
+      </c>
+      <c r="I183" t="n">
+        <v>66441</v>
+      </c>
+      <c r="J183" t="n">
+        <v>4</v>
+      </c>
+      <c r="K183" t="n">
+        <v>40</v>
+      </c>
+      <c r="L183" t="n">
+        <v>-0.146</v>
+      </c>
+      <c r="M183" t="n">
+        <v>-0.153</v>
+      </c>
+      <c r="N183" t="n">
+        <v>40</v>
+      </c>
+      <c r="O183" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="P183" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="Q183" t="n">
+        <v>-1.684</v>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S183" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>Oil Shipping Market Prices Surge Tenfold in Half a Year: Unprecedented Wild Skyrocketing Growth - eu.36kr.com</t>
+        </is>
+      </c>
+      <c r="V183" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE1uV0tVdTN6dG41UjRzRHBrLV9TdVdzWmg4THFzNWZ0TjY1SEw5WnVrTFZlQjFDQ2VFR1JvMjN2amc4YVhGRmtjSzdBdGlxRnc5bEp3?oc=5</t>
+        </is>
+      </c>
+      <c r="W183" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X183" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y183" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z183" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA183" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB183" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE00VzJTYmxIdkNabVVzbnY3V2lyT0tMYkxJOTBOVEUxN0oydU5BYlB3T1FiUFd6MUdLcXpqb0l0WDdKRXZLbmdydlRwWERJbVV6RkdqNVQ0RDZqUHJoZEtia3lB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC183" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD183" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-09-20T15:37:05+00:00</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="F184" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="G184" t="n">
+        <v>100.165</v>
+      </c>
+      <c r="H184" t="n">
+        <v>100.215</v>
+      </c>
+      <c r="I184" t="n">
+        <v>0</v>
+      </c>
+      <c r="J184" t="n">
+        <v>4</v>
+      </c>
+      <c r="K184" t="n">
+        <v>39</v>
+      </c>
+      <c r="L184" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="M184" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="N184" t="n">
+        <v>39</v>
+      </c>
+      <c r="O184" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="P184" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="Q184" t="n">
+        <v>5.294</v>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S184" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T184" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V184" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W184" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X184" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y184" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z184" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA184" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - mufgresearch.com</t>
+        </is>
+      </c>
+      <c r="AB184" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC184" t="inlineStr">
+        <is>
+          <t>Dovish Fed Bets Pummel Dollar, Boost Gold Ahead of NFP - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD184" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPZDNJaUJnTUhOckR3ODFMRjN3M3QtZ1NzUmtvYnRUOVlyWEo2Nzg4d3l5Tkl4SFNRMVJCUnlNeGxUYm5NQkxpNmxEdzVpU3ZHTkhRUXh0bEdhNld2WHFBVmNCRTBEY2dsUkxqVlYtYTUwX21GR1JZNnZjazk2OXBjNW80dWo3Nmx5TXZYLUY0WkZLei14eWV4dDlkRGVheWM?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-09-20T15:37:05+00:00</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>7690</v>
+      </c>
+      <c r="F185" t="n">
+        <v>7729.25</v>
+      </c>
+      <c r="G185" t="n">
+        <v>7686.25</v>
+      </c>
+      <c r="H185" t="n">
+        <v>7712.5</v>
+      </c>
+      <c r="I185" t="n">
+        <v>474169</v>
+      </c>
+      <c r="J185" t="n">
+        <v>4</v>
+      </c>
+      <c r="K185" t="n">
+        <v>40</v>
+      </c>
+      <c r="L185" t="n">
+        <v>-0.052</v>
+      </c>
+      <c r="M185" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="N185" t="n">
+        <v>40</v>
+      </c>
+      <c r="O185" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="P185" t="n">
+        <v>-0.016</v>
+      </c>
+      <c r="Q185" t="n">
+        <v>4.365</v>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S185" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 2: Dell Surges 16% on Soaring AI Backlog - finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="T185" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQWTRuSVIyTFR2RTZveHRTN3hEWnBwSDl4T2J4ZHZPT01OdEYzWUk3MXZJZjNIc0tTMGYtYmFIYnkxd1dfVVVKTks0MmhzTlc5Z014VHVMMHJVMmZkWWlYVXdHWlczYWRQNzRyYk5leV9ncFBQVE1CbVdTbGNxclNhTy1JNEQwSlVmNjhjOGZrQXBLZlFG?oc=5</t>
+        </is>
+      </c>
+      <c r="U185" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="V185" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="W185" t="inlineStr">
+        <is>
+          <t>SanDisk SNDK Stock Breaks Resistance as NAND Demand Strengthens but Memory Risks Remain - FXLeaders</t>
+        </is>
+      </c>
+      <c r="X185" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPSENjb3VhWEFEQTd5a0xIM0hGQWFUcTJfU1QyZXZ1VTluMndraDNNSnh2Y25xS0RkWjZJR2JsNDlnRk1KOGFwM0c1NlE3RGN1ZkFhVjA0SXBDNVhISXp1YUxkVnhpUzJGeHVOVHMxVExMTHhmZ0pVMExkSnNNV3BwV2MxMlBYZ1NTMlhmQmpxajdLaUtKNTFKSXllNGc1RUgydm5kZ1RXd1c4VmRBSlA1RUFvMm96QTN3QzdfZWh4MTJ0amY3bk16MDR3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y185" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z185" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA185" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="AB185" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC185" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD185" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-09-20T15:37:05+00:00</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>29728</v>
+      </c>
+      <c r="F186" t="n">
+        <v>29993.25</v>
+      </c>
+      <c r="G186" t="n">
+        <v>29719.75</v>
+      </c>
+      <c r="H186" t="n">
+        <v>29917.25</v>
+      </c>
+      <c r="I186" t="n">
+        <v>144899</v>
+      </c>
+      <c r="J186" t="n">
+        <v>4</v>
+      </c>
+      <c r="K186" t="n">
+        <v>40</v>
+      </c>
+      <c r="L186" t="n">
+        <v>-0.122</v>
+      </c>
+      <c r="M186" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="N186" t="n">
+        <v>38</v>
+      </c>
+      <c r="O186" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="P186" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="Q186" t="n">
+        <v>1.017</v>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S186" t="inlineStr">
+        <is>
+          <t>Tech Stocks Surge as Momentum Traps the Bears - finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQMHF3WHVnXzlRVW1XNld1X2lsdEc1eGpfUk1TWFJ1UC1vV21DXzBuRUozRjdValF3MWpydG90UDNRZGxKU005b2w4alk0OXduTnZ1aXVBUC0xZXdNVFlpQWFHeTU3SjhDYl9hZnFGTlBQY0prTUJaVUdJMl9Gb1I3aEJ3dnBnd3ljN3UyaXpoWUZxMVBWdW1ZQ3lhLTVuZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U186" t="inlineStr">
+        <is>
+          <t>AI Server Stocks Rally as the Hardware Bid Broadens: Hewlett Packard Enterprise Jumps 9%, Super Micro Climbs 6%, Dell Rises 3% - finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="V186" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNbUk4OGEtN1VjNjBIT1NxMGlpa2tEVC1sTExGOXpKUUpyc1VBX254dVlrTDEtSXN6VkxYM004OFY5eWlObFAwRV84NEVXSlh4WVhtRzFhTXV2eExDcjMxc2JDY1g3TW1DYldOanJmRFJ5eFozYzVLOXVyUExuRDMyak42MnlIcUNJaXRoWGQzbFhGNXNvekxWajhDZGs?oc=5</t>
+        </is>
+      </c>
+      <c r="W186" t="inlineStr">
+        <is>
+          <t>Tesla Swing Trade for NASDAQ:TSLA by Vasileios_Kairaktidis - TradingView</t>
+        </is>
+      </c>
+      <c r="X186" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE5RRTFlWVkxVDdrUUhKSE1MY3I0QWUtdy00WmpqVi1SZkhybUhIRkcwWTRBd2RSNjZHSGF0Ujd5RTV3dGhWWUxYa05tMjdlT2NQNkRaTDV3MHZoeFNucTZ1ZUU0WnA1ajhmdGs2ZHVKaFVnczRw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y186" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z186" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA186" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB186" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC186" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD186" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-09-20T15:37:05+00:00</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>80430.0469</v>
+      </c>
+      <c r="F187" t="n">
+        <v>80870.13280000001</v>
+      </c>
+      <c r="G187" t="n">
+        <v>80285.7812</v>
+      </c>
+      <c r="H187" t="n">
+        <v>80767.5312</v>
+      </c>
+      <c r="I187" t="n">
+        <v>1064646656</v>
+      </c>
+      <c r="J187" t="n">
+        <v>4</v>
+      </c>
+      <c r="K187" t="n">
+        <v>38</v>
+      </c>
+      <c r="L187" t="n">
+        <v>-0.039</v>
+      </c>
+      <c r="M187" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="N187" t="n">
+        <v>37</v>
+      </c>
+      <c r="O187" t="n">
+        <v>0.421</v>
+      </c>
+      <c r="P187" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="Q187" t="n">
+        <v>7.539</v>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S187" t="inlineStr">
+        <is>
+          <t>Best Crypto Presale To Buy Now: Remittix Gains Momentum as Institutional Crypto Access Expands - TechBullion</t>
+        </is>
+      </c>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPRXk2bEdHNHZEcVhCZXBLX3BnOHQ2SjZQdEhkNVJUZ3o3NW5wMDFNWVphXzVkUkVBcDBMMHAxWEc1cW1FMlEtUDFCY3BxTHAwcmZrOEhoQ1JBcU5tc1lMZlRUTjIxU1JUM2VuTXRIUUZPQW5VckhWWkJweHphWGxWaWZQLVI4bmtDMHpRZXZjNzUteG1WNWo2TzR2SWhkdWpkLWt3M3FpQlF6X0VHT2dvUllsdWVuYVRRMmc?oc=5</t>
+        </is>
+      </c>
+      <c r="U187" t="inlineStr">
+        <is>
+          <t>XRP Surges 6.9% as Bitcoin Rebound Reopens Door to Golden Cross - Decrypt</t>
+        </is>
+      </c>
+      <c r="V187" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ucm9hYldRNWMyRDBjREdzNUthTTVMa3RZcEY5WUdWWjNmOUMya0JSemRqUXE4Q2dNd3JpcFB1ejViT3ZvUWVMUGt5MDlTaHVXd0NVbE9vb0tQYU9Qd3o3czJBRFhBWmI4NGJlaC1sWjQxM3haR3NBM1lWRmJpZ9IBhgFBVV95cUxOM1RxOHBBS0hRVXpGLTlUS3JzUjhIYmFjTG1vdFZiWDhRUE9PV2VlWnBGMmRFMmNpWFhIcjdoeG9SOWJaZ0hwT2N6NG9rbkJuS3g2R01aMlo0allaRDh2WFdxY05neGlaejlwSUtIVGlYRVA1MlZOTUxHR3g0b2UweV9oenZoZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W187" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 5% to top $80,000 as investors look past Clarity Act's failure - finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="X187" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQQXFtZ2hIbkZNVDRDVlhiN2h2LUdSWHpNSFRscjBFZTFZRUdmNDZlaHdiaFJ1Qm5FY1E1bHlwQXB0bEVCNTBpanA4Vkp5bjM1Q3gwSVRfQ1hjZWpWRWhZcDBWZVpfQTNybGRwZ0tyeU9GS0czMl8tdFQybFlUZkNNWlJucnBNa3U2LTMtV3dDa1dUV3NneV83enJYdUgtOVFCa2JjTEc1VXVMdU90NU9XVktEYW1GSm9IM0RoNXZWN0QwUGprYVJ3ZjVn?oc=5</t>
+        </is>
+      </c>
+      <c r="Y187" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="Z187" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA187" t="inlineStr">
+        <is>
+          <t>Bitcoin Is 11 Days From Its First Winning Quarter in a Year. What Needs to Hold Until September 30? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB187" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQTU9EX0F6eUx0b0Q4cVhJMEtNLU92NXJPTmNvSGk2VVJmamw2dEhRdVN6Mi1xWThSbWY1MFRoVjlXWWVFUTdZcm1vajFTY3BXM0k0OHJYaFRZNmZ6dzZjRWFzUjFaeUstUlo5emkxNVhYay10WTJKT1JpbnZEM2xMUExDZ2YzM1dBWTYtbEpqS0pBUTRzUEFKeENRckJONVdnRTFGWm1mVUNOckc2dm4wSHRlQlhrcS1XUGlUQS10SjhlbGVxWFFxXy01VU1lMUNtMXdiX1U5OXBZUVhHRXN0V2lUZUJXYUhlSlFqUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC187" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - Crypto News</t>
+        </is>
+      </c>
+      <c r="AD187" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-20 18:34 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD187"/>
+  <dimension ref="A1:AD193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23535,6 +23535,762 @@
         </is>
       </c>
       <c r="AD187" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-09-20T18:32:42+00:00</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>4421.2002</v>
+      </c>
+      <c r="F188" t="n">
+        <v>4435.2002</v>
+      </c>
+      <c r="G188" t="n">
+        <v>4413.5</v>
+      </c>
+      <c r="H188" t="n">
+        <v>4424.8999</v>
+      </c>
+      <c r="I188" t="n">
+        <v>20009</v>
+      </c>
+      <c r="J188" t="n">
+        <v>4</v>
+      </c>
+      <c r="K188" t="n">
+        <v>39</v>
+      </c>
+      <c r="L188" t="n">
+        <v>-0.049</v>
+      </c>
+      <c r="M188" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="N188" t="n">
+        <v>40</v>
+      </c>
+      <c r="O188" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="P188" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="Q188" t="n">
+        <v>-1.206</v>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S188" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T188" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U188" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V188" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W188" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X188" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y188" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z188" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA188" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AB188" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC188" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AD188" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-09-20T18:32:42+00:00</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E189" t="n">
+        <v>95.98999999999999</v>
+      </c>
+      <c r="F189" t="n">
+        <v>96.17</v>
+      </c>
+      <c r="G189" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="H189" t="n">
+        <v>96.08</v>
+      </c>
+      <c r="I189" t="n">
+        <v>66441</v>
+      </c>
+      <c r="J189" t="n">
+        <v>4</v>
+      </c>
+      <c r="K189" t="n">
+        <v>40</v>
+      </c>
+      <c r="L189" t="n">
+        <v>-0.158</v>
+      </c>
+      <c r="M189" t="n">
+        <v>-0.171</v>
+      </c>
+      <c r="N189" t="n">
+        <v>40</v>
+      </c>
+      <c r="O189" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="P189" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="Q189" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S189" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T189" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U189" t="inlineStr">
+        <is>
+          <t>Oil Shipping Market Prices Surge Tenfold in Half a Year: Unprecedented Wild Skyrocketing Growth - 36氪</t>
+        </is>
+      </c>
+      <c r="V189" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE1uV0tVdTN6dG41UjRzRHBrLV9TdVdzWmg4THFzNWZ0TjY1SEw5WnVrTFZlQjFDQ2VFR1JvMjN2amc4YVhGRmtjSzdBdGlxRnc5bEp3?oc=5</t>
+        </is>
+      </c>
+      <c r="W189" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X189" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y189" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z189" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE00VzJTYmxIdkNabVVzbnY3V2lyT0tMYkxJOTBOVEUxN0oydU5BYlB3T1FiUFd6MUdLcXpqb0l0WDdKRXZLbmdydlRwWERJbVV6RkdqNVQ0RDZqUHJoZEtia3lB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA189" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB189" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC189" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD189" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-09-20T18:32:42+00:00</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="F190" t="n">
+        <v>100.298</v>
+      </c>
+      <c r="G190" t="n">
+        <v>100.165</v>
+      </c>
+      <c r="H190" t="n">
+        <v>100.215</v>
+      </c>
+      <c r="I190" t="n">
+        <v>0</v>
+      </c>
+      <c r="J190" t="n">
+        <v>4</v>
+      </c>
+      <c r="K190" t="n">
+        <v>39</v>
+      </c>
+      <c r="L190" t="n">
+        <v>0.103</v>
+      </c>
+      <c r="M190" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="N190" t="n">
+        <v>40</v>
+      </c>
+      <c r="O190" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="P190" t="n">
+        <v>-0.037</v>
+      </c>
+      <c r="Q190" t="n">
+        <v>2.086</v>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U190" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V190" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W190" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X190" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y190" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z190" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA190" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB190" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC190" t="inlineStr">
+        <is>
+          <t>FX Daily: Fed hold can hit the dollar today - think.ing.com</t>
+        </is>
+      </c>
+      <c r="AD190" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE91QWFPVUVXdGYyVGFxekZhSXBLNzFWN2xfWkJVRXNud05nSzJPQXpwN1hjbzJxZ0ZWLWdmTWhXbzI4NFRXdnpobUc2MllDT1VFQWtFbzhiZ1kzX0Z2c3FGal9nZF91Y19ISENwR1RVdnBRVVVhc0EtY3BmOEZKU1k?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-09-20T18:32:42+00:00</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>7690</v>
+      </c>
+      <c r="F191" t="n">
+        <v>7729.25</v>
+      </c>
+      <c r="G191" t="n">
+        <v>7686.25</v>
+      </c>
+      <c r="H191" t="n">
+        <v>7712.5</v>
+      </c>
+      <c r="I191" t="n">
+        <v>474169</v>
+      </c>
+      <c r="J191" t="n">
+        <v>4</v>
+      </c>
+      <c r="K191" t="n">
+        <v>40</v>
+      </c>
+      <c r="L191" t="n">
+        <v>-0.081</v>
+      </c>
+      <c r="M191" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="N191" t="n">
+        <v>40</v>
+      </c>
+      <c r="O191" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="P191" t="n">
+        <v>-0.036</v>
+      </c>
+      <c r="Q191" t="n">
+        <v>3.176</v>
+      </c>
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S191" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 2: Dell Surges 16% on Soaring AI Backlog - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T191" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQWTRuSVIyTFR2RTZveHRTN3hEWnBwSDl4T2J4ZHZPT01OdEYzWUk3MXZJZjNIc0tTMGYtYmFIYnkxd1dfVVVKTks0MmhzTlc5Z014VHVMMHJVMmZkWWlYVXdHWlczYWRQNzRyYk5leV9ncFBQVE1CbVdTbGNxclNhTy1JNEQwSlVmNjhjOGZrQXBLZlFG?oc=5</t>
+        </is>
+      </c>
+      <c r="U191" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="V191" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="W191" t="inlineStr">
+        <is>
+          <t>Dow surges to record close after a fresh tech rally and a plunge in oil prices - Business Insider</t>
+        </is>
+      </c>
+      <c r="X191" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOS0hLS2NLYi1nYlZnTmRJNTRtQXAyZUh5MExFZUVXcEtOTEhzVF9zeHozLThnVHVETGtwMVBFZFBUb3dVaDJlMmtmTUd6Y2ZmUVhMZjRxck41ZEJDZFNqSG5PRm96VXR6bE9tLWlybXBqVWh4NjRUSUJIcFVjdE9xRml2YWJVYTZvMmM4aTQ5bw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y191" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z191" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA191" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="AB191" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC191" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD191" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-09-20T18:32:42+00:00</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>29728</v>
+      </c>
+      <c r="F192" t="n">
+        <v>29993.25</v>
+      </c>
+      <c r="G192" t="n">
+        <v>29719.75</v>
+      </c>
+      <c r="H192" t="n">
+        <v>29917.25</v>
+      </c>
+      <c r="I192" t="n">
+        <v>144899</v>
+      </c>
+      <c r="J192" t="n">
+        <v>4</v>
+      </c>
+      <c r="K192" t="n">
+        <v>40</v>
+      </c>
+      <c r="L192" t="n">
+        <v>-0.144</v>
+      </c>
+      <c r="M192" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="N192" t="n">
+        <v>39</v>
+      </c>
+      <c r="O192" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="P192" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="Q192" t="n">
+        <v>-0.452</v>
+      </c>
+      <c r="R192" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S192" t="inlineStr">
+        <is>
+          <t>Samsung Electronics, SK hynix surge as U.S. tech stocks rally - 매일경제</t>
+        </is>
+      </c>
+      <c r="T192" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE55T0VWYmJHT1k0U1U3bldzSXpxTFNoNUVobHNVSHpjVmFhTGQzQUR3b0VDWkpvYlpHR0tFOWM2WXREa2U5NzQwbzE5TVFYT1BrSERZRjFhQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U192" t="inlineStr">
+        <is>
+          <t>AI Server Stocks Rally as the Hardware Bid Broadens: Hewlett Packard Enterprise Jumps 9%, Super Micro Climbs 6%, Dell Rises 3% - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="V192" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNbUk4OGEtN1VjNjBIT1NxMGlpa2tEVC1sTExGOXpKUUpyc1VBX254dVlrTDEtSXN6VkxYM004OFY5eWlObFAwRV84NEVXSlh4WVhtRzFhTXV2eExDcjMxc2JDY1g3TW1DYldOanJmRFJ5eFozYzVLOXVyUExuRDMyak42MnlIcUNJaXRoWGQzbFhGNXNvekxWajhDZGs?oc=5</t>
+        </is>
+      </c>
+      <c r="W192" t="inlineStr">
+        <is>
+          <t>Tesla Swing Trade for NASDAQ:TSLA by Vasileios_Kairaktidis - TradingView</t>
+        </is>
+      </c>
+      <c r="X192" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE5RRTFlWVkxVDdrUUhKSE1MY3I0QWUtdy00WmpqVi1SZkhybUhIRkcwWTRBd2RSNjZHSGF0Ujd5RTV3dGhWWUxYa05tMjdlT2NQNkRaTDV3MHZoeFNucTZ1ZUU0WnA1ajhmdGs2ZHVKaFVnczRw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y192" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z192" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA192" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB192" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC192" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD192" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-09-20T18:32:42+00:00</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E193" t="n">
+        <v>80639.5938</v>
+      </c>
+      <c r="F193" t="n">
+        <v>81472.03909999999</v>
+      </c>
+      <c r="G193" t="n">
+        <v>80635.07030000001</v>
+      </c>
+      <c r="H193" t="n">
+        <v>81221.99219999999</v>
+      </c>
+      <c r="I193" t="n">
+        <v>3645935616</v>
+      </c>
+      <c r="J193" t="n">
+        <v>4</v>
+      </c>
+      <c r="K193" t="n">
+        <v>37</v>
+      </c>
+      <c r="L193" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="M193" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="N193" t="n">
+        <v>37</v>
+      </c>
+      <c r="O193" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P193" t="n">
+        <v>-0.023</v>
+      </c>
+      <c r="Q193" t="n">
+        <v>12.404</v>
+      </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S193" t="inlineStr">
+        <is>
+          <t>Best Crypto Presale To Buy Now: Remittix Gains Momentum as Institutional Crypto Access Expands - TechBullion</t>
+        </is>
+      </c>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPRXk2bEdHNHZEcVhCZXBLX3BnOHQ2SjZQdEhkNVJUZ3o3NW5wMDFNWVphXzVkUkVBcDBMMHAxWEc1cW1FMlEtUDFCY3BxTHAwcmZrOEhoQ1JBcU5tc1lMZlRUTjIxU1JUM2VuTXRIUUZPQW5VckhWWkJweHphWGxWaWZQLVI4bmtDMHpRZXZjNzUteG1WNWo2TzR2SWhkdWpkLWt3M3FpQlF6X0VHT2dvUllsdWVuYVRRMmc?oc=5</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>XRP Surges 6.9% as Bitcoin Rebound Reopens Door to Golden Cross - Decrypt</t>
+        </is>
+      </c>
+      <c r="V193" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ucm9hYldRNWMyRDBjREdzNUthTTVMa3RZcEY5WUdWWjNmOUMya0JSemRqUXE4Q2dNd3JpcFB1ejViT3ZvUWVMUGt5MDlTaHVXd0NVbE9vb0tQYU9Qd3o3czJBRFhBWmI4NGJlaC1sWjQxM3haR3NBM1lWRmJpZ9IBhgFBVV95cUxOM1RxOHBBS0hRVXpGLTlUS3JzUjhIYmFjTG1vdFZiWDhRUE9PV2VlWnBGMmRFMmNpWFhIcjdoeG9SOWJaZ0hwT2N6NG9rbkJuS3g2R01aMlo0allaRDh2WFdxY05neGlaejlwSUtIVGlYRVA1MlZOTUxHR3g0b2UweV9oenZoZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W193" t="inlineStr">
+        <is>
+          <t>BlackRock clients buy $108M Bitcoin via IBIT as institutional demand stays strong - Pluang</t>
+        </is>
+      </c>
+      <c r="X193" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQbHV3QW80d1E2TzFjbVQ0QkltRlg5dmJ5eHJOVTFpUEstdWNPMWtnNG9qUUxxazBBMV91bVVjNnRJczRzRnJGV2FrLVpwX0xmdUljVnVETE9BelVrcklzc2M4SnoySlFuOXpLWk13d25qRGZuTmtTMlJXenZHNGNpYmxRbjkwSFRTMXdtS3lPQkRSQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y193" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="Z193" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA193" t="inlineStr">
+        <is>
+          <t>Bitcoin Is 11 Days From Its First Winning Quarter in a Year. What Needs to Hold Until September 30? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB193" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQTU9EX0F6eUx0b0Q4cVhJMEtNLU92NXJPTmNvSGk2VVJmamw2dEhRdVN6Mi1xWThSbWY1MFRoVjlXWWVFUTdZcm1vajFTY3BXM0k0OHJYaFRZNmZ6dzZjRWFzUjFaeUstUlo5emkxNVhYay10WTJKT1JpbnZEM2xMUExDZ2YzM1dBWTYtbEpqS0pBUTRzUEFKeENRckJONVdnRTFGWm1mVUNOckc2dm4wSHRlQlhrcS1XUGlUQS10SjhlbGVxWFFxXy01VU1lMUNtMXdiX1U5OXBZUVhHRXN0V2lUZUJXYUhlSlFqUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC193" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - Crypto News</t>
+        </is>
+      </c>
+      <c r="AD193" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-20 22:17 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD193"/>
+  <dimension ref="A1:AD199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24291,6 +24291,762 @@
         </is>
       </c>
       <c r="AD193" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-09-20T22:15:42+00:00</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>GCJ27.CMX</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>4464.5</v>
+      </c>
+      <c r="F194" t="n">
+        <v>4503.3999</v>
+      </c>
+      <c r="G194" t="n">
+        <v>4464.5</v>
+      </c>
+      <c r="H194" t="n">
+        <v>4498.5</v>
+      </c>
+      <c r="I194" t="n">
+        <v>1558</v>
+      </c>
+      <c r="J194" t="n">
+        <v>4</v>
+      </c>
+      <c r="K194" t="n">
+        <v>39</v>
+      </c>
+      <c r="L194" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="M194" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="N194" t="n">
+        <v>40</v>
+      </c>
+      <c r="O194" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="P194" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="Q194" t="n">
+        <v>-0.471</v>
+      </c>
+      <c r="R194" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S194" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T194" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U194" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V194" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W194" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X194" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y194" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z194" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA194" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AB194" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC194" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AD194" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-09-20T22:15:42+00:00</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E195" t="n">
+        <v>96</v>
+      </c>
+      <c r="F195" t="n">
+        <v>96.14</v>
+      </c>
+      <c r="G195" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="H195" t="n">
+        <v>96.08</v>
+      </c>
+      <c r="I195" t="n">
+        <v>45232</v>
+      </c>
+      <c r="J195" t="n">
+        <v>4</v>
+      </c>
+      <c r="K195" t="n">
+        <v>40</v>
+      </c>
+      <c r="L195" t="n">
+        <v>-0.134</v>
+      </c>
+      <c r="M195" t="n">
+        <v>-0.155</v>
+      </c>
+      <c r="N195" t="n">
+        <v>40</v>
+      </c>
+      <c r="O195" t="n">
+        <v>0.103</v>
+      </c>
+      <c r="P195" t="n">
+        <v>-0.065</v>
+      </c>
+      <c r="Q195" t="n">
+        <v>-0.608</v>
+      </c>
+      <c r="R195" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S195" t="inlineStr">
+        <is>
+          <t>Gold gains more than 2% on weaker dollar, easing oil prices - CNBC</t>
+        </is>
+      </c>
+      <c r="T195" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaG9YazhGMnhxa0V4TFlVbVFjSldNRkUwTUdRZV9FY0RQXzlTTFMzekN4WlVrMzdESVpZbmNNV0IwUXZDeGZCYmljN0pGTUNnZWxZdWRiSmh5a3VjcDB5a3hlbzhUclBCZTB6eVdhWGRWR2dBSE9Nc19hX3pPN0JfbThqbnI1dzJwcVJRTUdsQjBTYWxobkgzM9IBngFBVV95cUxPYzNuR1dpWnNWeDRxTWJCY1g3ZXR0T2ZlOWdMSXB1TGNYR3VBOHdyajR4ekxFalhIUk9hUGlLM1I4RjZXdl9NS1lUeVFvRDBpQjNYbU9uOG9XNkxnc2FsZWhaMXAtN3djMkNmTnVvSktqMV9uckpVRVlYTWJQbWtOT2U3X2F2b196ZjhsLVljSHNiaTAycUtsOGhTT192UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U195" t="inlineStr">
+        <is>
+          <t>Oil Shipping Market Prices Surge Tenfold in Half a Year: Unprecedented Wild Skyrocketing Growth - 36Kr</t>
+        </is>
+      </c>
+      <c r="V195" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE1uV0tVdTN6dG41UjRzRHBrLV9TdVdzWmg4THFzNWZ0TjY1SEw5WnVrTFZlQjFDQ2VFR1JvMjN2amc4YVhGRmtjSzdBdGlxRnc5bEp3?oc=5</t>
+        </is>
+      </c>
+      <c r="W195" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X195" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y195" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z195" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE00VzJTYmxIdkNabVVzbnY3V2lyT0tMYkxJOTBOVEUxN0oydU5BYlB3T1FiUFd6MUdLcXpqb0l0WDdKRXZLbmdydlRwWERJbVV6RkdqNVQ0RDZqUHJoZEtia3lB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA195" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB195" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC195" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD195" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-09-20T22:15:42+00:00</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>100.236</v>
+      </c>
+      <c r="F196" t="n">
+        <v>100.252</v>
+      </c>
+      <c r="G196" t="n">
+        <v>100.165</v>
+      </c>
+      <c r="H196" t="n">
+        <v>100.21</v>
+      </c>
+      <c r="I196" t="n">
+        <v>0</v>
+      </c>
+      <c r="J196" t="n">
+        <v>4</v>
+      </c>
+      <c r="K196" t="n">
+        <v>39</v>
+      </c>
+      <c r="L196" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="M196" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="N196" t="n">
+        <v>40</v>
+      </c>
+      <c r="O196" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="P196" t="n">
+        <v>-0.041</v>
+      </c>
+      <c r="Q196" t="n">
+        <v>2.621</v>
+      </c>
+      <c r="R196" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S196" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T196" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U196" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V196" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W196" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens as BOJ Dissent Clouds Rate-Hike Outlook - globalbankingandfinance.com</t>
+        </is>
+      </c>
+      <c r="X196" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPcDhOdGkwRnVsTWlBeXRTNXRfTENuNjcwbFNGMFVXMllsWTJVTXRSVVA0UC1tSGQyR3ljb1FxRUdCaDlDam5Lc2RFSUZLMWhzOUhlRW9OeDJObWg1MDNReWVZUXl1UF9Dc1lZT1NkWDBqU3hPYjNMTXlKM21qUjE0UTQxZktkSzJHSXpfMWFTOEo?oc=5</t>
+        </is>
+      </c>
+      <c r="Y196" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z196" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA196" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB196" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC196" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD196" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-09-20T22:15:42+00:00</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>7694.75</v>
+      </c>
+      <c r="F197" t="n">
+        <v>7729.25</v>
+      </c>
+      <c r="G197" t="n">
+        <v>7693</v>
+      </c>
+      <c r="H197" t="n">
+        <v>7712.5</v>
+      </c>
+      <c r="I197" t="n">
+        <v>414340</v>
+      </c>
+      <c r="J197" t="n">
+        <v>4</v>
+      </c>
+      <c r="K197" t="n">
+        <v>40</v>
+      </c>
+      <c r="L197" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="M197" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="N197" t="n">
+        <v>40</v>
+      </c>
+      <c r="O197" t="n">
+        <v>0.242</v>
+      </c>
+      <c r="P197" t="n">
+        <v>-0.052</v>
+      </c>
+      <c r="Q197" t="n">
+        <v>4.866</v>
+      </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S197" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="U197" t="inlineStr">
+        <is>
+          <t>SanDisk SNDK Stock Breaks Resistance as NAND Demand Strengthens but Memory Risks Remain - FXLeaders</t>
+        </is>
+      </c>
+      <c r="V197" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPSENjb3VhWEFEQTd5a0xIM0hGQWFUcTJfU1QyZXZ1VTluMndraDNNSnh2Y25xS0RkWjZJR2JsNDlnRk1KOGFwM0c1NlE3RGN1ZkFhVjA0SXBDNVhISXp1YUxkVnhpUzJGeHVOVHMxVExMTHhmZ0pVMExkSnNNV3BwV2MxMlBYZ1NTMlhmQmpxajdLaUtKNTFKSXllNGc1RUgydm5kZ1RXd1c4VmRBSlA1RUFvMm96QTN3QzdfZWh4MTJ0amY3bk16MDR3?oc=5</t>
+        </is>
+      </c>
+      <c r="W197" t="inlineStr">
+        <is>
+          <t>Dow surges to record close after a fresh tech rally and a plunge in oil prices - Business Insider</t>
+        </is>
+      </c>
+      <c r="X197" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOS0hLS2NLYi1nYlZnTmRJNTRtQXAyZUh5MExFZUVXcEtOTEhzVF9zeHozLThnVHVETGtwMVBFZFBUb3dVaDJlMmtmTUd6Y2ZmUVhMZjRxck41ZEJDZFNqSG5PRm96VXR6bE9tLWlybXBqVWh4NjRUSUJIcFVjdE9xRml2YWJVYTZvMmM4aTQ5bw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y197" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z197" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA197" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="AB197" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC197" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD197" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-09-20T22:15:42+00:00</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>29763</v>
+      </c>
+      <c r="F198" t="n">
+        <v>29993.25</v>
+      </c>
+      <c r="G198" t="n">
+        <v>29748</v>
+      </c>
+      <c r="H198" t="n">
+        <v>29917.25</v>
+      </c>
+      <c r="I198" t="n">
+        <v>119393</v>
+      </c>
+      <c r="J198" t="n">
+        <v>4</v>
+      </c>
+      <c r="K198" t="n">
+        <v>40</v>
+      </c>
+      <c r="L198" t="n">
+        <v>-0.097</v>
+      </c>
+      <c r="M198" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="N198" t="n">
+        <v>38</v>
+      </c>
+      <c r="O198" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="P198" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="Q198" t="n">
+        <v>1.542</v>
+      </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S198" t="inlineStr">
+        <is>
+          <t>German Medical Cannabis Sales Boost High Tide To Record Performance (NASDAQ:HITI) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPWk4xOHF4YTkxMlliTXAyRDl4bERlWU1ZcFR5ZDYyR1BvYnZUdXNrNXNxX0lVMVBPR0JVbk4wVUhLUDNzbDlrdndfRzRLUlZrWUY4aVVlZ0tneUtFRjF3M2ZnME96RVc3b3VrLWdKQWpDNFp6RmQtSHZLOXlNZzNqTHpQWDByV2JRM3JQcXI4QVBIdVA3enRnMWkzMUtfR29rZUNpcGRsXzZzXzZY?oc=5</t>
+        </is>
+      </c>
+      <c r="U198" t="inlineStr">
+        <is>
+          <t>Samsung Electronics, SK hynix surge as U.S. tech stocks rally - 매일경제</t>
+        </is>
+      </c>
+      <c r="V198" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE55T0VWYmJHT1k0U1U3bldzSXpxTFNoNUVobHNVSHpjVmFhTGQzQUR3b0VDWkpvYlpHR0tFOWM2WXREa2U5NzQwbzE5TVFYT1BrSERZRjFhQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W198" t="inlineStr">
+        <is>
+          <t>AI Server Stocks Rally as the Hardware Bid Broadens: Hewlett Packard Enterprise Jumps 9%, Super Micro Climbs 6%, Dell Rises 3% - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X198" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNbUk4OGEtN1VjNjBIT1NxMGlpa2tEVC1sTExGOXpKUUpyc1VBX254dVlrTDEtSXN6VkxYM004OFY5eWlObFAwRV84NEVXSlh4WVhtRzFhTXV2eExDcjMxc2JDY1g3TW1DYldOanJmRFJ5eFozYzVLOXVyUExuRDMyak42MnlIcUNJaXRoWGQzbFhGNXNvekxWajhDZGs?oc=5</t>
+        </is>
+      </c>
+      <c r="Y198" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="Z198" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA198" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AB198" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+      <c r="AC198" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="AD198" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-09-20T22:15:42+00:00</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>81030</v>
+      </c>
+      <c r="F199" t="n">
+        <v>81279.52340000001</v>
+      </c>
+      <c r="G199" t="n">
+        <v>80605.4219</v>
+      </c>
+      <c r="H199" t="n">
+        <v>81134.67969999999</v>
+      </c>
+      <c r="I199" t="n">
+        <v>802177024</v>
+      </c>
+      <c r="J199" t="n">
+        <v>4</v>
+      </c>
+      <c r="K199" t="n">
+        <v>37</v>
+      </c>
+      <c r="L199" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="M199" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="N199" t="n">
+        <v>37</v>
+      </c>
+      <c r="O199" t="n">
+        <v>0.351</v>
+      </c>
+      <c r="P199" t="n">
+        <v>-0.019</v>
+      </c>
+      <c r="Q199" t="n">
+        <v>9.795999999999999</v>
+      </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S199" t="inlineStr">
+        <is>
+          <t>XRP Surges 6.9% as Bitcoin Rebound Reopens Door to Golden Cross - Decrypt</t>
+        </is>
+      </c>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ucm9hYldRNWMyRDBjREdzNUthTTVMa3RZcEY5WUdWWjNmOUMya0JSemRqUXE4Q2dNd3JpcFB1ejViT3ZvUWVMUGt5MDlTaHVXd0NVbE9vb0tQYU9Qd3o3czJBRFhBWmI4NGJlaC1sWjQxM3haR3NBM1lWRmJpZ9IBhgFBVV95cUxOM1RxOHBBS0hRVXpGLTlUS3JzUjhIYmFjTG1vdFZiWDhRUE9PV2VlWnBGMmRFMmNpWFhIcjdoeG9SOWJaZ0hwT2N6NG9rbkJuS3g2R01aMlo0allaRDh2WFdxY05neGlaejlwSUtIVGlYRVA1MlZOTUxHR3g0b2UweV9oenZoZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U199" t="inlineStr">
+        <is>
+          <t>BlackRock clients buy $108M Bitcoin via IBIT as institutional demand stays strong - pluang.com</t>
+        </is>
+      </c>
+      <c r="V199" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQbHV3QW80d1E2TzFjbVQ0QkltRlg5dmJ5eHJOVTFpUEstdWNPMWtnNG9qUUxxazBBMV91bVVjNnRJczRzRnJGV2FrLVpwX0xmdUljVnVETE9BelVrcklzc2M4SnoySlFuOXpLWk13d25qRGZuTmtTMlJXenZHNGNpYmxRbjkwSFRTMXdtS3lPQkRSQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W199" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Surges Over $81,000 Despite Clarity Act Fail and Interest Rate Hike - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="X199" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE5DLVVDZWFpWWxfQzVoanF6dkl5QUc1cWkxZHNwWC1maFBiUG4wNjI4STZJRmRvZ01TNXE5emRHQ0VBdHpPb054TWhFUHhqS2sxU2k0SU1weVpWVG80VjlzSDdhd0NWNjRoNXExU3Izd2I2VHp3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y199" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="Z199" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA199" t="inlineStr">
+        <is>
+          <t>Bitcoin Is 11 Days From Its First Winning Quarter in a Year. What Needs to Hold Until September 30? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB199" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQTU9EX0F6eUx0b0Q4cVhJMEtNLU92NXJPTmNvSGk2VVJmamw2dEhRdVN6Mi1xWThSbWY1MFRoVjlXWWVFUTdZcm1vajFTY3BXM0k0OHJYaFRZNmZ6dzZjRWFzUjFaeUstUlo5emkxNVhYay10WTJKT1JpbnZEM2xMUExDZ2YzM1dBWTYtbEpqS0pBUTRzUEFKeENRckJONVdnRTFGWm1mVUNOckc2dm4wSHRlQlhrcS1XUGlUQS10SjhlbGVxWFFxXy01VU1lMUNtMXdiX1U5OXBZUVhHRXN0V2lUZUJXYUhlSlFqUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC199" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - Crypto News</t>
+        </is>
+      </c>
+      <c r="AD199" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-21 03:48 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD199"/>
+  <dimension ref="A1:AD205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25047,6 +25047,762 @@
         </is>
       </c>
       <c r="AD199" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-09-21T03:46:11+00:00</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>4411.5</v>
+      </c>
+      <c r="F200" t="n">
+        <v>4422.1001</v>
+      </c>
+      <c r="G200" t="n">
+        <v>4396.3999</v>
+      </c>
+      <c r="H200" t="n">
+        <v>4402.3999</v>
+      </c>
+      <c r="I200" t="n">
+        <v>18068</v>
+      </c>
+      <c r="J200" t="n">
+        <v>4</v>
+      </c>
+      <c r="K200" t="n">
+        <v>39</v>
+      </c>
+      <c r="L200" t="n">
+        <v>-0.028</v>
+      </c>
+      <c r="M200" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="N200" t="n">
+        <v>40</v>
+      </c>
+      <c r="O200" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P200" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="Q200" t="n">
+        <v>-0.042</v>
+      </c>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S200" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T200" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="U200" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="V200" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W200" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="X200" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y200" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z200" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA200" t="inlineStr">
+        <is>
+          <t>Gold ETF Trading Jumps 83%, Holdings Climb To Record 4,189 Tonnes - Yellow.com</t>
+        </is>
+      </c>
+      <c r="AB200" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBjVEpXV05CRmJaSnAzU2NsQzJYV3pnQno1UzE2M05HdVpUMVNoMXVfNkU0UG1MYXlJQi1QUU5RMDc4MlRVLWktYi1OMUczbE80U19lLUxNV0hfTzRXa2lNRUhpU25lbnowNFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC200" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - english.nv.ua</t>
+        </is>
+      </c>
+      <c r="AD200" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-09-21T03:46:11+00:00</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E201" t="n">
+        <v>95.66</v>
+      </c>
+      <c r="F201" t="n">
+        <v>95.86</v>
+      </c>
+      <c r="G201" t="n">
+        <v>93.58</v>
+      </c>
+      <c r="H201" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="I201" t="n">
+        <v>22478</v>
+      </c>
+      <c r="J201" t="n">
+        <v>4</v>
+      </c>
+      <c r="K201" t="n">
+        <v>40</v>
+      </c>
+      <c r="L201" t="n">
+        <v>-0.193</v>
+      </c>
+      <c r="M201" t="n">
+        <v>-0.177</v>
+      </c>
+      <c r="N201" t="n">
+        <v>40</v>
+      </c>
+      <c r="O201" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="P201" t="n">
+        <v>-0.08500000000000001</v>
+      </c>
+      <c r="Q201" t="n">
+        <v>-0.152</v>
+      </c>
+      <c r="R201" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S201" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T201" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U201" t="inlineStr">
+        <is>
+          <t>Oil Shipping Market Prices Surge Tenfold in Half a Year: Unprecedented Wild Skyrocketing Growth - 36Kr</t>
+        </is>
+      </c>
+      <c r="V201" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE1uV0tVdTN6dG41UjRzRHBrLV9TdVdzWmg4THFzNWZ0TjY1SEw5WnVrTFZlQjFDQ2VFR1JvMjN2amc4YVhGRmtjSzdBdGlxRnc5bEp3?oc=5</t>
+        </is>
+      </c>
+      <c r="W201" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X201" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y201" t="inlineStr">
+        <is>
+          <t>Market Recap: Semiconductor Stocks Surge as Oil Prices Drop Belo - GuruFocus</t>
+        </is>
+      </c>
+      <c r="Z201" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQVUhnUEpoS21NazZnR2F2dnQyU2JaTmNzWFc1VEdNTURSZTdKVFpJU3hBUDhTbkU1azV5dWxqNm5MVFdjWnpKS1gydVNuNHFYMXN3TjVjYnQ4bVVjRng4U1FDLVdfeVJ4cVpOV2g5RVdHbHBJWGVsRktjS3J5QVJjUzBXYk82Vi1JZ1pWWXF3Y1R6WjBkbUc1Z3JPTHZYeFp4aUd3QzBwYVNpY0k?oc=5</t>
+        </is>
+      </c>
+      <c r="AA201" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB201" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC201" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD201" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-09-21T03:46:11+00:00</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E202" t="n">
+        <v>100.279</v>
+      </c>
+      <c r="F202" t="n">
+        <v>100.312</v>
+      </c>
+      <c r="G202" t="n">
+        <v>100.201</v>
+      </c>
+      <c r="H202" t="n">
+        <v>100.295</v>
+      </c>
+      <c r="I202" t="n">
+        <v>0</v>
+      </c>
+      <c r="J202" t="n">
+        <v>4</v>
+      </c>
+      <c r="K202" t="n">
+        <v>39</v>
+      </c>
+      <c r="L202" t="n">
+        <v>0.151</v>
+      </c>
+      <c r="M202" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="N202" t="n">
+        <v>39</v>
+      </c>
+      <c r="O202" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="P202" t="n">
+        <v>-0.062</v>
+      </c>
+      <c r="Q202" t="n">
+        <v>5.943</v>
+      </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S202" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U202" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V202" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W202" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X202" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y202" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z202" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA202" t="inlineStr">
+        <is>
+          <t>ING lifts year-end EUR/USD forecast to 1.18 as dovish Fed view pressures Dollar - VT Markets</t>
+        </is>
+      </c>
+      <c r="AB202" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxORE5YdjZHQzh4V1B2REJUeHpXV3N6Y21ZeWh3VzhfNng4N0dsSk5xbEpCTW40a05ES2NPQkFqQ3RGWjR4ZnN4RUFhVXoxU1NPRFUzZnZRU3E3TzRSTUxxYWZ1dnVMVlVqVUZrR2JRYkt2QlVYVGtpUGN2Mmt6blhvRFVDWURtbkI4UGlyVHpmMHBSeFdTS0RNS0NENXZWQkFxSVNBdkQxSVczTmdMbDk4UVpzSWtZVUliVS1WVFZZdnRuYXM?oc=5</t>
+        </is>
+      </c>
+      <c r="AC202" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD202" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-09-21T03:46:11+00:00</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>7734.5</v>
+      </c>
+      <c r="F203" t="n">
+        <v>7746</v>
+      </c>
+      <c r="G203" t="n">
+        <v>7730.75</v>
+      </c>
+      <c r="H203" t="n">
+        <v>7743.75</v>
+      </c>
+      <c r="I203" t="n">
+        <v>34443</v>
+      </c>
+      <c r="J203" t="n">
+        <v>4</v>
+      </c>
+      <c r="K203" t="n">
+        <v>40</v>
+      </c>
+      <c r="L203" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="M203" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="N203" t="n">
+        <v>40</v>
+      </c>
+      <c r="O203" t="n">
+        <v>0.301</v>
+      </c>
+      <c r="P203" t="n">
+        <v>-0.051</v>
+      </c>
+      <c r="Q203" t="n">
+        <v>6.671</v>
+      </c>
+      <c r="R203" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S203" t="inlineStr">
+        <is>
+          <t>Nigerian Stock Market Surges As Investors Gain N316bn - dmarketforces.com</t>
+        </is>
+      </c>
+      <c r="T203" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOempJUzIyU0FVZkFkTWNFXzJ1U01EX1l3WXhBUHRZMmpyLVItMzJHb1FhaUEtYjIzRDd4NFpsVjZwLXJfM3hPa3ZGUWJ5NzFtUE9paGZmem5SblprZjlFNXdpWENKMU8xSUE0elB2bWFEeGI3enMwWUctTlQ5XzU1SUhfbGpwQmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U203" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="V203" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="W203" t="inlineStr">
+        <is>
+          <t>SanDisk SNDK Stock Breaks Resistance as NAND Demand Strengthens but Memory Risks Remain - FXLeaders</t>
+        </is>
+      </c>
+      <c r="X203" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPSENjb3VhWEFEQTd5a0xIM0hGQWFUcTJfU1QyZXZ1VTluMndraDNNSnh2Y25xS0RkWjZJR2JsNDlnRk1KOGFwM0c1NlE3RGN1ZkFhVjA0SXBDNVhISXp1YUxkVnhpUzJGeHVOVHMxVExMTHhmZ0pVMExkSnNNV3BwV2MxMlBYZ1NTMlhmQmpxajdLaUtKNTFKSXllNGc1RUgydm5kZ1RXd1c4VmRBSlA1RUFvMm96QTN3QzdfZWh4MTJ0amY3bk16MDR3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y203" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z203" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA203" t="inlineStr">
+        <is>
+          <t>Dow gains 250 points as oil prices and yields fall after Fed hike - qz.com</t>
+        </is>
+      </c>
+      <c r="AB203" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBIeU10VzFtempHaDBBYVhGSW5DenM0OVJnSWl3NXZWekdkcUJscTVfbzROZDNHSW83VUdIMTM0VjFfZlhnR01ONk1xTU5jNTBpak5LRFhSeGdxeXJoaktmQWhTend2bjY5eE14dTc3UE95QURIMWFrS0xEMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC203" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD203" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-09-21T03:46:11+00:00</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>30029.5</v>
+      </c>
+      <c r="F204" t="n">
+        <v>30130.5</v>
+      </c>
+      <c r="G204" t="n">
+        <v>30018</v>
+      </c>
+      <c r="H204" t="n">
+        <v>30084.5</v>
+      </c>
+      <c r="I204" t="n">
+        <v>27362</v>
+      </c>
+      <c r="J204" t="n">
+        <v>4</v>
+      </c>
+      <c r="K204" t="n">
+        <v>40</v>
+      </c>
+      <c r="L204" t="n">
+        <v>-0.114</v>
+      </c>
+      <c r="M204" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="N204" t="n">
+        <v>39</v>
+      </c>
+      <c r="O204" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="P204" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="Q204" t="n">
+        <v>-0.548</v>
+      </c>
+      <c r="R204" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S204" t="inlineStr">
+        <is>
+          <t>Samsung Electronics, SK hynix surge as U.S. tech stocks rally - 매일경제</t>
+        </is>
+      </c>
+      <c r="T204" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE55T0VWYmJHT1k0U1U3bldzSXpxTFNoNUVobHNVSHpjVmFhTGQzQUR3b0VDWkpvYlpHR0tFOWM2WXREa2U5NzQwbzE5TVFYT1BrSERZRjFhQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U204" t="inlineStr">
+        <is>
+          <t>Warren Buffett sends a strong warning to stock market investors - thestreet.com</t>
+        </is>
+      </c>
+      <c r="V204" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPNGMyemZrU3daYlVXenNWWWk1SHFzbVJCdkRUc1lWWlBZbVhDY1hOSUdzQXpoZUkxTjRaWHpsbFFUTzFfM2hmclZkaXdWeENNR3lvZzV2aTFYSjVsOVVFZmNhUVk3bGwwZ0pLckZNQVlyZkJYMUJqWDQ3Q1BqVnBlaW4xWHpCMTY5cDNpVlhxY1RhQU8tSVk3Rm5QVzltaS01OHpuc0NWQWdwZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W204" t="inlineStr">
+        <is>
+          <t>AI Server Stocks Rally as the Hardware Bid Broadens: Hewlett Packard Enterprise Jumps 9%, Super Micro Climbs 6%, Dell Rises 3% - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X204" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNbUk4OGEtN1VjNjBIT1NxMGlpa2tEVC1sTExGOXpKUUpyc1VBX254dVlrTDEtSXN6VkxYM004OFY5eWlObFAwRV84NEVXSlh4WVhtRzFhTXV2eExDcjMxc2JDY1g3TW1DYldOanJmRFJ5eFozYzVLOXVyUExuRDMyak42MnlIcUNJaXRoWGQzbFhGNXNvekxWajhDZGs?oc=5</t>
+        </is>
+      </c>
+      <c r="Y204" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: Fresh highs keep momentum strong near 29K - FOREX.com</t>
+        </is>
+      </c>
+      <c r="Z204" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQTZMQ21MMFIxaUJ2cUQtcUM1T1h4bGxsUmRiX3BUYndDbDRYMFhvU2ZXcU0yUVNrckthUVIxMDlpYWYzSXJwTDBrNThfOF91RVl5elRCZ3hyU3dGd0s4SUgzbkI4S2NzdlBpUEJoM0swT0NWSXlWWmQ0UWJfMTNyWnRIZGxQQ2MxajhnRTBTRHRVeFUtUjlLeUFLY0Y4VkVIVENoNnhYUjU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA204" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB204" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC204" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD204" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-09-21T03:46:11+00:00</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>81153.86719999999</v>
+      </c>
+      <c r="F205" t="n">
+        <v>82070.0938</v>
+      </c>
+      <c r="G205" t="n">
+        <v>80837.4688</v>
+      </c>
+      <c r="H205" t="n">
+        <v>81458.97659999999</v>
+      </c>
+      <c r="I205" t="n">
+        <v>5162641408</v>
+      </c>
+      <c r="J205" t="n">
+        <v>4</v>
+      </c>
+      <c r="K205" t="n">
+        <v>37</v>
+      </c>
+      <c r="L205" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="M205" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="N205" t="n">
+        <v>37</v>
+      </c>
+      <c r="O205" t="n">
+        <v>0.337</v>
+      </c>
+      <c r="P205" t="n">
+        <v>-0.056</v>
+      </c>
+      <c r="Q205" t="n">
+        <v>9.097</v>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S205" t="inlineStr">
+        <is>
+          <t>XRP Surges 6.9% as Bitcoin Rebound Reopens Door to Golden Cross - Decrypt</t>
+        </is>
+      </c>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ucm9hYldRNWMyRDBjREdzNUthTTVMa3RZcEY5WUdWWjNmOUMya0JSemRqUXE4Q2dNd3JpcFB1ejViT3ZvUWVMUGt5MDlTaHVXd0NVbE9vb0tQYU9Qd3o3czJBRFhBWmI4NGJlaC1sWjQxM3haR3NBM1lWRmJpZ9IBhgFBVV95cUxOM1RxOHBBS0hRVXpGLTlUS3JzUjhIYmFjTG1vdFZiWDhRUE9PV2VlWnBGMmRFMmNpWFhIcjdoeG9SOWJaZ0hwT2N6NG9rbkJuS3g2R01aMlo0allaRDh2WFdxY05neGlaejlwSUtIVGlYRVA1MlZOTUxHR3g0b2UweV9oenZoZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U205" t="inlineStr">
+        <is>
+          <t>Crypto markets rebound with Bitcoin over $80K; Akedo surges 400%, Stable drops 16%. - Pluang</t>
+        </is>
+      </c>
+      <c r="V205" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVTY5aEdmNHpYR0I5VmVuX2JYcm03YjcxT0pVRmtwenZYRjZLcGlmZUlIYThlLUstX1oxYzNRdXpfYXgyMEc4Y0UySjYyLUQ5LUZxTTgzU04yNUl5MUFrek9icFk0b2pERWhhNWtlaEk5NzR6NzJUYlhNZDdtYVhVZE8tUlFlVTdPQWtKSzJaXzRLWWdBNnc?oc=5</t>
+        </is>
+      </c>
+      <c r="W205" t="inlineStr">
+        <is>
+          <t>BlackRock clients buy $108M Bitcoin via IBIT as institutional demand stays strong - Pluang</t>
+        </is>
+      </c>
+      <c r="X205" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQbHV3QW80d1E2TzFjbVQ0QkltRlg5dmJ5eHJOVTFpUEstdWNPMWtnNG9qUUxxazBBMV91bVVjNnRJczRzRnJGV2FrLVpwX0xmdUljVnVETE9BelVrcklzc2M4SnoySlFuOXpLWk13d25qRGZuTmtTMlJXenZHNGNpYmxRbjkwSFRTMXdtS3lPQkRSQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y205" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="Z205" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA205" t="inlineStr">
+        <is>
+          <t>Bitcoin Is 11 Days From Its First Winning Quarter in a Year. What Needs to Hold Until September 30? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB205" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQTU9EX0F6eUx0b0Q4cVhJMEtNLU92NXJPTmNvSGk2VVJmamw2dEhRdVN6Mi1xWThSbWY1MFRoVjlXWWVFUTdZcm1vajFTY3BXM0k0OHJYaFRZNmZ6dzZjRWFzUjFaeUstUlo5emkxNVhYay10WTJKT1JpbnZEM2xMUExDZ2YzM1dBWTYtbEpqS0pBUTRzUEFKeENRckJONVdnRTFGWm1mVUNOckc2dm4wSHRlQlhrcS1XUGlUQS10SjhlbGVxWFFxXy01VU1lMUNtMXdiX1U5OXBZUVhHRXN0V2lUZUJXYUhlSlFqUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC205" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - Crypto News</t>
+        </is>
+      </c>
+      <c r="AD205" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-21 09:45 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD205"/>
+  <dimension ref="A1:AD211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25805,6 +25805,762 @@
       <c r="AD205" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-09-21T09:43:32+00:00</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E206" t="n">
+        <v>4387.8999</v>
+      </c>
+      <c r="F206" t="n">
+        <v>4395.2002</v>
+      </c>
+      <c r="G206" t="n">
+        <v>4377.5</v>
+      </c>
+      <c r="H206" t="n">
+        <v>4380.6001</v>
+      </c>
+      <c r="I206" t="n">
+        <v>17690</v>
+      </c>
+      <c r="J206" t="n">
+        <v>4</v>
+      </c>
+      <c r="K206" t="n">
+        <v>39</v>
+      </c>
+      <c r="L206" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="M206" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="N206" t="n">
+        <v>40</v>
+      </c>
+      <c r="O206" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="P206" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Q206" t="n">
+        <v>2.191</v>
+      </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S206" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T206" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="U206" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="V206" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W206" t="inlineStr">
+        <is>
+          <t>Gold hits record high as investors seek safety - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="X206" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVWt1Y1hBWG5uZFNjRUFtZHlqRUhfZGV6VzAtQ0tBT2VlVDVEZEJ2WHN0YndCcXRzSjNtVnFhUFZZZ2F4RFRxYkdsSF91eDk2MFl5R3JNWk1HREJjSVdhUE1uTTU1N1Z6Y2xfZzZCSDZ4YnhaT1czcWdXeHE3SjJBR2FqUm43Z0paUG5OVEdsWVdYYnZBWVHSAZsBQVVfeXFMTWh6VXlqZGZVbUl3SHVfQ195WFFveEVkLU9TU1RXMTZBdVhodU16UWxLLWVScDNsc2VGMThyT0RTTHB4SVNRYU1KWmRycHhnTEc0NTJ1RWgzdGc2Y0VkanR4QUtlUWFBSnB2cElORUltQk9XdWRLNXhKbU5jRUFqQVd6bG5YbURJakxhNTl3UEk4RzBaQzVJaVdRdFk?oc=5</t>
+        </is>
+      </c>
+      <c r="Y206" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z206" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQQmZsZ2tENzhwQTJ0SmZhaW5PcU9kZTh1WmZld0pySDQ0LTZDWnBTNkR0S3hKZTN2QXk4bjJrRmhqcGxjS1FQQkZ1X1VBNDVZTTJQRFAxVV81SGR1VUV4d2hVZnFBZ3NqSVRrQnQ5NmM1QUhCMUFHTktYMW9yaUo1dg?oc=5</t>
+        </is>
+      </c>
+      <c r="AA206" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="AB206" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC206" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD206" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-09-21T09:43:32+00:00</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="F207" t="n">
+        <v>94.78</v>
+      </c>
+      <c r="G207" t="n">
+        <v>93.45999999999999</v>
+      </c>
+      <c r="H207" t="n">
+        <v>94.15000000000001</v>
+      </c>
+      <c r="I207" t="n">
+        <v>30182</v>
+      </c>
+      <c r="J207" t="n">
+        <v>4</v>
+      </c>
+      <c r="K207" t="n">
+        <v>40</v>
+      </c>
+      <c r="L207" t="n">
+        <v>-0.058</v>
+      </c>
+      <c r="M207" t="n">
+        <v>-0.257</v>
+      </c>
+      <c r="N207" t="n">
+        <v>40</v>
+      </c>
+      <c r="O207" t="n">
+        <v>0.127</v>
+      </c>
+      <c r="P207" t="n">
+        <v>-0.063</v>
+      </c>
+      <c r="Q207" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S207" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T207" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U207" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - cnbc.com</t>
+        </is>
+      </c>
+      <c r="V207" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="W207" t="inlineStr">
+        <is>
+          <t>Oil prices surge 15% as Strait of Hormuz disruptions tighten supply - Offshore Technology</t>
+        </is>
+      </c>
+      <c r="X207" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPdndjemtyTkduUUpSVnR6aXJUNXBBR0JNd1FaaURNWmtvWm9WTkZUME50Qk1NVDUtdEtqcWE2R0xvUGRKNHBWZDMtblpaY1h1TE5zcmgycU5kS29mYU02N1BOdThBMUhUMDM0T1FScDZRY0JzYlRXTTJVajFYbkh3Rmp0MDFDeVZQcFhKSjhpaklySjZrVWJCZVoyWkw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y207" t="inlineStr">
+        <is>
+          <t>Market Recap: Semiconductor Stocks Surge as Oil Prices Drop Belo - GuruFocus</t>
+        </is>
+      </c>
+      <c r="Z207" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQVUhnUEpoS21NazZnR2F2dnQyU2JaTmNzWFc1VEdNTURSZTdKVFpJU3hBUDhTbkU1azV5dWxqNm5MVFdjWnpKS1gydVNuNHFYMXN3TjVjYnQ4bVVjRng4U1FDLVdfeVJ4cVpOV2g5RVdHbHBJWGVsRktjS3J5QVJjUzBXYk82Vi1JZ1pWWXF3Y1R6WjBkbUc1Z3JPTHZYeFp4aUd3QzBwYVNpY0k?oc=5</t>
+        </is>
+      </c>
+      <c r="AA207" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB207" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC207" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - cnbc.com</t>
+        </is>
+      </c>
+      <c r="AD207" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-09-21T09:43:32+00:00</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>100.337</v>
+      </c>
+      <c r="F208" t="n">
+        <v>100.375</v>
+      </c>
+      <c r="G208" t="n">
+        <v>100.257</v>
+      </c>
+      <c r="H208" t="n">
+        <v>100.323</v>
+      </c>
+      <c r="I208" t="n">
+        <v>0</v>
+      </c>
+      <c r="J208" t="n">
+        <v>4</v>
+      </c>
+      <c r="K208" t="n">
+        <v>39</v>
+      </c>
+      <c r="L208" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="M208" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="N208" t="n">
+        <v>39</v>
+      </c>
+      <c r="O208" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="P208" t="n">
+        <v>-0.007</v>
+      </c>
+      <c r="Q208" t="n">
+        <v>9.002000000000001</v>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S208" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - moomoo.com</t>
+        </is>
+      </c>
+      <c r="T208" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U208" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V208" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W208" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X208" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y208" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z208" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA208" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AB208" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC208" t="inlineStr">
+        <is>
+          <t>DXY Falls After Jobs Report - TradingView</t>
+        </is>
+      </c>
+      <c r="AD208" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNSEw2V2JQUlhSd1FvVjhhQlRoSGdrS1V2OUR6QnlSVUF0amg2dDNzWUd3cEh2Slg0ODBNNzVKejgzNGxPbFpZd3N2NG56eFhDYTBTLWpZSVd5WlY2RGQ2SnpKaTNoMkRUckNqQnl5MFZlUVlqWVpmcVBLWHgyLV9PcGhYdGY?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-09-21T09:43:32+00:00</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>7745.5</v>
+      </c>
+      <c r="F209" t="n">
+        <v>7764.25</v>
+      </c>
+      <c r="G209" t="n">
+        <v>7745.5</v>
+      </c>
+      <c r="H209" t="n">
+        <v>7761.5</v>
+      </c>
+      <c r="I209" t="n">
+        <v>62220</v>
+      </c>
+      <c r="J209" t="n">
+        <v>4</v>
+      </c>
+      <c r="K209" t="n">
+        <v>40</v>
+      </c>
+      <c r="L209" t="n">
+        <v>-0.123</v>
+      </c>
+      <c r="M209" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="N209" t="n">
+        <v>40</v>
+      </c>
+      <c r="O209" t="n">
+        <v>0.174</v>
+      </c>
+      <c r="P209" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="Q209" t="n">
+        <v>1.004</v>
+      </c>
+      <c r="R209" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S209" t="inlineStr">
+        <is>
+          <t>US stock market could ride earnings strength to more gains after S&amp;P 500 hits record - Reuters</t>
+        </is>
+      </c>
+      <c r="T209" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPRDhYYlFmZ3FHcjh0dS1TQ2Z3ampQM2tjSmZha3pHMzhVelB5Q0xzTE8zVThKM1haMFVuTWlpNkFXUHA3WlRORjE0NFhBcExMS1hWeVRIbUtxU3RmbEI2NS1FNmNtamhnZXY5QXlUa1FGN1FMRWc4cF9PMVVJM0pfeEFWQmJfY291UFVtLWFiN292QzMzQjNRQWFmY0RIeDBLQlZKS1dPbEZUMDVidHI3d1RSNkVqYjhlX2Y0Z295M3hDb0k?oc=5</t>
+        </is>
+      </c>
+      <c r="U209" t="inlineStr">
+        <is>
+          <t>Icon Energy Corp. Lifts Earnings Outlook as Dry Bulk Market Surges - The Globe and Mail</t>
+        </is>
+      </c>
+      <c r="V209" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxQR042dHRITEs0T0NDb0ROZE16MU8wNnJnaGl0Yjg5UnJWU0w4MXE3YUY1VkpIT1pUczZiWlRSQ2JIRnRSMkF4eEQ3Q3NIVEZYeWJ0MTNIMEZLbFU2bWFDN0VLTVhqV2N4NURadUhJWFhKalR4OVBxeW5mTlExZFVBUFBxQVFzN0lFMG96RTh6bW93eHl5dkJkWmtLOG9ieDUzVmk1RVpFY3Q0QUZaU2syMFlDWi1jWkRqdTY4MnFpdzNWVUp3ZmRkMVdUZklVNGtLTkliZ2pldDZldEhYMk1qR1lTTHg?oc=5</t>
+        </is>
+      </c>
+      <c r="W209" t="inlineStr">
+        <is>
+          <t>Illumina Stock Analysis: Bullish Trend Holds, Momentum in Focus - The Cryptonomist</t>
+        </is>
+      </c>
+      <c r="X209" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQaUstS2lxb25wVWhUUm9ZZjM4WUpYekk3Mk1VVjdHYWdaZUE2alhkXzVKMXlOOHZ0ekVOSE5EWXYtS1o2QjFyVGVockpyVWZPVXdhUTNsSFcyMEE5aFZqb0l4M045T3Z4cnNuU2t4ckpBYTNmZEhGZWstVlV2YlkzQW0zSkpNYUtzeTRYZ2NrMG9nWDhwQ0x2QTZsNVg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y209" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z209" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA209" t="inlineStr">
+        <is>
+          <t>Eramet shares rebound 2.5% and break back above key support - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB209" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNMGhPZjF6TzFuNjJyZjdRYUgydjVVX2I0d2FaM2c3RGU1RDhaVnNEOFhHTzVUcGxrM3FWbHpsZnEzNzZFbXItN0Vfc1lVZWphZFVrVmtOcnJZT1NLMFp2WkljT0lVREpzblBTV1ZBVkZ1eEZaN0xmMnVCTUFvLVlRVElpQnFvZEE1c05SdDVQMFVxUVBnOXdWZXdKUUNYTno0TGEzSmhpNzY1LW1zZlpqQjZnMXBFMEV4?oc=5</t>
+        </is>
+      </c>
+      <c r="AC209" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD209" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-09-21T09:43:32+00:00</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>30090.5</v>
+      </c>
+      <c r="F210" t="n">
+        <v>30262.5</v>
+      </c>
+      <c r="G210" t="n">
+        <v>30090.5</v>
+      </c>
+      <c r="H210" t="n">
+        <v>30252</v>
+      </c>
+      <c r="I210" t="n">
+        <v>27477</v>
+      </c>
+      <c r="J210" t="n">
+        <v>4</v>
+      </c>
+      <c r="K210" t="n">
+        <v>39</v>
+      </c>
+      <c r="L210" t="n">
+        <v>-0.237</v>
+      </c>
+      <c r="M210" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="N210" t="n">
+        <v>40</v>
+      </c>
+      <c r="O210" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="P210" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="Q210" t="n">
+        <v>-2.334</v>
+      </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S210" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="T210" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="U210" t="inlineStr">
+        <is>
+          <t>The S&amp;P 500 is back at a record high and the Dow just hit 54,000 | CNN Business - CNN</t>
+        </is>
+      </c>
+      <c r="V210" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE9sNTR6eTFUS1JYX1lnaWVIZGxJeVhmbENJMHN3SUc4TTlSaHpweUdwNUNLejJtSmIwb0x0SEQxalc2OVN1X2s1WFhPSWt2X2VrcFFVeXhVVVpxYVVnaUFjRDR3SUFxbzA?oc=5</t>
+        </is>
+      </c>
+      <c r="W210" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq boosted by chips to record closing highs - Reuters</t>
+        </is>
+      </c>
+      <c r="X210" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPOFFvTzhsTGtZYjFZd3ZLQUNtNGxSZTlyb0ZmX3pKSHFucWF1bnpGQlQydHhod21iUWE2bW54QzgyeEstVGZhQmRpSWZQZTMycFlMeTNtUGtfT0VHeWdaSlJCb0xrY29Gcy0tbm5XMWRDYkgyVUY4UDRycXgtMHRfc2hiUHN1Wmd2YTNEMFZ0ZVdqQXRGTnhETXJuZjYxTUpwRGpaU2N6ZEd0Yldh?oc=5</t>
+        </is>
+      </c>
+      <c r="Y210" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="Z210" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA210" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AB210" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+      <c r="AC210" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="AD210" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-09-21T09:43:32+00:00</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>81553.5</v>
+      </c>
+      <c r="F211" t="n">
+        <v>85152.9375</v>
+      </c>
+      <c r="G211" t="n">
+        <v>81386.36719999999</v>
+      </c>
+      <c r="H211" t="n">
+        <v>85006.00780000001</v>
+      </c>
+      <c r="I211" t="n">
+        <v>13365501952</v>
+      </c>
+      <c r="J211" t="n">
+        <v>4</v>
+      </c>
+      <c r="K211" t="n">
+        <v>38</v>
+      </c>
+      <c r="L211" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="M211" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="N211" t="n">
+        <v>37</v>
+      </c>
+      <c r="O211" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P211" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="Q211" t="n">
+        <v>11.634</v>
+      </c>
+      <c r="R211" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S211" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Recovery Surges Past $81,000 on Strong Market Signals - The Cryptonomist</t>
+        </is>
+      </c>
+      <c r="T211" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE1LclU5Y3NScVBlVHI5YlVwUS1fTWxKMFZYOUU5a04xNDBhU3k0VWR5UUFCZ0YxMHBPa0ZJcDlRRktOV0JjQVVlTUc0ZW9OdFRWUWpDTmFrcTktWGZuam10eDVYS29DTEk5YnNkVEw4RlFnNkpJTlE?oc=5</t>
+        </is>
+      </c>
+      <c r="U211" t="inlineStr">
+        <is>
+          <t>XRP Surges 6.9% as Bitcoin Rebound Reopens Door to Golden Cross - Decrypt</t>
+        </is>
+      </c>
+      <c r="V211" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ucm9hYldRNWMyRDBjREdzNUthTTVMa3RZcEY5WUdWWjNmOUMya0JSemRqUXE4Q2dNd3JpcFB1ejViT3ZvUWVMUGt5MDlTaHVXd0NVbE9vb0tQYU9Qd3o3czJBRFhBWmI4NGJlaC1sWjQxM3haR3NBM1lWRmJpZ9IBhgFBVV95cUxOM1RxOHBBS0hRVXpGLTlUS3JzUjhIYmFjTG1vdFZiWDhRUE9PV2VlWnBGMmRFMmNpWFhIcjdoeG9SOWJaZ0hwT2N6NG9rbkJuS3g2R01aMlo0allaRDh2WFdxY05neGlaejlwSUtIVGlYRVA1MlZOTUxHR3g0b2UweV9oenZoZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W211" t="inlineStr">
+        <is>
+          <t>BlackRock clients buy $108M Bitcoin via IBIT as institutional demand stays strong - Pluang</t>
+        </is>
+      </c>
+      <c r="X211" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQbHV3QW80d1E2TzFjbVQ0QkltRlg5dmJ5eHJOVTFpUEstdWNPMWtnNG9qUUxxazBBMV91bVVjNnRJczRzRnJGV2FrLVpwX0xmdUljVnVETE9BelVrcklzc2M4SnoySlFuOXpLWk13d25qRGZuTmtTMlJXenZHNGNpYmxRbjkwSFRTMXdtS3lPQkRSQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y211" t="inlineStr">
+        <is>
+          <t>Bitcoin surges above $80,000, triggering $183M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="Z211" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOU1htWHVWRE1uU2VTNTM0RkhnQVdMLUoxU3d1NGp1dU9GbmFyZXRDNUN0SzhnWERHNlFEMXZCdGZXUnRabFg1VmF4T3o4Njd1WmJPSkRnemRqblE5cFljZ29XXzhvOTF4cFo2eWI4V1MxclZzaThjVjdBUG4zS3hQSmhNOVdpU1NnSG0zSFhMT0Z0Z1M0bWZCNl9MTnBYVlJUd3ROQVl1U19ZQWhlalFqaURFTWxreUVzb0djQ09Ud203QndYZnZBTw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA211" t="inlineStr">
+        <is>
+          <t>Celsius estate sues BitMEX over $495M in Bitcoin liquidations - Crypto News</t>
+        </is>
+      </c>
+      <c r="AB211" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1rakZjRFpPdXJpWHBkNzF4T1kxVlR0UmhTeXZSbVA0WGphTkpLMEpsei1ZVGpSTTN0YWNqd2hrdXFKREZBdTkyaTB0OGNWb2Iwc0dXWXljYlFfS095Z25BMDRSZW1YTmlZaFp5VmZQaWgwd2xlbjlKek5tRkx0UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC211" t="inlineStr">
+        <is>
+          <t>Bitcoin Cracks $80,000, Ethereum, XRP Surge 4% on $170M Short Liquidations - Benzinga</t>
+        </is>
+      </c>
+      <c r="AD211" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQREJLU2hyMG1QZWU0TFM1eFYxUlljUW5hdzZVZjdoQnlqX3dVQ3ZQSlRWVzYyVkF3R0FodVRRRHktR2MzWkVldEJ3djFZVVROMzg3Yy0xRTZfbDFLS3d6NDZVVXNwSndDQV9QeUJqQ1ppbTE2Q3JUSGZYQS1faGxvSXJuUWhTT3dQSDAzS0dmdl81X3QtSTMtQlhBbmo3UWUzZlJyTVlOSFVRaEtYLXlQb1pkMEJzWGZSZlVsU2NTRXBxZnlIV1Npel9R?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-21 18:01 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD211"/>
+  <dimension ref="A1:AD217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26561,6 +26561,762 @@
       <c r="AD211" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQREJLU2hyMG1QZWU0TFM1eFYxUlljUW5hdzZVZjdoQnlqX3dVQ3ZQSlRWVzYyVkF3R0FodVRRRHktR2MzWkVldEJ3djFZVVROMzg3Yy0xRTZfbDFLS3d6NDZVVXNwSndDQV9QeUJqQ1ppbTE2Q3JUSGZYQS1faGxvSXJuUWhTT3dQSDAzS0dmdl81X3QtSTMtQlhBbmo3UWUzZlJyTVlOSFVRaEtYLXlQb1pkMEJzWGZSZlVsU2NTRXBxZnlIV1Npel9R?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-09-21T17:59:03+00:00</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>4383.7002</v>
+      </c>
+      <c r="F212" t="n">
+        <v>4395.7002</v>
+      </c>
+      <c r="G212" t="n">
+        <v>4360.2998</v>
+      </c>
+      <c r="H212" t="n">
+        <v>4381.1001</v>
+      </c>
+      <c r="I212" t="n">
+        <v>42805</v>
+      </c>
+      <c r="J212" t="n">
+        <v>4</v>
+      </c>
+      <c r="K212" t="n">
+        <v>39</v>
+      </c>
+      <c r="L212" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="M212" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="N212" t="n">
+        <v>40</v>
+      </c>
+      <c r="O212" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="P212" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="Q212" t="n">
+        <v>3.974</v>
+      </c>
+      <c r="R212" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S212" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T212" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="U212" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - azernews.az</t>
+        </is>
+      </c>
+      <c r="V212" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W212" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X212" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y212" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="Z212" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA212" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB212" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC212" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD212" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-09-21T17:59:03+00:00</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>92.56999999999999</v>
+      </c>
+      <c r="F213" t="n">
+        <v>92.67</v>
+      </c>
+      <c r="G213" t="n">
+        <v>91.19</v>
+      </c>
+      <c r="H213" t="n">
+        <v>92.23999999999999</v>
+      </c>
+      <c r="I213" t="n">
+        <v>113118</v>
+      </c>
+      <c r="J213" t="n">
+        <v>4</v>
+      </c>
+      <c r="K213" t="n">
+        <v>40</v>
+      </c>
+      <c r="L213" t="n">
+        <v>-0.184</v>
+      </c>
+      <c r="M213" t="n">
+        <v>-0.244</v>
+      </c>
+      <c r="N213" t="n">
+        <v>40</v>
+      </c>
+      <c r="O213" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="P213" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="Q213" t="n">
+        <v>-0.096</v>
+      </c>
+      <c r="R213" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S213" t="inlineStr">
+        <is>
+          <t>AI Demand Boosts Stocks as Oil Drops; Bonds Rally Worldwide - Global Banking &amp; Finance Review</t>
+        </is>
+      </c>
+      <c r="T213" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxQUi0zb3pMZTJuMWtSUWNEcXRqTElUWWRNa1JjLVQ3ZWtha0dlUEhaODk2V0g1dWtYRUVlN1ZnZEpQWWdVTXNtbkNqVTNpX1VMcVBObDcwQ0RnVVM0QllScFdpdENvMGxfVnBOcWdHLUl6VXl6R1lIMTQ1RThsbHJUTjh6QWpDXzg?oc=5</t>
+        </is>
+      </c>
+      <c r="U213" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="V213" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W213" t="inlineStr">
+        <is>
+          <t>Oil prices surge 15% as Strait of Hormuz disruptions tighten supply - offshore-technology.com</t>
+        </is>
+      </c>
+      <c r="X213" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPdndjemtyTkduUUpSVnR6aXJUNXBBR0JNd1FaaURNWmtvWm9WTkZUME50Qk1NVDUtdEtqcWE2R0xvUGRKNHBWZDMtblpaY1h1TE5zcmgycU5kS29mYU02N1BOdThBMUhUMDM0T1FScDZRY0JzYlRXTTJVajFYbkh3Rmp0MDFDeVZQcFhKSjhpaklySjZrVWJCZVoyWkw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y213" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 21, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z213" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5KS291VGxrSWo1UjJNRHhZRHlWeFNadWVKS3dfb2VXbzZpOUE4OU9lc0dpWDhJN19ENFlnbEsyUWFySVVyNF8yR2dkSUxzcXJCcHQ4dC1KVzltU0cyWHJ3ajNR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA213" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AB213" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC213" t="inlineStr">
+        <is>
+          <t>Soybean Oil tests $68 support after Fibonacci break: Live levels By Investing.com - Investing.com India</t>
+        </is>
+      </c>
+      <c r="AD213" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPOXJmd2Iycy1VdUZrQVBiYy1IRU1kZVp4NDNpb1V1Rm03WGoxMGo0Rk5QOGRPakMzeW10N1U3NmlYZUVQTTVZcEZMbVdMUDc4dnV1OGtjUGkzWUJGWUVnb25TLUNzVDc1eURWZF9vVTVzeHNxbVBBTS1Ec2VHbWpXdFlBR2I2Rl9tVm80NC12XzRjd2pUU0x2UjEzeUdiZ1YxSThTSDVvTllUMTgxRk00Y2pwcFVDdFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-09-21T17:59:03+00:00</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>100.363</v>
+      </c>
+      <c r="F214" t="n">
+        <v>100.418</v>
+      </c>
+      <c r="G214" t="n">
+        <v>100.334</v>
+      </c>
+      <c r="H214" t="n">
+        <v>100.414</v>
+      </c>
+      <c r="I214" t="n">
+        <v>0</v>
+      </c>
+      <c r="J214" t="n">
+        <v>4</v>
+      </c>
+      <c r="K214" t="n">
+        <v>39</v>
+      </c>
+      <c r="L214" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="M214" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="N214" t="n">
+        <v>39</v>
+      </c>
+      <c r="O214" t="n">
+        <v>0.194</v>
+      </c>
+      <c r="P214" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="Q214" t="n">
+        <v>6.898</v>
+      </c>
+      <c r="R214" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S214" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T214" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U214" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V214" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W214" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X214" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y214" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z214" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA214" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges Past ₺3.9 Million as Turkish Lira Hits Record Low - ccn.com</t>
+        </is>
+      </c>
+      <c r="AB214" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOTU9ZSDBLR2ItM2NIdklVS2dVUFV2S2k2bVVQV2ZpRG44SFpESzVheW9GVU9mcDNfTWFlU2NEQTVKVEg5T0lOeVlZcml5VnVOa1JXV0l5Q1I4a1BOUTRYeDVRVmplY3RqRXFuWHdCc0loVkQyb05oaDJaSzlSSGJ6Z3M4YWxqZXJ2dnIwY2JkR3Z0TVdlcnc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC214" t="inlineStr">
+        <is>
+          <t>FX Daily: Fed hold can hit the dollar today - think.ing.com</t>
+        </is>
+      </c>
+      <c r="AD214" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE91QWFPVUVXdGYyVGFxekZhSXBLNzFWN2xfWkJVRXNud05nSzJPQXpwN1hjbzJxZ0ZWLWdmTWhXbzI4NFRXdnpobUc2MllDT1VFQWtFbzhiZ1kzX0Z2c3FGal9nZF91Y19ISENwR1RVdnBRVVVhc0EtY3BmOEZKU1k?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-09-21T17:59:03+00:00</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>7774.75</v>
+      </c>
+      <c r="F215" t="n">
+        <v>7830</v>
+      </c>
+      <c r="G215" t="n">
+        <v>7767.75</v>
+      </c>
+      <c r="H215" t="n">
+        <v>7826.5</v>
+      </c>
+      <c r="I215" t="n">
+        <v>559816</v>
+      </c>
+      <c r="J215" t="n">
+        <v>4</v>
+      </c>
+      <c r="K215" t="n">
+        <v>40</v>
+      </c>
+      <c r="L215" t="n">
+        <v>-0.262</v>
+      </c>
+      <c r="M215" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="N215" t="n">
+        <v>40</v>
+      </c>
+      <c r="O215" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="P215" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="Q215" t="n">
+        <v>-1.939</v>
+      </c>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S215" t="inlineStr">
+        <is>
+          <t>Tech-Led Rally Lifts S&amp;P 500 To Best Day Since Early August - TheStreet Pro</t>
+        </is>
+      </c>
+      <c r="T215" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPOEQ1Z3N3emRUUUZvRmdOa0luVUdXZGVXeFpVcEk4U0ZQM2oxQnpVYU1DS1VwQ2p2dXZHTWpXeldqaGdMZW9rTGdjSXRnY0RuaGYxMTNqX1RVb3UzdnE0bkFEdjkySDg0YjNzV0NKd1F4TmJWdnFBTUNZZUh0aXR3cjdJSXkya1VTazdrWDBPVUlWV0pLLXo0b0x4LXUtWHprel9feg?oc=5</t>
+        </is>
+      </c>
+      <c r="U215" t="inlineStr">
+        <is>
+          <t>Dow jumps more than 250 points for record close and fifth winning day: Live updates - CNBC</t>
+        </is>
+      </c>
+      <c r="V215" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE8yenVSZnZSMHlWeHFLOUswVnExcnp5MVRSRXljcFJ0cGRMdF9ma3N2d0ZBYUNickZFc0dGV3RSWVRDRzRIbk82UnVDbUxjTXVGaHpEMTRZU2dpMjVwTWdLbWE0OHRidkJmTUYtbkxZSWNUUUd0T3VJ0gF8QVVfeXFMT2dHODc5S2N4X21SN1ZrcFVMaWxjaUo5Yi1ZNHR3aTN5RnpPNlF5NUxtNGhxNVpmQXg0VWpIWU1CUlZBWHNCSHlUVlh2eHAwYWhoSEJUd1kxQTljamczMEROTTlHbU4wTE9SaHVhMmtEMzRNYjdFbWc5ZFdwTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W215" t="inlineStr">
+        <is>
+          <t>Today’s Market Recap: AI Chip Stocks Gain, SanDisk Surges Nearly 11%, Micron Rises Nearly 4%, Bitcoin Reclaims $80,000 - TradingKey</t>
+        </is>
+      </c>
+      <c r="X215" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxOQW5IQUQ4c00ySlBQNE8wbmJ0VjR6QXVKM0F1VEgwX3d6R2ZrblpoTFdoRGhDRzR1Z05kaFRGY1NtWFMxMlZBRWtsaGFFUlp3MEJMNVBRTVlUOUN3Mi01cFVMdlE1dXcyMG83V0FXUEZ3Z1RHRHJJTTc3elBhdVpqOUFGT1BNSzI3cDZVNC1hTUoxeGxqdlB5ajNNRTNRNDNXX3F5LS1RMkNYSTBqVlRoNHFXWkNNRy0wbklNaHJROGdPV1l6cjVtT2NiMlRpR1NPOTUyNzNjN21DeVJk?oc=5</t>
+        </is>
+      </c>
+      <c r="Y215" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z215" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA215" t="inlineStr">
+        <is>
+          <t>Bank of America hikes S&amp;P 500 target after Al trade cracks - Rock Hill Herald</t>
+        </is>
+      </c>
+      <c r="AB215" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFB3R2RnanRNUElSa0tYdXpyekY3RVBlZXBwcXJZN1ZKc3dkQW5FalFVRlRjOS1lSE5CalBSRWczVTd0Y3NLRk5kbUpOcjdkWUJjYVFKNGVpUVRCWEFESjdnTS1QLWJjWU9ZeE9mSkk0Y3o4Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC215" t="inlineStr">
+        <is>
+          <t>Dow Drops 631, Nasdaq Slips 3, S&amp;P 500 Falls 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD215" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQVFVRNlU5aU5HaTYzZ2tnN1Nabng2cWNEd2VPQzdxcU96aHRDOFgyTUR0S3hQNXQ3MVVXQ2xDRGZKWkxNQVgyQl83eW1VQU8yX2hZVS0yR25COHJyTndBcG5xZUd2dFVvOUNPOE5BSkhnaVN4dGVQVFNreWQ0SmFFcTZwdFdmUlZqcTFsekRMcw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-09-21T17:59:03+00:00</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>30416.5</v>
+      </c>
+      <c r="F216" t="n">
+        <v>30724.5</v>
+      </c>
+      <c r="G216" t="n">
+        <v>30397</v>
+      </c>
+      <c r="H216" t="n">
+        <v>30714.5</v>
+      </c>
+      <c r="I216" t="n">
+        <v>216216</v>
+      </c>
+      <c r="J216" t="n">
+        <v>4</v>
+      </c>
+      <c r="K216" t="n">
+        <v>36</v>
+      </c>
+      <c r="L216" t="n">
+        <v>-0.184</v>
+      </c>
+      <c r="M216" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N216" t="n">
+        <v>40</v>
+      </c>
+      <c r="O216" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="P216" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="Q216" t="n">
+        <v>-3.163</v>
+      </c>
+      <c r="R216" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S216" t="inlineStr">
+        <is>
+          <t>AI Demand Boosts Stocks as Oil Drops; Bonds Rally Worldwide - Global Banking &amp; Finance Review</t>
+        </is>
+      </c>
+      <c r="T216" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxQUi0zb3pMZTJuMWtSUWNEcXRqTElUWWRNa1JjLVQ3ZWtha0dlUEhaODk2V0g1dWtYRUVlN1ZnZEpQWWdVTXNtbkNqVTNpX1VMcVBObDcwQ0RnVVM0QllScFdpdENvMGxfVnBOcWdHLUl6VXl6R1lIMTQ1RThsbHJUTjh6QWpDXzg?oc=5</t>
+        </is>
+      </c>
+      <c r="U216" t="inlineStr">
+        <is>
+          <t>Rally in bank and tech stocks lifts European shares - The Irish Times</t>
+        </is>
+      </c>
+      <c r="V216" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxOOF9EQmVSMHNBUUhmVExRTW56cEM5d2IyZDlsaEpjODZUYlI2VE1Wb3V0ZTNXSHFvcE5BVUtyYVc0THJKNkhSM3NXSzhjMVVJX1J1a0RYQTJBMHliRzJXMXYyT3RxajEtRzk3WmFHeHdGa2RGNUtyMGZwUlV4eWtrZVR6bHhpUy1KM1dFdzRGUl9BRVFGbV8xTHMyMV8wd2tY?oc=5</t>
+        </is>
+      </c>
+      <c r="W216" t="inlineStr">
+        <is>
+          <t>AMD Stock Hits Fresh Record High, Up 183% This Year - Advanced Micro Devices (NASDAQ:AMD), Oracle (NYSE:O - Benzinga</t>
+        </is>
+      </c>
+      <c r="X216" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxORWJKWG9XOWJiVkxCSEN1c1hwN3MycUhnMG1jdXRtSTd5eGZrcm9FeDU3R1JUb3oxc3F1T0ZTX2stek96R1BLcTFjckR0RUlxUUhMb0ZWZnZEaXNmaUR2ZGhPOXJCWkRaUWNybkdSeFVqek1iNjVKTV9uaWJVdGNjaG1IZkhSNEpZSWx1TmxlejdLM1Z1VjRQbTh0WkZOdm03SW9SRm41SnpZSUdO?oc=5</t>
+        </is>
+      </c>
+      <c r="Y216" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="Z216" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA216" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB216" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC216" t="inlineStr">
+        <is>
+          <t>European STOXX 600 Rises, Boosted by Tech Stocks and Falling Oil Prices - صحيفة مال</t>
+        </is>
+      </c>
+      <c r="AD216" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE5XZmhDU21GOHJLUzJvTzJzTmVhdU5ydHBrTjVKeHRrVHp0MmFFSDdZWGdHaDhjYUxJdWlBQTA5cUtEbGVFd2FVZ3h3SGh2OVdIajB6N3FMNkNDWEpIQ1pkQUdTeU00ZWptYlc2cW9n?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-09-21T17:59:03+00:00</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>85827</v>
+      </c>
+      <c r="F217" t="n">
+        <v>86348.99219999999</v>
+      </c>
+      <c r="G217" t="n">
+        <v>85619.11719999999</v>
+      </c>
+      <c r="H217" t="n">
+        <v>85846.2812</v>
+      </c>
+      <c r="I217" t="n">
+        <v>5441732608</v>
+      </c>
+      <c r="J217" t="n">
+        <v>4</v>
+      </c>
+      <c r="K217" t="n">
+        <v>37</v>
+      </c>
+      <c r="L217" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="M217" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="N217" t="n">
+        <v>36</v>
+      </c>
+      <c r="O217" t="n">
+        <v>0.354</v>
+      </c>
+      <c r="P217" t="n">
+        <v>-0.003</v>
+      </c>
+      <c r="Q217" t="n">
+        <v>7.134</v>
+      </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S217" t="inlineStr">
+        <is>
+          <t>Bitcoin surged to an eight-month high above $85,000 as oil fell and ETF inflows returned - qz.com</t>
+        </is>
+      </c>
+      <c r="T217" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9BRHhsSDNaZ2VlVnhzYmRsci1zNk1kQ2JWNHJxNTNVRHFDSHFqcmVoVFg2TkJxYTdZMUhfMEJpb1hFS3RabDlJcVZZWEh4M3VJUUpaX0JUSWtHd0pxNUctNzg3Nkx0Q2JoT21EN2cwV1ZtQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U217" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to $85,000 as $648M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="V217" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQRHZIOW9Xc2xkakVMRUlRV2F5a0thZHN0ZFREZ2lrOUowVjVWd0lBaE0yWmRMdkdxZW0zLUdnbTE1MFZsa05kRkRqbWhhZUdmMlFXa0NlUlJBRjlNVXVGcW9UdWl0RnlWUVhiZi11ZDlCSUxGRXVPYUNXaVZfbS01dnp3cFlfd3NMeHk2eUhzWkpyRVBfSWR5YUN6U0tRRnFDWGZJcDlQbTJCdG1FMGxrSHdpY0dmVHFDRkE?oc=5</t>
+        </is>
+      </c>
+      <c r="W217" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Surges Over $81,000 Despite Clarity Act Fail and Interest Rate Hike - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="X217" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE5DLVVDZWFpWWxfQzVoanF6dkl5QUc1cWkxZHNwWC1maFBiUG4wNjI4STZJRmRvZ01TNXE5emRHQ0VBdHpPb054TWhFUHhqS2sxU2k0SU1weVpWVG80VjlzSDdhd0NWNjRoNXExU3Izd2I2VHp3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y217" t="inlineStr">
+        <is>
+          <t>Bitcoin price tags $86K as analysis sees crypto in ‘new bull market’ - TradingView</t>
+        </is>
+      </c>
+      <c r="Z217" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOdGloQjlFZUswdXdaQnAyOTUzbmR4aGRnODZTcGRaZUs5ODBhaXpNWlM4bGl4U2d3aElrSGVEUmJfNnJQYzZqNFRWVS05eTkxeXRkTnltTTIxOV9sZFpaRFlhbll5OEdZRjJBNlpiX2UxOVltYURDQ3dhMl9rZk9JWVVCMGJtWGRkYy11Wkc2QlU2cDVEcHJMWDhlS3d0RnZ2SU5nMUU2STRMVlJSeFUxY3Nkak80Sm1ZYk0xV2VfalR5bGhpaS1YcA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA217" t="inlineStr">
+        <is>
+          <t>Bitcoin clears $85K as $648M in shorts are liquidated, per CoinGlass - Altcoin Buzz</t>
+        </is>
+      </c>
+      <c r="AB217" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxPdldlWXhkNnpXb1FYcEdMZHZ0WWtiSHpvMEo1RGd4ejZvQjVTcGFadWhURVFWcks2T2dlR0Y1cmxremJ0YS1DaFI1bW5hN3ptc0FfYWltM2lrdi0yNHo2YXBFdWxOSVBraXNqRGpaWUxXLWxPc0VFMEVFVi01WFUyOHlQZjNEcEUwVUFJ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC217" t="inlineStr">
+        <is>
+          <t>Senate Blocks Crypto Market Bill as Bitcoin Stocks Fall - Wealth Management</t>
+        </is>
+      </c>
+      <c r="AD217" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOLUF2Nm9sZE5pa0VtNW45bHFVZDBlaG9yYTAyZTJlMlhkX09EbjJ2Y25CMjdGUEp5ZVBZbGNaRWgwdVZseUd5MWhJbW4xeE00NFJoQW1BMGdDMkViRnZNUTRNUUxKQkhTMDR1bm5mMTRJandGX1Jhd1ZKOUJtMTdPdWdUN0RITkFmSWxJNFZJb1cwRjVuVzhiUWNKTEVnNnJvMmc?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-21 23:06 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD217"/>
+  <dimension ref="A1:AD223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27317,6 +27317,762 @@
       <c r="AD217" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOLUF2Nm9sZE5pa0VtNW45bHFVZDBlaG9yYTAyZTJlMlhkX09EbjJ2Y25CMjdGUEp5ZVBZbGNaRWgwdVZseUd5MWhJbW4xeE00NFJoQW1BMGdDMkViRnZNUTRNUUxKQkhTMDR1bm5mMTRJandGX1Jhd1ZKOUJtMTdPdWdUN0RITkFmSWxJNFZJb1cwRjVuVzhiUWNKTEVnNnJvMmc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-09-21T23:04:23+00:00</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>4383</v>
+      </c>
+      <c r="F218" t="n">
+        <v>4400.2998</v>
+      </c>
+      <c r="G218" t="n">
+        <v>4377.2998</v>
+      </c>
+      <c r="H218" t="n">
+        <v>4400</v>
+      </c>
+      <c r="I218" t="n">
+        <v>12304</v>
+      </c>
+      <c r="J218" t="n">
+        <v>4</v>
+      </c>
+      <c r="K218" t="n">
+        <v>40</v>
+      </c>
+      <c r="L218" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="M218" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="N218" t="n">
+        <v>40</v>
+      </c>
+      <c r="O218" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="P218" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="Q218" t="n">
+        <v>4.606</v>
+      </c>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S218" t="inlineStr">
+        <is>
+          <t>Gold Price Climbs to $4,620 as Safe-Haven Demand Returns Across Global Markets - CryptoRank</t>
+        </is>
+      </c>
+      <c r="T218" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMTFVdFU1RW5zWmFVMFF4ejVVWi1FVWZhYzBIT3RCN2ZybWY2cmV5ZnlEY21HRW5oZE1oeUd3TzkwNzhqRE5vR2UxeWZxUzcyVzNjN3JQMnFXdEdFYWUxU0p1SVBPZDlRSUVZTkRJdEw1cHFlVGE0cm0xU05URjMyRE12YmpvbkFvMUt3cVRNZ1FiOUd0NV9jelN3elBqd0tieU1ycjFxY0h6QWZKZlNjcGQ2aGk?oc=5</t>
+        </is>
+      </c>
+      <c r="U218" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V218" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W218" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X218" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y218" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="Z218" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA218" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="AB218" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC218" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD218" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-09-21T23:04:23+00:00</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>92.17</v>
+      </c>
+      <c r="F219" t="n">
+        <v>92.59</v>
+      </c>
+      <c r="G219" t="n">
+        <v>91.75</v>
+      </c>
+      <c r="H219" t="n">
+        <v>92.12</v>
+      </c>
+      <c r="I219" t="n">
+        <v>40761</v>
+      </c>
+      <c r="J219" t="n">
+        <v>4</v>
+      </c>
+      <c r="K219" t="n">
+        <v>40</v>
+      </c>
+      <c r="L219" t="n">
+        <v>-0.188</v>
+      </c>
+      <c r="M219" t="n">
+        <v>-0.238</v>
+      </c>
+      <c r="N219" t="n">
+        <v>40</v>
+      </c>
+      <c r="O219" t="n">
+        <v>0.228</v>
+      </c>
+      <c r="P219" t="n">
+        <v>-0.074</v>
+      </c>
+      <c r="Q219" t="n">
+        <v>0.8090000000000001</v>
+      </c>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T219" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U219" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="V219" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="W219" t="inlineStr">
+        <is>
+          <t>Europe's STOXX 600 rallies on tech, banks strength as oil prices retreat - Reuters</t>
+        </is>
+      </c>
+      <c r="X219" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNYWF0aU9mWUM0TjNtekhpT0I0NTM1RXoydldTZDlzNVM4Q0FnRXFCLTlaLUQxdEZfMS1qeU1XV0lsNHhvc09zMTBUQV9xVFhaakdCU196dW5sQ212UHdLVjVySHo5UWczV0dVS2dnY3d2Q2dTbWRkOWFRZ0g5aTlGaEtnQkFQcno2ZjdfdndQdGdSR1c3MjdEXzNCZlhRM216di1sdllQSl9OT3pkcWRSd3p3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y219" t="inlineStr">
+        <is>
+          <t>Brent Oil breaks below $103 support: Live levels By Investing.com - Investing.com Canada</t>
+        </is>
+      </c>
+      <c r="Z219" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNbVprR1I1Ukp5OTZuYlpCcW5mS0oxbW5ITGYyNlRSSWNjOG02dmpsalJVT2ZZN0FUTVdaTE5WVHlBNmxrZ2RfSmJmQ3N4YU0wcVpFVVJfMC1ZRVo5bmdtUWNhZ09wUF9jNzZnZnZ6UzVCN3VsRXR5b0N3c2QxOXdHTVZKemEyek5LT1puNTdMd3RZdFVrUW5XYk5tdnRnN3BIckRwdmUwWUJUcWpPY3dpZk83NDh0VElGT05lVm8wZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA219" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB219" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC219" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD219" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-09-21T23:04:23+00:00</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>100.429</v>
+      </c>
+      <c r="F220" t="n">
+        <v>100.435</v>
+      </c>
+      <c r="G220" t="n">
+        <v>100.383</v>
+      </c>
+      <c r="H220" t="n">
+        <v>100.425</v>
+      </c>
+      <c r="I220" t="n">
+        <v>0</v>
+      </c>
+      <c r="J220" t="n">
+        <v>4</v>
+      </c>
+      <c r="K220" t="n">
+        <v>39</v>
+      </c>
+      <c r="L220" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="M220" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="N220" t="n">
+        <v>39</v>
+      </c>
+      <c r="O220" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="P220" t="n">
+        <v>-0.012</v>
+      </c>
+      <c r="Q220" t="n">
+        <v>3.766</v>
+      </c>
+      <c r="R220" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T220" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U220" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V220" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W220" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X220" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y220" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z220" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA220" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges Past ₺3.9 Million as Turkish Lira Hits Record Low - CCN.com</t>
+        </is>
+      </c>
+      <c r="AB220" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOTU9ZSDBLR2ItM2NIdklVS2dVUFV2S2k2bVVQV2ZpRG44SFpESzVheW9GVU9mcDNfTWFlU2NEQTVKVEg5T0lOeVlZcml5VnVOa1JXV0l5Q1I4a1BOUTRYeDVRVmplY3RqRXFuWHdCc0loVkQyb05oaDJaSzlSSGJ6Z3M4YWxqZXJ2dnIwY2JkR3Z0TVdlcnc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC220" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD220" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-09-21T23:04:23+00:00</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>7827</v>
+      </c>
+      <c r="F221" t="n">
+        <v>7847.25</v>
+      </c>
+      <c r="G221" t="n">
+        <v>7826.5</v>
+      </c>
+      <c r="H221" t="n">
+        <v>7835.75</v>
+      </c>
+      <c r="I221" t="n">
+        <v>420761</v>
+      </c>
+      <c r="J221" t="n">
+        <v>4</v>
+      </c>
+      <c r="K221" t="n">
+        <v>39</v>
+      </c>
+      <c r="L221" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="M221" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="N221" t="n">
+        <v>40</v>
+      </c>
+      <c r="O221" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="P221" t="n">
+        <v>-0.024</v>
+      </c>
+      <c r="Q221" t="n">
+        <v>-5.327</v>
+      </c>
+      <c r="R221" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T221" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U221" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V221" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W221" t="inlineStr">
+        <is>
+          <t>Illumina Stock Analysis: Bullish Trend Holds, Momentum in Focus - The Cryptonomist</t>
+        </is>
+      </c>
+      <c r="X221" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQaUstS2lxb25wVWhUUm9ZZjM4WUpYekk3Mk1VVjdHYWdaZUE2alhkXzVKMXlOOHZ0ekVOSE5EWXYtS1o2QjFyVGVockpyVWZPVXdhUTNsSFcyMEE5aFZqb0l4M045T3Z4cnNuU2t4ckpBYTNmZEhGZWstVlV2YlkzQW0zSkpNYUtzeTRYZ2NrMG9nWDhwQ0x2QTZsNVg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y221" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z221" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA221" t="inlineStr">
+        <is>
+          <t>Eramet shares rebound 2.5% and break back above key support - Idéal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB221" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNMGhPZjF6TzFuNjJyZjdRYUgydjVVX2I0d2FaM2c3RGU1RDhaVnNEOFhHTzVUcGxrM3FWbHpsZnEzNzZFbXItN0Vfc1lVZWphZFVrVmtOcnJZT1NLMFp2WkljT0lVREpzblBTV1ZBVkZ1eEZaN0xmMnVCTUFvLVlRVElpQnFvZEE1c05SdDVQMFVxUVBnOXdWZXdKUUNYTno0TGEzSmhpNzY1LW1zZlpqQjZnMXBFMEV4?oc=5</t>
+        </is>
+      </c>
+      <c r="AC221" t="inlineStr">
+        <is>
+          <t>Bank of America hikes S&amp;P 500 target after Al trade cracks - Rock Hill Herald</t>
+        </is>
+      </c>
+      <c r="AD221" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFB3R2RnanRNUElSa0tYdXpyekY3RVBlZXBwcXJZN1ZKc3dkQW5FalFVRlRjOS1lSE5CalBSRWczVTd0Y3NLRk5kbUpOcjdkWUJjYVFKNGVpUVRCWEFESjdnTS1QLWJjWU9ZeE9mSkk0Y3o4Zw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-09-21T23:04:23+00:00</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>30712.75</v>
+      </c>
+      <c r="F222" t="n">
+        <v>30862.75</v>
+      </c>
+      <c r="G222" t="n">
+        <v>30712.5</v>
+      </c>
+      <c r="H222" t="n">
+        <v>30828.5</v>
+      </c>
+      <c r="I222" t="n">
+        <v>130576</v>
+      </c>
+      <c r="J222" t="n">
+        <v>4</v>
+      </c>
+      <c r="K222" t="n">
+        <v>35</v>
+      </c>
+      <c r="L222" t="n">
+        <v>-0.264</v>
+      </c>
+      <c r="M222" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="N222" t="n">
+        <v>38</v>
+      </c>
+      <c r="O222" t="n">
+        <v>-0.029</v>
+      </c>
+      <c r="P222" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="Q222" t="n">
+        <v>-6.67</v>
+      </c>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>Meta Platforms surges 12% amid AI monetization rally (META:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T222" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQYmJDOXZmZDZKcUZVVjE3a0NMVWtBMG5BazdXdlZVT0ZtZEltQjdUZEl1TjY3Ri1mbFF0Mzc0Z0JiMndydnI3SHYybUpoSGZ0Z2JyV0xkdGduY1RjdHNpZndzeWl4M0NSSGhpaEd5UlF4NVc0R2NSUUhTMjRVSC12Y2FYMEc2YlhHa3hvQ0ZHN3dxdVE?oc=5</t>
+        </is>
+      </c>
+      <c r="U222" t="inlineStr">
+        <is>
+          <t>US Stocks Surge as Nasdaq Rises Over 2% to Highest Since June; Tech and Chip Stocks Lead Gains, Meta Jumps 11% - TradingKey</t>
+        </is>
+      </c>
+      <c r="V222" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxORnJ6el84X0pHd2t0MjdieXpIUVlCMUxoa1A4aEt6ZWNaY3d3LXQ0N0ZtdEw0U0ZmYjl2cVdhVnA0d1YyWi1ueE41SnJGaHVNX3dsbmgyMFg0MWZHUWlTa0otOWZGd09OcXMtVU9EWjc5clJ6ZDdiS3k0bm41ajNfdUtOaWF6UTk5aFlhVDRWbDJ3ckxEQU52czFObnExX2F4MlNtSGx5TFNjN2Vqc2hvYkcwc2dVSWJ5NTJkLURNRUhoZjZxR3o4ZHMwbUdKZ1BVTTlBQXlHSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W222" t="inlineStr">
+        <is>
+          <t>Taiwanese shares buoyed by US tech rally and trade talks - Taipei Times</t>
+        </is>
+      </c>
+      <c r="X222" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBuTS1SbnpPUzVQVS11c2tORmxxVlJIY3kzYXl4amtCZERsRVM3STlKN0Y5Z2xMOUF5dkI2R2FTUXdhOWxkeVk0SW1Nb0Ytdk1MSmRvRnk4RUJaRHRRdXJCODVGT3p3WVJQMDAwV3AybFlaQ2hfS1E?oc=5</t>
+        </is>
+      </c>
+      <c r="Y222" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="Z222" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="AA222" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB222" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC222" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AD222" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-09-21T23:04:23+00:00</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>86550.75780000001</v>
+      </c>
+      <c r="F223" t="n">
+        <v>87373.7812</v>
+      </c>
+      <c r="G223" t="n">
+        <v>86274</v>
+      </c>
+      <c r="H223" t="n">
+        <v>86559.53909999999</v>
+      </c>
+      <c r="I223" t="n">
+        <v>6407229440</v>
+      </c>
+      <c r="J223" t="n">
+        <v>4</v>
+      </c>
+      <c r="K223" t="n">
+        <v>35</v>
+      </c>
+      <c r="L223" t="n">
+        <v>-0.074</v>
+      </c>
+      <c r="M223" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="N223" t="n">
+        <v>36</v>
+      </c>
+      <c r="O223" t="n">
+        <v>0.274</v>
+      </c>
+      <c r="P223" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="Q223" t="n">
+        <v>3.131</v>
+      </c>
+      <c r="R223" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to $87K, sparking talk of a $90K breakthrough amid strong inflows and market optimism. - Pluang</t>
+        </is>
+      </c>
+      <c r="T223" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNVml5bmpucDhzSmdrTF83UHZhU2t5cWQtaXE3QXJYVFhSSHU5MlROTTUtOG15aU5Cek5WM0Y4Z1FUQkFpcjdXUmxsLXhlX1JtRHI0eThJem1QSUFDanlQaHJqd2VzMnVsZElqaVJwVUZ1TU5WalB3eDd2MGlORXR2MVgxQWVnVTU2YnMxOWFNM3E0TW0zcEZzS0RleGxFYzl1TU41aU53?oc=5</t>
+        </is>
+      </c>
+      <c r="U223" t="inlineStr">
+        <is>
+          <t>Bitcoin surged to an eight-month high above $85,000 as oil fell and ETF inflows returned - qz.com</t>
+        </is>
+      </c>
+      <c r="V223" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9BRHhsSDNaZ2VlVnhzYmRsci1zNk1kQ2JWNHJxNTNVRHFDSHFqcmVoVFg2TkJxYTdZMUhfMEJpb1hFS3RabDlJcVZZWEh4M3VJUUpaX0JUSWtHd0pxNUctNzg3Nkx0Q2JoT21EN2cwV1ZtQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W223" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="X223" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y223" t="inlineStr">
+        <is>
+          <t>Bitcoin price tags $86K as analysis sees crypto in ‘new bull market’ - TradingView</t>
+        </is>
+      </c>
+      <c r="Z223" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOdGloQjlFZUswdXdaQnAyOTUzbmR4aGRnODZTcGRaZUs5ODBhaXpNWlM4bGl4U2d3aElrSGVEUmJfNnJQYzZqNFRWVS05eTkxeXRkTnltTTIxOV9sZFpaRFlhbll5OEdZRjJBNlpiX2UxOVltYURDQ3dhMl9rZk9JWVVCMGJtWGRkYy11Wkc2QlU2cDVEcHJMWDhlS3d0RnZ2SU5nMUU2STRMVlJSeFUxY3Nkak80Sm1ZYk0xV2VfalR5bGhpaS1YcA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA223" t="inlineStr">
+        <is>
+          <t>Bitcoin price rebounds above $85K after smaller holders reduce exposure amid market shakeout - Pluang</t>
+        </is>
+      </c>
+      <c r="AB223" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOTHNfMTFCdDN4RGF2U2o2a2JaSWRVMzNXZXdBRE5nTlEtWGVJbTFhTjNyRHNJSWNSdlc4NDRCdzlYT3RIa0NfWDkybVdDcEhuMDVPSExqSTlmcjgwT1FmNXQ3TVdWOFZJc0lXYV9MQThlTWRObG5vbkI4b0hiVlgzZk1LSnA3dUVhWS1nd3lscklBWWM?oc=5</t>
+        </is>
+      </c>
+      <c r="AC223" t="inlineStr">
+        <is>
+          <t>Bitcoin clears $85K as $648M in shorts are liquidated, per CoinGlass - Altcoin Buzz</t>
+        </is>
+      </c>
+      <c r="AD223" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxPdldlWXhkNnpXb1FYcEdMZHZ0WWtiSHpvMEo1RGd4ejZvQjVTcGFadWhURVFWcks2T2dlR0Y1cmxremJ0YS1DaFI1bW5hN3ptc0FfYWltM2lrdi0yNHo2YXBFdWxOSVBraXNqRGpaWUxXLWxPc0VFMEVFVi01WFUyOHlQZjNEcEUwVUFJ?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-22 03:46 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD223"/>
+  <dimension ref="A1:AD229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28073,6 +28073,762 @@
       <c r="AD223" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxPdldlWXhkNnpXb1FYcEdMZHZ0WWtiSHpvMEo1RGd4ejZvQjVTcGFadWhURVFWcks2T2dlR0Y1cmxremJ0YS1DaFI1bW5hN3ptc0FfYWltM2lrdi0yNHo2YXBFdWxOSVBraXNqRGpaWUxXLWxPc0VFMEVFVi01WFUyOHlQZjNEcEUwVUFJ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-09-22T03:44:21+00:00</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>4407</v>
+      </c>
+      <c r="F224" t="n">
+        <v>4414.1001</v>
+      </c>
+      <c r="G224" t="n">
+        <v>4376.2998</v>
+      </c>
+      <c r="H224" t="n">
+        <v>4384.2002</v>
+      </c>
+      <c r="I224" t="n">
+        <v>18225</v>
+      </c>
+      <c r="J224" t="n">
+        <v>4</v>
+      </c>
+      <c r="K224" t="n">
+        <v>40</v>
+      </c>
+      <c r="L224" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="M224" t="n">
+        <v>-0.015</v>
+      </c>
+      <c r="N224" t="n">
+        <v>40</v>
+      </c>
+      <c r="O224" t="n">
+        <v>0.222</v>
+      </c>
+      <c r="P224" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="Q224" t="n">
+        <v>5.957</v>
+      </c>
+      <c r="R224" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S224" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T224" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="U224" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="V224" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="W224" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="X224" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y224" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="Z224" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA224" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB224" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC224" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD224" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-09-22T03:44:21+00:00</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>92.27</v>
+      </c>
+      <c r="F225" t="n">
+        <v>93.27</v>
+      </c>
+      <c r="G225" t="n">
+        <v>92.11</v>
+      </c>
+      <c r="H225" t="n">
+        <v>93.12</v>
+      </c>
+      <c r="I225" t="n">
+        <v>10671</v>
+      </c>
+      <c r="J225" t="n">
+        <v>4</v>
+      </c>
+      <c r="K225" t="n">
+        <v>40</v>
+      </c>
+      <c r="L225" t="n">
+        <v>-0.103</v>
+      </c>
+      <c r="M225" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="N225" t="n">
+        <v>40</v>
+      </c>
+      <c r="O225" t="n">
+        <v>0.217</v>
+      </c>
+      <c r="P225" t="n">
+        <v>-0.068</v>
+      </c>
+      <c r="Q225" t="n">
+        <v>2.274</v>
+      </c>
+      <c r="R225" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S225" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="T225" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="U225" t="inlineStr">
+        <is>
+          <t>Europe's STOXX 600 rallies on tech, banks strength as oil prices retreat - Reuters</t>
+        </is>
+      </c>
+      <c r="V225" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNYWF0aU9mWUM0TjNtekhpT0I0NTM1RXoydldTZDlzNVM4Q0FnRXFCLTlaLUQxdEZfMS1qeU1XV0lsNHhvc09zMTBUQV9xVFhaakdCU196dW5sQ212UHdLVjVySHo5UWczV0dVS2dnY3d2Q2dTbWRkOWFRZ0g5aTlGaEtnQkFQcno2ZjdfdndQdGdSR1c3MjdEXzNCZlhRM216di1sdllQSl9OT3pkcWRSd3p3?oc=5</t>
+        </is>
+      </c>
+      <c r="W225" t="inlineStr">
+        <is>
+          <t>Oil prices surge 15% as Strait of Hormuz disruptions tighten supply - Offshore Technology</t>
+        </is>
+      </c>
+      <c r="X225" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPdndjemtyTkduUUpSVnR6aXJUNXBBR0JNd1FaaURNWmtvWm9WTkZUME50Qk1NVDUtdEtqcWE2R0xvUGRKNHBWZDMtblpaY1h1TE5zcmgycU5kS29mYU02N1BOdThBMUhUMDM0T1FScDZRY0JzYlRXTTJVajFYbkh3Rmp0MDFDeVZQcFhKSjhpaklySjZrVWJCZVoyWkw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y225" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z225" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA225" t="inlineStr">
+        <is>
+          <t>Brent Oil breaks below $103 support: Live levels By Investing.com - Investing.com Nigeria</t>
+        </is>
+      </c>
+      <c r="AB225" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQT1Z0V0k1ZTZrTEVrZU83eFRkV1FoMDZvZHlBdHBiS0xhWF9nOGdDM3Y5V1NxYnU3dm5JOXRmMFZYRU5oS3RKZ3FGYmw2dmFRN3psLXdMdkJTbXNyUHZ3Ujg1Y19nek50X0ZuYUs2ejdNNnBYNGZhU0lYNTdDZWFoQlhaX1hidlFPMDk4RTRCRVdDckg5Mzg0T2dNeTduaWxhUWZfV3FPM240c0ExS0xleTJIQ1p2U0NBODZnT01TVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC225" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD225" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-09-22T03:44:21+00:00</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>100.424</v>
+      </c>
+      <c r="F226" t="n">
+        <v>100.456</v>
+      </c>
+      <c r="G226" t="n">
+        <v>100.341</v>
+      </c>
+      <c r="H226" t="n">
+        <v>100.345</v>
+      </c>
+      <c r="I226" t="n">
+        <v>0</v>
+      </c>
+      <c r="J226" t="n">
+        <v>4</v>
+      </c>
+      <c r="K226" t="n">
+        <v>39</v>
+      </c>
+      <c r="L226" t="n">
+        <v>-0.058</v>
+      </c>
+      <c r="M226" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="N226" t="n">
+        <v>39</v>
+      </c>
+      <c r="O226" t="n">
+        <v>0.177</v>
+      </c>
+      <c r="P226" t="n">
+        <v>-0.019</v>
+      </c>
+      <c r="Q226" t="n">
+        <v>2.322</v>
+      </c>
+      <c r="R226" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S226" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T226" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U226" t="inlineStr">
+        <is>
+          <t>Yuan Strengthens Against Global Rate-Hike Tide as FX Settlement Cycle Fuels Independent Rally - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="V226" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE45ZHlodXZrMDVRa2xiS1A1cWJsZVlKRmRjeG0yTFNtYmFoN01jSm5xVjZDd2Y0V0U5Nno1VjdhdHlMbnYyMDFQblBrZlRERVVlZ0FlZ3lWQWpHS2dHWTFPR1VzYWVIM1ZvYjk1M1NidnBDYTVtYXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W226" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="X226" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y226" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z226" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA226" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges Past ₺3.9 Million as Turkish Lira Hits Record Low - CCN.com</t>
+        </is>
+      </c>
+      <c r="AB226" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOTU9ZSDBLR2ItM2NIdklVS2dVUFV2S2k2bVVQV2ZpRG44SFpESzVheW9GVU9mcDNfTWFlU2NEQTVKVEg5T0lOeVlZcml5VnVOa1JXV0l5Q1I4a1BOUTRYeDVRVmplY3RqRXFuWHdCc0loVkQyb05oaDJaSzlSSGJ6Z3M4YWxqZXJ2dnIwY2JkR3Z0TVdlcnc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC226" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD226" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-09-22T03:44:21+00:00</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E227" t="n">
+        <v>7835.25</v>
+      </c>
+      <c r="F227" t="n">
+        <v>7840</v>
+      </c>
+      <c r="G227" t="n">
+        <v>7831.75</v>
+      </c>
+      <c r="H227" t="n">
+        <v>7835</v>
+      </c>
+      <c r="I227" t="n">
+        <v>28191</v>
+      </c>
+      <c r="J227" t="n">
+        <v>4</v>
+      </c>
+      <c r="K227" t="n">
+        <v>40</v>
+      </c>
+      <c r="L227" t="n">
+        <v>-0.223</v>
+      </c>
+      <c r="M227" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="N227" t="n">
+        <v>40</v>
+      </c>
+      <c r="O227" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="P227" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="Q227" t="n">
+        <v>-0.832</v>
+      </c>
+      <c r="R227" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S227" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T227" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U227" t="inlineStr">
+        <is>
+          <t>South Korean shares climb nearly 2% as Wall Street rally boosts sentiment - TradingView</t>
+        </is>
+      </c>
+      <c r="V227" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOSUtCcEJDM2lJZU5sei1LQ0RMcERobnpPaUlycUhWOVdkZC1lMW03Ump1bnVwVHVFOFFCV2c5TG5HcFgxU1hJcW9heVRTSlNnQldieVdrelJRVFNxRHBLQUhxdm1HeHBhWW13QTdiNldKYURuSG9XMlpRZFhJQWsybC1ScHhOQTVTWXJWRmFkQVFUTlRfWEZtR3RBVE1tMGsxcnZMZDBTc0xPYUZSWmdFMTlzMl9KSkI3c2FEZDVlaDRtQ0xJcllETUllYV83Q3l0T05sVU40MnlsUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W227" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="X227" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y227" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z227" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA227" t="inlineStr">
+        <is>
+          <t>Dow Drops 631, Nasdaq Slips 3, S&amp;P 500 Falls 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB227" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQVFVRNlU5aU5HaTYzZ2tnN1Nabng2cWNEd2VPQzdxcU96aHRDOFgyTUR0S3hQNXQ3MVVXQ2xDRGZKWkxNQVgyQl83eW1VQU8yX2hZVS0yR25COHJyTndBcG5xZUd2dFVvOUNPOE5BSkhnaVN4dGVQVFNreWQ0SmFFcTZwdFdmUlZqcTFsekRMcw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC227" t="inlineStr">
+        <is>
+          <t>Darden Stock Breaks $207.25 as Earnings Week Puts $202.75 Support in Focus - TradingKey</t>
+        </is>
+      </c>
+      <c r="AD227" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPcEZ2cWsxRG44VFRXZkw3dWstakNwczBXVEVEOFpPZHVnSm1XME1QV2I4RUxZckNWcGxITF9LX2pVazVVc0JuNXlfLVUzaHBwWHZoQm91d0tSZmxiY25aVVFCeHNlTXdvZ3JpNWpaeV9QTDA4YS1wdzBmQUxmVnBFZjNCQ3Z2ZXplUnR3RjBWX0VGeTd6alRyTkZsQ01rZ0VNdkRXN2VpdkpnWm1OVU9tbQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-09-22T03:44:21+00:00</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E228" t="n">
+        <v>30852.25</v>
+      </c>
+      <c r="F228" t="n">
+        <v>30916.5</v>
+      </c>
+      <c r="G228" t="n">
+        <v>30850</v>
+      </c>
+      <c r="H228" t="n">
+        <v>30894.75</v>
+      </c>
+      <c r="I228" t="n">
+        <v>28852</v>
+      </c>
+      <c r="J228" t="n">
+        <v>4</v>
+      </c>
+      <c r="K228" t="n">
+        <v>35</v>
+      </c>
+      <c r="L228" t="n">
+        <v>-0.332</v>
+      </c>
+      <c r="M228" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="N228" t="n">
+        <v>39</v>
+      </c>
+      <c r="O228" t="n">
+        <v>-0.027</v>
+      </c>
+      <c r="P228" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="Q228" t="n">
+        <v>-8.339</v>
+      </c>
+      <c r="R228" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S228" t="inlineStr">
+        <is>
+          <t>Meta Platforms surges 12% amid AI monetization rally (META:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T228" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQYmJDOXZmZDZKcUZVVjE3a0NMVWtBMG5BazdXdlZVT0ZtZEltQjdUZEl1TjY3Ri1mbFF0Mzc0Z0JiMndydnI3SHYybUpoSGZ0Z2JyV0xkdGduY1RjdHNpZndzeWl4M0NSSGhpaEd5UlF4NVc0R2NSUUhTMjRVSC12Y2FYMEc2YlhHa3hvQ0ZHN3dxdVE?oc=5</t>
+        </is>
+      </c>
+      <c r="U228" t="inlineStr">
+        <is>
+          <t>US Stocks Surge as Nasdaq Rises Over 2% to Highest Since June; Tech and Chip Stocks Lead Gains, Meta Jumps 11% - TradingKey</t>
+        </is>
+      </c>
+      <c r="V228" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxORnJ6el84X0pHd2t0MjdieXpIUVlCMUxoa1A4aEt6ZWNaY3d3LXQ0N0ZtdEw0U0ZmYjl2cVdhVnA0d1YyWi1ueE41SnJGaHVNX3dsbmgyMFg0MWZHUWlTa0otOWZGd09OcXMtVU9EWjc5clJ6ZDdiS3k0bm41ajNfdUtOaWF6UTk5aFlhVDRWbDJ3ckxEQU52czFObnExX2F4MlNtSGx5TFNjN2Vqc2hvYkcwc2dVSWJ5NTJkLURNRUhoZjZxR3o4ZHMwbUdKZ1BVTTlBQXlHSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W228" t="inlineStr">
+        <is>
+          <t>Tech rally boosts Asian stocks, dollar firms on rate-hike wagers - Reuters</t>
+        </is>
+      </c>
+      <c r="X228" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBYNkdDWExac0tiSmtsc3Exd0ZHOTVDZFJCbTRtZW9jM3hTLU84b3JWbHQ1WmZsUE5pSmUzTHBFUXQzaHBnb01UQXV5ZUljTFl2cS1fbHhFMUtDblA3NHRjeXRzbEpYMjNZempPSmRPbEpIajV0T1BuRDl1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y228" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="Z228" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="AA228" t="inlineStr">
+        <is>
+          <t>Tech rally boosts Asian stocks, dollar firms on rate-hike wagers - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="AB228" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNcHJMUDBjcHVoTXZJN21mX0NMbll0NDFPSEVENHk0dzNPRUtOMXc2SVZuZXFfNmZpR1hIYzltM3VjQTdEUER6NHA2X2MtUUloYjdpV1BPTG4xVUdXZ0FoVy1NMThjQU1RLVdsUWNaSFNXakJYeTZENHdBWWYzbnBWQ200b0ZzQlhMVWR4bEZxMkprdVUyNEVlZk1Gaw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC228" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD228" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-09-22T03:44:21+00:00</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E229" t="n">
+        <v>86594.9375</v>
+      </c>
+      <c r="F229" t="n">
+        <v>86602.5938</v>
+      </c>
+      <c r="G229" t="n">
+        <v>85291.60159999999</v>
+      </c>
+      <c r="H229" t="n">
+        <v>85501.0469</v>
+      </c>
+      <c r="I229" t="n">
+        <v>4676423680</v>
+      </c>
+      <c r="J229" t="n">
+        <v>4</v>
+      </c>
+      <c r="K229" t="n">
+        <v>35</v>
+      </c>
+      <c r="L229" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="M229" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="N229" t="n">
+        <v>36</v>
+      </c>
+      <c r="O229" t="n">
+        <v>0.223</v>
+      </c>
+      <c r="P229" t="n">
+        <v>-0.039</v>
+      </c>
+      <c r="Q229" t="n">
+        <v>2.644</v>
+      </c>
+      <c r="R229" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S229" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to $87K, sparking talk of a $90K breakthrough amid strong inflows and market optimism. - Pluang</t>
+        </is>
+      </c>
+      <c r="T229" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNVml5bmpucDhzSmdrTF83UHZhU2t5cWQtaXE3QXJYVFhSSHU5MlROTTUtOG15aU5Cek5WM0Y4Z1FUQkFpcjdXUmxsLXhlX1JtRHI0eThJem1QSUFDanlQaHJqd2VzMnVsZElqaVJwVUZ1TU5WalB3eDd2MGlORXR2MVgxQWVnVTU2YnMxOWFNM3E0TW0zcEZzS0RleGxFYzl1TU41aU53?oc=5</t>
+        </is>
+      </c>
+      <c r="U229" t="inlineStr">
+        <is>
+          <t>Bitcoin surged to an eight-month high above $85,000 as oil fell and ETF inflows returned - qz.com</t>
+        </is>
+      </c>
+      <c r="V229" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9BRHhsSDNaZ2VlVnhzYmRsci1zNk1kQ2JWNHJxNTNVRHFDSHFqcmVoVFg2TkJxYTdZMUhfMEJpb1hFS3RabDlJcVZZWEh4M3VJUUpaX0JUSWtHd0pxNUctNzg3Nkx0Q2JoT21EN2cwV1ZtQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W229" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="X229" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y229" t="inlineStr">
+        <is>
+          <t>Bitcoin price tags $86K as analysis sees crypto in ‘new bull market’ - TradingView</t>
+        </is>
+      </c>
+      <c r="Z229" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOdGloQjlFZUswdXdaQnAyOTUzbmR4aGRnODZTcGRaZUs5ODBhaXpNWlM4bGl4U2d3aElrSGVEUmJfNnJQYzZqNFRWVS05eTkxeXRkTnltTTIxOV9sZFpaRFlhbll5OEdZRjJBNlpiX2UxOVltYURDQ3dhMl9rZk9JWVVCMGJtWGRkYy11Wkc2QlU2cDVEcHJMWDhlS3d0RnZ2SU5nMUU2STRMVlJSeFUxY3Nkak80Sm1ZYk0xV2VfalR5bGhpaS1YcA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA229" t="inlineStr">
+        <is>
+          <t>Bitcoin price rebounds above $85K after smaller holders reduce exposure amid market shakeout - Pluang</t>
+        </is>
+      </c>
+      <c r="AB229" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOTHNfMTFCdDN4RGF2U2o2a2JaSWRVMzNXZXdBRE5nTlEtWGVJbTFhTjNyRHNJSWNSdlc4NDRCdzlYT3RIa0NfWDkybVdDcEhuMDVPSExqSTlmcjgwT1FmNXQ3TVdWOFZJc0lXYV9MQThlTWRObG5vbkI4b0hiVlgzZk1LSnA3dUVhWS1nd3lscklBWWM?oc=5</t>
+        </is>
+      </c>
+      <c r="AC229" t="inlineStr">
+        <is>
+          <t>Senate Blocks Crypto Market Bill as Bitcoin Stocks Fall - Wealth Management</t>
+        </is>
+      </c>
+      <c r="AD229" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOLUF2Nm9sZE5pa0VtNW45bHFVZDBlaG9yYTAyZTJlMlhkX09EbjJ2Y25CMjdGUEp5ZVBZbGNaRWgwdVZseUd5MWhJbW4xeE00NFJoQW1BMGdDMkViRnZNUTRNUUxKQkhTMDR1bm5mMTRJandGX1Jhd1ZKOUJtMTdPdWdUN0RITkFmSWxJNFZJb1cwRjVuVzhiUWNKTEVnNnJvMmc?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-22 09:09 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD229"/>
+  <dimension ref="A1:AD235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28829,6 +28829,762 @@
       <c r="AD229" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOLUF2Nm9sZE5pa0VtNW45bHFVZDBlaG9yYTAyZTJlMlhkX09EbjJ2Y25CMjdGUEp5ZVBZbGNaRWgwdVZseUd5MWhJbW4xeE00NFJoQW1BMGdDMkViRnZNUTRNUUxKQkhTMDR1bm5mMTRJandGX1Jhd1ZKOUJtMTdPdWdUN0RITkFmSWxJNFZJb1cwRjVuVzhiUWNKTEVnNnJvMmc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-09-22T09:07:39+00:00</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E230" t="n">
+        <v>4379.6001</v>
+      </c>
+      <c r="F230" t="n">
+        <v>4384.2002</v>
+      </c>
+      <c r="G230" t="n">
+        <v>4327.6001</v>
+      </c>
+      <c r="H230" t="n">
+        <v>4369.1001</v>
+      </c>
+      <c r="I230" t="n">
+        <v>37355</v>
+      </c>
+      <c r="J230" t="n">
+        <v>4</v>
+      </c>
+      <c r="K230" t="n">
+        <v>39</v>
+      </c>
+      <c r="L230" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M230" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="N230" t="n">
+        <v>40</v>
+      </c>
+      <c r="O230" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="P230" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="Q230" t="n">
+        <v>4.238</v>
+      </c>
+      <c r="R230" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S230" t="inlineStr">
+        <is>
+          <t>Goldman Sachs Maintains Bullish Gold Outlook - businesskorea.co.kr</t>
+        </is>
+      </c>
+      <c r="T230" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE5aM0FhTU0tdzZUU1ZGcnJxZm1FN1pFVURiQXdyWmxKUi1MRGgzVWdEd3dTaVhWcUZnd01xNHlWaHpuSGowN29lQ1NBZjYxTUNQejYtc3p3VGdaNS0ySENZZFFOanpzV2R6RUZ4WWxBU05WZGU1?oc=5</t>
+        </is>
+      </c>
+      <c r="U230" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V230" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W230" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X230" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y230" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="Z230" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA230" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB230" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC230" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD230" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-09-22T09:07:39+00:00</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E231" t="n">
+        <v>93.38</v>
+      </c>
+      <c r="F231" t="n">
+        <v>93.84</v>
+      </c>
+      <c r="G231" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="H231" t="n">
+        <v>90.48999999999999</v>
+      </c>
+      <c r="I231" t="n">
+        <v>42794</v>
+      </c>
+      <c r="J231" t="n">
+        <v>4</v>
+      </c>
+      <c r="K231" t="n">
+        <v>40</v>
+      </c>
+      <c r="L231" t="n">
+        <v>-0.063</v>
+      </c>
+      <c r="M231" t="n">
+        <v>-0.203</v>
+      </c>
+      <c r="N231" t="n">
+        <v>40</v>
+      </c>
+      <c r="O231" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="P231" t="n">
+        <v>-0.092</v>
+      </c>
+      <c r="Q231" t="n">
+        <v>3.255</v>
+      </c>
+      <c r="R231" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S231" t="inlineStr">
+        <is>
+          <t>Asian Stocks Rise as AI Demand and Lower Oil Prices Lift Markets - Межа. Новини України.</t>
+        </is>
+      </c>
+      <c r="T231" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1LYUMyUDhiTlFhdDZDZWRJV3BXMzBHQmhxaWNhbHhieVJObjJpbU84WHUtaFlITmtnNWVJNW5CX1JrQ1RaTktaQ3pFYVdOZ3VmVkkxWkgtUDN2Zk90V1NwYjFlSF8?oc=5</t>
+        </is>
+      </c>
+      <c r="U231" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="V231" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="W231" t="inlineStr">
+        <is>
+          <t>Europe's STOXX 600 rallies on tech, banks strength as oil prices retreat - Reuters</t>
+        </is>
+      </c>
+      <c r="X231" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNYWF0aU9mWUM0TjNtekhpT0I0NTM1RXoydldTZDlzNVM4Q0FnRXFCLTlaLUQxdEZfMS1qeU1XV0lsNHhvc09zMTBUQV9xVFhaakdCU196dW5sQ212UHdLVjVySHo5UWczV0dVS2dnY3d2Q2dTbWRkOWFRZ0g5aTlGaEtnQkFQcno2ZjdfdndQdGdSR1c3MjdEXzNCZlhRM216di1sdllQSl9OT3pkcWRSd3p3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y231" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z231" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA231" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB231" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC231" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD231" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-09-22T09:07:39+00:00</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E232" t="n">
+        <v>100.328</v>
+      </c>
+      <c r="F232" t="n">
+        <v>100.667</v>
+      </c>
+      <c r="G232" t="n">
+        <v>100.327</v>
+      </c>
+      <c r="H232" t="n">
+        <v>100.439</v>
+      </c>
+      <c r="I232" t="n">
+        <v>0</v>
+      </c>
+      <c r="J232" t="n">
+        <v>4</v>
+      </c>
+      <c r="K232" t="n">
+        <v>39</v>
+      </c>
+      <c r="L232" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="M232" t="n">
+        <v>0.156</v>
+      </c>
+      <c r="N232" t="n">
+        <v>39</v>
+      </c>
+      <c r="O232" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="P232" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="Q232" t="n">
+        <v>4.269</v>
+      </c>
+      <c r="R232" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S232" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T232" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U232" t="inlineStr">
+        <is>
+          <t>Yuan Strengthens Against Global Rate-Hike Tide as FX Settlement Cycle Fuels Independent Rally - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="V232" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE45ZHlodXZrMDVRa2xiS1A1cWJsZVlKRmRjeG0yTFNtYmFoN01jSm5xVjZDd2Y0V0U5Nno1VjdhdHlMbnYyMDFQblBrZlRERVVlZ0FlZ3lWQWpHS2dHWTFPR1VzYWVIM1ZvYjk1M1NidnBDYTVtYXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W232" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="X232" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y232" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z232" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA232" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AB232" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC232" t="inlineStr">
+        <is>
+          <t>EUR/USD Forecast: The Euro Is Stabilising After Its Fed Sell-Off - Exchange Rates UK</t>
+        </is>
+      </c>
+      <c r="AD232" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNbHlBQS14NFJFRy1ac3ByY0F0aWN1NS1vSHNOLUQ5UmNUUzJGWUZ3dEZKZTlmaGw2aThaZVpnSmJ5NmtoTThiZlNOWVdsNF9zbXVQSXRQNGVac1dYbTJqaUxjZkVPX193XzB1d1NBbDdaQmo3YWdfbVRsU0dkUnJiRGEzTUJTejhsX0hOaTM0WE93QUpYN0Jud1RJdk5BelM2SGwxeEx4Nl9ld2hhTXFyaEdMRlZfVkFLUzRUcTRwZFo?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-09-22T09:07:39+00:00</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E233" t="n">
+        <v>7834.25</v>
+      </c>
+      <c r="F233" t="n">
+        <v>7839.5</v>
+      </c>
+      <c r="G233" t="n">
+        <v>7810.5</v>
+      </c>
+      <c r="H233" t="n">
+        <v>7833.5</v>
+      </c>
+      <c r="I233" t="n">
+        <v>90938</v>
+      </c>
+      <c r="J233" t="n">
+        <v>4</v>
+      </c>
+      <c r="K233" t="n">
+        <v>40</v>
+      </c>
+      <c r="L233" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="M233" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="N233" t="n">
+        <v>40</v>
+      </c>
+      <c r="O233" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="P233" t="n">
+        <v>-0.056</v>
+      </c>
+      <c r="Q233" t="n">
+        <v>-1.312</v>
+      </c>
+      <c r="R233" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S233" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T233" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U233" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V233" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W233" t="inlineStr">
+        <is>
+          <t>AbCellera Biologics (ABCL) Surges 34.78% as Shares Break Toward $9.81 Resistance - EMA Signal - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="X233" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPdUNOZndBWm5IMm9JRjRsTk5DNmtNQnR6YTFWMWlSTk5BT3J2TjNEdXlrMFl5Vi1sdDVyY1BybUlUU0taSnQtcktxZEV5ZkpYclc4dnBNa0lzamY3dFFRTGNMWXU5TFk3MUphb1hnak4zYS1vQ0s2NHdTeFFLOGEwdlRkcGE5VUs4a0t2bnk3SkJPMGk2RGM4VV9mclUwZmJQMGUtNXN0dUN5Z2M1U1E0cG5pckZOQlJ2TGdDSg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y233" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z233" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA233" t="inlineStr">
+        <is>
+          <t>Dow Drops 631, Nasdaq Slips 3, S&amp;P 500 Falls 34 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB233" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQVFVRNlU5aU5HaTYzZ2tnN1Nabng2cWNEd2VPQzdxcU96aHRDOFgyTUR0S3hQNXQ3MVVXQ2xDRGZKWkxNQVgyQl83eW1VQU8yX2hZVS0yR25COHJyTndBcG5xZUd2dFVvOUNPOE5BSkhnaVN4dGVQVFNreWQ0SmFFcTZwdFdmUlZqcTFsekRMcw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC233" t="inlineStr">
+        <is>
+          <t>Darden Stock Breaks $207.25 as Earnings Week Puts $202.75 Support in Focus - TradingKey</t>
+        </is>
+      </c>
+      <c r="AD233" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPcEZ2cWsxRG44VFRXZkw3dWstakNwczBXVEVEOFpPZHVnSm1XME1QV2I4RUxZckNWcGxITF9LX2pVazVVc0JuNXlfLVUzaHBwWHZoQm91d0tSZmxiY25aVVFCeHNlTXdvZ3JpNWpaeV9QTDA4YS1wdzBmQUxmVnBFZjNCQ3Z2ZXplUnR3RjBWX0VGeTd6alRyTkZsQ01rZ0VNdkRXN2VpdkpnWm1OVU9tbQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-09-22T09:07:39+00:00</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E234" t="n">
+        <v>30813</v>
+      </c>
+      <c r="F234" t="n">
+        <v>30844.75</v>
+      </c>
+      <c r="G234" t="n">
+        <v>30670</v>
+      </c>
+      <c r="H234" t="n">
+        <v>30786.5</v>
+      </c>
+      <c r="I234" t="n">
+        <v>39511</v>
+      </c>
+      <c r="J234" t="n">
+        <v>4</v>
+      </c>
+      <c r="K234" t="n">
+        <v>35</v>
+      </c>
+      <c r="L234" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="M234" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="N234" t="n">
+        <v>39</v>
+      </c>
+      <c r="O234" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="P234" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="Q234" t="n">
+        <v>-7.758</v>
+      </c>
+      <c r="R234" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S234" t="inlineStr">
+        <is>
+          <t>AI optimism lifts global stocks after Nasdaq nears record high - Financial Times</t>
+        </is>
+      </c>
+      <c r="T234" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPZExId29WNHdXUDRWQWpqQWpfV2d1LUp2Qk1hQVlwamNKQ0xrYXBJZGV1ZjYxU2FQNWNxVWgyZzY0Z1FFVTNNMUlUY3NjeEJLVmtHNVMzazdOMmE0OFRBV2JUUUdqR1ZZZEVOX0NKVmw0SDkxTlZ6T2xZSDJQSnFhbmwyY3g?oc=5</t>
+        </is>
+      </c>
+      <c r="U234" t="inlineStr">
+        <is>
+          <t>Meta Platforms surges 12% amid AI monetization rally (META:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V234" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQYmJDOXZmZDZKcUZVVjE3a0NMVWtBMG5BazdXdlZVT0ZtZEltQjdUZEl1TjY3Ri1mbFF0Mzc0Z0JiMndydnI3SHYybUpoSGZ0Z2JyV0xkdGduY1RjdHNpZndzeWl4M0NSSGhpaEd5UlF4NVc0R2NSUUhTMjRVSC12Y2FYMEc2YlhHa3hvQ0ZHN3dxdVE?oc=5</t>
+        </is>
+      </c>
+      <c r="W234" t="inlineStr">
+        <is>
+          <t>US Stocks Surge as Nasdaq Rises Over 2% to Highest Since June; Tech and Chip Stocks Lead Gains, Meta Jumps 11% - TradingKey</t>
+        </is>
+      </c>
+      <c r="X234" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxORnJ6el84X0pHd2t0MjdieXpIUVlCMUxoa1A4aEt6ZWNaY3d3LXQ0N0ZtdEw0U0ZmYjl2cVdhVnA0d1YyWi1ueE41SnJGaHVNX3dsbmgyMFg0MWZHUWlTa0otOWZGd09OcXMtVU9EWjc5clJ6ZDdiS3k0bm41ajNfdUtOaWF6UTk5aFlhVDRWbDJ3ckxEQU52czFObnExX2F4MlNtSGx5TFNjN2Vqc2hvYkcwc2dVSWJ5NTJkLURNRUhoZjZxR3o4ZHMwbUdKZ1BVTTlBQXlHSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y234" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investinglive.com</t>
+        </is>
+      </c>
+      <c r="Z234" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AA234" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB234" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC234" t="inlineStr">
+        <is>
+          <t>AI Stock Rally Lifts Nasdaq Near Record Highs as Oil Falls - Global Banking &amp; Finance Review</t>
+        </is>
+      </c>
+      <c r="AD234" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE9BOXpZbnVLRm1udm9zNXNQdFZUNWZMcGRkTWdYbmljQkRsdnVTUVFFa3lQSV9Ka3hRZ3ZRQ0RnXzBaQzRuRWlZTWlTQkpVSUdDSHdFdGJ2c3Q1c3AwWjh5bzFXRHVsM2R0OGlvRXZrYlg4QXpBMGdJN3c5SEllZFk?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-09-22T09:07:39+00:00</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E235" t="n">
+        <v>85411.96090000001</v>
+      </c>
+      <c r="F235" t="n">
+        <v>86331.5469</v>
+      </c>
+      <c r="G235" t="n">
+        <v>85150.02340000001</v>
+      </c>
+      <c r="H235" t="n">
+        <v>85882.36719999999</v>
+      </c>
+      <c r="I235" t="n">
+        <v>3664744448</v>
+      </c>
+      <c r="J235" t="n">
+        <v>4</v>
+      </c>
+      <c r="K235" t="n">
+        <v>34</v>
+      </c>
+      <c r="L235" t="n">
+        <v>-0.273</v>
+      </c>
+      <c r="M235" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="N235" t="n">
+        <v>36</v>
+      </c>
+      <c r="O235" t="n">
+        <v>0.277</v>
+      </c>
+      <c r="P235" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="Q235" t="n">
+        <v>-0.662</v>
+      </c>
+      <c r="R235" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S235" t="inlineStr">
+        <is>
+          <t>Bitcoin jumps nearly 5% to cross $85,000 as strong ETF inflows and institutional buying boost crypto momen - The Economic Times</t>
+        </is>
+      </c>
+      <c r="T235" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxQcGFmOUJLZlJEeERGcTlqN016NzFZemFrenJKcFpQa1BZMEZ6Z2dOYldneU9CaGk4dzBJSmZRVUs2eHhscUwtMmpKcE1GTHZQZWRiM0NhZXJGc2ZCeko4YWptOWVWX0dpbWx4RVUwODU3cmtyVUlVc0N1M252X1ZqaEtPNkEybHBfdWFOc3NNUXQ2MENSLVhrdUFKT29XQlNnYVRtckxLVjhYX0lkVWkyeHdsak9TcHRMWS1DOURlOUdoaHpCckZOX3NLazZVMmZRMWtKb0kyX2YwN1J6bV8wUEtxN1lBWmx5cExlbVVBYTBlRDFKb2FITHBoWUtiOFRPVGxwTnlrXzlWdHRRdWVzbdIBlgJBVV95cUxPNlNZM3JYRkx6cXBwUURPeHBJX1lMbzcyTUx4VlBlRVEydWtzRW90WDhObFZOekgxeEtoY244aFlmYUY3U21pUGxoUE52M05KOUZmeDRwV3RqNWhvbmVuMUNxZFZrQkhpbF93dm1FckZ2Y05YQWluTE9DVnZpYldOeWgxamI0YTFNLWNaUGdiZ2FDMTUxMHNKQ0RScXYxWDItWjlMMzdiUy1vWGxpY2I0YjhOSWY1dEp2TUVuZTVRSllrR2xtdUlmWHU1dXVrZXBjWHJ3SnM2Y25pbnJyWTY5OW9rWm1JXzhTcXA4azVHaDR0S0NvTkhpRklzUlRONUxHSmt3aXpLTWQ3eHFjekFfRkZWMFpWdw?oc=5</t>
+        </is>
+      </c>
+      <c r="U235" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to $87K, sparking talk of a $90K breakthrough amid strong inflows and market optimism. - Pluang</t>
+        </is>
+      </c>
+      <c r="V235" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNVml5bmpucDhzSmdrTF83UHZhU2t5cWQtaXE3QXJYVFhSSHU5MlROTTUtOG15aU5Cek5WM0Y4Z1FUQkFpcjdXUmxsLXhlX1JtRHI0eThJem1QSUFDanlQaHJqd2VzMnVsZElqaVJwVUZ1TU5WalB3eDd2MGlORXR2MVgxQWVnVTU2YnMxOWFNM3E0TW0zcEZzS0RleGxFYzl1TU41aU53?oc=5</t>
+        </is>
+      </c>
+      <c r="W235" t="inlineStr">
+        <is>
+          <t>Bitcoin surged to an eight-month high above $85,000 as oil fell and ETF inflows returned - qz.com</t>
+        </is>
+      </c>
+      <c r="X235" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9BRHhsSDNaZ2VlVnhzYmRsci1zNk1kQ2JWNHJxNTNVRHFDSHFqcmVoVFg2TkJxYTdZMUhfMEJpb1hFS3RabDlJcVZZWEh4M3VJUUpaX0JUSWtHd0pxNUctNzg3Nkx0Q2JoT21EN2cwV1ZtQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y235" t="inlineStr">
+        <is>
+          <t>Bitcoin price tags $86K as analysis sees crypto in ‘new bull market’ - TradingView</t>
+        </is>
+      </c>
+      <c r="Z235" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOdGloQjlFZUswdXdaQnAyOTUzbmR4aGRnODZTcGRaZUs5ODBhaXpNWlM4bGl4U2d3aElrSGVEUmJfNnJQYzZqNFRWVS05eTkxeXRkTnltTTIxOV9sZFpaRFlhbll5OEdZRjJBNlpiX2UxOVltYURDQ3dhMl9rZk9JWVVCMGJtWGRkYy11Wkc2QlU2cDVEcHJMWDhlS3d0RnZ2SU5nMUU2STRMVlJSeFUxY3Nkak80Sm1ZYk0xV2VfalR5bGhpaS1YcA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA235" t="inlineStr">
+        <is>
+          <t>Bitcoin price rebounds above $85K after smaller holders reduce exposure amid market shakeout - Pluang</t>
+        </is>
+      </c>
+      <c r="AB235" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOTHNfMTFCdDN4RGF2U2o2a2JaSWRVMzNXZXdBRE5nTlEtWGVJbTFhTjNyRHNJSWNSdlc4NDRCdzlYT3RIa0NfWDkybVdDcEhuMDVPSExqSTlmcjgwT1FmNXQ3TVdWOFZJc0lXYV9MQThlTWRObG5vbkI4b0hiVlgzZk1LSnA3dUVhWS1nd3lscklBWWM?oc=5</t>
+        </is>
+      </c>
+      <c r="AC235" t="inlineStr">
+        <is>
+          <t>Bitcoin clears $85K as $648M in shorts are liquidated, per CoinGlass - Altcoin Buzz</t>
+        </is>
+      </c>
+      <c r="AD235" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxPdldlWXhkNnpXb1FYcEdMZHZ0WWtiSHpvMEo1RGd4ejZvQjVTcGFadWhURVFWcks2T2dlR0Y1cmxremJ0YS1DaFI1bW5hN3ptc0FfYWltM2lrdi0yNHo2YXBFdWxOSVBraXNqRGpaWUxXLWxPc0VFMEVFVi01WFUyOHlQZjNEcEUwVUFJ?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-22 16:30 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD235"/>
+  <dimension ref="A1:AD241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29585,6 +29585,762 @@
       <c r="AD235" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxPdldlWXhkNnpXb1FYcEdMZHZ0WWtiSHpvMEo1RGd4ejZvQjVTcGFadWhURVFWcks2T2dlR0Y1cmxremJ0YS1DaFI1bW5hN3ptc0FfYWltM2lrdi0yNHo2YXBFdWxOSVBraXNqRGpaWUxXLWxPc0VFMEVFVi01WFUyOHlQZjNEcEUwVUFJ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-09-22T16:28:07+00:00</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E236" t="n">
+        <v>4371.6001</v>
+      </c>
+      <c r="F236" t="n">
+        <v>4381.8999</v>
+      </c>
+      <c r="G236" t="n">
+        <v>4351.7998</v>
+      </c>
+      <c r="H236" t="n">
+        <v>4361.7002</v>
+      </c>
+      <c r="I236" t="n">
+        <v>38346</v>
+      </c>
+      <c r="J236" t="n">
+        <v>4</v>
+      </c>
+      <c r="K236" t="n">
+        <v>40</v>
+      </c>
+      <c r="L236" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="M236" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="N236" t="n">
+        <v>40</v>
+      </c>
+      <c r="O236" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="P236" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="Q236" t="n">
+        <v>0.719</v>
+      </c>
+      <c r="R236" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S236" t="inlineStr">
+        <is>
+          <t>Goldman Sachs Maintains Bullish Gold Outlook - businesskorea.co.kr</t>
+        </is>
+      </c>
+      <c r="T236" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE5aM0FhTU0tdzZUU1ZGcnJxZm1FN1pFVURiQXdyWmxKUi1MRGgzVWdEd3dTaVhWcUZnd01xNHlWaHpuSGowN29lQ1NBZjYxTUNQejYtc3p3VGdaNS0ySENZZFFOanpzV2R6RUZ4WWxBU05WZGU1?oc=5</t>
+        </is>
+      </c>
+      <c r="U236" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V236" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W236" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X236" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y236" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="Z236" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA236" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="AB236" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC236" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD236" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-09-22T16:28:07+00:00</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E237" t="n">
+        <v>90.39</v>
+      </c>
+      <c r="F237" t="n">
+        <v>92.06</v>
+      </c>
+      <c r="G237" t="n">
+        <v>89.48</v>
+      </c>
+      <c r="H237" t="n">
+        <v>91.73999999999999</v>
+      </c>
+      <c r="I237" t="n">
+        <v>117063</v>
+      </c>
+      <c r="J237" t="n">
+        <v>4</v>
+      </c>
+      <c r="K237" t="n">
+        <v>40</v>
+      </c>
+      <c r="L237" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M237" t="n">
+        <v>-0.208</v>
+      </c>
+      <c r="N237" t="n">
+        <v>40</v>
+      </c>
+      <c r="O237" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="P237" t="n">
+        <v>-0.057</v>
+      </c>
+      <c r="Q237" t="n">
+        <v>4.987</v>
+      </c>
+      <c r="R237" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S237" t="inlineStr">
+        <is>
+          <t>Gasoline blending economics lift European naphtha demand - Quantum Commodity Intelligence</t>
+        </is>
+      </c>
+      <c r="T237" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNX0FiaEhNRzh6b0dnUVE1OTk2bC1hWkxTS3AzNXR6LXFkVlZUblBLOWtxbmNOTGxmTlg2ZWw0eEVoOXZiZTMzR0VhUVQ3QW1rTjRvR1R1blpqcWRBUHJaXzNHblZnaVVuZXJOSGh6dWJtdmxsNHk3VWNPWWZGQmRzM2g3ZnNaNWU5TGgyNmFpQlNLT19lc1ZYS0RJbGpBa2xP?oc=5</t>
+        </is>
+      </c>
+      <c r="U237" t="inlineStr">
+        <is>
+          <t>Surfactant Blend for Oil Recovery Market Forecast to Expand Toward 2035, Driven by Mature Field Revitalization - IndexBox</t>
+        </is>
+      </c>
+      <c r="V237" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPdDhJNWNKS3hTTjdibXRXTU55SkxhYW13S1Z2ZFp0OExVNVd5bTRjdzJzc3RHb3FpLUtmR2RhTkI3T0R5WlBNeTBOeHJHUjFyYWNUTU1od1lzRDBEWldUQjVlMFZpWmI0QzNzVGEwZ3U0S2tfSC0yVi11cVJEbkZTQUs4SU1HYTdJT2l0N2k2ZGxwNmRfdlUyTzRfV1lRY2tTb3dXYjl0Q0szWldlR0Z0aVA1RG5sTUpkUmRCbHltcG9rMUkxOXZueGM1aHZqWm4zWGhiUG9R?oc=5</t>
+        </is>
+      </c>
+      <c r="W237" t="inlineStr">
+        <is>
+          <t>Asian Stocks Rise as AI Demand and Lower Oil Prices Lift Markets - Межа. Новини України.</t>
+        </is>
+      </c>
+      <c r="X237" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1LYUMyUDhiTlFhdDZDZWRJV3BXMzBHQmhxaWNhbHhieVJObjJpbU84WHUtaFlITmtnNWVJNW5CX1JrQ1RaTktaQ3pFYVdOZ3VmVkkxWkgtUDN2Zk90V1NwYjFlSF8?oc=5</t>
+        </is>
+      </c>
+      <c r="Y237" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z237" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA237" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB237" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+      <c r="AC237" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD237" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-09-22T16:28:07+00:00</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>100.464</v>
+      </c>
+      <c r="F238" t="n">
+        <v>100.703</v>
+      </c>
+      <c r="G238" t="n">
+        <v>100.422</v>
+      </c>
+      <c r="H238" t="n">
+        <v>100.686</v>
+      </c>
+      <c r="I238" t="n">
+        <v>0</v>
+      </c>
+      <c r="J238" t="n">
+        <v>4</v>
+      </c>
+      <c r="K238" t="n">
+        <v>39</v>
+      </c>
+      <c r="L238" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="M238" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="N238" t="n">
+        <v>39</v>
+      </c>
+      <c r="O238" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="P238" t="n">
+        <v>-0.08599999999999999</v>
+      </c>
+      <c r="Q238" t="n">
+        <v>3.284</v>
+      </c>
+      <c r="R238" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S238" t="inlineStr">
+        <is>
+          <t>Safe-haven demand supports the US dollar; can Australia's better-than-expected GDP rescue the Australian dollar? - Moomoo</t>
+        </is>
+      </c>
+      <c r="T238" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPa2ZIYy1JQkhiaHZMZmZkNXhDd3M3S28wVEphV0Q5ODA0VFAwdExrYnFHSzRjRDhMMzFUTnY3c2g3RE5CbnFVaHI5cEstYjRJUGRjUV8wUlBYUE5CUFRhcWJGT1ZDcTRab1RIX1BONXpSZ1VVY1c4UENQd3Z0Z0wyS0JpOVhfcVVVRzd3WnpOY1JpdGViSTlZTl9LSVhONmM?oc=5</t>
+        </is>
+      </c>
+      <c r="U238" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="V238" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="W238" t="inlineStr">
+        <is>
+          <t>Gold price seen trading $4,000-4,500 range as strong dollar checks safe-haven demand - Khaleej Times</t>
+        </is>
+      </c>
+      <c r="X238" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQdDhNcUJyZkVSOWs4clk4Zmc1Z1hkSjY4ZVhNTkFGVEFKRzdzOFFxQm5mczhSQ2lSZ2daYnBHc0hhSkQzTFlaZ3NNa01wWEs1RFdiODFqY3NKOE1ZVUNSU24wZnl0R3VRUHhsWURpRGJoejZwNXRzREFHd2l0ZUZqRHNOWDRLdnd4SzQ1cENMZkVnTFRXMzJZemhIdWZUbm5heFQyRlN1RGNVQnU2bEctV3ZnTklleDIyY0lN0gHDAUFVX3lxTE1zQ1JjcnJXUE50Q0ZBTmRPMGlMS3dzWHRXcV9MbWprTE82d3JTdlluSFRORGJQWlh3ZmpqcmRoaDF1bVdlaEkzT2FiWk5TODBCZVNjMl9FY0hPZ1NKT2NycEFNY2QyM3JXb043UXRtUG43VzlXc1FCNlVBOV9nTElwVEdFV04xcURDOEdrVkRIbWlXanRUZVRXeExseHpiR0N6NGtSbW12YnFmdmJwNkliVlJUVGFnMW9jMEg3X0FHREdBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y238" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z238" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA238" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AB238" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC238" t="inlineStr">
+        <is>
+          <t>Gold rebounds from low as dollar weakens - Arab News</t>
+        </is>
+      </c>
+      <c r="AD238" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxOTnl6bjhtVDFfNHNGVUZCc2dxQkp1aG5OR2V6S3B0RE5CUUxpLWJRbkR3WGdqdElZckZnRDlLdVdjQzFBTE01Vjk2dGpLeVp2MTJ5VTNMWk1XTlhFeFRpVmtoNjI3YzlYZ2g0bGdTemRnR3RZbkJBdjlDS3hkMmlDU0paVEhxNElpa1E?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-09-22T16:28:07+00:00</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E239" t="n">
+        <v>7837</v>
+      </c>
+      <c r="F239" t="n">
+        <v>7848.5</v>
+      </c>
+      <c r="G239" t="n">
+        <v>7822.25</v>
+      </c>
+      <c r="H239" t="n">
+        <v>7826.75</v>
+      </c>
+      <c r="I239" t="n">
+        <v>497981</v>
+      </c>
+      <c r="J239" t="n">
+        <v>4</v>
+      </c>
+      <c r="K239" t="n">
+        <v>38</v>
+      </c>
+      <c r="L239" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="M239" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="N239" t="n">
+        <v>40</v>
+      </c>
+      <c r="O239" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="P239" t="n">
+        <v>-0.046</v>
+      </c>
+      <c r="Q239" t="n">
+        <v>2.912</v>
+      </c>
+      <c r="R239" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S239" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="T239" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="U239" t="inlineStr">
+        <is>
+          <t>GRAIL: Stock Surges As Market Digests FDA Briefing Docs - I Broadly Concur (Rating Upgrade) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V239" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPZ1M2ZmtfaHI5NjY2YjVyMUZBdHI1M1IxM09rLXVncjFHclVfUnRQRmlUN3p2S3Q4bnpGa3VMOURZbVRYS3RqQUdmdGFQM0xvbFotZEhhcHRQcHp6eHJFeDZTcVYyVFRqaUJEdy1fZ01TYkdpSEd1S05RTElsTjVnMjItbVIyVjM4a2tWbV9Md3NOc19JMy1WUmJGYzJXaElpQ3M4WE9YVDZfNzVqcGR3cVk1SUYwZGtJ?oc=5</t>
+        </is>
+      </c>
+      <c r="W239" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - Resistance Breakout Stocks - dars.gov.et</t>
+        </is>
+      </c>
+      <c r="X239" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQajNlZ0pyR21ESWttMzFab0VjcFktLTBhZmp0ODZaWHJfT0JHWEdHd3RhRFVUTVFYVWZaUjdnaE9HMzZmOEljWDlrRlJHZXF0TWdVRHBaMDhXNjRwTy1SNjA1ZTZ1d04zUFB3MmpZUk9FUXo3N0tPNFZZbFl1Mk56WkN5SXJXckVEbGlpOFJEcnVYTW11c2tYT0FvUTJWem84RXBwcg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y239" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z239" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA239" t="inlineStr">
+        <is>
+          <t>Darden Stock Breaks $207.25 as Earnings Week Puts $202.75 Support in Focus - TradingKey</t>
+        </is>
+      </c>
+      <c r="AB239" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPcEZ2cWsxRG44VFRXZkw3dWstakNwczBXVEVEOFpPZHVnSm1XME1QV2I4RUxZckNWcGxITF9LX2pVazVVc0JuNXlfLVUzaHBwWHZoQm91d0tSZmxiY25aVVFCeHNlTXdvZ3JpNWpaeV9QTDA4YS1wdzBmQUxmVnBFZjNCQ3Z2ZXplUnR3RjBWX0VGeTd6alRyTkZsQ01rZ0VNdkRXN2VpdkpnWm1OVU9tbQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC239" t="inlineStr">
+        <is>
+          <t>Nearly Two-Thirds Of The S&amp;P 500 Already Sell Off In A Big Way - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD239" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPUDR4Xzk0Qlp6SXVpbmZLZlFIR2QyODRNaUNzSWdCRm1yN1pMUFlNeVExZFBwT2xkVmJVa19hZjRNTVNXZ0g2NWp2SWlmVlVBV0U4M24yTlBCT3liTDk4X2RHelA0OXZkZ3F6cWxfa1ZQTS1YTTZJVVNjaWI3bDBHNEVENmxGOExJRER6SkN1Vk45MnRsM3hnRnpPazZGU0pYV2Yxc3FKZVluZw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-09-22T16:28:07+00:00</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E240" t="n">
+        <v>30753</v>
+      </c>
+      <c r="F240" t="n">
+        <v>30997.5</v>
+      </c>
+      <c r="G240" t="n">
+        <v>30748.75</v>
+      </c>
+      <c r="H240" t="n">
+        <v>30912.25</v>
+      </c>
+      <c r="I240" t="n">
+        <v>211470</v>
+      </c>
+      <c r="J240" t="n">
+        <v>4</v>
+      </c>
+      <c r="K240" t="n">
+        <v>35</v>
+      </c>
+      <c r="L240" t="n">
+        <v>-0.322</v>
+      </c>
+      <c r="M240" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="N240" t="n">
+        <v>39</v>
+      </c>
+      <c r="O240" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="P240" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="Q240" t="n">
+        <v>-6.764</v>
+      </c>
+      <c r="R240" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S240" t="inlineStr">
+        <is>
+          <t>AI optimism lifts global stocks after Nasdaq nears record high - Financial Times</t>
+        </is>
+      </c>
+      <c r="T240" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPZExId29WNHdXUDRWQWpqQWpfV2d1LUp2Qk1hQVlwamNKQ0xrYXBJZGV1ZjYxU2FQNWNxVWgyZzY0Z1FFVTNNMUlUY3NjeEJLVmtHNVMzazdOMmE0OFRBV2JUUUdqR1ZZZEVOX0NKVmw0SDkxTlZ6T2xZSDJQSnFhbmwyY3g?oc=5</t>
+        </is>
+      </c>
+      <c r="U240" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="V240" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W240" t="inlineStr">
+        <is>
+          <t>Nasdaq Hits Record High Ahead of Trump-Xi Meeting - TradingView</t>
+        </is>
+      </c>
+      <c r="X240" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxPVXdNbFk0MFJlelpwVzBnWWVlU3hkQkFPSVplSVBOQ0w5ellWSlIzajFDc2tPZTFsQlFTeDkyei1ob0dvUzc5SmFyQXQ2WWQ4bGhyMGhqbk1JUC1kLU1kUFMtNnNNWHRTVHcxT1JMb2phME5zQWc1eVpsQWZvbjdsa0NOZnhBaFQyOTRvMng5WnYydmszR0V0cHFnbW9lSHJIQnFFQ25naGJnYkhSS2c?oc=5</t>
+        </is>
+      </c>
+      <c r="Y240" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="Z240" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA240" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB240" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC240" t="inlineStr">
+        <is>
+          <t>AI Stock Rally Lifts Nasdaq Near Record Highs as Oil Falls - Global Banking &amp; Finance Review</t>
+        </is>
+      </c>
+      <c r="AD240" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE9BOXpZbnVLRm1udm9zNXNQdFZUNWZMcGRkTWdYbmljQkRsdnVTUVFFa3lQSV9Ka3hRZ3ZRQ0RnXzBaQzRuRWlZTWlTQkpVSUdDSHdFdGJ2c3Q1c3AwWjh5bzFXRHVsM2R0OGlvRXZrYlg4QXpBMGdJN3c5SEllZFk?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-09-22T16:28:07+00:00</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E241" t="n">
+        <v>86019.17969999999</v>
+      </c>
+      <c r="F241" t="n">
+        <v>86734</v>
+      </c>
+      <c r="G241" t="n">
+        <v>85452.92969999999</v>
+      </c>
+      <c r="H241" t="n">
+        <v>86118.03909999999</v>
+      </c>
+      <c r="I241" t="n">
+        <v>5689712640</v>
+      </c>
+      <c r="J241" t="n">
+        <v>4</v>
+      </c>
+      <c r="K241" t="n">
+        <v>36</v>
+      </c>
+      <c r="L241" t="n">
+        <v>-0.096</v>
+      </c>
+      <c r="M241" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="N241" t="n">
+        <v>36</v>
+      </c>
+      <c r="O241" t="n">
+        <v>0.314</v>
+      </c>
+      <c r="P241" t="n">
+        <v>-0.066</v>
+      </c>
+      <c r="Q241" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="R241" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S241" t="inlineStr">
+        <is>
+          <t>Bitcoin jumps nearly 5% to cross $85,000 as strong ETF inflows and institutional buying boost crypto momen - economictimes.com</t>
+        </is>
+      </c>
+      <c r="T241" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxQcGFmOUJLZlJEeERGcTlqN016NzFZemFrenJKcFpQa1BZMEZ6Z2dOYldneU9CaGk4dzBJSmZRVUs2eHhscUwtMmpKcE1GTHZQZWRiM0NhZXJGc2ZCeko4YWptOWVWX0dpbWx4RVUwODU3cmtyVUlVc0N1M252X1ZqaEtPNkEybHBfdWFOc3NNUXQ2MENSLVhrdUFKT29XQlNnYVRtckxLVjhYX0lkVWkyeHdsak9TcHRMWS1DOURlOUdoaHpCckZOX3NLazZVMmZRMWtKb0kyX2YwN1J6bV8wUEtxN1lBWmx5cExlbVVBYTBlRDFKb2FITHBoWUtiOFRPVGxwTnlrXzlWdHRRdWVzbdIBlgJBVV95cUxPNlNZM3JYRkx6cXBwUURPeHBJX1lMbzcyTUx4VlBlRVEydWtzRW90WDhObFZOekgxeEtoY244aFlmYUY3U21pUGxoUE52M05KOUZmeDRwV3RqNWhvbmVuMUNxZFZrQkhpbF93dm1FckZ2Y05YQWluTE9DVnZpYldOeWgxamI0YTFNLWNaUGdiZ2FDMTUxMHNKQ0RScXYxWDItWjlMMzdiUy1vWGxpY2I0YjhOSWY1dEp2TUVuZTVRSllrR2xtdUlmWHU1dXVrZXBjWHJ3SnM2Y25pbnJyWTY5OW9rWm1JXzhTcXA4azVHaDR0S0NvTkhpRklzUlRONUxHSmt3aXpLTWQ3eHFjekFfRkZWMFpWdw?oc=5</t>
+        </is>
+      </c>
+      <c r="U241" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to $87K, sparking talk of a $90K breakthrough amid strong inflows and market optimism. - Pluang</t>
+        </is>
+      </c>
+      <c r="V241" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNVml5bmpucDhzSmdrTF83UHZhU2t5cWQtaXE3QXJYVFhSSHU5MlROTTUtOG15aU5Cek5WM0Y4Z1FUQkFpcjdXUmxsLXhlX1JtRHI0eThJem1QSUFDanlQaHJqd2VzMnVsZElqaVJwVUZ1TU5WalB3eDd2MGlORXR2MVgxQWVnVTU2YnMxOWFNM3E0TW0zcEZzS0RleGxFYzl1TU41aU53?oc=5</t>
+        </is>
+      </c>
+      <c r="W241" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to 8-month high above $85,000 - qz.com</t>
+        </is>
+      </c>
+      <c r="X241" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9BRHhsSDNaZ2VlVnhzYmRsci1zNk1kQ2JWNHJxNTNVRHFDSHFqcmVoVFg2TkJxYTdZMUhfMEJpb1hFS3RabDlJcVZZWEh4M3VJUUpaX0JUSWtHd0pxNUctNzg3Nkx0Q2JoT21EN2cwV1ZtQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y241" t="inlineStr">
+        <is>
+          <t>Bitcoin price rebounds above $85K after smaller holders reduce exposure amid market shakeout - Pluang</t>
+        </is>
+      </c>
+      <c r="Z241" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOTHNfMTFCdDN4RGF2U2o2a2JaSWRVMzNXZXdBRE5nTlEtWGVJbTFhTjNyRHNJSWNSdlc4NDRCdzlYT3RIa0NfWDkybVdDcEhuMDVPSExqSTlmcjgwT1FmNXQ3TVdWOFZJc0lXYV9MQThlTWRObG5vbkI4b0hiVlgzZk1LSnA3dUVhWS1nd3lscklBWWM?oc=5</t>
+        </is>
+      </c>
+      <c r="AA241" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - Morningstar</t>
+        </is>
+      </c>
+      <c r="AB241" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC241" t="inlineStr">
+        <is>
+          <t>Bitcoin crashes, odds turn darker as MSTR, APLD lead crypto-stocks bloodbath - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="AD241" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPeGxFNjVybVhxTFdqQXBJUG1INDVZTllFTlpRZW9mZHdIMlBVOFEwSnNrZ29xYXRwelREYVhGRzBxWmJvMm16TFNONDJzQVVIQkNDM1dtOHVvbi13U0pRYUIzTnFFWEpPVmMwQTU2d00zbHQyd0hUM0h4YjZfT2J0ckJVdV91c1lGUERRLVZWazlhS3ZqOS1FQzZkano0SFUtS01sLUduc2JMMVJZcVNFZmlIOEUtX1k?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-22 22:50 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD241"/>
+  <dimension ref="A1:AD247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30341,6 +30341,762 @@
       <c r="AD241" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPeGxFNjVybVhxTFdqQXBJUG1INDVZTllFTlpRZW9mZHdIMlBVOFEwSnNrZ29xYXRwelREYVhGRzBxWmJvMm16TFNONDJzQVVIQkNDM1dtOHVvbi13U0pRYUIzTnFFWEpPVmMwQTU2d00zbHQyd0hUM0h4YjZfT2J0ckJVdV91c1lGUERRLVZWazlhS3ZqOS1FQzZkano0SFUtS01sLUduc2JMMVJZcVNFZmlIOEUtX1k?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:47:55+00:00</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>GCJ27.CMX</t>
+        </is>
+      </c>
+      <c r="E242" t="n">
+        <v>4448.3999</v>
+      </c>
+      <c r="F242" t="n">
+        <v>4450.2002</v>
+      </c>
+      <c r="G242" t="n">
+        <v>4438.2998</v>
+      </c>
+      <c r="H242" t="n">
+        <v>4450.2002</v>
+      </c>
+      <c r="I242" t="n">
+        <v>1669</v>
+      </c>
+      <c r="J242" t="n">
+        <v>4</v>
+      </c>
+      <c r="K242" t="n">
+        <v>39</v>
+      </c>
+      <c r="L242" t="n">
+        <v>-0.019</v>
+      </c>
+      <c r="M242" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="N242" t="n">
+        <v>40</v>
+      </c>
+      <c r="O242" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="P242" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="Q242" t="n">
+        <v>1.688</v>
+      </c>
+      <c r="R242" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S242" t="inlineStr">
+        <is>
+          <t>Goldman Sachs Maintains Bullish Gold Outlook - Businesskorea</t>
+        </is>
+      </c>
+      <c r="T242" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE5aM0FhTU0tdzZUU1ZGcnJxZm1FN1pFVURiQXdyWmxKUi1MRGgzVWdEd3dTaVhWcUZnd01xNHlWaHpuSGowN29lQ1NBZjYxTUNQejYtc3p3VGdaNS0ySENZZFFOanpzV2R6RUZ4WWxBU05WZGU1?oc=5</t>
+        </is>
+      </c>
+      <c r="U242" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V242" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W242" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X242" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y242" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="Z242" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA242" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB242" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC242" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD242" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:47:55+00:00</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E243" t="n">
+        <v>89.59999999999999</v>
+      </c>
+      <c r="F243" t="n">
+        <v>90.93000000000001</v>
+      </c>
+      <c r="G243" t="n">
+        <v>88.67</v>
+      </c>
+      <c r="H243" t="n">
+        <v>89.68000000000001</v>
+      </c>
+      <c r="I243" t="n">
+        <v>78404</v>
+      </c>
+      <c r="J243" t="n">
+        <v>4</v>
+      </c>
+      <c r="K243" t="n">
+        <v>40</v>
+      </c>
+      <c r="L243" t="n">
+        <v>-0.112</v>
+      </c>
+      <c r="M243" t="n">
+        <v>-0.233</v>
+      </c>
+      <c r="N243" t="n">
+        <v>40</v>
+      </c>
+      <c r="O243" t="n">
+        <v>0.331</v>
+      </c>
+      <c r="P243" t="n">
+        <v>-0.054</v>
+      </c>
+      <c r="Q243" t="n">
+        <v>4.381</v>
+      </c>
+      <c r="R243" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S243" t="inlineStr">
+        <is>
+          <t>Surfactant Blend for Oil Recovery Market Forecast to Expand Toward 2035, Driven by Mature Field Revitalization - IndexBox</t>
+        </is>
+      </c>
+      <c r="T243" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPdDhJNWNKS3hTTjdibXRXTU55SkxhYW13S1Z2ZFp0OExVNVd5bTRjdzJzc3RHb3FpLUtmR2RhTkI3T0R5WlBNeTBOeHJHUjFyYWNUTU1od1lzRDBEWldUQjVlMFZpWmI0QzNzVGEwZ3U0S2tfSC0yVi11cVJEbkZTQUs4SU1HYTdJT2l0N2k2ZGxwNmRfdlUyTzRfV1lRY2tTb3dXYjl0Q0szWldlR0Z0aVA1RG5sTUpkUmRCbHltcG9rMUkxOXZueGM1aHZqWm4zWGhiUG9R?oc=5</t>
+        </is>
+      </c>
+      <c r="U243" t="inlineStr">
+        <is>
+          <t>Asian Stocks Rise as AI Demand and Lower Oil Prices Lift Markets - Межа. Новини України.</t>
+        </is>
+      </c>
+      <c r="V243" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1LYUMyUDhiTlFhdDZDZWRJV3BXMzBHQmhxaWNhbHhieVJObjJpbU84WHUtaFlITmtnNWVJNW5CX1JrQ1RaTktaQ3pFYVdOZ3VmVkkxWkgtUDN2Zk90V1NwYjFlSF8?oc=5</t>
+        </is>
+      </c>
+      <c r="W243" t="inlineStr">
+        <is>
+          <t>Meta leads tech rally as oil prices fall - ft.com</t>
+        </is>
+      </c>
+      <c r="X243" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNRVVOOWNyQWNOZWc4NU9rMFFDZXhNZG91cDhxWFZTM0NXWnBCd2ktRkhnbXJzRGU3cUstOTZ2Y210a0ZpQ3lncF94endwRS15ell2TW1MSXo1WHpRQzFzNVgzLUd1Ymc0RGN6WVlwSkdweEVlV0RTZG45TnQ0RVpkS2x1dlA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y243" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z243" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA243" t="inlineStr">
+        <is>
+          <t>Oil prices hover around $100 a barrel - Transport Topics</t>
+        </is>
+      </c>
+      <c r="AB243" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTE1wYUFKb2JqTDVBUWJhODRORTIyWWh6bzZOMUFDd0ZzS1JUVzJobnd6MlpwNE5mRk5XRDdOVGNubXFtTXZDbktuLWNIZ3FQaVBjUHp2cE16NUdGbENfZHpXTEFEYlhpcDhpWnpz?oc=5</t>
+        </is>
+      </c>
+      <c r="AC243" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD243" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:47:55+00:00</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E244" t="n">
+        <v>100.601</v>
+      </c>
+      <c r="F244" t="n">
+        <v>100.605</v>
+      </c>
+      <c r="G244" t="n">
+        <v>100.481</v>
+      </c>
+      <c r="H244" t="n">
+        <v>100.541</v>
+      </c>
+      <c r="I244" t="n">
+        <v>0</v>
+      </c>
+      <c r="J244" t="n">
+        <v>4</v>
+      </c>
+      <c r="K244" t="n">
+        <v>39</v>
+      </c>
+      <c r="L244" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="M244" t="n">
+        <v>0.187</v>
+      </c>
+      <c r="N244" t="n">
+        <v>40</v>
+      </c>
+      <c r="O244" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="P244" t="n">
+        <v>-0.06900000000000001</v>
+      </c>
+      <c r="Q244" t="n">
+        <v>5.751</v>
+      </c>
+      <c r="R244" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S244" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T244" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U244" t="inlineStr">
+        <is>
+          <t>Gold price seen trading $4,000-4,500 range as strong dollar checks safe-haven demand - Khaleej Times</t>
+        </is>
+      </c>
+      <c r="V244" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQdDhNcUJyZkVSOWs4clk4Zmc1Z1hkSjY4ZVhNTkFGVEFKRzdzOFFxQm5mczhSQ2lSZ2daYnBHc0hhSkQzTFlaZ3NNa01wWEs1RFdiODFqY3NKOE1ZVUNSU24wZnl0R3VRUHhsWURpRGJoejZwNXRzREFHd2l0ZUZqRHNOWDRLdnd4SzQ1cENMZkVnTFRXMzJZemhIdWZUbm5heFQyRlN1RGNVQnU2bEctV3ZnTklleDIyY0lN0gHDAUFVX3lxTE1zQ1JjcnJXUE50Q0ZBTmRPMGlMS3dzWHRXcV9MbWprTE82d3JTdlluSFRORGJQWlh3ZmpqcmRoaDF1bVdlaEkzT2FiWk5TODBCZVNjMl9FY0hPZ1NKT2NycEFNY2QyM3JXb043UXRtUG43VzlXc1FCNlVBOV9nTElwVEdFV04xcURDOEdrVkRIbWlXanRUZVRXeExseHpiR0N6NGtSbW12YnFmdmJwNkliVlJUVGFnMW9jMEg3X0FHREdBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="W244" t="inlineStr">
+        <is>
+          <t>Canadian Dollar strengthens on rising oil prices ahead of potential US-Iran talks - FXStreet</t>
+        </is>
+      </c>
+      <c r="X244" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxObmphYlI3SXdxcVRpa3dJSldPd2VZeXJiYkl5Mzhia3pKWGlhd2poUEdNS2Jfc21BdkVoVktodE5HcVNJWTRWaDFDZjVYTTNkSE9YQjRBVzZzQTY3NUZuWWg3U3paSEdiN3h0N0R2UjBPc0ZERTNFMFUzUFpqa0xGZHJaLUpwQjlUa3Z3cDZNaDNTOGRkSlFOb2VzUjZDd0gwV0xEVEVCcWhCYktmemlOUlJWeGM3dHJZcUg5ME05aF9vQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y244" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z244" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA244" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AB244" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC244" t="inlineStr">
+        <is>
+          <t>Dovish Fed Bets Pummel Dollar, Boost Gold Ahead of NFP - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD244" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPZDNJaUJnTUhOckR3ODFMRjN3M3QtZ1NzUmtvYnRUOVlyWEo2Nzg4d3l5Tkl4SFNRMVJCUnlNeGxUYm5NQkxpNmxEdzVpU3ZHTkhRUXh0bEdhNld2WHFBVmNCRTBEY2dsUkxqVlYtYTUwX21GR1JZNnZjazk2OXBjNW80dWo3Nmx5TXZYLUY0WkZLei14eWV4dDlkRGVheWM?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:47:55+00:00</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E245" t="n">
+        <v>7837.5</v>
+      </c>
+      <c r="F245" t="n">
+        <v>7846.75</v>
+      </c>
+      <c r="G245" t="n">
+        <v>7826</v>
+      </c>
+      <c r="H245" t="n">
+        <v>7832.75</v>
+      </c>
+      <c r="I245" t="n">
+        <v>348607</v>
+      </c>
+      <c r="J245" t="n">
+        <v>4</v>
+      </c>
+      <c r="K245" t="n">
+        <v>39</v>
+      </c>
+      <c r="L245" t="n">
+        <v>-0.098</v>
+      </c>
+      <c r="M245" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="N245" t="n">
+        <v>40</v>
+      </c>
+      <c r="O245" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="P245" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="Q245" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="R245" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S245" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T245" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U245" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V245" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W245" t="inlineStr">
+        <is>
+          <t>GRAIL: Stock Surges As Market Digests FDA Briefing Docs - I Broadly Concur (Rating Upgrade) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="X245" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPZ1M2ZmtfaHI5NjY2YjVyMUZBdHI1M1IxM09rLXVncjFHclVfUnRQRmlUN3p2S3Q4bnpGa3VMOURZbVRYS3RqQUdmdGFQM0xvbFotZEhhcHRQcHp6eHJFeDZTcVYyVFRqaUJEdy1fZ01TYkdpSEd1S05RTElsTjVnMjItbVIyVjM4a2tWbV9Md3NOc19JMy1WUmJGYzJXaElpQ3M4WE9YVDZfNzVqcGR3cVk1SUYwZGtJ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y245" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z245" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA245" t="inlineStr">
+        <is>
+          <t>Stellantis stock breaks support as revenue grows 13 percent - AD HOC NEWS</t>
+        </is>
+      </c>
+      <c r="AB245" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQbnNpS1NfblNqOTl3MVU3T3lTSHZ6cWxHQnYzdE9sYmxLVnhrOU9vbVBxcGxuaHBtYUFYUEdmZFRRZEZxNnBDWTFScUg4VUNlZGVWaWJXYjlRUjR4Sm95MDZ6Rmc0cEh0RUV6LVBwVlRUeThRY05rVjVUOW8tYjJlZ1JfVFoyREdndFpXelB6U2ZIQzJycWs1RHVUa2puTHVkWVFieEJscldfaER5SWVBSVdORWdrQzlfSk55MFVzMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC245" t="inlineStr">
+        <is>
+          <t>Nike Shares Holding Steady After S&amp;P 100 Drop - WWD</t>
+        </is>
+      </c>
+      <c r="AD245" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxOdUFtOXo3NVlIS1AtR3l2RmRacC13czVFS1BMaC1uaEVRdHExREg0RlhUbV95cm5uY2tMT0puWFFSSThIRjJfX0tmRFRMdjVFLVN5aV85b29OWnZMTGplRmQtbHVjVUIzc05SSlBPaVpWRTd6Sko0UjhLV3cteXA2WWhaeTc3NnJmd1JVZHF3MVhrc3NtU1RjVDV4UklGSUVPYXRUSnBOTUlsSXRsOEE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:47:55+00:00</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E246" t="n">
+        <v>30977.25</v>
+      </c>
+      <c r="F246" t="n">
+        <v>31065.5</v>
+      </c>
+      <c r="G246" t="n">
+        <v>30951.25</v>
+      </c>
+      <c r="H246" t="n">
+        <v>31053</v>
+      </c>
+      <c r="I246" t="n">
+        <v>106123</v>
+      </c>
+      <c r="J246" t="n">
+        <v>4</v>
+      </c>
+      <c r="K246" t="n">
+        <v>32</v>
+      </c>
+      <c r="L246" t="n">
+        <v>-0.267</v>
+      </c>
+      <c r="M246" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="N246" t="n">
+        <v>38</v>
+      </c>
+      <c r="O246" t="n">
+        <v>-0.007</v>
+      </c>
+      <c r="P246" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="Q246" t="n">
+        <v>-7.409</v>
+      </c>
+      <c r="R246" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S246" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="T246" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U246" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="V246" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="W246" t="inlineStr">
+        <is>
+          <t>Nasdaq Hits Record High Ahead of Trump-Xi Meeting - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X246" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxQT0xKczFIMXh4aVRzSFVnLVNIUERhLTFWZ2lqVGt1RXpyemliZ3JFczFRQ1FLTUNLa0RpeGgxdjFCdW5tNUc0cDJNazVqWUszSXA3eDNveXQ4Q0lMN1JxRWJob2JETklBUzctR0xNRWpBOXFaekp4dlVvODlDQ0xoUE1janlVRTFyNDJIcHFMdUZLbm13YnRnZC13?oc=5</t>
+        </is>
+      </c>
+      <c r="Y246" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z246" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA246" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB246" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQVXdsbXlHdF9Xa0d3UFhXbk9jd1lRYV8xTzZMSUxtQVhWM1RybVpzbjFFclFFdHYzTTlrM1Q3V3pJMmFJNzliRmY0X3dIdXEtaldDNlpia1ppZUk1aC1FU0pHZW9uQm9NY0JWNHFYM2dMWWJLUjNYbWtERTh6LXFjZXQxbXpqc2YzOF9KM1dPMTUzUlVSY0FFc3podnk3MmNQMnBIQTUzMld3T1J2cFBFMFVTNkRvZTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC246" t="inlineStr">
+        <is>
+          <t>PayPal surges on Meta AI deal as tech rotation sinks financials - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD246" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOM0tOaEIydU41NDFVRlFLTi1Dbm4yT0FKYVJOd1ZuZ1VSMHZURnc2RGFCX2tzVXl6dWVrQ2Z3c05ETzNYeU5yUFduTGV0VElXNDNGYURLbndPVnJIQ1R4X0tzRW11SUtYcjVVUkpKdkhHNE54cnVqYjhkR2FHRUFaX1Q1UDhYWG91c0p4NWpudXVtaVRCajJJR05WRHZWclhfT29OcG1KXzVhRjVPeEtHZ2k1TQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:47:55+00:00</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E247" t="n">
+        <v>86474.4531</v>
+      </c>
+      <c r="F247" t="n">
+        <v>86606.2812</v>
+      </c>
+      <c r="G247" t="n">
+        <v>86014.0469</v>
+      </c>
+      <c r="H247" t="n">
+        <v>86193.75</v>
+      </c>
+      <c r="I247" t="n">
+        <v>2687467520</v>
+      </c>
+      <c r="J247" t="n">
+        <v>4</v>
+      </c>
+      <c r="K247" t="n">
+        <v>36</v>
+      </c>
+      <c r="L247" t="n">
+        <v>-0.06900000000000001</v>
+      </c>
+      <c r="M247" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="N247" t="n">
+        <v>37</v>
+      </c>
+      <c r="O247" t="n">
+        <v>0.451</v>
+      </c>
+      <c r="P247" t="n">
+        <v>-0.046</v>
+      </c>
+      <c r="Q247" t="n">
+        <v>6.586</v>
+      </c>
+      <c r="R247" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S247" t="inlineStr">
+        <is>
+          <t>Worldcoin (WLD) Surges 3.92% Amid Broad Market Rally - CoinMarketCap</t>
+        </is>
+      </c>
+      <c r="T247" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFBmVnI1LVFSVUJ4MkZjYnVKLXA1TlgxS0JVcXhYa0VGUXhLOEZjdWhnU2pfdU5TczhJaHB6OUpCRFNUdGdldWdhTGpVa0VNRU0zS0M2a3RBdm5jUW5sVVRZaHRhajYyVi1UTU5qcWptN28?oc=5</t>
+        </is>
+      </c>
+      <c r="U247" t="inlineStr">
+        <is>
+          <t>Bitcoin jumps nearly 5% to cross $85,000 as strong ETF inflows and institutional buying boost crypto momen - The Economic Times</t>
+        </is>
+      </c>
+      <c r="V247" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxQcGFmOUJLZlJEeERGcTlqN016NzFZemFrenJKcFpQa1BZMEZ6Z2dOYldneU9CaGk4dzBJSmZRVUs2eHhscUwtMmpKcE1GTHZQZWRiM0NhZXJGc2ZCeko4YWptOWVWX0dpbWx4RVUwODU3cmtyVUlVc0N1M252X1ZqaEtPNkEybHBfdWFOc3NNUXQ2MENSLVhrdUFKT29XQlNnYVRtckxLVjhYX0lkVWkyeHdsak9TcHRMWS1DOURlOUdoaHpCckZOX3NLazZVMmZRMWtKb0kyX2YwN1J6bV8wUEtxN1lBWmx5cExlbVVBYTBlRDFKb2FITHBoWUtiOFRPVGxwTnlrXzlWdHRRdWVzbdIBlgJBVV95cUxPNlNZM3JYRkx6cXBwUURPeHBJX1lMbzcyTUx4VlBlRVEydWtzRW90WDhObFZOekgxeEtoY244aFlmYUY3U21pUGxoUE52M05KOUZmeDRwV3RqNWhvbmVuMUNxZFZrQkhpbF93dm1FckZ2Y05YQWluTE9DVnZpYldOeWgxamI0YTFNLWNaUGdiZ2FDMTUxMHNKQ0RScXYxWDItWjlMMzdiUy1vWGxpY2I0YjhOSWY1dEp2TUVuZTVRSllrR2xtdUlmWHU1dXVrZXBjWHJ3SnM2Y25pbnJyWTY5OW9rWm1JXzhTcXA4azVHaDR0S0NvTkhpRklzUlRONUxHSmt3aXpLTWQ3eHFjekFfRkZWMFpWdw?oc=5</t>
+        </is>
+      </c>
+      <c r="W247" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to 8-month high above $85,000 - qz.com</t>
+        </is>
+      </c>
+      <c r="X247" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9BRHhsSDNaZ2VlVnhzYmRsci1zNk1kQ2JWNHJxNTNVRHFDSHFqcmVoVFg2TkJxYTdZMUhfMEJpb1hFS3RabDlJcVZZWEh4M3VJUUpaX0JUSWtHd0pxNUctNzg3Nkx0Q2JoT21EN2cwV1ZtQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y247" t="inlineStr">
+        <is>
+          <t>Bitcoin Is 11 Days From Its First Winning Quarter in a Year. What Needs to Hold Until September 30? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="Z247" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQTU9EX0F6eUx0b0Q4cVhJMEtNLU92NXJPTmNvSGk2VVJmamw2dEhRdVN6Mi1xWThSbWY1MFRoVjlXWWVFUTdZcm1vajFTY3BXM0k0OHJYaFRZNmZ6dzZjRWFzUjFaeUstUlo5emkxNVhYay10WTJKT1JpbnZEM2xMUExDZ2YzM1dBWTYtbEpqS0pBUTRzUEFKeENRckJONVdnRTFGWm1mVUNOckc2dm4wSHRlQlhrcS1XUGlUQS10SjhlbGVxWFFxXy01VU1lMUNtMXdiX1U5OXBZUVhHRXN0V2lUZUJXYUhlSlFqUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA247" t="inlineStr">
+        <is>
+          <t>Bitcoin ETFs Pull In Nearly $1 Billion as Short Sellers Get Liquidated - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="AB247" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNMTVWU1FadDJRSURCVEVweFRkbDRhY0YzM3dXVTI3dERaU0NWUzg0UFphRHhlZlVBNmwzeV9PTUxHQnU5Ni1TVUhDUm5DZHk2enp2dllIdUVJQXJEeGFza0VIUzQwcDlXcUJjdzIyM2syenEtclNoSnFzSUhRYmEtVzh3WTM4dDZCUDhFU0xWYzFvUWtRRHdvSEs0dThkZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC247" t="inlineStr">
+        <is>
+          <t>Bitcoin (BTC) price slides to $78,800 as BNB and DeFi tokens buck the selloff: Crypto Markets Today - CoinDesk</t>
+        </is>
+      </c>
+      <c r="AD247" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQTk1QUWpJdWlGclNwM2JhRzVfOW1XSVdtUzZ6a0E5a3l4ZUhYa3lmYVFkV0JVZlZKUzJMTXFyZmU1R29VMVZtaWhqeHl3dzVIaG1DQ2g1R1RLbW1JS1NscmlJcWxDbjZwM1ZQMWJuanVpWjhRZXR3dEJFVXlIM3NRSEkxUThTaEpKR3NNX3JKRW02X3pCbVJ4dVpCd2RYVTdSX1owWVZ5N0M3cXlUVDZv?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-23 03:45 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD247"/>
+  <dimension ref="A1:AD253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31097,6 +31097,762 @@
       <c r="AD247" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQTk1QUWpJdWlGclNwM2JhRzVfOW1XSVdtUzZ6a0E5a3l4ZUhYa3lmYVFkV0JVZlZKUzJMTXFyZmU1R29VMVZtaWhqeHl3dzVIaG1DQ2g1R1RLbW1JS1NscmlJcWxDbjZwM1ZQMWJuanVpWjhRZXR3dEJFVXlIM3NRSEkxUThTaEpKR3NNX3JKRW02X3pCbVJ4dVpCd2RYVTdSX1owWVZ5N0M3cXlUVDZv?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-09-23T03:43:30+00:00</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E248" t="n">
+        <v>4401.3999</v>
+      </c>
+      <c r="F248" t="n">
+        <v>4407.5</v>
+      </c>
+      <c r="G248" t="n">
+        <v>4370</v>
+      </c>
+      <c r="H248" t="n">
+        <v>4376.7998</v>
+      </c>
+      <c r="I248" t="n">
+        <v>14710</v>
+      </c>
+      <c r="J248" t="n">
+        <v>4</v>
+      </c>
+      <c r="K248" t="n">
+        <v>39</v>
+      </c>
+      <c r="L248" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="M248" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="N248" t="n">
+        <v>40</v>
+      </c>
+      <c r="O248" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="P248" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="Q248" t="n">
+        <v>1.331</v>
+      </c>
+      <c r="R248" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S248" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T248" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="U248" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="V248" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="W248" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="X248" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y248" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="Z248" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA248" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB248" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC248" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD248" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-09-23T03:43:30+00:00</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E249" t="n">
+        <v>89.56999999999999</v>
+      </c>
+      <c r="F249" t="n">
+        <v>90.38</v>
+      </c>
+      <c r="G249" t="n">
+        <v>89.45999999999999</v>
+      </c>
+      <c r="H249" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="I249" t="n">
+        <v>12684</v>
+      </c>
+      <c r="J249" t="n">
+        <v>4</v>
+      </c>
+      <c r="K249" t="n">
+        <v>40</v>
+      </c>
+      <c r="L249" t="n">
+        <v>-0.167</v>
+      </c>
+      <c r="M249" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="N249" t="n">
+        <v>40</v>
+      </c>
+      <c r="O249" t="n">
+        <v>0.247</v>
+      </c>
+      <c r="P249" t="n">
+        <v>-0.053</v>
+      </c>
+      <c r="Q249" t="n">
+        <v>1.604</v>
+      </c>
+      <c r="R249" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S249" t="inlineStr">
+        <is>
+          <t>Slack Wax Residue Market to Accelerate on Electronics Thermal Demand by 2035 - IndexBox</t>
+        </is>
+      </c>
+      <c r="T249" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOSUEwUUktaHFQWjJXZGNjTHdMaDFINFBhcjZPSExjWWJLcHlUY0RoWDV2VXdkTHVJM2lKbXF3QkJyQ2p4T3QwTXNoUjZyTzdMbm43cmRjWnBHZmpfQTdLanVYYmdvODZxQnFTcENGbWg1ZHdtQ1N6RnlHZi14UWhKaHNGTHhYWVlpLUtGRGw4NWpmZjRnQXQ1LVJnQXpsWUJ2Yk1ZM3lyMlBnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U249" t="inlineStr">
+        <is>
+          <t>Asian Stocks Rise as AI Demand and Lower Oil Prices Lift Markets - Межа. Новини України.</t>
+        </is>
+      </c>
+      <c r="V249" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1LYUMyUDhiTlFhdDZDZWRJV3BXMzBHQmhxaWNhbHhieVJObjJpbU84WHUtaFlITmtnNWVJNW5CX1JrQ1RaTktaQ3pFYVdOZ3VmVkkxWkgtUDN2Zk90V1NwYjFlSF8?oc=5</t>
+        </is>
+      </c>
+      <c r="W249" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X249" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y249" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z249" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA249" t="inlineStr">
+        <is>
+          <t>Oil prices hover around $100 a barrel - Transport Topics</t>
+        </is>
+      </c>
+      <c r="AB249" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTE1wYUFKb2JqTDVBUWJhODRORTIyWWh6bzZOMUFDd0ZzS1JUVzJobnd6MlpwNE5mRk5XRDdOVGNubXFtTXZDbktuLWNIZ3FQaVBjUHp2cE16NUdGbENfZHpXTEFEYlhpcDhpWnpz?oc=5</t>
+        </is>
+      </c>
+      <c r="AC249" t="inlineStr">
+        <is>
+          <t>Crude Oil sells off and takes it all back on Saudi cargoes through Oman - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD249" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMGtjZFowTldOS1FIY1N2eldvdW9LdVg1TFVXTjRvUDBKcnpxS2RYSkR4Tm1Td1hVVGxwdTVwU0JlX2ZZOWE4SmtYbmp2TVIzWjVFRU1WeHlyZy1VVU80bVVFTXJTMms5QXNIVW9DYS1lQjFXRWtVeHZnZmtlUU12Yy1kTE5YV1BiXy12REFYLUVxSFEzTE5CNVdYXzc4SkV0ZGhBWVEtMG1QZG8yX3dQS1FxTm8?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-09-23T03:43:30+00:00</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E250" t="n">
+        <v>100.552</v>
+      </c>
+      <c r="F250" t="n">
+        <v>100.704</v>
+      </c>
+      <c r="G250" t="n">
+        <v>100.545</v>
+      </c>
+      <c r="H250" t="n">
+        <v>100.676</v>
+      </c>
+      <c r="I250" t="n">
+        <v>0</v>
+      </c>
+      <c r="J250" t="n">
+        <v>4</v>
+      </c>
+      <c r="K250" t="n">
+        <v>39</v>
+      </c>
+      <c r="L250" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="M250" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="N250" t="n">
+        <v>40</v>
+      </c>
+      <c r="O250" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="P250" t="n">
+        <v>-0.026</v>
+      </c>
+      <c r="Q250" t="n">
+        <v>2.054</v>
+      </c>
+      <c r="R250" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S250" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T250" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U250" t="inlineStr">
+        <is>
+          <t>Gold price seen trading $4,000-4,500 range as strong dollar checks safe-haven demand - Khaleej Times</t>
+        </is>
+      </c>
+      <c r="V250" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQdDhNcUJyZkVSOWs4clk4Zmc1Z1hkSjY4ZVhNTkFGVEFKRzdzOFFxQm5mczhSQ2lSZ2daYnBHc0hhSkQzTFlaZ3NNa01wWEs1RFdiODFqY3NKOE1ZVUNSU24wZnl0R3VRUHhsWURpRGJoejZwNXRzREFHd2l0ZUZqRHNOWDRLdnd4SzQ1cENMZkVnTFRXMzJZemhIdWZUbm5heFQyRlN1RGNVQnU2bEctV3ZnTklleDIyY0lN0gHDAUFVX3lxTE1zQ1JjcnJXUE50Q0ZBTmRPMGlMS3dzWHRXcV9MbWprTE82d3JTdlluSFRORGJQWlh3ZmpqcmRoaDF1bVdlaEkzT2FiWk5TODBCZVNjMl9FY0hPZ1NKT2NycEFNY2QyM3JXb043UXRtUG43VzlXc1FCNlVBOV9nTElwVEdFV04xcURDOEdrVkRIbWlXanRUZVRXeExseHpiR0N6NGtSbW12YnFmdmJwNkliVlJUVGFnMW9jMEg3X0FHREdBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="W250" t="inlineStr">
+        <is>
+          <t>Canadian Dollar strengthens on rising oil prices ahead of potential US-Iran talks - FXStreet</t>
+        </is>
+      </c>
+      <c r="X250" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxObmphYlI3SXdxcVRpa3dJSldPd2VZeXJiYkl5Mzhia3pKWGlhd2poUEdNS2Jfc21BdkVoVktodE5HcVNJWTRWaDFDZjVYTTNkSE9YQjRBVzZzQTY3NUZuWWg3U3paSEdiN3h0N0R2UjBPc0ZERTNFMFUzUFpqa0xGZHJaLUpwQjlUa3Z3cDZNaDNTOGRkSlFOb2VzUjZDd0gwV0xEVEVCcWhCYktmemlOUlJWeGM3dHJZcUg5ME05aF9vQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y250" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z250" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA250" t="inlineStr">
+        <is>
+          <t>United States Dollar Index Price Forecast: Rising 20-day EMA backs bullish bias - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB250" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMVFrazh3MFdPaXh4RURLaS1CSm5LY3dRV0VmZ2t3MmFMOFZwdjhoTC1Gb1JsSm53S1hjVUJjUUhSUWdXcVBYUjZHdFktaVNkUDZBdzlvdEpwaWY4QXl2S0JhSGpCZkZ5Q2gzMGdzb2NNR3k4N3FMZUJEMkJ6NzNXWXBjMGNKb0txV1dHdlZia242dlNuRzI1cGgxdU9jbWVsSlVfMDBFdEt1aVlSUFN0LURmSWRhM0E3YUtXTXNB?oc=5</t>
+        </is>
+      </c>
+      <c r="AC250" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD250" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-09-23T03:43:30+00:00</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E251" t="n">
+        <v>7833.25</v>
+      </c>
+      <c r="F251" t="n">
+        <v>7836</v>
+      </c>
+      <c r="G251" t="n">
+        <v>7827.25</v>
+      </c>
+      <c r="H251" t="n">
+        <v>7836</v>
+      </c>
+      <c r="I251" t="n">
+        <v>24507</v>
+      </c>
+      <c r="J251" t="n">
+        <v>4</v>
+      </c>
+      <c r="K251" t="n">
+        <v>39</v>
+      </c>
+      <c r="L251" t="n">
+        <v>-0.047</v>
+      </c>
+      <c r="M251" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="N251" t="n">
+        <v>40</v>
+      </c>
+      <c r="O251" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="P251" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="Q251" t="n">
+        <v>-0.281</v>
+      </c>
+      <c r="R251" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T251" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U251" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V251" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W251" t="inlineStr">
+        <is>
+          <t>Stock market today: Dow hits record high, S&amp;P 500 and Nasdaq surge as Big Tech gains power rally - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X251" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPbkNnYmlpUUZ1UFBUdG13a1NLZlhpbXR4cEpMcUdqRkR5aXd1UjVKaEFFQTJyQ0JrQWFHN0I0Zk1wSDVOZ0RaRWM2aXpCb3BDQmE4c0dXaHFLQVhRcXdiZDZnSko3UGd6WlkwNlVncFNJdTVnbHVGaFJBTXltM0ttaUxkZ0ZFa2ptNVN5S3FTbXBPOTc3UHdZVEtVYVFqWXNMazVsZlhaY3hibzViazhyeXBta2RFWHF4Z1pN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y251" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z251" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA251" t="inlineStr">
+        <is>
+          <t>Stellantis stock breaks support as revenue grows 13 percent - AD HOC NEWS</t>
+        </is>
+      </c>
+      <c r="AB251" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQbnNpS1NfblNqOTl3MVU3T3lTSHZ6cWxHQnYzdE9sYmxLVnhrOU9vbVBxcGxuaHBtYUFYUEdmZFRRZEZxNnBDWTFScUg4VUNlZGVWaWJXYjlRUjR4Sm95MDZ6Rmc0cEh0RUV6LVBwVlRUeThRY05rVjVUOW8tYjJlZ1JfVFoyREdndFpXelB6U2ZIQzJycWs1RHVUa2puTHVkWVFieEJscldfaER5SWVBSVdORWdrQzlfSk55MFVzMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC251" t="inlineStr">
+        <is>
+          <t>Darden Stock Breaks $207.25 as Earnings Week Puts $202.75 Support in Focus - tradingkey.com</t>
+        </is>
+      </c>
+      <c r="AD251" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPcEZ2cWsxRG44VFRXZkw3dWstakNwczBXVEVEOFpPZHVnSm1XME1QV2I4RUxZckNWcGxITF9LX2pVazVVc0JuNXlfLVUzaHBwWHZoQm91d0tSZmxiY25aVVFCeHNlTXdvZ3JpNWpaeV9QTDA4YS1wdzBmQUxmVnBFZjNCQ3Z2ZXplUnR3RjBWX0VGeTd6alRyTkZsQ01rZ0VNdkRXN2VpdkpnWm1OVU9tbQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-09-23T03:43:30+00:00</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E252" t="n">
+        <v>31064.5</v>
+      </c>
+      <c r="F252" t="n">
+        <v>31065.75</v>
+      </c>
+      <c r="G252" t="n">
+        <v>30982.75</v>
+      </c>
+      <c r="H252" t="n">
+        <v>31012</v>
+      </c>
+      <c r="I252" t="n">
+        <v>22618</v>
+      </c>
+      <c r="J252" t="n">
+        <v>4</v>
+      </c>
+      <c r="K252" t="n">
+        <v>35</v>
+      </c>
+      <c r="L252" t="n">
+        <v>-0.229</v>
+      </c>
+      <c r="M252" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="N252" t="n">
+        <v>38</v>
+      </c>
+      <c r="O252" t="n">
+        <v>0.08799999999999999</v>
+      </c>
+      <c r="P252" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="Q252" t="n">
+        <v>-3.845</v>
+      </c>
+      <c r="R252" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="T252" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U252" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="V252" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="W252" t="inlineStr">
+        <is>
+          <t>Block Inc. stock holds at USD 76.28 after Nasdaq rally - AD HOC NEWS</t>
+        </is>
+      </c>
+      <c r="X252" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOX2xzZ2N0X1pmNVdGWWNvanktWXB3bkJPTWF4Q21qNDJZclExcUk0QnJFblE1ZkxvRWZsdkZnejY3SHZBdG01Y0hkSUdlTDlybW45a3ZVeWgwdmhXbDNHek1zczJROUEwbVNSRXplck5IR05rT0xGX3l2SzFadnFCUjg1QWZCdVdsZ0YwbHotZEFZemZyQmFPWmdWMm9EZlotbWlTcGk1ZlBzVU1DbmdRclBnWlhMcjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y252" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z252" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA252" t="inlineStr">
+        <is>
+          <t>PayPal surges on Meta AI deal as tech rotation sinks financials - Investing.com</t>
+        </is>
+      </c>
+      <c r="AB252" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOM0tOaEIydU41NDFVRlFLTi1Dbm4yT0FKYVJOd1ZuZ1VSMHZURnc2RGFCX2tzVXl6dWVrQ2Z3c05ETzNYeU5yUFduTGV0VElXNDNGYURLbndPVnJIQ1R4X0tzRW11SUtYcjVVUkpKdkhHNE54cnVqYjhkR2FHRUFaX1Q1UDhYWG91c0p4NWpudXVtaVRCajJJR05WRHZWclhfT29OcG1KXzVhRjVPeEtHZ2k1TQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC252" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AD252" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-09-23T03:43:30+00:00</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E253" t="n">
+        <v>86189.2188</v>
+      </c>
+      <c r="F253" t="n">
+        <v>86935.8281</v>
+      </c>
+      <c r="G253" t="n">
+        <v>86130</v>
+      </c>
+      <c r="H253" t="n">
+        <v>86825.14840000001</v>
+      </c>
+      <c r="I253" t="n">
+        <v>3378126848</v>
+      </c>
+      <c r="J253" t="n">
+        <v>4</v>
+      </c>
+      <c r="K253" t="n">
+        <v>37</v>
+      </c>
+      <c r="L253" t="n">
+        <v>-0.051</v>
+      </c>
+      <c r="M253" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="N253" t="n">
+        <v>37</v>
+      </c>
+      <c r="O253" t="n">
+        <v>0.354</v>
+      </c>
+      <c r="P253" t="n">
+        <v>-0.057</v>
+      </c>
+      <c r="Q253" t="n">
+        <v>5.594</v>
+      </c>
+      <c r="R253" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to 8-month high above $85,000 - qz.com</t>
+        </is>
+      </c>
+      <c r="T253" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9BRHhsSDNaZ2VlVnhzYmRsci1zNk1kQ2JWNHJxNTNVRHFDSHFqcmVoVFg2TkJxYTdZMUhfMEJpb1hFS3RabDlJcVZZWEh4M3VJUUpaX0JUSWtHd0pxNUctNzg3Nkx0Q2JoT21EN2cwV1ZtQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U253" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="V253" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="W253" t="inlineStr">
+        <is>
+          <t>Bitcoin: Surges Above $86,000 With $900M Liquidations - blockchain.news</t>
+        </is>
+      </c>
+      <c r="X253" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPWlJLVVp0NTE2ZWFUZHpuU2d3LXBsMUFZeDVKRy16X2VPZEpUQ19yM09qYkZ0U2o4S2pNZHlFUk56WjloUUtFbzBTdU1leVJXVTVpbExBUkg0T1ZhbllkOHRZUWdINTliV05wMFlRbVNWa0ZReGNMaFVIeFVFamsxNTJxQ00wZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y253" t="inlineStr">
+        <is>
+          <t>Bitcoin clears $85K as $648M in shorts are liquidated, per CoinGlass - altcoinbuzz.io</t>
+        </is>
+      </c>
+      <c r="Z253" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxPdldlWXhkNnpXb1FYcEdMZHZ0WWtiSHpvMEo1RGd4ejZvQjVTcGFadWhURVFWcks2T2dlR0Y1cmxremJ0YS1DaFI1bW5hN3ptc0FfYWltM2lrdi0yNHo2YXBFdWxOSVBraXNqRGpaWUxXLWxPc0VFMEVFVi01WFUyOHlQZjNEcEUwVUFJ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA253" t="inlineStr">
+        <is>
+          <t>Bitcoin Is 11 Days From Its First Winning Quarter in a Year. What Needs to Hold Until September 30? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB253" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQTU9EX0F6eUx0b0Q4cVhJMEtNLU92NXJPTmNvSGk2VVJmamw2dEhRdVN6Mi1xWThSbWY1MFRoVjlXWWVFUTdZcm1vajFTY3BXM0k0OHJYaFRZNmZ6dzZjRWFzUjFaeUstUlo5emkxNVhYay10WTJKT1JpbnZEM2xMUExDZ2YzM1dBWTYtbEpqS0pBUTRzUEFKeENRckJONVdnRTFGWm1mVUNOckc2dm4wSHRlQlhrcS1XUGlUQS10SjhlbGVxWFFxXy01VU1lMUNtMXdiX1U5OXBZUVhHRXN0V2lUZUJXYUhlSlFqUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC253" t="inlineStr">
+        <is>
+          <t>Bitcoin ETFs Pull In Nearly $1 Billion as Short Sellers Get Liquidated - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="AD253" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNMTVWU1FadDJRSURCVEVweFRkbDRhY0YzM3dXVTI3dERaU0NWUzg0UFphRHhlZlVBNmwzeV9PTUxHQnU5Ni1TVUhDUm5DZHk2enp2dllIdUVJQXJEeGFza0VIUzQwcDlXcUJjdzIyM2syenEtclNoSnFzSUhRYmEtVzh3WTM4dDZCUDhFU0xWYzFvUWtRRHdvSEs0dThkZw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-23 09:12 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD253"/>
+  <dimension ref="A1:AD259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31853,6 +31853,762 @@
       <c r="AD253" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNMTVWU1FadDJRSURCVEVweFRkbDRhY0YzM3dXVTI3dERaU0NWUzg0UFphRHhlZlVBNmwzeV9PTUxHQnU5Ni1TVUhDUm5DZHk2enp2dllIdUVJQXJEeGFza0VIUzQwcDlXcUJjdzIyM2syenEtclNoSnFzSUhRYmEtVzh3WTM4dDZCUDhFU0xWYzFvUWtRRHdvSEs0dThkZw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-09-23T09:10:01+00:00</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E254" t="n">
+        <v>4371.7998</v>
+      </c>
+      <c r="F254" t="n">
+        <v>4374.1001</v>
+      </c>
+      <c r="G254" t="n">
+        <v>4352.2002</v>
+      </c>
+      <c r="H254" t="n">
+        <v>4355.1001</v>
+      </c>
+      <c r="I254" t="n">
+        <v>15671</v>
+      </c>
+      <c r="J254" t="n">
+        <v>4</v>
+      </c>
+      <c r="K254" t="n">
+        <v>40</v>
+      </c>
+      <c r="L254" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M254" t="n">
+        <v>-0.017</v>
+      </c>
+      <c r="N254" t="n">
+        <v>40</v>
+      </c>
+      <c r="O254" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="P254" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="Q254" t="n">
+        <v>1.912</v>
+      </c>
+      <c r="R254" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T254" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="U254" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="V254" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="W254" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="X254" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y254" t="inlineStr">
+        <is>
+          <t>JPMorgan Says Bitcoin Could Beat Gold Once ETF Hedging Pressure Eases - Startup Fortune</t>
+        </is>
+      </c>
+      <c r="Z254" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOSXdwN2QyTldDZVRrZDh4TjZuQVFWTlBSaWJPV01kSzgxWk1sWVVTZm4tckp0N0tabDlWTmZJaHVqZFRfZDQ4Y0phZDFlX1JIODhxLU92YkJZaHQtZjFuRS13d2tIVWs1OXhWel9oY2xzM1NTV2JpTE80d21RVDl2d3p4NURVbExBdnFLUDNLZm9kZDdvUFNNQmJCMGZTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA254" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB254" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC254" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD254" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-09-23T09:10:01+00:00</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E255" t="n">
+        <v>89.29000000000001</v>
+      </c>
+      <c r="F255" t="n">
+        <v>90.52</v>
+      </c>
+      <c r="G255" t="n">
+        <v>89.08</v>
+      </c>
+      <c r="H255" t="n">
+        <v>89.92</v>
+      </c>
+      <c r="I255" t="n">
+        <v>29212</v>
+      </c>
+      <c r="J255" t="n">
+        <v>4</v>
+      </c>
+      <c r="K255" t="n">
+        <v>40</v>
+      </c>
+      <c r="L255" t="n">
+        <v>-0.012</v>
+      </c>
+      <c r="M255" t="n">
+        <v>-0.233</v>
+      </c>
+      <c r="N255" t="n">
+        <v>40</v>
+      </c>
+      <c r="O255" t="n">
+        <v>0.228</v>
+      </c>
+      <c r="P255" t="n">
+        <v>-0.049</v>
+      </c>
+      <c r="Q255" t="n">
+        <v>4.329</v>
+      </c>
+      <c r="R255" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S255" t="inlineStr">
+        <is>
+          <t>Slack Wax Residue Market to Accelerate on Electronics Thermal Demand by 2035 - IndexBox</t>
+        </is>
+      </c>
+      <c r="T255" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOSUEwUUktaHFQWjJXZGNjTHdMaDFINFBhcjZPSExjWWJLcHlUY0RoWDV2VXdkTHVJM2lKbXF3QkJyQ2p4T3QwTXNoUjZyTzdMbm43cmRjWnBHZmpfQTdLanVYYmdvODZxQnFTcENGbWg1ZHdtQ1N6RnlHZi14UWhKaHNGTHhYWVlpLUtGRGw4NWpmZjRnQXQ1LVJnQXpsWUJ2Yk1ZM3lyMlBnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U255" t="inlineStr">
+        <is>
+          <t>Asian Stocks Rise as AI Demand and Lower Oil Prices Lift Markets - Межа. Новини України.</t>
+        </is>
+      </c>
+      <c r="V255" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1LYUMyUDhiTlFhdDZDZWRJV3BXMzBHQmhxaWNhbHhieVJObjJpbU84WHUtaFlITmtnNWVJNW5CX1JrQ1RaTktaQ3pFYVdOZ3VmVkkxWkgtUDN2Zk90V1NwYjFlSF8?oc=5</t>
+        </is>
+      </c>
+      <c r="W255" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="X255" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y255" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z255" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA255" t="inlineStr">
+        <is>
+          <t>Oil prices hover around $100 a barrel - Transport Topics</t>
+        </is>
+      </c>
+      <c r="AB255" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTE1wYUFKb2JqTDVBUWJhODRORTIyWWh6bzZOMUFDd0ZzS1JUVzJobnd6MlpwNE5mRk5XRDdOVGNubXFtTXZDbktuLWNIZ3FQaVBjUHp2cE16NUdGbENfZHpXTEFEYlhpcDhpWnpz?oc=5</t>
+        </is>
+      </c>
+      <c r="AC255" t="inlineStr">
+        <is>
+          <t>End tax breaks on oil and gas - you.38degrees.org.uk</t>
+        </is>
+      </c>
+      <c r="AD255" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5gJBVV95cUxNMW1iTERSWU1IZnRiSm8xNFlCMlJILXlsUnZ1UlRXYkp0LUpDN0N1a2paNzNFQm5tM1Nwal9nNHpwSU1hMzh1dGIycW9mWmVtZVB3NGNtdnFXV29BU0ZSZVNwVTlTQmYzTC1CUUFNaW5YREVIUGktd2d3cEpHUWl4TGdfTWt4eGgzV3BKaVlSMlpOdFlIbzQwYnc5NzdTNTZOMzBCSGxyNzBEbzBJQjRPSDJvLUthQXdHNDVxa2RYWDVBZk1kdUVBZTZRS21DZTdSOVRVS3dfYWVSRXhIa1VpTE5ZXy1kUUk3OXVXUXA0TV9iSDlQYURzYWVhZWdLVnpWeXJDUGNpdHkzRENSbXExemwxcF9KcWtsVllBN0ZKRWtvenJNREVXX2hzbm5jVWVWM1J5QzhXSm5XdGV5ZzJlaW5mLXBoa0w0Z2ItWEozQmJIcFRmVXEycUxoX2ppZk1HalZmc0JB?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-09-23T09:10:01+00:00</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E256" t="n">
+        <v>100.731</v>
+      </c>
+      <c r="F256" t="n">
+        <v>100.862</v>
+      </c>
+      <c r="G256" t="n">
+        <v>100.707</v>
+      </c>
+      <c r="H256" t="n">
+        <v>100.801</v>
+      </c>
+      <c r="I256" t="n">
+        <v>0</v>
+      </c>
+      <c r="J256" t="n">
+        <v>4</v>
+      </c>
+      <c r="K256" t="n">
+        <v>39</v>
+      </c>
+      <c r="L256" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="M256" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="N256" t="n">
+        <v>39</v>
+      </c>
+      <c r="O256" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="P256" t="n">
+        <v>-0.024</v>
+      </c>
+      <c r="Q256" t="n">
+        <v>5.137</v>
+      </c>
+      <c r="R256" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S256" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T256" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U256" t="inlineStr">
+        <is>
+          <t>Gold price seen trading $4,000-4,500 range as strong dollar checks safe-haven demand - Khaleej Times</t>
+        </is>
+      </c>
+      <c r="V256" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQdDhNcUJyZkVSOWs4clk4Zmc1Z1hkSjY4ZVhNTkFGVEFKRzdzOFFxQm5mczhSQ2lSZ2daYnBHc0hhSkQzTFlaZ3NNa01wWEs1RFdiODFqY3NKOE1ZVUNSU24wZnl0R3VRUHhsWURpRGJoejZwNXRzREFHd2l0ZUZqRHNOWDRLdnd4SzQ1cENMZkVnTFRXMzJZemhIdWZUbm5heFQyRlN1RGNVQnU2bEctV3ZnTklleDIyY0lN0gHDAUFVX3lxTE1zQ1JjcnJXUE50Q0ZBTmRPMGlMS3dzWHRXcV9MbWprTE82d3JTdlluSFRORGJQWlh3ZmpqcmRoaDF1bVdlaEkzT2FiWk5TODBCZVNjMl9FY0hPZ1NKT2NycEFNY2QyM3JXb043UXRtUG43VzlXc1FCNlVBOV9nTElwVEdFV04xcURDOEdrVkRIbWlXanRUZVRXeExseHpiR0N6NGtSbW12YnFmdmJwNkliVlJUVGFnMW9jMEg3X0FHREdBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="W256" t="inlineStr">
+        <is>
+          <t>Canadian Dollar Strengthens On Rising Oil Prices Ahead Of Potential US-Iran Talks - InsuranceNewsNet</t>
+        </is>
+      </c>
+      <c r="X256" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOamYyNk9GZ1A3UFZpazcwVnlJZF84eGxxSWpWUDhsWWx6UURTajJKNjMySllWMkNnYnFTRlFuMXpKVEF2dEcyUEVJNjNNbXpPdkhZbmtXQTJnY19DMWQ2RjViYm8wMGJlM2xFZUhDb0pBbUFJeERIYm1JZngyV19pNjBCNWhEZDN5UWdUVlBwM01GTEliVVFSNE5JSzlrQkxQNk1FMDQ5ZUZMLXRIYVVZeDFrWi1mcUZFRHhN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y256" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z256" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA256" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AB256" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC256" t="inlineStr">
+        <is>
+          <t>Dovish Fed Bets Pummel Dollar, Boost Gold Ahead of NFP - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD256" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPZDNJaUJnTUhOckR3ODFMRjN3M3QtZ1NzUmtvYnRUOVlyWEo2Nzg4d3l5Tkl4SFNRMVJCUnlNeGxUYm5NQkxpNmxEdzVpU3ZHTkhRUXh0bEdhNld2WHFBVmNCRTBEY2dsUkxqVlYtYTUwX21GR1JZNnZjazk2OXBjNW80dWo3Nmx5TXZYLUY0WkZLei14eWV4dDlkRGVheWM?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-09-23T09:10:01+00:00</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E257" t="n">
+        <v>7836.5</v>
+      </c>
+      <c r="F257" t="n">
+        <v>7843.25</v>
+      </c>
+      <c r="G257" t="n">
+        <v>7834.25</v>
+      </c>
+      <c r="H257" t="n">
+        <v>7837</v>
+      </c>
+      <c r="I257" t="n">
+        <v>32048</v>
+      </c>
+      <c r="J257" t="n">
+        <v>4</v>
+      </c>
+      <c r="K257" t="n">
+        <v>39</v>
+      </c>
+      <c r="L257" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="M257" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="N257" t="n">
+        <v>40</v>
+      </c>
+      <c r="O257" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="P257" t="n">
+        <v>-0.038</v>
+      </c>
+      <c r="Q257" t="n">
+        <v>1.949</v>
+      </c>
+      <c r="R257" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S257" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T257" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U257" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V257" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W257" t="inlineStr">
+        <is>
+          <t>Stock market today: Dow hits record high, S&amp;P 500 and Nasdaq surge as Big Tech gains power rally - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X257" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPbkNnYmlpUUZ1UFBUdG13a1NLZlhpbXR4cEpMcUdqRkR5aXd1UjVKaEFFQTJyQ0JrQWFHN0I0Zk1wSDVOZ0RaRWM2aXpCb3BDQmE4c0dXaHFLQVhRcXdiZDZnSko3UGd6WlkwNlVncFNJdTVnbHVGaFJBTXltM0ttaUxkZ0ZFa2ptNVN5S3FTbXBPOTc3UHdZVEtVYVFqWXNMazVsZlhaY3hibzViazhyeXBta2RFWHF4Z1pN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y257" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z257" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA257" t="inlineStr">
+        <is>
+          <t>Stellantis stock breaks support as revenue grows 13 percent - AD HOC NEWS</t>
+        </is>
+      </c>
+      <c r="AB257" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQbnNpS1NfblNqOTl3MVU3T3lTSHZ6cWxHQnYzdE9sYmxLVnhrOU9vbVBxcGxuaHBtYUFYUEdmZFRRZEZxNnBDWTFScUg4VUNlZGVWaWJXYjlRUjR4Sm95MDZ6Rmc0cEh0RUV6LVBwVlRUeThRY05rVjVUOW8tYjJlZ1JfVFoyREdndFpXelB6U2ZIQzJycWs1RHVUa2puTHVkWVFieEJscldfaER5SWVBSVdORWdrQzlfSk55MFVzMA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC257" t="inlineStr">
+        <is>
+          <t>Nike Shares Holding Steady After S&amp;P 100 Drop - WWD</t>
+        </is>
+      </c>
+      <c r="AD257" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxOdUFtOXo3NVlIS1AtR3l2RmRacC13czVFS1BMaC1uaEVRdHExREg0RlhUbV95cm5uY2tMT0puWFFSSThIRjJfX0tmRFRMdjVFLVN5aV85b29OWnZMTGplRmQtbHVjVUIzc05SSlBPaVpWRTd6Sko0UjhLV3cteXA2WWhaeTc3NnJmd1JVZHF3MVhrc3NtU1RjVDV4UklGSUVPYXRUSnBOTUlsSXRsOEE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-09-23T09:10:01+00:00</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E258" t="n">
+        <v>31029.25</v>
+      </c>
+      <c r="F258" t="n">
+        <v>31094.75</v>
+      </c>
+      <c r="G258" t="n">
+        <v>31002</v>
+      </c>
+      <c r="H258" t="n">
+        <v>31019.25</v>
+      </c>
+      <c r="I258" t="n">
+        <v>18181</v>
+      </c>
+      <c r="J258" t="n">
+        <v>4</v>
+      </c>
+      <c r="K258" t="n">
+        <v>36</v>
+      </c>
+      <c r="L258" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="M258" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="N258" t="n">
+        <v>37</v>
+      </c>
+      <c r="O258" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="P258" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="Q258" t="n">
+        <v>-3.169</v>
+      </c>
+      <c r="R258" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S258" t="inlineStr">
+        <is>
+          <t>Asia Stocks Surge on Tech Rally as Oil Prices Slide Further - globalbankingandfinance.com</t>
+        </is>
+      </c>
+      <c r="T258" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOVUZYQjFQYWlmVnlzdlZNOFJtcFB2SUF0Q1Y1bjJTSnNsRmt5c2diZC1zQ252ZkIwZHdCT1Y0bnRTcGo1OEV3V3FfOXBtcnRPN2dZSjZMN1JQend1N1YyaTZEQ1UzVlYwR0pfR3JEbW8yMXYyZjVpbkdqeTRmbzlaYTV2NG9mQlpoYnNCSkJwYjUyNVkzNWhV?oc=5</t>
+        </is>
+      </c>
+      <c r="U258" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="V258" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W258" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="X258" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y258" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z258" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA258" t="inlineStr">
+        <is>
+          <t>PayPal surges on Meta AI deal as tech rotation sinks financials - Investing.com</t>
+        </is>
+      </c>
+      <c r="AB258" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOM0tOaEIydU41NDFVRlFLTi1Dbm4yT0FKYVJOd1ZuZ1VSMHZURnc2RGFCX2tzVXl6dWVrQ2Z3c05ETzNYeU5yUFduTGV0VElXNDNGYURLbndPVnJIQ1R4X0tzRW11SUtYcjVVUkpKdkhHNE54cnVqYjhkR2FHRUFaX1Q1UDhYWG91c0p4NWpudXVtaVRCajJJR05WRHZWclhfT29OcG1KXzVhRjVPeEtHZ2k1TQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC258" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AD258" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-09-23T09:10:01+00:00</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>86499.99219999999</v>
+      </c>
+      <c r="F259" t="n">
+        <v>86608.1875</v>
+      </c>
+      <c r="G259" t="n">
+        <v>85701.6562</v>
+      </c>
+      <c r="H259" t="n">
+        <v>85979.10159999999</v>
+      </c>
+      <c r="I259" t="n">
+        <v>4530638848</v>
+      </c>
+      <c r="J259" t="n">
+        <v>4</v>
+      </c>
+      <c r="K259" t="n">
+        <v>38</v>
+      </c>
+      <c r="L259" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="M259" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="N259" t="n">
+        <v>36</v>
+      </c>
+      <c r="O259" t="n">
+        <v>0.326</v>
+      </c>
+      <c r="P259" t="n">
+        <v>-0.058</v>
+      </c>
+      <c r="Q259" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="R259" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S259" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to 8-month high above $85,000 - qz.com</t>
+        </is>
+      </c>
+      <c r="T259" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9BRHhsSDNaZ2VlVnhzYmRsci1zNk1kQ2JWNHJxNTNVRHFDSHFqcmVoVFg2TkJxYTdZMUhfMEJpb1hFS3RabDlJcVZZWEh4M3VJUUpaX0JUSWtHd0pxNUctNzg3Nkx0Q2JoT21EN2cwV1ZtQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U259" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="V259" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="W259" t="inlineStr">
+        <is>
+          <t>Bitcoin: Surges Above $86,000 With $900M Liquidations - blockchain.news</t>
+        </is>
+      </c>
+      <c r="X259" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPWlJLVVp0NTE2ZWFUZHpuU2d3LXBsMUFZeDVKRy16X2VPZEpUQ19yM09qYkZ0U2o4S2pNZHlFUk56WjloUUtFbzBTdU1leVJXVTVpbExBUkg0T1ZhbllkOHRZUWdINTliV05wMFlRbVNWa0ZReGNMaFVIeFVFamsxNTJxQ00wZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y259" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Reaches $85,000 as Oil Crashes 10% and Pepeto Draws Capital BTC Cannot - TechBullion</t>
+        </is>
+      </c>
+      <c r="Z259" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNeGpPQmJlR0VEeXdiOGJBblBBcjk4TjBSTHpLcnhZOUpaenZ3enF2eWg2WXpZZlVfTjhCZG05cXpwaEFHN2o5X2lXdHFFV0RzWnFZZnpIS215V2hHelA0VGNUdk1WcUdKYTEzbVFmd2FxOTQzQkEyVjlsbzR3eUJZWnV2QVZpRkZDcWZ1R1M3Z0ZVTzV2RWkwQWtrT21UV2otOHBCZEdFbzhDUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA259" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - Morningstar</t>
+        </is>
+      </c>
+      <c r="AB259" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC259" t="inlineStr">
+        <is>
+          <t>Bitcoin’s crashes are shrinking, and Wall Street is starting to notice - coindesk.com</t>
+        </is>
+      </c>
+      <c r="AD259" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxPTUNDOGdpNU11bkFfZGRiMmlTeUNDS05VMjhiQzhhbnl4dUVFNjdSSTlPV3VyT0dzN1JRajhZQm5ITGtpRHVndVdfTXN0dzF2b0t1MWpWbGhIQW5wUVYtN29JTWxiOXRpVUdteFV0UHhFOHVqNjdBcjZPNVl3VkZUaGZTRnM1NkxFQlo4NXJCcmx2dkdNWVVzdVBpUVVhY3RrYUhpaWxveTR1WXBIV0NiZUFYaw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-23 16:21 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD259"/>
+  <dimension ref="A1:AD265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32609,6 +32609,762 @@
       <c r="AD259" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxPTUNDOGdpNU11bkFfZGRiMmlTeUNDS05VMjhiQzhhbnl4dUVFNjdSSTlPV3VyT0dzN1JRajhZQm5ITGtpRHVndVdfTXN0dzF2b0t1MWpWbGhIQW5wUVYtN29JTWxiOXRpVUdteFV0UHhFOHVqNjdBcjZPNVl3VkZUaGZTRnM1NkxFQlo4NXJCcmx2dkdNWVVzdVBpUVVhY3RrYUhpaWxveTR1WXBIV0NiZUFYaw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-09-23T16:18:16+00:00</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>4346.2998</v>
+      </c>
+      <c r="F260" t="n">
+        <v>4350.6001</v>
+      </c>
+      <c r="G260" t="n">
+        <v>4313.2998</v>
+      </c>
+      <c r="H260" t="n">
+        <v>4319.7002</v>
+      </c>
+      <c r="I260" t="n">
+        <v>47883</v>
+      </c>
+      <c r="J260" t="n">
+        <v>4</v>
+      </c>
+      <c r="K260" t="n">
+        <v>39</v>
+      </c>
+      <c r="L260" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="M260" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="N260" t="n">
+        <v>40</v>
+      </c>
+      <c r="O260" t="n">
+        <v>-0.095</v>
+      </c>
+      <c r="P260" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="Q260" t="n">
+        <v>-2.427</v>
+      </c>
+      <c r="R260" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S260" t="inlineStr">
+        <is>
+          <t>TD Securities sees gold entering new bull phase as positioning, ETFs and central bank buying underpin gains - VT Markets</t>
+        </is>
+      </c>
+      <c r="T260" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxQeU1nYzhqTl91TXQtYkNnWGpfb2VURHlkTXBBMkVSRHdMNDRCc2hMc1JiRjA5ODRkdURKSElDR1BmVkdmVXlISVFKOTNoRjVmVEYzTjlPUWVuSUtJaXBidk1EajlmbUFyTUduS0pqZFAtYVozM3Vua3hJSDlBOUdKQnFSMFVySU1nVG8zekdjYl9NQzFBaWFtUng3VG5qRHlGMTB3TlJKZGxNb3FFV2hRajZPLVUyZ1psd0JqcVN0LVVsNXc4Qk1RUXA5aHZucUl2WS1oYjRnR0tVZElSMHVsOHZhcm1WcFdzRFE?oc=5</t>
+        </is>
+      </c>
+      <c r="U260" t="inlineStr">
+        <is>
+          <t>Gold surges by most in six months as dollar drops; copper rises to new record (GLD:NYSEARCA) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V260" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNMUxKaHZFbTh1MERIbGtIeU1xSXlETnIwNXZ2eVZMeEw0SlM1ZGpsRjJIb2UzNWZGMl8zQXoyQV9mUnRHSXBUYXBoSmhFdDJ6WG8tc3RKVkloeFoyYW9BaUNqUWFMM1d0UGdFRzVOMEwtZVFXVUtHWmhEZlZuMVVGN1FXYjRTMVp3OFdVM25JSG1BbXZaS1BrSkdBdzZYVE8xU3E3Qm56dVI3UlBUTHV2eVh4cWM?oc=5</t>
+        </is>
+      </c>
+      <c r="W260" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X260" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y260" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="Z260" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA260" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB260" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC260" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD260" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-09-23T16:18:16+00:00</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E261" t="n">
+        <v>91.06</v>
+      </c>
+      <c r="F261" t="n">
+        <v>92.89</v>
+      </c>
+      <c r="G261" t="n">
+        <v>90.70999999999999</v>
+      </c>
+      <c r="H261" t="n">
+        <v>92.67</v>
+      </c>
+      <c r="I261" t="n">
+        <v>124732</v>
+      </c>
+      <c r="J261" t="n">
+        <v>4</v>
+      </c>
+      <c r="K261" t="n">
+        <v>40</v>
+      </c>
+      <c r="L261" t="n">
+        <v>-0.109</v>
+      </c>
+      <c r="M261" t="n">
+        <v>-0.214</v>
+      </c>
+      <c r="N261" t="n">
+        <v>40</v>
+      </c>
+      <c r="O261" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="P261" t="n">
+        <v>-0.034</v>
+      </c>
+      <c r="Q261" t="n">
+        <v>1.184</v>
+      </c>
+      <c r="R261" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S261" t="inlineStr">
+        <is>
+          <t>Asian Stocks Rise as AI Demand and Lower Oil Prices Lift Markets - Межа. Новини України.</t>
+        </is>
+      </c>
+      <c r="T261" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1LYUMyUDhiTlFhdDZDZWRJV3BXMzBHQmhxaWNhbHhieVJObjJpbU84WHUtaFlITmtnNWVJNW5CX1JrQ1RaTktaQ3pFYVdOZ3VmVkkxWkgtUDN2Zk90V1NwYjFlSF8?oc=5</t>
+        </is>
+      </c>
+      <c r="U261" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V261" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W261" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="X261" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y261" t="inlineStr">
+        <is>
+          <t>US stocks slip after bond yields jump on higher oil prices and a strong economic report - Baltimore Sun</t>
+        </is>
+      </c>
+      <c r="Z261" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPRnFzdHBsNkdUbVpoYS0xdzF5U2lNckVTajVGYjFxMXhPU2RPMW5pMU5Ra2ZTTUY2Yl9mcmczOHNBajdGN1hieXcxeFJVNWczUjRNTXJDY01JWk1tYnFTbEJtTVpTU0FGWGFJbUk1SkZvXzJ1S2t2WkxkTTUzQkI3cXA5endCSU9WckNsenRn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA261" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AB261" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC261" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="AD261" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-09-23T16:18:16+00:00</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>100.895</v>
+      </c>
+      <c r="F262" t="n">
+        <v>101.122</v>
+      </c>
+      <c r="G262" t="n">
+        <v>100.83</v>
+      </c>
+      <c r="H262" t="n">
+        <v>101.058</v>
+      </c>
+      <c r="I262" t="n">
+        <v>0</v>
+      </c>
+      <c r="J262" t="n">
+        <v>4</v>
+      </c>
+      <c r="K262" t="n">
+        <v>38</v>
+      </c>
+      <c r="L262" t="n">
+        <v>-0.053</v>
+      </c>
+      <c r="M262" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="N262" t="n">
+        <v>40</v>
+      </c>
+      <c r="O262" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="P262" t="n">
+        <v>-0.054</v>
+      </c>
+      <c r="Q262" t="n">
+        <v>-0.5649999999999999</v>
+      </c>
+      <c r="R262" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S262" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T262" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U262" t="inlineStr">
+        <is>
+          <t>Gold price seen trading $4,000-4,500 range as strong dollar checks safe-haven demand - Khaleej Times</t>
+        </is>
+      </c>
+      <c r="V262" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQdDhNcUJyZkVSOWs4clk4Zmc1Z1hkSjY4ZVhNTkFGVEFKRzdzOFFxQm5mczhSQ2lSZ2daYnBHc0hhSkQzTFlaZ3NNa01wWEs1RFdiODFqY3NKOE1ZVUNSU24wZnl0R3VRUHhsWURpRGJoejZwNXRzREFHd2l0ZUZqRHNOWDRLdnd4SzQ1cENMZkVnTFRXMzJZemhIdWZUbm5heFQyRlN1RGNVQnU2bEctV3ZnTklleDIyY0lN0gHDAUFVX3lxTE1zQ1JjcnJXUE50Q0ZBTmRPMGlMS3dzWHRXcV9MbWprTE82d3JTdlluSFRORGJQWlh3ZmpqcmRoaDF1bVdlaEkzT2FiWk5TODBCZVNjMl9FY0hPZ1NKT2NycEFNY2QyM3JXb043UXRtUG43VzlXc1FCNlVBOV9nTElwVEdFV04xcURDOEdrVkRIbWlXanRUZVRXeExseHpiR0N6NGtSbW12YnFmdmJwNkliVlJUVGFnMW9jMEg3X0FHREdBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="W262" t="inlineStr">
+        <is>
+          <t>Canadian Dollar Strengthens On Rising Oil Prices Ahead Of Potential US-Iran Talks - InsuranceNewsNet</t>
+        </is>
+      </c>
+      <c r="X262" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOamYyNk9GZ1A3UFZpazcwVnlJZF84eGxxSWpWUDhsWWx6UURTajJKNjMySllWMkNnYnFTRlFuMXpKVEF2dEcyUEVJNjNNbXpPdkhZbmtXQTJnY19DMWQ2RjViYm8wMGJlM2xFZUhDb0pBbUFJeERIYm1JZngyV19pNjBCNWhEZDN5UWdUVlBwM01GTEliVVFSNE5JSzlrQkxQNk1FMDQ5ZUZMLXRIYVVZeDFrWi1mcUZFRHhN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y262" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z262" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA262" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - mufgresearch.com</t>
+        </is>
+      </c>
+      <c r="AB262" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC262" t="inlineStr">
+        <is>
+          <t>Dollar rebounds from losses sparked by Treasury buyback plan - Reuters</t>
+        </is>
+      </c>
+      <c r="AD262" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPamFxZlBhRm1DcmRBZF9VSDd4aXllSmNTWEttZ2dLUkprSnJ5c2xBNXRKT1lQTDdrbXlUUjBnTXdWdVRrWENPYkRkal9pbm9UVDNueFd0am56Z3JCakxsZ2ZHclBRMHpyUUMzeVJHV1FPcVp1dXBYNUtMNk81Z3k1QkRmV1RnRHdPVjhDU3hNYS1xaWxYOU4wMUQwWk5nTDJPWG9kblZIQV9xOG11QTJR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-09-23T16:18:16+00:00</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>7823.75</v>
+      </c>
+      <c r="F263" t="n">
+        <v>7826.25</v>
+      </c>
+      <c r="G263" t="n">
+        <v>7776.5</v>
+      </c>
+      <c r="H263" t="n">
+        <v>7778.75</v>
+      </c>
+      <c r="I263" t="n">
+        <v>646312</v>
+      </c>
+      <c r="J263" t="n">
+        <v>4</v>
+      </c>
+      <c r="K263" t="n">
+        <v>40</v>
+      </c>
+      <c r="L263" t="n">
+        <v>-0.095</v>
+      </c>
+      <c r="M263" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="N263" t="n">
+        <v>40</v>
+      </c>
+      <c r="O263" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="P263" t="n">
+        <v>-0.036</v>
+      </c>
+      <c r="Q263" t="n">
+        <v>0.422</v>
+      </c>
+      <c r="R263" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S263" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T263" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U263" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V263" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W263" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 nears record highs as tech and AI optimism boost market, with potential to exceed 8000 points. - Pluang</t>
+        </is>
+      </c>
+      <c r="X263" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBzSHJ2YV9mU09pcDRfNHdoNm9MYmhNcDdITmJ3RUdxSHoyMTBNUGRGZm9PdGZfT1JtaTN1NFR0MnlwZmdlSi1DRGhONUNwWXRwYTB6cXhWdzVYOVp5VU5NSWVabVJvNk1HcVY4Wm9xekJFVC1uQXJoVzFhNA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y263" t="inlineStr">
+        <is>
+          <t>Rejecting the "U.S. stock market crash" narrative! Goldman Sachs and Deutsche Bank share a bullish outlook - Moomoo</t>
+        </is>
+      </c>
+      <c r="Z263" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQYjVpSnhxZUVPbjJMRm11VkhkRklGNkFQVVY0c3JWdTN6c2UzeUE4ZFozTUNTekI3NXYzazlsRE9ZdTNUcEktSDY3eWhhVVZpM2MzT2FPR0RsenNNbEN3RlFmVGFuemI4Xy1ncEpiSU9Sa0wwdEwwekh3VG9mRlJXd3VZUTRVQjd3TmxWX0tHRTZzWnRYVWFsRE83dWRHdEp2VFM0aGFiS282VWc?oc=5</t>
+        </is>
+      </c>
+      <c r="AA263" t="inlineStr">
+        <is>
+          <t>US stocks slip after bond yields jump on higher oil prices and a strong economic report - Orlando Sentinel</t>
+        </is>
+      </c>
+      <c r="AB263" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPRWE1dEMyY3pVME1JZ2ZYNlNqWllsX0UzbTJLZTlIMkoybFhMeE1zdUJKOU5tU3FvS3hxeUswWFRDOWhEbGhTSjlVWXpMOENiWXljMEwzT00wcFpJaDlWekJWcDMwcjFNdkJIQlhNbWxQVFpjX2xNWTlURWYzTkFNZms4ZzFPS0NMM2FwSk5BN1N1UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC263" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="AD263" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-09-23T16:18:16+00:00</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E264" t="n">
+        <v>30968</v>
+      </c>
+      <c r="F264" t="n">
+        <v>31013</v>
+      </c>
+      <c r="G264" t="n">
+        <v>30642.75</v>
+      </c>
+      <c r="H264" t="n">
+        <v>30739.5</v>
+      </c>
+      <c r="I264" t="n">
+        <v>257400</v>
+      </c>
+      <c r="J264" t="n">
+        <v>4</v>
+      </c>
+      <c r="K264" t="n">
+        <v>34</v>
+      </c>
+      <c r="L264" t="n">
+        <v>-0.186</v>
+      </c>
+      <c r="M264" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="N264" t="n">
+        <v>37</v>
+      </c>
+      <c r="O264" t="n">
+        <v>0.251</v>
+      </c>
+      <c r="P264" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="Q264" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="R264" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S264" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="T264" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U264" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="V264" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="W264" t="inlineStr">
+        <is>
+          <t>Muse Tops Charts, Igniting AI Frenzy as Nasdaq Hits Record and Memory Stocks Surge - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="X264" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBHOC1ndUtleTlXM1FPUlBFa3Rfa0RXMnZDX0xsZ0JBU1dVVmxWRHRSNzJDb3d3UF9rMm9qVE03dEY5YlZ0dm15eVcwUlZGMnhCVHF4RVZ1T1Q2WnU3VTNOdVA4b1pCbHBwc194MEl3dDdmQ096ZUE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y264" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="Z264" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AA264" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AB264" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+      <c r="AC264" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="AD264" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-09-23T16:18:16+00:00</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E265" t="n">
+        <v>85482.1094</v>
+      </c>
+      <c r="F265" t="n">
+        <v>85918.82030000001</v>
+      </c>
+      <c r="G265" t="n">
+        <v>83556.21090000001</v>
+      </c>
+      <c r="H265" t="n">
+        <v>84215</v>
+      </c>
+      <c r="I265" t="n">
+        <v>14680895488</v>
+      </c>
+      <c r="J265" t="n">
+        <v>4</v>
+      </c>
+      <c r="K265" t="n">
+        <v>38</v>
+      </c>
+      <c r="L265" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="M265" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="N265" t="n">
+        <v>35</v>
+      </c>
+      <c r="O265" t="n">
+        <v>0.312</v>
+      </c>
+      <c r="P265" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="Q265" t="n">
+        <v>8.935</v>
+      </c>
+      <c r="R265" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S265" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to 8-month high above $85,000 - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T265" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOeTBySkNJSmR2RUFYbjk3Si1YaDB5WEFQYVdxakN4Xy1aUm5KOVdkb1U3eGtFUUxMLUlJcGltRkhKZUdkQjc1aUdyZjNjV2pmZ1VEUXBoVDZfY2lQck93NzVVX00tNkpkS2lOQ1NfS0FnNU5GMzhzaTFtSGRsQ0FyYWRMbmUxV0N2T3lPQ2Q5SndrdHB2TGRV?oc=5</t>
+        </is>
+      </c>
+      <c r="U265" t="inlineStr">
+        <is>
+          <t>Korea's crypto trading volumes surge 17-fold as Bitcoin rally draws investors back - KED Global</t>
+        </is>
+      </c>
+      <c r="V265" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAwQWt5MXdVS3E1RlE0aVZuQkJOTWw4VTdidDEwNDA3Wl94R2d2aksyS3BoMjFNcHZYaWZ2M2V3VGk4VEtYVmRMX0E3ZEt0emlDUDY5bWZydmVkVTVVVjRjU1ctU3ZwTHdLYUZISVRZWDlaU0FiS2c?oc=5</t>
+        </is>
+      </c>
+      <c r="W265" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="X265" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y265" t="inlineStr">
+        <is>
+          <t>Price jump recalculated: 49 cases from two years - CryptoTicker</t>
+        </is>
+      </c>
+      <c r="Z265" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE1kVTVWcW9PaS1icGItLWRKZDdwcXUyTjFNcXVmM3RmV0pWd2tYUGllak1XTGZJbTJyLVFuQUhSZFptR25GdTh5dUh1RFJKaF9kR0J1b0Q5MDd2T1ZHNERCUHFpZU8tUzh3algxQXBOVlBkYktEYUM4?oc=5</t>
+        </is>
+      </c>
+      <c r="AA265" t="inlineStr">
+        <is>
+          <t>What Is the Best Crypto to Buy Before the Trump and Xi Meeting on September 24? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB265" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQd3JmR3RxRWpZNW1DSWJ4WTBNbFNrRW5xNjNEV0x4dVViYXVwT1dqRGxZVlJvX3hZUGs3dlVuRFdFZVJvdk9hSWk0RFNMTVJCZEJHaHlJcGs5aUFzSlpvVUg5X2s5ZkNNb1NnM05rMkk5QzVadEgyRXRYN2NodWYtTl9Xck4tRWQ4MDdObjlSRlhmdDN6TUhqTmljZWNES3B2OG9nWXp3aktzNFl0MDROd0I5anFoWTQ4ckZLYkJkcnpyd2k1RkExVlZJdFFNRGdJa3FJ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC265" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - Morningstar</t>
+        </is>
+      </c>
+      <c r="AD265" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-23 22:48 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD265"/>
+  <dimension ref="A1:AD271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33365,6 +33365,762 @@
       <c r="AD265" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-09-23T22:47:02+00:00</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>4326.7002</v>
+      </c>
+      <c r="F266" t="n">
+        <v>4329.8999</v>
+      </c>
+      <c r="G266" t="n">
+        <v>4317.2998</v>
+      </c>
+      <c r="H266" t="n">
+        <v>4326</v>
+      </c>
+      <c r="I266" t="n">
+        <v>151588</v>
+      </c>
+      <c r="J266" t="n">
+        <v>4</v>
+      </c>
+      <c r="K266" t="n">
+        <v>39</v>
+      </c>
+      <c r="L266" t="n">
+        <v>-0.027</v>
+      </c>
+      <c r="M266" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="N266" t="n">
+        <v>40</v>
+      </c>
+      <c r="O266" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="P266" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="Q266" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="R266" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S266" t="inlineStr">
+        <is>
+          <t>TD Securities sees gold entering new bull phase as positioning, ETFs and central bank buying underpin gains - VT Markets</t>
+        </is>
+      </c>
+      <c r="T266" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxQeU1nYzhqTl91TXQtYkNnWGpfb2VURHlkTXBBMkVSRHdMNDRCc2hMc1JiRjA5ODRkdURKSElDR1BmVkdmVXlISVFKOTNoRjVmVEYzTjlPUWVuSUtJaXBidk1EajlmbUFyTUduS0pqZFAtYVozM3Vua3hJSDlBOUdKQnFSMFVySU1nVG8zekdjYl9NQzFBaWFtUng3VG5qRHlGMTB3TlJKZGxNb3FFV2hRajZPLVUyZ1psd0JqcVN0LVVsNXc4Qk1RUXA5aHZucUl2WS1oYjRnR0tVZElSMHVsOHZhcm1WcFdzRFE?oc=5</t>
+        </is>
+      </c>
+      <c r="U266" t="inlineStr">
+        <is>
+          <t>Gold price will hit $4,900/oz in 2026 on strong sovereign demand as China buys 75% more than reported in July – Goldman Sachs - kitco.com</t>
+        </is>
+      </c>
+      <c r="V266" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOdmIweWNUQkhQS0N4SVhSTjEzWjBlUU9IX2Vxa2c4cGVvM1RQN3BqRkVRWFBYSHAzdFNqcmdYSFhVWUViVWV5Wmp6cHhERHVOSHNnbTcxYnlaaFZ1Y3lsOWpWRDdxbUR4ZDNlRVlQWEZERkhuLWZaT0VxRkhEamE3QmRGMDNvX3Z1VlVPNnczTFBWbEhlbEZqMkZJYTRsM2FKSXpkWUJIbkVUcGtwaXdwRUUxbDBHTFJ1ZmpjZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W266" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X266" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y266" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="Z266" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA266" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB266" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+      <c r="AC266" t="inlineStr">
+        <is>
+          <t>Gold ETFs Shine in H1 2026 with Unprecedented Liquidity - Investing News Network</t>
+        </is>
+      </c>
+      <c r="AD266" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE1JaGRkaHpGODN4bGpQdFl6S3VyUjZKYzRvWUxjUjhyQ0lVXzZMZEltdGkwMEo2d0lhVWVmMDVUYUJfRXF4emdyX0ZTd0N6SVgwN3kxMFVXTkt5WXZJbE8ybVNRLUJYTVZy?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-09-23T22:47:02+00:00</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E267" t="n">
+        <v>91.66</v>
+      </c>
+      <c r="F267" t="n">
+        <v>93.03</v>
+      </c>
+      <c r="G267" t="n">
+        <v>91.65000000000001</v>
+      </c>
+      <c r="H267" t="n">
+        <v>92.45</v>
+      </c>
+      <c r="I267" t="n">
+        <v>45602</v>
+      </c>
+      <c r="J267" t="n">
+        <v>4</v>
+      </c>
+      <c r="K267" t="n">
+        <v>40</v>
+      </c>
+      <c r="L267" t="n">
+        <v>-0.078</v>
+      </c>
+      <c r="M267" t="n">
+        <v>-0.156</v>
+      </c>
+      <c r="N267" t="n">
+        <v>40</v>
+      </c>
+      <c r="O267" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="P267" t="n">
+        <v>-0.062</v>
+      </c>
+      <c r="Q267" t="n">
+        <v>-0.877</v>
+      </c>
+      <c r="R267" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S267" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="T267" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U267" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="V267" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+      <c r="W267" t="inlineStr">
+        <is>
+          <t>Europe's STOXX 600 rallies on tech, banks strength as oil prices retreat - Reuters</t>
+        </is>
+      </c>
+      <c r="X267" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNYWF0aU9mWUM0TjNtekhpT0I0NTM1RXoydldTZDlzNVM4Q0FnRXFCLTlaLUQxdEZfMS1qeU1XV0lsNHhvc09zMTBUQV9xVFhaakdCU196dW5sQ212UHdLVjVySHo5UWczV0dVS2dnY3d2Q2dTbWRkOWFRZ0g5aTlGaEtnQkFQcno2ZjdfdndQdGdSR1c3MjdEXzNCZlhRM216di1sdllQSl9OT3pkcWRSd3p3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y267" t="inlineStr">
+        <is>
+          <t>US stocks fall after bond yields jump on higher oil prices and a strong economic report - Stamford Advocate</t>
+        </is>
+      </c>
+      <c r="Z267" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNMWVPMFpRaUxVSWhoZGJ4UTlDZEFmdmtUOTlqeWxDTmpZZkpVa1g4MjE5UTRUclhGa3hubC1ady1KWkxQVWlyYlJ3bFE2RkdTb3VjX1NQY1daaDZWVjRsU2YxNkZxMThLbVdjZWRoZ3g3Zkx1NWZqc0swMWxYcnd3a2F5QWQzYkxKVXlYMzRQU05IVEI2SGxKeExud2hpc2o3WVVuZTJnejV3Wlk0SXAwNGtKZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA267" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AB267" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC267" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="AD267" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-09-23T22:47:02+00:00</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E268" t="n">
+        <v>101.096</v>
+      </c>
+      <c r="F268" t="n">
+        <v>101.146</v>
+      </c>
+      <c r="G268" t="n">
+        <v>101.076</v>
+      </c>
+      <c r="H268" t="n">
+        <v>101.115</v>
+      </c>
+      <c r="I268" t="n">
+        <v>0</v>
+      </c>
+      <c r="J268" t="n">
+        <v>4</v>
+      </c>
+      <c r="K268" t="n">
+        <v>38</v>
+      </c>
+      <c r="L268" t="n">
+        <v>-0.054</v>
+      </c>
+      <c r="M268" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="N268" t="n">
+        <v>40</v>
+      </c>
+      <c r="O268" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="P268" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="Q268" t="n">
+        <v>-0.401</v>
+      </c>
+      <c r="R268" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S268" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T268" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U268" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="V268" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W268" t="inlineStr">
+        <is>
+          <t>US Dollar Price Forecast: Hawkish Fed Supports DXY as EUR and GBP Struggle - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X268" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPZzU5UmRLaEJSVG5xMURPTU91clkycEdGaE92b0dUalJNMXhSUEFURmdjMF9fS09HV2Zoelh1blI0X29mcDhJWkU4cXZDVjlCdk5VZUpyVHotZE1teDU5dzNwRjgxdmxqZlplQWRNWV81T05RWW8tNndfRjN3UTgwY3NVM3c2YUw4eS03eGpzNWRPcTFNby1iR1lCcS1iaFduZjlN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y268" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z268" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA268" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AB268" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC268" t="inlineStr">
+        <is>
+          <t>Fed Rate Hike Expectations Cool as Dollar Index Heads for 0.7% Weekly Drop; Yen Posts Strongest Week Since July - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="AD268" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE94WlM1ZkNvNFh0OHpwd2NJSERscXJnUlFBSnZfQkF1SnVOU0RRVExqU2V1VHhkSjFPb0RzNzBabjEyQ0RxVnpvdzY3ekF5eWdBM2JYNWJOZHVzV2hZSEpSYnowczBuNDJVOFZFcktSUTVsQnktZUE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-09-23T22:47:02+00:00</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E269" t="n">
+        <v>7784.25</v>
+      </c>
+      <c r="F269" t="n">
+        <v>7784.75</v>
+      </c>
+      <c r="G269" t="n">
+        <v>7761</v>
+      </c>
+      <c r="H269" t="n">
+        <v>7775</v>
+      </c>
+      <c r="I269" t="n">
+        <v>410802</v>
+      </c>
+      <c r="J269" t="n">
+        <v>4</v>
+      </c>
+      <c r="K269" t="n">
+        <v>40</v>
+      </c>
+      <c r="L269" t="n">
+        <v>-0.064</v>
+      </c>
+      <c r="M269" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="N269" t="n">
+        <v>40</v>
+      </c>
+      <c r="O269" t="n">
+        <v>0.172</v>
+      </c>
+      <c r="P269" t="n">
+        <v>-0.019</v>
+      </c>
+      <c r="Q269" t="n">
+        <v>2.163</v>
+      </c>
+      <c r="R269" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S269" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T269" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U269" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V269" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W269" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 nears record highs as tech and AI optimism boost market, with potential to exceed 8000 points. - Pluang</t>
+        </is>
+      </c>
+      <c r="X269" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBzSHJ2YV9mU09pcDRfNHdoNm9MYmhNcDdITmJ3RUdxSHoyMTBNUGRGZm9PdGZfT1JtaTN1NFR0MnlwZmdlSi1DRGhONUNwWXRwYTB6cXhWdzVYOVp5VU5NSWVabVJvNk1HcVY4Wm9xekJFVC1uQXJoVzFhNA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y269" t="inlineStr">
+        <is>
+          <t>US stocks fall after bond yields jump on higher oil prices and a strong economic report - Stamford Advocate</t>
+        </is>
+      </c>
+      <c r="Z269" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNMWVPMFpRaUxVSWhoZGJ4UTlDZEFmdmtUOTlqeWxDTmpZZkpVa1g4MjE5UTRUclhGa3hubC1ady1KWkxQVWlyYlJ3bFE2RkdTb3VjX1NQY1daaDZWVjRsU2YxNkZxMThLbVdjZWRoZ3g3Zkx1NWZqc0swMWxYcnd3a2F5QWQzYkxKVXlYMzRQU05IVEI2SGxKeExud2hpc2o3WVVuZTJnejV3Wlk0SXAwNGtKZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA269" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="AB269" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC269" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 Falls as 10-Year Treasury Yield Tops 5% After Five-Year PMI High - CryptoRank</t>
+        </is>
+      </c>
+      <c r="AD269" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOWElOdlZ6cHE2dnZ6b3llQzhrRm1NRXgxNnNtRUZzaktQVUpMUWkzemdYTFBhOE9LVXF5STJic0ZjOXNuVElJaUN1QmVMVGNTZm9yaFp6SmQ2R19tMmFsNlJ1aFY3UU1Ec3lYdkI3aWJSb0V3U01zRE4xbl9FVXQ4dHAxLUs5V2lrQmtJZFh4NlNWQTk5U3RFSWxrQmpjNjN6eEZmYmZPTVN2amJR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-09-23T22:47:02+00:00</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E270" t="n">
+        <v>30771</v>
+      </c>
+      <c r="F270" t="n">
+        <v>30813</v>
+      </c>
+      <c r="G270" t="n">
+        <v>30710</v>
+      </c>
+      <c r="H270" t="n">
+        <v>30784.75</v>
+      </c>
+      <c r="I270" t="n">
+        <v>101231</v>
+      </c>
+      <c r="J270" t="n">
+        <v>4</v>
+      </c>
+      <c r="K270" t="n">
+        <v>35</v>
+      </c>
+      <c r="L270" t="n">
+        <v>-0.197</v>
+      </c>
+      <c r="M270" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="N270" t="n">
+        <v>38</v>
+      </c>
+      <c r="O270" t="n">
+        <v>0.192</v>
+      </c>
+      <c r="P270" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="Q270" t="n">
+        <v>-1.29</v>
+      </c>
+      <c r="R270" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S270" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="T270" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U270" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="V270" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="W270" t="inlineStr">
+        <is>
+          <t>Muse Tops Charts, Igniting AI Frenzy as Nasdaq Hits Record and Memory Stocks Surge - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="X270" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBHOC1ndUtleTlXM1FPUlBFa3Rfa0RXMnZDX0xsZ0JBU1dVVmxWRHRSNzJDb3d3UF9rMm9qVE03dEY5YlZ0dm15eVcwUlZGMnhCVHF4RVZ1T1Q2WnU3VTNOdVA4b1pCbHBwc194MEl3dDdmQ096ZUE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y270" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z270" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA270" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB270" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC270" t="inlineStr">
+        <is>
+          <t>Nasdaq rebounds sharply after Fed-driven sell-off - Proactive financial news</t>
+        </is>
+      </c>
+      <c r="AD270" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQb0QtMjVCMlh0RzBoMWp5R1ZPck9HVTMyR1Zvd1BBZFVleDZvNFBHcFdYLWxKRlg4UVFhanhibnY5RUZNQXpuRGRoQkxCc1MzU2xjQWVfdVZMYUlDS0ZrMTV3NnpsRHhvZTN0a2NldlRCT3JDWXotOGRUbjBOcVVza09WWkIzVUpWel80T2V1b09BLWU3S3hPWWdVc19lcmtqSFVHM0xxUDI3TTNuV0FBb3lPN0k0eEloN3N4Rg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-09-23T22:47:02+00:00</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E271" t="n">
+        <v>84323.63280000001</v>
+      </c>
+      <c r="F271" t="n">
+        <v>84659.0781</v>
+      </c>
+      <c r="G271" t="n">
+        <v>84206.1875</v>
+      </c>
+      <c r="H271" t="n">
+        <v>84578.77340000001</v>
+      </c>
+      <c r="I271" t="n">
+        <v>3246104576</v>
+      </c>
+      <c r="J271" t="n">
+        <v>4</v>
+      </c>
+      <c r="K271" t="n">
+        <v>36</v>
+      </c>
+      <c r="L271" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="M271" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="N271" t="n">
+        <v>35</v>
+      </c>
+      <c r="O271" t="n">
+        <v>0.434</v>
+      </c>
+      <c r="P271" t="n">
+        <v>-0.054</v>
+      </c>
+      <c r="Q271" t="n">
+        <v>8.255000000000001</v>
+      </c>
+      <c r="R271" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to 8-month high above $85,000 - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T271" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOeTBySkNJSmR2RUFYbjk3Si1YaDB5WEFQYVdxakN4Xy1aUm5KOVdkb1U3eGtFUUxMLUlJcGltRkhKZUdkQjc1aUdyZjNjV2pmZ1VEUXBoVDZfY2lQck93NzVVX00tNkpkS2lOQ1NfS0FnNU5GMzhzaTFtSGRsQ0FyYWRMbmUxV0N2T3lPQ2Q5SndrdHB2TGRV?oc=5</t>
+        </is>
+      </c>
+      <c r="U271" t="inlineStr">
+        <is>
+          <t>Korea's crypto trading volumes surge 17-fold as Bitcoin rally draws investors back - KED Global</t>
+        </is>
+      </c>
+      <c r="V271" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAwQWt5MXdVS3E1RlE0aVZuQkJOTWw4VTdidDEwNDA3Wl94R2d2aksyS3BoMjFNcHZYaWZ2M2V3VGk4VEtYVmRMX0E3ZEt0emlDUDY5bWZydmVkVTVVVjRjU1ctU3ZwTHdLYUZISVRZWDlaU0FiS2c?oc=5</t>
+        </is>
+      </c>
+      <c r="W271" t="inlineStr">
+        <is>
+          <t>Bitcoin: Surges Above $86,000 With $900M Liquidations - blockchain.news</t>
+        </is>
+      </c>
+      <c r="X271" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPWlJLVVp0NTE2ZWFUZHpuU2d3LXBsMUFZeDVKRy16X2VPZEpUQ19yM09qYkZ0U2o4S2pNZHlFUk56WjloUUtFbzBTdU1leVJXVTVpbExBUkg0T1ZhbllkOHRZUWdINTliV05wMFlRbVNWa0ZReGNMaFVIeFVFamsxNTJxQ00wZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y271" t="inlineStr">
+        <is>
+          <t>What Is the Best Crypto to Buy Before the Trump and Xi Meeting on September 24? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="Z271" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQd3JmR3RxRWpZNW1DSWJ4WTBNbFNrRW5xNjNEV0x4dVViYXVwT1dqRGxZVlJvX3hZUGs3dlVuRFdFZVJvdk9hSWk0RFNMTVJCZEJHaHlJcGs5aUFzSlpvVUg5X2s5ZkNNb1NnM05rMkk5QzVadEgyRXRYN2NodWYtTl9Xck4tRWQ4MDdObjlSRlhmdDN6TUhqTmljZWNES3B2OG9nWXp3aktzNFl0MDROd0I5anFoWTQ4ckZLYkJkcnpyd2k1RkExVlZJdFFNRGdJa3FJ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA271" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - Morningstar</t>
+        </is>
+      </c>
+      <c r="AB271" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC271" t="inlineStr">
+        <is>
+          <t>BitMEX Has Shut Down: Where Do Its Traders Go Now? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AD271" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOM2hMNnhmbnEzc3NCcjZBZjJHd3VZdzZCQnBRaFI3OXN0MC1NMlAtOTVFXzJqWVhtemE1cF9oMjRNVHNTRTlUbWxSTVNSejgtN09iNkZoQnFWbmtTaHlIbGJBUW0weE01bDJnckpoaXFDYk9hYnViSkFHX1JBbU1KVnltSmdNRXFSU0p0ZzZxaDI4NWRjTjA4MXctdkZvYjdpQzdLakc0eGVJMXM?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-24 03:37 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD271"/>
+  <dimension ref="A1:AD277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34121,6 +34121,762 @@
       <c r="AD271" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOM2hMNnhmbnEzc3NCcjZBZjJHd3VZdzZCQnBRaFI3OXN0MC1NMlAtOTVFXzJqWVhtemE1cF9oMjRNVHNTRTlUbWxSTVNSejgtN09iNkZoQnFWbmtTaHlIbGJBUW0weE01bDJnckpoaXFDYk9hYnViSkFHX1JBbU1KVnltSmdNRXFSU0p0ZzZxaDI4NWRjTjA4MXctdkZvYjdpQzdLakc0eGVJMXM?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-09-24T03:34:51+00:00</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>4324.1001</v>
+      </c>
+      <c r="F272" t="n">
+        <v>4338</v>
+      </c>
+      <c r="G272" t="n">
+        <v>4308</v>
+      </c>
+      <c r="H272" t="n">
+        <v>4323</v>
+      </c>
+      <c r="I272" t="n">
+        <v>20594</v>
+      </c>
+      <c r="J272" t="n">
+        <v>4</v>
+      </c>
+      <c r="K272" t="n">
+        <v>39</v>
+      </c>
+      <c r="L272" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="M272" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="N272" t="n">
+        <v>40</v>
+      </c>
+      <c r="O272" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="P272" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="Q272" t="n">
+        <v>0.398</v>
+      </c>
+      <c r="R272" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S272" t="inlineStr">
+        <is>
+          <t>Gold price will hit $4,900/oz in 2026 on strong sovereign demand as China buys 75% more than reported in July – Goldman Sachs - Kitco</t>
+        </is>
+      </c>
+      <c r="T272" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOdmIweWNUQkhQS0N4SVhSTjEzWjBlUU9IX2Vxa2c4cGVvM1RQN3BqRkVRWFBYSHAzdFNqcmdYSFhVWUViVWV5Wmp6cHhERHVOSHNnbTcxYnlaaFZ1Y3lsOWpWRDdxbUR4ZDNlRVlQWEZERkhuLWZaT0VxRkhEamE3QmRGMDNvX3Z1VlVPNnczTFBWbEhlbEZqMkZJYTRsM2FKSXpkWUJIbkVUcGtwaXdwRUUxbDBHTFJ1ZmpjZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U272" t="inlineStr">
+        <is>
+          <t>Gold and silver buybacks hit record levels in North America - Mining.com.au</t>
+        </is>
+      </c>
+      <c r="V272" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPWC0xZVBSelpNZFRHOWI4djBDdnZxYkhjdThyaVNfSVUwcTZsOHZ1bTg2eWxlOWI3bWZQNE5WeTFfdFZoRlIyX0FjdmtLOFRMVFM0TDVzM09ZaEdVeG1tdFZzazlINmxyTDZFMTU0MjliajlYRUVnTzJyaWFQc3FpcmhUc1pWaGc2cWc?oc=5</t>
+        </is>
+      </c>
+      <c r="W272" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X272" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y272" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - english.nv.ua</t>
+        </is>
+      </c>
+      <c r="Z272" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA272" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB272" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC272" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD272" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-09-24T03:34:51+00:00</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E273" t="n">
+        <v>92.14</v>
+      </c>
+      <c r="F273" t="n">
+        <v>92.18000000000001</v>
+      </c>
+      <c r="G273" t="n">
+        <v>91.25</v>
+      </c>
+      <c r="H273" t="n">
+        <v>91.33</v>
+      </c>
+      <c r="I273" t="n">
+        <v>12519</v>
+      </c>
+      <c r="J273" t="n">
+        <v>4</v>
+      </c>
+      <c r="K273" t="n">
+        <v>40</v>
+      </c>
+      <c r="L273" t="n">
+        <v>-0.095</v>
+      </c>
+      <c r="M273" t="n">
+        <v>-0.182</v>
+      </c>
+      <c r="N273" t="n">
+        <v>40</v>
+      </c>
+      <c r="O273" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="P273" t="n">
+        <v>-0.053</v>
+      </c>
+      <c r="Q273" t="n">
+        <v>-0.838</v>
+      </c>
+      <c r="R273" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S273" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="T273" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U273" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="V273" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+      <c r="W273" t="inlineStr">
+        <is>
+          <t>Current price of oil as of July 30, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X273" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9odGxncTZBdXJrcnd4Zm1GSENJSFpJQUJxbGphdTV2dTRfQTVmMzVFQ21PTGhzY19DSGVFUWpoeEtGMDZhNzRveUNoaDBlcDVLSmRpaFh6ZnA1emJSVllSYTNR?oc=5</t>
+        </is>
+      </c>
+      <c r="Y273" t="inlineStr">
+        <is>
+          <t>US stocks fall after bond yields jump on higher oil prices and a strong economic report - WSLS</t>
+        </is>
+      </c>
+      <c r="Z273" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOVkVPYmx3cHBQQ0FuM3hLQzY2SXpIZjRjdVRhWmh4NllobGlvVjdFV2E3alNiRF93c2l3ZjhhN2o5UGZJeWJnN1ZXRUE0SUN1bU90VGliQnV0U0tvdGhYaUx3b2d0Mk9iRWNxR3JQWXJ1TzBHdGRaTFFlczNoN0xkN2hSNnVaQU5UYjcwX1JWZ2pIbGV4dlFDeEJBdkxoUV9uSGxvbFMyZ2JPeFVacW5hbFg0N0w5U1BvVlV3cTZPTzFBTEhYU0E?oc=5</t>
+        </is>
+      </c>
+      <c r="AA273" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 21, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB273" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5KS291VGxrSWo1UjJNRHhZRHlWeFNadWVKS3dfb2VXbzZpOUE4OU9lc0dpWDhJN19ENFlnbEsyUWFySVVyNF8yR2dkSUxzcXJCcHQ4dC1KVzltU0cyWHJ3ajNR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC273" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AD273" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-09-24T03:34:51+00:00</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E274" t="n">
+        <v>101.134</v>
+      </c>
+      <c r="F274" t="n">
+        <v>101.219</v>
+      </c>
+      <c r="G274" t="n">
+        <v>101.062</v>
+      </c>
+      <c r="H274" t="n">
+        <v>101.096</v>
+      </c>
+      <c r="I274" t="n">
+        <v>0</v>
+      </c>
+      <c r="J274" t="n">
+        <v>4</v>
+      </c>
+      <c r="K274" t="n">
+        <v>38</v>
+      </c>
+      <c r="L274" t="n">
+        <v>-0.036</v>
+      </c>
+      <c r="M274" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="N274" t="n">
+        <v>39</v>
+      </c>
+      <c r="O274" t="n">
+        <v>0.143</v>
+      </c>
+      <c r="P274" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="Q274" t="n">
+        <v>1.611</v>
+      </c>
+      <c r="R274" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S274" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="T274" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U274" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens as T-Note Yields Soar - TradingView</t>
+        </is>
+      </c>
+      <c r="V274" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxOTkdqT3BLeGczVldhZ2thVE5QdHVXV3E3eGxPTUh4dFZZVjlCc0c4MG14enJ4RFp0RzNEcEJ5WlNHbDRMVW1HdThSRHNkeWZGWTUta05zcUNDOVlyUnNtMHV0SFg2b1FjcWVQTmcyM2tNUkk5di1uZ3NqMlZ3ZndvbGhKYXIxS29Hck5KNzZuV3UzdVpuTGdMbzU3TnR4WE5O?oc=5</t>
+        </is>
+      </c>
+      <c r="W274" t="inlineStr">
+        <is>
+          <t>US Dollar Price Forecast: Hawkish Fed Supports DXY as EUR and GBP Struggle - finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="X274" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPZzU5UmRLaEJSVG5xMURPTU91clkycEdGaE92b0dUalJNMXhSUEFURmdjMF9fS09HV2Zoelh1blI0X29mcDhJWkU4cXZDVjlCdk5VZUpyVHotZE1teDU5dzNwRjgxdmxqZlplQWRNWV81T05RWW8tNndfRjN3UTgwY3NVM3c2YUw4eS03eGpzNWRPcTFNby1iR1lCcS1iaFduZjlN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y274" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z274" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA274" t="inlineStr">
+        <is>
+          <t>Euro weakens below 1.1400 as Fed rate hike expectations reinforce US Dollar strength - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB274" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxQdDBKc2VPX2hDOXVFbGVUYXVLekI4U3lMb3dSRnEtb0ZaNU93MHA5RkxmTWVfa3hGS2k1eS1lOEZWdmZhXzBpX3FiQ2ExcTlpQTFKNGJRb2NNRHdpNThGM0pHUW15bjR5NHZFa0lJRFhLUzF2YWMyaFMtOEtyOFRrbXJXdGhkQ3pIRXRCSlhBS0REWHJRaFJBM3Ixc3huTWR0LUlXSVd6SGg1N053MmpLY3VBTFU3cW1JTXdBWDdrRUJGaV9h?oc=5</t>
+        </is>
+      </c>
+      <c r="AC274" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD274" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-09-24T03:34:51+00:00</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E275" t="n">
+        <v>7768.25</v>
+      </c>
+      <c r="F275" t="n">
+        <v>7769.75</v>
+      </c>
+      <c r="G275" t="n">
+        <v>7758</v>
+      </c>
+      <c r="H275" t="n">
+        <v>7759</v>
+      </c>
+      <c r="I275" t="n">
+        <v>32217</v>
+      </c>
+      <c r="J275" t="n">
+        <v>4</v>
+      </c>
+      <c r="K275" t="n">
+        <v>40</v>
+      </c>
+      <c r="L275" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="M275" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="N275" t="n">
+        <v>40</v>
+      </c>
+      <c r="O275" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="P275" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="Q275" t="n">
+        <v>4.648</v>
+      </c>
+      <c r="R275" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S275" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="T275" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U275" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V275" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W275" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 posts 3% summer rally. Some on Wall Street think the gains can continue - CNBC</t>
+        </is>
+      </c>
+      <c r="X275" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOZnpTM0tYdTdvczYtRGQyZklaTWhHZFFBRW5SOU1KamRZWFhSTTFQeFpoYnhIX2huUXUtUUFqRTVMRGxjMW1lN3VveGhhYTF1QUx2Y1VBOHYzWThIRU91Y2FGRUVWSmVlRTBlQ1pyMVFha3JtRmpyVktlcUgyTWRoX1oyUTVOSTI0Z1RvQzQtNFZFM3dYVGFtR3hyRVlCLWRQcDFxVHpuUXkzcnM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y275" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z275" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA275" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB275" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC275" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD275" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-09-24T03:34:51+00:00</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E276" t="n">
+        <v>30753.5</v>
+      </c>
+      <c r="F276" t="n">
+        <v>30761</v>
+      </c>
+      <c r="G276" t="n">
+        <v>30700.25</v>
+      </c>
+      <c r="H276" t="n">
+        <v>30707.25</v>
+      </c>
+      <c r="I276" t="n">
+        <v>20964</v>
+      </c>
+      <c r="J276" t="n">
+        <v>4</v>
+      </c>
+      <c r="K276" t="n">
+        <v>35</v>
+      </c>
+      <c r="L276" t="n">
+        <v>-0.356</v>
+      </c>
+      <c r="M276" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N276" t="n">
+        <v>33</v>
+      </c>
+      <c r="O276" t="n">
+        <v>0.269</v>
+      </c>
+      <c r="P276" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="Q276" t="n">
+        <v>-0.791</v>
+      </c>
+      <c r="R276" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S276" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="T276" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U276" t="inlineStr">
+        <is>
+          <t>Stock market today: Dow hits record high, S&amp;P 500 and Nasdaq surge as Big Tech gains power rally - finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="V276" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPbkNnYmlpUUZ1UFBUdG13a1NLZlhpbXR4cEpMcUdqRkR5aXd1UjVKaEFFQTJyQ0JrQWFHN0I0Zk1wSDVOZ0RaRWM2aXpCb3BDQmE4c0dXaHFLQVhRcXdiZDZnSko3UGd6WlkwNlVncFNJdTVnbHVGaFJBTXltM0ttaUxkZ0ZFa2ptNVN5S3FTbXBPOTc3UHdZVEtVYVFqWXNMazVsZlhaY3hibzViazhyeXBta2RFWHF4Z1pN?oc=5</t>
+        </is>
+      </c>
+      <c r="W276" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="X276" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y276" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="Z276" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AA276" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB276" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC276" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD276" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-09-24T03:34:51+00:00</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E277" t="n">
+        <v>84378.3125</v>
+      </c>
+      <c r="F277" t="n">
+        <v>84479.9219</v>
+      </c>
+      <c r="G277" t="n">
+        <v>83727.4375</v>
+      </c>
+      <c r="H277" t="n">
+        <v>83987.02340000001</v>
+      </c>
+      <c r="I277" t="n">
+        <v>3439443968</v>
+      </c>
+      <c r="J277" t="n">
+        <v>4</v>
+      </c>
+      <c r="K277" t="n">
+        <v>37</v>
+      </c>
+      <c r="L277" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="M277" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="N277" t="n">
+        <v>36</v>
+      </c>
+      <c r="O277" t="n">
+        <v>0.545</v>
+      </c>
+      <c r="P277" t="n">
+        <v>-0.011</v>
+      </c>
+      <c r="Q277" t="n">
+        <v>10.904</v>
+      </c>
+      <c r="R277" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S277" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T277" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U277" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to 8-month high above $85,000 - finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="V277" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOeTBySkNJSmR2RUFYbjk3Si1YaDB5WEFQYVdxakN4Xy1aUm5KOVdkb1U3eGtFUUxMLUlJcGltRkhKZUdkQjc1aUdyZjNjV2pmZ1VEUXBoVDZfY2lQck93NzVVX00tNkpkS2lOQ1NfS0FnNU5GMzhzaTFtSGRsQ0FyYWRMbmUxV0N2T3lPQ2Q5SndrdHB2TGRV?oc=5</t>
+        </is>
+      </c>
+      <c r="W277" t="inlineStr">
+        <is>
+          <t>Korea's crypto trading volumes surge 17-fold as Bitcoin rally draws investors back - KED Global</t>
+        </is>
+      </c>
+      <c r="X277" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAwQWt5MXdVS3E1RlE0aVZuQkJOTWw4VTdidDEwNDA3Wl94R2d2aksyS3BoMjFNcHZYaWZ2M2V3VGk4VEtYVmRMX0E3ZEt0emlDUDY5bWZydmVkVTVVVjRjU1ctU3ZwTHdLYUZISVRZWDlaU0FiS2c?oc=5</t>
+        </is>
+      </c>
+      <c r="Y277" t="inlineStr">
+        <is>
+          <t>What Is the Best Crypto to Buy Before the Trump and Xi Meeting on September 24? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="Z277" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQd3JmR3RxRWpZNW1DSWJ4WTBNbFNrRW5xNjNEV0x4dVViYXVwT1dqRGxZVlJvX3hZUGs3dlVuRFdFZVJvdk9hSWk0RFNMTVJCZEJHaHlJcGs5aUFzSlpvVUg5X2s5ZkNNb1NnM05rMkk5QzVadEgyRXRYN2NodWYtTl9Xck4tRWQ4MDdObjlSRlhmdDN6TUhqTmljZWNES3B2OG9nWXp3aktzNFl0MDROd0I5anFoWTQ4ckZLYkJkcnpyd2k1RkExVlZJdFFNRGdJa3FJ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA277" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Reaches $85,000 as Oil Crashes 10% and Remittix Draws Capital With Its PayFi Opportunity - TechBullion</t>
+        </is>
+      </c>
+      <c r="AB277" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNeWpqd2dycVdrekt5ZUhpX09tUl8tTEhUY0x1TlFkSWMwOUlVdU9DWUJkT0x1THNtQ3RNbVRQd3h3VXJpYWR3LWd5V0ZrWDlEQ3ZxVEt3WW1jbktZUTNsbXI3emJRbWdGbFIxVmY4LVliZE4zTHB4U3h4SjhIYkxHZ0Rxb2hDWjR1ZVdZNXV6TDJjNmI2aUxsbGxuQVVWaUFlVTQyV3Nrc3EtSzZXQi03V2tDSHpjRzlZeGcweHZaU2twUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC277" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - Morningstar</t>
+        </is>
+      </c>
+      <c r="AD277" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-24 09:07 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD277"/>
+  <dimension ref="A1:AD283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34877,6 +34877,762 @@
       <c r="AD277" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-09-24T09:05:00+00:00</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>4324.3999</v>
+      </c>
+      <c r="F278" t="n">
+        <v>4331.2002</v>
+      </c>
+      <c r="G278" t="n">
+        <v>4295.6001</v>
+      </c>
+      <c r="H278" t="n">
+        <v>4296.2002</v>
+      </c>
+      <c r="I278" t="n">
+        <v>21127</v>
+      </c>
+      <c r="J278" t="n">
+        <v>4</v>
+      </c>
+      <c r="K278" t="n">
+        <v>39</v>
+      </c>
+      <c r="L278" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="M278" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="N278" t="n">
+        <v>40</v>
+      </c>
+      <c r="O278" t="n">
+        <v>-0.082</v>
+      </c>
+      <c r="P278" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="Q278" t="n">
+        <v>-1.429</v>
+      </c>
+      <c r="R278" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S278" t="inlineStr">
+        <is>
+          <t>Gold price will hit $4,900/oz in 2026 on strong sovereign demand as China buys 75% more than reported in July – Goldman Sachs - Kitco</t>
+        </is>
+      </c>
+      <c r="T278" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOdmIweWNUQkhQS0N4SVhSTjEzWjBlUU9IX2Vxa2c4cGVvM1RQN3BqRkVRWFBYSHAzdFNqcmdYSFhVWUViVWV5Wmp6cHhERHVOSHNnbTcxYnlaaFZ1Y3lsOWpWRDdxbUR4ZDNlRVlQWEZERkhuLWZaT0VxRkhEamE3QmRGMDNvX3Z1VlVPNnczTFBWbEhlbEZqMkZJYTRsM2FKSXpkWUJIbkVUcGtwaXdwRUUxbDBHTFJ1ZmpjZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U278" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="V278" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="W278" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="X278" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y278" t="inlineStr">
+        <is>
+          <t>Founders Metals (TSXV:FDR) Falls 5.65% as Profit-Taking Tests Strong Antino Gold Momentum - kalkine.ca</t>
+        </is>
+      </c>
+      <c r="Z278" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQWjZmSkNZV2p0c3pfYWd1Y2U0NnVtdlNaTGdEU3dDbEZ1QTV2WVZCUXp2bmZFVE5ETHByVmc4R1lBUFlDU2JsejNyNkNCcEk3R2lUQUpPbnl5ZS1aeWZGN0lISTVocl9leXVOdTBrN2dKdGJyVl85N0pUQlFtaEZvTXF3V2MzU0xNcTFydU5fNWZsamhnNDVqSThhVEVuaHYweTI5c1g3ZDlDOWplQl8zVGJqa3JnZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA278" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="AB278" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC278" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD278" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-09-24T09:05:00+00:00</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>91.45999999999999</v>
+      </c>
+      <c r="F279" t="n">
+        <v>94.69</v>
+      </c>
+      <c r="G279" t="n">
+        <v>91.33</v>
+      </c>
+      <c r="H279" t="n">
+        <v>94.37</v>
+      </c>
+      <c r="I279" t="n">
+        <v>47730</v>
+      </c>
+      <c r="J279" t="n">
+        <v>4</v>
+      </c>
+      <c r="K279" t="n">
+        <v>40</v>
+      </c>
+      <c r="L279" t="n">
+        <v>-0.055</v>
+      </c>
+      <c r="M279" t="n">
+        <v>-0.184</v>
+      </c>
+      <c r="N279" t="n">
+        <v>40</v>
+      </c>
+      <c r="O279" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="P279" t="n">
+        <v>-0.095</v>
+      </c>
+      <c r="Q279" t="n">
+        <v>2.851</v>
+      </c>
+      <c r="R279" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S279" t="inlineStr">
+        <is>
+          <t>Road Tanker Equipment Market Industry Outlook Strengthens Amid Rising Global Demand - EIN News</t>
+        </is>
+      </c>
+      <c r="T279" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxNdjZFb0VzdVVYTlgtZ2xrcVVobF84V01sWlAzak1fbjM2Y3pyeGR5YWt0cEVmdXBtcUJYd0pZT0V2TmgyM2M1bUhWMUFQMXM3b0ZieURGV3AxX1NBUk1jRmcyNDZlWlR5ODM3U2RfaGxBRDJZVlllVHpfS0ktRUtGSjh5d0NrdDBPY2tILVFjeTZWeHFZZ2JhQkhXRDdKNms2NzFvRkhzNC1qbGJsWWNhVi1tWjJ1MG1aQnNFQjE1ZEhxY3M?oc=5</t>
+        </is>
+      </c>
+      <c r="U279" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="V279" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+      <c r="W279" t="inlineStr">
+        <is>
+          <t>Europe's STOXX 600 rallies on tech, banks strength as oil prices retreat - Reuters</t>
+        </is>
+      </c>
+      <c r="X279" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNYWF0aU9mWUM0TjNtekhpT0I0NTM1RXoydldTZDlzNVM4Q0FnRXFCLTlaLUQxdEZfMS1qeU1XV0lsNHhvc09zMTBUQV9xVFhaakdCU196dW5sQ212UHdLVjVySHo5UWczV0dVS2dnY3d2Q2dTbWRkOWFRZ0g5aTlGaEtnQkFQcno2ZjdfdndQdGdSR1c3MjdEXzNCZlhRM216di1sdllQSl9OT3pkcWRSd3p3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y279" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 21, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z279" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5KS291VGxrSWo1UjJNRHhZRHlWeFNadWVKS3dfb2VXbzZpOUE4OU9lc0dpWDhJN19ENFlnbEsyUWFySVVyNF8yR2dkSUxzcXJCcHQ4dC1KVzltU0cyWHJ3ajNR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA279" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AB279" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC279" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="AD279" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-09-24T09:05:00+00:00</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>101.08</v>
+      </c>
+      <c r="F280" t="n">
+        <v>101.178</v>
+      </c>
+      <c r="G280" t="n">
+        <v>101.001</v>
+      </c>
+      <c r="H280" t="n">
+        <v>101.163</v>
+      </c>
+      <c r="I280" t="n">
+        <v>0</v>
+      </c>
+      <c r="J280" t="n">
+        <v>4</v>
+      </c>
+      <c r="K280" t="n">
+        <v>40</v>
+      </c>
+      <c r="L280" t="n">
+        <v>-0.027</v>
+      </c>
+      <c r="M280" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="N280" t="n">
+        <v>39</v>
+      </c>
+      <c r="O280" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="P280" t="n">
+        <v>-0.011</v>
+      </c>
+      <c r="Q280" t="n">
+        <v>3.187</v>
+      </c>
+      <c r="R280" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S280" t="inlineStr">
+        <is>
+          <t>New Zealand Dollar gains as US Dollar declines despite hawkish Fed tone - FXStreet</t>
+        </is>
+      </c>
+      <c r="T280" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQZ2dHNGdueVY2N2hwcFMyWlAyTHgtZVNKdlFHZHlERm5FUnBvam5tRXFBZjYycUlQTmI1RUI4WVJoU3R6T0M2ZGJJLUNXU2tuVzFCOVA4VWRXY1VON0l3S1U3SVFLb3NNbU1uV2R5QWVyX0NDTlJkdlVlQzlnakdmUEtGaloxcndaQU5kYzlYZFhIdWU0OVBoMXhhRnYtaFVscXBrYnlhTkxWVjdZNWlIZTNtSGM?oc=5</t>
+        </is>
+      </c>
+      <c r="U280" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - virginiabusiness.com</t>
+        </is>
+      </c>
+      <c r="V280" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W280" t="inlineStr">
+        <is>
+          <t>EUR/USD outlook: Hawkish Fed puts euro on the ropes - stonex.com</t>
+        </is>
+      </c>
+      <c r="X280" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNOFk3LTVtQlhSTWRNN2RfT0VtX2JHdlVUT0tPNUxuQWZ3QUNWUDNvX3lvUVZZT29LbkJxQ05tTnA2VlkxNjNlWWxKVENyN3ktTW1ITmFKQS16TXBaeUFUbTltdV9jaGRmSUFLZVU0NUs5cFR0NWxwUkc5NThqU3lLNmYxcHZJbXo3bDlWNlMyWTh2TzYwd1k4MVNzS296WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y280" t="inlineStr">
+        <is>
+          <t>Strong U.S. Economic Data Lifts Dollar; Taiwan Dollar Weakens Past NT$31.8 Ahead of Long Holiday - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="Z280" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE5wcW5TZnFJMGZyMlF3TmxYZnNwNzlTTUdUWld3ODVCYXkyNmVqTUpWbThlTmhGSFI3NUJycDI0d0NzM1czYTQ2Tk9VTC1lX3hLbWlGd3ZlTkYwVnhlbE94M3NXSWxiWGVrMG9ZNVRya000OTdXWEE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA280" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="AB280" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC280" t="inlineStr">
+        <is>
+          <t>Euro weakens below 1.1400 as Fed rate hike expectations reinforce US Dollar strength - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD280" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxQdDBKc2VPX2hDOXVFbGVUYXVLekI4U3lMb3dSRnEtb0ZaNU93MHA5RkxmTWVfa3hGS2k1eS1lOEZWdmZhXzBpX3FiQ2ExcTlpQTFKNGJRb2NNRHdpNThGM0pHUW15bjR5NHZFa0lJRFhLUzF2YWMyaFMtOEtyOFRrbXJXdGhkQ3pIRXRCSlhBS0REWHJRaFJBM3Ixc3huTWR0LUlXSVd6SGg1N053MmpLY3VBTFU3cW1JTXdBWDdrRUJGaV9h?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-09-24T09:05:00+00:00</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E281" t="n">
+        <v>7754.25</v>
+      </c>
+      <c r="F281" t="n">
+        <v>7760</v>
+      </c>
+      <c r="G281" t="n">
+        <v>7721</v>
+      </c>
+      <c r="H281" t="n">
+        <v>7721.75</v>
+      </c>
+      <c r="I281" t="n">
+        <v>87498</v>
+      </c>
+      <c r="J281" t="n">
+        <v>4</v>
+      </c>
+      <c r="K281" t="n">
+        <v>40</v>
+      </c>
+      <c r="L281" t="n">
+        <v>-0.014</v>
+      </c>
+      <c r="M281" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="N281" t="n">
+        <v>40</v>
+      </c>
+      <c r="O281" t="n">
+        <v>0.191</v>
+      </c>
+      <c r="P281" t="n">
+        <v>-0.031</v>
+      </c>
+      <c r="Q281" t="n">
+        <v>3.526</v>
+      </c>
+      <c r="R281" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S281" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T281" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U281" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V281" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W281" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 posts 3% summer rally. Some on Wall Street think the gains can continue - CNBC</t>
+        </is>
+      </c>
+      <c r="X281" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOZnpTM0tYdTdvczYtRGQyZklaTWhHZFFBRW5SOU1KamRZWFhSTTFQeFpoYnhIX2huUXUtUUFqRTVMRGxjMW1lN3VveGhhYTF1QUx2Y1VBOHYzWThIRU91Y2FGRUVWSmVlRTBlQ1pyMVFha3JtRmpyVktlcUgyTWRoX1oyUTVOSTI0Z1RvQzQtNFZFM3dYVGFtR3hyRVlCLWRQcDFxVHpuUXkzcnM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y281" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z281" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA281" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB281" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+      <c r="AC281" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 Falls as 10-Year Treasury Yield Tops 5% After Five-Year PMI High - CryptoRank</t>
+        </is>
+      </c>
+      <c r="AD281" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOWElOdlZ6cHE2dnZ6b3llQzhrRm1NRXgxNnNtRUZzaktQVUpMUWkzemdYTFBhOE9LVXF5STJic0ZjOXNuVElJaUN1QmVMVGNTZm9yaFp6SmQ2R19tMmFsNlJ1aFY3UU1Ec3lYdkI3aWJSb0V3U01zRE4xbl9FVXQ4dHAxLUs5V2lrQmtJZFh4NlNWQTk5U3RFSWxrQmpjNjN6eEZmYmZPTVN2amJR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-09-24T09:05:00+00:00</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E282" t="n">
+        <v>30685.75</v>
+      </c>
+      <c r="F282" t="n">
+        <v>30716</v>
+      </c>
+      <c r="G282" t="n">
+        <v>30407.25</v>
+      </c>
+      <c r="H282" t="n">
+        <v>30423.25</v>
+      </c>
+      <c r="I282" t="n">
+        <v>51331</v>
+      </c>
+      <c r="J282" t="n">
+        <v>4</v>
+      </c>
+      <c r="K282" t="n">
+        <v>35</v>
+      </c>
+      <c r="L282" t="n">
+        <v>-0.288</v>
+      </c>
+      <c r="M282" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="N282" t="n">
+        <v>34</v>
+      </c>
+      <c r="O282" t="n">
+        <v>0.321</v>
+      </c>
+      <c r="P282" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="Q282" t="n">
+        <v>0.925</v>
+      </c>
+      <c r="R282" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S282" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T282" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U282" t="inlineStr">
+        <is>
+          <t>Stock market today: Dow hits record high, S&amp;P 500 and Nasdaq surge as Big Tech gains power rally - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="V282" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPbkNnYmlpUUZ1UFBUdG13a1NLZlhpbXR4cEpMcUdqRkR5aXd1UjVKaEFFQTJyQ0JrQWFHN0I0Zk1wSDVOZ0RaRWM2aXpCb3BDQmE4c0dXaHFLQVhRcXdiZDZnSko3UGd6WlkwNlVncFNJdTVnbHVGaFJBTXltM0ttaUxkZ0ZFa2ptNVN5S3FTbXBPOTc3UHdZVEtVYVFqWXNMazVsZlhaY3hibzViazhyeXBta2RFWHF4Z1pN?oc=5</t>
+        </is>
+      </c>
+      <c r="W282" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - staradvertiser.com</t>
+        </is>
+      </c>
+      <c r="X282" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y282" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="Z282" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AA282" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB282" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+      <c r="AC282" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="AD282" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-09-24T09:05:00+00:00</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E283" t="n">
+        <v>83963.9688</v>
+      </c>
+      <c r="F283" t="n">
+        <v>84606</v>
+      </c>
+      <c r="G283" t="n">
+        <v>83314.5469</v>
+      </c>
+      <c r="H283" t="n">
+        <v>83604.07030000001</v>
+      </c>
+      <c r="I283" t="n">
+        <v>5337989120</v>
+      </c>
+      <c r="J283" t="n">
+        <v>4</v>
+      </c>
+      <c r="K283" t="n">
+        <v>37</v>
+      </c>
+      <c r="L283" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="M283" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="N283" t="n">
+        <v>36</v>
+      </c>
+      <c r="O283" t="n">
+        <v>0.495</v>
+      </c>
+      <c r="P283" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q283" t="n">
+        <v>10.456</v>
+      </c>
+      <c r="R283" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S283" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T283" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U283" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to 8-month high above $85,000 - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="V283" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOeTBySkNJSmR2RUFYbjk3Si1YaDB5WEFQYVdxakN4Xy1aUm5KOVdkb1U3eGtFUUxMLUlJcGltRkhKZUdkQjc1aUdyZjNjV2pmZ1VEUXBoVDZfY2lQck93NzVVX00tNkpkS2lOQ1NfS0FnNU5GMzhzaTFtSGRsQ0FyYWRMbmUxV0N2T3lPQ2Q5SndrdHB2TGRV?oc=5</t>
+        </is>
+      </c>
+      <c r="W283" t="inlineStr">
+        <is>
+          <t>Korea's crypto trading volumes surge 17-fold as Bitcoin rally draws investors back - KED Global</t>
+        </is>
+      </c>
+      <c r="X283" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAwQWt5MXdVS3E1RlE0aVZuQkJOTWw4VTdidDEwNDA3Wl94R2d2aksyS3BoMjFNcHZYaWZ2M2V3VGk4VEtYVmRMX0E3ZEt0emlDUDY5bWZydmVkVTVVVjRjU1ctU3ZwTHdLYUZISVRZWDlaU0FiS2c?oc=5</t>
+        </is>
+      </c>
+      <c r="Y283" t="inlineStr">
+        <is>
+          <t>BTC, ETH, DOGE price news: Doge slides 8%, Bitcoin under $84,000 in crypto sell-off - coindesk.com</t>
+        </is>
+      </c>
+      <c r="Z283" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNaE9Ja2tiYTUyalVRNl9qNkVOVVBlZXBEMU5QTnZRMVpBcXVtZTlXZ0g0YnB3YU43cC1NR3NpT19xaEdZWHl0N3FMMjEwMjh1b0U4RmQwVENJZ2drZ2pXcjZUM3JpV3VtWkFtcWVxSVFGSndVdFFQZ2dPdFpiZW5IUXJiR0hfM19FRzBNYUNIbTBlQkhzZVI5N2d2dkxPM242dVphV1FnbU5EQkRKb3dDYkVuTW13aTBTRHVhSUwwV0FRdzRxdnI3cTJsdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA283" t="inlineStr">
+        <is>
+          <t>Chainalysis 2026 Crypto Adoption Index: Brazil Leads, Bear Market Resilience Highlighted - KuCoin</t>
+        </is>
+      </c>
+      <c r="AB283" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQeGFHQlYxdm9Ed1h3d25WY3lOcDFNQlA4cWcxZnVOWnRUTnBVc3VwNmxlQlBHc3FOdnQyQ3pQSHVQRDQ2VzRES2JjMkMyVDhRT3RLY3dTc0RQX3M3cC1zYTFkbHpnd1Z4Q2hpc0ZoTWRuREVseXpQak1Bamx1ZGxFVEhuNU9ybk9TLTQxeGVKS2tod2VNQ1Z0U0FEcDhtc2w4QUlQY20yaXZlZnBRWXRubThRZ09PNndxUERocw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC283" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Reaches $85,000 as Oil Crashes 10% and Remittix Draws Capital With Its PayFi Opportunity - TechBullion</t>
+        </is>
+      </c>
+      <c r="AD283" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNeWpqd2dycVdrekt5ZUhpX09tUl8tTEhUY0x1TlFkSWMwOUlVdU9DWUJkT0x1THNtQ3RNbVRQd3h3VXJpYWR3LWd5V0ZrWDlEQ3ZxVEt3WW1jbktZUTNsbXI3emJRbWdGbFIxVmY4LVliZE4zTHB4U3h4SjhIYkxHZ0Rxb2hDWjR1ZVdZNXV6TDJjNmI2aUxsbGxuQVVWaUFlVTQyV3Nrc3EtSzZXQi03V2tDSHpjRzlZeGcweHZaU2twUQ?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-24 16:43 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD283"/>
+  <dimension ref="A1:AD289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35633,6 +35633,762 @@
       <c r="AD283" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNeWpqd2dycVdrekt5ZUhpX09tUl8tTEhUY0x1TlFkSWMwOUlVdU9DWUJkT0x1THNtQ3RNbVRQd3h3VXJpYWR3LWd5V0ZrWDlEQ3ZxVEt3WW1jbktZUTNsbXI3emJRbWdGbFIxVmY4LVliZE4zTHB4U3h4SjhIYkxHZ0Rxb2hDWjR1ZVdZNXV6TDJjNmI2aUxsbGxuQVVWaUFlVTQyV3Nrc3EtSzZXQi03V2tDSHpjRzlZeGcweHZaU2twUQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-09-24T16:40:36+00:00</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E284" t="n">
+        <v>4316.2002</v>
+      </c>
+      <c r="F284" t="n">
+        <v>4324.2998</v>
+      </c>
+      <c r="G284" t="n">
+        <v>4279.5</v>
+      </c>
+      <c r="H284" t="n">
+        <v>4311.2998</v>
+      </c>
+      <c r="I284" t="n">
+        <v>45598</v>
+      </c>
+      <c r="J284" t="n">
+        <v>4</v>
+      </c>
+      <c r="K284" t="n">
+        <v>39</v>
+      </c>
+      <c r="L284" t="n">
+        <v>-0.048</v>
+      </c>
+      <c r="M284" t="n">
+        <v>-0.014</v>
+      </c>
+      <c r="N284" t="n">
+        <v>40</v>
+      </c>
+      <c r="O284" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="P284" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="Q284" t="n">
+        <v>-0.991</v>
+      </c>
+      <c r="R284" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S284" t="inlineStr">
+        <is>
+          <t>Gold price will hit $4,900/oz in 2026 on strong sovereign demand as China buys 75% more than reported in July – Goldman Sachs - Kitco</t>
+        </is>
+      </c>
+      <c r="T284" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOdmIweWNUQkhQS0N4SVhSTjEzWjBlUU9IX2Vxa2c4cGVvM1RQN3BqRkVRWFBYSHAzdFNqcmdYSFhVWUViVWV5Wmp6cHhERHVOSHNnbTcxYnlaaFZ1Y3lsOWpWRDdxbUR4ZDNlRVlQWEZERkhuLWZaT0VxRkhEamE3QmRGMDNvX3Z1VlVPNnczTFBWbEhlbEZqMkZJYTRsM2FKSXpkWUJIbkVUcGtwaXdwRUUxbDBHTFJ1ZmpjZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U284" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="V284" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="W284" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="X284" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y284" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="Z284" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA284" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB284" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC284" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD284" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-09-24T16:40:36+00:00</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E285" t="n">
+        <v>93.92</v>
+      </c>
+      <c r="F285" t="n">
+        <v>96.78</v>
+      </c>
+      <c r="G285" t="n">
+        <v>93.52</v>
+      </c>
+      <c r="H285" t="n">
+        <v>94.03</v>
+      </c>
+      <c r="I285" t="n">
+        <v>154098</v>
+      </c>
+      <c r="J285" t="n">
+        <v>4</v>
+      </c>
+      <c r="K285" t="n">
+        <v>40</v>
+      </c>
+      <c r="L285" t="n">
+        <v>-0.003</v>
+      </c>
+      <c r="M285" t="n">
+        <v>-0.211</v>
+      </c>
+      <c r="N285" t="n">
+        <v>40</v>
+      </c>
+      <c r="O285" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="P285" t="n">
+        <v>-0.07099999999999999</v>
+      </c>
+      <c r="Q285" t="n">
+        <v>1.827</v>
+      </c>
+      <c r="R285" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S285" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="T285" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+      <c r="U285" t="inlineStr">
+        <is>
+          <t>Europe's STOXX 600 rallies on tech, banks strength as oil prices retreat - Reuters</t>
+        </is>
+      </c>
+      <c r="V285" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNYWF0aU9mWUM0TjNtekhpT0I0NTM1RXoydldTZDlzNVM4Q0FnRXFCLTlaLUQxdEZfMS1qeU1XV0lsNHhvc09zMTBUQV9xVFhaakdCU196dW5sQ212UHdLVjVySHo5UWczV0dVS2dnY3d2Q2dTbWRkOWFRZ0g5aTlGaEtnQkFQcno2ZjdfdndQdGdSR1c3MjdEXzNCZlhRM216di1sdllQSl9OT3pkcWRSd3p3?oc=5</t>
+        </is>
+      </c>
+      <c r="W285" t="inlineStr">
+        <is>
+          <t>BTC Breaks Resistance, Eyes $85K–$95K Range - Action Forex</t>
+        </is>
+      </c>
+      <c r="X285" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNZGVLanR1Sy05Tm5XSDFLdDdEeW40UTdSUm9ZT2t2Z3JRNHdaYlpxU1BTeDd4VkR1eGw2d3JJNlFaMDI3Tksycm5zcE9sUm5pM1VEM1lkVkQzWDRNUmswQUYyT2NFa09UcnZQdkFKRXBoOEtFVVRzbVpSbnpYa1NLbWJOaFFxZWNHTTAzQy1LS2xoekVYZGZCVTVDajZCY2VoQi12NXRBdFl5bnBYemJz?oc=5</t>
+        </is>
+      </c>
+      <c r="Y285" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z285" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA285" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AB285" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC285" t="inlineStr">
+        <is>
+          <t>Brent Oil breaks below $103 support: Live levels - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD285" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPVXk0bHVBcmVMZGtMeTFpVUVfTWFXSE9Qd20tc3JDMHgyVi00ZFpodkdya0ZHLXI4MUdQTDZzS2M2MzVMWnBIMUZicXBYZld5Tl9jTTZsM1hOUHJJdFNqcE1SZVRSU2FFR01iQTJ3UlZTWmdPakZFNkpoQlhjMzVJU0VsY3p0Zndwa005eUQwMldkbFhHckFhMTJxdFBPNEpBYmZXWVBUSjBsbXlWQy1mLWhYbVc2U19Scy1VOE1CQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-09-24T16:40:36+00:00</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E286" t="n">
+        <v>101.232</v>
+      </c>
+      <c r="F286" t="n">
+        <v>101.377</v>
+      </c>
+      <c r="G286" t="n">
+        <v>101.134</v>
+      </c>
+      <c r="H286" t="n">
+        <v>101.202</v>
+      </c>
+      <c r="I286" t="n">
+        <v>0</v>
+      </c>
+      <c r="J286" t="n">
+        <v>4</v>
+      </c>
+      <c r="K286" t="n">
+        <v>40</v>
+      </c>
+      <c r="L286" t="n">
+        <v>-0.118</v>
+      </c>
+      <c r="M286" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="N286" t="n">
+        <v>40</v>
+      </c>
+      <c r="O286" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="P286" t="n">
+        <v>-0.008999999999999999</v>
+      </c>
+      <c r="Q286" t="n">
+        <v>0.547</v>
+      </c>
+      <c r="R286" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S286" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T286" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U286" t="inlineStr">
+        <is>
+          <t>New Zealand Dollar gains as US Dollar declines despite hawkish Fed tone - FXStreet</t>
+        </is>
+      </c>
+      <c r="V286" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQZ2dHNGdueVY2N2hwcFMyWlAyTHgtZVNKdlFHZHlERm5FUnBvam5tRXFBZjYycUlQTmI1RUI4WVJoU3R6T0M2ZGJJLUNXU2tuVzFCOVA4VWRXY1VON0l3S1U3SVFLb3NNbU1uV2R5QWVyX0NDTlJkdlVlQzlnakdmUEtGaloxcndaQU5kYzlYZFhIdWU0OVBoMXhhRnYtaFVscXBrYnlhTkxWVjdZNWlIZTNtSGM?oc=5</t>
+        </is>
+      </c>
+      <c r="W286" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="X286" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y286" t="inlineStr">
+        <is>
+          <t>Strong U.S. Economic Data Lifts Dollar; Taiwan Dollar Weakens Past NT$31.8 Ahead of Long Holiday - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="Z286" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE5wcW5TZnFJMGZyMlF3TmxYZnNwNzlTTUdUWld3ODVCYXkyNmVqTUpWbThlTmhGSFI3NUJycDI0d0NzM1czYTQ2Tk9VTC1lX3hLbWlGd3ZlTkYwVnhlbE94M3NXSWxiWGVrMG9ZNVRya000OTdXWEE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA286" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="AB286" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC286" t="inlineStr">
+        <is>
+          <t>Euro weakens below 1.1400 as Fed rate hike expectations reinforce US Dollar strength - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD286" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxQdDBKc2VPX2hDOXVFbGVUYXVLekI4U3lMb3dSRnEtb0ZaNU93MHA5RkxmTWVfa3hGS2k1eS1lOEZWdmZhXzBpX3FiQ2ExcTlpQTFKNGJRb2NNRHdpNThGM0pHUW15bjR5NHZFa0lJRFhLUzF2YWMyaFMtOEtyOFRrbXJXdGhkQ3pIRXRCSlhBS0REWHJRaFJBM3Ixc3huTWR0LUlXSVd6SGg1N053MmpLY3VBTFU3cW1JTXdBWDdrRUJGaV9h?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-09-24T16:40:36+00:00</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E287" t="n">
+        <v>7734.75</v>
+      </c>
+      <c r="F287" t="n">
+        <v>7778</v>
+      </c>
+      <c r="G287" t="n">
+        <v>7725.25</v>
+      </c>
+      <c r="H287" t="n">
+        <v>7758</v>
+      </c>
+      <c r="I287" t="n">
+        <v>685926</v>
+      </c>
+      <c r="J287" t="n">
+        <v>4</v>
+      </c>
+      <c r="K287" t="n">
+        <v>39</v>
+      </c>
+      <c r="L287" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="M287" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="N287" t="n">
+        <v>40</v>
+      </c>
+      <c r="O287" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="P287" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="Q287" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="R287" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S287" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T287" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U287" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V287" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W287" t="inlineStr">
+        <is>
+          <t>Stock market today: Dow hits record high, S&amp;P 500 and Nasdaq surge as Big Tech gains power rally - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X287" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPbkNnYmlpUUZ1UFBUdG13a1NLZlhpbXR4cEpMcUdqRkR5aXd1UjVKaEFFQTJyQ0JrQWFHN0I0Zk1wSDVOZ0RaRWM2aXpCb3BDQmE4c0dXaHFLQVhRcXdiZDZnSko3UGd6WlkwNlVncFNJdTVnbHVGaFJBTXltM0ttaUxkZ0ZFa2ptNVN5S3FTbXBPOTc3UHdZVEtVYVFqWXNMazVsZlhaY3hibzViazhyeXBta2RFWHF4Z1pN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y287" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics Surges 11.39% as CRSP Stock Breaks Above $58 - RSI Oversold Picks - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z287" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOb3N1QlpQbGN6ci1CNHo3MHFGMHBLVVd1YkNwYU9MX0JQUThkcWt3b3pOMzIyZDI1OGN4UmIya3MzNkd3ZmRoTUFqam90MVlPX0VxaGxUY1YyclN0SWY3b1dSZ3FKQ08zcUEwNHF2NUxfLW9hWThBOHJlQXNOU3FZVm9JZTJObGJnbDZ2eHN6MWIzamtpZ1JCRW5ydXNEU3ZuX3hxaEdua2UzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA287" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB287" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC287" t="inlineStr">
+        <is>
+          <t>FTSE 100 flat again after Wall Street drops - UK Investor Magazine</t>
+        </is>
+      </c>
+      <c r="AD287" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQSnI3anlJTS0tUGJsWjAyc1hYbE40c0dRUklVc2Y5U0QyYU45R1JVT2JyZjE3S3ZHNnVqaU1sWkFacGV0SlJIZ3NyRHBkYUZYaG1Jc0pHeV9oMXlMNmxTSElNNzkxR09rM3dOb2NCODdVTlF4MmIyMVBFX0ZKUHEyVzFSUQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-09-24T16:40:36+00:00</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>30486.5</v>
+      </c>
+      <c r="F288" t="n">
+        <v>30748</v>
+      </c>
+      <c r="G288" t="n">
+        <v>30484.25</v>
+      </c>
+      <c r="H288" t="n">
+        <v>30668.75</v>
+      </c>
+      <c r="I288" t="n">
+        <v>283213</v>
+      </c>
+      <c r="J288" t="n">
+        <v>4</v>
+      </c>
+      <c r="K288" t="n">
+        <v>35</v>
+      </c>
+      <c r="L288" t="n">
+        <v>-0.316</v>
+      </c>
+      <c r="M288" t="n">
+        <v>0.136</v>
+      </c>
+      <c r="N288" t="n">
+        <v>34</v>
+      </c>
+      <c r="O288" t="n">
+        <v>0.295</v>
+      </c>
+      <c r="P288" t="n">
+        <v>0.136</v>
+      </c>
+      <c r="Q288" t="n">
+        <v>-0.014</v>
+      </c>
+      <c r="R288" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S288" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T288" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U288" t="inlineStr">
+        <is>
+          <t>Stock market today: Dow hits record high, S&amp;P 500 and Nasdaq surge as Big Tech gains power rally - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="V288" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPbkNnYmlpUUZ1UFBUdG13a1NLZlhpbXR4cEpMcUdqRkR5aXd1UjVKaEFFQTJyQ0JrQWFHN0I0Zk1wSDVOZ0RaRWM2aXpCb3BDQmE4c0dXaHFLQVhRcXdiZDZnSko3UGd6WlkwNlVncFNJdTVnbHVGaFJBTXltM0ttaUxkZ0ZFa2ptNVN5S3FTbXBPOTc3UHdZVEtVYVFqWXNMazVsZlhaY3hibzViazhyeXBta2RFWHF4Z1pN?oc=5</t>
+        </is>
+      </c>
+      <c r="W288" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="X288" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y288" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z288" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA288" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB288" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC288" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD288" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-09-24T16:40:36+00:00</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>83581.64840000001</v>
+      </c>
+      <c r="F289" t="n">
+        <v>84894.11719999999</v>
+      </c>
+      <c r="G289" t="n">
+        <v>83387.21090000001</v>
+      </c>
+      <c r="H289" t="n">
+        <v>84802.8906</v>
+      </c>
+      <c r="I289" t="n">
+        <v>2696982528</v>
+      </c>
+      <c r="J289" t="n">
+        <v>4</v>
+      </c>
+      <c r="K289" t="n">
+        <v>37</v>
+      </c>
+      <c r="L289" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="M289" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="N289" t="n">
+        <v>36</v>
+      </c>
+      <c r="O289" t="n">
+        <v>0.434</v>
+      </c>
+      <c r="P289" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="Q289" t="n">
+        <v>9.114000000000001</v>
+      </c>
+      <c r="R289" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S289" t="inlineStr">
+        <is>
+          <t>Bitcoin: Surges Above $86,000 With $900M Liquidations - blockchain.news</t>
+        </is>
+      </c>
+      <c r="T289" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPWlJLVVp0NTE2ZWFUZHpuU2d3LXBsMUFZeDVKRy16X2VPZEpUQ19yM09qYkZ0U2o4S2pNZHlFUk56WjloUUtFbzBTdU1leVJXVTVpbExBUkg0T1ZhbllkOHRZUWdINTliV05wMFlRbVNWa0ZReGNMaFVIeFVFamsxNTJxQ00wZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U289" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to $85,000 as $648M in shorts liquidated - TradingView</t>
+        </is>
+      </c>
+      <c r="V289" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQRHZIOW9Xc2xkakVMRUlRV2F5a0thZHN0ZFREZ2lrOUowVjVWd0lBaE0yWmRMdkdxZW0zLUdnbTE1MFZsa05kRkRqbWhhZUdmMlFXa0NlUlJBRjlNVXVGcW9UdWl0RnlWUVhiZi11ZDlCSUxGRXVPYUNXaVZfbS01dnp3cFlfd3NMeHk2eUhzWkpyRVBfSWR5YUN6U0tRRnFDWGZJcDlQbTJCdG1FMGxrSHdpY0dmVHFDRkE?oc=5</t>
+        </is>
+      </c>
+      <c r="W289" t="inlineStr">
+        <is>
+          <t>'It’s crypto spring': 4 reasons for bitcoin’s surge above $85,000 - Yahoo Finance UK</t>
+        </is>
+      </c>
+      <c r="X289" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNZzU1dUlEakhTNVlkT2pTU0xzeS1fNU9PQkJybHd5U0dmalhUTnZVNHN2UFV6MkdOT05OejhwbkY1MlZocVFvZ2NhMF9iVHVFbFlxcjY1S2ktN3lncGRVaWVYUjdfTUJLQ25QdE1VSTNyYVFMWm1WU3FuM3NFWkx4SlNaa3hGaFE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y289" t="inlineStr">
+        <is>
+          <t>Bitcoin miners sell 20,000 BTC to Binance witho... - Pluang</t>
+        </is>
+      </c>
+      <c r="Z289" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOVW1uRV9RaHZHWDE3TnpyWExZbm8xYkdvaWdGWTI2M3VRamtBa3V0Q2lxano2eFFZdkhwZzF3MmlPMWRDSVUyZ3BGTlZQVlIwZUdjVk4wZm1iU2MtTW8yMDNuSlFzdzNtbEN0TFFhV1dCcGNCQ2p3VVlDb3NzR1Q2NGVoY2hsVU4tRWtpbHV1S0pDdTJXSmxKLTBDLVFLZkp4b2hnRw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA289" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - global.morningstar.com</t>
+        </is>
+      </c>
+      <c r="AB289" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC289" t="inlineStr">
+        <is>
+          <t>Bitcoin Price LIVE: JGB Sell-Off Puts $81,178 in Focus as BTC Breaks $84,304 Equilibrium - CryptoRank</t>
+        </is>
+      </c>
+      <c r="AD289" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPVExlTUQtSEl1aUFtdjc4Y0s3b2dXT2xjTHY3ODB5REY4d2JGa21kZ2VORmMxQ25kMHNKQ2JrR25COS1Ia1dXMWNVbmcxaE9RNlFuR19teDNPbEwzOVFBREoySHV2Xzg2czN3VVdyaXFWWlpGQXBkaHRNT05xZWhKU012RFpTZWpkd2tBdWNidG5YNlJQeGRiTVZUR2NJYUViVHNqM3FILVIzeHdabUxSNnpfa1U5XzhjQXZfRTFR?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-24 23:07 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD289"/>
+  <dimension ref="A1:AD295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36389,6 +36389,762 @@
       <c r="AD289" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPVExlTUQtSEl1aUFtdjc4Y0s3b2dXT2xjTHY3ODB5REY4d2JGa21kZ2VORmMxQ25kMHNKQ2JrR25COS1Ia1dXMWNVbmcxaE9RNlFuR19teDNPbEwzOVFBREoySHV2Xzg2czN3VVdyaXFWWlpGQXBkaHRNT05xZWhKU012RFpTZWpkd2tBdWNidG5YNlJQeGRiTVZUR2NJYUViVHNqM3FILVIzeHdabUxSNnpfa1U5XzhjQXZfRTFR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-09-24T23:04:54+00:00</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>4300.2002</v>
+      </c>
+      <c r="F290" t="n">
+        <v>4317.2002</v>
+      </c>
+      <c r="G290" t="n">
+        <v>4291.2998</v>
+      </c>
+      <c r="H290" t="n">
+        <v>4307.5</v>
+      </c>
+      <c r="I290" t="n">
+        <v>18420</v>
+      </c>
+      <c r="J290" t="n">
+        <v>4</v>
+      </c>
+      <c r="K290" t="n">
+        <v>39</v>
+      </c>
+      <c r="L290" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="M290" t="n">
+        <v>-0.028</v>
+      </c>
+      <c r="N290" t="n">
+        <v>40</v>
+      </c>
+      <c r="O290" t="n">
+        <v>-0.036</v>
+      </c>
+      <c r="P290" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="Q290" t="n">
+        <v>-2.099</v>
+      </c>
+      <c r="R290" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S290" t="inlineStr">
+        <is>
+          <t>Gold price will hit $4,900/oz in 2026 on strong sovereign demand as China buys 75% more than reported in July – Goldman Sachs - kitco.com</t>
+        </is>
+      </c>
+      <c r="T290" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOdmIweWNUQkhQS0N4SVhSTjEzWjBlUU9IX2Vxa2c4cGVvM1RQN3BqRkVRWFBYSHAzdFNqcmdYSFhVWUViVWV5Wmp6cHhERHVOSHNnbTcxYnlaaFZ1Y3lsOWpWRDdxbUR4ZDNlRVlQWEZERkhuLWZaT0VxRkhEamE3QmRGMDNvX3Z1VlVPNnczTFBWbEhlbEZqMkZJYTRsM2FKSXpkWUJIbkVUcGtwaXdwRUUxbDBHTFJ1ZmpjZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U290" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="V290" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="W290" t="inlineStr">
+        <is>
+          <t>Gold hits record high as investors seek safety - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="X290" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVWt1Y1hBWG5uZFNjRUFtZHlqRUhfZGV6VzAtQ0tBT2VlVDVEZEJ2WHN0YndCcXRzSjNtVnFhUFZZZ2F4RFRxYkdsSF91eDk2MFl5R3JNWk1HREJjSVdhUE1uTTU1N1Z6Y2xfZzZCSDZ4YnhaT1czcWdXeHE3SjJBR2FqUm43Z0paUG5OVEdsWVdYYnZBWVHSAZsBQVVfeXFMTWh6VXlqZGZVbUl3SHVfQ195WFFveEVkLU9TU1RXMTZBdVhodU16UWxLLWVScDNsc2VGMThyT0RTTHB4SVNRYU1KWmRycHhnTEc0NTJ1RWgzdGc2Y0VkanR4QUtlUWFBSnB2cElORUltQk9XdWRLNXhKbU5jRUFqQVd6bG5YbURJakxhNTl3UEk4RzBaQzVJaVdRdFk?oc=5</t>
+        </is>
+      </c>
+      <c r="Y290" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="Z290" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA290" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - kitco.com</t>
+        </is>
+      </c>
+      <c r="AB290" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC290" t="inlineStr">
+        <is>
+          <t>EUR/USD and GBP/USD break support – Gold and Silver on a knife’s edge [Video] - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD290" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQcWJpUEpUOTF2dzFZcktNQ2UwWGQ3MWpXMHlLbkhEcHJCQkJiVUdIZEFxYzdfc01jVXQwNjd3VG1HMnF4UWdpVkJiWFplT3Y5NmJkOWhxcjhxVDNSZ0N4LWtuSVBfX01WUFhxOWVic0dmLUhpbWNxS1BqWUlDZnJ0LWRCYzdZalhueVFBYVAzTFZnbnRvRTJHU1MzOC12aWVDZkpRZlFoY01BQTA3MDJXNF9NeWJUOVFQMFBz?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-09-24T23:04:54+00:00</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>95.3</v>
+      </c>
+      <c r="F291" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="G291" t="n">
+        <v>93.88</v>
+      </c>
+      <c r="H291" t="n">
+        <v>94.38</v>
+      </c>
+      <c r="I291" t="n">
+        <v>55344</v>
+      </c>
+      <c r="J291" t="n">
+        <v>4</v>
+      </c>
+      <c r="K291" t="n">
+        <v>40</v>
+      </c>
+      <c r="L291" t="n">
+        <v>-0.005</v>
+      </c>
+      <c r="M291" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="N291" t="n">
+        <v>40</v>
+      </c>
+      <c r="O291" t="n">
+        <v>0.136</v>
+      </c>
+      <c r="P291" t="n">
+        <v>-0.08699999999999999</v>
+      </c>
+      <c r="Q291" t="n">
+        <v>2.607</v>
+      </c>
+      <c r="R291" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S291" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - energynow.com</t>
+        </is>
+      </c>
+      <c r="T291" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U291" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 24, 2026 - au.finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="V291" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxOb2pJQmtvNklTblpFU0RUUXF0SHZHdTl6Ujh1NDg3bEc4TnYyZVFtNU1zU2tpdHFYRVR3alVaTTNsM0VyLVp3eV9NVmtjWHVKMHYwN3dLUjh0elZtcW9LcHBJaUlfaExpZjNOYzFvazB2MEg5QXc5QWo2QlRLdzQyR1oyU3N4dw?oc=5</t>
+        </is>
+      </c>
+      <c r="W291" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X291" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y291" t="inlineStr">
+        <is>
+          <t>US Equity Markets End Mixed Amid Rising Oil Prices, Strong Macroeconomic Data - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="Z291" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxON3VpM1dxR25YQUhXSlZLcWxWWDJXaTFtZWptazNyLTVhVG9sakhkdTlWSGdHcUJkSG9lVmZuS1lEcWE1TUVVN3dNRUJHWVhadnBwSGpSbVQtZUxJdWtTaXdZNkhFQnlhbXY4TnZZY09DODJEdm1GcjBWTWhQUzFXb1ZEVGxzSHNhVW9xRzdueWtYM1YxLXlR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA291" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AB291" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC291" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD291" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-09-24T23:04:54+00:00</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>101.285</v>
+      </c>
+      <c r="F292" t="n">
+        <v>101.316</v>
+      </c>
+      <c r="G292" t="n">
+        <v>101.24</v>
+      </c>
+      <c r="H292" t="n">
+        <v>101.248</v>
+      </c>
+      <c r="I292" t="n">
+        <v>0</v>
+      </c>
+      <c r="J292" t="n">
+        <v>4</v>
+      </c>
+      <c r="K292" t="n">
+        <v>40</v>
+      </c>
+      <c r="L292" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="M292" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="N292" t="n">
+        <v>40</v>
+      </c>
+      <c r="O292" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="P292" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="Q292" t="n">
+        <v>3.048</v>
+      </c>
+      <c r="R292" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S292" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T292" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U292" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="V292" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQNkZhLVNRRzlQWGRxQnZUa0tLX0Y4LXF3dXd4NEtpTVlHREtlX0RpRWw4T2tyakdpWFc5U2x5Y3B4Q1ZrclB0MEdwMEFjM0xia1J0UHRaLU41bEM1UFRaQ3lFMU5haXRjcUQtY0w3N2tZUzBSMC1CeXNVendmaWU5OXFFY0wteWk4N2h6dmhXSnhPaVdpalJsYV9VOGMtaGRmc0FNX3FpTnFfNXhnT0ZqMU5qUHRxOFgzRE9HaQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W292" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="X292" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y292" t="inlineStr">
+        <is>
+          <t>Strong U.S. Economic Data Lifts Dollar; Taiwan Dollar Weakens Past NT$31.8 Ahead of Long Holiday - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="Z292" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE5wcW5TZnFJMGZyMlF3TmxYZnNwNzlTTUdUWld3ODVCYXkyNmVqTUpWbThlTmhGSFI3NUJycDI0d0NzM1czYTQ2Tk9VTC1lX3hLbWlGd3ZlTkYwVnhlbE94M3NXSWxiWGVrMG9ZNVRya000OTdXWEE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA292" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="AB292" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AC292" t="inlineStr">
+        <is>
+          <t>Hungarian forint weakens past 366 per euro - Daily News Hungary</t>
+        </is>
+      </c>
+      <c r="AD292" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE8wYUpiZWt0eUY0R2pDRFhlNU9NR1A2NmVvSi1FRHlVejZyb01YZWoweHNCM0t4WXhlTnhwQ3pqTDhQTTBKVlduZENjMThucUJ0Tm5MbVZPSjQ3QUhXVTJ6dnl3cHBZSFJWRlVMWHcwcHJDY3EtUkJoSUo4bjA?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-09-24T23:04:54+00:00</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>7763.25</v>
+      </c>
+      <c r="F293" t="n">
+        <v>7777.75</v>
+      </c>
+      <c r="G293" t="n">
+        <v>7748.75</v>
+      </c>
+      <c r="H293" t="n">
+        <v>7756.75</v>
+      </c>
+      <c r="I293" t="n">
+        <v>404179</v>
+      </c>
+      <c r="J293" t="n">
+        <v>4</v>
+      </c>
+      <c r="K293" t="n">
+        <v>38</v>
+      </c>
+      <c r="L293" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="M293" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="N293" t="n">
+        <v>40</v>
+      </c>
+      <c r="O293" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="P293" t="n">
+        <v>-0.014</v>
+      </c>
+      <c r="Q293" t="n">
+        <v>5.169</v>
+      </c>
+      <c r="R293" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S293" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - aol.com</t>
+        </is>
+      </c>
+      <c r="T293" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="U293" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 set for strong year-end rally despite r... - Pluang</t>
+        </is>
+      </c>
+      <c r="V293" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTFBJY3VWNDgwOEZQdnZSWlROZjZ3RGY1eXJsR1poYVhoelM0ZlZLZGVoY1FuRWtaa2QtWnVyUjd5YS1INGlZbExIaVpPR0dPb3RfUHNBeU1MdUwwTEhwbzNMeHVDb3c3UE5fakhCUURHQXJWaHpLWjBJT2Z3?oc=5</t>
+        </is>
+      </c>
+      <c r="W293" t="inlineStr">
+        <is>
+          <t>Global benchmarks mostly rise after Wall Street's rally - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="X293" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQQzQ4eHpITXFBQXAzWTczOVJxa2NxcVdTcWhRVXZwYTVCTUJjM1QzZkI5M0szbmRnQnlwOXdaM1BEQ0V3U3pqU1o4MkVFSHJPM180eXJKalNjWUttdDFXVnR3RXRqaGJOQllmMjhHWFpGOUxROUJRbjQ4N1hablgtQ29md2lGcWl4T21WSm9seWVYS0Zp0gGaAUFVX3lxTE1xV1lTRnoyWGZUcVFqNVA1dDhKU1lLM0ZEcFVWa0xLRURGSU1JM2hEWng0OTZsY3pkcTNCNmswY3Bjd0hzRTNpT2ZwWWlrNE5sQTJzNlplS0lGMjNUNTF1NzZZQV9RX0VhT3UxZDZYV0NGenJjWmotQlR5WGpJQnNWNTJneW5PWFFTU1ZMbkpUdHpvQjNqamJ4QWc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y293" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z293" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA293" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AB293" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC293" t="inlineStr">
+        <is>
+          <t>If There's a Stock Market Crash Ahead, History Highlights the Best Strategy for Investors - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="AD293" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOLUduUjZLVDVGbEVES2xrSENCZmxRUG5Dbmt0V1FlRWgtbmdMb2ZwdjExcjZTVExTMzJvMHd5X2NDUHlMamFZZWJOT0FJZTI0ZUc2eHBwakt5Uzc1UU52NEJVNERGS0E5M3NmMFBUbkFaeDZDNHBrb29tMmhmNUJuWW0wRzhmcG4yZ2t0ZmpoOEFhWUgtMWc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-09-24T23:04:54+00:00</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>30697.5</v>
+      </c>
+      <c r="F294" t="n">
+        <v>30792.5</v>
+      </c>
+      <c r="G294" t="n">
+        <v>30622</v>
+      </c>
+      <c r="H294" t="n">
+        <v>30728.25</v>
+      </c>
+      <c r="I294" t="n">
+        <v>125756</v>
+      </c>
+      <c r="J294" t="n">
+        <v>4</v>
+      </c>
+      <c r="K294" t="n">
+        <v>36</v>
+      </c>
+      <c r="L294" t="n">
+        <v>-0.326</v>
+      </c>
+      <c r="M294" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="N294" t="n">
+        <v>33</v>
+      </c>
+      <c r="O294" t="n">
+        <v>0.219</v>
+      </c>
+      <c r="P294" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="Q294" t="n">
+        <v>-0.763</v>
+      </c>
+      <c r="R294" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S294" t="inlineStr">
+        <is>
+          <t>Stock market today: Dow hits record high, S&amp;P 500 and Nasdaq surge as Big Tech gains power rally - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T294" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPbkNnYmlpUUZ1UFBUdG13a1NLZlhpbXR4cEpMcUdqRkR5aXd1UjVKaEFFQTJyQ0JrQWFHN0I0Zk1wSDVOZ0RaRWM2aXpCb3BDQmE4c0dXaHFLQVhRcXdiZDZnSko3UGd6WlkwNlVncFNJdTVnbHVGaFJBTXltM0ttaUxkZ0ZFa2ptNVN5S3FTbXBPOTc3UHdZVEtVYVFqWXNMazVsZlhaY3hibzViazhyeXBta2RFWHF4Z1pN?oc=5</t>
+        </is>
+      </c>
+      <c r="U294" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="V294" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W294" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="X294" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y294" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z294" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA294" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB294" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC294" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD294" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-09-24T23:04:54+00:00</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>84365.2812</v>
+      </c>
+      <c r="F295" t="n">
+        <v>84488.5</v>
+      </c>
+      <c r="G295" t="n">
+        <v>83945.3594</v>
+      </c>
+      <c r="H295" t="n">
+        <v>84338.52340000001</v>
+      </c>
+      <c r="I295" t="n">
+        <v>2464092160</v>
+      </c>
+      <c r="J295" t="n">
+        <v>4</v>
+      </c>
+      <c r="K295" t="n">
+        <v>38</v>
+      </c>
+      <c r="L295" t="n">
+        <v>-0.016</v>
+      </c>
+      <c r="M295" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="N295" t="n">
+        <v>37</v>
+      </c>
+      <c r="O295" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="P295" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="Q295" t="n">
+        <v>9.138</v>
+      </c>
+      <c r="R295" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S295" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T295" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U295" t="inlineStr">
+        <is>
+          <t>Bitcoin: Surges Above $86,000 With $900M Liquidations - blockchain.news</t>
+        </is>
+      </c>
+      <c r="V295" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPWlJLVVp0NTE2ZWFUZHpuU2d3LXBsMUFZeDVKRy16X2VPZEpUQ19yM09qYkZ0U2o4S2pNZHlFUk56WjloUUtFbzBTdU1leVJXVTVpbExBUkg0T1ZhbllkOHRZUWdINTliV05wMFlRbVNWa0ZReGNMaFVIeFVFamsxNTJxQ00wZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W295" t="inlineStr">
+        <is>
+          <t>'It’s crypto spring': 4 reasons for bitcoin’s surge above $85,000 - Yahoo Finance UK</t>
+        </is>
+      </c>
+      <c r="X295" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNZzU1dUlEakhTNVlkT2pTU0xzeS1fNU9PQkJybHd5U0dmalhUTnZVNHN2UFV6MkdOT05OejhwbkY1MlZocVFvZ2NhMF9iVHVFbFlxcjY1S2ktN3lncGRVaWVYUjdfTUJLQ25QdE1VSTNyYVFMWm1WU3FuM3NFWkx4SlNaa3hGaFE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y295" t="inlineStr">
+        <is>
+          <t>Uniswap drops 11% amid market pullback but holds key $9 support with strong buyer interest. - Pluang</t>
+        </is>
+      </c>
+      <c r="Z295" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNSnpwMUZXVHB4Xzd6eXY1bmN2TXM0VHd4QjhhbjhpejVjMWxhdGI0UjFEUTBBRnZmYU9DMVUyaXREUGJkQnBQVTA0MlIzVXEyNm8xOS1tYndSaUFuV3FtbG9ENkQ0UW1yTnNTbHFJcEZXTnJBSU5rWW1uelZ2Y3N6cWRYd3JrOUpwNWFoYWs3UnFveHRfeFdUcnNR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA295" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="AB295" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AC295" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Prediction: Levels, Tax and Leverage Check - CryptoTicker</t>
+        </is>
+      </c>
+      <c r="AD295" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaXV3ang1VjN6VzlqcVR1empzLS12Q3pnSjdaZUh3SVcyRXdUc0k0c1Y5RGFfTjdPRmRUT0tzaGd4TEZDSjhXelJhOHdpSzdZQ1gxMTBKWjVsdE1ZTHZsRzZodEZpZGR6OEYycGJiYkZUWTBicVVsWms5OXBTcXhrdTRRamhvSVVNY1pLOFBZbw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-25 03:54 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD295"/>
+  <dimension ref="A1:AD301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37145,6 +37145,762 @@
       <c r="AD295" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaXV3ang1VjN6VzlqcVR1empzLS12Q3pnSjdaZUh3SVcyRXdUc0k0c1Y5RGFfTjdPRmRUT0tzaGd4TEZDSjhXelJhOHdpSzdZQ1gxMTBKWjVsdE1ZTHZsRzZodEZpZGR6OEYycGJiYkZUWTBicVVsWms5OXBTcXhrdTRRamhvSVVNY1pLOFBZbw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-09-25T03:51:20+00:00</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>4299.8999</v>
+      </c>
+      <c r="F296" t="n">
+        <v>4331</v>
+      </c>
+      <c r="G296" t="n">
+        <v>4299.2998</v>
+      </c>
+      <c r="H296" t="n">
+        <v>4309.2002</v>
+      </c>
+      <c r="I296" t="n">
+        <v>11223</v>
+      </c>
+      <c r="J296" t="n">
+        <v>4</v>
+      </c>
+      <c r="K296" t="n">
+        <v>39</v>
+      </c>
+      <c r="L296" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M296" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="N296" t="n">
+        <v>40</v>
+      </c>
+      <c r="O296" t="n">
+        <v>-0.054</v>
+      </c>
+      <c r="P296" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="Q296" t="n">
+        <v>-0.411</v>
+      </c>
+      <c r="R296" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S296" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="T296" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="U296" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="V296" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="W296" t="inlineStr">
+        <is>
+          <t>Gold hits record high as investors seek safety - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="X296" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVWt1Y1hBWG5uZFNjRUFtZHlqRUhfZGV6VzAtQ0tBT2VlVDVEZEJ2WHN0YndCcXRzSjNtVnFhUFZZZ2F4RFRxYkdsSF91eDk2MFl5R3JNWk1HREJjSVdhUE1uTTU1N1Z6Y2xfZzZCSDZ4YnhaT1czcWdXeHE3SjJBR2FqUm43Z0paUG5OVEdsWVdYYnZBWVHSAZsBQVVfeXFMTWh6VXlqZGZVbUl3SHVfQ195WFFveEVkLU9TU1RXMTZBdVhodU16UWxLLWVScDNsc2VGMThyT0RTTHB4SVNRYU1KWmRycHhnTEc0NTJ1RWgzdGc2Y0VkanR4QUtlUWFBSnB2cElORUltQk9XdWRLNXhKbU5jRUFqQVd6bG5YbURJakxhNTl3UEk4RzBaQzVJaVdRdFk?oc=5</t>
+        </is>
+      </c>
+      <c r="Y296" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="Z296" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA296" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AB296" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC296" t="inlineStr">
+        <is>
+          <t>Gold breaks $4,320 support, bears target $4,261: Live levels - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD296" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPME13WGVlVjFRRTNPak02V1FBTDZVR25FMHh5Yjc5NWZqZUZfZ3pyUjRxTU5HcWRDS1I3RVRQQ0V0eTZOZmMxMk9aMlc1WGsyd0FPQzU3ZzlMSUp4cVFBSUR6ZkJucl9WSTNlRWRPdHlxY1o1emxISC10OXJib2tlaV80RGpxaW9hR3BydHhPOVNMdFFDSDd1c3RzVGc1MmJpNm1WTDkySUplMkZyZks2bQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-09-25T03:51:20+00:00</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>93.97</v>
+      </c>
+      <c r="F297" t="n">
+        <v>94.06999999999999</v>
+      </c>
+      <c r="G297" t="n">
+        <v>92.72</v>
+      </c>
+      <c r="H297" t="n">
+        <v>93.08</v>
+      </c>
+      <c r="I297" t="n">
+        <v>18394</v>
+      </c>
+      <c r="J297" t="n">
+        <v>4</v>
+      </c>
+      <c r="K297" t="n">
+        <v>40</v>
+      </c>
+      <c r="L297" t="n">
+        <v>-0.038</v>
+      </c>
+      <c r="M297" t="n">
+        <v>-0.195</v>
+      </c>
+      <c r="N297" t="n">
+        <v>40</v>
+      </c>
+      <c r="O297" t="n">
+        <v>0.192</v>
+      </c>
+      <c r="P297" t="n">
+        <v>-0.095</v>
+      </c>
+      <c r="Q297" t="n">
+        <v>3.082</v>
+      </c>
+      <c r="R297" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S297" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T297" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U297" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="V297" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="W297" t="inlineStr">
+        <is>
+          <t>Europe's STOXX 600 rallies on tech, banks strength as oil prices retreat - Reuters</t>
+        </is>
+      </c>
+      <c r="X297" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNYWF0aU9mWUM0TjNtekhpT0I0NTM1RXoydldTZDlzNVM4Q0FnRXFCLTlaLUQxdEZfMS1qeU1XV0lsNHhvc09zMTBUQV9xVFhaakdCU196dW5sQ212UHdLVjVySHo5UWczV0dVS2dnY3d2Q2dTbWRkOWFRZ0g5aTlGaEtnQkFQcno2ZjdfdndQdGdSR1c3MjdEXzNCZlhRM216di1sdllQSl9OT3pkcWRSd3p3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y297" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z297" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA297" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AB297" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC297" t="inlineStr">
+        <is>
+          <t>Brent Oil breaks below $103 support: Live levels - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD297" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPVXk0bHVBcmVMZGtMeTFpVUVfTWFXSE9Qd20tc3JDMHgyVi00ZFpodkdya0ZHLXI4MUdQTDZzS2M2MzVMWnBIMUZicXBYZld5Tl9jTTZsM1hOUHJJdFNqcE1SZVRSU2FFR01iQTJ3UlZTWmdPakZFNkpoQlhjMzVJU0VsY3p0Zndwa005eUQwMldkbFhHckFhMTJxdFBPNEpBYmZXWVBUSjBsbXlWQy1mLWhYbVc2U19Scy1VOE1CQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-09-25T03:51:20+00:00</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>101.297</v>
+      </c>
+      <c r="F298" t="n">
+        <v>101.305</v>
+      </c>
+      <c r="G298" t="n">
+        <v>101.209</v>
+      </c>
+      <c r="H298" t="n">
+        <v>101.284</v>
+      </c>
+      <c r="I298" t="n">
+        <v>0</v>
+      </c>
+      <c r="J298" t="n">
+        <v>4</v>
+      </c>
+      <c r="K298" t="n">
+        <v>39</v>
+      </c>
+      <c r="L298" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="M298" t="n">
+        <v>0.151</v>
+      </c>
+      <c r="N298" t="n">
+        <v>40</v>
+      </c>
+      <c r="O298" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="P298" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="Q298" t="n">
+        <v>4.887</v>
+      </c>
+      <c r="R298" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S298" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T298" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U298" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="V298" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQNkZhLVNRRzlQWGRxQnZUa0tLX0Y4LXF3dXd4NEtpTVlHREtlX0RpRWw4T2tyakdpWFc5U2x5Y3B4Q1ZrclB0MEdwMEFjM0xia1J0UHRaLU41bEM1UFRaQ3lFMU5haXRjcUQtY0w3N2tZUzBSMC1CeXNVendmaWU5OXFFY0wteWk4N2h6dmhXSnhPaVdpalJsYV9VOGMtaGRmc0FNX3FpTnFfNXhnT0ZqMU5qUHRxOFgzRE9HaQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W298" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="X298" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y298" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z298" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA298" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AB298" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+      <c r="AC298" t="inlineStr">
+        <is>
+          <t>US Dollar: Higher yields support currency – MUFG - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD298" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQM0g3eExicnBMSVplbGZrNVl5d215aFlSVlVkbkdvRzhELWVOWkg3dllXMTZwa0Z6SVE3YUxqTFRLRGtROTJxUHEzNVdUNkJFRW9pbVl1MDludEI3RS1xVmVLcXNPbGFRTVJNSHY3TW16QTljbkVwMGlZd0lvZHk3NE9EdDctN2MtVmhDZFNzV25BUQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-09-25T03:51:20+00:00</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E299" t="n">
+        <v>7751.25</v>
+      </c>
+      <c r="F299" t="n">
+        <v>7767.25</v>
+      </c>
+      <c r="G299" t="n">
+        <v>7748.5</v>
+      </c>
+      <c r="H299" t="n">
+        <v>7765</v>
+      </c>
+      <c r="I299" t="n">
+        <v>35211</v>
+      </c>
+      <c r="J299" t="n">
+        <v>4</v>
+      </c>
+      <c r="K299" t="n">
+        <v>38</v>
+      </c>
+      <c r="L299" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M299" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="N299" t="n">
+        <v>40</v>
+      </c>
+      <c r="O299" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="P299" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="Q299" t="n">
+        <v>3.434</v>
+      </c>
+      <c r="R299" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S299" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="T299" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="U299" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 set for strong year-end rally despite r... - Pluang</t>
+        </is>
+      </c>
+      <c r="V299" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTFBJY3VWNDgwOEZQdnZSWlROZjZ3RGY1eXJsR1poYVhoelM0ZlZLZGVoY1FuRWtaa2QtWnVyUjd5YS1INGlZbExIaVpPR0dPb3RfUHNBeU1MdUwwTEhwbzNMeHVDb3c3UE5fakhCUURHQXJWaHpLWjBJT2Z3?oc=5</t>
+        </is>
+      </c>
+      <c r="W299" t="inlineStr">
+        <is>
+          <t>Global benchmarks mostly rise after Wall Street's rally - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="X299" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQQzQ4eHpITXFBQXAzWTczOVJxa2NxcVdTcWhRVXZwYTVCTUJjM1QzZkI5M0szbmRnQnlwOXdaM1BEQ0V3U3pqU1o4MkVFSHJPM180eXJKalNjWUttdDFXVnR3RXRqaGJOQllmMjhHWFpGOUxROUJRbjQ4N1hablgtQ29md2lGcWl4T21WSm9seWVYS0Zp0gGaAUFVX3lxTE1xV1lTRnoyWGZUcVFqNVA1dDhKU1lLM0ZEcFVWa0xLRURGSU1JM2hEWng0OTZsY3pkcTNCNmswY3Bjd0hzRTNpT2ZwWWlrNE5sQTJzNlplS0lGMjNUNTF1NzZZQV9RX0VhT3UxZDZYV0NGenJjWmotQlR5WGpJQnNWNTJneW5PWFFTU1ZMbkpUdHpvQjNqamJ4QWc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y299" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="Z299" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA299" t="inlineStr">
+        <is>
+          <t>FTSE 100 flat again after Wall Street drops - UK Investor Magazine</t>
+        </is>
+      </c>
+      <c r="AB299" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQSnI3anlJTS0tUGJsWjAyc1hYbE40c0dRUklVc2Y5U0QyYU45R1JVT2JyZjE3S3ZHNnVqaU1sWkFacGV0SlJIZ3NyRHBkYUZYaG1Jc0pHeV9oMXlMNmxTSElNNzkxR09rM3dOb2NCODdVTlF4MmIyMVBFX0ZKUHEyVzFSUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC299" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 Falls as 10-Year Treasury Yield Tops 5% After Five-Year PMI High - CryptoRank</t>
+        </is>
+      </c>
+      <c r="AD299" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOWElOdlZ6cHE2dnZ6b3llQzhrRm1NRXgxNnNtRUZzaktQVUpMUWkzemdYTFBhOE9LVXF5STJic0ZjOXNuVElJaUN1QmVMVGNTZm9yaFp6SmQ2R19tMmFsNlJ1aFY3UU1Ec3lYdkI3aWJSb0V3U01zRE4xbl9FVXQ4dHAxLUs5V2lrQmtJZFh4NlNWQTk5U3RFSWxrQmpjNjN6eEZmYmZPTVN2amJR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-09-25T03:51:20+00:00</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>30687</v>
+      </c>
+      <c r="F300" t="n">
+        <v>30814.5</v>
+      </c>
+      <c r="G300" t="n">
+        <v>30679</v>
+      </c>
+      <c r="H300" t="n">
+        <v>30805</v>
+      </c>
+      <c r="I300" t="n">
+        <v>21667</v>
+      </c>
+      <c r="J300" t="n">
+        <v>4</v>
+      </c>
+      <c r="K300" t="n">
+        <v>35</v>
+      </c>
+      <c r="L300" t="n">
+        <v>-0.367</v>
+      </c>
+      <c r="M300" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="N300" t="n">
+        <v>32</v>
+      </c>
+      <c r="O300" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="P300" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="Q300" t="n">
+        <v>-2.189</v>
+      </c>
+      <c r="R300" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S300" t="inlineStr">
+        <is>
+          <t>Stock market today: Dow hits record high, S&amp;P 500 and Nasdaq surge as Big Tech gains power rally - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T300" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPbkNnYmlpUUZ1UFBUdG13a1NLZlhpbXR4cEpMcUdqRkR5aXd1UjVKaEFFQTJyQ0JrQWFHN0I0Zk1wSDVOZ0RaRWM2aXpCb3BDQmE4c0dXaHFLQVhRcXdiZDZnSko3UGd6WlkwNlVncFNJdTVnbHVGaFJBTXltM0ttaUxkZ0ZFa2ptNVN5S3FTbXBPOTc3UHdZVEtVYVFqWXNMazVsZlhaY3hibzViazhyeXBta2RFWHF4Z1pN?oc=5</t>
+        </is>
+      </c>
+      <c r="U300" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="V300" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W300" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="X300" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y300" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z300" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA300" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB300" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC300" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD300" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-09-25T03:51:20+00:00</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>84388.46090000001</v>
+      </c>
+      <c r="F301" t="n">
+        <v>84870.3906</v>
+      </c>
+      <c r="G301" t="n">
+        <v>84052.1875</v>
+      </c>
+      <c r="H301" t="n">
+        <v>84179.11719999999</v>
+      </c>
+      <c r="I301" t="n">
+        <v>1245421568</v>
+      </c>
+      <c r="J301" t="n">
+        <v>4</v>
+      </c>
+      <c r="K301" t="n">
+        <v>37</v>
+      </c>
+      <c r="L301" t="n">
+        <v>-0.074</v>
+      </c>
+      <c r="M301" t="n">
+        <v>0.131</v>
+      </c>
+      <c r="N301" t="n">
+        <v>37</v>
+      </c>
+      <c r="O301" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="P301" t="n">
+        <v>-0.052</v>
+      </c>
+      <c r="Q301" t="n">
+        <v>7.554</v>
+      </c>
+      <c r="R301" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S301" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T301" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U301" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="V301" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="W301" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="X301" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y301" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="Z301" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AA301" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Prediction: What to Check on Levels, Holding Period and Leverage Before the October 28 Rate Decision - CryptoTicker</t>
+        </is>
+      </c>
+      <c r="AB301" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaXV3ang1VjN6VzlqcVR1empzLS12Q3pnSjdaZUh3SVcyRXdUc0k0c1Y5RGFfTjdPRmRUT0tzaGd4TEZDSjhXelJhOHdpSzdZQ1gxMTBKWjVsdE1ZTHZsRzZodEZpZGR6OEYycGJiYkZUWTBicVVsWms5OXBTcXhrdTRRamhvSVVNY1pLOFBZbw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC301" t="inlineStr">
+        <is>
+          <t>Bitcoin holds near $84,500 as crypto liquidatio... - Pluang</t>
+        </is>
+      </c>
+      <c r="AD301" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQb2NnZlF4Zk94UEJad3FYRnk1dFNmcUs2Y0NRMlJnQnc0WFluUmstUmFDOTlSV2xSQ3p3NlJZb0lDdHZpYTgzSWF3c0tKb1NDQVhrX1ZLalhDSTB2UGR1ZHVPdWhqMVB5WFAxazhBc3B3T2tHdGFsb0dubmZrWkN6aUhKWm52d2NITy1zbFhB?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-25 09:30 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD301"/>
+  <dimension ref="A1:AD307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37899,6 +37899,762 @@
         </is>
       </c>
       <c r="AD301" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQb2NnZlF4Zk94UEJad3FYRnk1dFNmcUs2Y0NRMlJnQnc0WFluUmstUmFDOTlSV2xSQ3p3NlJZb0lDdHZpYTgzSWF3c0tKb1NDQVhrX1ZLalhDSTB2UGR1ZHVPdWhqMVB5WFAxazhBc3B3T2tHdGFsb0dubmZrWkN6aUhKWm52d2NITy1zbFhB?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-09-25T09:28:12+00:00</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>4301.1001</v>
+      </c>
+      <c r="F302" t="n">
+        <v>4333.5</v>
+      </c>
+      <c r="G302" t="n">
+        <v>4300.7998</v>
+      </c>
+      <c r="H302" t="n">
+        <v>4327.2002</v>
+      </c>
+      <c r="I302" t="n">
+        <v>14594</v>
+      </c>
+      <c r="J302" t="n">
+        <v>4</v>
+      </c>
+      <c r="K302" t="n">
+        <v>39</v>
+      </c>
+      <c r="L302" t="n">
+        <v>-0.047</v>
+      </c>
+      <c r="M302" t="n">
+        <v>-0.023</v>
+      </c>
+      <c r="N302" t="n">
+        <v>40</v>
+      </c>
+      <c r="O302" t="n">
+        <v>-0.004</v>
+      </c>
+      <c r="P302" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="Q302" t="n">
+        <v>-1.498</v>
+      </c>
+      <c r="R302" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S302" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="T302" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="U302" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="V302" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="W302" t="inlineStr">
+        <is>
+          <t>Gold hits record high as investors seek safety - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="X302" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVWt1Y1hBWG5uZFNjRUFtZHlqRUhfZGV6VzAtQ0tBT2VlVDVEZEJ2WHN0YndCcXRzSjNtVnFhUFZZZ2F4RFRxYkdsSF91eDk2MFl5R3JNWk1HREJjSVdhUE1uTTU1N1Z6Y2xfZzZCSDZ4YnhaT1czcWdXeHE3SjJBR2FqUm43Z0paUG5OVEdsWVdYYnZBWVHSAZsBQVVfeXFMTWh6VXlqZGZVbUl3SHVfQ195WFFveEVkLU9TU1RXMTZBdVhodU16UWxLLWVScDNsc2VGMThyT0RTTHB4SVNRYU1KWmRycHhnTEc0NTJ1RWgzdGc2Y0VkanR4QUtlUWFBSnB2cElORUltQk9XdWRLNXhKbU5jRUFqQVd6bG5YbURJakxhNTl3UEk4RzBaQzVJaVdRdFk?oc=5</t>
+        </is>
+      </c>
+      <c r="Y302" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="Z302" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA302" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AB302" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC302" t="inlineStr">
+        <is>
+          <t>Gold breaks below key MAs, eyes $4,260 support: Live levels - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD302" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPME13WGVlVjFRRTNPak02V1FBTDZVR25FMHh5Yjc5NWZqZUZfZ3pyUjRxTU5HcWRDS1I3RVRQQ0V0eTZOZmMxMk9aMlc1WGsyd0FPQzU3ZzlMSUp4cVFBSUR6ZkJucl9WSTNlRWRPdHlxY1o1emxISC10OXJib2tlaV80RGpxaW9hR3BydHhPOVNMdFFDSDd1c3RzVGc1MmJpNm1WTDkySUplMkZyZks2bQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-09-25T09:28:12+00:00</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="F303" t="n">
+        <v>93.73999999999999</v>
+      </c>
+      <c r="G303" t="n">
+        <v>92.14</v>
+      </c>
+      <c r="H303" t="n">
+        <v>92.87</v>
+      </c>
+      <c r="I303" t="n">
+        <v>33720</v>
+      </c>
+      <c r="J303" t="n">
+        <v>4</v>
+      </c>
+      <c r="K303" t="n">
+        <v>40</v>
+      </c>
+      <c r="L303" t="n">
+        <v>-0.078</v>
+      </c>
+      <c r="M303" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="N303" t="n">
+        <v>40</v>
+      </c>
+      <c r="O303" t="n">
+        <v>0.191</v>
+      </c>
+      <c r="P303" t="n">
+        <v>-0.066</v>
+      </c>
+      <c r="Q303" t="n">
+        <v>2.252</v>
+      </c>
+      <c r="R303" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S303" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T303" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U303" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V303" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W303" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X303" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y303" t="inlineStr">
+        <is>
+          <t>US stocks fall after bond yields jump on higher oil prices and a strong economic report - WSLS</t>
+        </is>
+      </c>
+      <c r="Z303" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOVkVPYmx3cHBQQ0FuM3hLQzY2SXpIZjRjdVRhWmh4NllobGlvVjdFV2E3alNiRF93c2l3ZjhhN2o5UGZJeWJnN1ZXRUE0SUN1bU90VGliQnV0U0tvdGhYaUx3b2d0Mk9iRWNxR3JQWXJ1TzBHdGRaTFFlczNoN0xkN2hSNnVaQU5UYjcwX1JWZ2pIbGV4dlFDeEJBdkxoUV9uSGxvbFMyZ2JPeFVacW5hbFg0N0w5U1BvVlV3cTZPTzFBTEhYU0E?oc=5</t>
+        </is>
+      </c>
+      <c r="AA303" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AB303" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC303" t="inlineStr">
+        <is>
+          <t>nano Crude Oil Fut (Jan 2027) Trade Ideas — COINBASE:NOLF2027 - TradingView</t>
+        </is>
+      </c>
+      <c r="AD303" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNc1BOTkRSU0FuQ1IyRE5kUGJzb2V4Mnl1SW5JYVZVWEV0WGZPT1BQN3BEbHpFNU1SQUhMbUdmM04tZG5fbkVMb2hmeDE1M0lIUUd6cHhSdWU2VExUSEJZc3YzY2pNUXFpTUNlNm5Pd2wydU1lU0Ztb1UzT2ZLaUx2SFhWQ2dJQ25QR0E?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-09-25T09:28:12+00:00</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>101.23</v>
+      </c>
+      <c r="F304" t="n">
+        <v>101.23</v>
+      </c>
+      <c r="G304" t="n">
+        <v>101.058</v>
+      </c>
+      <c r="H304" t="n">
+        <v>101.066</v>
+      </c>
+      <c r="I304" t="n">
+        <v>0</v>
+      </c>
+      <c r="J304" t="n">
+        <v>4</v>
+      </c>
+      <c r="K304" t="n">
+        <v>39</v>
+      </c>
+      <c r="L304" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="M304" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="N304" t="n">
+        <v>39</v>
+      </c>
+      <c r="O304" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="P304" t="n">
+        <v>-0.011</v>
+      </c>
+      <c r="Q304" t="n">
+        <v>1.413</v>
+      </c>
+      <c r="R304" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S304" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T304" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U304" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="V304" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="W304" t="inlineStr">
+        <is>
+          <t>Canadian Dollar Strengthens On Rising Oil Prices Ahead Of Potential US-Iran Talks - InsuranceNewsNet</t>
+        </is>
+      </c>
+      <c r="X304" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOamYyNk9GZ1A3UFZpazcwVnlJZF84eGxxSWpWUDhsWWx6UURTajJKNjMySllWMkNnYnFTRlFuMXpKVEF2dEcyUEVJNjNNbXpPdkhZbmtXQTJnY19DMWQ2RjViYm8wMGJlM2xFZUhDb0pBbUFJeERIYm1JZngyV19pNjBCNWhEZDN5UWdUVlBwM01GTEliVVFSNE5JSzlrQkxQNk1FMDQ5ZUZMLXRIYVVZeDFrWi1mcUZFRHhN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y304" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z304" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA304" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ing think</t>
+        </is>
+      </c>
+      <c r="AB304" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC304" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD304" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-09-25T09:28:12+00:00</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>7770</v>
+      </c>
+      <c r="F305" t="n">
+        <v>7792.5</v>
+      </c>
+      <c r="G305" t="n">
+        <v>7769.75</v>
+      </c>
+      <c r="H305" t="n">
+        <v>7790</v>
+      </c>
+      <c r="I305" t="n">
+        <v>54069</v>
+      </c>
+      <c r="J305" t="n">
+        <v>4</v>
+      </c>
+      <c r="K305" t="n">
+        <v>38</v>
+      </c>
+      <c r="L305" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="M305" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="N305" t="n">
+        <v>40</v>
+      </c>
+      <c r="O305" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="P305" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="Q305" t="n">
+        <v>3.215</v>
+      </c>
+      <c r="R305" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S305" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="T305" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="U305" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 set for strong year-end rally despite r... - Pluang</t>
+        </is>
+      </c>
+      <c r="V305" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTFBJY3VWNDgwOEZQdnZSWlROZjZ3RGY1eXJsR1poYVhoelM0ZlZLZGVoY1FuRWtaa2QtWnVyUjd5YS1INGlZbExIaVpPR0dPb3RfUHNBeU1MdUwwTEhwbzNMeHVDb3c3UE5fakhCUURHQXJWaHpLWjBJT2Z3?oc=5</t>
+        </is>
+      </c>
+      <c r="W305" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 posts 3% summer rally. Some on Wall Street think the gains can continue - CNBC</t>
+        </is>
+      </c>
+      <c r="X305" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOZnpTM0tYdTdvczYtRGQyZklaTWhHZFFBRW5SOU1KamRZWFhSTTFQeFpoYnhIX2huUXUtUUFqRTVMRGxjMW1lN3VveGhhYTF1QUx2Y1VBOHYzWThIRU91Y2FGRUVWSmVlRTBlQ1pyMVFha3JtRmpyVktlcUgyTWRoX1oyUTVOSTI0Z1RvQzQtNFZFM3dYVGFtR3hyRVlCLWRQcDFxVHpuUXkzcnM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y305" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z305" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA305" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AB305" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC305" t="inlineStr">
+        <is>
+          <t>If There's a Stock Market Crash Ahead, History Highlights the Best Strategy for Investors - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="AD305" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOLUduUjZLVDVGbEVES2xrSENCZmxRUG5Dbmt0V1FlRWgtbmdMb2ZwdjExcjZTVExTMzJvMHd5X2NDUHlMamFZZWJOT0FJZTI0ZUc2eHBwakt5Uzc1UU52NEJVNERGS0E5M3NmMFBUbkFaeDZDNHBrb29tMmhmNUJuWW0wRzhmcG4yZ2t0ZmpoOEFhWUgtMWc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-09-25T09:28:12+00:00</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>30850.5</v>
+      </c>
+      <c r="F306" t="n">
+        <v>30963.25</v>
+      </c>
+      <c r="G306" t="n">
+        <v>30838</v>
+      </c>
+      <c r="H306" t="n">
+        <v>30951</v>
+      </c>
+      <c r="I306" t="n">
+        <v>23585</v>
+      </c>
+      <c r="J306" t="n">
+        <v>4</v>
+      </c>
+      <c r="K306" t="n">
+        <v>34</v>
+      </c>
+      <c r="L306" t="n">
+        <v>-0.294</v>
+      </c>
+      <c r="M306" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="N306" t="n">
+        <v>33</v>
+      </c>
+      <c r="O306" t="n">
+        <v>0.231</v>
+      </c>
+      <c r="P306" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="Q306" t="n">
+        <v>-0.681</v>
+      </c>
+      <c r="R306" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S306" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="T306" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U306" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="V306" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="W306" t="inlineStr">
+        <is>
+          <t>Nasdaq Hits Record High Ahead of Trump-Xi Meeting - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X306" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxQT0xKczFIMXh4aVRzSFVnLVNIUERhLTFWZ2lqVGt1RXpyemliZ3JFczFRQ1FLTUNLa0RpeGgxdjFCdW5tNUc0cDJNazVqWUszSXA3eDNveXQ4Q0lMN1JxRWJob2JETklBUzctR0xNRWpBOXFaekp4dlVvODlDQ0xoUE1janlVRTFyNDJIcHFMdUZLbm13YnRnZC13?oc=5</t>
+        </is>
+      </c>
+      <c r="Y306" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z306" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA306" t="inlineStr">
+        <is>
+          <t>Hong Kong stocks fall as tech shares slide, Trump-Xi summit in focus - TradingView</t>
+        </is>
+      </c>
+      <c r="AB306" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPRDdiTzljR3dfdGUwdGFCaHB1TGRJakd6UDdIMURaTkJxRGZCQW4zZlhfSHhaYXY0SHF5ZnRiX2QzaXNCNjRVTm84Qmh2Sml2QXJub3hUN05tOVA2LVBLUEhLNGg1SkpSSGRITUl3QUMwQ29VMDFjaGJBdk9EZndiZWplODQ0ajNkME44Z0VCbnVSX0JZb1JhNi1MODRsXzJOb202WnRRV1NDaFBNcnZCQUVLVXFCZWgtODlEeGFUX3dnVjdIOUVXdEpVX2p5blI5M1A4?oc=5</t>
+        </is>
+      </c>
+      <c r="AC306" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AD306" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-09-25T09:28:12+00:00</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>84178.2812</v>
+      </c>
+      <c r="F307" t="n">
+        <v>84832.7031</v>
+      </c>
+      <c r="G307" t="n">
+        <v>83751</v>
+      </c>
+      <c r="H307" t="n">
+        <v>84771.1562</v>
+      </c>
+      <c r="I307" t="n">
+        <v>1547022336</v>
+      </c>
+      <c r="J307" t="n">
+        <v>4</v>
+      </c>
+      <c r="K307" t="n">
+        <v>37</v>
+      </c>
+      <c r="L307" t="n">
+        <v>-0.026</v>
+      </c>
+      <c r="M307" t="n">
+        <v>0.141</v>
+      </c>
+      <c r="N307" t="n">
+        <v>36</v>
+      </c>
+      <c r="O307" t="n">
+        <v>0.524</v>
+      </c>
+      <c r="P307" t="n">
+        <v>-0.065</v>
+      </c>
+      <c r="Q307" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="R307" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S307" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T307" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U307" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="V307" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="W307" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="X307" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y307" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="Z307" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AA307" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Prediction: What to Check on Levels, Holding Period and Leverage Before the October 28 Rate Decision - CryptoTicker</t>
+        </is>
+      </c>
+      <c r="AB307" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaXV3ang1VjN6VzlqcVR1empzLS12Q3pnSjdaZUh3SVcyRXdUc0k0c1Y5RGFfTjdPRmRUT0tzaGd4TEZDSjhXelJhOHdpSzdZQ1gxMTBKWjVsdE1ZTHZsRzZodEZpZGR6OEYycGJiYkZUWTBicVVsWms5OXBTcXhrdTRRamhvSVVNY1pLOFBZbw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC307" t="inlineStr">
+        <is>
+          <t>Bitcoin holds near $84,500 as crypto liquidatio... - Pluang</t>
+        </is>
+      </c>
+      <c r="AD307" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQb2NnZlF4Zk94UEJad3FYRnk1dFNmcUs2Y0NRMlJnQnc0WFluUmstUmFDOTlSV2xSQ3p3NlJZb0lDdHZpYTgzSWF3c0tKb1NDQVhrX1ZLalhDSTB2UGR1ZHVPdWhqMVB5WFAxazhBc3B3T2tHdGFsb0dubmZrWkN6aUhKWm52d2NITy1zbFhB?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-25 16:47 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD307"/>
+  <dimension ref="A1:AD313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38657,6 +38657,762 @@
       <c r="AD307" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQb2NnZlF4Zk94UEJad3FYRnk1dFNmcUs2Y0NRMlJnQnc0WFluUmstUmFDOTlSV2xSQ3p3NlJZb0lDdHZpYTgzSWF3c0tKb1NDQVhrX1ZLalhDSTB2UGR1ZHVPdWhqMVB5WFAxazhBc3B3T2tHdGFsb0dubmZrWkN6aUhKWm52d2NITy1zbFhB?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-09-25T16:45:43+00:00</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>4333.8999</v>
+      </c>
+      <c r="F308" t="n">
+        <v>4336</v>
+      </c>
+      <c r="G308" t="n">
+        <v>4289.2002</v>
+      </c>
+      <c r="H308" t="n">
+        <v>4320.7998</v>
+      </c>
+      <c r="I308" t="n">
+        <v>51482</v>
+      </c>
+      <c r="J308" t="n">
+        <v>4</v>
+      </c>
+      <c r="K308" t="n">
+        <v>39</v>
+      </c>
+      <c r="L308" t="n">
+        <v>-0.139</v>
+      </c>
+      <c r="M308" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="N308" t="n">
+        <v>40</v>
+      </c>
+      <c r="O308" t="n">
+        <v>-0.041</v>
+      </c>
+      <c r="P308" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="Q308" t="n">
+        <v>-4.032</v>
+      </c>
+      <c r="R308" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S308" t="inlineStr">
+        <is>
+          <t>Lundin Gold Hits Record Grade at Bonza Sur With 204 g/t Gold Over 3 Metres Intercept - the deep dive</t>
+        </is>
+      </c>
+      <c r="T308" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNaDdPLWtTOVlMN0c3OWFFWmF1dUZfT28xLWducTQyQVo5XzRUZzU5YWxUZ1JlZzZqcHRtcG5FUENMZE9LN1ZEQXdpTDBMa3c2Ry1aakpaMjBtTlV6bTNDenB4d2d1OEltQmxadjVsTHFWY0J5alI2Sko2YVdfa1VHZDd3bGVtdUlOaXVaZU0xcFo0UHBjNXZTX2dKS1dtX1J5d2JBX2NxSW9TMS1P?oc=5</t>
+        </is>
+      </c>
+      <c r="U308" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="V308" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="W308" t="inlineStr">
+        <is>
+          <t>Gold hits record high as investors seek safety - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="X308" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVWt1Y1hBWG5uZFNjRUFtZHlqRUhfZGV6VzAtQ0tBT2VlVDVEZEJ2WHN0YndCcXRzSjNtVnFhUFZZZ2F4RFRxYkdsSF91eDk2MFl5R3JNWk1HREJjSVdhUE1uTTU1N1Z6Y2xfZzZCSDZ4YnhaT1czcWdXeHE3SjJBR2FqUm43Z0paUG5OVEdsWVdYYnZBWVHSAZsBQVVfeXFMTWh6VXlqZGZVbUl3SHVfQ195WFFveEVkLU9TU1RXMTZBdVhodU16UWxLLWVScDNsc2VGMThyT0RTTHB4SVNRYU1KWmRycHhnTEc0NTJ1RWgzdGc2Y0VkanR4QUtlUWFBSnB2cElORUltQk9XdWRLNXhKbU5jRUFqQVd6bG5YbURJakxhNTl3UEk4RzBaQzVJaVdRdFk?oc=5</t>
+        </is>
+      </c>
+      <c r="Y308" t="inlineStr">
+        <is>
+          <t>Kremlin begins record-breaking gold sell-off from central bank reserves - The New Voice of Ukraine</t>
+        </is>
+      </c>
+      <c r="Z308" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOMExQRGhrZkRfVzVScmRCNVNJRE5UY2lvMEtSempTckduN2xwU20ycFd0TEZZSDJZZUdQYmdOa2pKcFpqWEQ3TkRsNEZ4Z1M3REtJTUo0S1VrSUVueGFaMm41R0R1VTNsRDNFcHQtNXFQcjN0X0Q4YkVzUjljUTdHUEpsbHA1U3lkdW9IbF82dEtxdC03NUFqMUFkY3lBYzjSAZgBQVVfeXFMT1ZFLW1wbm11dmppazdlbkVvX1Y1Qm1pclI0NTFRQmM5a29yci0wa3l2OWhjMXhBTWI2TXdSbXZMczhMaHdTR0J0UTZLa2loNGxTUG5HTlFhVjFZNzZ6clFQSXVaYTY2MnByQzVZMENFdHEyazBrOTV0cU9ncFh3ZEl5amlrYXZEb19iRlZ3Yl84QTAxXzNMTzE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA308" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB308" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC308" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AD308" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-09-25T16:45:43+00:00</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E309" t="n">
+        <v>92.53</v>
+      </c>
+      <c r="F309" t="n">
+        <v>94.23</v>
+      </c>
+      <c r="G309" t="n">
+        <v>91.51000000000001</v>
+      </c>
+      <c r="H309" t="n">
+        <v>92.23999999999999</v>
+      </c>
+      <c r="I309" t="n">
+        <v>134598</v>
+      </c>
+      <c r="J309" t="n">
+        <v>4</v>
+      </c>
+      <c r="K309" t="n">
+        <v>40</v>
+      </c>
+      <c r="L309" t="n">
+        <v>-0.039</v>
+      </c>
+      <c r="M309" t="n">
+        <v>-0.134</v>
+      </c>
+      <c r="N309" t="n">
+        <v>40</v>
+      </c>
+      <c r="O309" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="P309" t="n">
+        <v>-0.003</v>
+      </c>
+      <c r="Q309" t="n">
+        <v>2.723</v>
+      </c>
+      <c r="R309" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S309" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T309" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U309" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V309" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W309" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X309" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y309" t="inlineStr">
+        <is>
+          <t>A reprieve from rising oil prices helps steady the US stock and bond markets - Union-Bulletin</t>
+        </is>
+      </c>
+      <c r="Z309" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNbkhMTHRncTNzVXpuSElYX3Q5cU5MMHFPYWt6LVBFVkV5TlgwRzU2WFc4NXlNQkRtVUgxRVdNekdnYTNlTm9PUUc4czh4Q2NqU0VySWhfM2NCQTdveTFtLWZFSFp5WmpMVXVjWWpDNXpBeW9uaFBYUXVOYmREcGpJUFhrNjhSSG5BdHpIaTJ1OXJfcVI5NWhQOE94LVR4RnpSVFpONWE2ZkRuNGxaVWFkUWpmSVZMQVVYWTRqdVBzOFVUT1FfMGpXb0s1blNMZEI2QUcxT3dKeXRVb3VscjhaUVpFZHJQMXlqTnU2TEgzV3ZjUzRQNG5KTG5KOW9mQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA309" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AB309" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC309" t="inlineStr">
+        <is>
+          <t>nano Crude Oil Fut (Jan 2027) Trade Ideas — COINBASE:NOLF2027 - TradingView</t>
+        </is>
+      </c>
+      <c r="AD309" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNc1BOTkRSU0FuQ1IyRE5kUGJzb2V4Mnl1SW5JYVZVWEV0WGZPT1BQN3BEbHpFNU1SQUhMbUdmM04tZG5fbkVMb2hmeDE1M0lIUUd6cHhSdWU2VExUSEJZc3YzY2pNUXFpTUNlNm5Pd2wydU1lU0Ztb1UzT2ZLaUx2SFhWQ2dJQ25QR0E?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-09-25T16:45:43+00:00</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>100.982</v>
+      </c>
+      <c r="F310" t="n">
+        <v>101.099</v>
+      </c>
+      <c r="G310" t="n">
+        <v>100.872</v>
+      </c>
+      <c r="H310" t="n">
+        <v>101.018</v>
+      </c>
+      <c r="I310" t="n">
+        <v>0</v>
+      </c>
+      <c r="J310" t="n">
+        <v>4</v>
+      </c>
+      <c r="K310" t="n">
+        <v>39</v>
+      </c>
+      <c r="L310" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="M310" t="n">
+        <v>0.156</v>
+      </c>
+      <c r="N310" t="n">
+        <v>40</v>
+      </c>
+      <c r="O310" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="P310" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="Q310" t="n">
+        <v>2.316</v>
+      </c>
+      <c r="R310" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S310" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T310" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U310" t="inlineStr">
+        <is>
+          <t>U.S. dollar strengthens as traders see resilient US economy - Forex Factory</t>
+        </is>
+      </c>
+      <c r="V310" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPUzNuYUY3Y0xYRjV5UHMzckJMZEs1WGRncEwtTVdXbjZlSEJhb19uWmF0WFk0WEVGZld5TjdUZ1l5QjhhS05TbHJUX01YNDNIVFRJVmlHMFJvQjV4MWhkZkVlcE1EMnVGTERUcVRULThyaldDbjJmN1Z2RmxMeTVvenZsVklyLURIdWduOGpBOF9ibnlmVEZjckJDS21GbmljbTVvckJIZEF1YjTSAZoBQVVfeXFMUEYxZDNRZEJUMGgzNzcxb2ZWTS1JUkVlSlFTSnNiTmdyUkYxNXZWemFaNFNJam1PR1RWOGFyVmd3NG9kcUxkeklXS0FyYTdwaDZXa1hPLWtoSTMwUTVWcjQxcmVVdEk1cldRYjB2bnlEWWFLOF9XRlFOZVNXNEQzQ09jYWFxbHNPRVFNTXd3cWtDcFRBSjM3MzZhZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W310" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="X310" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y310" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z310" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA310" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB310" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC310" t="inlineStr">
+        <is>
+          <t>Canadian financial close: Canadian dollar weakens - producer.com</t>
+        </is>
+      </c>
+      <c r="AD310" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPa2d4UUItci1PNGZTWXRocTJTNzZOYWxiS1hWTWdzUGFzZFZDb3BRMVR3YXpRekluS3FEMEE3V1lWWGgtZ20zVG5KRlR0dFY1RU1NaGRYWkFEckdhWHVEbmx4cm5iOG93M1lGWi1xZDNpWGx6VWkwV0xQTTNCaTBHeHFpVVR0Y3k2WHhLMmZvUENYdw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-09-25T16:45:43+00:00</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>7785</v>
+      </c>
+      <c r="F311" t="n">
+        <v>7811</v>
+      </c>
+      <c r="G311" t="n">
+        <v>7752.75</v>
+      </c>
+      <c r="H311" t="n">
+        <v>7803.5</v>
+      </c>
+      <c r="I311" t="n">
+        <v>836980</v>
+      </c>
+      <c r="J311" t="n">
+        <v>4</v>
+      </c>
+      <c r="K311" t="n">
+        <v>40</v>
+      </c>
+      <c r="L311" t="n">
+        <v>-0.191</v>
+      </c>
+      <c r="M311" t="n">
+        <v>0.148</v>
+      </c>
+      <c r="N311" t="n">
+        <v>40</v>
+      </c>
+      <c r="O311" t="n">
+        <v>0.173</v>
+      </c>
+      <c r="P311" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="Q311" t="n">
+        <v>-0.348</v>
+      </c>
+      <c r="R311" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S311" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T311" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U311" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V311" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W311" t="inlineStr">
+        <is>
+          <t>Litecoin, Cardano, Stellar, and Chainlink All Outperformed Bitcoin This Week. Which Rally Has the Strongest Support? - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="X311" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxOampGT2pHS01lUzJHdmZhbi1XUjRKaEZWNW1xU0xmS0VkcE94THBjRWNWVENsdF9fR3BCb01hLU8weFMzdVJGaTEybzk0bDZ0Z1ZWbWFNUjIyNkxsb1lPbEVDelgwcmh5SmdROVEzZHo0OXBUVGM5dFBxZ1BYclQyZHdlTVVzV1gzWEI5alp1WG1CNFZJdWVXbVJfRnBvYVppM1B3aWZJMGJJMTg5WFlaMG5mQWNSbzFyRGJfdS1DN3pxTmtpREcwVHBpWENjMC1zbklHX2tCanowTmNtWlNfVmhrMDYyREZkZHE1d3NLcng2LUljXzFjbDV1MUJTQ2s?oc=5</t>
+        </is>
+      </c>
+      <c r="Y311" t="inlineStr">
+        <is>
+          <t>If There's a Stock Market Crash Ahead, History Highlights the Best Strategy for Investors - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="Z311" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOQjlSRnVrTllBQ18wak5KWFByYjA4V24ydVJiNnNuV0dQQ1VKVDNnZVp0YUtZdzlhOTNfekZjUW1BckF6UUZFbGZ6cDNwbkVERzZGSlpSa1pueHdxZTdMeVNXWV9BMDh5Z24yU2JEd09IZllEcU1oN0RidTZicDltdy1YRkNzd2dNa2JpZ3FfV1Rha1ZrTVc3NDNxZHQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA311" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB311" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC311" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AD311" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-09-25T16:45:43+00:00</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E312" t="n">
+        <v>30878</v>
+      </c>
+      <c r="F312" t="n">
+        <v>30951.5</v>
+      </c>
+      <c r="G312" t="n">
+        <v>30684</v>
+      </c>
+      <c r="H312" t="n">
+        <v>30909.25</v>
+      </c>
+      <c r="I312" t="n">
+        <v>310579</v>
+      </c>
+      <c r="J312" t="n">
+        <v>4</v>
+      </c>
+      <c r="K312" t="n">
+        <v>35</v>
+      </c>
+      <c r="L312" t="n">
+        <v>-0.196</v>
+      </c>
+      <c r="M312" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="N312" t="n">
+        <v>36</v>
+      </c>
+      <c r="O312" t="n">
+        <v>0.306</v>
+      </c>
+      <c r="P312" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="Q312" t="n">
+        <v>1.586</v>
+      </c>
+      <c r="R312" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S312" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="T312" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="U312" t="inlineStr">
+        <is>
+          <t>Nasdaq Hits Record High Ahead of Trump-Xi Meeting - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="V312" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxQT0xKczFIMXh4aVRzSFVnLVNIUERhLTFWZ2lqVGt1RXpyemliZ3JFczFRQ1FLTUNLa0RpeGgxdjFCdW5tNUc0cDJNazVqWUszSXA3eDNveXQ4Q0lMN1JxRWJob2JETklBUzctR0xNRWpBOXFaekp4dlVvODlDQ0xoUE1janlVRTFyNDJIcHFMdUZLbm13YnRnZC13?oc=5</t>
+        </is>
+      </c>
+      <c r="W312" t="inlineStr">
+        <is>
+          <t>Stock Market Split As Nasdaq Hits High, Dow Jones Slides Amid Surging Treasury Yields: Weekly Review - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="X312" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPMEdvdk5ZTHduYS1XYjZlUExBRFFIT0Z2aWVGVW9zdmNmdF9TUXkzQnJRcmxNbnd1U3BkbWpueU9lSk1XWFFFOXVGZl9XRHE0eHRjSW5OMlhqdHZ0WUh0RXd5UlZRQVNZa2o2Z3FuZHpMTnQ3M1NuQVpqczFvYVBhalF4VnFpNGNoSERFVkg5cHZTajJyenA1OHRlcFRrYnVqejcwdk1qby03WmVE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y312" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z312" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA312" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB312" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC312" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD312" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-09-25T16:45:43+00:00</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E313" t="n">
+        <v>84437.77340000001</v>
+      </c>
+      <c r="F313" t="n">
+        <v>84556.1875</v>
+      </c>
+      <c r="G313" t="n">
+        <v>83155.99219999999</v>
+      </c>
+      <c r="H313" t="n">
+        <v>83793.5625</v>
+      </c>
+      <c r="I313" t="n">
+        <v>9038090240</v>
+      </c>
+      <c r="J313" t="n">
+        <v>4</v>
+      </c>
+      <c r="K313" t="n">
+        <v>37</v>
+      </c>
+      <c r="L313" t="n">
+        <v>-0.106</v>
+      </c>
+      <c r="M313" t="n">
+        <v>0.148</v>
+      </c>
+      <c r="N313" t="n">
+        <v>35</v>
+      </c>
+      <c r="O313" t="n">
+        <v>0.481</v>
+      </c>
+      <c r="P313" t="n">
+        <v>-0.059</v>
+      </c>
+      <c r="Q313" t="n">
+        <v>7.453</v>
+      </c>
+      <c r="R313" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S313" t="inlineStr">
+        <is>
+          <t>XRP, Solana Lead Crypto Majors With Bitcoin Stuck Below $85K, BTC ETF Inflows Turning Positive For 2026 - TradingView</t>
+        </is>
+      </c>
+      <c r="T313" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOSTZPSHFoWDhhaEFHTFcxQ0RjcHNmZVZxNXY5VUxvRjFMVUpUY3hibVdTNHBWRUxRSU9ibDdjZkVCSmkwQmJpWjZ1eGh1WmpBRlBDMlVSbkZ3aWFUOUhRanQxT05KdVhsenRJVkNURWI1U09ILWF4dVhiZWRocTE3bXJnVVBaZlBub2ZmYkdLRVdKLWFFcGoxZnVYVXpMY2kyTVduNXA3bXN0SWowMEljOEtJTHA5dnFfT3F0OFF6LWYxaTYwTGpNZTc5YW15YndqRnROUnhCRjBhLWxiOVVvRmlpeXZ1NWxRNldRMU5PaVd3Yk0?oc=5</t>
+        </is>
+      </c>
+      <c r="U313" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="V313" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="W313" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X313" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y313" t="inlineStr">
+        <is>
+          <t>Crypto Prices Today: Bitcoin Slides to $84,000 While Altcoins Rally Hard - CryptoTicker</t>
+        </is>
+      </c>
+      <c r="Z313" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNaWVhbE9DbTFqTjFKVzEwVFJIZzdZZVlTakpMOHJmdnY5SHUxWHdFeVhRd3NjUW5seWw4cmlqOGpqV1RTMFhaQlpkT3A3SGV0YTloTWFHNzNZT2RqVGZqaDlLMk1tbW15UzRZVDlwbURXMGhJM3dXV1laRUVfaWdXQw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA313" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="AB313" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AC313" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Prediction: What to Check on Levels, Holding Period and Leverage Before the October 28 Rate Decision - CryptoTicker</t>
+        </is>
+      </c>
+      <c r="AD313" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaXV3ang1VjN6VzlqcVR1empzLS12Q3pnSjdaZUh3SVcyRXdUc0k0c1Y5RGFfTjdPRmRUT0tzaGd4TEZDSjhXelJhOHdpSzdZQ1gxMTBKWjVsdE1ZTHZsRzZodEZpZGR6OEYycGJiYkZUWTBicVVsWms5OXBTcXhrdTRRamhvSVVNY1pLOFBZbw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-25 23:11 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD313"/>
+  <dimension ref="A1:AD319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39411,6 +39411,762 @@
         </is>
       </c>
       <c r="AD313" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaXV3ang1VjN6VzlqcVR1empzLS12Q3pnSjdaZUh3SVcyRXdUc0k0c1Y5RGFfTjdPRmRUT0tzaGd4TEZDSjhXelJhOHdpSzdZQ1gxMTBKWjVsdE1ZTHZsRzZodEZpZGR6OEYycGJiYkZUWTBicVVsWms5OXBTcXhrdTRRamhvSVVNY1pLOFBZbw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:09:40+00:00</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E314" t="n">
+        <v>4321.6001</v>
+      </c>
+      <c r="F314" t="n">
+        <v>4332.3999</v>
+      </c>
+      <c r="G314" t="n">
+        <v>4314.5</v>
+      </c>
+      <c r="H314" t="n">
+        <v>4320.5</v>
+      </c>
+      <c r="I314" t="n">
+        <v>17239</v>
+      </c>
+      <c r="J314" t="n">
+        <v>4</v>
+      </c>
+      <c r="K314" t="n">
+        <v>40</v>
+      </c>
+      <c r="L314" t="n">
+        <v>-0.187</v>
+      </c>
+      <c r="M314" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="N314" t="n">
+        <v>40</v>
+      </c>
+      <c r="O314" t="n">
+        <v>-0.027</v>
+      </c>
+      <c r="P314" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="Q314" t="n">
+        <v>-4.269</v>
+      </c>
+      <c r="R314" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S314" t="inlineStr">
+        <is>
+          <t>Lundin Gold Hits Record Grade at Bonza Sur With 204 g/t Gold Over 3 Metres Intercept - the deep dive</t>
+        </is>
+      </c>
+      <c r="T314" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNaDdPLWtTOVlMN0c3OWFFWmF1dUZfT28xLWducTQyQVo5XzRUZzU5YWxUZ1JlZzZqcHRtcG5FUENMZE9LN1ZEQXdpTDBMa3c2Ry1aakpaMjBtTlV6bTNDenB4d2d1OEltQmxadjVsTHFWY0J5alI2Sko2YVdfa1VHZDd3bGVtdUlOaXVaZU0xcFo0UHBjNXZTX2dKS1dtX1J5d2JBX2NxSW9TMS1P?oc=5</t>
+        </is>
+      </c>
+      <c r="U314" t="inlineStr">
+        <is>
+          <t>Gold price will hit $4,900/oz in 2026 on strong sovereign demand as China buys 75% more than reported in July – Goldman Sachs - Kitco</t>
+        </is>
+      </c>
+      <c r="V314" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOdmIweWNUQkhQS0N4SVhSTjEzWjBlUU9IX2Vxa2c4cGVvM1RQN3BqRkVRWFBYSHAzdFNqcmdYSFhVWUViVWV5Wmp6cHhERHVOSHNnbTcxYnlaaFZ1Y3lsOWpWRDdxbUR4ZDNlRVlQWEZERkhuLWZaT0VxRkhEamE3QmRGMDNvX3Z1VlVPNnczTFBWbEhlbEZqMkZJYTRsM2FKSXpkWUJIbkVUcGtwaXdwRUUxbDBHTFJ1ZmpjZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W314" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X314" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y314" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="Z314" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA314" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AB314" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC314" t="inlineStr">
+        <is>
+          <t>Gold breaks below key MAs, eyes $4,260 support: Live levels - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD314" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPME13WGVlVjFRRTNPak02V1FBTDZVR25FMHh5Yjc5NWZqZUZfZ3pyUjRxTU5HcWRDS1I3RVRQQ0V0eTZOZmMxMk9aMlc1WGsyd0FPQzU3ZzlMSUp4cVFBSUR6ZkJucl9WSTNlRWRPdHlxY1o1emxISC10OXJib2tlaV80RGpxaW9hR3BydHhPOVNMdFFDSDd1c3RzVGc1MmJpNm1WTDkySUplMkZyZks2bQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:09:40+00:00</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E315" t="n">
+        <v>92.23999999999999</v>
+      </c>
+      <c r="F315" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="G315" t="n">
+        <v>91.81999999999999</v>
+      </c>
+      <c r="H315" t="n">
+        <v>92.44</v>
+      </c>
+      <c r="I315" t="n">
+        <v>72759</v>
+      </c>
+      <c r="J315" t="n">
+        <v>4</v>
+      </c>
+      <c r="K315" t="n">
+        <v>40</v>
+      </c>
+      <c r="L315" t="n">
+        <v>-0</v>
+      </c>
+      <c r="M315" t="n">
+        <v>-0.163</v>
+      </c>
+      <c r="N315" t="n">
+        <v>40</v>
+      </c>
+      <c r="O315" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="P315" t="n">
+        <v>-0.125</v>
+      </c>
+      <c r="Q315" t="n">
+        <v>3.547</v>
+      </c>
+      <c r="R315" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S315" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T315" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U315" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V315" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W315" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="X315" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y315" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z315" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA315" t="inlineStr">
+        <is>
+          <t>nano Crude Oil Fut (Jan 2027) Trade Ideas — COINBASE:NOLF2027 - TradingView</t>
+        </is>
+      </c>
+      <c r="AB315" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNc1BOTkRSU0FuQ1IyRE5kUGJzb2V4Mnl1SW5JYVZVWEV0WGZPT1BQN3BEbHpFNU1SQUhMbUdmM04tZG5fbkVMb2hmeDE1M0lIUUd6cHhSdWU2VExUSEJZc3YzY2pNUXFpTUNlNm5Pd2wydU1lU0Ztb1UzT2ZLaUx2SFhWQ2dJQ25QR0E?oc=5</t>
+        </is>
+      </c>
+      <c r="AC315" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="AD315" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:09:40+00:00</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E316" t="n">
+        <v>101.022</v>
+      </c>
+      <c r="F316" t="n">
+        <v>101.077</v>
+      </c>
+      <c r="G316" t="n">
+        <v>100.954</v>
+      </c>
+      <c r="H316" t="n">
+        <v>101.035</v>
+      </c>
+      <c r="I316" t="n">
+        <v>0</v>
+      </c>
+      <c r="J316" t="n">
+        <v>4</v>
+      </c>
+      <c r="K316" t="n">
+        <v>39</v>
+      </c>
+      <c r="L316" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="M316" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="N316" t="n">
+        <v>40</v>
+      </c>
+      <c r="O316" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="P316" t="n">
+        <v>-0.004</v>
+      </c>
+      <c r="Q316" t="n">
+        <v>2.884</v>
+      </c>
+      <c r="R316" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S316" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T316" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U316" t="inlineStr">
+        <is>
+          <t>U.S. dollar strengthens as traders see resilient US economy - Forex Factory</t>
+        </is>
+      </c>
+      <c r="V316" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPUzNuYUY3Y0xYRjV5UHMzckJMZEs1WGRncEwtTVdXbjZlSEJhb19uWmF0WFk0WEVGZld5TjdUZ1l5QjhhS05TbHJUX01YNDNIVFRJVmlHMFJvQjV4MWhkZkVlcE1EMnVGTERUcVRULThyaldDbjJmN1Z2RmxMeTVvenZsVklyLURIdWduOGpBOF9ibnlmVEZjckJDS21GbmljbTVvckJIZEF1YjTSAZoBQVVfeXFMUEYxZDNRZEJUMGgzNzcxb2ZWTS1JUkVlSlFTSnNiTmdyUkYxNXZWemFaNFNJam1PR1RWOGFyVmd3NG9kcUxkeklXS0FyYTdwaDZXa1hPLWtoSTMwUTVWcjQxcmVVdEk1cldRYjB2bnlEWWFLOF9XRlFOZVNXNEQzQ09jYWFxbHNPRVFNTXd3cWtDcFRBSjM3MzZhZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W316" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="X316" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="Y316" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z316" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA316" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB316" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC316" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD316" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:09:40+00:00</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E317" t="n">
+        <v>7795.25</v>
+      </c>
+      <c r="F317" t="n">
+        <v>7814.75</v>
+      </c>
+      <c r="G317" t="n">
+        <v>7793.25</v>
+      </c>
+      <c r="H317" t="n">
+        <v>7805.75</v>
+      </c>
+      <c r="I317" t="n">
+        <v>473791</v>
+      </c>
+      <c r="J317" t="n">
+        <v>4</v>
+      </c>
+      <c r="K317" t="n">
+        <v>40</v>
+      </c>
+      <c r="L317" t="n">
+        <v>-0.177</v>
+      </c>
+      <c r="M317" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="N317" t="n">
+        <v>40</v>
+      </c>
+      <c r="O317" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="P317" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="Q317" t="n">
+        <v>-1.506</v>
+      </c>
+      <c r="R317" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S317" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T317" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U317" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V317" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W317" t="inlineStr">
+        <is>
+          <t>Stock market today: Dow hits record high, S&amp;P 500 and Nasdaq surge as Big Tech gains power rally - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X317" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPbkNnYmlpUUZ1UFBUdG13a1NLZlhpbXR4cEpMcUdqRkR5aXd1UjVKaEFFQTJyQ0JrQWFHN0I0Zk1wSDVOZ0RaRWM2aXpCb3BDQmE4c0dXaHFLQVhRcXdiZDZnSko3UGd6WlkwNlVncFNJdTVnbHVGaFJBTXltM0ttaUxkZ0ZFa2ptNVN5S3FTbXBPOTc3UHdZVEtVYVFqWXNMazVsZlhaY3hibzViazhyeXBta2RFWHF4Z1pN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y317" t="inlineStr">
+        <is>
+          <t>If There's a Stock Market Crash Ahead, History Highlights the Best Strategy for Investors - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="Z317" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOQjlSRnVrTllBQ18wak5KWFByYjA4V24ydVJiNnNuV0dQQ1VKVDNnZVp0YUtZdzlhOTNfekZjUW1BckF6UUZFbGZ6cDNwbkVERzZGSlpSa1pueHdxZTdMeVNXWV9BMDh5Z24yU2JEd09IZllEcU1oN0RidTZicDltdy1YRkNzd2dNa2JpZ3FfV1Rha1ZrTVc3NDNxZHQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA317" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB317" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC317" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AD317" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:09:40+00:00</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E318" t="n">
+        <v>30912</v>
+      </c>
+      <c r="F318" t="n">
+        <v>30935</v>
+      </c>
+      <c r="G318" t="n">
+        <v>30845</v>
+      </c>
+      <c r="H318" t="n">
+        <v>30921.75</v>
+      </c>
+      <c r="I318" t="n">
+        <v>83633</v>
+      </c>
+      <c r="J318" t="n">
+        <v>4</v>
+      </c>
+      <c r="K318" t="n">
+        <v>35</v>
+      </c>
+      <c r="L318" t="n">
+        <v>-0.073</v>
+      </c>
+      <c r="M318" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="N318" t="n">
+        <v>35</v>
+      </c>
+      <c r="O318" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="P318" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="Q318" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="R318" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S318" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally (AMD:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T318" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNRTNUV0JnS3haREZESHpOTVREazZUWkNwUE43OEQxMFJYajZnU3JhaWFKOEt1MVEtLTJYdlg5YnVUUnE3WnFnN0FoRDRJUFZlVEpNN2pCaWFpSEQ5NmlIM2hoQ2VDcHNHRHpTcWpiQ1RCVFRPbDd2cExKOF9adGxta2FWMUN1NjRvamQ0QUpYcFBUM2hSZkk4YWVibw?oc=5</t>
+        </is>
+      </c>
+      <c r="U318" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally - TradingView</t>
+        </is>
+      </c>
+      <c r="V318" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOcEVXNVpEUFAyU1hJbU1QMk1PYVBBSUNoRmRZMTR0d1Bib2FHeFEwS1N4QXpTLXVva3VXYTh6TG1Wd0Y5NnQ4ZGprUC1hR0d4eWc0TmUyR3lRN0xfX3YwRlpic0hmSU82RTZtZnRudXRlNzBkclZaTW1kNGFURDdac29ZX09obU9OWjRBVXoyRHc2R2ZVbTc5dFZYdlhXc0tqZGhJUUszampxSVMwWENrbk1abUtMemVnbHFpVA?oc=5</t>
+        </is>
+      </c>
+      <c r="W318" t="inlineStr">
+        <is>
+          <t>S&amp;P500, Nasdaq End Higher, Dow Hits Record High On Strong Mag 7 Performance And Falling Oil Prices — BA, XOM, CVX, HOOD, AMD In Focus - Stocktwits</t>
+        </is>
+      </c>
+      <c r="X318" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPbHVRbDJ4YUNuNGtIUDJpZEROMVZkbzB5Rkp5YWhJaENZOG9LR3FJQWRQRHgxbElCSkM5eXdsT3Jzek9zSm5saEFNalpPMFltRU5IVTlqMGhZZEVNNDFDQVJseE9pRXJ5cUhfTVdMWHRBeThHbXNEWDZxWHFlNE1UdDZMRjdUWWdKYmJpWG5tRVBmMHNoX2ZWR1hyRExpaWhvVnBjNnhWellxSkh6N3JaVlppb3p0dXoweFZQWXVaOWhXY1RQdmhwYm52c3pQdVM2UjZHbU94NlA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y318" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z318" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA318" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB318" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC318" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD318" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:09:40+00:00</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E319" t="n">
+        <v>84006.5469</v>
+      </c>
+      <c r="F319" t="n">
+        <v>84176.9688</v>
+      </c>
+      <c r="G319" t="n">
+        <v>83615.00780000001</v>
+      </c>
+      <c r="H319" t="n">
+        <v>84087.9219</v>
+      </c>
+      <c r="I319" t="n">
+        <v>422236160</v>
+      </c>
+      <c r="J319" t="n">
+        <v>4</v>
+      </c>
+      <c r="K319" t="n">
+        <v>38</v>
+      </c>
+      <c r="L319" t="n">
+        <v>-0.093</v>
+      </c>
+      <c r="M319" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="N319" t="n">
+        <v>35</v>
+      </c>
+      <c r="O319" t="n">
+        <v>0.602</v>
+      </c>
+      <c r="P319" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="Q319" t="n">
+        <v>10.257</v>
+      </c>
+      <c r="R319" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S319" t="inlineStr">
+        <is>
+          <t>XRP, Solana Lead Crypto Majors With Bitcoin Stuck Below $85K, BTC ETF Inflows Turning Positive For 2026 - TradingView</t>
+        </is>
+      </c>
+      <c r="T319" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOSTZPSHFoWDhhaEFHTFcxQ0RjcHNmZVZxNXY5VUxvRjFMVUpUY3hibVdTNHBWRUxRSU9ibDdjZkVCSmkwQmJpWjZ1eGh1WmpBRlBDMlVSbkZ3aWFUOUhRanQxT05KdVhsenRJVkNURWI1U09ILWF4dVhiZWRocTE3bXJnVVBaZlBub2ZmYkdLRVdKLWFFcGoxZnVYVXpMY2kyTVduNXA3bXN0SWowMEljOEtJTHA5dnFfT3F0OFF6LWYxaTYwTGpNZTc5YW15YndqRnROUnhCRjBhLWxiOVVvRmlpeXZ1NWxRNldRMU5PaVd3Yk0?oc=5</t>
+        </is>
+      </c>
+      <c r="U319" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="V319" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="W319" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X319" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y319" t="inlineStr">
+        <is>
+          <t>Crypto Prices Today: Bitcoin Slides to $84,000 While Altcoins Rally Hard - CryptoTicker</t>
+        </is>
+      </c>
+      <c r="Z319" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNaWVhbE9DbTFqTjFKVzEwVFJIZzdZZVlTakpMOHJmdnY5SHUxWHdFeVhRd3NjUW5seWw4cmlqOGpqV1RTMFhaQlpkT3A3SGV0YTloTWFHNzNZT2RqVGZqaDlLMk1tbW15UzRZVDlwbURXMGhJM3dXV1laRUVfaWdXQw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA319" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="AB319" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AC319" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Prediction: What to Check on Levels, Holding Period and Leverage Before the October 28 Rate Decision - CryptoTicker</t>
+        </is>
+      </c>
+      <c r="AD319" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaXV3ang1VjN6VzlqcVR1empzLS12Q3pnSjdaZUh3SVcyRXdUc0k0c1Y5RGFfTjdPRmRUT0tzaGd4TEZDSjhXelJhOHdpSzdZQ1gxMTBKWjVsdE1ZTHZsRzZodEZpZGR6OEYycGJiYkZUWTBicVVsWms5OXBTcXhrdTRRamhvSVVNY1pLOFBZbw?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-25 23:50 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD319"/>
+  <dimension ref="A1:AD325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40167,6 +40167,762 @@
         </is>
       </c>
       <c r="AD319" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaXV3ang1VjN6VzlqcVR1empzLS12Q3pnSjdaZUh3SVcyRXdUc0k0c1Y5RGFfTjdPRmRUT0tzaGd4TEZDSjhXelJhOHdpSzdZQ1gxMTBKWjVsdE1ZTHZsRzZodEZpZGR6OEYycGJiYkZUWTBicVVsWms5OXBTcXhrdTRRamhvSVVNY1pLOFBZbw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:48:49+00:00</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E320" t="n">
+        <v>4321.6001</v>
+      </c>
+      <c r="F320" t="n">
+        <v>4332.3999</v>
+      </c>
+      <c r="G320" t="n">
+        <v>4314.5</v>
+      </c>
+      <c r="H320" t="n">
+        <v>4320.5</v>
+      </c>
+      <c r="I320" t="n">
+        <v>17239</v>
+      </c>
+      <c r="J320" t="n">
+        <v>4</v>
+      </c>
+      <c r="K320" t="n">
+        <v>40</v>
+      </c>
+      <c r="L320" t="n">
+        <v>-0.136</v>
+      </c>
+      <c r="M320" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="N320" t="n">
+        <v>40</v>
+      </c>
+      <c r="O320" t="n">
+        <v>-0.027</v>
+      </c>
+      <c r="P320" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="Q320" t="n">
+        <v>-3.251</v>
+      </c>
+      <c r="R320" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S320" t="inlineStr">
+        <is>
+          <t>Lundin Gold Hits Record Grade at Bonza Sur With 204 g/t Gold Over 3 Metres Intercept - the deep dive</t>
+        </is>
+      </c>
+      <c r="T320" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNaDdPLWtTOVlMN0c3OWFFWmF1dUZfT28xLWducTQyQVo5XzRUZzU5YWxUZ1JlZzZqcHRtcG5FUENMZE9LN1ZEQXdpTDBMa3c2Ry1aakpaMjBtTlV6bTNDenB4d2d1OEltQmxadjVsTHFWY0J5alI2Sko2YVdfa1VHZDd3bGVtdUlOaXVaZU0xcFo0UHBjNXZTX2dKS1dtX1J5d2JBX2NxSW9TMS1P?oc=5</t>
+        </is>
+      </c>
+      <c r="U320" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="V320" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="W320" t="inlineStr">
+        <is>
+          <t>Precious Metals Surge: Gold Approaches $4,500 Mark, Silver Reclaims $66 - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="X320" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAxTUhJVFR3RXFNV3VTVFBNTl9OUXhvNmx6R01EZjFqSW05UWJjN3JIUGltNUNobFJKazVGR0lhb1J2bS1iRDdSeC1Fa0YtNU1BQi1xM1hnVjhaZklSUjFpU0ZHWV9GOHlncUtZMmtKTzRxQV8zM2c?oc=5</t>
+        </is>
+      </c>
+      <c r="Y320" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="Z320" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA320" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AB320" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC320" t="inlineStr">
+        <is>
+          <t>Gold breaks below key MAs, eyes $4,260 support: Live levels - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD320" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPME13WGVlVjFRRTNPak02V1FBTDZVR25FMHh5Yjc5NWZqZUZfZ3pyUjRxTU5HcWRDS1I3RVRQQ0V0eTZOZmMxMk9aMlc1WGsyd0FPQzU3ZzlMSUp4cVFBSUR6ZkJucl9WSTNlRWRPdHlxY1o1emxISC10OXJib2tlaV80RGpxaW9hR3BydHhPOVNMdFFDSDd1c3RzVGc1MmJpNm1WTDkySUplMkZyZks2bQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:48:49+00:00</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E321" t="n">
+        <v>92.23999999999999</v>
+      </c>
+      <c r="F321" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="G321" t="n">
+        <v>91.81999999999999</v>
+      </c>
+      <c r="H321" t="n">
+        <v>92.44</v>
+      </c>
+      <c r="I321" t="n">
+        <v>72759</v>
+      </c>
+      <c r="J321" t="n">
+        <v>4</v>
+      </c>
+      <c r="K321" t="n">
+        <v>40</v>
+      </c>
+      <c r="L321" t="n">
+        <v>-0</v>
+      </c>
+      <c r="M321" t="n">
+        <v>-0.163</v>
+      </c>
+      <c r="N321" t="n">
+        <v>40</v>
+      </c>
+      <c r="O321" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="P321" t="n">
+        <v>-0.092</v>
+      </c>
+      <c r="Q321" t="n">
+        <v>2.589</v>
+      </c>
+      <c r="R321" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S321" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T321" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U321" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V321" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W321" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="X321" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y321" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z321" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA321" t="inlineStr">
+        <is>
+          <t>nano Crude Oil Fut (Jan 2027) Trade Ideas — COINBASE:NOLF2027 - TradingView</t>
+        </is>
+      </c>
+      <c r="AB321" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNc1BOTkRSU0FuQ1IyRE5kUGJzb2V4Mnl1SW5JYVZVWEV0WGZPT1BQN3BEbHpFNU1SQUhMbUdmM04tZG5fbkVMb2hmeDE1M0lIUUd6cHhSdWU2VExUSEJZc3YzY2pNUXFpTUNlNm5Pd2wydU1lU0Ztb1UzT2ZLaUx2SFhWQ2dJQ25QR0E?oc=5</t>
+        </is>
+      </c>
+      <c r="AC321" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="AD321" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:48:49+00:00</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E322" t="n">
+        <v>101.022</v>
+      </c>
+      <c r="F322" t="n">
+        <v>101.077</v>
+      </c>
+      <c r="G322" t="n">
+        <v>100.954</v>
+      </c>
+      <c r="H322" t="n">
+        <v>101.035</v>
+      </c>
+      <c r="I322" t="n">
+        <v>0</v>
+      </c>
+      <c r="J322" t="n">
+        <v>4</v>
+      </c>
+      <c r="K322" t="n">
+        <v>39</v>
+      </c>
+      <c r="L322" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="M322" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="N322" t="n">
+        <v>40</v>
+      </c>
+      <c r="O322" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="P322" t="n">
+        <v>-0.004</v>
+      </c>
+      <c r="Q322" t="n">
+        <v>2.883</v>
+      </c>
+      <c r="R322" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S322" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T322" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U322" t="inlineStr">
+        <is>
+          <t>U.S. dollar strengthens as traders see resilient US economy - Forex Factory</t>
+        </is>
+      </c>
+      <c r="V322" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPUzNuYUY3Y0xYRjV5UHMzckJMZEs1WGRncEwtTVdXbjZlSEJhb19uWmF0WFk0WEVGZld5TjdUZ1l5QjhhS05TbHJUX01YNDNIVFRJVmlHMFJvQjV4MWhkZkVlcE1EMnVGTERUcVRULThyaldDbjJmN1Z2RmxMeTVvenZsVklyLURIdWduOGpBOF9ibnlmVEZjckJDS21GbmljbTVvckJIZEF1YjTSAZoBQVVfeXFMUEYxZDNRZEJUMGgzNzcxb2ZWTS1JUkVlSlFTSnNiTmdyUkYxNXZWemFaNFNJam1PR1RWOGFyVmd3NG9kcUxkeklXS0FyYTdwaDZXa1hPLWtoSTMwUTVWcjQxcmVVdEk1cldRYjB2bnlEWWFLOF9XRlFOZVNXNEQzQ09jYWFxbHNPRVFNTXd3cWtDcFRBSjM3MzZhZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W322" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="X322" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="Y322" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z322" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA322" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB322" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC322" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD322" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:48:49+00:00</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E323" t="n">
+        <v>7795.25</v>
+      </c>
+      <c r="F323" t="n">
+        <v>7814.75</v>
+      </c>
+      <c r="G323" t="n">
+        <v>7793.25</v>
+      </c>
+      <c r="H323" t="n">
+        <v>7805.75</v>
+      </c>
+      <c r="I323" t="n">
+        <v>473791</v>
+      </c>
+      <c r="J323" t="n">
+        <v>4</v>
+      </c>
+      <c r="K323" t="n">
+        <v>40</v>
+      </c>
+      <c r="L323" t="n">
+        <v>-0.175</v>
+      </c>
+      <c r="M323" t="n">
+        <v>0.163</v>
+      </c>
+      <c r="N323" t="n">
+        <v>32</v>
+      </c>
+      <c r="O323" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="P323" t="n">
+        <v>-0.007</v>
+      </c>
+      <c r="Q323" t="n">
+        <v>0.5639999999999999</v>
+      </c>
+      <c r="R323" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S323" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T323" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U323" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - aol.com</t>
+        </is>
+      </c>
+      <c r="V323" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W323" t="inlineStr">
+        <is>
+          <t>Stock market today: Dow hits record high, S&amp;P 500 and Nasdaq surge as Big Tech gains power rally - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X323" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPbkNnYmlpUUZ1UFBUdG13a1NLZlhpbXR4cEpMcUdqRkR5aXd1UjVKaEFFQTJyQ0JrQWFHN0I0Zk1wSDVOZ0RaRWM2aXpCb3BDQmE4c0dXaHFLQVhRcXdiZDZnSko3UGd6WlkwNlVncFNJdTVnbHVGaFJBTXltM0ttaUxkZ0ZFa2ptNVN5S3FTbXBPOTc3UHdZVEtVYVFqWXNMazVsZlhaY3hibzViazhyeXBta2RFWHF4Z1pN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y323" t="inlineStr">
+        <is>
+          <t>If There's a Stock Market Crash Ahead, History Highlights the Best Strategy for Investors - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="Z323" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOQjlSRnVrTllBQ18wak5KWFByYjA4V24ydVJiNnNuV0dQQ1VKVDNnZVp0YUtZdzlhOTNfekZjUW1BckF6UUZFbGZ6cDNwbkVERzZGSlpSa1pueHdxZTdMeVNXWV9BMDh5Z24yU2JEd09IZllEcU1oN0RidTZicDltdy1YRkNzd2dNa2JpZ3FfV1Rha1ZrTVc3NDNxZHQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA323" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB323" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC323" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AD323" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:48:49+00:00</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E324" t="n">
+        <v>30912</v>
+      </c>
+      <c r="F324" t="n">
+        <v>30935</v>
+      </c>
+      <c r="G324" t="n">
+        <v>30845</v>
+      </c>
+      <c r="H324" t="n">
+        <v>30921.75</v>
+      </c>
+      <c r="I324" t="n">
+        <v>83633</v>
+      </c>
+      <c r="J324" t="n">
+        <v>4</v>
+      </c>
+      <c r="K324" t="n">
+        <v>35</v>
+      </c>
+      <c r="L324" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="M324" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N324" t="n">
+        <v>34</v>
+      </c>
+      <c r="O324" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="P324" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="Q324" t="n">
+        <v>1.656</v>
+      </c>
+      <c r="R324" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S324" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally (AMD:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T324" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNRTNUV0JnS3haREZESHpOTVREazZUWkNwUE43OEQxMFJYajZnU3JhaWFKOEt1MVEtLTJYdlg5YnVUUnE3WnFnN0FoRDRJUFZlVEpNN2pCaWFpSEQ5NmlIM2hoQ2VDcHNHRHpTcWpiQ1RCVFRPbDd2cExKOF9adGxta2FWMUN1NjRvamQ0QUpYcFBUM2hSZkk4YWVibw?oc=5</t>
+        </is>
+      </c>
+      <c r="U324" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as chipmakers fuel stock gains - Reuters</t>
+        </is>
+      </c>
+      <c r="V324" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQUUdXdXVKYkpsa2JoQmRNeVpVWWhwb1pIVmUwcUl0QVRFVEFjRDJtREJPbXJWaXVEc0NQSWZZUlhwTl80T3h4eGM1dE9oaXRsWlVueWx0MWt3YXlWbV9PYkZDWVVPb1ZveThvalZfWnBvQ2J5Sjg1UkNOQmU5eDdWN0FvVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W324" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally - TradingView</t>
+        </is>
+      </c>
+      <c r="X324" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOcEVXNVpEUFAyU1hJbU1QMk1PYVBBSUNoRmRZMTR0d1Bib2FHeFEwS1N4QXpTLXVva3VXYTh6TG1Wd0Y5NnQ4ZGprUC1hR0d4eWc0TmUyR3lRN0xfX3YwRlpic0hmSU82RTZtZnRudXRlNzBkclZaTW1kNGFURDdac29ZX09obU9OWjRBVXoyRHc2R2ZVbTc5dFZYdlhXc0tqZGhJUUszampxSVMwWENrbk1abUtMemVnbHFpVA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y324" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z324" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA324" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB324" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC324" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD324" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:48:49+00:00</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E325" t="n">
+        <v>84006.5469</v>
+      </c>
+      <c r="F325" t="n">
+        <v>84176.9688</v>
+      </c>
+      <c r="G325" t="n">
+        <v>83615.00780000001</v>
+      </c>
+      <c r="H325" t="n">
+        <v>84066</v>
+      </c>
+      <c r="I325" t="n">
+        <v>567984128</v>
+      </c>
+      <c r="J325" t="n">
+        <v>4</v>
+      </c>
+      <c r="K325" t="n">
+        <v>38</v>
+      </c>
+      <c r="L325" t="n">
+        <v>-0.093</v>
+      </c>
+      <c r="M325" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="N325" t="n">
+        <v>35</v>
+      </c>
+      <c r="O325" t="n">
+        <v>0.5580000000000001</v>
+      </c>
+      <c r="P325" t="n">
+        <v>-0.073</v>
+      </c>
+      <c r="Q325" t="n">
+        <v>9.491</v>
+      </c>
+      <c r="R325" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S325" t="inlineStr">
+        <is>
+          <t>XRP, Solana Lead Crypto Majors With Bitcoin Stuck Below $85K, BTC ETF Inflows Turning Positive For 2026 - TradingView</t>
+        </is>
+      </c>
+      <c r="T325" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOSTZPSHFoWDhhaEFHTFcxQ0RjcHNmZVZxNXY5VUxvRjFMVUpUY3hibVdTNHBWRUxRSU9ibDdjZkVCSmkwQmJpWjZ1eGh1WmpBRlBDMlVSbkZ3aWFUOUhRanQxT05KdVhsenRJVkNURWI1U09ILWF4dVhiZWRocTE3bXJnVVBaZlBub2ZmYkdLRVdKLWFFcGoxZnVYVXpMY2kyTVduNXA3bXN0SWowMEljOEtJTHA5dnFfT3F0OFF6LWYxaTYwTGpNZTc5YW15YndqRnROUnhCRjBhLWxiOVVvRmlpeXZ1NWxRNldRMU5PaVd3Yk0?oc=5</t>
+        </is>
+      </c>
+      <c r="U325" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="V325" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="W325" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X325" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y325" t="inlineStr">
+        <is>
+          <t>Crypto Prices Today: Bitcoin Slides to $84,000 While Altcoins Rally Hard - CryptoTicker</t>
+        </is>
+      </c>
+      <c r="Z325" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNaWVhbE9DbTFqTjFKVzEwVFJIZzdZZVlTakpMOHJmdnY5SHUxWHdFeVhRd3NjUW5seWw4cmlqOGpqV1RTMFhaQlpkT3A3SGV0YTloTWFHNzNZT2RqVGZqaDlLMk1tbW15UzRZVDlwbURXMGhJM3dXV1laRUVfaWdXQw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA325" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="AB325" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AC325" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Prediction: What to Check on Levels, Holding Period and Leverage Before the October 28 Rate Decision - CryptoTicker</t>
+        </is>
+      </c>
+      <c r="AD325" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaXV3ang1VjN6VzlqcVR1empzLS12Q3pnSjdaZUh3SVcyRXdUc0k0c1Y5RGFfTjdPRmRUT0tzaGd4TEZDSjhXelJhOHdpSzdZQ1gxMTBKWjVsdE1ZTHZsRzZodEZpZGR6OEYycGJiYkZUWTBicVVsWms5OXBTcXhrdTRRamhvSVVNY1pLOFBZbw?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-26 03:59 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD325"/>
+  <dimension ref="A1:AD331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40341,7 +40341,7 @@
         <v>40</v>
       </c>
       <c r="L321" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M321" t="n">
         <v>-0.163</v>
@@ -40923,6 +40923,762 @@
         </is>
       </c>
       <c r="AD325" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaXV3ang1VjN6VzlqcVR1empzLS12Q3pnSjdaZUh3SVcyRXdUc0k0c1Y5RGFfTjdPRmRUT0tzaGd4TEZDSjhXelJhOHdpSzdZQ1gxMTBKWjVsdE1ZTHZsRzZodEZpZGR6OEYycGJiYkZUWTBicVVsWms5OXBTcXhrdTRRamhvSVVNY1pLOFBZbw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-09-26T03:57:01+00:00</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E326" t="n">
+        <v>4321.6001</v>
+      </c>
+      <c r="F326" t="n">
+        <v>4332.3999</v>
+      </c>
+      <c r="G326" t="n">
+        <v>4314.5</v>
+      </c>
+      <c r="H326" t="n">
+        <v>4320.5</v>
+      </c>
+      <c r="I326" t="n">
+        <v>17239</v>
+      </c>
+      <c r="J326" t="n">
+        <v>4</v>
+      </c>
+      <c r="K326" t="n">
+        <v>39</v>
+      </c>
+      <c r="L326" t="n">
+        <v>-0.196</v>
+      </c>
+      <c r="M326" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="N326" t="n">
+        <v>40</v>
+      </c>
+      <c r="O326" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="P326" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="Q326" t="n">
+        <v>-4.137</v>
+      </c>
+      <c r="R326" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S326" t="inlineStr">
+        <is>
+          <t>Lundin Gold Hits Record Grade at Bonza Sur With 204 g/t Gold Over 3 Metres Intercept - the deep dive</t>
+        </is>
+      </c>
+      <c r="T326" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNaDdPLWtTOVlMN0c3OWFFWmF1dUZfT28xLWducTQyQVo5XzRUZzU5YWxUZ1JlZzZqcHRtcG5FUENMZE9LN1ZEQXdpTDBMa3c2Ry1aakpaMjBtTlV6bTNDenB4d2d1OEltQmxadjVsTHFWY0J5alI2Sko2YVdfa1VHZDd3bGVtdUlOaXVaZU0xcFo0UHBjNXZTX2dKS1dtX1J5d2JBX2NxSW9TMS1P?oc=5</t>
+        </is>
+      </c>
+      <c r="U326" t="inlineStr">
+        <is>
+          <t>Gold Q4 2026 outlook: Resilience in the face of rallying dollar and yields - FOREX.com</t>
+        </is>
+      </c>
+      <c r="V326" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPUk9TLVFNaXZQZXZINE1scGhtYk9IRVB0a2Z4SnoxT1dwN1B3V3M2WUpubFIyZk9CcmwyVGNxd09LRFZLRGhuQnFpSjgxbUJHYUM1ME40LU5ZTjFSZmh2NncyUHF5MEdwcW84dXUwOU9XR20wYmRXZTFNb1N3LUtZdEpIOENoTU01Uno1OGIweXZHcnR5cDM3TTF0X19xa05ROW5mVXlnNElaRXRRcGxPdUh1NnB4SzUtZUd0dA?oc=5</t>
+        </is>
+      </c>
+      <c r="W326" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="X326" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="Y326" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - fxstreet.com</t>
+        </is>
+      </c>
+      <c r="Z326" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA326" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AB326" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC326" t="inlineStr">
+        <is>
+          <t>Gold breaks below key MAs, eyes $4,260 support: Live levels - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD326" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPME13WGVlVjFRRTNPak02V1FBTDZVR25FMHh5Yjc5NWZqZUZfZ3pyUjRxTU5HcWRDS1I3RVRQQ0V0eTZOZmMxMk9aMlc1WGsyd0FPQzU3ZzlMSUp4cVFBSUR6ZkJucl9WSTNlRWRPdHlxY1o1emxISC10OXJib2tlaV80RGpxaW9hR3BydHhPOVNMdFFDSDd1c3RzVGc1MmJpNm1WTDkySUplMkZyZks2bQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-09-26T03:57:01+00:00</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E327" t="n">
+        <v>92.23999999999999</v>
+      </c>
+      <c r="F327" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="G327" t="n">
+        <v>91.81999999999999</v>
+      </c>
+      <c r="H327" t="n">
+        <v>92.44</v>
+      </c>
+      <c r="I327" t="n">
+        <v>72759</v>
+      </c>
+      <c r="J327" t="n">
+        <v>4</v>
+      </c>
+      <c r="K327" t="n">
+        <v>40</v>
+      </c>
+      <c r="L327" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="M327" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="N327" t="n">
+        <v>40</v>
+      </c>
+      <c r="O327" t="n">
+        <v>0.201</v>
+      </c>
+      <c r="P327" t="n">
+        <v>-0.074</v>
+      </c>
+      <c r="Q327" t="n">
+        <v>4.547</v>
+      </c>
+      <c r="R327" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S327" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T327" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U327" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V327" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W327" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - Reuters</t>
+        </is>
+      </c>
+      <c r="X327" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPWEdjS0pVMy1JLXZFN0V6ZFhjdjNOOXpjRnUtYXdYZEdjbzNaR2R6TGU4UTRDVEdLazJuMS12eHp6d0hWQjI0ZzdhRTUtbVBqR3NhSGRES0UxbG1TZ29QX1hjaWZFNWs1RWNWV1E0azdPVDNIR2x4TGJYMzdDZ3YtVUN1VzZEam5Tb3pXYy1TejN0VFMxYjI1U3ByeFZDZmZ1UnFYX053R3N3YzhST3dSWGdB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y327" t="inlineStr">
+        <is>
+          <t>A reprieve from rising oil prices helps US stocks finish the week higher - WRAL</t>
+        </is>
+      </c>
+      <c r="Z327" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNTzNxamtacnJZaXVrRGRhTXRoRE5DbmluNlpjNGRIRnRfTWI0WFBoZTRxWkxMcmxnakxtdHU3VEVJNWhZaDlQMDNuMHdISTRqN1VJTVJoaldxLVllLU1Kb2RzQnlKWFRoaGFHM1VkdmtGZjVMLTRMTU9DZ2RuX2RlaXhYS1p0MlJrNktCM1ZTcFVNTlVzYW9jZnNXSWpzOHM4RlY0YmVraTJsYTBV?oc=5</t>
+        </is>
+      </c>
+      <c r="AA327" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AB327" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC327" t="inlineStr">
+        <is>
+          <t>nano Crude Oil Fut (Jan 2027) Trade Ideas — COINBASE:NOLF2027 - TradingView</t>
+        </is>
+      </c>
+      <c r="AD327" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNc1BOTkRSU0FuQ1IyRE5kUGJzb2V4Mnl1SW5JYVZVWEV0WGZPT1BQN3BEbHpFNU1SQUhMbUdmM04tZG5fbkVMb2hmeDE1M0lIUUd6cHhSdWU2VExUSEJZc3YzY2pNUXFpTUNlNm5Pd2wydU1lU0Ztb1UzT2ZLaUx2SFhWQ2dJQ25QR0E?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-09-26T03:57:01+00:00</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E328" t="n">
+        <v>101.022</v>
+      </c>
+      <c r="F328" t="n">
+        <v>101.077</v>
+      </c>
+      <c r="G328" t="n">
+        <v>100.954</v>
+      </c>
+      <c r="H328" t="n">
+        <v>101.035</v>
+      </c>
+      <c r="I328" t="n">
+        <v>0</v>
+      </c>
+      <c r="J328" t="n">
+        <v>4</v>
+      </c>
+      <c r="K328" t="n">
+        <v>39</v>
+      </c>
+      <c r="L328" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="M328" t="n">
+        <v>0.157</v>
+      </c>
+      <c r="N328" t="n">
+        <v>40</v>
+      </c>
+      <c r="O328" t="n">
+        <v>0.089</v>
+      </c>
+      <c r="P328" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="Q328" t="n">
+        <v>3.183</v>
+      </c>
+      <c r="R328" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S328" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T328" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U328" t="inlineStr">
+        <is>
+          <t>U.S. dollar strengthens as traders see resilient US economy - Forex Factory</t>
+        </is>
+      </c>
+      <c r="V328" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPUzNuYUY3Y0xYRjV5UHMzckJMZEs1WGRncEwtTVdXbjZlSEJhb19uWmF0WFk0WEVGZld5TjdUZ1l5QjhhS05TbHJUX01YNDNIVFRJVmlHMFJvQjV4MWhkZkVlcE1EMnVGTERUcVRULThyaldDbjJmN1Z2RmxMeTVvenZsVklyLURIdWduOGpBOF9ibnlmVEZjckJDS21GbmljbTVvckJIZEF1YjTSAZoBQVVfeXFMUEYxZDNRZEJUMGgzNzcxb2ZWTS1JUkVlSlFTSnNiTmdyUkYxNXZWemFaNFNJam1PR1RWOGFyVmd3NG9kcUxkeklXS0FyYTdwaDZXa1hPLWtoSTMwUTVWcjQxcmVVdEk1cldRYjB2bnlEWWFLOF9XRlFOZVNXNEQzQ09jYWFxbHNPRVFNTXd3cWtDcFRBSjM3MzZhZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W328" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="X328" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="Y328" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z328" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA328" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB328" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC328" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD328" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-09-26T03:57:01+00:00</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E329" t="n">
+        <v>7795.25</v>
+      </c>
+      <c r="F329" t="n">
+        <v>7814.75</v>
+      </c>
+      <c r="G329" t="n">
+        <v>7793.25</v>
+      </c>
+      <c r="H329" t="n">
+        <v>7805.75</v>
+      </c>
+      <c r="I329" t="n">
+        <v>473791</v>
+      </c>
+      <c r="J329" t="n">
+        <v>4</v>
+      </c>
+      <c r="K329" t="n">
+        <v>40</v>
+      </c>
+      <c r="L329" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="M329" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="N329" t="n">
+        <v>40</v>
+      </c>
+      <c r="O329" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="P329" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="Q329" t="n">
+        <v>0.127</v>
+      </c>
+      <c r="R329" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S329" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T329" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U329" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V329" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W329" t="inlineStr">
+        <is>
+          <t>AbCellera Biologics (ABCL) Surges 34.78% as Shares Break Toward $9.81 Resistance - EMA Signal - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="X329" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPdUNOZndBWm5IMm9JRjRsTk5DNmtNQnR6YTFWMWlSTk5BT3J2TjNEdXlrMFl5Vi1sdDVyY1BybUlUU0taSnQtcktxZEV5ZkpYclc4dnBNa0lzamY3dFFRTGNMWXU5TFk3MUphb1hnak4zYS1vQ0s2NHdTeFFLOGEwdlRkcGE5VUs4a0t2bnk3SkJPMGk2RGM4VV9mclUwZmJQMGUtNXN0dUN5Z2M1U1E0cG5pckZOQlJ2TGdDSg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y329" t="inlineStr">
+        <is>
+          <t>If There's a Stock Market Crash Ahead, History Highlights the Best Strategy for Investors - AOL.com</t>
+        </is>
+      </c>
+      <c r="Z329" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxObDRyTS13c3JCdDU5NmNhU3g3NnlUNkpoamlFR1Fic09CTzltRV9zcS1fUUwzdG45dExiY3k3N2c2VnItZ2twWnBZNktPXzItSmRMRVBveS1GdWljRDFpTmtxN3c1OG41a1dhTzFwNU44WkpGTm5oNjMtdzVtaURxVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA329" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB329" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC329" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - foxbusiness.com</t>
+        </is>
+      </c>
+      <c r="AD329" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-09-26T03:57:01+00:00</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E330" t="n">
+        <v>30912</v>
+      </c>
+      <c r="F330" t="n">
+        <v>30935</v>
+      </c>
+      <c r="G330" t="n">
+        <v>30845</v>
+      </c>
+      <c r="H330" t="n">
+        <v>30921.75</v>
+      </c>
+      <c r="I330" t="n">
+        <v>83633</v>
+      </c>
+      <c r="J330" t="n">
+        <v>4</v>
+      </c>
+      <c r="K330" t="n">
+        <v>35</v>
+      </c>
+      <c r="L330" t="n">
+        <v>-0.089</v>
+      </c>
+      <c r="M330" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="N330" t="n">
+        <v>34</v>
+      </c>
+      <c r="O330" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="P330" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="Q330" t="n">
+        <v>2.477</v>
+      </c>
+      <c r="R330" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S330" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally (AMD:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T330" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNRTNUV0JnS3haREZESHpOTVREazZUWkNwUE43OEQxMFJYajZnU3JhaWFKOEt1MVEtLTJYdlg5YnVUUnE3WnFnN0FoRDRJUFZlVEpNN2pCaWFpSEQ5NmlIM2hoQ2VDcHNHRHpTcWpiQ1RCVFRPbDd2cExKOF9adGxta2FWMUN1NjRvamQ0QUpYcFBUM2hSZkk4YWVibw?oc=5</t>
+        </is>
+      </c>
+      <c r="U330" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally - TradingView</t>
+        </is>
+      </c>
+      <c r="V330" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOcEVXNVpEUFAyU1hJbU1QMk1PYVBBSUNoRmRZMTR0d1Bib2FHeFEwS1N4QXpTLXVva3VXYTh6TG1Wd0Y5NnQ4ZGprUC1hR0d4eWc0TmUyR3lRN0xfX3YwRlpic0hmSU82RTZtZnRudXRlNzBkclZaTW1kNGFURDdac29ZX09obU9OWjRBVXoyRHc2R2ZVbTc5dFZYdlhXc0tqZGhJUUszampxSVMwWENrbk1abUtMemVnbHFpVA?oc=5</t>
+        </is>
+      </c>
+      <c r="W330" t="inlineStr">
+        <is>
+          <t>S&amp;P500, Nasdaq End Higher, Dow Hits Record High On Strong Mag 7 Performance And Falling Oil Prices — BA, XOM, CVX, HOOD, AMD In Focus - Stocktwits</t>
+        </is>
+      </c>
+      <c r="X330" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPbHVRbDJ4YUNuNGtIUDJpZEROMVZkbzB5Rkp5YWhJaENZOG9LR3FJQWRQRHgxbElCSkM5eXdsT3Jzek9zSm5saEFNalpPMFltRU5IVTlqMGhZZEVNNDFDQVJseE9pRXJ5cUhfTVdMWHRBeThHbXNEWDZxWHFlNE1UdDZMRjdUWWdKYmJpWG5tRVBmMHNoX2ZWR1hyRExpaWhvVnBjNnhWellxSkh6N3JaVlppb3p0dXoweFZQWXVaOWhXY1RQdmhwYm52c3pQdVM2UjZHbU94NlA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y330" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z330" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA330" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB330" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC330" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD330" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-09-26T03:57:01+00:00</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E331" t="n">
+        <v>84096.00780000001</v>
+      </c>
+      <c r="F331" t="n">
+        <v>84135.10159999999</v>
+      </c>
+      <c r="G331" t="n">
+        <v>83777.7812</v>
+      </c>
+      <c r="H331" t="n">
+        <v>83930.46090000001</v>
+      </c>
+      <c r="I331" t="n">
+        <v>635058176</v>
+      </c>
+      <c r="J331" t="n">
+        <v>4</v>
+      </c>
+      <c r="K331" t="n">
+        <v>37</v>
+      </c>
+      <c r="L331" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="M331" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="N331" t="n">
+        <v>35</v>
+      </c>
+      <c r="O331" t="n">
+        <v>0.481</v>
+      </c>
+      <c r="P331" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="Q331" t="n">
+        <v>8.585000000000001</v>
+      </c>
+      <c r="R331" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S331" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="T331" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U331" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="V331" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="W331" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="X331" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y331" t="inlineStr">
+        <is>
+          <t>Crypto Prices Today: Bitcoin Slides to $84,000 While Altcoins Rally Hard - CryptoTicker</t>
+        </is>
+      </c>
+      <c r="Z331" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNaWVhbE9DbTFqTjFKVzEwVFJIZzdZZVlTakpMOHJmdnY5SHUxWHdFeVhRd3NjUW5seWw4cmlqOGpqV1RTMFhaQlpkT3A3SGV0YTloTWFHNzNZT2RqVGZqaDlLMk1tbW15UzRZVDlwbURXMGhJM3dXV1laRUVfaWdXQw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA331" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="AB331" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AC331" t="inlineStr">
+        <is>
+          <t>Bitcoin Price Prediction: What to Check on Levels, Holding Period and Leverage Before the October 28 Rate Decision - CryptoTicker</t>
+        </is>
+      </c>
+      <c r="AD331" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaXV3ang1VjN6VzlqcVR1empzLS12Q3pnSjdaZUh3SVcyRXdUc0k0c1Y5RGFfTjdPRmRUT0tzaGd4TEZDSjhXelJhOHdpSzdZQ1gxMTBKWjVsdE1ZTHZsRzZodEZpZGR6OEYycGJiYkZUWTBicVVsWms5OXBTcXhrdTRRamhvSVVNY1pLOFBZbw?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-26 09:16 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD331"/>
+  <dimension ref="A1:AD337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41681,6 +41681,762 @@
       <c r="AD331" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaXV3ang1VjN6VzlqcVR1empzLS12Q3pnSjdaZUh3SVcyRXdUc0k0c1Y5RGFfTjdPRmRUT0tzaGd4TEZDSjhXelJhOHdpSzdZQ1gxMTBKWjVsdE1ZTHZsRzZodEZpZGR6OEYycGJiYkZUWTBicVVsWms5OXBTcXhrdTRRamhvSVVNY1pLOFBZbw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-09-26T09:13:52+00:00</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E332" t="n">
+        <v>4321.6001</v>
+      </c>
+      <c r="F332" t="n">
+        <v>4332.3999</v>
+      </c>
+      <c r="G332" t="n">
+        <v>4314.5</v>
+      </c>
+      <c r="H332" t="n">
+        <v>4321.2002</v>
+      </c>
+      <c r="I332" t="n">
+        <v>17239</v>
+      </c>
+      <c r="J332" t="n">
+        <v>4</v>
+      </c>
+      <c r="K332" t="n">
+        <v>39</v>
+      </c>
+      <c r="L332" t="n">
+        <v>-0.163</v>
+      </c>
+      <c r="M332" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="N332" t="n">
+        <v>40</v>
+      </c>
+      <c r="O332" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="P332" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="Q332" t="n">
+        <v>-3.37</v>
+      </c>
+      <c r="R332" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S332" t="inlineStr">
+        <is>
+          <t>Lundin Gold Hits Record Grade at Bonza Sur With 204 g/t Gold Over 3 Metres Intercept - the deep dive</t>
+        </is>
+      </c>
+      <c r="T332" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNaDdPLWtTOVlMN0c3OWFFWmF1dUZfT28xLWducTQyQVo5XzRUZzU5YWxUZ1JlZzZqcHRtcG5FUENMZE9LN1ZEQXdpTDBMa3c2Ry1aakpaMjBtTlV6bTNDenB4d2d1OEltQmxadjVsTHFWY0J5alI2Sko2YVdfa1VHZDd3bGVtdUlOaXVaZU0xcFo0UHBjNXZTX2dKS1dtX1J5d2JBX2NxSW9TMS1P?oc=5</t>
+        </is>
+      </c>
+      <c r="U332" t="inlineStr">
+        <is>
+          <t>Gold Q4 2026 outlook: Resilience in the face of rallying dollar and yields - FOREX.com</t>
+        </is>
+      </c>
+      <c r="V332" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPUk9TLVFNaXZQZXZINE1scGhtYk9IRVB0a2Z4SnoxT1dwN1B3V3M2WUpubFIyZk9CcmwyVGNxd09LRFZLRGhuQnFpSjgxbUJHYUM1ME40LU5ZTjFSZmh2NncyUHF5MEdwcW84dXUwOU9XR20wYmRXZTFNb1N3LUtZdEpIOENoTU01Uno1OGIweXZHcnR5cDM3TTF0X19xa05ROW5mVXlnNElaRXRRcGxPdUh1NnB4SzUtZUd0dA?oc=5</t>
+        </is>
+      </c>
+      <c r="W332" t="inlineStr">
+        <is>
+          <t>Precious Metals Surge: Gold Approaches $4,500 Mark, Silver Reclaims $66 - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="X332" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAxTUhJVFR3RXFNV3VTVFBNTl9OUXhvNmx6R01EZjFqSW05UWJjN3JIUGltNUNobFJKazVGR0lhb1J2bS1iRDdSeC1Fa0YtNU1BQi1xM1hnVjhaZklSUjFpU0ZHWV9GOHlncUtZMmtKTzRxQV8zM2c?oc=5</t>
+        </is>
+      </c>
+      <c r="Y332" t="inlineStr">
+        <is>
+          <t>Record: Chinese investors pull $2.22 billion from Gold ETFs in June, the highest monthly outflow ever - FXStreet</t>
+        </is>
+      </c>
+      <c r="Z332" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSFRKQTdTLTFRejA5ZGxYc0lkZGFQNlplRlBCemlQVEwyMVdDNFkxTENCMXgwZ3NjZEdzdWNkcjJDdno0d0xyVHl1S2Zlal85Q2pkaTVvbm5VMGVUaE9naDhITzdVV2xPeGRlQmdYQlZCNGc2VDVnLU5hMGxHQklJMUZXY2xUSmxVQVU0ZmVISlVPR1dPTVNfOE9iOVJ3TlpXbThVcWlMRmJUeENhYkdLTkVxZ05qeXRHSDlkejk1R2V3bHpsd3h4ZHEwLVA0Q2VvajhqMmRCTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA332" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AB332" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC332" t="inlineStr">
+        <is>
+          <t>Gold breaks below key MAs, eyes $4,260 support: Live levels - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD332" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPME13WGVlVjFRRTNPak02V1FBTDZVR25FMHh5Yjc5NWZqZUZfZ3pyUjRxTU5HcWRDS1I3RVRQQ0V0eTZOZmMxMk9aMlc1WGsyd0FPQzU3ZzlMSUp4cVFBSUR6ZkJucl9WSTNlRWRPdHlxY1o1emxISC10OXJib2tlaV80RGpxaW9hR3BydHhPOVNMdFFDSDd1c3RzVGc1MmJpNm1WTDkySUplMkZyZks2bQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-09-26T09:13:52+00:00</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E333" t="n">
+        <v>92.23999999999999</v>
+      </c>
+      <c r="F333" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="G333" t="n">
+        <v>91.81999999999999</v>
+      </c>
+      <c r="H333" t="n">
+        <v>92.41</v>
+      </c>
+      <c r="I333" t="n">
+        <v>72759</v>
+      </c>
+      <c r="J333" t="n">
+        <v>4</v>
+      </c>
+      <c r="K333" t="n">
+        <v>40</v>
+      </c>
+      <c r="L333" t="n">
+        <v>-0.089</v>
+      </c>
+      <c r="M333" t="n">
+        <v>-0.175</v>
+      </c>
+      <c r="N333" t="n">
+        <v>40</v>
+      </c>
+      <c r="O333" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="P333" t="n">
+        <v>-0.142</v>
+      </c>
+      <c r="Q333" t="n">
+        <v>1.366</v>
+      </c>
+      <c r="R333" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S333" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T333" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U333" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V333" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W333" t="inlineStr">
+        <is>
+          <t>India LPG Production Up 20% in September as Festive Demand Meets Middle East Import Limits - News and Statistics - IndexBox</t>
+        </is>
+      </c>
+      <c r="X333" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOQ0tOLWtGVXFnTmFYWFZmQXM5ODFpb3hJZ1dHenBzVHRWQWwyWm9sT0dVS0Z1eWpxY2RLRURxb3pEXzRmN09oVG1FRXFzYUZidnpQbHNCNG1jbWg2WWJ3Z2s5MUlWQndxNldmZmR2QXJJeTVvdkZXN3lxUTZGZEN4cG9MdFN3Q2NBX2dEdHZNMUU2MUhVbXdGN3RsbDl0bzZ2RmpxNTBMZ1doak04b092N0Qtaw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y333" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="Z333" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA333" t="inlineStr">
+        <is>
+          <t>nano Crude Oil Fut (Jan 2027) Trade Ideas — COINBASE:NOLF2027 - TradingView</t>
+        </is>
+      </c>
+      <c r="AB333" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNc1BOTkRSU0FuQ1IyRE5kUGJzb2V4Mnl1SW5JYVZVWEV0WGZPT1BQN3BEbHpFNU1SQUhMbUdmM04tZG5fbkVMb2hmeDE1M0lIUUd6cHhSdWU2VExUSEJZc3YzY2pNUXFpTUNlNm5Pd2wydU1lU0Ztb1UzT2ZLaUx2SFhWQ2dJQ25QR0E?oc=5</t>
+        </is>
+      </c>
+      <c r="AC333" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 25, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AD333" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9DVE10MHdQOXV3X0ZlbGNJS0J4ZXg2Tm1GSVVQcmdJVExmVUo5R2FPbjBDRVJ3eUZLeWd2SC1CVnZLUHNYZkx6M1NoNnFkMGpKUHFBZjh4clhDZDZlZ1Vmak5B?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-09-26T09:13:52+00:00</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E334" t="n">
+        <v>101.022</v>
+      </c>
+      <c r="F334" t="n">
+        <v>101.077</v>
+      </c>
+      <c r="G334" t="n">
+        <v>100.954</v>
+      </c>
+      <c r="H334" t="n">
+        <v>101.035</v>
+      </c>
+      <c r="I334" t="n">
+        <v>0</v>
+      </c>
+      <c r="J334" t="n">
+        <v>4</v>
+      </c>
+      <c r="K334" t="n">
+        <v>39</v>
+      </c>
+      <c r="L334" t="n">
+        <v>-0.016</v>
+      </c>
+      <c r="M334" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="N334" t="n">
+        <v>40</v>
+      </c>
+      <c r="O334" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="P334" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Q334" t="n">
+        <v>1.268</v>
+      </c>
+      <c r="R334" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S334" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T334" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U334" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="V334" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="W334" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="X334" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y334" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z334" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA334" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB334" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC334" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD334" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-09-26T09:13:52+00:00</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E335" t="n">
+        <v>7795.25</v>
+      </c>
+      <c r="F335" t="n">
+        <v>7814.75</v>
+      </c>
+      <c r="G335" t="n">
+        <v>7793.25</v>
+      </c>
+      <c r="H335" t="n">
+        <v>7803.75</v>
+      </c>
+      <c r="I335" t="n">
+        <v>473791</v>
+      </c>
+      <c r="J335" t="n">
+        <v>4</v>
+      </c>
+      <c r="K335" t="n">
+        <v>40</v>
+      </c>
+      <c r="L335" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="M335" t="n">
+        <v>0.152</v>
+      </c>
+      <c r="N335" t="n">
+        <v>40</v>
+      </c>
+      <c r="O335" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="P335" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="Q335" t="n">
+        <v>-2.877</v>
+      </c>
+      <c r="R335" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S335" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T335" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U335" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V335" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W335" t="inlineStr">
+        <is>
+          <t>Stock market today: Dow hits record high, S&amp;P 500 and Nasdaq surge as Big Tech gains power rally - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X335" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPbkNnYmlpUUZ1UFBUdG13a1NLZlhpbXR4cEpMcUdqRkR5aXd1UjVKaEFFQTJyQ0JrQWFHN0I0Zk1wSDVOZ0RaRWM2aXpCb3BDQmE4c0dXaHFLQVhRcXdiZDZnSko3UGd6WlkwNlVncFNJdTVnbHVGaFJBTXltM0ttaUxkZ0ZFa2ptNVN5S3FTbXBPOTc3UHdZVEtVYVFqWXNMazVsZlhaY3hibzViazhyeXBta2RFWHF4Z1pN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y335" t="inlineStr">
+        <is>
+          <t>If There's a Stock Market Crash Ahead, History Highlights the Best Strategy for Investors - AOL.com</t>
+        </is>
+      </c>
+      <c r="Z335" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxObDRyTS13c3JCdDU5NmNhU3g3NnlUNkpoamlFR1Fic09CTzltRV9zcS1fUUwzdG45dExiY3k3N2c2VnItZ2twWnBZNktPXzItSmRMRVBveS1GdWljRDFpTmtxN3c1OG41a1dhTzFwNU44WkpGTm5oNjMtdzVtaURxVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA335" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB335" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC335" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - foxbusiness.com</t>
+        </is>
+      </c>
+      <c r="AD335" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-09-26T09:13:52+00:00</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E336" t="n">
+        <v>30912</v>
+      </c>
+      <c r="F336" t="n">
+        <v>30935</v>
+      </c>
+      <c r="G336" t="n">
+        <v>30845</v>
+      </c>
+      <c r="H336" t="n">
+        <v>30889.25</v>
+      </c>
+      <c r="I336" t="n">
+        <v>83633</v>
+      </c>
+      <c r="J336" t="n">
+        <v>4</v>
+      </c>
+      <c r="K336" t="n">
+        <v>35</v>
+      </c>
+      <c r="L336" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="M336" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="N336" t="n">
+        <v>34</v>
+      </c>
+      <c r="O336" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="P336" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="Q336" t="n">
+        <v>2.678</v>
+      </c>
+      <c r="R336" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S336" t="inlineStr">
+        <is>
+          <t>Nasdaq sets record high, oil dips on improved crude flows - Reuters</t>
+        </is>
+      </c>
+      <c r="T336" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBYNkdDWExac0tiSmtsc3Exd0ZHOTVDZFJCbTRtZW9jM3hTLU84b3JWbHQ1WmZsUE5pSmUzTHBFUXQzaHBnb01UQXV5ZUljTFl2cS1fbHhFMUtDblA3NHRjeXRzbEpYMjNZempPSmRPbEpIajV0T1BuRDl1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U336" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally (AMD:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V336" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNRTNUV0JnS3haREZESHpOTVREazZUWkNwUE43OEQxMFJYajZnU3JhaWFKOEt1MVEtLTJYdlg5YnVUUnE3WnFnN0FoRDRJUFZlVEpNN2pCaWFpSEQ5NmlIM2hoQ2VDcHNHRHpTcWpiQ1RCVFRPbDd2cExKOF9adGxta2FWMUN1NjRvamQ0QUpYcFBUM2hSZkk4YWVibw?oc=5</t>
+        </is>
+      </c>
+      <c r="W336" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally - TradingView</t>
+        </is>
+      </c>
+      <c r="X336" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOcEVXNVpEUFAyU1hJbU1QMk1PYVBBSUNoRmRZMTR0d1Bib2FHeFEwS1N4QXpTLXVva3VXYTh6TG1Wd0Y5NnQ4ZGprUC1hR0d4eWc0TmUyR3lRN0xfX3YwRlpic0hmSU82RTZtZnRudXRlNzBkclZaTW1kNGFURDdac29ZX09obU9OWjRBVXoyRHc2R2ZVbTc5dFZYdlhXc0tqZGhJUUszampxSVMwWENrbk1abUtMemVnbHFpVA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y336" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z336" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA336" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB336" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC336" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD336" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-09-26T09:13:52+00:00</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E337" t="n">
+        <v>83918.35159999999</v>
+      </c>
+      <c r="F337" t="n">
+        <v>84323.7031</v>
+      </c>
+      <c r="G337" t="n">
+        <v>83867.52340000001</v>
+      </c>
+      <c r="H337" t="n">
+        <v>83993.97659999999</v>
+      </c>
+      <c r="I337" t="n">
+        <v>177268736</v>
+      </c>
+      <c r="J337" t="n">
+        <v>4</v>
+      </c>
+      <c r="K337" t="n">
+        <v>38</v>
+      </c>
+      <c r="L337" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="M337" t="n">
+        <v>0.183</v>
+      </c>
+      <c r="N337" t="n">
+        <v>35</v>
+      </c>
+      <c r="O337" t="n">
+        <v>0.431</v>
+      </c>
+      <c r="P337" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="Q337" t="n">
+        <v>10.467</v>
+      </c>
+      <c r="R337" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S337" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="T337" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U337" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="V337" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="W337" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="X337" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y337" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="Z337" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AA337" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - global.morningstar.com</t>
+        </is>
+      </c>
+      <c r="AB337" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC337" t="inlineStr">
+        <is>
+          <t>Bitcoin Price LIVE: JGB Sell-Off Puts $81,178 in Focus as BTC Breaks $84,304 Equilibrium - CryptoRank</t>
+        </is>
+      </c>
+      <c r="AD337" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPVExlTUQtSEl1aUFtdjc4Y0s3b2dXT2xjTHY3ODB5REY4d2JGa21kZ2VORmMxQ25kMHNKQ2JrR25COS1Ia1dXMWNVbmcxaE9RNlFuR19teDNPbEwzOVFBREoySHV2Xzg2czN3VVdyaXFWWlpGQXBkaHRNT05xZWhKU012RFpTZWpkd2tBdWNidG5YNlJQeGRiTVZUR2NJYUViVHNqM3FILVIzeHdabUxSNnpfa1U5XzhjQXZfRTFR?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-26 15:59 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD337"/>
+  <dimension ref="A1:AD343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42437,6 +42437,762 @@
       <c r="AD337" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPVExlTUQtSEl1aUFtdjc4Y0s3b2dXT2xjTHY3ODB5REY4d2JGa21kZ2VORmMxQ25kMHNKQ2JrR25COS1Ia1dXMWNVbmcxaE9RNlFuR19teDNPbEwzOVFBREoySHV2Xzg2czN3VVdyaXFWWlpGQXBkaHRNT05xZWhKU012RFpTZWpkd2tBdWNidG5YNlJQeGRiTVZUR2NJYUViVHNqM3FILVIzeHdabUxSNnpfa1U5XzhjQXZfRTFR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-09-26T15:57:49+00:00</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E338" t="n">
+        <v>4321.6001</v>
+      </c>
+      <c r="F338" t="n">
+        <v>4332.3999</v>
+      </c>
+      <c r="G338" t="n">
+        <v>4314.5</v>
+      </c>
+      <c r="H338" t="n">
+        <v>4321.2002</v>
+      </c>
+      <c r="I338" t="n">
+        <v>17239</v>
+      </c>
+      <c r="J338" t="n">
+        <v>4</v>
+      </c>
+      <c r="K338" t="n">
+        <v>39</v>
+      </c>
+      <c r="L338" t="n">
+        <v>-0.195</v>
+      </c>
+      <c r="M338" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="N338" t="n">
+        <v>40</v>
+      </c>
+      <c r="O338" t="n">
+        <v>-0.033</v>
+      </c>
+      <c r="P338" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="Q338" t="n">
+        <v>-4.971</v>
+      </c>
+      <c r="R338" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S338" t="inlineStr">
+        <is>
+          <t>Gold Q4 2026 outlook: Resilience in the face of rallying dollar and yields - FOREX.com</t>
+        </is>
+      </c>
+      <c r="T338" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPUk9TLVFNaXZQZXZINE1scGhtYk9IRVB0a2Z4SnoxT1dwN1B3V3M2WUpubFIyZk9CcmwyVGNxd09LRFZLRGhuQnFpSjgxbUJHYUM1ME40LU5ZTjFSZmh2NncyUHF5MEdwcW84dXUwOU9XR20wYmRXZTFNb1N3LUtZdEpIOENoTU01Uno1OGIweXZHcnR5cDM3TTF0X19xa05ROW5mVXlnNElaRXRRcGxPdUh1NnB4SzUtZUd0dA?oc=5</t>
+        </is>
+      </c>
+      <c r="U338" t="inlineStr">
+        <is>
+          <t>Precious Metals Surge: Gold Approaches $4,500 Mark, Silver Reclaims $66 - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="V338" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAxTUhJVFR3RXFNV3VTVFBNTl9OUXhvNmx6R01EZjFqSW05UWJjN3JIUGltNUNobFJKazVGR0lhb1J2bS1iRDdSeC1Fa0YtNU1BQi1xM1hnVjhaZklSUjFpU0ZHWV9GOHlncUtZMmtKTzRxQV8zM2c?oc=5</t>
+        </is>
+      </c>
+      <c r="W338" t="inlineStr">
+        <is>
+          <t>Gold rises above $4,130 as geopolitical uncertainty supports safe-haven demand - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X338" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPVC0wdnlpU1I2eWVTbnhmbHhvdFBmWUM4c3J4dk9NZFVBMGZBOVBJall6QmY2UkxxTm15TS1ycGs1ZW42RFFNaWdiUlJuajNKWmhOZ0sxYWlOSUZpcTAySkV3NHhST0dGRVZtVmVVVmt4WFFja2hjOW1RVVF5UFdGaUxaOXhOSTUwX21ab1FQQlh4dE0yOUVn?oc=5</t>
+        </is>
+      </c>
+      <c r="Y338" t="inlineStr">
+        <is>
+          <t>First-half gold ETF flows remained positive – World Gold Council - Mining Weekly</t>
+        </is>
+      </c>
+      <c r="Z338" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQMVFWRF9NZVpGV2M1dlNDd1FuTVRkYTdZTXpVUlhHdmVBOW1MN1BMZzZWSzB6b2VjeW5UaWJUUFdqUXJ0U2U5QUxXTGM1SmY4aDhtczgwRTFzNWJpZ2dDLWFrZVNwRndDaW1SdWlBdzVzMEJnZW1uSjBRQlpyV0l4cWpSbUdsd0V4MFBvbTFtNTJLZ01ncUR6am8wRE01cHFvcHcxN1lPdnhjSTZOb2hB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA338" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AB338" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC338" t="inlineStr">
+        <is>
+          <t>Gold breaks below key MAs, eyes $4,260 support: Live levels - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD338" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPME13WGVlVjFRRTNPak02V1FBTDZVR25FMHh5Yjc5NWZqZUZfZ3pyUjRxTU5HcWRDS1I3RVRQQ0V0eTZOZmMxMk9aMlc1WGsyd0FPQzU3ZzlMSUp4cVFBSUR6ZkJucl9WSTNlRWRPdHlxY1o1emxISC10OXJib2tlaV80RGpxaW9hR3BydHhPOVNMdFFDSDd1c3RzVGc1MmJpNm1WTDkySUplMkZyZks2bQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-09-26T15:57:49+00:00</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E339" t="n">
+        <v>92.23999999999999</v>
+      </c>
+      <c r="F339" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="G339" t="n">
+        <v>91.81999999999999</v>
+      </c>
+      <c r="H339" t="n">
+        <v>92.41</v>
+      </c>
+      <c r="I339" t="n">
+        <v>72759</v>
+      </c>
+      <c r="J339" t="n">
+        <v>4</v>
+      </c>
+      <c r="K339" t="n">
+        <v>40</v>
+      </c>
+      <c r="L339" t="n">
+        <v>-0.136</v>
+      </c>
+      <c r="M339" t="n">
+        <v>-0.182</v>
+      </c>
+      <c r="N339" t="n">
+        <v>40</v>
+      </c>
+      <c r="O339" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="P339" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="Q339" t="n">
+        <v>2.144</v>
+      </c>
+      <c r="R339" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S339" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T339" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U339" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V339" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W339" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X339" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y339" t="inlineStr">
+        <is>
+          <t>OPEC Monthly Oil Market Report, September 2026 - Peak Oil Barrel</t>
+        </is>
+      </c>
+      <c r="Z339" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9faVVpVXlFX1hFRG4tM2FnZTE5Q1ROMG1RWmxCTWVWcTdLcmo0VlBIbTlQcnhYOUQxeUxvaTE4VVo5Ulo3cExYYVViZUxWcU9VUzRIRXhQRTJLb19hWFhJc2V5WkxmMGhtSk92QVJndFZlV1NQeWxkM2Z3WWc?oc=5</t>
+        </is>
+      </c>
+      <c r="AA339" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AB339" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC339" t="inlineStr">
+        <is>
+          <t>nano Crude Oil Fut (Jan 2027) Trade Ideas — COINBASE:NOLF2027 - TradingView</t>
+        </is>
+      </c>
+      <c r="AD339" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNc1BOTkRSU0FuQ1IyRE5kUGJzb2V4Mnl1SW5JYVZVWEV0WGZPT1BQN3BEbHpFNU1SQUhMbUdmM04tZG5fbkVMb2hmeDE1M0lIUUd6cHhSdWU2VExUSEJZc3YzY2pNUXFpTUNlNm5Pd2wydU1lU0Ztb1UzT2ZLaUx2SFhWQ2dJQ25QR0E?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-09-26T15:57:49+00:00</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E340" t="n">
+        <v>101.022</v>
+      </c>
+      <c r="F340" t="n">
+        <v>101.077</v>
+      </c>
+      <c r="G340" t="n">
+        <v>100.954</v>
+      </c>
+      <c r="H340" t="n">
+        <v>101.035</v>
+      </c>
+      <c r="I340" t="n">
+        <v>0</v>
+      </c>
+      <c r="J340" t="n">
+        <v>4</v>
+      </c>
+      <c r="K340" t="n">
+        <v>40</v>
+      </c>
+      <c r="L340" t="n">
+        <v>-0.028</v>
+      </c>
+      <c r="M340" t="n">
+        <v>0.177</v>
+      </c>
+      <c r="N340" t="n">
+        <v>40</v>
+      </c>
+      <c r="O340" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="P340" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Q340" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="R340" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S340" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T340" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U340" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="V340" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="W340" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="X340" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y340" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z340" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA340" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ing think</t>
+        </is>
+      </c>
+      <c r="AB340" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC340" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD340" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-09-26T15:57:49+00:00</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E341" t="n">
+        <v>7795.25</v>
+      </c>
+      <c r="F341" t="n">
+        <v>7814.75</v>
+      </c>
+      <c r="G341" t="n">
+        <v>7793.25</v>
+      </c>
+      <c r="H341" t="n">
+        <v>7803.75</v>
+      </c>
+      <c r="I341" t="n">
+        <v>473791</v>
+      </c>
+      <c r="J341" t="n">
+        <v>4</v>
+      </c>
+      <c r="K341" t="n">
+        <v>39</v>
+      </c>
+      <c r="L341" t="n">
+        <v>-0.152</v>
+      </c>
+      <c r="M341" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="N341" t="n">
+        <v>40</v>
+      </c>
+      <c r="O341" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="P341" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="Q341" t="n">
+        <v>-0.6919999999999999</v>
+      </c>
+      <c r="R341" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S341" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T341" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U341" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V341" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W341" t="inlineStr">
+        <is>
+          <t>Stock market today: Dow hits record high, S&amp;P 500 and Nasdaq surge as Big Tech gains power rally - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X341" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPbkNnYmlpUUZ1UFBUdG13a1NLZlhpbXR4cEpMcUdqRkR5aXd1UjVKaEFFQTJyQ0JrQWFHN0I0Zk1wSDVOZ0RaRWM2aXpCb3BDQmE4c0dXaHFLQVhRcXdiZDZnSko3UGd6WlkwNlVncFNJdTVnbHVGaFJBTXltM0ttaUxkZ0ZFa2ptNVN5S3FTbXBPOTc3UHdZVEtVYVFqWXNMazVsZlhaY3hibzViazhyeXBta2RFWHF4Z1pN?oc=5</t>
+        </is>
+      </c>
+      <c r="Y341" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z341" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA341" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AB341" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC341" t="inlineStr">
+        <is>
+          <t>If There's a Stock Market Crash Ahead, History Highlights the Best Strategy for Investors - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="AD341" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOLUduUjZLVDVGbEVES2xrSENCZmxRUG5Dbmt0V1FlRWgtbmdMb2ZwdjExcjZTVExTMzJvMHd5X2NDUHlMamFZZWJOT0FJZTI0ZUc2eHBwakt5Uzc1UU52NEJVNERGS0E5M3NmMFBUbkFaeDZDNHBrb29tMmhmNUJuWW0wRzhmcG4yZ2t0ZmpoOEFhWUgtMWc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-09-26T15:57:49+00:00</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E342" t="n">
+        <v>30912</v>
+      </c>
+      <c r="F342" t="n">
+        <v>30935</v>
+      </c>
+      <c r="G342" t="n">
+        <v>30845</v>
+      </c>
+      <c r="H342" t="n">
+        <v>30889.25</v>
+      </c>
+      <c r="I342" t="n">
+        <v>83633</v>
+      </c>
+      <c r="J342" t="n">
+        <v>4</v>
+      </c>
+      <c r="K342" t="n">
+        <v>34</v>
+      </c>
+      <c r="L342" t="n">
+        <v>-0.126</v>
+      </c>
+      <c r="M342" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="N342" t="n">
+        <v>34</v>
+      </c>
+      <c r="O342" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="P342" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="Q342" t="n">
+        <v>1.239</v>
+      </c>
+      <c r="R342" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S342" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally (AMD:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T342" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNRTNUV0JnS3haREZESHpOTVREazZUWkNwUE43OEQxMFJYajZnU3JhaWFKOEt1MVEtLTJYdlg5YnVUUnE3WnFnN0FoRDRJUFZlVEpNN2pCaWFpSEQ5NmlIM2hoQ2VDcHNHRHpTcWpiQ1RCVFRPbDd2cExKOF9adGxta2FWMUN1NjRvamQ0QUpYcFBUM2hSZkk4YWVibw?oc=5</t>
+        </is>
+      </c>
+      <c r="U342" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="V342" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W342" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="X342" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y342" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z342" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA342" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB342" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC342" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD342" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-09-26T15:57:49+00:00</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E343" t="n">
+        <v>84158.82030000001</v>
+      </c>
+      <c r="F343" t="n">
+        <v>84190.4688</v>
+      </c>
+      <c r="G343" t="n">
+        <v>83846.39840000001</v>
+      </c>
+      <c r="H343" t="n">
+        <v>84145.39840000001</v>
+      </c>
+      <c r="I343" t="n">
+        <v>39250944</v>
+      </c>
+      <c r="J343" t="n">
+        <v>4</v>
+      </c>
+      <c r="K343" t="n">
+        <v>37</v>
+      </c>
+      <c r="L343" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="M343" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="N343" t="n">
+        <v>36</v>
+      </c>
+      <c r="O343" t="n">
+        <v>0.419</v>
+      </c>
+      <c r="P343" t="n">
+        <v>-0.079</v>
+      </c>
+      <c r="Q343" t="n">
+        <v>10.154</v>
+      </c>
+      <c r="R343" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S343" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="T343" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U343" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="V343" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="W343" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="X343" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y343" t="inlineStr">
+        <is>
+          <t>Bitcoin Price LIVE: JGB Sell-Off Puts $81,178 in Focus as BTC Breaks $84,304 Equilibrium - CryptoRank</t>
+        </is>
+      </c>
+      <c r="Z343" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPVExlTUQtSEl1aUFtdjc4Y0s3b2dXT2xjTHY3ODB5REY4d2JGa21kZ2VORmMxQ25kMHNKQ2JrR25COS1Ia1dXMWNVbmcxaE9RNlFuR19teDNPbEwzOVFBREoySHV2Xzg2czN3VVdyaXFWWlpGQXBkaHRNT05xZWhKU012RFpTZWpkd2tBdWNidG5YNlJQeGRiTVZUR2NJYUViVHNqM3FILVIzeHdabUxSNnpfa1U5XzhjQXZfRTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA343" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - bitcoinmagazine.com</t>
+        </is>
+      </c>
+      <c r="AB343" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AC343" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - Morningstar</t>
+        </is>
+      </c>
+      <c r="AD343" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-26 19:08 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD343"/>
+  <dimension ref="A1:AD349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43191,6 +43191,762 @@
         </is>
       </c>
       <c r="AD343" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-09-26T19:06:01+00:00</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E344" t="n">
+        <v>4321.6001</v>
+      </c>
+      <c r="F344" t="n">
+        <v>4332.3999</v>
+      </c>
+      <c r="G344" t="n">
+        <v>4314.5</v>
+      </c>
+      <c r="H344" t="n">
+        <v>4321.2002</v>
+      </c>
+      <c r="I344" t="n">
+        <v>17239</v>
+      </c>
+      <c r="J344" t="n">
+        <v>4</v>
+      </c>
+      <c r="K344" t="n">
+        <v>39</v>
+      </c>
+      <c r="L344" t="n">
+        <v>-0.192</v>
+      </c>
+      <c r="M344" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="N344" t="n">
+        <v>40</v>
+      </c>
+      <c r="O344" t="n">
+        <v>-0.018</v>
+      </c>
+      <c r="P344" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="Q344" t="n">
+        <v>-4.589</v>
+      </c>
+      <c r="R344" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S344" t="inlineStr">
+        <is>
+          <t>Lundin Gold Hits Record Grade at Bonza Sur With 204 g/t Gold Over 3 Metres Intercept - the deep dive</t>
+        </is>
+      </c>
+      <c r="T344" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNaDdPLWtTOVlMN0c3OWFFWmF1dUZfT28xLWducTQyQVo5XzRUZzU5YWxUZ1JlZzZqcHRtcG5FUENMZE9LN1ZEQXdpTDBMa3c2Ry1aakpaMjBtTlV6bTNDenB4d2d1OEltQmxadjVsTHFWY0J5alI2Sko2YVdfa1VHZDd3bGVtdUlOaXVaZU0xcFo0UHBjNXZTX2dKS1dtX1J5d2JBX2NxSW9TMS1P?oc=5</t>
+        </is>
+      </c>
+      <c r="U344" t="inlineStr">
+        <is>
+          <t>Gold price will hit $4,900/oz in 2026 on strong sovereign demand as China buys 75% more than reported in July – Goldman Sachs - Kitco</t>
+        </is>
+      </c>
+      <c r="V344" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOdmIweWNUQkhQS0N4SVhSTjEzWjBlUU9IX2Vxa2c4cGVvM1RQN3BqRkVRWFBYSHAzdFNqcmdYSFhVWUViVWV5Wmp6cHhERHVOSHNnbTcxYnlaaFZ1Y3lsOWpWRDdxbUR4ZDNlRVlQWEZERkhuLWZaT0VxRkhEamE3QmRGMDNvX3Z1VlVPNnczTFBWbEhlbEZqMkZJYTRsM2FKSXpkWUJIbkVUcGtwaXdwRUUxbDBHTFJ1ZmpjZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W344" t="inlineStr">
+        <is>
+          <t>Precious Metals Surge: Gold Approaches $4,500 Mark, Silver Reclaims $66 - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="X344" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAxTUhJVFR3RXFNV3VTVFBNTl9OUXhvNmx6R01EZjFqSW05UWJjN3JIUGltNUNobFJKazVGR0lhb1J2bS1iRDdSeC1Fa0YtNU1BQi1xM1hnVjhaZklSUjFpU0ZHWV9GOHlncUtZMmtKTzRxQV8zM2c?oc=5</t>
+        </is>
+      </c>
+      <c r="Y344" t="inlineStr">
+        <is>
+          <t>First-half gold ETF flows remained positive – World Gold Council - Mining Weekly</t>
+        </is>
+      </c>
+      <c r="Z344" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQMVFWRF9NZVpGV2M1dlNDd1FuTVRkYTdZTXpVUlhHdmVBOW1MN1BMZzZWSzB6b2VjeW5UaWJUUFdqUXJ0U2U5QUxXTGM1SmY4aDhtczgwRTFzNWJpZ2dDLWFrZVNwRndDaW1SdWlBdzVzMEJnZW1uSjBRQlpyV0l4cWpSbUdsd0V4MFBvbTFtNTJLZ01ncUR6am8wRE01cHFvcHcxN1lPdnhjSTZOb2hB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA344" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AB344" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC344" t="inlineStr">
+        <is>
+          <t>Gold breaks below key MAs, eyes $4,260 support: Live levels - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD344" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPME13WGVlVjFRRTNPak02V1FBTDZVR25FMHh5Yjc5NWZqZUZfZ3pyUjRxTU5HcWRDS1I3RVRQQ0V0eTZOZmMxMk9aMlc1WGsyd0FPQzU3ZzlMSUp4cVFBSUR6ZkJucl9WSTNlRWRPdHlxY1o1emxISC10OXJib2tlaV80RGpxaW9hR3BydHhPOVNMdFFDSDd1c3RzVGc1MmJpNm1WTDkySUplMkZyZks2bQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-09-26T19:06:01+00:00</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E345" t="n">
+        <v>92.23999999999999</v>
+      </c>
+      <c r="F345" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="G345" t="n">
+        <v>91.81999999999999</v>
+      </c>
+      <c r="H345" t="n">
+        <v>92.41</v>
+      </c>
+      <c r="I345" t="n">
+        <v>72759</v>
+      </c>
+      <c r="J345" t="n">
+        <v>4</v>
+      </c>
+      <c r="K345" t="n">
+        <v>40</v>
+      </c>
+      <c r="L345" t="n">
+        <v>-0.092</v>
+      </c>
+      <c r="M345" t="n">
+        <v>-0.161</v>
+      </c>
+      <c r="N345" t="n">
+        <v>40</v>
+      </c>
+      <c r="O345" t="n">
+        <v>0.219</v>
+      </c>
+      <c r="P345" t="n">
+        <v>-0.127</v>
+      </c>
+      <c r="Q345" t="n">
+        <v>2.541</v>
+      </c>
+      <c r="R345" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S345" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T345" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U345" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V345" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W345" t="inlineStr">
+        <is>
+          <t>Oil prices surge 15% as Strait of Hormuz disruptions tighten supply - offshore-technology.com</t>
+        </is>
+      </c>
+      <c r="X345" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPdndjemtyTkduUUpSVnR6aXJUNXBBR0JNd1FaaURNWmtvWm9WTkZUME50Qk1NVDUtdEtqcWE2R0xvUGRKNHBWZDMtblpaY1h1TE5zcmgycU5kS29mYU02N1BOdThBMUhUMDM0T1FScDZRY0JzYlRXTTJVajFYbkh3Rmp0MDFDeVZQcFhKSjhpaklySjZrVWJCZVoyWkw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y345" t="inlineStr">
+        <is>
+          <t>OPEC Monthly Oil Market Report, September 2026 - Peak Oil Barrel</t>
+        </is>
+      </c>
+      <c r="Z345" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9faVVpVXlFX1hFRG4tM2FnZTE5Q1ROMG1RWmxCTWVWcTdLcmo0VlBIbTlQcnhYOUQxeUxvaTE4VVo5Ulo3cExYYVViZUxWcU9VUzRIRXhQRTJLb19hWFhJc2V5WkxmMGhtSk92QVJndFZlV1NQeWxkM2Z3WWc?oc=5</t>
+        </is>
+      </c>
+      <c r="AA345" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AB345" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC345" t="inlineStr">
+        <is>
+          <t>nano Crude Oil Fut (Jan 2027) Trade Ideas — COINBASE:NOLF2027 - TradingView</t>
+        </is>
+      </c>
+      <c r="AD345" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNc1BOTkRSU0FuQ1IyRE5kUGJzb2V4Mnl1SW5JYVZVWEV0WGZPT1BQN3BEbHpFNU1SQUhMbUdmM04tZG5fbkVMb2hmeDE1M0lIUUd6cHhSdWU2VExUSEJZc3YzY2pNUXFpTUNlNm5Pd2wydU1lU0Ztb1UzT2ZLaUx2SFhWQ2dJQ25QR0E?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-09-26T19:06:01+00:00</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E346" t="n">
+        <v>101.022</v>
+      </c>
+      <c r="F346" t="n">
+        <v>101.077</v>
+      </c>
+      <c r="G346" t="n">
+        <v>100.954</v>
+      </c>
+      <c r="H346" t="n">
+        <v>101.035</v>
+      </c>
+      <c r="I346" t="n">
+        <v>0</v>
+      </c>
+      <c r="J346" t="n">
+        <v>4</v>
+      </c>
+      <c r="K346" t="n">
+        <v>39</v>
+      </c>
+      <c r="L346" t="n">
+        <v>-0.053</v>
+      </c>
+      <c r="M346" t="n">
+        <v>0.203</v>
+      </c>
+      <c r="N346" t="n">
+        <v>40</v>
+      </c>
+      <c r="O346" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="P346" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="Q346" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="R346" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S346" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T346" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U346" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="V346" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="W346" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="X346" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y346" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z346" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA346" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ing think</t>
+        </is>
+      </c>
+      <c r="AB346" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC346" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD346" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-09-26T19:06:01+00:00</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E347" t="n">
+        <v>7795.25</v>
+      </c>
+      <c r="F347" t="n">
+        <v>7814.75</v>
+      </c>
+      <c r="G347" t="n">
+        <v>7793.25</v>
+      </c>
+      <c r="H347" t="n">
+        <v>7803.75</v>
+      </c>
+      <c r="I347" t="n">
+        <v>473791</v>
+      </c>
+      <c r="J347" t="n">
+        <v>4</v>
+      </c>
+      <c r="K347" t="n">
+        <v>40</v>
+      </c>
+      <c r="L347" t="n">
+        <v>-0.233</v>
+      </c>
+      <c r="M347" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="N347" t="n">
+        <v>40</v>
+      </c>
+      <c r="O347" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="P347" t="n">
+        <v>-0.033</v>
+      </c>
+      <c r="Q347" t="n">
+        <v>-1.158</v>
+      </c>
+      <c r="R347" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S347" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T347" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U347" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V347" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W347" t="inlineStr">
+        <is>
+          <t>AbCellera Biologics (ABCL) Surges 34.78% as Shares Break Toward $9.81 Resistance - EMA Signal - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="X347" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPdUNOZndBWm5IMm9JRjRsTk5DNmtNQnR6YTFWMWlSTk5BT3J2TjNEdXlrMFl5Vi1sdDVyY1BybUlUU0taSnQtcktxZEV5ZkpYclc4dnBNa0lzamY3dFFRTGNMWXU5TFk3MUphb1hnak4zYS1vQ0s2NHdTeFFLOGEwdlRkcGE5VUs4a0t2bnk3SkJPMGk2RGM4VV9mclUwZmJQMGUtNXN0dUN5Z2M1U1E0cG5pckZOQlJ2TGdDSg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y347" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z347" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA347" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AB347" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC347" t="inlineStr">
+        <is>
+          <t>If There's a Stock Market Crash Ahead, History Highlights the Best Strategy for Investors - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="AD347" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOLUduUjZLVDVGbEVES2xrSENCZmxRUG5Dbmt0V1FlRWgtbmdMb2ZwdjExcjZTVExTMzJvMHd5X2NDUHlMamFZZWJOT0FJZTI0ZUc2eHBwakt5Uzc1UU52NEJVNERGS0E5M3NmMFBUbkFaeDZDNHBrb29tMmhmNUJuWW0wRzhmcG4yZ2t0ZmpoOEFhWUgtMWc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-09-26T19:06:01+00:00</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E348" t="n">
+        <v>30912</v>
+      </c>
+      <c r="F348" t="n">
+        <v>30935</v>
+      </c>
+      <c r="G348" t="n">
+        <v>30845</v>
+      </c>
+      <c r="H348" t="n">
+        <v>30889.25</v>
+      </c>
+      <c r="I348" t="n">
+        <v>83633</v>
+      </c>
+      <c r="J348" t="n">
+        <v>4</v>
+      </c>
+      <c r="K348" t="n">
+        <v>35</v>
+      </c>
+      <c r="L348" t="n">
+        <v>-0.031</v>
+      </c>
+      <c r="M348" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="N348" t="n">
+        <v>33</v>
+      </c>
+      <c r="O348" t="n">
+        <v>0.269</v>
+      </c>
+      <c r="P348" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="Q348" t="n">
+        <v>4.894</v>
+      </c>
+      <c r="R348" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S348" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally (AMD:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T348" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNRTNUV0JnS3haREZESHpOTVREazZUWkNwUE43OEQxMFJYajZnU3JhaWFKOEt1MVEtLTJYdlg5YnVUUnE3WnFnN0FoRDRJUFZlVEpNN2pCaWFpSEQ5NmlIM2hoQ2VDcHNHRHpTcWpiQ1RCVFRPbDd2cExKOF9adGxta2FWMUN1NjRvamQ0QUpYcFBUM2hSZkk4YWVibw?oc=5</t>
+        </is>
+      </c>
+      <c r="U348" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - staradvertiser.com</t>
+        </is>
+      </c>
+      <c r="V348" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W348" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="X348" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y348" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z348" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA348" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB348" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC348" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD348" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-09-26T19:06:01+00:00</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E349" t="n">
+        <v>84150.32030000001</v>
+      </c>
+      <c r="F349" t="n">
+        <v>84156.49219999999</v>
+      </c>
+      <c r="G349" t="n">
+        <v>83967.61719999999</v>
+      </c>
+      <c r="H349" t="n">
+        <v>84015.89840000001</v>
+      </c>
+      <c r="I349" t="n">
+        <v>257557504</v>
+      </c>
+      <c r="J349" t="n">
+        <v>4</v>
+      </c>
+      <c r="K349" t="n">
+        <v>38</v>
+      </c>
+      <c r="L349" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="M349" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="N349" t="n">
+        <v>35</v>
+      </c>
+      <c r="O349" t="n">
+        <v>0.454</v>
+      </c>
+      <c r="P349" t="n">
+        <v>-0.079</v>
+      </c>
+      <c r="Q349" t="n">
+        <v>11.563</v>
+      </c>
+      <c r="R349" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S349" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="T349" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U349" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="V349" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="W349" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="X349" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y349" t="inlineStr">
+        <is>
+          <t>Bitcoin Price LIVE: JGB Sell-Off Puts $81,178 in Focus as BTC Breaks $84,304 Equilibrium - CryptoRank</t>
+        </is>
+      </c>
+      <c r="Z349" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPVExlTUQtSEl1aUFtdjc4Y0s3b2dXT2xjTHY3ODB5REY4d2JGa21kZ2VORmMxQ25kMHNKQ2JrR25COS1Ia1dXMWNVbmcxaE9RNlFuR19teDNPbEwzOVFBREoySHV2Xzg2czN3VVdyaXFWWlpGQXBkaHRNT05xZWhKU012RFpTZWpkd2tBdWNidG5YNlJQeGRiTVZUR2NJYUViVHNqM3FILVIzeHdabUxSNnpfa1U5XzhjQXZfRTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AA349" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - bitcoinmagazine.com</t>
+        </is>
+      </c>
+      <c r="AB349" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AC349" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - Morningstar</t>
+        </is>
+      </c>
+      <c r="AD349" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-26 22:29 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD349"/>
+  <dimension ref="A1:AD355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43947,6 +43947,762 @@
         </is>
       </c>
       <c r="AD349" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-09-26T22:26:57+00:00</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E350" t="n">
+        <v>4321.6001</v>
+      </c>
+      <c r="F350" t="n">
+        <v>4332.3999</v>
+      </c>
+      <c r="G350" t="n">
+        <v>4314.5</v>
+      </c>
+      <c r="H350" t="n">
+        <v>4321.2002</v>
+      </c>
+      <c r="I350" t="n">
+        <v>17239</v>
+      </c>
+      <c r="J350" t="n">
+        <v>4</v>
+      </c>
+      <c r="K350" t="n">
+        <v>39</v>
+      </c>
+      <c r="L350" t="n">
+        <v>-0.103</v>
+      </c>
+      <c r="M350" t="n">
+        <v>-0.011</v>
+      </c>
+      <c r="N350" t="n">
+        <v>40</v>
+      </c>
+      <c r="O350" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="P350" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="Q350" t="n">
+        <v>-2.631</v>
+      </c>
+      <c r="R350" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S350" t="inlineStr">
+        <is>
+          <t>Lundin Gold Hits Record Grade at Bonza Sur With 204 g/t Gold Over 3 Metres Intercept - the deep dive</t>
+        </is>
+      </c>
+      <c r="T350" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNaDdPLWtTOVlMN0c3OWFFWmF1dUZfT28xLWducTQyQVo5XzRUZzU5YWxUZ1JlZzZqcHRtcG5FUENMZE9LN1ZEQXdpTDBMa3c2Ry1aakpaMjBtTlV6bTNDenB4d2d1OEltQmxadjVsTHFWY0J5alI2Sko2YVdfa1VHZDd3bGVtdUlOaXVaZU0xcFo0UHBjNXZTX2dKS1dtX1J5d2JBX2NxSW9TMS1P?oc=5</t>
+        </is>
+      </c>
+      <c r="U350" t="inlineStr">
+        <is>
+          <t>Precious Metals Surge: Gold Approaches $4,500 Mark, Silver Reclaims $66 - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="V350" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAxTUhJVFR3RXFNV3VTVFBNTl9OUXhvNmx6R01EZjFqSW05UWJjN3JIUGltNUNobFJKazVGR0lhb1J2bS1iRDdSeC1Fa0YtNU1BQi1xM1hnVjhaZklSUjFpU0ZHWV9GOHlncUtZMmtKTzRxQV8zM2c?oc=5</t>
+        </is>
+      </c>
+      <c r="W350" t="inlineStr">
+        <is>
+          <t>Gold rises above $4,130 as geopolitical uncertainty supports safe-haven demand - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X350" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPVC0wdnlpU1I2eWVTbnhmbHhvdFBmWUM4c3J4dk9NZFVBMGZBOVBJall6QmY2UkxxTm15TS1ycGs1ZW42RFFNaWdiUlJuajNKWmhOZ0sxYWlOSUZpcTAySkV3NHhST0dGRVZtVmVVVmt4WFFja2hjOW1RVVF5UFdGaUxaOXhOSTUwX21ab1FQQlh4dE0yOUVn?oc=5</t>
+        </is>
+      </c>
+      <c r="Y350" t="inlineStr">
+        <is>
+          <t>First-half gold ETF flows remained positive – World Gold Council - Mining Weekly</t>
+        </is>
+      </c>
+      <c r="Z350" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQMVFWRF9NZVpGV2M1dlNDd1FuTVRkYTdZTXpVUlhHdmVBOW1MN1BMZzZWSzB6b2VjeW5UaWJUUFdqUXJ0U2U5QUxXTGM1SmY4aDhtczgwRTFzNWJpZ2dDLWFrZVNwRndDaW1SdWlBdzVzMEJnZW1uSjBRQlpyV0l4cWpSbUdsd0V4MFBvbTFtNTJLZ01ncUR6am8wRE01cHFvcHcxN1lPdnhjSTZOb2hB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA350" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AB350" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC350" t="inlineStr">
+        <is>
+          <t>Gold ETFs Shine in H1 2026 with Unprecedented Liquidity - investingnews.com</t>
+        </is>
+      </c>
+      <c r="AD350" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE1JaGRkaHpGODN4bGpQdFl6S3VyUjZKYzRvWUxjUjhyQ0lVXzZMZEltdGkwMEo2d0lhVWVmMDVUYUJfRXF4emdyX0ZTd0N6SVgwN3kxMFVXTkt5WXZJbE8ybVNRLUJYTVZy?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-09-26T22:26:57+00:00</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E351" t="n">
+        <v>92.23999999999999</v>
+      </c>
+      <c r="F351" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="G351" t="n">
+        <v>91.81999999999999</v>
+      </c>
+      <c r="H351" t="n">
+        <v>92.41</v>
+      </c>
+      <c r="I351" t="n">
+        <v>72759</v>
+      </c>
+      <c r="J351" t="n">
+        <v>4</v>
+      </c>
+      <c r="K351" t="n">
+        <v>40</v>
+      </c>
+      <c r="L351" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="M351" t="n">
+        <v>-0.161</v>
+      </c>
+      <c r="N351" t="n">
+        <v>40</v>
+      </c>
+      <c r="O351" t="n">
+        <v>0.254</v>
+      </c>
+      <c r="P351" t="n">
+        <v>-0.081</v>
+      </c>
+      <c r="Q351" t="n">
+        <v>3.272</v>
+      </c>
+      <c r="R351" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S351" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T351" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U351" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V351" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W351" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X351" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y351" t="inlineStr">
+        <is>
+          <t>OPEC Monthly Oil Market Report, September 2026 - Peak Oil Barrel</t>
+        </is>
+      </c>
+      <c r="Z351" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9faVVpVXlFX1hFRG4tM2FnZTE5Q1ROMG1RWmxCTWVWcTdLcmo0VlBIbTlQcnhYOUQxeUxvaTE4VVo5Ulo3cExYYVViZUxWcU9VUzRIRXhQRTJLb19hWFhJc2V5WkxmMGhtSk92QVJndFZlV1NQeWxkM2Z3WWc?oc=5</t>
+        </is>
+      </c>
+      <c r="AA351" t="inlineStr">
+        <is>
+          <t>nano Crude Oil Fut (Jan 2027) Trade Ideas — COINBASE:NOLF2027 - TradingView</t>
+        </is>
+      </c>
+      <c r="AB351" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNc1BOTkRSU0FuQ1IyRE5kUGJzb2V4Mnl1SW5JYVZVWEV0WGZPT1BQN3BEbHpFNU1SQUhMbUdmM04tZG5fbkVMb2hmeDE1M0lIUUd6cHhSdWU2VExUSEJZc3YzY2pNUXFpTUNlNm5Pd2wydU1lU0Ztb1UzT2ZLaUx2SFhWQ2dJQ25QR0E?oc=5</t>
+        </is>
+      </c>
+      <c r="AC351" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 25, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AD351" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9DVE10MHdQOXV3X0ZlbGNJS0J4ZXg2Tm1GSVVQcmdJVExmVUo5R2FPbjBDRVJ3eUZLeWd2SC1CVnZLUHNYZkx6M1NoNnFkMGpKUHFBZjh4clhDZDZlZ1Vmak5B?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-09-26T22:26:57+00:00</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E352" t="n">
+        <v>101.022</v>
+      </c>
+      <c r="F352" t="n">
+        <v>101.077</v>
+      </c>
+      <c r="G352" t="n">
+        <v>100.954</v>
+      </c>
+      <c r="H352" t="n">
+        <v>101.035</v>
+      </c>
+      <c r="I352" t="n">
+        <v>0</v>
+      </c>
+      <c r="J352" t="n">
+        <v>4</v>
+      </c>
+      <c r="K352" t="n">
+        <v>39</v>
+      </c>
+      <c r="L352" t="n">
+        <v>-0.054</v>
+      </c>
+      <c r="M352" t="n">
+        <v>0.203</v>
+      </c>
+      <c r="N352" t="n">
+        <v>40</v>
+      </c>
+      <c r="O352" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="P352" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="Q352" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="R352" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S352" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T352" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U352" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="V352" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="W352" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="X352" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y352" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z352" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA352" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ing think</t>
+        </is>
+      </c>
+      <c r="AB352" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC352" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD352" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-09-26T22:26:57+00:00</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E353" t="n">
+        <v>7795.25</v>
+      </c>
+      <c r="F353" t="n">
+        <v>7814.75</v>
+      </c>
+      <c r="G353" t="n">
+        <v>7793.25</v>
+      </c>
+      <c r="H353" t="n">
+        <v>7803.75</v>
+      </c>
+      <c r="I353" t="n">
+        <v>473791</v>
+      </c>
+      <c r="J353" t="n">
+        <v>4</v>
+      </c>
+      <c r="K353" t="n">
+        <v>40</v>
+      </c>
+      <c r="L353" t="n">
+        <v>-0.121</v>
+      </c>
+      <c r="M353" t="n">
+        <v>0.138</v>
+      </c>
+      <c r="N353" t="n">
+        <v>40</v>
+      </c>
+      <c r="O353" t="n">
+        <v>0.209</v>
+      </c>
+      <c r="P353" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="Q353" t="n">
+        <v>1.775</v>
+      </c>
+      <c r="R353" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S353" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T353" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U353" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V353" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W353" t="inlineStr">
+        <is>
+          <t>AbCellera Biologics (ABCL) Surges 34.78% as Shares Break Toward $9.81 Resistance - EMA Signal - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="X353" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPdUNOZndBWm5IMm9JRjRsTk5DNmtNQnR6YTFWMWlSTk5BT3J2TjNEdXlrMFl5Vi1sdDVyY1BybUlUU0taSnQtcktxZEV5ZkpYclc4dnBNa0lzamY3dFFRTGNMWXU5TFk3MUphb1hnak4zYS1vQ0s2NHdTeFFLOGEwdlRkcGE5VUs4a0t2bnk3SkJPMGk2RGM4VV9mclUwZmJQMGUtNXN0dUN5Z2M1U1E0cG5pckZOQlJ2TGdDSg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y353" t="inlineStr">
+        <is>
+          <t>If There's a Stock Market Crash Ahead, History Highlights the Best Strategy for Investors - AOL.com</t>
+        </is>
+      </c>
+      <c r="Z353" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxObDRyTS13c3JCdDU5NmNhU3g3NnlUNkpoamlFR1Fic09CTzltRV9zcS1fUUwzdG45dExiY3k3N2c2VnItZ2twWnBZNktPXzItSmRMRVBveS1GdWljRDFpTmtxN3c1OG41a1dhTzFwNU44WkpGTm5oNjMtdzVtaURxVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA353" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB353" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC353" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AD353" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-09-26T22:26:57+00:00</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E354" t="n">
+        <v>30912</v>
+      </c>
+      <c r="F354" t="n">
+        <v>30935</v>
+      </c>
+      <c r="G354" t="n">
+        <v>30845</v>
+      </c>
+      <c r="H354" t="n">
+        <v>30889.25</v>
+      </c>
+      <c r="I354" t="n">
+        <v>83633</v>
+      </c>
+      <c r="J354" t="n">
+        <v>4</v>
+      </c>
+      <c r="K354" t="n">
+        <v>35</v>
+      </c>
+      <c r="L354" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="M354" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="N354" t="n">
+        <v>34</v>
+      </c>
+      <c r="O354" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="P354" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="Q354" t="n">
+        <v>1.893</v>
+      </c>
+      <c r="R354" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S354" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="T354" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U354" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="V354" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="W354" t="inlineStr">
+        <is>
+          <t>Stock Market Split As Nasdaq Hits High, Dow Jones Slides Amid Surging Treasury Yields: Weekly Review - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="X354" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPMEdvdk5ZTHduYS1XYjZlUExBRFFIT0Z2aWVGVW9zdmNmdF9TUXkzQnJRcmxNbnd1U3BkbWpueU9lSk1XWFFFOXVGZl9XRHE0eHRjSW5OMlhqdHZ0WUh0RXd5UlZRQVNZa2o2Z3FuZHpMTnQ3M1NuQVpqczFvYVBhalF4VnFpNGNoSERFVkg5cHZTajJyenA1OHRlcFRrYnVqejcwdk1qby03WmVE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y354" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z354" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA354" t="inlineStr">
+        <is>
+          <t>Palantir Technologies (NASDAQ: PLTR) Stock Price Falls Against Market Trend As Analysts Hold Strong Buy Rating - foreignpolicyjournal.com</t>
+        </is>
+      </c>
+      <c r="AB354" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPMGF1R05yZm50ZU84bGZvYS1nVjBoTF9GQUxqaERwSXpkdVZ0MzkwcTV2UF9uRVF5S2hCTW5uU21BYjR1eTVhamUwU1JrV1lOVnBXcnQ2WXlJeTRxdVFGZHVWMzFPMnJnUmc5eHBtSkFZV255NVAwajN3WkJQQnVKTjBQUnM1VjZ5ZEthMlIwVFQwMlpZTmlIU1ZsWnAyeXVZeHVzeHdRdHRaNGtzN0dQQWNNUldNdkZBZktSNXIzS1JxLVZaNmdlMUx0MnZJeVZqaTZXdG1rVHFiTnZReDVUaWV6Y3RVOWdQekh3cg?oc=5</t>
+        </is>
+      </c>
+      <c r="AC354" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AD354" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-09-26T22:26:57+00:00</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E355" t="n">
+        <v>83994.63280000001</v>
+      </c>
+      <c r="F355" t="n">
+        <v>84394.6562</v>
+      </c>
+      <c r="G355" t="n">
+        <v>83814.07030000001</v>
+      </c>
+      <c r="H355" t="n">
+        <v>84328.24219999999</v>
+      </c>
+      <c r="I355" t="n">
+        <v>1286210560</v>
+      </c>
+      <c r="J355" t="n">
+        <v>4</v>
+      </c>
+      <c r="K355" t="n">
+        <v>38</v>
+      </c>
+      <c r="L355" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="M355" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="N355" t="n">
+        <v>35</v>
+      </c>
+      <c r="O355" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="P355" t="n">
+        <v>-0.08699999999999999</v>
+      </c>
+      <c r="Q355" t="n">
+        <v>10.984</v>
+      </c>
+      <c r="R355" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S355" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="T355" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U355" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="V355" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="W355" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="X355" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y355" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="Z355" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AA355" t="inlineStr">
+        <is>
+          <t>Bitcoin Price LIVE: JGB Sell-Off Puts $81,178 in Focus as BTC Breaks $84,304 Equilibrium - CryptoRank</t>
+        </is>
+      </c>
+      <c r="AB355" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPVExlTUQtSEl1aUFtdjc4Y0s3b2dXT2xjTHY3ODB5REY4d2JGa21kZ2VORmMxQ25kMHNKQ2JrR25COS1Ia1dXMWNVbmcxaE9RNlFuR19teDNPbEwzOVFBREoySHV2Xzg2czN3VVdyaXFWWlpGQXBkaHRNT05xZWhKU012RFpTZWpkd2tBdWNidG5YNlJQeGRiTVZUR2NJYUViVHNqM3FILVIzeHdabUxSNnpfa1U5XzhjQXZfRTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC355" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - Morningstar</t>
+        </is>
+      </c>
+      <c r="AD355" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-27 04:09 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD355"/>
+  <dimension ref="A1:AD361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44703,6 +44703,762 @@
         </is>
       </c>
       <c r="AD355" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-09-27T04:07:21+00:00</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E356" t="n">
+        <v>4321.6001</v>
+      </c>
+      <c r="F356" t="n">
+        <v>4332.3999</v>
+      </c>
+      <c r="G356" t="n">
+        <v>4314.5</v>
+      </c>
+      <c r="H356" t="n">
+        <v>4321.2002</v>
+      </c>
+      <c r="I356" t="n">
+        <v>17239</v>
+      </c>
+      <c r="J356" t="n">
+        <v>4</v>
+      </c>
+      <c r="K356" t="n">
+        <v>39</v>
+      </c>
+      <c r="L356" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="M356" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="N356" t="n">
+        <v>40</v>
+      </c>
+      <c r="O356" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="P356" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="Q356" t="n">
+        <v>-1.351</v>
+      </c>
+      <c r="R356" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S356" t="inlineStr">
+        <is>
+          <t>Precious Metals Surge: Gold Approaches $4,500 Mark, Silver Reclaims $66 - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="T356" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAxTUhJVFR3RXFNV3VTVFBNTl9OUXhvNmx6R01EZjFqSW05UWJjN3JIUGltNUNobFJKazVGR0lhb1J2bS1iRDdSeC1Fa0YtNU1BQi1xM1hnVjhaZklSUjFpU0ZHWV9GOHlncUtZMmtKTzRxQV8zM2c?oc=5</t>
+        </is>
+      </c>
+      <c r="U356" t="inlineStr">
+        <is>
+          <t>Gold hits record high as investors seek safety - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="V356" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVWt1Y1hBWG5uZFNjRUFtZHlqRUhfZGV6VzAtQ0tBT2VlVDVEZEJ2WHN0YndCcXRzSjNtVnFhUFZZZ2F4RFRxYkdsSF91eDk2MFl5R3JNWk1HREJjSVdhUE1uTTU1N1Z6Y2xfZzZCSDZ4YnhaT1czcWdXeHE3SjJBR2FqUm43Z0paUG5OVEdsWVdYYnZBWVHSAZsBQVVfeXFMTWh6VXlqZGZVbUl3SHVfQ195WFFveEVkLU9TU1RXMTZBdVhodU16UWxLLWVScDNsc2VGMThyT0RTTHB4SVNRYU1KWmRycHhnTEc0NTJ1RWgzdGc2Y0VkanR4QUtlUWFBSnB2cElORUltQk9XdWRLNXhKbU5jRUFqQVd6bG5YbURJakxhNTl3UEk4RzBaQzVJaVdRdFk?oc=5</t>
+        </is>
+      </c>
+      <c r="W356" t="inlineStr">
+        <is>
+          <t>Gold rises above $4,130 as geopolitical uncertainty supports safe-haven demand - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X356" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPVC0wdnlpU1I2eWVTbnhmbHhvdFBmWUM4c3J4dk9NZFVBMGZBOVBJall6QmY2UkxxTm15TS1ycGs1ZW42RFFNaWdiUlJuajNKWmhOZ0sxYWlOSUZpcTAySkV3NHhST0dGRVZtVmVVVmt4WFFja2hjOW1RVVF5UFdGaUxaOXhOSTUwX21ab1FQQlh4dE0yOUVn?oc=5</t>
+        </is>
+      </c>
+      <c r="Y356" t="inlineStr">
+        <is>
+          <t>First-half gold ETF flows remained positive – World Gold Council - miningweekly.com</t>
+        </is>
+      </c>
+      <c r="Z356" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQMVFWRF9NZVpGV2M1dlNDd1FuTVRkYTdZTXpVUlhHdmVBOW1MN1BMZzZWSzB6b2VjeW5UaWJUUFdqUXJ0U2U5QUxXTGM1SmY4aDhtczgwRTFzNWJpZ2dDLWFrZVNwRndDaW1SdWlBdzVzMEJnZW1uSjBRQlpyV0l4cWpSbUdsd0V4MFBvbTFtNTJLZ01ncUR6am8wRE01cHFvcHcxN1lPdnhjSTZOb2hB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA356" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - kitco.com</t>
+        </is>
+      </c>
+      <c r="AB356" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC356" t="inlineStr">
+        <is>
+          <t>Wall Street split on gold price path after drop below $4,300, Main Street maintains bullish majority as jobs take center stage - kitco.com</t>
+        </is>
+      </c>
+      <c r="AD356" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQbWtUQVJKczJHZ1lWRDRZUEpOc1JuMVJHNmxQR18wSFlJbWJaemlYMXozWXdJTXRxRDVzWWRnWVFobWJCWEZqdUVqa2VMemE3NlI0MDJKdVFBWkJ0a3NrZE01WEJ2NS1mVUhaLTJYNnM4MUdHNHlDTnhYa0JZdS1lN2Vqdk5YOUhhWlhkMXc3S3pFaURQeFVKUU9pbVN5cWYzY0FwdThESE1IQ2JMVEo3T2JZbw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-09-27T04:07:21+00:00</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E357" t="n">
+        <v>92.23999999999999</v>
+      </c>
+      <c r="F357" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="G357" t="n">
+        <v>91.81999999999999</v>
+      </c>
+      <c r="H357" t="n">
+        <v>92.41</v>
+      </c>
+      <c r="I357" t="n">
+        <v>72759</v>
+      </c>
+      <c r="J357" t="n">
+        <v>4</v>
+      </c>
+      <c r="K357" t="n">
+        <v>40</v>
+      </c>
+      <c r="L357" t="n">
+        <v>-0.055</v>
+      </c>
+      <c r="M357" t="n">
+        <v>-0.189</v>
+      </c>
+      <c r="N357" t="n">
+        <v>40</v>
+      </c>
+      <c r="O357" t="n">
+        <v>0.276</v>
+      </c>
+      <c r="P357" t="n">
+        <v>-0.101</v>
+      </c>
+      <c r="Q357" t="n">
+        <v>4.417</v>
+      </c>
+      <c r="R357" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S357" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T357" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U357" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="V357" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="W357" t="inlineStr">
+        <is>
+          <t>Europe's STOXX 600 rallies on tech, banks strength as oil prices retreat - Reuters</t>
+        </is>
+      </c>
+      <c r="X357" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNYWF0aU9mWUM0TjNtekhpT0I0NTM1RXoydldTZDlzNVM4Q0FnRXFCLTlaLUQxdEZfMS1qeU1XV0lsNHhvc09zMTBUQV9xVFhaakdCU196dW5sQ212UHdLVjVySHo5UWczV0dVS2dnY3d2Q2dTbWRkOWFRZ0g5aTlGaEtnQkFQcno2ZjdfdndQdGdSR1c3MjdEXzNCZlhRM216di1sdllQSl9OT3pkcWRSd3p3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y357" t="inlineStr">
+        <is>
+          <t>OPEC Monthly Oil Market Report, September 2026 - Peak Oil Barrel</t>
+        </is>
+      </c>
+      <c r="Z357" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9faVVpVXlFX1hFRG4tM2FnZTE5Q1ROMG1RWmxCTWVWcTdLcmo0VlBIbTlQcnhYOUQxeUxvaTE4VVo5Ulo3cExYYVViZUxWcU9VUzRIRXhQRTJLb19hWFhJc2V5WkxmMGhtSk92QVJndFZlV1NQeWxkM2Z3WWc?oc=5</t>
+        </is>
+      </c>
+      <c r="AA357" t="inlineStr">
+        <is>
+          <t>nano Crude Oil Fut (Jan 2027) Trade Ideas — COINBASE:NOLF2027 - TradingView</t>
+        </is>
+      </c>
+      <c r="AB357" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNc1BOTkRSU0FuQ1IyRE5kUGJzb2V4Mnl1SW5JYVZVWEV0WGZPT1BQN3BEbHpFNU1SQUhMbUdmM04tZG5fbkVMb2hmeDE1M0lIUUd6cHhSdWU2VExUSEJZc3YzY2pNUXFpTUNlNm5Pd2wydU1lU0Ztb1UzT2ZLaUx2SFhWQ2dJQ25QR0E?oc=5</t>
+        </is>
+      </c>
+      <c r="AC357" t="inlineStr">
+        <is>
+          <t>Current price of oil as of September 25, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AD357" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9DVE10MHdQOXV3X0ZlbGNJS0J4ZXg2Tm1GSVVQcmdJVExmVUo5R2FPbjBDRVJ3eUZLeWd2SC1CVnZLUHNYZkx6M1NoNnFkMGpKUHFBZjh4clhDZDZlZ1Vmak5B?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-09-27T04:07:21+00:00</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E358" t="n">
+        <v>101.022</v>
+      </c>
+      <c r="F358" t="n">
+        <v>101.077</v>
+      </c>
+      <c r="G358" t="n">
+        <v>100.954</v>
+      </c>
+      <c r="H358" t="n">
+        <v>101.035</v>
+      </c>
+      <c r="I358" t="n">
+        <v>0</v>
+      </c>
+      <c r="J358" t="n">
+        <v>4</v>
+      </c>
+      <c r="K358" t="n">
+        <v>40</v>
+      </c>
+      <c r="L358" t="n">
+        <v>-0.038</v>
+      </c>
+      <c r="M358" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="N358" t="n">
+        <v>40</v>
+      </c>
+      <c r="O358" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="P358" t="n">
+        <v>-0.005</v>
+      </c>
+      <c r="Q358" t="n">
+        <v>1.824</v>
+      </c>
+      <c r="R358" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S358" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T358" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U358" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="V358" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="W358" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="X358" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y358" t="inlineStr">
+        <is>
+          <t>A hawkish Fed and a dovish SNB are driving gains in USDCHF - marketpulse.com</t>
+        </is>
+      </c>
+      <c r="Z358" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNNDRQWG91elN3ajdjOGFCNWR2ZWg3dG93VFlWLW8xcExpSU80TE0tWHY4bzNTdllfLThVT1o1TnY5dmFlVkE0cGhlcWlsblQyVVFXRzdMSnJpcW9lNmxWbWU0eVRDOEYtVk5GYzFBSzBJS0VjYUVLRzI5T0N0UGc2QWd2WWxCc1dadlctb25ScjJLdmpZTGZ4d3BZNA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA358" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ing think</t>
+        </is>
+      </c>
+      <c r="AB358" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC358" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD358" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-09-27T04:07:21+00:00</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E359" t="n">
+        <v>7795.25</v>
+      </c>
+      <c r="F359" t="n">
+        <v>7814.75</v>
+      </c>
+      <c r="G359" t="n">
+        <v>7793.25</v>
+      </c>
+      <c r="H359" t="n">
+        <v>7803.75</v>
+      </c>
+      <c r="I359" t="n">
+        <v>473791</v>
+      </c>
+      <c r="J359" t="n">
+        <v>4</v>
+      </c>
+      <c r="K359" t="n">
+        <v>40</v>
+      </c>
+      <c r="L359" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="M359" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="N359" t="n">
+        <v>40</v>
+      </c>
+      <c r="O359" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="P359" t="n">
+        <v>-0.012</v>
+      </c>
+      <c r="Q359" t="n">
+        <v>2.004</v>
+      </c>
+      <c r="R359" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S359" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T359" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U359" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V359" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W359" t="inlineStr">
+        <is>
+          <t>AbCellera Biologics (ABCL) Surges 34.78% as Shares Break Toward $9.81 Resistance - EMA Signal - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="X359" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPdUNOZndBWm5IMm9JRjRsTk5DNmtNQnR6YTFWMWlSTk5BT3J2TjNEdXlrMFl5Vi1sdDVyY1BybUlUU0taSnQtcktxZEV5ZkpYclc4dnBNa0lzamY3dFFRTGNMWXU5TFk3MUphb1hnak4zYS1vQ0s2NHdTeFFLOGEwdlRkcGE5VUs4a0t2bnk3SkJPMGk2RGM4VV9mclUwZmJQMGUtNXN0dUN5Z2M1U1E0cG5pckZOQlJ2TGdDSg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y359" t="inlineStr">
+        <is>
+          <t>PolyPid (PYPD) Surges 7%: Biotech Stock Breaks Above Key Support Level - Retracement Entry - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="Z359" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQaklvOUYyZ2dSbXZCNEM1TU9LR3l6akk4bnZSZkhSSWNxYW5JWUZGcUttMDBBcENoc0Z4eEZpNmx3cDNwMDhSc0lDSlpIaVR2Zng2ZzZ0em5NOEd6cFJXMXpSdkhQbUlZb2hVTzd4bmJYM1B6R09XOU1raHFMUWdweDRKTVJFQU1RQy1PMmFWc0dJMVlXdGNyWVh3SV9wd0F6UFFrQ3A4Z1pyTjJhNGtldWdB?oc=5</t>
+        </is>
+      </c>
+      <c r="AA359" t="inlineStr">
+        <is>
+          <t>Wall Street split on gold price path after drop below $4,300, Main Street maintains bullish majority as jobs take center stage - kitco.com</t>
+        </is>
+      </c>
+      <c r="AB359" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQbWtUQVJKczJHZ1lWRDRZUEpOc1JuMVJHNmxQR18wSFlJbWJaemlYMXozWXdJTXRxRDVzWWRnWVFobWJCWEZqdUVqa2VMemE3NlI0MDJKdVFBWkJ0a3NrZE01WEJ2NS1mVUhaLTJYNnM4MUdHNHlDTnhYa0JZdS1lN2Vqdk5YOUhhWlhkMXc3S3pFaURQeFVKUU9pbVN5cWYzY0FwdThESE1IQ2JMVEo3T2JZbw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC359" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD359" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-09-27T04:07:21+00:00</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E360" t="n">
+        <v>30912</v>
+      </c>
+      <c r="F360" t="n">
+        <v>30935</v>
+      </c>
+      <c r="G360" t="n">
+        <v>30845</v>
+      </c>
+      <c r="H360" t="n">
+        <v>30889.25</v>
+      </c>
+      <c r="I360" t="n">
+        <v>83633</v>
+      </c>
+      <c r="J360" t="n">
+        <v>4</v>
+      </c>
+      <c r="K360" t="n">
+        <v>34</v>
+      </c>
+      <c r="L360" t="n">
+        <v>-0.208</v>
+      </c>
+      <c r="M360" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="N360" t="n">
+        <v>34</v>
+      </c>
+      <c r="O360" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="P360" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="Q360" t="n">
+        <v>0.627</v>
+      </c>
+      <c r="R360" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S360" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally (AMD:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T360" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNRTNUV0JnS3haREZESHpOTVREazZUWkNwUE43OEQxMFJYajZnU3JhaWFKOEt1MVEtLTJYdlg5YnVUUnE3WnFnN0FoRDRJUFZlVEpNN2pCaWFpSEQ5NmlIM2hoQ2VDcHNHRHpTcWpiQ1RCVFRPbDd2cExKOF9adGxta2FWMUN1NjRvamQ0QUpYcFBUM2hSZkk4YWVibw?oc=5</t>
+        </is>
+      </c>
+      <c r="U360" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as chipmakers fuel stock gains - Reuters</t>
+        </is>
+      </c>
+      <c r="V360" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQUUdXdXVKYkpsa2JoQmRNeVpVWWhwb1pIVmUwcUl0QVRFVEFjRDJtREJPbXJWaXVEc0NQSWZZUlhwTl80T3h4eGM1dE9oaXRsWlVueWx0MWt3YXlWbV9PYkZDWVVPb1ZveThvalZfWnBvQ2J5Sjg1UkNOQmU5eDdWN0FvVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W360" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="X360" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y360" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z360" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA360" t="inlineStr">
+        <is>
+          <t>Palantir Technologies (NASDAQ: PLTR) Stock Price Falls Against Market Trend As Analysts Hold Strong Buy Rating - foreignpolicyjournal.com</t>
+        </is>
+      </c>
+      <c r="AB360" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPMGF1R05yZm50ZU84bGZvYS1nVjBoTF9GQUxqaERwSXpkdVZ0MzkwcTV2UF9uRVF5S2hCTW5uU21BYjR1eTVhamUwU1JrV1lOVnBXcnQ2WXlJeTRxdVFGZHVWMzFPMnJnUmc5eHBtSkFZV255NVAwajN3WkJQQnVKTjBQUnM1VjZ5ZEthMlIwVFQwMlpZTmlIU1ZsWnAyeXVZeHVzeHdRdHRaNGtzN0dQQWNNUldNdkZBZktSNXIzS1JxLVZaNmdlMUx0MnZJeVZqaTZXdG1rVHFiTnZReDVUaWV6Y3RVOWdQekh3cg?oc=5</t>
+        </is>
+      </c>
+      <c r="AC360" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AD360" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-09-27T04:07:21+00:00</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E361" t="n">
+        <v>84291.21090000001</v>
+      </c>
+      <c r="F361" t="n">
+        <v>84560.4688</v>
+      </c>
+      <c r="G361" t="n">
+        <v>84261.2812</v>
+      </c>
+      <c r="H361" t="n">
+        <v>84408.7969</v>
+      </c>
+      <c r="I361" t="n">
+        <v>732500992</v>
+      </c>
+      <c r="J361" t="n">
+        <v>4</v>
+      </c>
+      <c r="K361" t="n">
+        <v>37</v>
+      </c>
+      <c r="L361" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="M361" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="N361" t="n">
+        <v>35</v>
+      </c>
+      <c r="O361" t="n">
+        <v>0.442</v>
+      </c>
+      <c r="P361" t="n">
+        <v>-0.079</v>
+      </c>
+      <c r="Q361" t="n">
+        <v>9.045</v>
+      </c>
+      <c r="R361" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S361" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - cnbc.com</t>
+        </is>
+      </c>
+      <c r="T361" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U361" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="V361" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="W361" t="inlineStr">
+        <is>
+          <t>Bitcoin surges to over 7-month high as tokenized-stock move lifts crypto sentiment - Investing.com</t>
+        </is>
+      </c>
+      <c r="X361" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYkhkWmxhUGhucUhoNHZIdkxiMnNjNEQ1MXBOSXU3dFljTXZVVjBpbTJJMDVjckpiOF9UZTgyTnZZZHNZNUFYeFVqVWEwbVd5Z1RxYmVsVWdPUGNiZjNJUTZTMzdfZE0weHFpdWlJbWx2YnZuQkJBZ1ZYTE9HY2QxcWQtSTZaVnVVbE4wdk8yYVg4d3N0SU1lXzdTMnBVX1ZuakFiX0pvODVuNXhIY0pRVWQ1cUNQdHFLTmVDaWc4TF9XMTh4bzVQWXZBMA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y361" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="Z361" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AA361" t="inlineStr">
+        <is>
+          <t>Bitcoin Price LIVE: JGB Sell-Off Puts $81,178 in Focus as BTC Breaks $84,304 Equilibrium - CryptoRank</t>
+        </is>
+      </c>
+      <c r="AB361" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPVExlTUQtSEl1aUFtdjc4Y0s3b2dXT2xjTHY3ODB5REY4d2JGa21kZ2VORmMxQ25kMHNKQ2JrR25COS1Ia1dXMWNVbmcxaE9RNlFuR19teDNPbEwzOVFBREoySHV2Xzg2czN3VVdyaXFWWlpGQXBkaHRNT05xZWhKU012RFpTZWpkd2tBdWNidG5YNlJQeGRiTVZUR2NJYUViVHNqM3FILVIzeHdabUxSNnpfa1U5XzhjQXZfRTFR?oc=5</t>
+        </is>
+      </c>
+      <c r="AC361" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - Morningstar</t>
+        </is>
+      </c>
+      <c r="AD361" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-27 13:38 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD361"/>
+  <dimension ref="A1:AD367"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45461,6 +45461,762 @@
       <c r="AD361" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-09-27T13:36:32+00:00</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E362" t="n">
+        <v>4321.6001</v>
+      </c>
+      <c r="F362" t="n">
+        <v>4332.3999</v>
+      </c>
+      <c r="G362" t="n">
+        <v>4314.5</v>
+      </c>
+      <c r="H362" t="n">
+        <v>4321.2002</v>
+      </c>
+      <c r="I362" t="n">
+        <v>17239</v>
+      </c>
+      <c r="J362" t="n">
+        <v>4</v>
+      </c>
+      <c r="K362" t="n">
+        <v>39</v>
+      </c>
+      <c r="L362" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="M362" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="N362" t="n">
+        <v>40</v>
+      </c>
+      <c r="O362" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="P362" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="Q362" t="n">
+        <v>-1.697</v>
+      </c>
+      <c r="R362" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S362" t="inlineStr">
+        <is>
+          <t>Lundin Gold Hits Record Grade at Bonza Sur With 204 g/t Gold Over 3 Metres Intercept - the deep dive</t>
+        </is>
+      </c>
+      <c r="T362" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNaDdPLWtTOVlMN0c3OWFFWmF1dUZfT28xLWducTQyQVo5XzRUZzU5YWxUZ1JlZzZqcHRtcG5FUENMZE9LN1ZEQXdpTDBMa3c2Ry1aakpaMjBtTlV6bTNDenB4d2d1OEltQmxadjVsTHFWY0J5alI2Sko2YVdfa1VHZDd3bGVtdUlOaXVaZU0xcFo0UHBjNXZTX2dKS1dtX1J5d2JBX2NxSW9TMS1P?oc=5</t>
+        </is>
+      </c>
+      <c r="U362" t="inlineStr">
+        <is>
+          <t>Precious Metals Surge: Gold Approaches $4,500 Mark, Silver Reclaims $66 - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="V362" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAxTUhJVFR3RXFNV3VTVFBNTl9OUXhvNmx6R01EZjFqSW05UWJjN3JIUGltNUNobFJKazVGR0lhb1J2bS1iRDdSeC1Fa0YtNU1BQi1xM1hnVjhaZklSUjFpU0ZHWV9GOHlncUtZMmtKTzRxQV8zM2c?oc=5</t>
+        </is>
+      </c>
+      <c r="W362" t="inlineStr">
+        <is>
+          <t>Gold rises above $4,130 as geopolitical uncertainty supports safe-haven demand - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X362" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPVC0wdnlpU1I2eWVTbnhmbHhvdFBmWUM4c3J4dk9NZFVBMGZBOVBJall6QmY2UkxxTm15TS1ycGs1ZW42RFFNaWdiUlJuajNKWmhOZ0sxYWlOSUZpcTAySkV3NHhST0dGRVZtVmVVVmt4WFFja2hjOW1RVVF5UFdGaUxaOXhOSTUwX21ab1FQQlh4dE0yOUVn?oc=5</t>
+        </is>
+      </c>
+      <c r="Y362" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="Z362" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA362" t="inlineStr">
+        <is>
+          <t>Gold (XAU/USD) Price Forecast for Today, Tomorrow, Next Week, and the Next 30 Days - LiteFinance</t>
+        </is>
+      </c>
+      <c r="AB362" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxOZ1BXeVdPR08tTmQ4MHdZMkloUzlsNjRjSE5VVmxyeVRrdDZqbDI3Tm5VVUdfYTdZM0dOYjkzVFBuMGhJUzZEM3E0RDBkc0RTUXd2VFdMdm5uenpPXzJobUNvRklvRkt0S0pfYkZ0UWRXaWRDc09MR1pBUkVDRXN2Y2FINkVmUDBlRkZHNGhzZkNyNk5LUzZrM2VUV1pVOV9N?oc=5</t>
+        </is>
+      </c>
+      <c r="AC362" t="inlineStr">
+        <is>
+          <t>Gold breaks below key MAs, eyes $4,260 support: Live levels - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD362" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPME13WGVlVjFRRTNPak02V1FBTDZVR25FMHh5Yjc5NWZqZUZfZ3pyUjRxTU5HcWRDS1I3RVRQQ0V0eTZOZmMxMk9aMlc1WGsyd0FPQzU3ZzlMSUp4cVFBSUR6ZkJucl9WSTNlRWRPdHlxY1o1emxISC10OXJib2tlaV80RGpxaW9hR3BydHhPOVNMdFFDSDd1c3RzVGc1MmJpNm1WTDkySUplMkZyZks2bQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-09-27T13:36:32+00:00</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E363" t="n">
+        <v>92.23999999999999</v>
+      </c>
+      <c r="F363" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="G363" t="n">
+        <v>91.81999999999999</v>
+      </c>
+      <c r="H363" t="n">
+        <v>92.41</v>
+      </c>
+      <c r="I363" t="n">
+        <v>72759</v>
+      </c>
+      <c r="J363" t="n">
+        <v>4</v>
+      </c>
+      <c r="K363" t="n">
+        <v>40</v>
+      </c>
+      <c r="L363" t="n">
+        <v>-0.203</v>
+      </c>
+      <c r="M363" t="n">
+        <v>-0.154</v>
+      </c>
+      <c r="N363" t="n">
+        <v>40</v>
+      </c>
+      <c r="O363" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="P363" t="n">
+        <v>-0.121</v>
+      </c>
+      <c r="Q363" t="n">
+        <v>-1.295</v>
+      </c>
+      <c r="R363" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S363" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T363" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U363" t="inlineStr">
+        <is>
+          <t>Oil surges 6%, Brent and US crude both surpass $100 on more tanker attacks - Reuters</t>
+        </is>
+      </c>
+      <c r="V363" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPVTlKVk5vOWlpYndFb2Flck9IczhtU2k5X1I3a0tlMjA2dkRmMEJncVFZdWctZW9wX05NaU9vUzNwMU5ld3UycklJMjhHaHB3WDdZVF81Z0t1WWNZak8tTFFwdDZtTHZvUnozMnVpUmtEanVsN2ZxM1A2QkxZS3IydDByTlQtd3RFYThzVnlwVmR0eGMyT1RQQldPZVp4VE1oSm5TcHBXVTd1dXM?oc=5</t>
+        </is>
+      </c>
+      <c r="W363" t="inlineStr">
+        <is>
+          <t>Europe's STOXX 600 rallies on tech, banks strength as oil prices retreat - Reuters</t>
+        </is>
+      </c>
+      <c r="X363" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNYWF0aU9mWUM0TjNtekhpT0I0NTM1RXoydldTZDlzNVM4Q0FnRXFCLTlaLUQxdEZfMS1qeU1XV0lsNHhvc09zMTBUQV9xVFhaakdCU196dW5sQ212UHdLVjVySHo5UWczV0dVS2dnY3d2Q2dTbWRkOWFRZ0g5aTlGaEtnQkFQcno2ZjdfdndQdGdSR1c3MjdEXzNCZlhRM216di1sdllQSl9OT3pkcWRSd3p3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y363" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 25, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z363" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9DVE10MHdQOXV3X0ZlbGNJS0J4ZXg2Tm1GSVVQcmdJVExmVUo5R2FPbjBDRVJ3eUZLeWd2SC1CVnZLUHNYZkx6M1NoNnFkMGpKUHFBZjh4clhDZDZlZ1Vmak5B?oc=5</t>
+        </is>
+      </c>
+      <c r="AA363" t="inlineStr">
+        <is>
+          <t>OPEC Monthly Oil Market Report, September 2026 - Peak Oil Barrel</t>
+        </is>
+      </c>
+      <c r="AB363" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9faVVpVXlFX1hFRG4tM2FnZTE5Q1ROMG1RWmxCTWVWcTdLcmo0VlBIbTlQcnhYOUQxeUxvaTE4VVo5Ulo3cExYYVViZUxWcU9VUzRIRXhQRTJLb19hWFhJc2V5WkxmMGhtSk92QVJndFZlV1NQeWxkM2Z3WWc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC363" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AD363" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-09-27T13:36:32+00:00</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E364" t="n">
+        <v>101.022</v>
+      </c>
+      <c r="F364" t="n">
+        <v>101.077</v>
+      </c>
+      <c r="G364" t="n">
+        <v>100.954</v>
+      </c>
+      <c r="H364" t="n">
+        <v>101.035</v>
+      </c>
+      <c r="I364" t="n">
+        <v>0</v>
+      </c>
+      <c r="J364" t="n">
+        <v>4</v>
+      </c>
+      <c r="K364" t="n">
+        <v>39</v>
+      </c>
+      <c r="L364" t="n">
+        <v>-0.038</v>
+      </c>
+      <c r="M364" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="N364" t="n">
+        <v>40</v>
+      </c>
+      <c r="O364" t="n">
+        <v>0.131</v>
+      </c>
+      <c r="P364" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="Q364" t="n">
+        <v>1.381</v>
+      </c>
+      <c r="R364" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S364" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T364" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U364" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="V364" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="W364" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="X364" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y364" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z364" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA364" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB364" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC364" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD364" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-09-27T13:36:32+00:00</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E365" t="n">
+        <v>7795.25</v>
+      </c>
+      <c r="F365" t="n">
+        <v>7814.75</v>
+      </c>
+      <c r="G365" t="n">
+        <v>7793.25</v>
+      </c>
+      <c r="H365" t="n">
+        <v>7803.75</v>
+      </c>
+      <c r="I365" t="n">
+        <v>473791</v>
+      </c>
+      <c r="J365" t="n">
+        <v>4</v>
+      </c>
+      <c r="K365" t="n">
+        <v>40</v>
+      </c>
+      <c r="L365" t="n">
+        <v>-0.019</v>
+      </c>
+      <c r="M365" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="N365" t="n">
+        <v>40</v>
+      </c>
+      <c r="O365" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="P365" t="n">
+        <v>-0.047</v>
+      </c>
+      <c r="Q365" t="n">
+        <v>3.922</v>
+      </c>
+      <c r="R365" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S365" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="T365" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOUmw5dTU0bUtGQk1BdkpteVFtOFpEN0tycVhJNnIwQndiRVVaZjlMcG9lanhVZkxLd1lMVlRRMGMyNXctZkRDVnE4YVNXQkg2QUFxcEhKdVJ0eWl6Yk9HOXRKMTNoUWNyNmtMX2FZOEdJd0FETUU4Mmc1SVFXcllLVmt1bDhoMUdWRzN2VGUzMnVIWk1qRXBONUZSN3BkMDBvOG9zMTA3WUdVLVFDTXlj?oc=5</t>
+        </is>
+      </c>
+      <c r="U365" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - AOL.com</t>
+        </is>
+      </c>
+      <c r="V365" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="W365" t="inlineStr">
+        <is>
+          <t>AbCellera Biologics (ABCL) Surges 34.78% as Shares Break Toward $9.81 Resistance - EMA Signal - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="X365" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPdUNOZndBWm5IMm9JRjRsTk5DNmtNQnR6YTFWMWlSTk5BT3J2TjNEdXlrMFl5Vi1sdDVyY1BybUlUU0taSnQtcktxZEV5ZkpYclc4dnBNa0lzamY3dFFRTGNMWXU5TFk3MUphb1hnak4zYS1vQ0s2NHdTeFFLOGEwdlRkcGE5VUs4a0t2bnk3SkJPMGk2RGM4VV9mclUwZmJQMGUtNXN0dUN5Z2M1U1E0cG5pckZOQlJ2TGdDSg?oc=5</t>
+        </is>
+      </c>
+      <c r="Y365" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z365" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA365" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - foxbusiness.com</t>
+        </is>
+      </c>
+      <c r="AB365" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC365" t="inlineStr">
+        <is>
+          <t>Dow Drops 317, Nasdaq Sinks 172, S&amp;P 500 Falls 45 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD365" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ3VXaWVra21SbURkNk5DcVRTX1JSX280Zm9pV05MaUx5dkF3S1ZBZUFvcWk2SS1LZGRVd1c1ODFXSlFJUHdvdEZ4OXFFaDA4V2tIUHJqOW9TenRSTlJibmJNSm5JWks4eFpPYm9rRjBSOGVRM1YyZ05HY3NFNWZBM1VBaFdjbVlHZDJwVTZtY203UQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-09-27T13:36:32+00:00</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E366" t="n">
+        <v>30912</v>
+      </c>
+      <c r="F366" t="n">
+        <v>30935</v>
+      </c>
+      <c r="G366" t="n">
+        <v>30845</v>
+      </c>
+      <c r="H366" t="n">
+        <v>30889.25</v>
+      </c>
+      <c r="I366" t="n">
+        <v>83633</v>
+      </c>
+      <c r="J366" t="n">
+        <v>4</v>
+      </c>
+      <c r="K366" t="n">
+        <v>35</v>
+      </c>
+      <c r="L366" t="n">
+        <v>-0.138</v>
+      </c>
+      <c r="M366" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="N366" t="n">
+        <v>34</v>
+      </c>
+      <c r="O366" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="P366" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="Q366" t="n">
+        <v>2.189</v>
+      </c>
+      <c r="R366" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S366" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally (AMD:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T366" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNRTNUV0JnS3haREZESHpOTVREazZUWkNwUE43OEQxMFJYajZnU3JhaWFKOEt1MVEtLTJYdlg5YnVUUnE3WnFnN0FoRDRJUFZlVEpNN2pCaWFpSEQ5NmlIM2hoQ2VDcHNHRHpTcWpiQ1RCVFRPbDd2cExKOF9adGxta2FWMUN1NjRvamQ0QUpYcFBUM2hSZkk4YWVibw?oc=5</t>
+        </is>
+      </c>
+      <c r="U366" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="V366" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W366" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq, Dow Forecast: Wall Street Split Widens Into Month-End - forex.com</t>
+        </is>
+      </c>
+      <c r="X366" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOZ25WbG0xb0NqbzZlYWZyUmRoNVR2VDV2MHBURzFWbFcxS0xOdjIwYURDbGxxcTRoYVVZclFNT3NHbG1GSlBYREo2RlVKUnl5MGROc3lXbmlwSjVTeHREbWwxeUtqdTNHSzNTZU5mQ3JJaGg5NV9BTXZLTGJSMHJ3anBRQlg1a3BsMk1oMmY5bE9xWjBmRTJ3OTd4MjlrelZXTy05MF90ZzVFYjc0LW1MUVJxUlVUbHFKUk9reG5oX096R3Fy?oc=5</t>
+        </is>
+      </c>
+      <c r="Y366" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z366" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA366" t="inlineStr">
+        <is>
+          <t>Palantir Technologies (NASDAQ: PLTR) Stock Price Falls Against Market Trend As Analysts Hold Strong Buy Rating - foreignpolicyjournal.com</t>
+        </is>
+      </c>
+      <c r="AB366" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPMGF1R05yZm50ZU84bGZvYS1nVjBoTF9GQUxqaERwSXpkdVZ0MzkwcTV2UF9uRVF5S2hCTW5uU21BYjR1eTVhamUwU1JrV1lOVnBXcnQ2WXlJeTRxdVFGZHVWMzFPMnJnUmc5eHBtSkFZV255NVAwajN3WkJQQnVKTjBQUnM1VjZ5ZEthMlIwVFQwMlpZTmlIU1ZsWnAyeXVZeHVzeHdRdHRaNGtzN0dQQWNNUldNdkZBZktSNXIzS1JxLVZaNmdlMUx0MnZJeVZqaTZXdG1rVHFiTnZReDVUaWV6Y3RVOWdQekh3cg?oc=5</t>
+        </is>
+      </c>
+      <c r="AC366" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AD366" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-09-27T13:36:32+00:00</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E367" t="n">
+        <v>84927.72659999999</v>
+      </c>
+      <c r="F367" t="n">
+        <v>85140.49219999999</v>
+      </c>
+      <c r="G367" t="n">
+        <v>84625.75</v>
+      </c>
+      <c r="H367" t="n">
+        <v>84889.1875</v>
+      </c>
+      <c r="I367" t="n">
+        <v>1498497024</v>
+      </c>
+      <c r="J367" t="n">
+        <v>4</v>
+      </c>
+      <c r="K367" t="n">
+        <v>38</v>
+      </c>
+      <c r="L367" t="n">
+        <v>-0.003</v>
+      </c>
+      <c r="M367" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="N367" t="n">
+        <v>35</v>
+      </c>
+      <c r="O367" t="n">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="P367" t="n">
+        <v>-0.019</v>
+      </c>
+      <c r="Q367" t="n">
+        <v>11.374</v>
+      </c>
+      <c r="R367" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S367" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T367" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U367" t="inlineStr">
+        <is>
+          <t>Bitcoin may reach $94,000 by October 2026, with strong institutional demand and Uptober optimism. - Pluang</t>
+        </is>
+      </c>
+      <c r="V367" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQRXFhOHd4Sl9SZ2I0dEhnbHdtaXFJSWFMXzBsRGRmS0w3c0pzSlpodU9raEE0aVNteWQxUlpKbmhiN3RUaWZscGxIZUZWQ1I4OUduLUQ4b3Q3ejc4d05jd3NscS0yNlNRM1NPU0J0V3BNSDNSQUdHTmVJdGR3cF9XaFhNRVNVUERGbTY2eQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W367" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X367" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y367" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="Z367" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AA367" t="inlineStr">
+        <is>
+          <t>Bitcoin Holders Are Selling, But This Time It’s Different: What You Need to Know - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB367" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxNY1pjQzFadG5wOXBrS3lYNVppbjF2eVp3WTBCN0xWa04yWU9jSDZVYkhNRnM2aXg1cFdRZ0FHQVIyRUhfUUNCTHYtaFhjdENNTzJ3ZEJJSVIwMFB0SEZ1RXdYSWdZejFoY0oxbTJlZjBoNWZtMTR2VHFmOEMySnpOMGMxT1NVWXNQOEhoN3pYRjZTQ29VS1NfbDlubTc0b1MzLVcyQTdSYjJGNlBYTVROem9wNUNMSXRhNVJXV3NaWlZfdUdZbHYzTTdjWEgxVFJsM3c?oc=5</t>
+        </is>
+      </c>
+      <c r="AC367" t="inlineStr">
+        <is>
+          <t>Crypto’s Latest Rebound is Fueled By More Liquidations - Bloomberg</t>
+        </is>
+      </c>
+      <c r="AD367" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcTZKMERXNUtEc1UtZTlmNy1RS21TYTV1ZXJuUzF3Rjkza1Zwbk4yWW5aRmxQSDRoWW4wU0ZadTVydVdiS01pNGlnYjZ3R0loMmp4YzNQT0N4TjVsNERrLWhzRm5QWEJFNFVFZ2lxZzNtRkM0c3Q5RkV6YzlubW9RSFZ6SFF0OHJXdHlONS1TS2Itd0JSaG5IVHJmdzNOY3l1RjNsNHFsckU?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-27 19:39 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD367"/>
+  <dimension ref="A1:AD373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46215,6 +46215,762 @@
         </is>
       </c>
       <c r="AD367" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcTZKMERXNUtEc1UtZTlmNy1RS21TYTV1ZXJuUzF3Rjkza1Zwbk4yWW5aRmxQSDRoWW4wU0ZadTVydVdiS01pNGlnYjZ3R0loMmp4YzNQT0N4TjVsNERrLWhzRm5QWEJFNFVFZ2lxZzNtRkM0c3Q5RkV6YzlubW9RSFZ6SFF0OHJXdHlONS1TS2Itd0JSaG5IVHJmdzNOY3l1RjNsNHFsckU?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-09-27T19:36:40+00:00</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E368" t="n">
+        <v>4321.6001</v>
+      </c>
+      <c r="F368" t="n">
+        <v>4332.3999</v>
+      </c>
+      <c r="G368" t="n">
+        <v>4314.5</v>
+      </c>
+      <c r="H368" t="n">
+        <v>4321.2002</v>
+      </c>
+      <c r="I368" t="n">
+        <v>17239</v>
+      </c>
+      <c r="J368" t="n">
+        <v>4</v>
+      </c>
+      <c r="K368" t="n">
+        <v>39</v>
+      </c>
+      <c r="L368" t="n">
+        <v>-0.082</v>
+      </c>
+      <c r="M368" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="N368" t="n">
+        <v>40</v>
+      </c>
+      <c r="O368" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="P368" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="Q368" t="n">
+        <v>-1.247</v>
+      </c>
+      <c r="R368" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S368" t="inlineStr">
+        <is>
+          <t>Lundin Gold Hits Record Grade at Bonza Sur With 204 g/t Gold Over 3 Metres Intercept - the deep dive</t>
+        </is>
+      </c>
+      <c r="T368" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNaDdPLWtTOVlMN0c3OWFFWmF1dUZfT28xLWducTQyQVo5XzRUZzU5YWxUZ1JlZzZqcHRtcG5FUENMZE9LN1ZEQXdpTDBMa3c2Ry1aakpaMjBtTlV6bTNDenB4d2d1OEltQmxadjVsTHFWY0J5alI2Sko2YVdfa1VHZDd3bGVtdUlOaXVaZU0xcFo0UHBjNXZTX2dKS1dtX1J5d2JBX2NxSW9TMS1P?oc=5</t>
+        </is>
+      </c>
+      <c r="U368" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="V368" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W368" t="inlineStr">
+        <is>
+          <t>Precious Metals Surge: Gold Approaches $4,500 Mark, Silver Reclaims $66 - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="X368" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAxTUhJVFR3RXFNV3VTVFBNTl9OUXhvNmx6R01EZjFqSW05UWJjN3JIUGltNUNobFJKazVGR0lhb1J2bS1iRDdSeC1Fa0YtNU1BQi1xM1hnVjhaZklSUjFpU0ZHWV9GOHlncUtZMmtKTzRxQV8zM2c?oc=5</t>
+        </is>
+      </c>
+      <c r="Y368" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="Z368" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA368" t="inlineStr">
+        <is>
+          <t>Gold (XAU/USD) Price Forecast for Today, Tomorrow, Next Week, and the Next 30 Days - LiteFinance</t>
+        </is>
+      </c>
+      <c r="AB368" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxOZ1BXeVdPR08tTmQ4MHdZMkloUzlsNjRjSE5VVmxyeVRrdDZqbDI3Tm5VVUdfYTdZM0dOYjkzVFBuMGhJUzZEM3E0RDBkc0RTUXd2VFdMdm5uenpPXzJobUNvRklvRkt0S0pfYkZ0UWRXaWRDc09MR1pBUkVDRXN2Y2FINkVmUDBlRkZHNGhzZkNyNk5LUzZrM2VUV1pVOV9N?oc=5</t>
+        </is>
+      </c>
+      <c r="AC368" t="inlineStr">
+        <is>
+          <t>Gold ETFs Shine in H1 2026 with Unprecedented Liquidity - investingnews.com</t>
+        </is>
+      </c>
+      <c r="AD368" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE1JaGRkaHpGODN4bGpQdFl6S3VyUjZKYzRvWUxjUjhyQ0lVXzZMZEltdGkwMEo2d0lhVWVmMDVUYUJfRXF4emdyX0ZTd0N6SVgwN3kxMFVXTkt5WXZJbE8ybVNRLUJYTVZy?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-09-27T19:36:40+00:00</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E369" t="n">
+        <v>92.23999999999999</v>
+      </c>
+      <c r="F369" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="G369" t="n">
+        <v>91.81999999999999</v>
+      </c>
+      <c r="H369" t="n">
+        <v>92.41</v>
+      </c>
+      <c r="I369" t="n">
+        <v>72759</v>
+      </c>
+      <c r="J369" t="n">
+        <v>4</v>
+      </c>
+      <c r="K369" t="n">
+        <v>40</v>
+      </c>
+      <c r="L369" t="n">
+        <v>-0.155</v>
+      </c>
+      <c r="M369" t="n">
+        <v>-0.184</v>
+      </c>
+      <c r="N369" t="n">
+        <v>40</v>
+      </c>
+      <c r="O369" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="P369" t="n">
+        <v>-0.153</v>
+      </c>
+      <c r="Q369" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="R369" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S369" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T369" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U369" t="inlineStr">
+        <is>
+          <t>Oil surges 6%, Brent and US crude both surpass $100 on more tanker attacks - Reuters</t>
+        </is>
+      </c>
+      <c r="V369" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPVTlKVk5vOWlpYndFb2Flck9IczhtU2k5X1I3a0tlMjA2dkRmMEJncVFZdWctZW9wX05NaU9vUzNwMU5ld3UycklJMjhHaHB3WDdZVF81Z0t1WWNZak8tTFFwdDZtTHZvUnozMnVpUmtEanVsN2ZxM1A2QkxZS3IydDByTlQtd3RFYThzVnlwVmR0eGMyT1RQQldPZVp4VE1oSm5TcHBXVTd1dXM?oc=5</t>
+        </is>
+      </c>
+      <c r="W369" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 17, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X369" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE5fSXp3bHBkaFNMQi1VVDJLRnVSZEQ4bkVYaFB4UUhYZjR5S0JLS3lWcm12X0cwZ2NndlpTMG5lLWJZSUpscFVIclBwcFloaGh1ZnZ3VVVib2w2Wld6WkpsaFZB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y369" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 25, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z369" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9DVE10MHdQOXV3X0ZlbGNJS0J4ZXg2Tm1GSVVQcmdJVExmVUo5R2FPbjBDRVJ3eUZLeWd2SC1CVnZLUHNYZkx6M1NoNnFkMGpKUHFBZjh4clhDZDZlZ1Vmak5B?oc=5</t>
+        </is>
+      </c>
+      <c r="AA369" t="inlineStr">
+        <is>
+          <t>OPEC Monthly Oil Market Report, September 2026 - Peak Oil Barrel</t>
+        </is>
+      </c>
+      <c r="AB369" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9faVVpVXlFX1hFRG4tM2FnZTE5Q1ROMG1RWmxCTWVWcTdLcmo0VlBIbTlQcnhYOUQxeUxvaTE4VVo5Ulo3cExYYVViZUxWcU9VUzRIRXhQRTJLb19hWFhJc2V5WkxmMGhtSk92QVJndFZlV1NQeWxkM2Z3WWc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC369" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AD369" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-09-27T19:36:40+00:00</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E370" t="n">
+        <v>101.022</v>
+      </c>
+      <c r="F370" t="n">
+        <v>101.077</v>
+      </c>
+      <c r="G370" t="n">
+        <v>100.954</v>
+      </c>
+      <c r="H370" t="n">
+        <v>101.035</v>
+      </c>
+      <c r="I370" t="n">
+        <v>0</v>
+      </c>
+      <c r="J370" t="n">
+        <v>4</v>
+      </c>
+      <c r="K370" t="n">
+        <v>39</v>
+      </c>
+      <c r="L370" t="n">
+        <v>-0.068</v>
+      </c>
+      <c r="M370" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="N370" t="n">
+        <v>40</v>
+      </c>
+      <c r="O370" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="P370" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Q370" t="n">
+        <v>1.096</v>
+      </c>
+      <c r="R370" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S370" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T370" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U370" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="V370" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="W370" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="X370" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y370" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z370" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA370" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB370" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC370" t="inlineStr">
+        <is>
+          <t>Asia FX Talk - USD holds firm, yen falls, regional CPI in focus - MUFG Research</t>
+        </is>
+      </c>
+      <c r="AD370" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNRUZEM3VLaUtVaEZNNzlGMFlmOXJxenVDMG9qSk1Pb0pxVWwzLW1ndmtfVzJ3bExHSWlnR2J3YmFlbHN4RFE0WXl5b21FaXh2TllraVI5MHhfdWhLeDhXTi02bXZTRUJuVzJHb1NqMXB5dTdmSV82WmNwMW1oYUdiRFd4VFZYWW1Wd0RFWkMtd2w3a0Z3dXpyR212eEtycGpWQ09FcXA5dVh4T1c0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-09-27T19:36:40+00:00</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E371" t="n">
+        <v>7795.25</v>
+      </c>
+      <c r="F371" t="n">
+        <v>7814.75</v>
+      </c>
+      <c r="G371" t="n">
+        <v>7793.25</v>
+      </c>
+      <c r="H371" t="n">
+        <v>7803.75</v>
+      </c>
+      <c r="I371" t="n">
+        <v>473791</v>
+      </c>
+      <c r="J371" t="n">
+        <v>4</v>
+      </c>
+      <c r="K371" t="n">
+        <v>39</v>
+      </c>
+      <c r="L371" t="n">
+        <v>0.303</v>
+      </c>
+      <c r="M371" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="N371" t="n">
+        <v>40</v>
+      </c>
+      <c r="O371" t="n">
+        <v>0.211</v>
+      </c>
+      <c r="P371" t="n">
+        <v>-0.116</v>
+      </c>
+      <c r="Q371" t="n">
+        <v>9.638999999999999</v>
+      </c>
+      <c r="R371" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S371" t="inlineStr">
+        <is>
+          <t>Stock market today: Nasdaq surges 2% to record high, Dow and S&amp;P 500 gain as chip stocks rally, oil falls - aol.com</t>
+        </is>
+      </c>
+      <c r="T371" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5zcWd0VnY2YzZFVGMwSnZaOE5NcVN1dF9LRHRCbEpJdHFwOGpWR1FNelJiWTA2Y01oVHRhbXJpand2d1RHV194bWwwX3ItdkROekdzNkd6STlzZnh4SU5OejhmSDdxVllMRDRFZFhNUFVuWjlrRXBN?oc=5</t>
+        </is>
+      </c>
+      <c r="U371" t="inlineStr">
+        <is>
+          <t>AbCellera Biologics (ABCL) Surges 34.78% as Shares Break Toward $9.81 Resistance - EMA Signal - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="V371" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPdUNOZndBWm5IMm9JRjRsTk5DNmtNQnR6YTFWMWlSTk5BT3J2TjNEdXlrMFl5Vi1sdDVyY1BybUlUU0taSnQtcktxZEV5ZkpYclc4dnBNa0lzamY3dFFRTGNMWXU5TFk3MUphb1hnak4zYS1vQ0s2NHdTeFFLOGEwdlRkcGE5VUs4a0t2bnk3SkJPMGk2RGM4VV9mclUwZmJQMGUtNXN0dUN5Z2M1U1E0cG5pckZOQlJ2TGdDSg?oc=5</t>
+        </is>
+      </c>
+      <c r="W371" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 21: Meta Surges on Excitement Over Muse Personal AI Agent - The Globe and Mail</t>
+        </is>
+      </c>
+      <c r="X371" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxQSWZkbHdXQnI1czhKLV84RzVXWDJvaElPdzNTQlZ4MjZSaENrdzkxN3lHZFFhWV9uR1RPeTZYSnBnSHNPUGM0NERzYkk1dWJfdUR0YjZiYkE2ZFZSb25SbVFUaVBqTFAwSURBOEdDVDhvS1hxMUZrcDZ1NmhIWGV2YjZIU3hHbnE4VUpoRUp6UGh1QUNVYzRSV0NxSXFzOVdiODFrOS11OW5ZODNIWEFXNS1lVFhaT0JVbGdIQ0RlSlV0c2ZaNzlsMnJLenFCNEc4aXBWNUN0VVBTNktTS1B1N3EwN05BbVotUWduMlhlUXFvdzlWdEMwdw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y371" t="inlineStr">
+        <is>
+          <t>AMD Beat Revenue at $11.5B and Data Center +107% — But the Stock Just Broke $476 Support - tradingkey.com</t>
+        </is>
+      </c>
+      <c r="Z371" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxPV3ZFcXFwS28tbkhsdGFscXlhbjZoQjY1TE9Fbk1mTU5lNGJWQUtvTjZmTHRtdTAwLWN6NHBocmN4WGlKNlhuU0UxaGF4b1BTMFRoVzRwdTVqckZyT2c2TlF1ZkJLNl8xOVlfajBCZUV1Y2lKYlBPUVBHaXZXUjJpWURwcDBZR0Z3VERmeDRERHRNR1VFOXU1ZmwxX2FsLTBEdHV6US04RDJXYUF3SWluYXAwelFwUlpwUXNJTkxOSFRSZmREU1lDOFV5TTYzUlVCM3k2bmlsbw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA371" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB371" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC371" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AD371" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-09-27T19:36:40+00:00</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E372" t="n">
+        <v>30912</v>
+      </c>
+      <c r="F372" t="n">
+        <v>30935</v>
+      </c>
+      <c r="G372" t="n">
+        <v>30845</v>
+      </c>
+      <c r="H372" t="n">
+        <v>30889.25</v>
+      </c>
+      <c r="I372" t="n">
+        <v>83633</v>
+      </c>
+      <c r="J372" t="n">
+        <v>4</v>
+      </c>
+      <c r="K372" t="n">
+        <v>35</v>
+      </c>
+      <c r="L372" t="n">
+        <v>-0.131</v>
+      </c>
+      <c r="M372" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="N372" t="n">
+        <v>34</v>
+      </c>
+      <c r="O372" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="P372" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="Q372" t="n">
+        <v>2.809</v>
+      </c>
+      <c r="R372" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S372" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally (AMD:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T372" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNRTNUV0JnS3haREZESHpOTVREazZUWkNwUE43OEQxMFJYajZnU3JhaWFKOEt1MVEtLTJYdlg5YnVUUnE3WnFnN0FoRDRJUFZlVEpNN2pCaWFpSEQ5NmlIM2hoQ2VDcHNHRHpTcWpiQ1RCVFRPbDd2cExKOF9adGxta2FWMUN1NjRvamQ0QUpYcFBUM2hSZkk4YWVibw?oc=5</t>
+        </is>
+      </c>
+      <c r="U372" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as chipmakers fuel stock gains - Reuters</t>
+        </is>
+      </c>
+      <c r="V372" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQUUdXdXVKYkpsa2JoQmRNeVpVWWhwb1pIVmUwcUl0QVRFVEFjRDJtREJPbXJWaXVEc0NQSWZZUlhwTl80T3h4eGM1dE9oaXRsWlVueWx0MWt3YXlWbV9PYkZDWVVPb1ZveThvalZfWnBvQ2J5Sjg1UkNOQmU5eDdWN0FvVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W372" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investinglive.com</t>
+        </is>
+      </c>
+      <c r="X372" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y372" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z372" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA372" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investinglive.com</t>
+        </is>
+      </c>
+      <c r="AB372" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC372" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD372" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-09-27T19:36:40+00:00</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E373" t="n">
+        <v>84446.0938</v>
+      </c>
+      <c r="F373" t="n">
+        <v>84830.8438</v>
+      </c>
+      <c r="G373" t="n">
+        <v>84317.2812</v>
+      </c>
+      <c r="H373" t="n">
+        <v>84766.03909999999</v>
+      </c>
+      <c r="I373" t="n">
+        <v>2925985792</v>
+      </c>
+      <c r="J373" t="n">
+        <v>4</v>
+      </c>
+      <c r="K373" t="n">
+        <v>36</v>
+      </c>
+      <c r="L373" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="M373" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="N373" t="n">
+        <v>37</v>
+      </c>
+      <c r="O373" t="n">
+        <v>0.543</v>
+      </c>
+      <c r="P373" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="Q373" t="n">
+        <v>11.054</v>
+      </c>
+      <c r="R373" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S373" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T373" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U373" t="inlineStr">
+        <is>
+          <t>Bitcoin may reach $94,000 by October 2026, with strong institutional demand and Uptober optimism. - Pluang</t>
+        </is>
+      </c>
+      <c r="V373" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQRXFhOHd4Sl9SZ2I0dEhnbHdtaXFJSWFMXzBsRGRmS0w3c0pzSlpodU9raEE0aVNteWQxUlpKbmhiN3RUaWZscGxIZUZWQ1I4OUduLUQ4b3Q3ejc4d05jd3NscS0yNlNRM1NPU0J0V3BNSDNSQUdHTmVJdGR3cF9XaFhNRVNVUERGbTY2eQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W373" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X373" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y373" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="Z373" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AA373" t="inlineStr">
+        <is>
+          <t>Bitcoin Holders Are Selling, But This Time It’s Different: What You Need to Know - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB373" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxNY1pjQzFadG5wOXBrS3lYNVppbjF2eVp3WTBCN0xWa04yWU9jSDZVYkhNRnM2aXg1cFdRZ0FHQVIyRUhfUUNCTHYtaFhjdENNTzJ3ZEJJSVIwMFB0SEZ1RXdYSWdZejFoY0oxbTJlZjBoNWZtMTR2VHFmOEMySnpOMGMxT1NVWXNQOEhoN3pYRjZTQ29VS1NfbDlubTc0b1MzLVcyQTdSYjJGNlBYTVROem9wNUNMSXRhNVJXV3NaWlZfdUdZbHYzTTdjWEgxVFJsM3c?oc=5</t>
+        </is>
+      </c>
+      <c r="AC373" t="inlineStr">
+        <is>
+          <t>Crypto’s Latest Rebound is Fueled By More Liquidations - Bloomberg</t>
+        </is>
+      </c>
+      <c r="AD373" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcTZKMERXNUtEc1UtZTlmNy1RS21TYTV1ZXJuUzF3Rjkza1Zwbk4yWW5aRmxQSDRoWW4wU0ZadTVydVdiS01pNGlnYjZ3R0loMmp4YzNQT0N4TjVsNERrLWhzRm5QWEJFNFVFZ2lxZzNtRkM0c3Q5RkV6YzlubW9RSFZ6SFF0OHJXdHlONS1TS2Itd0JSaG5IVHJmdzNOY3l1RjNsNHFsckU?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-27 22:55 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD373"/>
+  <dimension ref="A1:AD379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46527,7 +46527,7 @@
         <v>0.146</v>
       </c>
       <c r="P370" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q370" t="n">
         <v>1.096</v>
@@ -46973,6 +46973,762 @@
       <c r="AD373" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcTZKMERXNUtEc1UtZTlmNy1RS21TYTV1ZXJuUzF3Rjkza1Zwbk4yWW5aRmxQSDRoWW4wU0ZadTVydVdiS01pNGlnYjZ3R0loMmp4YzNQT0N4TjVsNERrLWhzRm5QWEJFNFVFZ2lxZzNtRkM0c3Q5RkV6YzlubW9RSFZ6SFF0OHJXdHlONS1TS2Itd0JSaG5IVHJmdzNOY3l1RjNsNHFsckU?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:53:21+00:00</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E374" t="n">
+        <v>4318.2998</v>
+      </c>
+      <c r="F374" t="n">
+        <v>4332.3999</v>
+      </c>
+      <c r="G374" t="n">
+        <v>4296.2998</v>
+      </c>
+      <c r="H374" t="n">
+        <v>4297</v>
+      </c>
+      <c r="I374" t="n">
+        <v>12508</v>
+      </c>
+      <c r="J374" t="n">
+        <v>4</v>
+      </c>
+      <c r="K374" t="n">
+        <v>39</v>
+      </c>
+      <c r="L374" t="n">
+        <v>-0.183</v>
+      </c>
+      <c r="M374" t="n">
+        <v>-0.007</v>
+      </c>
+      <c r="N374" t="n">
+        <v>40</v>
+      </c>
+      <c r="O374" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="P374" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="Q374" t="n">
+        <v>-2.353</v>
+      </c>
+      <c r="R374" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S374" t="inlineStr">
+        <is>
+          <t>Lundin Gold Hits Record Grade at Bonza Sur With 204 g/t Gold Over 3 Metres Intercept - the deep dive</t>
+        </is>
+      </c>
+      <c r="T374" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNaDdPLWtTOVlMN0c3OWFFWmF1dUZfT28xLWducTQyQVo5XzRUZzU5YWxUZ1JlZzZqcHRtcG5FUENMZE9LN1ZEQXdpTDBMa3c2Ry1aakpaMjBtTlV6bTNDenB4d2d1OEltQmxadjVsTHFWY0J5alI2Sko2YVdfa1VHZDd3bGVtdUlOaXVaZU0xcFo0UHBjNXZTX2dKS1dtX1J5d2JBX2NxSW9TMS1P?oc=5</t>
+        </is>
+      </c>
+      <c r="U374" t="inlineStr">
+        <is>
+          <t>Gold Q4 2026 outlook: Resilience in the face of rallying dollar and yields - FOREX.com</t>
+        </is>
+      </c>
+      <c r="V374" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPZWYyaG9XSnA0TEs3VTYtRXVhY1RUOWFwSkJOOXZLMGxGTlF1eU5VZzNJR2VGazZZVUlYNEJCVmJNZV90YkVJd0VtZmxTck9pemxwTV9XTUY4MmpBUDZEZkVYbkh5UEVnQU5VS0ZOWDJ4WnFRTGNvZ3ZKOUdNdk94SlBTUnU5TlRHcjVHVlRTN2I3OGluWllqS3MyZU1LYVRDOXY4RG13cUpDUnluVnR4Z1NfRHpjSUxMMUk1cQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W374" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X374" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y374" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="Z374" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA374" t="inlineStr">
+        <is>
+          <t>Gold price prediction: Experts predict Gold rate for last three months of 2026, first half of 2027 - The Economic Times</t>
+        </is>
+      </c>
+      <c r="AB374" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQckxsNld0Z0c3SXk5S3ZSeDdEYlZTMzRwVkRubG04eHAwNko2OExnZnVCNlkxOXlyUWt3d3JMX1p4aFJBcXNIWVFhMllvbVJrV21yaFczd3lSUExIZ25pOEZsVEE3U3NYVU1OVjBEb295eURCYlJFS1Nxbl8yOE9NbHhwcmRfaDRPeEFBZHdBd1MwZjdDcmdpLUhhSlNYeTJNZzU2QWdOQ29rRWVYU09DeTNQcHlSTFlpNGxMd3NrRDJWX3E4aURvem1YbmRYTHZwRThKMklaUnMxbEs4bUkyQ0NMSVlTR29CSk5xbWZPRXlkZUVWZWdTb01kMWxWUHFqTUHSAYcCQVVfeXFMUFRXd01oZ3BNc3hSLUpQRUlFSTVfb2pzUTJjME0wN2VsRVpzSHBSbGU5eUFWVFRZeERUd2hleWhWZU4wdkQ1OFRIUkYzV3BITHNRZXRqR0h1WFgzSGlpYTVmOGNfZXlTR3BCcGZjMUx2NFJLZ3FkTU9oeHFfZTl4amFKdHprVzVJUnFBVTRIUmlNTlgyd0NrM0dPalJpV0hXV3E4WEJHYmtQdlBYNEZwRGgyOVRxcDZ5alh0WlRCS2pZSC03WktEY2N3dHlDSFJaNF9UQk9KaVg4OHdodktfVWtoZTcxY3JfUU03ZFVYYWRCVEhYQ3hiUURpNGVDTVhwV1Q2NWpRcHc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC374" t="inlineStr">
+        <is>
+          <t>Gold (XAU/USD) Price Forecast for Today, Tomorrow, Next Week, and the Next 30 Days - LiteFinance</t>
+        </is>
+      </c>
+      <c r="AD374" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxOZ1BXeVdPR08tTmQ4MHdZMkloUzlsNjRjSE5VVmxyeVRrdDZqbDI3Tm5VVUdfYTdZM0dOYjkzVFBuMGhJUzZEM3E0RDBkc0RTUXd2VFdMdm5uenpPXzJobUNvRklvRkt0S0pfYkZ0UWRXaWRDc09MR1pBUkVDRXN2Y2FINkVmUDBlRkZHNGhzZkNyNk5LUzZrM2VUV1pVOV9N?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:53:21+00:00</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E375" t="n">
+        <v>92.16</v>
+      </c>
+      <c r="F375" t="n">
+        <v>93.66</v>
+      </c>
+      <c r="G375" t="n">
+        <v>91.81999999999999</v>
+      </c>
+      <c r="H375" t="n">
+        <v>93.56999999999999</v>
+      </c>
+      <c r="I375" t="n">
+        <v>52283</v>
+      </c>
+      <c r="J375" t="n">
+        <v>4</v>
+      </c>
+      <c r="K375" t="n">
+        <v>40</v>
+      </c>
+      <c r="L375" t="n">
+        <v>-0.188</v>
+      </c>
+      <c r="M375" t="n">
+        <v>-0.175</v>
+      </c>
+      <c r="N375" t="n">
+        <v>40</v>
+      </c>
+      <c r="O375" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="P375" t="n">
+        <v>-0.169</v>
+      </c>
+      <c r="Q375" t="n">
+        <v>-0.855</v>
+      </c>
+      <c r="R375" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S375" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T375" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U375" t="inlineStr">
+        <is>
+          <t>Europe's STOXX 600 rallies on tech, banks strength as oil prices retreat - Reuters</t>
+        </is>
+      </c>
+      <c r="V375" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNYWF0aU9mWUM0TjNtekhpT0I0NTM1RXoydldTZDlzNVM4Q0FnRXFCLTlaLUQxdEZfMS1qeU1XV0lsNHhvc09zMTBUQV9xVFhaakdCU196dW5sQ212UHdLVjVySHo5UWczV0dVS2dnY3d2Q2dTbWRkOWFRZ0g5aTlGaEtnQkFQcno2ZjdfdndQdGdSR1c3MjdEXzNCZlhRM216di1sdllQSl9OT3pkcWRSd3p3?oc=5</t>
+        </is>
+      </c>
+      <c r="W375" t="inlineStr">
+        <is>
+          <t>Oil prices surge 15% as Strait of Hormuz disruptions tighten supply - Offshore Technology</t>
+        </is>
+      </c>
+      <c r="X375" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPdndjemtyTkduUUpSVnR6aXJUNXBBR0JNd1FaaURNWmtvWm9WTkZUME50Qk1NVDUtdEtqcWE2R0xvUGRKNHBWZDMtblpaY1h1TE5zcmgycU5kS29mYU02N1BOdThBMUhUMDM0T1FScDZRY0JzYlRXTTJVajFYbkh3Rmp0MDFDeVZQcFhKSjhpaklySjZrVWJCZVoyWkw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y375" t="inlineStr">
+        <is>
+          <t>OPEC Monthly Oil Market Report, September 2026 - Peak Oil Barrel</t>
+        </is>
+      </c>
+      <c r="Z375" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9faVVpVXlFX1hFRG4tM2FnZTE5Q1ROMG1RWmxCTWVWcTdLcmo0VlBIbTlQcnhYOUQxeUxvaTE4VVo5Ulo3cExYYVViZUxWcU9VUzRIRXhQRTJLb19hWFhJc2V5WkxmMGhtSk92QVJndFZlV1NQeWxkM2Z3WWc?oc=5</t>
+        </is>
+      </c>
+      <c r="AA375" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 25, 2026 - fortune.com</t>
+        </is>
+      </c>
+      <c r="AB375" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9DVE10MHdQOXV3X0ZlbGNJS0J4ZXg2Tm1GSVVQcmdJVExmVUo5R2FPbjBDRVJ3eUZLeWd2SC1CVnZLUHNYZkx6M1NoNnFkMGpKUHFBZjh4clhDZDZlZ1Vmak5B?oc=5</t>
+        </is>
+      </c>
+      <c r="AC375" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AD375" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:53:21+00:00</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E376" t="n">
+        <v>101.022</v>
+      </c>
+      <c r="F376" t="n">
+        <v>101.077</v>
+      </c>
+      <c r="G376" t="n">
+        <v>100.954</v>
+      </c>
+      <c r="H376" t="n">
+        <v>101.035</v>
+      </c>
+      <c r="I376" t="n">
+        <v>0</v>
+      </c>
+      <c r="J376" t="n">
+        <v>4</v>
+      </c>
+      <c r="K376" t="n">
+        <v>39</v>
+      </c>
+      <c r="L376" t="n">
+        <v>-0.055</v>
+      </c>
+      <c r="M376" t="n">
+        <v>0.173</v>
+      </c>
+      <c r="N376" t="n">
+        <v>40</v>
+      </c>
+      <c r="O376" t="n">
+        <v>0.148</v>
+      </c>
+      <c r="P376" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="Q376" t="n">
+        <v>1.393</v>
+      </c>
+      <c r="R376" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S376" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T376" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U376" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="V376" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="W376" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - tradingview.com</t>
+        </is>
+      </c>
+      <c r="X376" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y376" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z376" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA376" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB376" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC376" t="inlineStr">
+        <is>
+          <t>ING lifts year-end EUR/USD forecast to 1.18 as dovish Fed view pressures Dollar - VT Markets</t>
+        </is>
+      </c>
+      <c r="AD376" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxORE5YdjZHQzh4V1B2REJUeHpXV3N6Y21ZeWh3VzhfNng4N0dsSk5xbEpCTW40a05ES2NPQkFqQ3RGWjR4ZnN4RUFhVXoxU1NPRFUzZnZRU3E3TzRSTUxxYWZ1dnVMVlVqVUZrR2JRYkt2QlVYVGtpUGN2Mmt6blhvRFVDWURtbkI4UGlyVHpmMHBSeFdTS0RNS0NENXZWQkFxSVNBdkQxSVczTmdMbDk4UVpzSWtZVUliVS1WVFZZdnRuYXM?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:53:21+00:00</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E377" t="n">
+        <v>7802.75</v>
+      </c>
+      <c r="F377" t="n">
+        <v>7814.75</v>
+      </c>
+      <c r="G377" t="n">
+        <v>7781.5</v>
+      </c>
+      <c r="H377" t="n">
+        <v>7783.25</v>
+      </c>
+      <c r="I377" t="n">
+        <v>378921</v>
+      </c>
+      <c r="J377" t="n">
+        <v>4</v>
+      </c>
+      <c r="K377" t="n">
+        <v>39</v>
+      </c>
+      <c r="L377" t="n">
+        <v>0.266</v>
+      </c>
+      <c r="M377" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="N377" t="n">
+        <v>40</v>
+      </c>
+      <c r="O377" t="n">
+        <v>0.216</v>
+      </c>
+      <c r="P377" t="n">
+        <v>-0.118</v>
+      </c>
+      <c r="Q377" t="n">
+        <v>8.994</v>
+      </c>
+      <c r="R377" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S377" t="inlineStr">
+        <is>
+          <t>AbCellera Biologics (ABCL) Surges 34.78% as Shares Break Toward $9.81 Resistance - EMA Signal - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="T377" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPdUNOZndBWm5IMm9JRjRsTk5DNmtNQnR6YTFWMWlSTk5BT3J2TjNEdXlrMFl5Vi1sdDVyY1BybUlUU0taSnQtcktxZEV5ZkpYclc4dnBNa0lzamY3dFFRTGNMWXU5TFk3MUphb1hnak4zYS1vQ0s2NHdTeFFLOGEwdlRkcGE5VUs4a0t2bnk3SkJPMGk2RGM4VV9mclUwZmJQMGUtNXN0dUN5Z2M1U1E0cG5pckZOQlJ2TGdDSg?oc=5</t>
+        </is>
+      </c>
+      <c r="U377" t="inlineStr">
+        <is>
+          <t>Dow surges to record close after a fresh tech rally and a plunge in oil prices - Business Insider</t>
+        </is>
+      </c>
+      <c r="V377" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOS0hLS2NLYi1nYlZnTmRJNTRtQXAyZUh5MExFZUVXcEtOTEhzVF9zeHozLThnVHVETGtwMVBFZFBUb3dVaDJlMmtmTUd6Y2ZmUVhMZjRxck41ZEJDZFNqSG5PRm96VXR6bE9tLWlybXBqVWh4NjRUSUJIcFVjdE9xRml2YWJVYTZvMmM4aTQ5bw?oc=5</t>
+        </is>
+      </c>
+      <c r="W377" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 21: Meta Surges on Excitement Over Muse Personal AI Agent - The Globe and Mail</t>
+        </is>
+      </c>
+      <c r="X377" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxQSWZkbHdXQnI1czhKLV84RzVXWDJvaElPdzNTQlZ4MjZSaENrdzkxN3lHZFFhWV9uR1RPeTZYSnBnSHNPUGM0NERzYkk1dWJfdUR0YjZiYkE2ZFZSb25SbVFUaVBqTFAwSURBOEdDVDhvS1hxMUZrcDZ1NmhIWGV2YjZIU3hHbnE4VUpoRUp6UGh1QUNVYzRSV0NxSXFzOVdiODFrOS11OW5ZODNIWEFXNS1lVFhaT0JVbGdIQ0RlSlV0c2ZaNzlsMnJLenFCNEc4aXBWNUN0VVBTNktTS1B1N3EwN05BbVotUWduMlhlUXFvdzlWdEMwdw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y377" t="inlineStr">
+        <is>
+          <t>AMD Beat Revenue at $11.5B and Data Center +107% — But the Stock Just Broke $476 Support - TradingKey</t>
+        </is>
+      </c>
+      <c r="Z377" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxPV3ZFcXFwS28tbkhsdGFscXlhbjZoQjY1TE9Fbk1mTU5lNGJWQUtvTjZmTHRtdTAwLWN6NHBocmN4WGlKNlhuU0UxaGF4b1BTMFRoVzRwdTVqckZyT2c2TlF1ZkJLNl8xOVlfajBCZUV1Y2lKYlBPUVBHaXZXUjJpWURwcDBZR0Z3VERmeDRERHRNR1VFOXU1ZmwxX2FsLTBEdHV6US04RDJXYUF3SWluYXAwelFwUlpwUXNJTkxOSFRSZmREU1lDOFV5TTYzUlVCM3k2bmlsbw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA377" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB377" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC377" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AD377" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:53:21+00:00</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E378" t="n">
+        <v>30869</v>
+      </c>
+      <c r="F378" t="n">
+        <v>30935</v>
+      </c>
+      <c r="G378" t="n">
+        <v>30795.75</v>
+      </c>
+      <c r="H378" t="n">
+        <v>30806.5</v>
+      </c>
+      <c r="I378" t="n">
+        <v>59802</v>
+      </c>
+      <c r="J378" t="n">
+        <v>4</v>
+      </c>
+      <c r="K378" t="n">
+        <v>35</v>
+      </c>
+      <c r="L378" t="n">
+        <v>-0.081</v>
+      </c>
+      <c r="M378" t="n">
+        <v>0.089</v>
+      </c>
+      <c r="N378" t="n">
+        <v>34</v>
+      </c>
+      <c r="O378" t="n">
+        <v>0.257</v>
+      </c>
+      <c r="P378" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="Q378" t="n">
+        <v>3.451</v>
+      </c>
+      <c r="R378" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S378" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally (AMD:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T378" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNRTNUV0JnS3haREZESHpOTVREazZUWkNwUE43OEQxMFJYajZnU3JhaWFKOEt1MVEtLTJYdlg5YnVUUnE3WnFnN0FoRDRJUFZlVEpNN2pCaWFpSEQ5NmlIM2hoQ2VDcHNHRHpTcWpiQ1RCVFRPbDd2cExKOF9adGxta2FWMUN1NjRvamQ0QUpYcFBUM2hSZkk4YWVibw?oc=5</t>
+        </is>
+      </c>
+      <c r="U378" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as chipmakers fuel stock gains - Reuters</t>
+        </is>
+      </c>
+      <c r="V378" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQUUdXdXVKYkpsa2JoQmRNeVpVWWhwb1pIVmUwcUl0QVRFVEFjRDJtREJPbXJWaXVEc0NQSWZZUlhwTl80T3h4eGM1dE9oaXRsWlVueWx0MWt3YXlWbV9PYkZDWVVPb1ZveThvalZfWnBvQ2J5Sjg1UkNOQmU5eDdWN0FvVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W378" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="X378" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y378" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z378" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA378" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="AB378" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC378" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD378" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:53:21+00:00</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E379" t="n">
+        <v>84802.97659999999</v>
+      </c>
+      <c r="F379" t="n">
+        <v>84830.8438</v>
+      </c>
+      <c r="G379" t="n">
+        <v>84120</v>
+      </c>
+      <c r="H379" t="n">
+        <v>84218.10159999999</v>
+      </c>
+      <c r="I379" t="n">
+        <v>1475979264</v>
+      </c>
+      <c r="J379" t="n">
+        <v>4</v>
+      </c>
+      <c r="K379" t="n">
+        <v>36</v>
+      </c>
+      <c r="L379" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="M379" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="N379" t="n">
+        <v>37</v>
+      </c>
+      <c r="O379" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="P379" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="Q379" t="n">
+        <v>10.618</v>
+      </c>
+      <c r="R379" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S379" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T379" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U379" t="inlineStr">
+        <is>
+          <t>Bitcoin may reach $94,000 by October 2026, with strong institutional demand and Uptober optimism. - Pluang</t>
+        </is>
+      </c>
+      <c r="V379" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQRXFhOHd4Sl9SZ2I0dEhnbHdtaXFJSWFMXzBsRGRmS0w3c0pzSlpodU9raEE0aVNteWQxUlpKbmhiN3RUaWZscGxIZUZWQ1I4OUduLUQ4b3Q3ejc4d05jd3NscS0yNlNRM1NPU0J0V3BNSDNSQUdHTmVJdGR3cF9XaFhNRVNVUERGbTY2eQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W379" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X379" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y379" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="Z379" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AA379" t="inlineStr">
+        <is>
+          <t>Bitcoin Holders Are Selling, But This Time It’s Different: What You Need to Know - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB379" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxNY1pjQzFadG5wOXBrS3lYNVppbjF2eVp3WTBCN0xWa04yWU9jSDZVYkhNRnM2aXg1cFdRZ0FHQVIyRUhfUUNCTHYtaFhjdENNTzJ3ZEJJSVIwMFB0SEZ1RXdYSWdZejFoY0oxbTJlZjBoNWZtMTR2VHFmOEMySnpOMGMxT1NVWXNQOEhoN3pYRjZTQ29VS1NfbDlubTc0b1MzLVcyQTdSYjJGNlBYTVROem9wNUNMSXRhNVJXV3NaWlZfdUdZbHYzTTdjWEgxVFJsM3c?oc=5</t>
+        </is>
+      </c>
+      <c r="AC379" t="inlineStr">
+        <is>
+          <t>Will Bitcoin Price Breakout Towards $100,000? One Candle Will Decide This Week - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="AD379" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQdGFudS1DOXZsRlFtMHNtZnpDdklNbGNPc045OEZuMjZXZ2RZWlk1NldxNy1jNXdJbU9KX05zZHJ3VXhPVS0tVV9oZVRlSEYwS3FHWXpMaU1GNC1JQU5lMnJnWVRnUVRYdWY3YW9FVjhzd1E0dW13dGJMU2szdm4yU1BlWlFSNTQzRHFlV3NzU0ZaaXBNVFRiX05rNllJLTdi?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-28 04:11 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD379"/>
+  <dimension ref="A1:AD385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47729,6 +47729,762 @@
       <c r="AD379" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQdGFudS1DOXZsRlFtMHNtZnpDdklNbGNPc045OEZuMjZXZ2RZWlk1NldxNy1jNXdJbU9KX05zZHJ3VXhPVS0tVV9oZVRlSEYwS3FHWXpMaU1GNC1JQU5lMnJnWVRnUVRYdWY3YW9FVjhzd1E0dW13dGJMU2szdm4yU1BlWlFSNTQzRHFlV3NzU0ZaaXBNVFRiX05rNllJLTdi?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-09-28T04:09:03+00:00</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E380" t="n">
+        <v>4308.7998</v>
+      </c>
+      <c r="F380" t="n">
+        <v>4310</v>
+      </c>
+      <c r="G380" t="n">
+        <v>4252.3999</v>
+      </c>
+      <c r="H380" t="n">
+        <v>4256.8999</v>
+      </c>
+      <c r="I380" t="n">
+        <v>16922</v>
+      </c>
+      <c r="J380" t="n">
+        <v>4</v>
+      </c>
+      <c r="K380" t="n">
+        <v>39</v>
+      </c>
+      <c r="L380" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="M380" t="n">
+        <v>0</v>
+      </c>
+      <c r="N380" t="n">
+        <v>40</v>
+      </c>
+      <c r="O380" t="n">
+        <v>0.132</v>
+      </c>
+      <c r="P380" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="Q380" t="n">
+        <v>2.617</v>
+      </c>
+      <c r="R380" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S380" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="T380" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="U380" t="inlineStr">
+        <is>
+          <t>Gold hits record high as investors seek safety - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="V380" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVWt1Y1hBWG5uZFNjRUFtZHlqRUhfZGV6VzAtQ0tBT2VlVDVEZEJ2WHN0YndCcXRzSjNtVnFhUFZZZ2F4RFRxYkdsSF91eDk2MFl5R3JNWk1HREJjSVdhUE1uTTU1N1Z6Y2xfZzZCSDZ4YnhaT1czcWdXeHE3SjJBR2FqUm43Z0paUG5OVEdsWVdYYnZBWVHSAZsBQVVfeXFMTWh6VXlqZGZVbUl3SHVfQ195WFFveEVkLU9TU1RXMTZBdVhodU16UWxLLWVScDNsc2VGMThyT0RTTHB4SVNRYU1KWmRycHhnTEc0NTJ1RWgzdGc2Y0VkanR4QUtlUWFBSnB2cElORUltQk9XdWRLNXhKbU5jRUFqQVd6bG5YbURJakxhNTl3UEk4RzBaQzVJaVdRdFk?oc=5</t>
+        </is>
+      </c>
+      <c r="W380" t="inlineStr">
+        <is>
+          <t>Gold rises above $4,130 as geopolitical uncertainty supports safe-haven demand - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X380" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPVC0wdnlpU1I2eWVTbnhmbHhvdFBmWUM4c3J4dk9NZFVBMGZBOVBJall6QmY2UkxxTm15TS1ycGs1ZW42RFFNaWdiUlJuajNKWmhOZ0sxYWlOSUZpcTAySkV3NHhST0dGRVZtVmVVVmt4WFFja2hjOW1RVVF5UFdGaUxaOXhOSTUwX21ab1FQQlh4dE0yOUVn?oc=5</t>
+        </is>
+      </c>
+      <c r="Y380" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="Z380" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA380" t="inlineStr">
+        <is>
+          <t>Gold price prediction: Experts predict Gold rate for last three months of 2026, first half of 2027 - The Economic Times</t>
+        </is>
+      </c>
+      <c r="AB380" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQckxsNld0Z0c3SXk5S3ZSeDdEYlZTMzRwVkRubG04eHAwNko2OExnZnVCNlkxOXlyUWt3d3JMX1p4aFJBcXNIWVFhMllvbVJrV21yaFczd3lSUExIZ25pOEZsVEE3U3NYVU1OVjBEb295eURCYlJFS1Nxbl8yOE9NbHhwcmRfaDRPeEFBZHdBd1MwZjdDcmdpLUhhSlNYeTJNZzU2QWdOQ29rRWVYU09DeTNQcHlSTFlpNGxMd3NrRDJWX3E4aURvem1YbmRYTHZwRThKMklaUnMxbEs4bUkyQ0NMSVlTR29CSk5xbWZPRXlkZUVWZWdTb01kMWxWUHFqTUHSAYcCQVVfeXFMUFRXd01oZ3BNc3hSLUpQRUlFSTVfb2pzUTJjME0wN2VsRVpzSHBSbGU5eUFWVFRZeERUd2hleWhWZU4wdkQ1OFRIUkYzV3BITHNRZXRqR0h1WFgzSGlpYTVmOGNfZXlTR3BCcGZjMUx2NFJLZ3FkTU9oeHFfZTl4amFKdHprVzVJUnFBVTRIUmlNTlgyd0NrM0dPalJpV0hXV3E4WEJHYmtQdlBYNEZwRGgyOVRxcDZ5alh0WlRCS2pZSC03WktEY2N3dHlDSFJaNF9UQk9KaVg4OHdodktfVWtoZTcxY3JfUU03ZFVYYWRCVEhYQ3hiUURpNGVDTVhwV1Q2NWpRcHc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC380" t="inlineStr">
+        <is>
+          <t>Gold (XAU/USD) Price Forecast for Today, Tomorrow, Next Week, and the Next 30 Days - LiteFinance</t>
+        </is>
+      </c>
+      <c r="AD380" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxOZ1BXeVdPR08tTmQ4MHdZMkloUzlsNjRjSE5VVmxyeVRrdDZqbDI3Tm5VVUdfYTdZM0dOYjkzVFBuMGhJUzZEM3E0RDBkc0RTUXd2VFdMdm5uenpPXzJobUNvRklvRkt0S0pfYkZ0UWRXaWRDc09MR1pBUkVDRXN2Y2FINkVmUDBlRkZHNGhzZkNyNk5LUzZrM2VUV1pVOV9N?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-09-28T04:09:03+00:00</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E381" t="n">
+        <v>93.28</v>
+      </c>
+      <c r="F381" t="n">
+        <v>93.76000000000001</v>
+      </c>
+      <c r="G381" t="n">
+        <v>92.90000000000001</v>
+      </c>
+      <c r="H381" t="n">
+        <v>93.08</v>
+      </c>
+      <c r="I381" t="n">
+        <v>9127</v>
+      </c>
+      <c r="J381" t="n">
+        <v>3</v>
+      </c>
+      <c r="K381" t="n">
+        <v>40</v>
+      </c>
+      <c r="L381" t="n">
+        <v>-0.139</v>
+      </c>
+      <c r="M381" t="n">
+        <v>-0.204</v>
+      </c>
+      <c r="N381" t="n">
+        <v>40</v>
+      </c>
+      <c r="O381" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="P381" t="n">
+        <v>-0.118</v>
+      </c>
+      <c r="Q381" t="n">
+        <v>-1.362</v>
+      </c>
+      <c r="R381" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S381" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - energynow.com</t>
+        </is>
+      </c>
+      <c r="T381" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U381" t="inlineStr">
+        <is>
+          <t>Oil prices surge 15% as Strait of Hormuz disruptions tighten supply - Offshore Technology</t>
+        </is>
+      </c>
+      <c r="V381" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPdndjemtyTkduUUpSVnR6aXJUNXBBR0JNd1FaaURNWmtvWm9WTkZUME50Qk1NVDUtdEtqcWE2R0xvUGRKNHBWZDMtblpaY1h1TE5zcmgycU5kS29mYU02N1BOdThBMUhUMDM0T1FScDZRY0JzYlRXTTJVajFYbkh3Rmp0MDFDeVZQcFhKSjhpaklySjZrVWJCZVoyWkw?oc=5</t>
+        </is>
+      </c>
+      <c r="W381" t="inlineStr">
+        <is>
+          <t>BTC Breaks Resistance, Eyes $85K–$95K Range - Action Forex</t>
+        </is>
+      </c>
+      <c r="X381" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNZGVLanR1Sy05Tm5XSDFLdDdEeW40UTdSUm9ZT2t2Z3JRNHdaYlpxU1BTeDd4VkR1eGw2d3JJNlFaMDI3Tksycm5zcE9sUm5pM1VEM1lkVkQzWDRNUmswQUYyT2NFa09UcnZQdkFKRXBoOEtFVVRzbVpSbnpYa1NLbWJOaFFxZWNHTTAzQy1LS2xoekVYZGZCVTVDajZCY2VoQi12NXRBdFl5bnBYemJz?oc=5</t>
+        </is>
+      </c>
+      <c r="Y381" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 25, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z381" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9DVE10MHdQOXV3X0ZlbGNJS0J4ZXg2Tm1GSVVQcmdJVExmVUo5R2FPbjBDRVJ3eUZLeWd2SC1CVnZLUHNYZkx6M1NoNnFkMGpKUHFBZjh4clhDZDZlZ1Vmak5B?oc=5</t>
+        </is>
+      </c>
+      <c r="AA381" t="inlineStr">
+        <is>
+          <t>OPEC Monthly Oil Market Report, September 2026 - Peak Oil Barrel</t>
+        </is>
+      </c>
+      <c r="AB381" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9faVVpVXlFX1hFRG4tM2FnZTE5Q1ROMG1RWmxCTWVWcTdLcmo0VlBIbTlQcnhYOUQxeUxvaTE4VVo5Ulo3cExYYVViZUxWcU9VUzRIRXhQRTJLb19hWFhJc2V5WkxmMGhtSk92QVJndFZlV1NQeWxkM2Z3WWc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC381" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AD381" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-09-28T04:09:03+00:00</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E382" t="n">
+        <v>101.12</v>
+      </c>
+      <c r="F382" t="n">
+        <v>101.12</v>
+      </c>
+      <c r="G382" t="n">
+        <v>101.12</v>
+      </c>
+      <c r="H382" t="n">
+        <v>101.12</v>
+      </c>
+      <c r="I382" t="n">
+        <v>0</v>
+      </c>
+      <c r="J382" t="n">
+        <v>1</v>
+      </c>
+      <c r="K382" t="n">
+        <v>40</v>
+      </c>
+      <c r="L382" t="n">
+        <v>-0.08799999999999999</v>
+      </c>
+      <c r="M382" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N382" t="n">
+        <v>40</v>
+      </c>
+      <c r="O382" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="P382" t="n">
+        <v>-0.003</v>
+      </c>
+      <c r="Q382" t="n">
+        <v>1.424</v>
+      </c>
+      <c r="R382" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S382" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T382" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U382" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="V382" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="W382" t="inlineStr">
+        <is>
+          <t>Dollar Strengthens Further - TradingView</t>
+        </is>
+      </c>
+      <c r="X382" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxObzB4WE8ybzdmSFlHSW5oWVpiYmp1eF9haUlwVzA2SVkxckotTWVvZC1MNkYyem1LZTBwOFE3bDlJY3NQczdjLXdQXy1iQkQtR096QkZkeVNuXzk2aXd3SGpibVVDOUNiekFJRU1MalhOSmFUWHVLMW5rcHc2UUozaFVNOA?oc=5</t>
+        </is>
+      </c>
+      <c r="Y382" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z382" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA382" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB382" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC382" t="inlineStr">
+        <is>
+          <t>British Pound gains as US Dollar weakens despite hawkish Fed, geopolitical tensions - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD382" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPS2g2djM3bEE4SmNheEM2X09OUDBWaTRYNFdaOWJKVDZpWHkzRlp1SVFENXJOR0VDQTNmQWx5bVU3dFFub3lERF9JUUNRV2d4akR0aURPa3R4T29pWENCU3pjeVZhRktqU0Jjb29HUGxWX3QyVHRlUnVVbFM3YU1rWEFPVWxUemQ5OGZzdjRYZFUyTTFuWFZXQ0NlLTBwZmxXdnM3d1JzRklDaHdhZW1WaDdrM2lnVGpScW93LWp1bWtza2s?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-09-28T04:09:03+00:00</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E383" t="n">
+        <v>7791</v>
+      </c>
+      <c r="F383" t="n">
+        <v>7792.25</v>
+      </c>
+      <c r="G383" t="n">
+        <v>7772.25</v>
+      </c>
+      <c r="H383" t="n">
+        <v>7772.25</v>
+      </c>
+      <c r="I383" t="n">
+        <v>29294</v>
+      </c>
+      <c r="J383" t="n">
+        <v>4</v>
+      </c>
+      <c r="K383" t="n">
+        <v>39</v>
+      </c>
+      <c r="L383" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="M383" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="N383" t="n">
+        <v>40</v>
+      </c>
+      <c r="O383" t="n">
+        <v>0.211</v>
+      </c>
+      <c r="P383" t="n">
+        <v>-0.059</v>
+      </c>
+      <c r="Q383" t="n">
+        <v>9.345000000000001</v>
+      </c>
+      <c r="R383" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S383" t="inlineStr">
+        <is>
+          <t>AbCellera Biologics (ABCL) Surges 34.78% as Shares Break Toward $9.81 Resistance - EMA Signal - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="T383" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPdUNOZndBWm5IMm9JRjRsTk5DNmtNQnR6YTFWMWlSTk5BT3J2TjNEdXlrMFl5Vi1sdDVyY1BybUlUU0taSnQtcktxZEV5ZkpYclc4dnBNa0lzamY3dFFRTGNMWXU5TFk3MUphb1hnak4zYS1vQ0s2NHdTeFFLOGEwdlRkcGE5VUs4a0t2bnk3SkJPMGk2RGM4VV9mclUwZmJQMGUtNXN0dUN5Z2M1U1E0cG5pckZOQlJ2TGdDSg?oc=5</t>
+        </is>
+      </c>
+      <c r="U383" t="inlineStr">
+        <is>
+          <t>Dow surges to record close after a fresh tech rally and a plunge in oil prices - Business Insider</t>
+        </is>
+      </c>
+      <c r="V383" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOS0hLS2NLYi1nYlZnTmRJNTRtQXAyZUh5MExFZUVXcEtOTEhzVF9zeHozLThnVHVETGtwMVBFZFBUb3dVaDJlMmtmTUd6Y2ZmUVhMZjRxck41ZEJDZFNqSG5PRm96VXR6bE9tLWlybXBqVWh4NjRUSUJIcFVjdE9xRml2YWJVYTZvMmM4aTQ5bw?oc=5</t>
+        </is>
+      </c>
+      <c r="W383" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 21: Meta Surges on Excitement Over Muse Personal AI Agent - The Globe and Mail</t>
+        </is>
+      </c>
+      <c r="X383" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxQSWZkbHdXQnI1czhKLV84RzVXWDJvaElPdzNTQlZ4MjZSaENrdzkxN3lHZFFhWV9uR1RPeTZYSnBnSHNPUGM0NERzYkk1dWJfdUR0YjZiYkE2ZFZSb25SbVFUaVBqTFAwSURBOEdDVDhvS1hxMUZrcDZ1NmhIWGV2YjZIU3hHbnE4VUpoRUp6UGh1QUNVYzRSV0NxSXFzOVdiODFrOS11OW5ZODNIWEFXNS1lVFhaT0JVbGdIQ0RlSlV0c2ZaNzlsMnJLenFCNEc4aXBWNUN0VVBTNktTS1B1N3EwN05BbVotUWduMlhlUXFvdzlWdEMwdw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y383" t="inlineStr">
+        <is>
+          <t>If There's a Stock Market Crash Ahead, History Highlights the Best Strategy for Investors - AOL.com</t>
+        </is>
+      </c>
+      <c r="Z383" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxObDRyTS13c3JCdDU5NmNhU3g3NnlUNkpoamlFR1Fic09CTzltRV9zcS1fUUwzdG45dExiY3k3N2c2VnItZ2twWnBZNktPXzItSmRMRVBveS1GdWljRDFpTmtxN3c1OG41a1dhTzFwNU44WkpGTm5oNjMtdzVtaURxVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA383" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AB383" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC383" t="inlineStr">
+        <is>
+          <t>A Bear Market Is Coming Eventually. Here's How I'm Preparing My Investments. - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="AD383" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOZFgxaGViZ3NYZ2xMUmc5YURqMkJKQzMtMGRkV0MyVjZCVUZVaS1hZDJDVlZxY2NCUnk4cExpWXB6ME45YXlyYlJWOW1xWHBJVncxMHczOU11NklXM01DdWhzSG95dHk4MXhCV2x1LUwtdDVTdEdXeGhQaGE2M0pGdEkwbUhSYzN3U2NYeDZwY1B5QkQyazNETDZVZ2JvMUVfQUE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-09-28T04:09:03+00:00</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E384" t="n">
+        <v>30844.5</v>
+      </c>
+      <c r="F384" t="n">
+        <v>30898.25</v>
+      </c>
+      <c r="G384" t="n">
+        <v>30643.25</v>
+      </c>
+      <c r="H384" t="n">
+        <v>30643.25</v>
+      </c>
+      <c r="I384" t="n">
+        <v>23401</v>
+      </c>
+      <c r="J384" t="n">
+        <v>4</v>
+      </c>
+      <c r="K384" t="n">
+        <v>34</v>
+      </c>
+      <c r="L384" t="n">
+        <v>-0.064</v>
+      </c>
+      <c r="M384" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="N384" t="n">
+        <v>35</v>
+      </c>
+      <c r="O384" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="P384" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="Q384" t="n">
+        <v>4.102</v>
+      </c>
+      <c r="R384" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S384" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as chipmakers fuel stock gains - reuters.com</t>
+        </is>
+      </c>
+      <c r="T384" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQUUdXdXVKYkpsa2JoQmRNeVpVWWhwb1pIVmUwcUl0QVRFVEFjRDJtREJPbXJWaXVEc0NQSWZZUlhwTl80T3h4eGM1dE9oaXRsWlVueWx0MWt3YXlWbV9PYkZDWVVPb1ZveThvalZfWnBvQ2J5Sjg1UkNOQmU5eDdWN0FvVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U384" t="inlineStr">
+        <is>
+          <t>Nasdaq gains 2% for the week driven by mid-week tech rally (AMD:NASDAQ) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="V384" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNRTNUV0JnS3haREZESHpOTVREazZUWkNwUE43OEQxMFJYajZnU3JhaWFKOEt1MVEtLTJYdlg5YnVUUnE3WnFnN0FoRDRJUFZlVEpNN2pCaWFpSEQ5NmlIM2hoQ2VDcHNHRHpTcWpiQ1RCVFRPbDd2cExKOF9adGxta2FWMUN1NjRvamQ0QUpYcFBUM2hSZkk4YWVibw?oc=5</t>
+        </is>
+      </c>
+      <c r="W384" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="X384" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y384" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z384" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA384" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB384" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+      <c r="AC384" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - tvnewscheck.com</t>
+        </is>
+      </c>
+      <c r="AD384" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-09-28T04:09:03+00:00</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E385" t="n">
+        <v>84120.9531</v>
+      </c>
+      <c r="F385" t="n">
+        <v>84210.9219</v>
+      </c>
+      <c r="G385" t="n">
+        <v>83190.32030000001</v>
+      </c>
+      <c r="H385" t="n">
+        <v>83354.02340000001</v>
+      </c>
+      <c r="I385" t="n">
+        <v>6422020096</v>
+      </c>
+      <c r="J385" t="n">
+        <v>4</v>
+      </c>
+      <c r="K385" t="n">
+        <v>37</v>
+      </c>
+      <c r="L385" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="M385" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N385" t="n">
+        <v>36</v>
+      </c>
+      <c r="O385" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="P385" t="n">
+        <v>-0.015</v>
+      </c>
+      <c r="Q385" t="n">
+        <v>10.585</v>
+      </c>
+      <c r="R385" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S385" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T385" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U385" t="inlineStr">
+        <is>
+          <t>Bitcoin may reach $94,000 by October 2026, with strong institutional demand and Uptober optimism. - Pluang</t>
+        </is>
+      </c>
+      <c r="V385" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQRXFhOHd4Sl9SZ2I0dEhnbHdtaXFJSWFMXzBsRGRmS0w3c0pzSlpodU9raEE0aVNteWQxUlpKbmhiN3RUaWZscGxIZUZWQ1I4OUduLUQ4b3Q3ejc4d05jd3NscS0yNlNRM1NPU0J0V3BNSDNSQUdHTmVJdGR3cF9XaFhNRVNVUERGbTY2eQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W385" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X385" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y385" t="inlineStr">
+        <is>
+          <t>Institutions Held Their Bitcoin Through Crash — and Some Bought More: Report - Bitcoin Magazine</t>
+        </is>
+      </c>
+      <c r="Z385" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5TejE3cXRtYXN0Qm5POU9ISHVfT3NGQW90UVViWXRxbURFeFc0V3hzSUF3dUhBTUxJS2d5cHpqT1ExRDhmb3RQa1FTdWlxZkZ0TFUyYWF6RkY1LXJjN2NiTk1DRnF6LU1acm51dy1UbGVla29UWmNoeWZ2REY?oc=5</t>
+        </is>
+      </c>
+      <c r="AA385" t="inlineStr">
+        <is>
+          <t>Bitcoin Holders Are Selling, But This Time It’s Different: What You Need to Know - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="AB385" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxNY1pjQzFadG5wOXBrS3lYNVppbjF2eVp3WTBCN0xWa04yWU9jSDZVYkhNRnM2aXg1cFdRZ0FHQVIyRUhfUUNCTHYtaFhjdENNTzJ3ZEJJSVIwMFB0SEZ1RXdYSWdZejFoY0oxbTJlZjBoNWZtMTR2VHFmOEMySnpOMGMxT1NVWXNQOEhoN3pYRjZTQ29VS1NfbDlubTc0b1MzLVcyQTdSYjJGNlBYTVROem9wNUNMSXRhNVJXV3NaWlZfdUdZbHYzTTdjWEgxVFJsM3c?oc=5</t>
+        </is>
+      </c>
+      <c r="AC385" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - global.morningstar.com</t>
+        </is>
+      </c>
+      <c r="AD385" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-28 16:35 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD385"/>
+  <dimension ref="A1:AD391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48485,6 +48485,762 @@
       <c r="AD385" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-09-28T16:33:01+00:00</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E386" t="n">
+        <v>4186.1001</v>
+      </c>
+      <c r="F386" t="n">
+        <v>4193.2002</v>
+      </c>
+      <c r="G386" t="n">
+        <v>4143.1001</v>
+      </c>
+      <c r="H386" t="n">
+        <v>4162.3999</v>
+      </c>
+      <c r="I386" t="n">
+        <v>57335</v>
+      </c>
+      <c r="J386" t="n">
+        <v>4</v>
+      </c>
+      <c r="K386" t="n">
+        <v>40</v>
+      </c>
+      <c r="L386" t="n">
+        <v>-0.022</v>
+      </c>
+      <c r="M386" t="n">
+        <v>-0.017</v>
+      </c>
+      <c r="N386" t="n">
+        <v>40</v>
+      </c>
+      <c r="O386" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="P386" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="Q386" t="n">
+        <v>-0.156</v>
+      </c>
+      <c r="R386" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S386" t="inlineStr">
+        <is>
+          <t>Silver hits record high above $100/oz as gold closes in on $5,000 milestone - CNBC</t>
+        </is>
+      </c>
+      <c r="T386" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPR2ZOdnZ4aThnN0lBV01aSE9BMXBjZVc1U1NyekxkSU11d1VDYXM4LUtEV042aW52YmJGNzEtQTlBNjUzWE8yNkRoaW4yVkwyeGlHcXZkTEljZTFmZi0zejNWekFWMHBqcVJCeTJyLUp5bG9oUWVsUnhvV21UYWRLd3YydTBIbW4wSlBHLURxWmgzVzRWNWdZN2h30gGfAUFVX3lxTFBqOWgxMXdKRzlZNUtyemMyaUV0TXI5Z3lSM0NiNDhOUWhTZnFGMHpsRURaUGJUWVVxalZtNFpyNXJ0UWE3TTNIWEtvQUYxQlJRRlFkU0RhOFJ4TE1tRVB1cDJfM1d3M3ZKX29LQ2JqR1R3YTBzc0F2eF8tRFVYa1RIVkdINmxOWE42MXpMbEEyd2xOM3RHOUF6YTAwRjZ3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="U386" t="inlineStr">
+        <is>
+          <t>Gold rises above $4,130 as geopolitical uncertainty supports safe-haven demand - finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="V386" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPVC0wdnlpU1I2eWVTbnhmbHhvdFBmWUM4c3J4dk9NZFVBMGZBOVBJall6QmY2UkxxTm15TS1ycGs1ZW42RFFNaWdiUlJuajNKWmhOZ0sxYWlOSUZpcTAySkV3NHhST0dGRVZtVmVVVmt4WFFja2hjOW1RVVF5UFdGaUxaOXhOSTUwX21ab1FQQlh4dE0yOUVn?oc=5</t>
+        </is>
+      </c>
+      <c r="W386" t="inlineStr">
+        <is>
+          <t>Gold hits record high as investors seek safety - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="X386" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVWt1Y1hBWG5uZFNjRUFtZHlqRUhfZGV6VzAtQ0tBT2VlVDVEZEJ2WHN0YndCcXRzSjNtVnFhUFZZZ2F4RFRxYkdsSF91eDk2MFl5R3JNWk1HREJjSVdhUE1uTTU1N1Z6Y2xfZzZCSDZ4YnhaT1czcWdXeHE3SjJBR2FqUm43Z0paUG5OVEdsWVdYYnZBWVHSAZsBQVVfeXFMTWh6VXlqZGZVbUl3SHVfQ195WFFveEVkLU9TU1RXMTZBdVhodU16UWxLLWVScDNsc2VGMThyT0RTTHB4SVNRYU1KWmRycHhnTEc0NTJ1RWgzdGc2Y0VkanR4QUtlUWFBSnB2cElORUltQk9XdWRLNXhKbU5jRUFqQVd6bG5YbURJakxhNTl3UEk4RzBaQzVJaVdRdFk?oc=5</t>
+        </is>
+      </c>
+      <c r="Y386" t="inlineStr">
+        <is>
+          <t>Gold - Breaks Key Support As Rising US Yields Sap Demand - eFXdata</t>
+        </is>
+      </c>
+      <c r="Z386" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE1vWmp3NWY1TURNaGVjOGM0Q2h3UWdPT19qNzJKa1VPeFVOYnBDcG5IZ2lrd2JQdmdDZ2xTYUc2cFc2QmRLbkFjbHQyWjUwTlgzOEhWWFRnYzdjS3JGVFZOTnkxclY1V0tyUE54SVNUT0VaNlBLTHBRcmFB0gF_QVVfeXFMUHlzQjl2bW4zTlllTUFwbndXQ2VGMGVmNDdMbHM3T1haTjdIWno3Y0dsNVJ1ajRlT2NIZEFJcS00VzFLZDcwZEl5SHJmOWxjV0lJWXJ2MFEwMi1rSUY2VDNqX3Vtd3RGYkxfUzNZUS1wa0xWYzdreWluR3h1dmtKcw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA386" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AB386" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC386" t="inlineStr">
+        <is>
+          <t>Gold ETFs Shine in H1 2026 with Unprecedented Liquidity - Investing News Network</t>
+        </is>
+      </c>
+      <c r="AD386" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE1JaGRkaHpGODN4bGpQdFl6S3VyUjZKYzRvWUxjUjhyQ0lVXzZMZEltdGkwMEo2d0lhVWVmMDVUYUJfRXF4emdyX0ZTd0N6SVgwN3kxMFVXTkt5WXZJbE8ybVNRLUJYTVZy?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-09-28T16:33:01+00:00</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E387" t="n">
+        <v>94.23999999999999</v>
+      </c>
+      <c r="F387" t="n">
+        <v>95.7</v>
+      </c>
+      <c r="G387" t="n">
+        <v>93.14</v>
+      </c>
+      <c r="H387" t="n">
+        <v>93.25</v>
+      </c>
+      <c r="I387" t="n">
+        <v>102390</v>
+      </c>
+      <c r="J387" t="n">
+        <v>4</v>
+      </c>
+      <c r="K387" t="n">
+        <v>40</v>
+      </c>
+      <c r="L387" t="n">
+        <v>-0.08400000000000001</v>
+      </c>
+      <c r="M387" t="n">
+        <v>-0.197</v>
+      </c>
+      <c r="N387" t="n">
+        <v>40</v>
+      </c>
+      <c r="O387" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="P387" t="n">
+        <v>-0.103</v>
+      </c>
+      <c r="Q387" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="R387" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S387" t="inlineStr">
+        <is>
+          <t>Russian oil supply to India tightens on reduced exports, strong Chinese demand - marketscreener.com</t>
+        </is>
+      </c>
+      <c r="T387" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNRXJ2bElPQ1kzYWFxQWxuN01qRmdIUHdoelBHdlRMNUF6THo0RldHWDVqMm8yTTAwSzRVYUctTEc0VmV3ajFPQkJ0QVZYSzJqb1RjNG1HcGVpXzh3VXc3NGYycHV3ZU5VQnV2djZGQllXOHNXTzJNU3JFSHhXQ284dklmaTVob3Q5TzRJaXdjYkM1M1JKamxUc3Q4dzBtaFIzcEJvLTlnTkYzbkFlNGpJYUhIbm1Nak5VSm5TN1FjRm81VHFmdlVRdTBB?oc=5</t>
+        </is>
+      </c>
+      <c r="U387" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="V387" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W387" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="X387" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y387" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 28, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z387" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9rRk9pZkN0bERaRFVvU0wyVmU3SVQwWEpsYm1EMkR1eWg5dnJjNDBzNGlpZHpyVmFiRUlJYUF1MnhYMnFSalRMWXRSWWZfWHpNX0hJNXJyaTg2T2ZKckNOSFVn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA387" t="inlineStr">
+        <is>
+          <t>OPEC Monthly Oil Market Report, September 2026 - Peak Oil Barrel</t>
+        </is>
+      </c>
+      <c r="AB387" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9faVVpVXlFX1hFRG4tM2FnZTE5Q1ROMG1RWmxCTWVWcTdLcmo0VlBIbTlQcnhYOUQxeUxvaTE4VVo5Ulo3cExYYVViZUxWcU9VUzRIRXhQRTJLb19hWFhJc2V5WkxmMGhtSk92QVJndFZlV1NQeWxkM2Z3WWc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC387" t="inlineStr">
+        <is>
+          <t>Oil falls on oversupply after Hormuz reopening; Michigan sentiment improves - equiti.com</t>
+        </is>
+      </c>
+      <c r="AD387" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQNW5vUTdIRGFyRVl2N2RoaktRTEFFdFh5al9GckxJSVJOd1V6UkR0UzdzMFNrVlAyRnMzZGVUOUM0S2x6WWcwc0ZZR2kwb2o1TVYxRl9pdG9hMWlrc3NDdEJYWU1aZjEtSVVrRnVqMTEzVEEwNUNRV3JiT2pVY2pPeXBiTG44YUtLcTFKUHdXMEIwMmk2cVFQN04zamI2MTN6Nm9LOWdTY3lnMWduazh6OGpXeW5SVjZOVHgyeUxR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-09-28T16:33:01+00:00</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E388" t="n">
+        <v>101.162</v>
+      </c>
+      <c r="F388" t="n">
+        <v>101.308</v>
+      </c>
+      <c r="G388" t="n">
+        <v>101.125</v>
+      </c>
+      <c r="H388" t="n">
+        <v>101.132</v>
+      </c>
+      <c r="I388" t="n">
+        <v>0</v>
+      </c>
+      <c r="J388" t="n">
+        <v>4</v>
+      </c>
+      <c r="K388" t="n">
+        <v>40</v>
+      </c>
+      <c r="L388" t="n">
+        <v>-0.155</v>
+      </c>
+      <c r="M388" t="n">
+        <v>0.141</v>
+      </c>
+      <c r="N388" t="n">
+        <v>40</v>
+      </c>
+      <c r="O388" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="P388" t="n">
+        <v>-0.028</v>
+      </c>
+      <c r="Q388" t="n">
+        <v>-0.348</v>
+      </c>
+      <c r="R388" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S388" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T388" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U388" t="inlineStr">
+        <is>
+          <t>United States Dollar Index remains stronger as hawkish Fed signals drive rate hike bets - FXStreet</t>
+        </is>
+      </c>
+      <c r="V388" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOUHRaUk85MWJmMkZjUlFUM01CQktxTmF4VDM1NFNsS056S0NuMjM5RXo3U2hqaURkQkctUXdWWHUzdmFJWW9OazJfaWs1T1Z0SDdMaUJWYng4TmZ3LVBNRjVqdlpNc0wtaFAxSWdxUTBuQ0liNHU2bjBQMW5KSXUtWG0ydFRYcTBORk1xdm1OZzg4bC12blBhS3gxSFF0QUZGREpBTzVUdFh3ZXV0Tkpja1VRMjN4bFJRSmtjMUV3RmxXbkQxWTZndUV3?oc=5</t>
+        </is>
+      </c>
+      <c r="W388" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X388" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y388" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z388" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA388" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB388" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC388" t="inlineStr">
+        <is>
+          <t>British Pound gains as US Dollar weakens despite hawkish Fed, geopolitical tensions - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD388" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPS2g2djM3bEE4SmNheEM2X09OUDBWaTRYNFdaOWJKVDZpWHkzRlp1SVFENXJOR0VDQTNmQWx5bVU3dFFub3lERF9JUUNRV2d4akR0aURPa3R4T29pWENCU3pjeVZhRktqU0Jjb29HUGxWX3QyVHRlUnVVbFM3YU1rWEFPVWxUemQ5OGZzdjRYZFUyTTFuWFZXQ0NlLTBwZmxXdnM3d1JzRklDaHdhZW1WaDdrM2lnVGpScW93LWp1bWtza2s?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-09-28T16:33:01+00:00</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E389" t="n">
+        <v>7780.5</v>
+      </c>
+      <c r="F389" t="n">
+        <v>7780.5</v>
+      </c>
+      <c r="G389" t="n">
+        <v>7726</v>
+      </c>
+      <c r="H389" t="n">
+        <v>7767.75</v>
+      </c>
+      <c r="I389" t="n">
+        <v>708755</v>
+      </c>
+      <c r="J389" t="n">
+        <v>4</v>
+      </c>
+      <c r="K389" t="n">
+        <v>39</v>
+      </c>
+      <c r="L389" t="n">
+        <v>0.166</v>
+      </c>
+      <c r="M389" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="N389" t="n">
+        <v>40</v>
+      </c>
+      <c r="O389" t="n">
+        <v>0.247</v>
+      </c>
+      <c r="P389" t="n">
+        <v>-0.068</v>
+      </c>
+      <c r="Q389" t="n">
+        <v>7.67</v>
+      </c>
+      <c r="R389" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S389" t="inlineStr">
+        <is>
+          <t>AbCellera Biologics (ABCL) Surges 34.78% as Shares Break Toward $9.81 Resistance - EMA Signal - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="T389" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPdUNOZndBWm5IMm9JRjRsTk5DNmtNQnR6YTFWMWlSTk5BT3J2TjNEdXlrMFl5Vi1sdDVyY1BybUlUU0taSnQtcktxZEV5ZkpYclc4dnBNa0lzamY3dFFRTGNMWXU5TFk3MUphb1hnak4zYS1vQ0s2NHdTeFFLOGEwdlRkcGE5VUs4a0t2bnk3SkJPMGk2RGM4VV9mclUwZmJQMGUtNXN0dUN5Z2M1U1E0cG5pckZOQlJ2TGdDSg?oc=5</t>
+        </is>
+      </c>
+      <c r="U389" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 9: Meta Surges Over 6.5% on Muse AI Agent Launch - finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="V389" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPSEdBOEZMVVlEODVXN3FfVjlfYnUtV2NDMEtpRkwyeUkxeHBUb2Nfc2FaYzZ2VE9QbDU5NjJNV2o0cG5MN19UcGc5OFk3R09pWVpGckptOFJJdXdnbkhxOXdQZzhrNmk3OEw4M3pVdjNEUTI5Q1dzRzE1M3lDYno4Wlp2TnV1c0JBcnViMVROYnVuLUFT?oc=5</t>
+        </is>
+      </c>
+      <c r="W389" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 rises 1.2%, nearing record high despite slower GDP growth forecast - Pluang</t>
+        </is>
+      </c>
+      <c r="X389" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQYkF1MzJGdi1STjFWVG5jeG1pRVRCZXZWRUxZMGh6OGVjYkdCVWduNHVsWnBIUzRpNEJiZ0JwTHpHOTNyMGJuNzVGTllHRG45RDJYSFNacHJMMnJ4SFczN2pFbFhSZFl0RDNRaXl4T3E0ZEZfNEhVeW5WY3d0OWZSdTFXWXNTRUNLaFF4TEJYQ2Q3OTFnTm1yYUIxMExJdw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y389" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z389" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA389" t="inlineStr">
+        <is>
+          <t>Nanobiotix stock breaks through 27.94 € support level, lagging the SBF 120 index - Ideal Investisseur</t>
+        </is>
+      </c>
+      <c r="AB389" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNam1pVTNZWEFqODA0WlNlVkhwVWpNQ1hZYmpKR085TVZtU1lMREhQZENQUXdUTGlzSGpHa3MySTVSTWo0OG5rZFhFVkYyM1JORDZzWTNJV0tXanBSVVZnOE5wRFhuZVBrSFNQUzVJbU44bWVrZnN6emhoZi0tZW5EZGU2WHAxZHBjNkd4OVZIU3BjUFcxREE0NGVkSVRBYW1WMTZjd1o3d0E1d0tORVBza2YtTzNRS3N2ZEdlWjhGR3l2N1ZfMHRKVEVtbHhJWWppUUVQSktHZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC389" t="inlineStr">
+        <is>
+          <t>Wall Street split on gold price path after drop below $4,300, Main Street maintains bullish majority as jobs take center stage - Kitco</t>
+        </is>
+      </c>
+      <c r="AD389" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQbWtUQVJKczJHZ1lWRDRZUEpOc1JuMVJHNmxQR18wSFlJbWJaemlYMXozWXdJTXRxRDVzWWRnWVFobWJCWEZqdUVqa2VMemE3NlI0MDJKdVFBWkJ0a3NrZE01WEJ2NS1mVUhaLTJYNnM4MUdHNHlDTnhYa0JZdS1lN2Vqdk5YOUhhWlhkMXc3S3pFaURQeFVKUU9pbVN5cWYzY0FwdThESE1IQ2JMVEo3T2JZbw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-09-28T16:33:01+00:00</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E390" t="n">
+        <v>30739.25</v>
+      </c>
+      <c r="F390" t="n">
+        <v>30759.25</v>
+      </c>
+      <c r="G390" t="n">
+        <v>30356.75</v>
+      </c>
+      <c r="H390" t="n">
+        <v>30635.25</v>
+      </c>
+      <c r="I390" t="n">
+        <v>299378</v>
+      </c>
+      <c r="J390" t="n">
+        <v>4</v>
+      </c>
+      <c r="K390" t="n">
+        <v>36</v>
+      </c>
+      <c r="L390" t="n">
+        <v>-0.044</v>
+      </c>
+      <c r="M390" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="N390" t="n">
+        <v>37</v>
+      </c>
+      <c r="O390" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="P390" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="Q390" t="n">
+        <v>4.112</v>
+      </c>
+      <c r="R390" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S390" t="inlineStr">
+        <is>
+          <t>Three AI chip stocks are outperforming the 50-day SMA amid the Nasdaq rally. - KuCoin</t>
+        </is>
+      </c>
+      <c r="T390" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQaUhtRWpGemZZSlRpcXdhU2hBY012YlgtRzFEX1lzQ2ZYU0ptSUszQUtyYlFWQ2VhOWJnYnY2a3RnNG5mZTVaeXM2WEpKXzE2cWVlS0dtSjZzTG5yTzVJZ0xmN3lTcEFZNjRCUmlNaWUwVW5uY3pNa3ZOdEdDalJhR0N2SXBDYW5aeDdWNm90RFJzbVB3QVBaZ1V5TktHQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U390" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="V390" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W390" t="inlineStr">
+        <is>
+          <t>Nasdaq indices surge as buyers break above key resistance - investingLive</t>
+        </is>
+      </c>
+      <c r="X390" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNQTZPX3FUV2ZpQ1NIekg5VHBoTm85UFFqaFg5clBON19hejFFX2pPVlA1VjdKODAxWll5azI0cUpid2NsVVBiYmpILVFJRzFFeWV3N1pfLWMzV05Xb3VWc3BIUllaQXJPclFKU3g3bWNNa0ROcklaWEd4U2owRC1ZWlJpRGwzV0l3Smtzd2ItYmtWcXlWWGc?oc=5</t>
+        </is>
+      </c>
+      <c r="Y390" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z390" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA390" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AB390" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+      <c r="AC390" t="inlineStr">
+        <is>
+          <t>Nasdaq Breaks Support As Chip Sell-Off Deepens; Knight-Swift, Canadian Pacific, AbbVie In Focus - Video - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD390" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOa0VQNUt2ZDVDYmZpdDB6V3lwVVdxemtUWU5xU0wyTHVKdmtuNzJEU29WUGNSVkNtRjFXV0xIRnQ5N3RodFF3d2JyOFBBbkZQTDVrZWV3R2QzeWctZ1JCS09Bc2VOU2JqWnM4VnlMZjFQVUh2VHNqdzBocUJ3Zm5XSTQ2b19jU3pvZFhvYWNucF9ydU5uLVhqNWN0SDUxZ3BKMXdN?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-09-28T16:33:01+00:00</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E391" t="n">
+        <v>83549.1406</v>
+      </c>
+      <c r="F391" t="n">
+        <v>84158.14840000001</v>
+      </c>
+      <c r="G391" t="n">
+        <v>82573.5</v>
+      </c>
+      <c r="H391" t="n">
+        <v>83939.1719</v>
+      </c>
+      <c r="I391" t="n">
+        <v>6773606400</v>
+      </c>
+      <c r="J391" t="n">
+        <v>4</v>
+      </c>
+      <c r="K391" t="n">
+        <v>39</v>
+      </c>
+      <c r="L391" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M391" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="N391" t="n">
+        <v>35</v>
+      </c>
+      <c r="O391" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="P391" t="n">
+        <v>-0.049</v>
+      </c>
+      <c r="Q391" t="n">
+        <v>10.606</v>
+      </c>
+      <c r="R391" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S391" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T391" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U391" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="V391" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W391" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X391" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y391" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - Morningstar</t>
+        </is>
+      </c>
+      <c r="Z391" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA391" t="inlineStr">
+        <is>
+          <t>Bitcoin Long Liquidations Reach $10.36 Million in One Hour - tokenpost.com</t>
+        </is>
+      </c>
+      <c r="AB391" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5yS3RCWGxyU3ljd213Nk1UZm1OYWluX0MxcDJ1SE1uQlAxZkJGcDhqX1doNXB6RmhlNW9KYXRITWtBMS1BVFRvMzJxbkJlVi1XMUdaQnNWeGNQUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC391" t="inlineStr">
+        <is>
+          <t>Hunter Biden’s ‘$LAPTOP’ crypto coin crashes minutes after launch - The Washington Post</t>
+        </is>
+      </c>
+      <c r="AD391" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNNlBPY25HX1E5UmZ2LVE1MmhmYjBEcEkzaTY5WlpGUmdZc2JURlVzYVRTNzBROF95OHdaTXhHX1lJY3pEdl9XNVl1ek1oblk4c0VPTEt6TGJ6a1pPSGJqWTMyNGJNYVpRNml0UlhiMWJHVTVlOW9WLVRFck9QMkZnSTJJRm1CWVUyRkhURnV2SHZJNTJwOWtpTUZtU3pKOVdUYTBIWGp5NVE0ZFdUbGFtZ1RqTQ?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-29 00:17 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD391"/>
+  <dimension ref="A1:AD397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49241,6 +49241,762 @@
       <c r="AD391" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNNlBPY25HX1E5UmZ2LVE1MmhmYjBEcEkzaTY5WlpGUmdZc2JURlVzYVRTNzBROF95OHdaTXhHX1lJY3pEdl9XNVl1ek1oblk4c0VPTEt6TGJ6a1pPSGJqWTMyNGJNYVpRNml0UlhiMWJHVTVlOW9WLVRFck9QMkZnSTJJRm1CWVUyRkhURnV2SHZJNTJwOWtpTUZtU3pKOVdUYTBIWGp5NVE0ZFdUbGFtZ1RqTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-09-29T00:15:55+00:00</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E392" t="n">
+        <v>4156.1001</v>
+      </c>
+      <c r="F392" t="n">
+        <v>4161.3999</v>
+      </c>
+      <c r="G392" t="n">
+        <v>4144.2002</v>
+      </c>
+      <c r="H392" t="n">
+        <v>4155.3999</v>
+      </c>
+      <c r="I392" t="n">
+        <v>6769</v>
+      </c>
+      <c r="J392" t="n">
+        <v>4</v>
+      </c>
+      <c r="K392" t="n">
+        <v>39</v>
+      </c>
+      <c r="L392" t="n">
+        <v>-0.157</v>
+      </c>
+      <c r="M392" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="N392" t="n">
+        <v>40</v>
+      </c>
+      <c r="O392" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="P392" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="Q392" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="R392" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S392" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - azernews.az</t>
+        </is>
+      </c>
+      <c r="T392" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U392" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="V392" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="W392" t="inlineStr">
+        <is>
+          <t>Gold Q4 2026 outlook: Resilience in the face of rallying dollar and yields - stonex.com</t>
+        </is>
+      </c>
+      <c r="X392" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNTko5U0Y2X2ZERERoQ2VBTW5KUTdpSlNwX1Z1OEpjMDZuZDN5ZkllVE9nSjhrRnU5anZyaXVtVkF6aHZWQUhiOHJrNFpoYi1vUkhsYXVvcTNjekRwNVBtM0ZIeUJ2NEctSDBGWlUwMEVoTDdqQmUwMktvVXU4bzZTUXNLaFByaG1sRy11OEhHQ0pudDR3ZHJlTGc5a1JHRWtVeHRob1FzYzBzdDA5SXhMeFlaTGJpUUZBVW1sYy12TEM?oc=5</t>
+        </is>
+      </c>
+      <c r="Y392" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="Z392" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA392" t="inlineStr">
+        <is>
+          <t>Gold ETFs Shine in H1 2026 with Unprecedented Liquidity - Investing News Network</t>
+        </is>
+      </c>
+      <c r="AB392" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE1JaGRkaHpGODN4bGpQdFl6S3VyUjZKYzRvWUxjUjhyQ0lVXzZMZEltdGkwMEo2d0lhVWVmMDVUYUJfRXF4emdyX0ZTd0N6SVgwN3kxMFVXTkt5WXZJbE8ybVNRLUJYTVZy?oc=5</t>
+        </is>
+      </c>
+      <c r="AC392" t="inlineStr">
+        <is>
+          <t>Gold breaks below $4,200 with RSI at 28.6: Live levels - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD392" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQMFF4cXpFOXY3cWx4YlB4eGVMYkRadXJvQW03Y1k0ZjJJMTloM2Q4OTczYzZ1cW5ZT3VPN3FCcFRVQ0J2RmlROS1pZ1dtZ3ozNVd5cjR6bExESG52QzN3Z2FuWThjcVJmQVdJT0JSaU1uRzB2MVVlMGptNXRKN3pGUWd6X0wzZnZMRFl1VVZOY1pyd1RiNmY5T0lKOHA4eFlfVlp1UWlNcElaV04tM1ZKTw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-09-29T00:15:55+00:00</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E393" t="n">
+        <v>93.23</v>
+      </c>
+      <c r="F393" t="n">
+        <v>93.77</v>
+      </c>
+      <c r="G393" t="n">
+        <v>92.83</v>
+      </c>
+      <c r="H393" t="n">
+        <v>93.45</v>
+      </c>
+      <c r="I393" t="n">
+        <v>6900</v>
+      </c>
+      <c r="J393" t="n">
+        <v>4</v>
+      </c>
+      <c r="K393" t="n">
+        <v>40</v>
+      </c>
+      <c r="L393" t="n">
+        <v>-0.147</v>
+      </c>
+      <c r="M393" t="n">
+        <v>-0.188</v>
+      </c>
+      <c r="N393" t="n">
+        <v>40</v>
+      </c>
+      <c r="O393" t="n">
+        <v>0.257</v>
+      </c>
+      <c r="P393" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="Q393" t="n">
+        <v>2.199</v>
+      </c>
+      <c r="R393" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S393" t="inlineStr">
+        <is>
+          <t>Russian oil supply to India tightens on reduced exports, strong Chinese demand - marketscreener.com</t>
+        </is>
+      </c>
+      <c r="T393" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNRXJ2bElPQ1kzYWFxQWxuN01qRmdIUHdoelBHdlRMNUF6THo0RldHWDVqMm8yTTAwSzRVYUctTEc0VmV3ajFPQkJ0QVZYSzJqb1RjNG1HcGVpXzh3VXc3NGYycHV3ZU5VQnV2djZGQllXOHNXTzJNU3JFSHhXQ284dklmaTVob3Q5TzRJaXdjYkM1M1JKamxUc3Q4dzBtaFIzcEJvLTlnTkYzbkFlNGpJYUhIbm1Nak5VSm5TN1FjRm81VHFmdlVRdTBB?oc=5</t>
+        </is>
+      </c>
+      <c r="U393" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="V393" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W393" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="X393" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y393" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 28, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z393" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9rRk9pZkN0bERaRFVvU0wyVmU3SVQwWEpsYm1EMkR1eWg5dnJjNDBzNGlpZHpyVmFiRUlJYUF1MnhYMnFSalRMWXRSWWZfWHpNX0hJNXJyaTg2T2ZKckNOSFVn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA393" t="inlineStr">
+        <is>
+          <t>OPEC Monthly Oil Market Report, September 2026 - Peak Oil Barrel</t>
+        </is>
+      </c>
+      <c r="AB393" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9faVVpVXlFX1hFRG4tM2FnZTE5Q1ROMG1RWmxCTWVWcTdLcmo0VlBIbTlQcnhYOUQxeUxvaTE4VVo5Ulo3cExYYVViZUxWcU9VUzRIRXhQRTJLb19hWFhJc2V5WkxmMGhtSk92QVJndFZlV1NQeWxkM2Z3WWc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC393" t="inlineStr">
+        <is>
+          <t>Brent Oil breaks $101.50 neckline, eyes $97.49 support: Live By Investing.com - Investing.com Nigeria</t>
+        </is>
+      </c>
+      <c r="AD393" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQcjJSZzJxN1ZmdFlDSmtsYXZhbU5xdUNxMV9MSFYyTS10RHNhV2kxSDJfSEVDZ00zRTFWZlJaVmU2dnktYUVLTUNSWExUU2k1Mi1Jd3hzaW53OXc5d0lrM1JLbXZMbkdELUhKWFIwbGJoNFlWZDFfdFByRW1iUDJ6OGlpTUdaQjRDYS10MVo1eE5fUktYd0ZVeUZIWDdRaGdWaDlubHVpR2Q3U1VXekNGUDZZNUVMdw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-09-29T00:15:55+00:00</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E394" t="n">
+        <v>101.19</v>
+      </c>
+      <c r="F394" t="n">
+        <v>101.231</v>
+      </c>
+      <c r="G394" t="n">
+        <v>101.167</v>
+      </c>
+      <c r="H394" t="n">
+        <v>101.226</v>
+      </c>
+      <c r="I394" t="n">
+        <v>0</v>
+      </c>
+      <c r="J394" t="n">
+        <v>4</v>
+      </c>
+      <c r="K394" t="n">
+        <v>40</v>
+      </c>
+      <c r="L394" t="n">
+        <v>-0.201</v>
+      </c>
+      <c r="M394" t="n">
+        <v>0.126</v>
+      </c>
+      <c r="N394" t="n">
+        <v>40</v>
+      </c>
+      <c r="O394" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="P394" t="n">
+        <v>-0.014</v>
+      </c>
+      <c r="Q394" t="n">
+        <v>-2.33</v>
+      </c>
+      <c r="R394" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S394" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T394" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U394" t="inlineStr">
+        <is>
+          <t>United States Dollar Index remains stronger as hawkish Fed signals drive rate hike bets - FXStreet</t>
+        </is>
+      </c>
+      <c r="V394" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOUHRaUk85MWJmMkZjUlFUM01CQktxTmF4VDM1NFNsS056S0NuMjM5RXo3U2hqaURkQkctUXdWWHUzdmFJWW9OazJfaWs1T1Z0SDdMaUJWYng4TmZ3LVBNRjVqdlpNc0wtaFAxSWdxUTBuQ0liNHU2bjBQMW5KSXUtWG0ydFRYcTBORk1xdm1OZzg4bC12blBhS3gxSFF0QUZGREpBTzVUdFh3ZXV0Tkpja1VRMjN4bFJRSmtjMUV3RmxXbkQxWTZndUV3?oc=5</t>
+        </is>
+      </c>
+      <c r="W394" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X394" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y394" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z394" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA394" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB394" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC394" t="inlineStr">
+        <is>
+          <t>British Pound gains as US Dollar weakens despite hawkish Fed, geopolitical tensions - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD394" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPS2g2djM3bEE4SmNheEM2X09OUDBWaTRYNFdaOWJKVDZpWHkzRlp1SVFENXJOR0VDQTNmQWx5bVU3dFFub3lERF9JUUNRV2d4akR0aURPa3R4T29pWENCU3pjeVZhRktqU0Jjb29HUGxWX3QyVHRlUnVVbFM3YU1rWEFPVWxUemQ5OGZzdjRYZFUyTTFuWFZXQ0NlLTBwZmxXdnM3d1JzRklDaHdhZW1WaDdrM2lnVGpScW93LWp1bWtza2s?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-09-29T00:15:55+00:00</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E395" t="n">
+        <v>7746.25</v>
+      </c>
+      <c r="F395" t="n">
+        <v>7752.75</v>
+      </c>
+      <c r="G395" t="n">
+        <v>7740.5</v>
+      </c>
+      <c r="H395" t="n">
+        <v>7749.5</v>
+      </c>
+      <c r="I395" t="n">
+        <v>55086</v>
+      </c>
+      <c r="J395" t="n">
+        <v>4</v>
+      </c>
+      <c r="K395" t="n">
+        <v>39</v>
+      </c>
+      <c r="L395" t="n">
+        <v>0.181</v>
+      </c>
+      <c r="M395" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="N395" t="n">
+        <v>39</v>
+      </c>
+      <c r="O395" t="n">
+        <v>0.323</v>
+      </c>
+      <c r="P395" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="Q395" t="n">
+        <v>9.843999999999999</v>
+      </c>
+      <c r="R395" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S395" t="inlineStr">
+        <is>
+          <t>Navitas Semiconductor stock surges 20% on U.S. defense contract - Investing.com</t>
+        </is>
+      </c>
+      <c r="T395" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQNEh0SWNBYm1CU01OYXNoTkU3aUl4RmN6X21XS1I4ejBTbnNCMXJKZXFHRWdhc3FUNm1BcFYxakdQMlNCSzg4a1J3UUo0RC1BMC1OeGVRUXVScmJnUkR5VGhBWjRqQkg1dUEzUmdRcFk2b1VBT1RoNWx0SjJ6T241ZkhyVndHR2w2YURDTm11N2x2WnVmWUgyVXRxYUxrdTdZTW90MC0zZ3ZBNlNyWWRHaHNueUQ3YTBa?oc=5</t>
+        </is>
+      </c>
+      <c r="U395" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 9: Meta Surges Over 6.5% on Muse AI Agent Launch - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="V395" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPSEdBOEZMVVlEODVXN3FfVjlfYnUtV2NDMEtpRkwyeUkxeHBUb2Nfc2FaYzZ2VE9QbDU5NjJNV2o0cG5MN19UcGc5OFk3R09pWVpGckptOFJJdXdnbkhxOXdQZzhrNmk3OEw4M3pVdjNEUTI5Q1dzRzE1M3lDYno4Wlp2TnV1c0JBcnViMVROYnVuLUFT?oc=5</t>
+        </is>
+      </c>
+      <c r="W395" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 rises 1.2%, nearing record high despite slower GDP growth forecast - Pluang</t>
+        </is>
+      </c>
+      <c r="X395" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQYkF1MzJGdi1STjFWVG5jeG1pRVRCZXZWRUxZMGh6OGVjYkdCVWduNHVsWnBIUzRpNEJiZ0JwTHpHOTNyMGJuNzVGTllHRG45RDJYSFNacHJMMnJ4SFczN2pFbFhSZFl0RDNRaXl4T3E0ZEZfNEhVeW5WY3d0OWZSdTFXWXNTRUNLaFF4TEJYQ2Q3OTFnTm1yYUIxMExJdw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y395" t="inlineStr">
+        <is>
+          <t>Dow Drops 352, Nasdaq Sinks 308, S&amp;P 500 Falls 59 - TV News Check</t>
+        </is>
+      </c>
+      <c r="Z395" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOU01EZGE0SW03eXhMd0NqUFllNlVQUHBhcG83aTE2NmVHR09yLWdYZ3pRV3pNeTZ3a1dCQXB6UTd3MHZXenlNc2N1UzlWSm5kd2FzNjA0cVV6NmVXNEgtcHlma09OZzhfZVNZRk0xdmgyblZnb1k2aXd1RjlwNXk5cVI3STR2RUlRcklTSXRpbFlTdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA395" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AB395" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC395" t="inlineStr">
+        <is>
+          <t>Nanobiotix stock breaks through 27.94 € support level, lagging the SBF 120 index - Ideal Investisseur</t>
+        </is>
+      </c>
+      <c r="AD395" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNam1pVTNZWEFqODA0WlNlVkhwVWpNQ1hZYmpKR085TVZtU1lMREhQZENQUXdUTGlzSGpHa3MySTVSTWo0OG5rZFhFVkYyM1JORDZzWTNJV0tXanBSVVZnOE5wRFhuZVBrSFNQUzVJbU44bWVrZnN6emhoZi0tZW5EZGU2WHAxZHBjNkd4OVZIU3BjUFcxREE0NGVkSVRBYW1WMTZjd1o3d0E1d0tORVBza2YtTzNRS3N2ZEdlWjhGR3l2N1ZfMHRKVEVtbHhJWWppUUVQSktHZw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-09-29T00:15:55+00:00</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E396" t="n">
+        <v>30567</v>
+      </c>
+      <c r="F396" t="n">
+        <v>30616</v>
+      </c>
+      <c r="G396" t="n">
+        <v>30533</v>
+      </c>
+      <c r="H396" t="n">
+        <v>30585.75</v>
+      </c>
+      <c r="I396" t="n">
+        <v>22788</v>
+      </c>
+      <c r="J396" t="n">
+        <v>4</v>
+      </c>
+      <c r="K396" t="n">
+        <v>36</v>
+      </c>
+      <c r="L396" t="n">
+        <v>-0.053</v>
+      </c>
+      <c r="M396" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="N396" t="n">
+        <v>37</v>
+      </c>
+      <c r="O396" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="P396" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="Q396" t="n">
+        <v>4.717</v>
+      </c>
+      <c r="R396" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S396" t="inlineStr">
+        <is>
+          <t>Tech Stocks Surge as Apple (AAPL) Hits Record High - GuruFocus</t>
+        </is>
+      </c>
+      <c r="T396" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPbUtsdjFuWFdnMjZ2b2RGMjQzVzhXSG03Y1dYUmxXNmxjZlhiRkx3aVRPbEhyWk1XX3I0UUw3bjVkVTFzR2JTc1hSTFVEUVlSbnVDZm9rb0lCZFNvRnZKdnJ2ZjBhU1J2Tzl2V1VJY3UwckZqTE53YXdZdW10M3gxdUFxN1o2LUVjWkhDZXlnM18?oc=5</t>
+        </is>
+      </c>
+      <c r="U396" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq, Dow Forecast: Wall Street Split Widens Into Month-End - stonex.com</t>
+        </is>
+      </c>
+      <c r="V396" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNcy04QTN2dUFjZ0V3MkxNNkhYSTZ4THBjNXpqbkczLTlJQkpEeHFXbERVOG90YUdDMFZTRk9iUUFzbnlzVW84TG5FQ19LaE5sWmp4WGNadmN5QmVwaWVKc3QxM1ZQTVI3Y01vZlpUWmJmeWd2R3k1UEwzTE1QUmFEc2hTOFlWVjRabkJYdGxXcjFVckhsUkJ2UmYwQjc5cm1JaGlqdzluUWNlWC1GWnc2bWJQMzZMNTdE?oc=5</t>
+        </is>
+      </c>
+      <c r="W396" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="X396" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y396" t="inlineStr">
+        <is>
+          <t>Stock Market Today: Small Caps, Gold Miners Spanked Amid Sell-Off; Meta Makes A Bullish Move - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="Z396" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPQ1FiOVdEVEtTNHJ0OE1RQm5wXzJrbkg4cloxSmtreGtnR3Q3WlNNS1ZidDZwWjItSENaWXJpSDl1b3MySjVqUE9oTUxSd0lMY0ZxMDNiVGZtN3I2c2x5dzJvQ0NJdllKbjZva2VZQlpvV0hpb1JBbWxJVTdIclFLd2c5UE5UdUtBVHdQVklnWndnaVk0NmxYYkpSTG1NOXpWNG9yZDN2NDVLcjNC?oc=5</t>
+        </is>
+      </c>
+      <c r="AA396" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="AB396" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC396" t="inlineStr">
+        <is>
+          <t>Nasdaq Breaks Support As Chip Sell-Off Deepens; Knight-Swift, Canadian Pacific, AbbVie In Focus - Video - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD396" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOa0VQNUt2ZDVDYmZpdDB6V3lwVVdxemtUWU5xU0wyTHVKdmtuNzJEU29WUGNSVkNtRjFXV0xIRnQ5N3RodFF3d2JyOFBBbkZQTDVrZWV3R2QzeWctZ1JCS09Bc2VOU2JqWnM4VnlMZjFQVUh2VHNqdzBocUJ3Zm5XSTQ2b19jU3pvZFhvYWNucF9ydU5uLVhqNWN0SDUxZ3BKMXdN?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-09-29T00:15:55+00:00</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E397" t="n">
+        <v>84024.0312</v>
+      </c>
+      <c r="F397" t="n">
+        <v>84024.0312</v>
+      </c>
+      <c r="G397" t="n">
+        <v>83073.02340000001</v>
+      </c>
+      <c r="H397" t="n">
+        <v>83369.02340000001</v>
+      </c>
+      <c r="I397" t="n">
+        <v>970489856</v>
+      </c>
+      <c r="J397" t="n">
+        <v>4</v>
+      </c>
+      <c r="K397" t="n">
+        <v>37</v>
+      </c>
+      <c r="L397" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="M397" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="N397" t="n">
+        <v>34</v>
+      </c>
+      <c r="O397" t="n">
+        <v>0.126</v>
+      </c>
+      <c r="P397" t="n">
+        <v>-0.078</v>
+      </c>
+      <c r="Q397" t="n">
+        <v>6.755</v>
+      </c>
+      <c r="R397" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S397" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T397" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U397" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="V397" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W397" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X397" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y397" t="inlineStr">
+        <is>
+          <t>Bitcoin Short Liquidations Reach $13.82 Million in One Hour - tokenpost.com</t>
+        </is>
+      </c>
+      <c r="Z397" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBzSExMTl95TVZUY1JQSWhwZlJoR3BOOHR5ME1fRlZhXzBOVlRUMFRqS3JyeHJzbXpOWW5JMnBDSFp2SWt1MTRGalo0dHl4dnRVa0w1WlJSdlVYZw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA397" t="inlineStr">
+        <is>
+          <t>Crypto’s Latest Rebound is Fueled By More Liquidations - Bloomberg.com</t>
+        </is>
+      </c>
+      <c r="AB397" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcTZKMERXNUtEc1UtZTlmNy1RS21TYTV1ZXJuUzF3Rjkza1Zwbk4yWW5aRmxQSDRoWW4wU0ZadTVydVdiS01pNGlnYjZ3R0loMmp4YzNQT0N4TjVsNERrLWhzRm5QWEJFNFVFZ2lxZzNtRkM0c3Q5RkV6YzlubW9RSFZ6SFF0OHJXdHlONS1TS2Itd0JSaG5IVHJmdzNOY3l1RjNsNHFsckU?oc=5</t>
+        </is>
+      </c>
+      <c r="AC397" t="inlineStr">
+        <is>
+          <t>Crypto Winter or the Big Crash? Where the Bitcoin Price Goes Now - Morningstar</t>
+        </is>
+      </c>
+      <c r="AD397" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-29 10:31 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD397"/>
+  <dimension ref="A1:AD403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49997,6 +49997,762 @@
       <c r="AD397" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYXh2TjlMak92TzdhZ09YbkhyRmd3S0c1RWl5bnRETnBidU81TlV1U0JKbGd5bEsxNXBxVzJzZGxuZDVHLUp6VTFISE82TFE1dlVtckpPbVpqRldwQjZBa01NaTROYlFPN0F6RVhGM2xRVy1ZT2NOa1F4ZnRoT2JQb1J0M29ndjhvV2xBWW9RTXZaekppN1NuR09vdk5sM2Z3TFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-09-29T10:29:13+00:00</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E398" t="n">
+        <v>4171.8999</v>
+      </c>
+      <c r="F398" t="n">
+        <v>4182.7998</v>
+      </c>
+      <c r="G398" t="n">
+        <v>4167.3999</v>
+      </c>
+      <c r="H398" t="n">
+        <v>4181.3999</v>
+      </c>
+      <c r="I398" t="n">
+        <v>15111</v>
+      </c>
+      <c r="J398" t="n">
+        <v>4</v>
+      </c>
+      <c r="K398" t="n">
+        <v>39</v>
+      </c>
+      <c r="L398" t="n">
+        <v>-0.136</v>
+      </c>
+      <c r="M398" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="N398" t="n">
+        <v>40</v>
+      </c>
+      <c r="O398" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P398" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="Q398" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="R398" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S398" t="inlineStr">
+        <is>
+          <t>Highest Gold Price Ever: How Gold Reached $5,595 Faster Than Past Cycles - EBC Financial Group</t>
+        </is>
+      </c>
+      <c r="T398" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFBLSnpPSTJsQUlsSlBhQXFWc0RlWXNGbmtOU1VIc0xzYi13Y3gzRGgwN25odF9hTlowR2ZIb3hoNUVhcERaX1Juclc3dmlvMFB0U3ZiMFVYOTZJUS1lSkF3M2ZiX3VvcVpBa09vUktjV0dmd2Jpb3pj?oc=5</t>
+        </is>
+      </c>
+      <c r="U398" t="inlineStr">
+        <is>
+          <t>Lundin Gold Hits Record Grade at Bonza Sur With 204 g/t Gold Over 3 Metres Intercept - the deep dive</t>
+        </is>
+      </c>
+      <c r="V398" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNaDdPLWtTOVlMN0c3OWFFWmF1dUZfT28xLWducTQyQVo5XzRUZzU5YWxUZ1JlZzZqcHRtcG5FUENMZE9LN1ZEQXdpTDBMa3c2Ry1aakpaMjBtTlV6bTNDenB4d2d1OEltQmxadjVsTHFWY0J5alI2Sko2YVdfa1VHZDd3bGVtdUlOaXVaZU0xcFo0UHBjNXZTX2dKS1dtX1J5d2JBX2NxSW9TMS1P?oc=5</t>
+        </is>
+      </c>
+      <c r="W398" t="inlineStr">
+        <is>
+          <t>Gold surges toward $4,500 as investors seek safe haven from economic risks - AzerNews</t>
+        </is>
+      </c>
+      <c r="X398" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9PWVJtWlh5TmhEaEQxdkFxNmR5OE5BM1c4QURIOWozVnZwbHdMcndfejh5NGduQkZXaG15Q05GMzhBbzJsM1VaZGlPdnJRYWNwUXFiZmU1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y398" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="Z398" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA398" t="inlineStr">
+        <is>
+          <t>Wall Street split on gold price path after drop below $4,300, Main Street maintains bullish majority - Shanghai Metals Market</t>
+        </is>
+      </c>
+      <c r="AB398" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPTlNGU0Z3RlVTUlhNYldCZFJkWjg3cUdXVFdpUUJ6TVl4Tkdad2x0YXREdFc2M1BMa0FIRGwxMVJVdHE3cUwySjJBTFp2SnI3UHNNWVVpYk1NV2tuZU14S0hadXVHR2JWT2ZwTTNLejBwQnhmMnNuek9zRTZ2YnpfX1FmazY0MWdLbTNjaFAtdkcweG0xcWNncDI5Xy10TFpiNGphMEswaFl4ZHpwUnF0QmlNQjBuVFFHY2xBWm1ncG9Md1ZhRlFFMkZxYWh4cVQ3WHJpSUh2aHBObXF3Smc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC398" t="inlineStr">
+        <is>
+          <t>Gold ETFs Shine in H1 2026 with Unprecedented Liquidity - Investing News Network</t>
+        </is>
+      </c>
+      <c r="AD398" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE1JaGRkaHpGODN4bGpQdFl6S3VyUjZKYzRvWUxjUjhyQ0lVXzZMZEltdGkwMEo2d0lhVWVmMDVUYUJfRXF4emdyX0ZTd0N6SVgwN3kxMFVXTkt5WXZJbE8ybVNRLUJYTVZy?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-09-29T10:29:13+00:00</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E399" t="n">
+        <v>93.95999999999999</v>
+      </c>
+      <c r="F399" t="n">
+        <v>94.09</v>
+      </c>
+      <c r="G399" t="n">
+        <v>92.08</v>
+      </c>
+      <c r="H399" t="n">
+        <v>92.3</v>
+      </c>
+      <c r="I399" t="n">
+        <v>32694</v>
+      </c>
+      <c r="J399" t="n">
+        <v>4</v>
+      </c>
+      <c r="K399" t="n">
+        <v>40</v>
+      </c>
+      <c r="L399" t="n">
+        <v>-0.073</v>
+      </c>
+      <c r="M399" t="n">
+        <v>-0.151</v>
+      </c>
+      <c r="N399" t="n">
+        <v>40</v>
+      </c>
+      <c r="O399" t="n">
+        <v>0.224</v>
+      </c>
+      <c r="P399" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="Q399" t="n">
+        <v>3.023</v>
+      </c>
+      <c r="R399" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S399" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T399" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U399" t="inlineStr">
+        <is>
+          <t>Oil prices gain as focus shifts to supply recovery and demand - CNBC</t>
+        </is>
+      </c>
+      <c r="V399" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaFA3TG9MdVViYl8xUnV2c2U2T0FDLU1oRGM0VlA5bEVsaG9oOG9oOC03VWowRjBieTVuMEFRMDBJR2M5ODhIOGt1LTZDNUNXTkVvN1Bva3ljSlJqUUJQLW5KR18zVkFtUjdZVzZ5RmZpOV90TlpKLUhwd0hqYXV3alZFRDRqQ0ZjM2RJTGdrR1dtZTR0MmhLRHVPNWdRb03SAaQBQVVfeXFMT3VZUUFQRjJ6VnNtOGxsRVBXNkUyckprRnQ3UDhfZnN5NzVOZGRCNFJ1dnpmb0dvaDhEaWVXaE9Fa3drUXE3Vm1WbW5wbklwLTBvUERWX1RvMElsZW56dHdoNmUzWGliNEFHOTMydU1qRDVyeWxlMkpNdkZZVnl0QjNEeHNHb3dFTUY0RktoQ0ZMY2NtODg2X2pTS0Q0bVlJTkJTVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W399" t="inlineStr">
+        <is>
+          <t>Current price of oil as of August 6, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="X399" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTFA0dDhDZFBwQnNBWXBPbWp6RVRoMTdCMzdWVlZCdnk2YThTbGl5cWtjX2g4bFh2Vy1kOHZPT0QwVHRlbXVIVWRENTJSaGJNb3ZReVpoc1lybEVVaGpvS2V0LWNB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y399" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 28, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z399" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9rRk9pZkN0bERaRFVvU0wyVmU3SVQwWEpsYm1EMkR1eWg5dnJjNDBzNGlpZHpyVmFiRUlJYUF1MnhYMnFSalRMWXRSWWZfWHpNX0hJNXJyaTg2T2ZKckNOSFVn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA399" t="inlineStr">
+        <is>
+          <t>OPEC Monthly Oil Market Report, September 2026 - Peak Oil Barrel</t>
+        </is>
+      </c>
+      <c r="AB399" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9faVVpVXlFX1hFRG4tM2FnZTE5Q1ROMG1RWmxCTWVWcTdLcmo0VlBIbTlQcnhYOUQxeUxvaTE4VVo5Ulo3cExYYVViZUxWcU9VUzRIRXhQRTJLb19hWFhJc2V5WkxmMGhtSk92QVJndFZlV1NQeWxkM2Z3WWc?oc=5</t>
+        </is>
+      </c>
+      <c r="AC399" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD399" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-09-29T10:29:13+00:00</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E400" t="n">
+        <v>101.281</v>
+      </c>
+      <c r="F400" t="n">
+        <v>101.487</v>
+      </c>
+      <c r="G400" t="n">
+        <v>101.263</v>
+      </c>
+      <c r="H400" t="n">
+        <v>101.443</v>
+      </c>
+      <c r="I400" t="n">
+        <v>0</v>
+      </c>
+      <c r="J400" t="n">
+        <v>4</v>
+      </c>
+      <c r="K400" t="n">
+        <v>40</v>
+      </c>
+      <c r="L400" t="n">
+        <v>-0.155</v>
+      </c>
+      <c r="M400" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="N400" t="n">
+        <v>40</v>
+      </c>
+      <c r="O400" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="P400" t="n">
+        <v>-0.016</v>
+      </c>
+      <c r="Q400" t="n">
+        <v>-1.168</v>
+      </c>
+      <c r="R400" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S400" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T400" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U400" t="inlineStr">
+        <is>
+          <t>United States Dollar Index remains stronger as hawkish Fed signals drive rate hike bets - FXStreet</t>
+        </is>
+      </c>
+      <c r="V400" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOUHRaUk85MWJmMkZjUlFUM01CQktxTmF4VDM1NFNsS056S0NuMjM5RXo3U2hqaURkQkctUXdWWHUzdmFJWW9OazJfaWs1T1Z0SDdMaUJWYng4TmZ3LVBNRjVqdlpNc0wtaFAxSWdxUTBuQ0liNHU2bjBQMW5KSXUtWG0ydFRYcTBORk1xdm1OZzg4bC12blBhS3gxSFF0QUZGREpBTzVUdFh3ZXV0Tkpja1VRMjN4bFJRSmtjMUV3RmxXbkQxWTZndUV3?oc=5</t>
+        </is>
+      </c>
+      <c r="W400" t="inlineStr">
+        <is>
+          <t>United States Dollar Index strengthens as oil surge bolster Fed rate hike bets - FXStreet</t>
+        </is>
+      </c>
+      <c r="X400" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNQTE2ck15MDY5S1lfRWRKRVZsdmRLSnVMSlhLYmd5cEJLSm5YdVRnMGpHTGNjall0dVFvV0hZNFVoOGRMQTd2Y292T0Rva1RhU0tnXzAzZXgxZzlqbEtTZU9vdVlTZEZVckdBZlJmbnIwaDRZaDh0ZnpaLVRWYzV2YXpxdnVMTDYyUmZfcThpX2ZFZGVoQXlQVkg1dHFiVFdyajFfZGp2YzJETkdfNi11RG1HUXhfblhiNVQ2NHdn?oc=5</t>
+        </is>
+      </c>
+      <c r="Y400" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z400" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA400" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB400" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC400" t="inlineStr">
+        <is>
+          <t>British Pound gains as US Dollar weakens despite hawkish Fed, geopolitical tensions - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD400" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPS2g2djM3bEE4SmNheEM2X09OUDBWaTRYNFdaOWJKVDZpWHkzRlp1SVFENXJOR0VDQTNmQWx5bVU3dFFub3lERF9JUUNRV2d4akR0aURPa3R4T29pWENCU3pjeVZhRktqU0Jjb29HUGxWX3QyVHRlUnVVbFM3YU1rWEFPVWxUemQ5OGZzdjRYZFUyTTFuWFZXQ0NlLTBwZmxXdnM3d1JzRklDaHdhZW1WaDdrM2lnVGpScW93LWp1bWtza2s?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-09-29T10:29:13+00:00</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E401" t="n">
+        <v>7743</v>
+      </c>
+      <c r="F401" t="n">
+        <v>7754.5</v>
+      </c>
+      <c r="G401" t="n">
+        <v>7736.25</v>
+      </c>
+      <c r="H401" t="n">
+        <v>7743.5</v>
+      </c>
+      <c r="I401" t="n">
+        <v>61581</v>
+      </c>
+      <c r="J401" t="n">
+        <v>4</v>
+      </c>
+      <c r="K401" t="n">
+        <v>39</v>
+      </c>
+      <c r="L401" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="M401" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="N401" t="n">
+        <v>40</v>
+      </c>
+      <c r="O401" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="P401" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="Q401" t="n">
+        <v>5.383</v>
+      </c>
+      <c r="R401" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S401" t="inlineStr">
+        <is>
+          <t>Navitas Semiconductor stock surges 20% on U.S. defense contract - Investing.com</t>
+        </is>
+      </c>
+      <c r="T401" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQNEh0SWNBYm1CU01OYXNoTkU3aUl4RmN6X21XS1I4ejBTbnNCMXJKZXFHRWdhc3FUNm1BcFYxakdQMlNCSzg4a1J3UUo0RC1BMC1OeGVRUXVScmJnUkR5VGhBWjRqQkg1dUEzUmdRcFk2b1VBT1RoNWx0SjJ6T241ZkhyVndHR2w2YURDTm11N2x2WnVmWUgyVXRxYUxrdTdZTW90MC0zZ3ZBNlNyWWRHaHNueUQ3YTBa?oc=5</t>
+        </is>
+      </c>
+      <c r="U401" t="inlineStr">
+        <is>
+          <t>Dr Reddy's Stock Surges Over 2%; Outperforms Peers As Nifty Pharma Bucks Broader Weakness - NDTV Profit</t>
+        </is>
+      </c>
+      <c r="V401" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxPaFpUYVp1bWFOVjhWU2d1d1JfczVoNGFfSWNfbTd1ZjRKVDBqdWdiRTlyNEhfdUJkZ05aS1NjckRyOENPQ0d1dTRSdFhqWHJVc01UNmNHV0pRUHdHYWlNY1c5VnRBWTk4TS1zb0d0U0FMaU5kRVhWd3NyZmZFMkRKUy01MlFSV19qS3EydGNvYm0xbjhlQnRBYjV2dlF3SV9ubmVOUWhCZE4yZWJSMXc2MnBFckExbUdxWTNjOHNkQUJhV25RalZqRDcxWGpvZFBGR1pxcDVGN3BnS3NS0gHkAUFVX3lxTE4ybzZoR2tPTWFpT3VfTzNIbHpBeHoxTDVXZlJNaVpUZmlNaFpZeXZ4ZUx5YzZMM1RnMWNTNEJiUEtDLXdrYnBlN2FoU3Ywc081TURvVHNXZ2p1ZzV3TTBVZjBQSkd0eWtTTHBYYVdLYWl6dlNSQ0g3M0ZIa0N3cmFta29SNldXa1hEdnU2UFo0aHY5WlA5UGdwWnZqOXJvQjJVSWF5RXVEbDRSTXc4LUhlRHJHd2dwdm9sYjJvWjRqcVRnVlVpYzNya21nVU1CdmdXZnhHN2QtbXhXLXBBYmFnREUxSA?oc=5</t>
+        </is>
+      </c>
+      <c r="W401" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq, Dow Forecast: Wall Street Split Widens Into Month-End - stonex.com</t>
+        </is>
+      </c>
+      <c r="X401" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNcy04QTN2dUFjZ0V3MkxNNkhYSTZ4THBjNXpqbkczLTlJQkpEeHFXbERVOG90YUdDMFZTRk9iUUFzbnlzVW84TG5FQ19LaE5sWmp4WGNadmN5QmVwaWVKc3QxM1ZQTVI3Y01vZlpUWmJmeWd2R3k1UEwzTE1QUmFEc2hTOFlWVjRabkJYdGxXcjFVckhsUkJ2UmYwQjc5cm1JaGlqdzluUWNlWC1GWnc2bWJQMzZMNTdE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y401" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="Z401" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA401" t="inlineStr">
+        <is>
+          <t>Markets News, Sept. 28, 2026: Nasdaq, AI Stocks Fall to Start Week; Treasury Yields Jump - Investopedia</t>
+        </is>
+      </c>
+      <c r="AB401" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOVGptdWozalY5bFNzUDJ6Ykl2NVNkS28zWjlGcXIxQU50aG4tYU8xZVJmeHVqT3ZNU0xEOFdzRzNTTHhUMWc0WXItSjI0bS1OMUJ5cTB2bGF5U09EMWEyQktaaHhMdUZuNWFkMWxnS2ZfeFZrV1pURXdVTlNqNHhjUUlJSTZ1QWViSTdkaGFlWEE?oc=5</t>
+        </is>
+      </c>
+      <c r="AC401" t="inlineStr">
+        <is>
+          <t>Wall Street split on gold price path after drop below $4,300, Main Street maintains bullish majority as jobs take center stage - Kitco</t>
+        </is>
+      </c>
+      <c r="AD401" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQbWtUQVJKczJHZ1lWRDRZUEpOc1JuMVJHNmxQR18wSFlJbWJaemlYMXozWXdJTXRxRDVzWWRnWVFobWJCWEZqdUVqa2VMemE3NlI0MDJKdVFBWkJ0a3NrZE01WEJ2NS1mVUhaLTJYNnM4MUdHNHlDTnhYa0JZdS1lN2Vqdk5YOUhhWlhkMXc3S3pFaURQeFVKUU9pbVN5cWYzY0FwdThESE1IQ2JMVEo3T2JZbw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-09-29T10:29:13+00:00</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E402" t="n">
+        <v>30548.75</v>
+      </c>
+      <c r="F402" t="n">
+        <v>30635.25</v>
+      </c>
+      <c r="G402" t="n">
+        <v>30527.75</v>
+      </c>
+      <c r="H402" t="n">
+        <v>30589</v>
+      </c>
+      <c r="I402" t="n">
+        <v>23184</v>
+      </c>
+      <c r="J402" t="n">
+        <v>4</v>
+      </c>
+      <c r="K402" t="n">
+        <v>36</v>
+      </c>
+      <c r="L402" t="n">
+        <v>-0.104</v>
+      </c>
+      <c r="M402" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="N402" t="n">
+        <v>39</v>
+      </c>
+      <c r="O402" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="P402" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="Q402" t="n">
+        <v>4.031</v>
+      </c>
+      <c r="R402" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S402" t="inlineStr">
+        <is>
+          <t>Tech Stocks Surge as Apple (AAPL) Hits Record High - GuruFocus</t>
+        </is>
+      </c>
+      <c r="T402" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPbUtsdjFuWFdnMjZ2b2RGMjQzVzhXSG03Y1dYUmxXNmxjZlhiRkx3aVRPbEhyWk1XX3I0UUw3bjVkVTFzR2JTc1hSTFVEUVlSbnVDZm9rb0lCZFNvRnZKdnJ2ZjBhU1J2Tzl2V1VJY3UwckZqTE53YXdZdW10M3gxdUFxN1o2LUVjWkhDZXlnM18?oc=5</t>
+        </is>
+      </c>
+      <c r="U402" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq, Dow Forecast: Wall Street Split Widens Into Month-End - stonex.com</t>
+        </is>
+      </c>
+      <c r="V402" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNcy04QTN2dUFjZ0V3MkxNNkhYSTZ4THBjNXpqbkczLTlJQkpEeHFXbERVOG90YUdDMFZTRk9iUUFzbnlzVW84TG5FQ19LaE5sWmp4WGNadmN5QmVwaWVKc3QxM1ZQTVI3Y01vZlpUWmJmeWd2R3k1UEwzTE1QUmFEc2hTOFlWVjRabkJYdGxXcjFVckhsUkJ2UmYwQjc5cm1JaGlqdzluUWNlWC1GWnc2bWJQMzZMNTdE?oc=5</t>
+        </is>
+      </c>
+      <c r="W402" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="X402" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y402" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX extends gains as oil, Treasury yields fall - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z402" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOEYwd1BtWVl1OTlFSDhYVWRTSWxkbHZ0SmEwaVFmM25iRlNCY2JsQXhZbW5Id1hLUG5hcmZkaDUxWHhYTFozSFQySjhGcTZfZFgweTZOazlTQTZ6eWFyN1hXbS1KdjhBX3gtbDlfd1lUVEFWQ3VvWHdGTkE3aUdPZEs4TFNVbVVfQWthN01laUV0Zk42T1JWLS1Ja0tscnc4Nlk0U3NfbmZocWlWRlp1NjhTOA?oc=5</t>
+        </is>
+      </c>
+      <c r="AA402" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="AB402" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC402" t="inlineStr">
+        <is>
+          <t>Nasdaq Breaks Support As Chip Sell-Off Deepens; Knight-Swift, Canadian Pacific, AbbVie In Focus - Video - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD402" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOa0VQNUt2ZDVDYmZpdDB6V3lwVVdxemtUWU5xU0wyTHVKdmtuNzJEU29WUGNSVkNtRjFXV0xIRnQ5N3RodFF3d2JyOFBBbkZQTDVrZWV3R2QzeWctZ1JCS09Bc2VOU2JqWnM4VnlMZjFQVUh2VHNqdzBocUJ3Zm5XSTQ2b19jU3pvZFhvYWNucF9ydU5uLVhqNWN0SDUxZ3BKMXdN?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-09-29T10:29:13+00:00</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E403" t="n">
+        <v>83976</v>
+      </c>
+      <c r="F403" t="n">
+        <v>84330.99219999999</v>
+      </c>
+      <c r="G403" t="n">
+        <v>83729.64840000001</v>
+      </c>
+      <c r="H403" t="n">
+        <v>84096.0469</v>
+      </c>
+      <c r="I403" t="n">
+        <v>1319133184</v>
+      </c>
+      <c r="J403" t="n">
+        <v>4</v>
+      </c>
+      <c r="K403" t="n">
+        <v>39</v>
+      </c>
+      <c r="L403" t="n">
+        <v>0.138</v>
+      </c>
+      <c r="M403" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="N403" t="n">
+        <v>35</v>
+      </c>
+      <c r="O403" t="n">
+        <v>0.312</v>
+      </c>
+      <c r="P403" t="n">
+        <v>-0.079</v>
+      </c>
+      <c r="Q403" t="n">
+        <v>10.152</v>
+      </c>
+      <c r="R403" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S403" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T403" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U403" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - CNBC</t>
+        </is>
+      </c>
+      <c r="V403" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W403" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X403" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y403" t="inlineStr">
+        <is>
+          <t>XRP Price Prediction for October 2026 - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="Z403" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOb252ZDRzQ2lYVUhvM1JnR0hEaGNpTm1qbU5ZNml2NHRzMGFWVzVJRkRHejBhbnlnVXdYTGUyXzFNSTR2YlJ2Q3o1UGhObzgxQ1k0VnFWWU5GTVpmUU9xNWNtTGJxZXQwSlhfOVRyU0Z3X29BUEg1cEZFQU5PakR0QjVqUUxhdllSc0FiZ1BfVDMxUHpSR3AzWlFSZjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA403" t="inlineStr">
+        <is>
+          <t>Current price of Bitcoin for Sept. 28, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB403" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE10TUZGTV9PZWFjUUFTTUwwLTJRZGllSjJEbk5zLVVaTnJSOUd1LUw2OGN3bWl4azRQcDd5VDBuenoxYm93UDdlNS1GWk84Vk5yR3lmYVpma09tOHI4M2NNWGhwYVIwWUU?oc=5</t>
+        </is>
+      </c>
+      <c r="AC403" t="inlineStr">
+        <is>
+          <t>Crypto’s Latest Rebound is Fueled By More Liquidations - Bloomberg</t>
+        </is>
+      </c>
+      <c r="AD403" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcTZKMERXNUtEc1UtZTlmNy1RS21TYTV1ZXJuUzF3Rjkza1Zwbk4yWW5aRmxQSDRoWW4wU0ZadTVydVdiS01pNGlnYjZ3R0loMmp4YzNQT0N4TjVsNERrLWhzRm5QWEJFNFVFZ2lxZzNtRkM0c3Q5RkV6YzlubW9RSFZ6SFF0OHJXdHlONS1TS2Itd0JSaG5IVHJmdzNOY3l1RjNsNHFsckU?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-29 17:50 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD403"/>
+  <dimension ref="A1:AD409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50753,6 +50753,762 @@
       <c r="AD403" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcTZKMERXNUtEc1UtZTlmNy1RS21TYTV1ZXJuUzF3Rjkza1Zwbk4yWW5aRmxQSDRoWW4wU0ZadTVydVdiS01pNGlnYjZ3R0loMmp4YzNQT0N4TjVsNERrLWhzRm5QWEJFNFVFZ2lxZzNtRkM0c3Q5RkV6YzlubW9RSFZ6SFF0OHJXdHlONS1TS2Itd0JSaG5IVHJmdzNOY3l1RjNsNHFsckU?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-09-29T17:48:52+00:00</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E404" t="n">
+        <v>4189.5</v>
+      </c>
+      <c r="F404" t="n">
+        <v>4207.2002</v>
+      </c>
+      <c r="G404" t="n">
+        <v>4176.2998</v>
+      </c>
+      <c r="H404" t="n">
+        <v>4177</v>
+      </c>
+      <c r="I404" t="n">
+        <v>37106</v>
+      </c>
+      <c r="J404" t="n">
+        <v>4</v>
+      </c>
+      <c r="K404" t="n">
+        <v>39</v>
+      </c>
+      <c r="L404" t="n">
+        <v>-0.032</v>
+      </c>
+      <c r="M404" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="N404" t="n">
+        <v>40</v>
+      </c>
+      <c r="O404" t="n">
+        <v>0.192</v>
+      </c>
+      <c r="P404" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="Q404" t="n">
+        <v>2.719</v>
+      </c>
+      <c r="R404" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S404" t="inlineStr">
+        <is>
+          <t>Gold hits record above $5,100 as geopolitics drive safe‑haven rush - Reuters</t>
+        </is>
+      </c>
+      <c r="T404" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeEVJaEpsQjFWNXBMR1dObVJJUUN5Vjc1ZVhOOUxIN1lfUzBzZUlQSDBUakVkdnVqc0VJYnlzbm5GSDZqeWVBS1BaSTE2Um1YWUViWV93MFU4d19KTUJnNnZhWERidE9JWE53Sk9CdGQza1hkVWNXQ3ltc092V2YyRDZFeHBIUFVwQ3dfd05IVndaVEN3N1VYekRPYlI0WFU?oc=5</t>
+        </is>
+      </c>
+      <c r="U404" t="inlineStr">
+        <is>
+          <t>Gold hits record high as investors seek safety - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="V404" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVWt1Y1hBWG5uZFNjRUFtZHlqRUhfZGV6VzAtQ0tBT2VlVDVEZEJ2WHN0YndCcXRzSjNtVnFhUFZZZ2F4RFRxYkdsSF91eDk2MFl5R3JNWk1HREJjSVdhUE1uTTU1N1Z6Y2xfZzZCSDZ4YnhaT1czcWdXeHE3SjJBR2FqUm43Z0paUG5OVEdsWVdYYnZBWVHSAZsBQVVfeXFMTWh6VXlqZGZVbUl3SHVfQ195WFFveEVkLU9TU1RXMTZBdVhodU16UWxLLWVScDNsc2VGMThyT0RTTHB4SVNRYU1KWmRycHhnTEc0NTJ1RWgzdGc2Y0VkanR4QUtlUWFBSnB2cElORUltQk9XdWRLNXhKbU5jRUFqQVd6bG5YbURJakxhNTl3UEk4RzBaQzVJaVdRdFk?oc=5</t>
+        </is>
+      </c>
+      <c r="W404" t="inlineStr">
+        <is>
+          <t>Gold rises above $4,130 as geopolitical uncertainty supports safe-haven demand - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="X404" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPVC0wdnlpU1I2eWVTbnhmbHhvdFBmWUM4c3J4dk9NZFVBMGZBOVBJall6QmY2UkxxTm15TS1ycGs1ZW42RFFNaWdiUlJuajNKWmhOZ0sxYWlOSUZpcTAySkV3NHhST0dGRVZtVmVVVmt4WFFja2hjOW1RVVF5UFdGaUxaOXhOSTUwX21ab1FQQlh4dE0yOUVn?oc=5</t>
+        </is>
+      </c>
+      <c r="Y404" t="inlineStr">
+        <is>
+          <t>Gold - Breaks Key Support As Rising US Yields Sap Demand - eFXdata</t>
+        </is>
+      </c>
+      <c r="Z404" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE1vWmp3NWY1TURNaGVjOGM0Q2h3UWdPT19qNzJKa1VPeFVOYnBDcG5IZ2lrd2JQdmdDZ2xTYUc2cFc2QmRLbkFjbHQyWjUwTlgzOEhWWFRnYzdjS3JGVFZOTnkxclY1V0tyUE54SVNUT0VaNlBLTHBRcmFB0gF_QVVfeXFMUHlzQjl2bW4zTlllTUFwbndXQ2VGMGVmNDdMbHM3T1haTjdIWno3Y0dsNVJ1ajRlT2NIZEFJcS00VzFLZDcwZEl5SHJmOWxjV0lJWXJ2MFEwMi1rSUY2VDNqX3Vtd3RGYkxfUzNZUS1wa0xWYzdreWluR3h1dmtKcw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA404" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AB404" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC404" t="inlineStr">
+        <is>
+          <t>Gold rebounds 0.9% after sell-off, but Fed rate hike fears cap gains - Moneycontrol.com</t>
+        </is>
+      </c>
+      <c r="AD404" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOd1RDOVU3VHdGV0YzNk14dFdSdDczak9INXBqQkhwY2ZnVGh4bElsNFZ3VnBlM0VCc18wUWI2RjJwSkxRMVFJNTFPRE81WjhWUDlkX2tzTjhJdmtDOFdtMGdHalZWdXJEWUFUT2xFRFJUS3RPQ0pVeUtOS3lBMmNNQXkyeW5yYVZNaTg0MmRSWloxV2hWSXJaSjFkRFU4dkhJeHV3S05rajU5OVQ0amhzdUdFUjc4UWp4aURhRWNrSzJtdFZ1Ul8tUnUtTnd2UzNzcmFEMlM3b9IB3AFBVV95cUxPVlBMdl9fWnMySEdYQ3pGaXliNmJraWw1WVVsYS1xcndpdDNqSUNmSTdIbEtzeWRFb1FoWEJ4YXNqX2JGZUNjM29vRUlseHR4R3BObXR6S2kzVC12dDFXem1GWnc0UVh1Y0JDRGxxdEVTZ1dRUlBGYVpDdDR5LXNpeTcxT0U4cVRFeGZCdmtpd3NnaDJrbFBESHA2R21OdGc5aG9pTUc4RHlCaVBCdzJxdnE5dnJHTXN3dk4zNTl4QkRNQTZaOEp0NFRkTlVzak5ybkRJXzdYZndLTm1i?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-09-29T17:48:52+00:00</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E405" t="n">
+        <v>90.89</v>
+      </c>
+      <c r="F405" t="n">
+        <v>91.76000000000001</v>
+      </c>
+      <c r="G405" t="n">
+        <v>90.06</v>
+      </c>
+      <c r="H405" t="n">
+        <v>90.3</v>
+      </c>
+      <c r="I405" t="n">
+        <v>127221</v>
+      </c>
+      <c r="J405" t="n">
+        <v>4</v>
+      </c>
+      <c r="K405" t="n">
+        <v>40</v>
+      </c>
+      <c r="L405" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="M405" t="n">
+        <v>-0.264</v>
+      </c>
+      <c r="N405" t="n">
+        <v>40</v>
+      </c>
+      <c r="O405" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="P405" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="Q405" t="n">
+        <v>3.824</v>
+      </c>
+      <c r="R405" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S405" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - energynow.com</t>
+        </is>
+      </c>
+      <c r="T405" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U405" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - cnbc.com</t>
+        </is>
+      </c>
+      <c r="V405" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="W405" t="inlineStr">
+        <is>
+          <t>Oil prices surge 15% as Strait of Hormuz disruptions tighten supply - Offshore Technology</t>
+        </is>
+      </c>
+      <c r="X405" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPdndjemtyTkduUUpSVnR6aXJUNXBBR0JNd1FaaURNWmtvWm9WTkZUME50Qk1NVDUtdEtqcWE2R0xvUGRKNHBWZDMtblpaY1h1TE5zcmgycU5kS29mYU02N1BOdThBMUhUMDM0T1FScDZRY0JzYlRXTTJVajFYbkh3Rmp0MDFDeVZQcFhKSjhpaklySjZrVWJCZVoyWkw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y405" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 28, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z405" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9rRk9pZkN0bERaRFVvU0wyVmU3SVQwWEpsYm1EMkR1eWg5dnJjNDBzNGlpZHpyVmFiRUlJYUF1MnhYMnFSalRMWXRSWWZfWHpNX0hJNXJyaTg2T2ZKckNOSFVn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA405" t="inlineStr">
+        <is>
+          <t>Brent Oil breaks below $103 support: Live levels By Investing.com - Investing.com Nigeria</t>
+        </is>
+      </c>
+      <c r="AB405" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQT1Z0V0k1ZTZrTEVrZU83eFRkV1FoMDZvZHlBdHBiS0xhWF9nOGdDM3Y5V1NxYnU3dm5JOXRmMFZYRU5oS3RKZ3FGYmw2dmFRN3psLXdMdkJTbXNyUHZ3Ujg1Y19nek50X0ZuYUs2ejdNNnBYNGZhU0lYNTdDZWFoQlhaX1hidlFPMDk4RTRCRVdDckg5Mzg0T2dNeTduaWxhUWZfV3FPM240c0ExS0xleTJIQ1p2U0NBODZnT01TVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC405" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - cnbc.com</t>
+        </is>
+      </c>
+      <c r="AD405" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-09-29T17:48:52+00:00</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E406" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="F406" t="n">
+        <v>101.612</v>
+      </c>
+      <c r="G406" t="n">
+        <v>101.364</v>
+      </c>
+      <c r="H406" t="n">
+        <v>101.587</v>
+      </c>
+      <c r="I406" t="n">
+        <v>0</v>
+      </c>
+      <c r="J406" t="n">
+        <v>4</v>
+      </c>
+      <c r="K406" t="n">
+        <v>40</v>
+      </c>
+      <c r="L406" t="n">
+        <v>-0.242</v>
+      </c>
+      <c r="M406" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="N406" t="n">
+        <v>40</v>
+      </c>
+      <c r="O406" t="n">
+        <v>0.089</v>
+      </c>
+      <c r="P406" t="n">
+        <v>-0.038</v>
+      </c>
+      <c r="Q406" t="n">
+        <v>-3.053</v>
+      </c>
+      <c r="R406" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S406" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T406" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U406" t="inlineStr">
+        <is>
+          <t>United States Dollar Index strengthens as oil surge bolster Fed rate hike bets - FXStreet</t>
+        </is>
+      </c>
+      <c r="V406" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNQTE2ck15MDY5S1lfRWRKRVZsdmRLSnVMSlhLYmd5cEJLSm5YdVRnMGpHTGNjall0dVFvV0hZNFVoOGRMQTd2Y292T0Rva1RhU0tnXzAzZXgxZzlqbEtTZU9vdVlTZEZVckdBZlJmbnIwaDRZaDh0ZnpaLVRWYzV2YXpxdnVMTDYyUmZfcThpX2ZFZGVoQXlQVkg1dHFiVFdyajFfZGp2YzJETkdfNi11RG1HUXhfblhiNVQ2NHdn?oc=5</t>
+        </is>
+      </c>
+      <c r="W406" t="inlineStr">
+        <is>
+          <t>Dollar Gains on US Economic Strength and Hawkish Fed Comments - TradingView</t>
+        </is>
+      </c>
+      <c r="X406" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOaEdRYWt1NjlZdUc2SmN1aENJRmhOU0Rxc095SVpSMmZ5UzA3MW9zRWRtR20yX1VlV0xkblZ3QlRSYkNzbHh0Ui1ZVmpyY0hxNk9nXzVERmZBeXc5azJkMUhKaFBobTZqeWo3WWtPaXE3R3RFaEZycXVGYjdfOTlLR1RybjRCamxFMGlyeGNuYkxNRnJaU3E0cDVrYnBQdGZ3R29lcmpmYWFDaEtmSUdzSExDcnVyT1RhVVJj?oc=5</t>
+        </is>
+      </c>
+      <c r="Y406" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z406" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA406" t="inlineStr">
+        <is>
+          <t>ING lifts year-end EUR/USD forecast to 1.18 as dovish Fed view pressures Dollar - VT Markets</t>
+        </is>
+      </c>
+      <c r="AB406" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxORE5YdjZHQzh4V1B2REJUeHpXV3N6Y21ZeWh3VzhfNng4N0dsSk5xbEpCTW40a05ES2NPQkFqQ3RGWjR4ZnN4RUFhVXoxU1NPRFUzZnZRU3E3TzRSTUxxYWZ1dnVMVlVqVUZrR2JRYkt2QlVYVGtpUGN2Mmt6blhvRFVDWURtbkI4UGlyVHpmMHBSeFdTS0RNS0NENXZWQkFxSVNBdkQxSVczTmdMbDk4UVpzSWtZVUliVS1WVFZZdnRuYXM?oc=5</t>
+        </is>
+      </c>
+      <c r="AC406" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - think.ing.com</t>
+        </is>
+      </c>
+      <c r="AD406" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-09-29T17:48:52+00:00</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E407" t="n">
+        <v>7736.25</v>
+      </c>
+      <c r="F407" t="n">
+        <v>7747</v>
+      </c>
+      <c r="G407" t="n">
+        <v>7712.25</v>
+      </c>
+      <c r="H407" t="n">
+        <v>7720.75</v>
+      </c>
+      <c r="I407" t="n">
+        <v>629061</v>
+      </c>
+      <c r="J407" t="n">
+        <v>4</v>
+      </c>
+      <c r="K407" t="n">
+        <v>39</v>
+      </c>
+      <c r="L407" t="n">
+        <v>0.181</v>
+      </c>
+      <c r="M407" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="N407" t="n">
+        <v>40</v>
+      </c>
+      <c r="O407" t="n">
+        <v>0.242</v>
+      </c>
+      <c r="P407" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="Q407" t="n">
+        <v>7.872</v>
+      </c>
+      <c r="R407" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S407" t="inlineStr">
+        <is>
+          <t>Cruise Stocks Rally as Carnival's Q3 Results Land: Carnival Surges 12%, Royal Caribbean Gains 7%, Norwegian Rises 5% - 24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="T407" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxOMmZaTF9PRUhuc1JFaDRuVk1Qcmg5d01XaE4zaHpEYlpuRU1lLU91UFY2d2VWWnZtbkNfbzA4RF8zMTZXVE5Kc2ZNQU5UdU1LaURHQzE2NUZ2blNySFEyN0pYZUkyQTc4N0dSVUVTdmE1dHk0azcyWmQ0SnZ0YzhSdGxKeUU0cWl4V0ZpQ2JBYWh3Z1lGX3FOZG1sbGt4OXRvNXZiUWtiUExpakZZYTBzMmkxSjZjRzdaTGhpVk1kUUFxR0dOYW9tdzduNHloa3BVYUtpNkxyN1NLNjNuaUJ2WFBGRGJLNUpf?oc=5</t>
+        </is>
+      </c>
+      <c r="U407" t="inlineStr">
+        <is>
+          <t>Navitas Semiconductor stock surges 20% on U.S. defense contract - Investing.com</t>
+        </is>
+      </c>
+      <c r="V407" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQNEh0SWNBYm1CU01OYXNoTkU3aUl4RmN6X21XS1I4ejBTbnNCMXJKZXFHRWdhc3FUNm1BcFYxakdQMlNCSzg4a1J3UUo0RC1BMC1OeGVRUXVScmJnUkR5VGhBWjRqQkg1dUEzUmdRcFk2b1VBT1RoNWx0SjJ6T241ZkhyVndHR2w2YURDTm11N2x2WnVmWUgyVXRxYUxrdTdZTW90MC0zZ3ZBNlNyWWRHaHNueUQ3YTBa?oc=5</t>
+        </is>
+      </c>
+      <c r="W407" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq, Dow Forecast: Wall Street Split Widens Into Month-End - stonex.com</t>
+        </is>
+      </c>
+      <c r="X407" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNcy04QTN2dUFjZ0V3MkxNNkhYSTZ4THBjNXpqbkczLTlJQkpEeHFXbERVOG90YUdDMFZTRk9iUUFzbnlzVW84TG5FQ19LaE5sWmp4WGNadmN5QmVwaWVKc3QxM1ZQTVI3Y01vZlpUWmJmeWd2R3k1UEwzTE1QUmFEc2hTOFlWVjRabkJYdGxXcjFVckhsUkJ2UmYwQjc5cm1JaGlqdzluUWNlWC1GWnc2bWJQMzZMNTdE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y407" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - foxbusiness.com</t>
+        </is>
+      </c>
+      <c r="Z407" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA407" t="inlineStr">
+        <is>
+          <t>If a Stock Market Crash Is Coming, History Says This ETF Could Be the Smartest Buy for Investors - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="AB407" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPNmZsYzdSQlYxVjBRQ0I5czFNbmxLLURMRTluU1FGRENsUzgzOWpJV3pYN1RfckE1T3dlbHdxMlFUcTUzaFZiOUp0clFxN3dQRWpMTHVuRG9XbG94Z3ctSmdpWkVLR1A1Rm4yZTd1bnVmaDNwV09EVTQwSVVlYXlpdWU2MlY3TTY0RnJvQ1FJVEc2Y2ZaNjkzcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC407" t="inlineStr">
+        <is>
+          <t>Markets News, Sept. 28, 2026: Nasdaq, AI Stocks Fall to Start Week; Treasury Yields Jump - Investopedia</t>
+        </is>
+      </c>
+      <c r="AD407" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOVGptdWozalY5bFNzUDJ6Ykl2NVNkS28zWjlGcXIxQU50aG4tYU8xZVJmeHVqT3ZNU0xEOFdzRzNTTHhUMWc0WXItSjI0bS1OMUJ5cTB2bGF5U09EMWEyQktaaHhMdUZuNWFkMWxnS2ZfeFZrV1pURXdVTlNqNHhjUUlJSTZ1QWViSTdkaGFlWEE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-09-29T17:48:52+00:00</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E408" t="n">
+        <v>30608.25</v>
+      </c>
+      <c r="F408" t="n">
+        <v>30706.25</v>
+      </c>
+      <c r="G408" t="n">
+        <v>30504.5</v>
+      </c>
+      <c r="H408" t="n">
+        <v>30562.75</v>
+      </c>
+      <c r="I408" t="n">
+        <v>236806</v>
+      </c>
+      <c r="J408" t="n">
+        <v>4</v>
+      </c>
+      <c r="K408" t="n">
+        <v>35</v>
+      </c>
+      <c r="L408" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="M408" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="N408" t="n">
+        <v>37</v>
+      </c>
+      <c r="O408" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="P408" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="Q408" t="n">
+        <v>8.138</v>
+      </c>
+      <c r="R408" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S408" t="inlineStr">
+        <is>
+          <t>Fox Factory Can Ride This Rally Higher (NASDAQ:FOXF) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T408" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxNR3dERjZqYldnZlUySXJibzlKQ0MxdUk5dUNIdHYxR0ZwcmdUM19EdVZaRUtKQXlSSnAwdGdJVkZLdzA3bDBvNWtuNWlPNUZGRVZmN2s1VHg1c1hjS1d0M1l1WFRZNWFlRFpPMHJtakFzSUVtencwY1FJRGRNaXFtODdGRW1GZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U408" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq, Dow Forecast: Wall Street Split Widens Into Month-End - stonex.com</t>
+        </is>
+      </c>
+      <c r="V408" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNcy04QTN2dUFjZ0V3MkxNNkhYSTZ4THBjNXpqbkczLTlJQkpEeHFXbERVOG90YUdDMFZTRk9iUUFzbnlzVW84TG5FQ19LaE5sWmp4WGNadmN5QmVwaWVKc3QxM1ZQTVI3Y01vZlpUWmJmeWd2R3k1UEwzTE1QUmFEc2hTOFlWVjRabkJYdGxXcjFVckhsUkJ2UmYwQjc5cm1JaGlqdzluUWNlWC1GWnc2bWJQMzZMNTdE?oc=5</t>
+        </is>
+      </c>
+      <c r="W408" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="X408" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y408" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX rises as oil eases and tech gains - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z408" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPLW1jVmJFX0hHWElrSWo5SHdxc1dYVEVBbHlydHp6eDlXSmpOd2w5SHZfTlYtOU82RnhkYzZCNVpjRWI1TjV3OU80cVdGRkJwdFMtVjdNMEk5bUVTVWdnemtQQ1FHV2s4dm9GLXZFa3VmZDE2UHpGT2lDWjE1U212eUdtMERfSFlzWWl6TUNJanJmeHdSMlE0eW11Ri16Z2c1U3hRd1RCRW8?oc=5</t>
+        </is>
+      </c>
+      <c r="AA408" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="AB408" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC408" t="inlineStr">
+        <is>
+          <t>Katie Stockton: Bracing for volatility after Nasdaq broke below recent support - cnbc.com</t>
+        </is>
+      </c>
+      <c r="AD408" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLWhuVXhhdF9LbEhfSTV2RlNTZ0IyVjBlcUxGS0RQLXA5S0xjUWFZa3c3Nm1OZmxSRU5mVmVLZzRkbEFKYWd1YWFoVHdadUpRRXlMc1BSVi1BY2Q5RlVLRzVoa2xuRkxZdThVS0VVTzRYY256MHZha1l6RDlrU0NaVXZGZW1qZFRWbTBOUFBTRGxUck9ZWk9tWlY4bl9LcU1BVG5Ka0RVVURXallmZGhqT1BacEpBYnFTUzBIRQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-09-29T17:48:52+00:00</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E409" t="n">
+        <v>84189.67969999999</v>
+      </c>
+      <c r="F409" t="n">
+        <v>84262.49219999999</v>
+      </c>
+      <c r="G409" t="n">
+        <v>82869.9688</v>
+      </c>
+      <c r="H409" t="n">
+        <v>83037.24219999999</v>
+      </c>
+      <c r="I409" t="n">
+        <v>94326784</v>
+      </c>
+      <c r="J409" t="n">
+        <v>4</v>
+      </c>
+      <c r="K409" t="n">
+        <v>39</v>
+      </c>
+      <c r="L409" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="M409" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="N409" t="n">
+        <v>34</v>
+      </c>
+      <c r="O409" t="n">
+        <v>0.339</v>
+      </c>
+      <c r="P409" t="n">
+        <v>-0.023</v>
+      </c>
+      <c r="Q409" t="n">
+        <v>9.515000000000001</v>
+      </c>
+      <c r="R409" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S409" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - cnbc.com</t>
+        </is>
+      </c>
+      <c r="T409" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U409" t="inlineStr">
+        <is>
+          <t>Bitcoin surged to an eight-month high above $85,000 as oil fell and ETF inflows returned - qz.com</t>
+        </is>
+      </c>
+      <c r="V409" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9BRHhsSDNaZ2VlVnhzYmRsci1zNk1kQ2JWNHJxNTNVRHFDSHFqcmVoVFg2TkJxYTdZMUhfMEJpb1hFS3RabDlJcVZZWEh4M3VJUUpaX0JUSWtHd0pxNUctNzg3Nkx0Q2JoT21EN2cwV1ZtQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W409" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X409" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y409" t="inlineStr">
+        <is>
+          <t>Curve DAO Gains 14% Amid Broader Market Decline - KuCoin</t>
+        </is>
+      </c>
+      <c r="Z409" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNLTZ4QTE1dG16NVhDTzFhSXd2SnFQUXl6UXVvb2ZBeWpfdGlUdkdZaExKRmZVOFNNN0JJX2lFMjVzR0FjUEZBQXl4ajE2em1hem1FdWRtSXNSZXlsWVkzVUd4WGowdmJLa3AtRXR4SkQ3TGh0Z29ibUc5UVdpcUszWnU2RVhOUUE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA409" t="inlineStr">
+        <is>
+          <t>Current price of Bitcoin for Sept. 28, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="AB409" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE10TUZGTV9PZWFjUUFTTUwwLTJRZGllSjJEbk5zLVVaTnJSOUd1LUw2OGN3bWl4azRQcDd5VDBuenoxYm93UDdlNS1GWk84Vk5yR3lmYVpma09tOHI4M2NNWGhwYVIwWUU?oc=5</t>
+        </is>
+      </c>
+      <c r="AC409" t="inlineStr">
+        <is>
+          <t>Zcash Volatility Explained: Liquidations, Whales, Sector Shifts - CoinMarketCap</t>
+        </is>
+      </c>
+      <c r="AD409" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9TbE5mMkZiN0psUzFJMU83ZUhUTXpuX1hwYlE1dXJqSzY4MVVlMC1vczZQa0d0M2ljWG1tRG5fR2RaeExkTmhlT0ltLWJ3WnVwa2FJLWtTLVM0REg5VFp3MGxaX2tSWlhLYlRVSXdPS18?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-29 23:33 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD409"/>
+  <dimension ref="A1:AD415"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51509,6 +51509,762 @@
       <c r="AD409" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9TbE5mMkZiN0psUzFJMU83ZUhUTXpuX1hwYlE1dXJqSzY4MVVlMC1vczZQa0d0M2ljWG1tRG5fR2RaeExkTmhlT0ltLWJ3WnVwa2FJLWtTLVM0REg5VFp3MGxaX2tSWlhLYlRVSXdPS18?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-09-29T23:31:03+00:00</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E410" t="n">
+        <v>4203.7002</v>
+      </c>
+      <c r="F410" t="n">
+        <v>4218.1001</v>
+      </c>
+      <c r="G410" t="n">
+        <v>4200.3999</v>
+      </c>
+      <c r="H410" t="n">
+        <v>4213.7998</v>
+      </c>
+      <c r="I410" t="n">
+        <v>9121</v>
+      </c>
+      <c r="J410" t="n">
+        <v>4</v>
+      </c>
+      <c r="K410" t="n">
+        <v>39</v>
+      </c>
+      <c r="L410" t="n">
+        <v>-0.122</v>
+      </c>
+      <c r="M410" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="N410" t="n">
+        <v>40</v>
+      </c>
+      <c r="O410" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="P410" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="Q410" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="R410" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S410" t="inlineStr">
+        <is>
+          <t>Highest Gold Price Ever: How Gold Reached $5,595 Faster Than Past Cycles - EBC Financial Group</t>
+        </is>
+      </c>
+      <c r="T410" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFBLSnpPSTJsQUlsSlBhQXFWc0RlWXNGbmtOU1VIc0xzYi13Y3gzRGgwN25odF9hTlowR2ZIb3hoNUVhcERaX1Juclc3dmlvMFB0U3ZiMFVYOTZJUS1lSkF3M2ZiX3VvcVpBa09vUktjV0dmd2Jpb3pj?oc=5</t>
+        </is>
+      </c>
+      <c r="U410" t="inlineStr">
+        <is>
+          <t>Gold: Prior floor becomes resistance — NFP breaks the structure and bears own the tape - FXStreet</t>
+        </is>
+      </c>
+      <c r="V410" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNZmpYbjdKbktMMGFsV2xjZmRjaVJMR2h6OUJIcF94NDRHTHZTaE1NSXlsSzR2dS1aa0JCeTZ5a05IbVpjYjZ6SDNlSU9HSFEySmlqbl9yUFBrcF9Na2JKNEtPRzRmS1BPc1Zia1ZLcTZLOEM2YVB4dHRrQjZkQ2JmTTZJS2k5YkFnWUxqdVAtVFVqeTItc3JDUHd6M1JVM2p1aW1uNWpNc1VRbUVNWlE4NGszRW1KRlB1RXNGcFpYNERPRURoTEFXOTl3?oc=5</t>
+        </is>
+      </c>
+      <c r="W410" t="inlineStr">
+        <is>
+          <t>China’s central bank buys 20.2 tonnes of gold in August, largest purchase since 2023 - Kitco</t>
+        </is>
+      </c>
+      <c r="X410" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWDFEUjBvUmhpWnhKb1dmOC1Kd1U3MjVCNG1WSUxXdFdydW1EekdVUDdDb1BDY3FBSVZEMzl0bV9UZGZJV1ZuSDFEb250emQzTm5PY3pfZFktZUdxOV9LNUxzNGFvNHVOcndfWENQVnpzVldMWHJHWHhxdHZHS0ZQYm1FaHFTaVhwRXRsb0hZMUs0WThnNkppalB3OHlOQUhZT1Awakl4dEdudW01aEtnTjFFOUdjZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y410" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="Z410" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA410" t="inlineStr">
+        <is>
+          <t>Gold rebounds 0.9% after sell-off, but Fed rate hike fears cap gains - Moneycontrol.com</t>
+        </is>
+      </c>
+      <c r="AB410" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOd1RDOVU3VHdGV0YzNk14dFdSdDczak9INXBqQkhwY2ZnVGh4bElsNFZ3VnBlM0VCc18wUWI2RjJwSkxRMVFJNTFPRE81WjhWUDlkX2tzTjhJdmtDOFdtMGdHalZWdXJEWUFUT2xFRFJUS3RPQ0pVeUtOS3lBMmNNQXkyeW5yYVZNaTg0MmRSWloxV2hWSXJaSjFkRFU4dkhJeHV3S05rajU5OVQ0amhzdUdFUjc4UWp4aURhRWNrSzJtdFZ1Ul8tUnUtTnd2UzNzcmFEMlM3b9IB3AFBVV95cUxPVlBMdl9fWnMySEdYQ3pGaXliNmJraWw1WVVsYS1xcndpdDNqSUNmSTdIbEtzeWRFb1FoWEJ4YXNqX2JGZUNjM29vRUlseHR4R3BObXR6S2kzVC12dDFXem1GWnc0UVh1Y0JDRGxxdEVTZ1dRUlBGYVpDdDR5LXNpeTcxT0U4cVRFeGZCdmtpd3NnaDJrbFBESHA2R21OdGc5aG9pTUc4RHlCaVBCdzJxdnE5dnJHTXN3dk4zNTl4QkRNQTZaOEp0NFRkTlVzak5ybkRJXzdYZndLTm1i?oc=5</t>
+        </is>
+      </c>
+      <c r="AC410" t="inlineStr">
+        <is>
+          <t>Gold ETFs Shine in H1 2026 with Unprecedented Liquidity - Investing News Network</t>
+        </is>
+      </c>
+      <c r="AD410" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE1JaGRkaHpGODN4bGpQdFl6S3VyUjZKYzRvWUxjUjhyQ0lVXzZMZEltdGkwMEo2d0lhVWVmMDVUYUJfRXF4emdyX0ZTd0N6SVgwN3kxMFVXTkt5WXZJbE8ybVNRLUJYTVZy?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-09-29T23:31:03+00:00</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E411" t="n">
+        <v>89.45</v>
+      </c>
+      <c r="F411" t="n">
+        <v>89.56999999999999</v>
+      </c>
+      <c r="G411" t="n">
+        <v>88.58</v>
+      </c>
+      <c r="H411" t="n">
+        <v>89.34</v>
+      </c>
+      <c r="I411" t="n">
+        <v>17259</v>
+      </c>
+      <c r="J411" t="n">
+        <v>4</v>
+      </c>
+      <c r="K411" t="n">
+        <v>40</v>
+      </c>
+      <c r="L411" t="n">
+        <v>-0.052</v>
+      </c>
+      <c r="M411" t="n">
+        <v>-0.222</v>
+      </c>
+      <c r="N411" t="n">
+        <v>40</v>
+      </c>
+      <c r="O411" t="n">
+        <v>0.223</v>
+      </c>
+      <c r="P411" t="n">
+        <v>-0.08799999999999999</v>
+      </c>
+      <c r="Q411" t="n">
+        <v>3.419</v>
+      </c>
+      <c r="R411" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S411" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T411" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U411" t="inlineStr">
+        <is>
+          <t>Oil surges 6%, Brent and US crude both surpass $100 on more tanker attacks - Reuters</t>
+        </is>
+      </c>
+      <c r="V411" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPVTlKVk5vOWlpYndFb2Flck9IczhtU2k5X1I3a0tlMjA2dkRmMEJncVFZdWctZW9wX05NaU9vUzNwMU5ld3UycklJMjhHaHB3WDdZVF81Z0t1WWNZak8tTFFwdDZtTHZvUnozMnVpUmtEanVsN2ZxM1A2QkxZS3IydDByTlQtd3RFYThzVnlwVmR0eGMyT1RQQldPZVp4VE1oSm5TcHBXVTd1dXM?oc=5</t>
+        </is>
+      </c>
+      <c r="W411" t="inlineStr">
+        <is>
+          <t>OPEC+ keeps oil output policy unchanged for October - CNBC</t>
+        </is>
+      </c>
+      <c r="X411" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1Jb3JjX3FIRFp4VzJLdzM2R3lSSWdsWk1kOTZiWkxWeTc0RlQtVFQzOG1oVUF2Ym5YRVgzOVA1SHJBTXU3YTV2RUxvTXF1bEJNQkpaVlB6ZXpLS1BVRGVkUXQ3VFhMSEJBVFd5RdIBckFVX3lxTE9MTjdQYzRBcGtFSno4b2hSanRVNm1XdVVQd2dZQl8zNHpaa3ctV1I0T0JJT3I5LUllUWRSazVFYjZDSHFGNmktbVl4X0JyMHNXc1VneTBvSDZWRjFPMEtUZndITlpXS1R6ZVRoRGg5TURudw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y411" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 28, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z411" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9rRk9pZkN0bERaRFVvU0wyVmU3SVQwWEpsYm1EMkR1eWg5dnJjNDBzNGlpZHpyVmFiRUlJYUF1MnhYMnFSalRMWXRSWWZfWHpNX0hJNXJyaTg2T2ZKckNOSFVn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA411" t="inlineStr">
+        <is>
+          <t>Brent Oil breaks below $103 support: Live levels By Investing.com - Investing.com Nigeria</t>
+        </is>
+      </c>
+      <c r="AB411" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQT1Z0V0k1ZTZrTEVrZU83eFRkV1FoMDZvZHlBdHBiS0xhWF9nOGdDM3Y5V1NxYnU3dm5JOXRmMFZYRU5oS3RKZ3FGYmw2dmFRN3psLXdMdkJTbXNyUHZ3Ujg1Y19nek50X0ZuYUs2ejdNNnBYNGZhU0lYNTdDZWFoQlhaX1hidlFPMDk4RTRCRVdDckg5Mzg0T2dNeTduaWxhUWZfV3FPM240c0ExS0xleTJIQ1p2U0NBODZnT01TVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC411" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - CNBC</t>
+        </is>
+      </c>
+      <c r="AD411" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-09-29T23:31:03+00:00</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E412" t="n">
+        <v>101.372</v>
+      </c>
+      <c r="F412" t="n">
+        <v>101.444</v>
+      </c>
+      <c r="G412" t="n">
+        <v>101.361</v>
+      </c>
+      <c r="H412" t="n">
+        <v>101.377</v>
+      </c>
+      <c r="I412" t="n">
+        <v>0</v>
+      </c>
+      <c r="J412" t="n">
+        <v>4</v>
+      </c>
+      <c r="K412" t="n">
+        <v>40</v>
+      </c>
+      <c r="L412" t="n">
+        <v>-0.212</v>
+      </c>
+      <c r="M412" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="N412" t="n">
+        <v>40</v>
+      </c>
+      <c r="O412" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="P412" t="n">
+        <v>-0.046</v>
+      </c>
+      <c r="Q412" t="n">
+        <v>-3.694</v>
+      </c>
+      <c r="R412" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S412" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T412" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U412" t="inlineStr">
+        <is>
+          <t>United States Dollar Index strengthens as oil surge bolster Fed rate hike bets - FXStreet</t>
+        </is>
+      </c>
+      <c r="V412" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNQTE2ck15MDY5S1lfRWRKRVZsdmRLSnVMSlhLYmd5cEJLSm5YdVRnMGpHTGNjall0dVFvV0hZNFVoOGRMQTd2Y292T0Rva1RhU0tnXzAzZXgxZzlqbEtTZU9vdVlTZEZVckdBZlJmbnIwaDRZaDh0ZnpaLVRWYzV2YXpxdnVMTDYyUmZfcThpX2ZFZGVoQXlQVkg1dHFiVFdyajFfZGp2YzJETkdfNi11RG1HUXhfblhiNVQ2NHdn?oc=5</t>
+        </is>
+      </c>
+      <c r="W412" t="inlineStr">
+        <is>
+          <t>United States Dollar Index approaches yearly peak on hawkish Fed outlook - FXStreet</t>
+        </is>
+      </c>
+      <c r="X412" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQdUVDWVdBQ1FGa1UtNFpxLXFPQ2h6R3REb2gyWm5ZcWhoLUNEbmJVZGl1V1VGdlNmNW9XdHZleXNRV1lMQVF4NnRTWlpEamJMTTk1U1ptU0pNY005RFh3dUhncjVvRFFWRWR3akIyeVVuWlI1TWZtdGZydm0wblpodDVZNzJ2MkdWM0RhdFJWZExfYV8tckwwYXFVZkdrb21zRm9jRlJyenlkV0FDRlBLMXcyTHFZZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y412" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z412" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA412" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB412" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC412" t="inlineStr">
+        <is>
+          <t>British Pound gains as US Dollar weakens despite hawkish Fed, geopolitical tensions - FXStreet</t>
+        </is>
+      </c>
+      <c r="AD412" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPS2g2djM3bEE4SmNheEM2X09OUDBWaTRYNFdaOWJKVDZpWHkzRlp1SVFENXJOR0VDQTNmQWx5bVU3dFFub3lERF9JUUNRV2d4akR0aURPa3R4T29pWENCU3pjeVZhRktqU0Jjb29HUGxWX3QyVHRlUnVVbFM3YU1rWEFPVWxUemQ5OGZzdjRYZFUyTTFuWFZXQ0NlLTBwZmxXdnM3d1JzRklDaHdhZW1WaDdrM2lnVGpScW93LWp1bWtza2s?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-09-29T23:31:03+00:00</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E413" t="n">
+        <v>7737.25</v>
+      </c>
+      <c r="F413" t="n">
+        <v>7749.25</v>
+      </c>
+      <c r="G413" t="n">
+        <v>7727</v>
+      </c>
+      <c r="H413" t="n">
+        <v>7743.25</v>
+      </c>
+      <c r="I413" t="n">
+        <v>279367</v>
+      </c>
+      <c r="J413" t="n">
+        <v>4</v>
+      </c>
+      <c r="K413" t="n">
+        <v>39</v>
+      </c>
+      <c r="L413" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="M413" t="n">
+        <v>-0.004</v>
+      </c>
+      <c r="N413" t="n">
+        <v>40</v>
+      </c>
+      <c r="O413" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="P413" t="n">
+        <v>-0.014</v>
+      </c>
+      <c r="Q413" t="n">
+        <v>9.382999999999999</v>
+      </c>
+      <c r="R413" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S413" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 29: Carnival Surges 13% on Record Bookings, Raised Guidance - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="T413" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxNLThyaTVvUmFCc0VKZEluVjF1WkxxTjJGX0JJcVFnVmhnSjh0RjBIX01COGJDV2VlUXBFSVo5RG1EZmdSUmhmRVZUZHNOU1JPN3NhSW1PRjZvZmhEdFNGU1J0cWhsNm1ldWloY3BmUXg1a1VwUGxrbnJiMTAzdnkzekNnaTV4MjZZczEwQURmSjhYWlY1SUk4VjFwUy1qZUJnRUxsbVJDcGRzZGZ6NDFfMzNONjFFOWFnenE3TnZzN0JBOFlQTEliajM1WEJxQkdPZjlNdXYyQ00?oc=5</t>
+        </is>
+      </c>
+      <c r="U413" t="inlineStr">
+        <is>
+          <t>Navitas Semiconductor stock surges 20% on U.S. defense contract - Investing.com</t>
+        </is>
+      </c>
+      <c r="V413" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQNEh0SWNBYm1CU01OYXNoTkU3aUl4RmN6X21XS1I4ejBTbnNCMXJKZXFHRWdhc3FUNm1BcFYxakdQMlNCSzg4a1J3UUo0RC1BMC1OeGVRUXVScmJnUkR5VGhBWjRqQkg1dUEzUmdRcFk2b1VBT1RoNWx0SjJ6T241ZkhyVndHR2w2YURDTm11N2x2WnVmWUgyVXRxYUxrdTdZTW90MC0zZ3ZBNlNyWWRHaHNueUQ3YTBa?oc=5</t>
+        </is>
+      </c>
+      <c r="W413" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq, Dow Forecast: Wall Street Split Widens Into Month-End - stonex.com</t>
+        </is>
+      </c>
+      <c r="X413" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNcy04QTN2dUFjZ0V3MkxNNkhYSTZ4THBjNXpqbkczLTlJQkpEeHFXbERVOG90YUdDMFZTRk9iUUFzbnlzVW84TG5FQ19LaE5sWmp4WGNadmN5QmVwaWVKc3QxM1ZQTVI3Y01vZlpUWmJmeWd2R3k1UEwzTE1QUmFEc2hTOFlWVjRabkJYdGxXcjFVckhsUkJ2UmYwQjc5cm1JaGlqdzluUWNlWC1GWnc2bWJQMzZMNTdE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y413" t="inlineStr">
+        <is>
+          <t>If a Stock Market Crash Is Coming, History Says This ETF Could Be the Smartest Buy for Investors - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="Z413" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQS1JvNzZmU2xWbFRsWEd2SjlVWnRDandpVHgwcXBFWVZCSlJUZ3hWend0RFlzOURVM2xTSVJJVEFSZVZCcnlwR3lKazBDTEZlOEp4Q0M5SlhfQlhVSTJtX0hnM2lNV3VMTnNUd2thYXJCam41VGZOUDlFbG1hczZ5ek1obkxrQ08zVV83ZzMtM0stU0tCYVIwbWZ3c29ycGM?oc=5</t>
+        </is>
+      </c>
+      <c r="AA413" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AB413" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC413" t="inlineStr">
+        <is>
+          <t>If a Stock Market Crash Is Coming, History Says This ETF Could Be the Smartest Buy for Investors - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="AD413" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPNmZsYzdSQlYxVjBRQ0I5czFNbmxLLURMRTluU1FGRENsUzgzOWpJV3pYN1RfckE1T3dlbHdxMlFUcTUzaFZiOUp0clFxN3dQRWpMTHVuRG9XbG94Z3ctSmdpWkVLR1A1Rm4yZTd1bnVmaDNwV09EVTQwSVVlYXlpdWU2MlY3TTY0RnJvQ1FJVEc2Y2ZaNjkzcQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-09-29T23:31:03+00:00</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E414" t="n">
+        <v>30647</v>
+      </c>
+      <c r="F414" t="n">
+        <v>30708.75</v>
+      </c>
+      <c r="G414" t="n">
+        <v>30592.25</v>
+      </c>
+      <c r="H414" t="n">
+        <v>30671.25</v>
+      </c>
+      <c r="I414" t="n">
+        <v>68389</v>
+      </c>
+      <c r="J414" t="n">
+        <v>4</v>
+      </c>
+      <c r="K414" t="n">
+        <v>37</v>
+      </c>
+      <c r="L414" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="M414" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="N414" t="n">
+        <v>38</v>
+      </c>
+      <c r="O414" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="P414" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="Q414" t="n">
+        <v>11.562</v>
+      </c>
+      <c r="R414" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S414" t="inlineStr">
+        <is>
+          <t>Fox Factory Can Ride This Rally Higher (NASDAQ:FOXF) - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="T414" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxNR3dERjZqYldnZlUySXJibzlKQ0MxdUk5dUNIdHYxR0ZwcmdUM19EdVZaRUtKQXlSSnAwdGdJVkZLdzA3bDBvNWtuNWlPNUZGRVZmN2s1VHg1c1hjS1d0M1l1WFRZNWFlRFpPMHJtakFzSUVtencwY1FJRGRNaXFtODdGRW1GZw?oc=5</t>
+        </is>
+      </c>
+      <c r="U414" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq, Dow Forecast: Wall Street Split Widens Into Month-End - stonex.com</t>
+        </is>
+      </c>
+      <c r="V414" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNcy04QTN2dUFjZ0V3MkxNNkhYSTZ4THBjNXpqbkczLTlJQkpEeHFXbERVOG90YUdDMFZTRk9iUUFzbnlzVW84TG5FQ19LaE5sWmp4WGNadmN5QmVwaWVKc3QxM1ZQTVI3Y01vZlpUWmJmeWd2R3k1UEwzTE1QUmFEc2hTOFlWVjRabkJYdGxXcjFVckhsUkJ2UmYwQjc5cm1JaGlqdzluUWNlWC1GWnc2bWJQMzZMNTdE?oc=5</t>
+        </is>
+      </c>
+      <c r="W414" t="inlineStr">
+        <is>
+          <t>Nasdaq hits record high as AI chip rally lifts tech stocks - Honolulu Star-Advertiser</t>
+        </is>
+      </c>
+      <c r="X414" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQmp4bXNYaENJQTJSWXJRY0F0dDJFaHB6eUQzM195M1hvSmlqXzd2ckJWQVZKaHhLLWZTYkJReG93OTZfQTdOLU9rRktNamhHeURBX3JBS25ja0h5WjAxa1dPamktbDhlUHFsbUl0ZWgxRTJ3cWhPVHA3TVA1UzBvSHhLM0pFZkRfX3NfZ3lwQWlSVU5hRG5TLUM5V1g4aGxpa08zSk5uZU5zVnZzQUhuSl9iQUFXZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y414" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="Z414" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AA414" t="inlineStr">
+        <is>
+          <t>Dow Drops 132, Nasdaq Loses 23, S&amp;P 500 Falls 13 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AB414" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOWVl3dU1hNlNGdGJkaWVqRWptcFVWRnBlSDdIVVFrVnVVMFBpWFpRVmtCejVpMDMzY1BvRGNKUUg1ZHNoQ2laOVhleHR5QzVESjU5b2ExUWRKcThMeTlsRHRVbDNtemcxRFZVZ2pwdFFOWG1WQVdudUloUTdHZngzVWpycFJ1Mk9aM19lU2xscVY?oc=5</t>
+        </is>
+      </c>
+      <c r="AC414" t="inlineStr">
+        <is>
+          <t>Nasdaq Breaks Support As Chip Sell-Off Deepens; Knight-Swift, Canadian Pacific, AbbVie In Focus - Video - Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="AD414" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOa0VQNUt2ZDVDYmZpdDB6V3lwVVdxemtUWU5xU0wyTHVKdmtuNzJEU29WUGNSVkNtRjFXV0xIRnQ5N3RodFF3d2JyOFBBbkZQTDVrZWV3R2QzeWctZ1JCS09Bc2VOU2JqWnM4VnlMZjFQVUh2VHNqdzBocUJ3Zm5XSTQ2b19jU3pvZFhvYWNucF9ydU5uLVhqNWN0SDUxZ3BKMXdN?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-09-29T23:31:03+00:00</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E415" t="n">
+        <v>83579.8594</v>
+      </c>
+      <c r="F415" t="n">
+        <v>83821.49219999999</v>
+      </c>
+      <c r="G415" t="n">
+        <v>83338.57030000001</v>
+      </c>
+      <c r="H415" t="n">
+        <v>83681.8906</v>
+      </c>
+      <c r="I415" t="n">
+        <v>896215040</v>
+      </c>
+      <c r="J415" t="n">
+        <v>4</v>
+      </c>
+      <c r="K415" t="n">
+        <v>39</v>
+      </c>
+      <c r="L415" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="M415" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="N415" t="n">
+        <v>35</v>
+      </c>
+      <c r="O415" t="n">
+        <v>0.447</v>
+      </c>
+      <c r="P415" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="Q415" t="n">
+        <v>11.451</v>
+      </c>
+      <c r="R415" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S415" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - CNBC</t>
+        </is>
+      </c>
+      <c r="T415" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U415" t="inlineStr">
+        <is>
+          <t>Bitcoin surged to an eight-month high above $85,000 as oil fell and ETF inflows returned - qz.com</t>
+        </is>
+      </c>
+      <c r="V415" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9BRHhsSDNaZ2VlVnhzYmRsci1zNk1kQ2JWNHJxNTNVRHFDSHFqcmVoVFg2TkJxYTdZMUhfMEJpb1hFS3RabDlJcVZZWEh4M3VJUUpaX0JUSWtHd0pxNUctNzg3Nkx0Q2JoT21EN2cwV1ZtQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W415" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X415" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y415" t="inlineStr">
+        <is>
+          <t>Current price of Bitcoin for Sept. 28, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z415" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE10TUZGTV9PZWFjUUFTTUwwLTJRZGllSjJEbk5zLVVaTnJSOUd1LUw2OGN3bWl4azRQcDd5VDBuenoxYm93UDdlNS1GWk84Vk5yR3lmYVpma09tOHI4M2NNWGhwYVIwWUU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA415" t="inlineStr">
+        <is>
+          <t>Zcash Volatility Explained: Liquidations, Whales, Sector Shifts - CoinMarketCap</t>
+        </is>
+      </c>
+      <c r="AB415" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9TbE5mMkZiN0psUzFJMU83ZUhUTXpuX1hwYlE1dXJqSzY4MVVlMC1vczZQa0d0M2ljWG1tRG5fR2RaeExkTmhlT0ltLWJ3WnVwa2FJLWtTLVM0REg5VFp3MGxaX2tSWlhLYlRVSXdPS18?oc=5</t>
+        </is>
+      </c>
+      <c r="AC415" t="inlineStr">
+        <is>
+          <t>$297M Bitcoin moved by Strategy was internal, n... - Pluang</t>
+        </is>
+      </c>
+      <c r="AD415" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQOFM4dVVNY1R2S2t6VGYzV0h6djJhQUptTEJ5YXJMVjFtczRxVWxXX254VlhyaG5rVk4yZHRNQ3ZOdC1VUlA1d2hWOFlpWjRkNkZDbkxQYm5hQ1RfM19xcUdoZXY1SEp3bmFUNTF3NllkZ3BzZml0Tk1kRlo4dzFibXhPNnk3eldOUXROdmctU0N6TFZoMlgtcUhpdHY2NkRFeWVkMS15MkpQVHI3?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan: 2026-09-30 04:27 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD415"/>
+  <dimension ref="A1:AD421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52263,6 +52263,762 @@
         </is>
       </c>
       <c r="AD415" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQOFM4dVVNY1R2S2t6VGYzV0h6djJhQUptTEJ5YXJMVjFtczRxVWxXX254VlhyaG5rVk4yZHRNQ3ZOdC1VUlA1d2hWOFlpWjRkNkZDbkxQYm5hQ1RfM19xcUdoZXY1SEp3bmFUNTF3NllkZ3BzZml0Tk1kRlo4dzFibXhPNnk3eldOUXROdmctU0N6TFZoMlgtcUhpdHY2NkRFeWVkMS15MkpQVHI3?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-09-30T04:25:27+00:00</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E416" t="n">
+        <v>4208.2998</v>
+      </c>
+      <c r="F416" t="n">
+        <v>4216</v>
+      </c>
+      <c r="G416" t="n">
+        <v>4198.6001</v>
+      </c>
+      <c r="H416" t="n">
+        <v>4206.7998</v>
+      </c>
+      <c r="I416" t="n">
+        <v>10612</v>
+      </c>
+      <c r="J416" t="n">
+        <v>4</v>
+      </c>
+      <c r="K416" t="n">
+        <v>39</v>
+      </c>
+      <c r="L416" t="n">
+        <v>-0.038</v>
+      </c>
+      <c r="M416" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="N416" t="n">
+        <v>40</v>
+      </c>
+      <c r="O416" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="P416" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="Q416" t="n">
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="R416" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S416" t="inlineStr">
+        <is>
+          <t>Highest Gold Price Ever: How Gold Reached $5,595 Faster Than Past Cycles - EBC Financial Group</t>
+        </is>
+      </c>
+      <c r="T416" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFBLSnpPSTJsQUlsSlBhQXFWc0RlWXNGbmtOU1VIc0xzYi13Y3gzRGgwN25odF9hTlowR2ZIb3hoNUVhcERaX1Juclc3dmlvMFB0U3ZiMFVYOTZJUS1lSkF3M2ZiX3VvcVpBa09vUktjV0dmd2Jpb3pj?oc=5</t>
+        </is>
+      </c>
+      <c r="U416" t="inlineStr">
+        <is>
+          <t>Gold: Prior floor becomes resistance — NFP breaks the structure and bears own the tape - FXStreet</t>
+        </is>
+      </c>
+      <c r="V416" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNZmpYbjdKbktMMGFsV2xjZmRjaVJMR2h6OUJIcF94NDRHTHZTaE1NSXlsSzR2dS1aa0JCeTZ5a05IbVpjYjZ6SDNlSU9HSFEySmlqbl9yUFBrcF9Na2JKNEtPRzRmS1BPc1Zia1ZLcTZLOEM2YVB4dHRrQjZkQ2JmTTZJS2k5YkFnWUxqdVAtVFVqeTItc3JDUHd6M1JVM2p1aW1uNWpNc1VRbUVNWlE4NGszRW1KRlB1RXNGcFpYNERPRURoTEFXOTl3?oc=5</t>
+        </is>
+      </c>
+      <c r="W416" t="inlineStr">
+        <is>
+          <t>China’s central bank buys 20.2 tonnes of gold in August, largest purchase since 2023 - Kitco</t>
+        </is>
+      </c>
+      <c r="X416" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWDFEUjBvUmhpWnhKb1dmOC1Kd1U3MjVCNG1WSUxXdFdydW1EekdVUDdDb1BDY3FBSVZEMzl0bV9UZGZJV1ZuSDFEb250emQzTm5PY3pfZFktZUdxOV9LNUxzNGFvNHVOcndfWENQVnpzVldMWHJHWHhxdHZHS0ZQYm1FaHFTaVhwRXRsb0hZMUs0WThnNkppalB3OHlOQUhZT1Awakl4dEdudW01aEtnTjFFOUdjZw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y416" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="Z416" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AA416" t="inlineStr">
+        <is>
+          <t>Gold rebounds 0.9% after sell-off, but Fed rate hike fears cap gains - Moneycontrol.com</t>
+        </is>
+      </c>
+      <c r="AB416" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOd1RDOVU3VHdGV0YzNk14dFdSdDczak9INXBqQkhwY2ZnVGh4bElsNFZ3VnBlM0VCc18wUWI2RjJwSkxRMVFJNTFPRE81WjhWUDlkX2tzTjhJdmtDOFdtMGdHalZWdXJEWUFUT2xFRFJUS3RPQ0pVeUtOS3lBMmNNQXkyeW5yYVZNaTg0MmRSWloxV2hWSXJaSjFkRFU4dkhJeHV3S05rajU5OVQ0amhzdUdFUjc4UWp4aURhRWNrSzJtdFZ1Ul8tUnUtTnd2UzNzcmFEMlM3b9IB3AFBVV95cUxPVlBMdl9fWnMySEdYQ3pGaXliNmJraWw1WVVsYS1xcndpdDNqSUNmSTdIbEtzeWRFb1FoWEJ4YXNqX2JGZUNjM29vRUlseHR4R3BObXR6S2kzVC12dDFXem1GWnc0UVh1Y0JDRGxxdEVTZ1dRUlBGYVpDdDR5LXNpeTcxT0U4cVRFeGZCdmtpd3NnaDJrbFBESHA2R21OdGc5aG9pTUc4RHlCaVBCdzJxdnE5dnJHTXN3dk4zNTl4QkRNQTZaOEp0NFRkTlVzak5ybkRJXzdYZndLTm1i?oc=5</t>
+        </is>
+      </c>
+      <c r="AC416" t="inlineStr">
+        <is>
+          <t>Wall Street split on gold price path after drop below $4,300, Main Street maintains bullish majority - Shanghai Metals Market</t>
+        </is>
+      </c>
+      <c r="AD416" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOQTlBcTVpdi1lQm5EaGtBUGtQeDVBckRQX1hrcXE0a2NDYm40ZHloc2N6VHI2OUQzVXBnMzkzMDhQT3dwYjdxWE1CN2twdGttTFdBRjl4aVBBcnozbkVBeC1WQk9ac1lraXJ4MEl1ZUlRVndzNmJWdjZlckxIT1RRcURTd2ZsZW1majBMRWt6aG5nTWpzc01QOWk3Q1B3UzdfLUZiQkxiaDRfS25fT1l2MjYwQ1hvS185ZWxKYWp3VTdkd1BQLVhxc1ZWMmVvdkJFaWhaLXY4ekUtQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-09-30T04:25:27+00:00</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E417" t="n">
+        <v>89.34</v>
+      </c>
+      <c r="F417" t="n">
+        <v>89.89</v>
+      </c>
+      <c r="G417" t="n">
+        <v>89.23</v>
+      </c>
+      <c r="H417" t="n">
+        <v>89.68000000000001</v>
+      </c>
+      <c r="I417" t="n">
+        <v>9840</v>
+      </c>
+      <c r="J417" t="n">
+        <v>4</v>
+      </c>
+      <c r="K417" t="n">
+        <v>40</v>
+      </c>
+      <c r="L417" t="n">
+        <v>-0.043</v>
+      </c>
+      <c r="M417" t="n">
+        <v>-0.227</v>
+      </c>
+      <c r="N417" t="n">
+        <v>40</v>
+      </c>
+      <c r="O417" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="P417" t="n">
+        <v>-0.08400000000000001</v>
+      </c>
+      <c r="Q417" t="n">
+        <v>2.823</v>
+      </c>
+      <c r="R417" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S417" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T417" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U417" t="inlineStr">
+        <is>
+          <t>Current price of oil as of July 30, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="V417" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9odGxncTZBdXJrcnd4Zm1GSENJSFpJQUJxbGphdTV2dTRfQTVmMzVFQ21PTGhzY19DSGVFUWpoeEtGMDZhNzRveUNoaDBlcDVLSmRpaFh6ZnA1emJSVllSYTNR?oc=5</t>
+        </is>
+      </c>
+      <c r="W417" t="inlineStr">
+        <is>
+          <t>Oil prices surge 15% as Strait of Hormuz disruptions tighten supply - Offshore Technology</t>
+        </is>
+      </c>
+      <c r="X417" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPdndjemtyTkduUUpSVnR6aXJUNXBBR0JNd1FaaURNWmtvWm9WTkZUME50Qk1NVDUtdEtqcWE2R0xvUGRKNHBWZDMtblpaY1h1TE5zcmgycU5kS29mYU02N1BOdThBMUhUMDM0T1FScDZRY0JzYlRXTTJVajFYbkh3Rmp0MDFDeVZQcFhKSjhpaklySjZrVWJCZVoyWkw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y417" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 28, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z417" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9rRk9pZkN0bERaRFVvU0wyVmU3SVQwWEpsYm1EMkR1eWg5dnJjNDBzNGlpZHpyVmFiRUlJYUF1MnhYMnFSalRMWXRSWWZfWHpNX0hJNXJyaTg2T2ZKckNOSFVn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA417" t="inlineStr">
+        <is>
+          <t>Brent Oil breaks below $103 support: Live levels By Investing.com - Investing.com Nigeria</t>
+        </is>
+      </c>
+      <c r="AB417" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQT1Z0V0k1ZTZrTEVrZU83eFRkV1FoMDZvZHlBdHBiS0xhWF9nOGdDM3Y5V1NxYnU3dm5JOXRmMFZYRU5oS3RKZ3FGYmw2dmFRN3psLXdMdkJTbXNyUHZ3Ujg1Y19nek50X0ZuYUs2ejdNNnBYNGZhU0lYNTdDZWFoQlhaX1hidlFPMDk4RTRCRVdDckg5Mzg0T2dNeTduaWxhUWZfV3FPM240c0ExS0xleTJIQ1p2U0NBODZnT01TVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC417" t="inlineStr">
+        <is>
+          <t>Oil prices edge higher after sharp drop as Middle East supply recovers - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD417" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPQ2U3QjBSRFpSSTIzU1RjeEt4bmVidmRVVEg0Y1cwYktEVi0ycVB5MFFXa1B0ajc5ZFhKNlgzLVVvRXBLNFJoRmpuT3JadlpYZ0F5Q2NIM3VtQ01GazVIM0ZHSXhxLWRrRHc5RmJQUWo3TVpXT1gxWmNrS01pUE9FS21kQVg4dVMtX3ljSzRwQXJZSkM5a09JMXNnWFY0dVd0WDZmSnFSenprTkVzbVNiYnI1Wld1RC1jYW9ibFYwbGVnRWRN?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-09-30T04:25:27+00:00</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E418" t="n">
+        <v>101.389</v>
+      </c>
+      <c r="F418" t="n">
+        <v>101.425</v>
+      </c>
+      <c r="G418" t="n">
+        <v>101.311</v>
+      </c>
+      <c r="H418" t="n">
+        <v>101.421</v>
+      </c>
+      <c r="I418" t="n">
+        <v>0</v>
+      </c>
+      <c r="J418" t="n">
+        <v>4</v>
+      </c>
+      <c r="K418" t="n">
+        <v>40</v>
+      </c>
+      <c r="L418" t="n">
+        <v>-0.115</v>
+      </c>
+      <c r="M418" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="N418" t="n">
+        <v>40</v>
+      </c>
+      <c r="O418" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="P418" t="n">
+        <v>-0.065</v>
+      </c>
+      <c r="Q418" t="n">
+        <v>-1.458</v>
+      </c>
+      <c r="R418" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S418" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T418" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U418" t="inlineStr">
+        <is>
+          <t>United States Dollar Index approaches yearly peak on hawkish Fed outlook - FXStreet</t>
+        </is>
+      </c>
+      <c r="V418" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQdUVDWVdBQ1FGa1UtNFpxLXFPQ2h6R3REb2gyWm5ZcWhoLUNEbmJVZGl1V1VGdlNmNW9XdHZleXNRV1lMQVF4NnRTWlpEamJMTTk1U1ptU0pNY005RFh3dUhncjVvRFFWRWR3akIyeVVuWlI1TWZtdGZydm0wblpodDVZNzJ2MkdWM0RhdFJWZExfYV8tckwwYXFVZkdrb21zRm9jRlJyenlkV0FDRlBLMXcyTHFZZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W418" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X418" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y418" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z418" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA418" t="inlineStr">
+        <is>
+          <t>British Pound gains as US Dollar weakens despite hawkish Fed, geopolitical tensions - FXStreet</t>
+        </is>
+      </c>
+      <c r="AB418" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPS2g2djM3bEE4SmNheEM2X09OUDBWaTRYNFdaOWJKVDZpWHkzRlp1SVFENXJOR0VDQTNmQWx5bVU3dFFub3lERF9JUUNRV2d4akR0aURPa3R4T29pWENCU3pjeVZhRktqU0Jjb29HUGxWX3QyVHRlUnVVbFM3YU1rWEFPVWxUemQ5OGZzdjRYZFUyTTFuWFZXQ0NlLTBwZmxXdnM3d1JzRklDaHdhZW1WaDdrM2lnVGpScW93LWp1bWtza2s?oc=5</t>
+        </is>
+      </c>
+      <c r="AC418" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - think.ing.com</t>
+        </is>
+      </c>
+      <c r="AD418" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-09-30T04:25:27+00:00</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>ES=F</t>
+        </is>
+      </c>
+      <c r="E419" t="n">
+        <v>7744.25</v>
+      </c>
+      <c r="F419" t="n">
+        <v>7751.25</v>
+      </c>
+      <c r="G419" t="n">
+        <v>7740.5</v>
+      </c>
+      <c r="H419" t="n">
+        <v>7749.75</v>
+      </c>
+      <c r="I419" t="n">
+        <v>24583</v>
+      </c>
+      <c r="J419" t="n">
+        <v>4</v>
+      </c>
+      <c r="K419" t="n">
+        <v>39</v>
+      </c>
+      <c r="L419" t="n">
+        <v>0.181</v>
+      </c>
+      <c r="M419" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="N419" t="n">
+        <v>40</v>
+      </c>
+      <c r="O419" t="n">
+        <v>0.203</v>
+      </c>
+      <c r="P419" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="Q419" t="n">
+        <v>7.091</v>
+      </c>
+      <c r="R419" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S419" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Sept. 29: Carnival Surges 13% on Record Bookings, Raised Guidance - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="T419" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxNLThyaTVvUmFCc0VKZEluVjF1WkxxTjJGX0JJcVFnVmhnSjh0RjBIX01COGJDV2VlUXBFSVo5RG1EZmdSUmhmRVZUZHNOU1JPN3NhSW1PRjZvZmhEdFNGU1J0cWhsNm1ldWloY3BmUXg1a1VwUGxrbnJiMTAzdnkzekNnaTV4MjZZczEwQURmSjhYWlY1SUk4VjFwUy1qZUJnRUxsbVJDcGRzZGZ6NDFfMzNONjFFOWFnenE3TnZzN0JBOFlQTEliajM1WEJxQkdPZjlNdXYyQ00?oc=5</t>
+        </is>
+      </c>
+      <c r="U419" t="inlineStr">
+        <is>
+          <t>Navitas Semiconductor stock surges 20% on U.S. defense contract - Investing.com</t>
+        </is>
+      </c>
+      <c r="V419" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQNEh0SWNBYm1CU01OYXNoTkU3aUl4RmN6X21XS1I4ejBTbnNCMXJKZXFHRWdhc3FUNm1BcFYxakdQMlNCSzg4a1J3UUo0RC1BMC1OeGVRUXVScmJnUkR5VGhBWjRqQkg1dUEzUmdRcFk2b1VBT1RoNWx0SjJ6T241ZkhyVndHR2w2YURDTm11N2x2WnVmWUgyVXRxYUxrdTdZTW90MC0zZ3ZBNlNyWWRHaHNueUQ3YTBa?oc=5</t>
+        </is>
+      </c>
+      <c r="W419" t="inlineStr">
+        <is>
+          <t>OSR Holdings (OSRH) Surges 15%: Small-Cap Stock Breaks Resistance, Eyes $0.50 Level - Dividend ETF - careplusvn.com</t>
+        </is>
+      </c>
+      <c r="X419" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPeU1GWGNLRllfbnJweWwzWDBwZnZTOGphUXlMOVFLMFcwc0RqUGJXVGFxcmx1Mkdwa25XanZ5ZGVRbDczQkd2bzZRX3k3UXRuZlFkYWp0dzVacWkzbzQtaG9adEhDWi00cGx0eXlGc2Z4Q0I4UUZqR1czN2ltaHc3MkdsRnBuY1pLRXR6UjlaMHRpSHctSXVtVDJxZkVwekxNbUhKd3lIaVpmeUNxU3NLRnYwM0pJdE9BU2cxdmxB?oc=5</t>
+        </is>
+      </c>
+      <c r="Y419" t="inlineStr">
+        <is>
+          <t>If a Stock Market Crash Is Coming, History Says This ETF Could Be the Smartest Buy for Investors - finance.yahoo.com</t>
+        </is>
+      </c>
+      <c r="Z419" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQS1JvNzZmU2xWbFRsWEd2SjlVWnRDandpVHgwcXBFWVZCSlJUZ3hWend0RFlzOURVM2xTSVJJVEFSZVZCcnlwR3lKazBDTEZlOEp4Q0M5SlhfQlhVSTJtX0hnM2lNV3VMTnNUd2thYXJCam41VGZOUDlFbG1hczZ5ek1obkxrQ08zVV83ZzMtM0stU0tCYVIwbWZ3c29ycGM?oc=5</t>
+        </is>
+      </c>
+      <c r="AA419" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 falls for third straight day - Fox Business</t>
+        </is>
+      </c>
+      <c r="AB419" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5mVGZhR2M2RXNUaW82ZXZfOGVwTjBCcVNaTXpZUFpSNXdKY1RIZENnWk9sLUMyOGNwSVNnRmRfTWJZeEZEOGVhQXd2a1VKdTA0SmhTM3cxQjZGWjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC419" t="inlineStr">
+        <is>
+          <t>If a Stock Market Crash Is Coming, History Says This ETF Could Be the Smartest Buy for Investors - The Motley Fool</t>
+        </is>
+      </c>
+      <c r="AD419" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPNmZsYzdSQlYxVjBRQ0I5czFNbmxLLURMRTluU1FGRENsUzgzOWpJV3pYN1RfckE1T3dlbHdxMlFUcTUzaFZiOUp0clFxN3dQRWpMTHVuRG9XbG94Z3ctSmdpWkVLR1A1Rm4yZTd1bnVmaDNwV09EVTQwSVVlYXlpdWU2MlY3TTY0RnJvQ1FJVEc2Y2ZaNjkzcQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-09-30T04:25:27+00:00</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>NQ=F</t>
+        </is>
+      </c>
+      <c r="E420" t="n">
+        <v>30653.75</v>
+      </c>
+      <c r="F420" t="n">
+        <v>30669.5</v>
+      </c>
+      <c r="G420" t="n">
+        <v>30571</v>
+      </c>
+      <c r="H420" t="n">
+        <v>30650.75</v>
+      </c>
+      <c r="I420" t="n">
+        <v>19024</v>
+      </c>
+      <c r="J420" t="n">
+        <v>4</v>
+      </c>
+      <c r="K420" t="n">
+        <v>37</v>
+      </c>
+      <c r="L420" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="M420" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="N420" t="n">
+        <v>38</v>
+      </c>
+      <c r="O420" t="n">
+        <v>0.264</v>
+      </c>
+      <c r="P420" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="Q420" t="n">
+        <v>9.01</v>
+      </c>
+      <c r="R420" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S420" t="inlineStr">
+        <is>
+          <t>Tech Stocks Surge as Apple (AAPL) Hits Record High - GuruFocus</t>
+        </is>
+      </c>
+      <c r="T420" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPbUtsdjFuWFdnMjZ2b2RGMjQzVzhXSG03Y1dYUmxXNmxjZlhiRkx3aVRPbEhyWk1XX3I0UUw3bjVkVTFzR2JTc1hSTFVEUVlSbnVDZm9rb0lCZFNvRnZKdnJ2ZjBhU1J2Tzl2V1VJY3UwckZqTE53YXdZdW10M3gxdUFxN1o2LUVjWkhDZXlnM18?oc=5</t>
+        </is>
+      </c>
+      <c r="U420" t="inlineStr">
+        <is>
+          <t>Stocks boosted by tech earnings; bond yields hit multi-year highs - Reuters</t>
+        </is>
+      </c>
+      <c r="V420" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxPNlVXYXdFRjZLcGRvZUdsRkVNc0ZwYUJzNE1rcHdzN3VQOC00WF90TVNOdXhudGZVY3BqWlJ5ZUVTUDZYLVVhd2VEekFRX25rdnZwck13QThNMUhLOEpuVUZHUDhMV3d5ZmlKbDJOTmJmRDQ2Y29uTDBONzZSZ2d5aGtNZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W420" t="inlineStr">
+        <is>
+          <t>S&amp;P 500, Nasdaq, Dow Forecast: Wall Street Split Widens Into Month-End - stonex.com</t>
+        </is>
+      </c>
+      <c r="X420" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNcy04QTN2dUFjZ0V3MkxNNkhYSTZ4THBjNXpqbkczLTlJQkpEeHFXbERVOG90YUdDMFZTRk9iUUFzbnlzVW84TG5FQ19LaE5sWmp4WGNadmN5QmVwaWVKc3QxM1ZQTVI3Y01vZlpUWmJmeWd2R3k1UEwzTE1QUmFEc2hTOFlWVjRabkJYdGxXcjFVckhsUkJ2UmYwQjc5cm1JaGlqdzluUWNlWC1GWnc2bWJQMzZMNTdE?oc=5</t>
+        </is>
+      </c>
+      <c r="Y420" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 Forecast: NDX rises as oil eases and tech gains - stonex.com</t>
+        </is>
+      </c>
+      <c r="Z420" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPLW1jVmJFX0hHWElrSWo5SHdxc1dYVEVBbHlydHp6eDlXSmpOd2w5SHZfTlYtOU82RnhkYzZCNVpjRWI1TjV3OU80cVdGRkJwdFMtVjdNMEk5bUVTVWdnemtQQ1FHV2s4dm9GLXZFa3VmZDE2UHpGT2lDWjE1U212eUdtMERfSFlzWWl6TUNJanJmeHdSMlE0eW11Ri16Z2c1U3hRd1RCRW8?oc=5</t>
+        </is>
+      </c>
+      <c r="AA420" t="inlineStr">
+        <is>
+          <t>Nasdaq analysis today at investingLive.com - TradingView</t>
+        </is>
+      </c>
+      <c r="AB420" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQdm0tWXlKR0hxZHRBUEJpSEkyX3RBZkxjU2x6UzUyUkIwRS1OclFFRmhJWHJ4WmFxU1BXOW83elNPTFNtNW1sTzc4RTRILXhwYjNwSy16T0dubWhvUlpjX2lwMTNEVkZhejRSWnRUdVhIX2FNUEQ0TEprajlRdkR4RmFVSHhlazZ6MGRwRWpqXzN6UVN0RmxRMWI3M2RVd2ptOHFUMQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC420" t="inlineStr">
+        <is>
+          <t>Dow Drops 132, Nasdaq Loses 23, S&amp;P 500 Falls 13 - TV News Check</t>
+        </is>
+      </c>
+      <c r="AD420" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOWVl3dU1hNlNGdGJkaWVqRWptcFVWRnBlSDdIVVFrVnVVMFBpWFpRVmtCejVpMDMzY1BvRGNKUUg1ZHNoQ2laOVhleHR5QzVESjU5b2ExUWRKcThMeTlsRHRVbDNtemcxRFZVZ2pwdFFOWG1WQVdudUloUTdHZngzVWpycFJ1Mk9aM19lU2xscVY?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-09-30T04:25:27+00:00</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E421" t="n">
+        <v>83417.07030000001</v>
+      </c>
+      <c r="F421" t="n">
+        <v>83584</v>
+      </c>
+      <c r="G421" t="n">
+        <v>83129.3438</v>
+      </c>
+      <c r="H421" t="n">
+        <v>83376.35159999999</v>
+      </c>
+      <c r="I421" t="n">
+        <v>218028032</v>
+      </c>
+      <c r="J421" t="n">
+        <v>4</v>
+      </c>
+      <c r="K421" t="n">
+        <v>39</v>
+      </c>
+      <c r="L421" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="M421" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="N421" t="n">
+        <v>34</v>
+      </c>
+      <c r="O421" t="n">
+        <v>0.465</v>
+      </c>
+      <c r="P421" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="Q421" t="n">
+        <v>14.993</v>
+      </c>
+      <c r="R421" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S421" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 12% in two days as Trump, crypto execs lead last ditch effort for Clarity Act - cnbc.com</t>
+        </is>
+      </c>
+      <c r="T421" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOYW5ydk13NmdWaS1wZXd0MC1KQnpxOUdGY3R6SFpYMDVIZFNfMW5RQTU2b1dfYXVtMDhiWERTMXdwdjlEQWl5V2dsSm00NE5pY2phS0I1R015QWJ3cEVHaG0wUjZXYU5oUm1LWFl2bVZuNmF2WUZRZlI5LUItQVZNdjF1X0VKeW50b2l4WG5SWWdEN25oajl0bi1qU0ZabEh2c1owQV9jSVDSAa4BQVVfeXFMT3lZRHR0SU5wSjZla2VFbldPbk04ejJ3UUJjLVNaUndRQlgyR2F0SnJsOXltSVV0NTVDemd6VzhyOTlidWNwUXp2WjctTkNRYS1rTjdRblRHcTdVQ05KNXVrdFM5Ulk1NjgtOC1lNWlobUp6NWhXNzNoNlBEWWpnUXVuSy0tTm05VDBIT0JaOTJ4X3BKaW5scUNQYUFIRTR1OG9TQzM5ZFYyUTFhWmln?oc=5</t>
+        </is>
+      </c>
+      <c r="U421" t="inlineStr">
+        <is>
+          <t>Bitcoin surges 22% for the week as investor optimism floods back - cnbc.com</t>
+        </is>
+      </c>
+      <c r="V421" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOcjRGYUZ1N0FTMjBSWUZKS3BUU2dhVVVxYzdLQ0lMRkhNZ0hua3c3Uzg2N3AyNThYb3JfR3BYQ09sWkl1Ni1Pd3R3UEFkNFRRUGtMNW9TTllKQ2huZ1c3UWN5ME85dHFOblprdVNjWk5GN2xvRXBXSU1HdTNyRmpyVUtZTUZDV08xVzN3dUJR0gGTAUFVX3lxTE91YXlLVVY1aGtjTzVEU05mWTU4c0pFT0I4ZW5OOHltMk1zV0FwNTVQZnZrQzlVazVIOTgtWkp6d3lxTmljc0ptZUwtU05oUEs0MXNRYXlDVmpjUHVuRnFMdzBEbGMzWDFrekdnbmY2ajl1TzRkQ09TcDZTWlBYWlJGak4xOFkzMElveWZOVzBKcEpxWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="W421" t="inlineStr">
+        <is>
+          <t>Bitcoin Surges as Institutional Demand, Short Covering, Clarity Act Progress Converge - WSJ</t>
+        </is>
+      </c>
+      <c r="X421" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYVg0QkZmc3p2MENoYl9xejdUYzd2NmxxWERxaWl2VGJNSTFIaVVQZzNOYS1fYVA4X0Y4RVc4QnR3ZjdCaGktTEtuSld3R2tQQ3ZGX19fc2YxcVZNRE1jd0kyOVlpNGZoYXVYVHRUNGt5Z0ZQWHNpUnFEMF8tVHI4N1Z0M2hvNXMteEd0T3g1NDVlSHNQZmRlSzNJNXg0eGNuajBXdzVRdmYzOVNnY2V1bkVUZlJwYXRyYlBMel9yR042VTRJMTlXTm01dw?oc=5</t>
+        </is>
+      </c>
+      <c r="Y421" t="inlineStr">
+        <is>
+          <t>Current price of Bitcoin for Sept. 28, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z421" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE10TUZGTV9PZWFjUUFTTUwwLTJRZGllSjJEbk5zLVVaTnJSOUd1LUw2OGN3bWl4azRQcDd5VDBuenoxYm93UDdlNS1GWk84Vk5yR3lmYVpma09tOHI4M2NNWGhwYVIwWUU?oc=5</t>
+        </is>
+      </c>
+      <c r="AA421" t="inlineStr">
+        <is>
+          <t>Zcash Volatility Explained: Liquidations, Whales, Sector Shifts - CoinMarketCap</t>
+        </is>
+      </c>
+      <c r="AB421" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9TbE5mMkZiN0psUzFJMU83ZUhUTXpuX1hwYlE1dXJqSzY4MVVlMC1vczZQa0d0M2ljWG1tRG5fR2RaeExkTmhlT0ltLWJ3WnVwa2FJLWtTLVM0REg5VFp3MGxaX2tSWlhLYlRVSXdPS18?oc=5</t>
+        </is>
+      </c>
+      <c r="AC421" t="inlineStr">
+        <is>
+          <t>$297M Bitcoin moved by Strategy was internal, n... - Pluang</t>
+        </is>
+      </c>
+      <c r="AD421" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQOFM4dVVNY1R2S2t6VGYzV0h6djJhQUptTEJ5YXJMVjFtczRxVWxXX254VlhyaG5rVk4yZHRNQ3ZOdC1VUlA1d2hWOFlpWjRkNkZDbkxQYm5hQ1RfM19xcUdoZXY1SEp3bmFUNTF3NllkZ3BzZml0Tk1kRlo4dzFibXhPNnk3eldOUXROdmctU0N6TFZoMlgtcUhpdHY2NkRFeWVkMS15MkpQVHI3?oc=5</t>
         </is>

</xml_diff>

<commit_message>
Scan: 2026-09-30 14:45 UTC
</commit_message>
<xml_diff>
--- a/data/asset_sentiment_log.xlsx
+++ b/data/asset_sentiment_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD421"/>
+  <dimension ref="A1:AD427"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53021,6 +53021,762 @@
       <c r="AD421" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQOFM4dVVNY1R2S2t6VGYzV0h6djJhQUptTEJ5YXJMVjFtczRxVWxXX254VlhyaG5rVk4yZHRNQ3ZOdC1VUlA1d2hWOFlpWjRkNkZDbkxQYm5hQ1RfM19xcUdoZXY1SEp3bmFUNTF3NllkZ3BzZml0Tk1kRlo4dzFibXhPNnk3eldOUXROdmctU0N6TFZoMlgtcUhpdHY2NkRFeWVkMS15MkpQVHI3?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-09-30T14:43:03+00:00</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>GCZ26.CMX</t>
+        </is>
+      </c>
+      <c r="E422" t="n">
+        <v>4215.8999</v>
+      </c>
+      <c r="F422" t="n">
+        <v>4251.1001</v>
+      </c>
+      <c r="G422" t="n">
+        <v>4197.5</v>
+      </c>
+      <c r="H422" t="n">
+        <v>4201.7002</v>
+      </c>
+      <c r="I422" t="n">
+        <v>50618</v>
+      </c>
+      <c r="J422" t="n">
+        <v>4</v>
+      </c>
+      <c r="K422" t="n">
+        <v>40</v>
+      </c>
+      <c r="L422" t="n">
+        <v>-0.122</v>
+      </c>
+      <c r="M422" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="N422" t="n">
+        <v>40</v>
+      </c>
+      <c r="O422" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="P422" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="Q422" t="n">
+        <v>-2.083</v>
+      </c>
+      <c r="R422" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S422" t="inlineStr">
+        <is>
+          <t>Precious Metals Surge: Gold Approaches $4,500 Mark, Silver Reclaims $66 - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="T422" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAxTUhJVFR3RXFNV3VTVFBNTl9OUXhvNmx6R01EZjFqSW05UWJjN3JIUGltNUNobFJKazVGR0lhb1J2bS1iRDdSeC1Fa0YtNU1BQi1xM1hnVjhaZklSUjFpU0ZHWV9GOHlncUtZMmtKTzRxQV8zM2c?oc=5</t>
+        </is>
+      </c>
+      <c r="U422" t="inlineStr">
+        <is>
+          <t>Gold hits record high as investors seek safety - ABC News - Breaking News, Latest News and Videos</t>
+        </is>
+      </c>
+      <c r="V422" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVWt1Y1hBWG5uZFNjRUFtZHlqRUhfZGV6VzAtQ0tBT2VlVDVEZEJ2WHN0YndCcXRzSjNtVnFhUFZZZ2F4RFRxYkdsSF91eDk2MFl5R3JNWk1HREJjSVdhUE1uTTU1N1Z6Y2xfZzZCSDZ4YnhaT1czcWdXeHE3SjJBR2FqUm43Z0paUG5OVEdsWVdYYnZBWVHSAZsBQVVfeXFMTWh6VXlqZGZVbUl3SHVfQ195WFFveEVkLU9TU1RXMTZBdVhodU16UWxLLWVScDNsc2VGMThyT0RTTHB4SVNRYU1KWmRycHhnTEc0NTJ1RWgzdGc2Y0VkanR4QUtlUWFBSnB2cElORUltQk9XdWRLNXhKbU5jRUFqQVd6bG5YbURJakxhNTl3UEk4RzBaQzVJaVdRdFk?oc=5</t>
+        </is>
+      </c>
+      <c r="W422" t="inlineStr">
+        <is>
+          <t>Gold: Prior floor becomes resistance — NFP breaks the structure and bears own the tape - FXStreet</t>
+        </is>
+      </c>
+      <c r="X422" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNZmpYbjdKbktMMGFsV2xjZmRjaVJMR2h6OUJIcF94NDRHTHZTaE1NSXlsSzR2dS1aa0JCeTZ5a05IbVpjYjZ6SDNlSU9HSFEySmlqbl9yUFBrcF9Na2JKNEtPRzRmS1BPc1Zia1ZLcTZLOEM2YVB4dHRrQjZkQ2JmTTZJS2k5YkFnWUxqdVAtVFVqeTItc3JDUHd6M1JVM2p1aW1uNWpNc1VRbUVNWlE4NGszRW1KRlB1RXNGcFpYNERPRURoTEFXOTl3?oc=5</t>
+        </is>
+      </c>
+      <c r="Y422" t="inlineStr">
+        <is>
+          <t>Global demand drives record holdings - World Gold Council</t>
+        </is>
+      </c>
+      <c r="Z422" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE1IUWRIWVBPTDdNaTdkeDdLSUlIZ21SMHJNU2wzbi1ldl9SOWl1WWNYZHNRY3ljSm5Kdlg0WWdDcml1Z1dhbHpwVm0zbEE1a0d2NmllWlFqQkdfTUYyM19ZYjB5M0RkVU5LZkE2dTQxRXY4cldoNkJJa3F5VlFXdEE?oc=5</t>
+        </is>
+      </c>
+      <c r="AA422" t="inlineStr">
+        <is>
+          <t>Gold market sees positive ETF inflows in July, ending two months of outflows - Kitco</t>
+        </is>
+      </c>
+      <c r="AB422" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNcGdBZURLclpjb21vODJwTDdrcndNR2ZCUGdqRGVoYXhkWkdFZEpHT2wyMnNORDJnRUtxcGhZTGxWcGxfNVhxLVpHNlh2c2VpbW5JOENUeFpJT1QxMnVCRWdsNFROQzZuYjNxbmptZGVWbTliMWJTcVBVU2hrMGs0Qlpkb2p6Y1hydWZJQVlWcS1kejhZTDZyU2UwQmVBNHpLMkp5UUxsNmJvV2c5ZU9vMEdNZk1Zdw?oc=5</t>
+        </is>
+      </c>
+      <c r="AC422" t="inlineStr">
+        <is>
+          <t>Gold ETFs Shine in H1 2026 with Unprecedented Liquidity - Investing News Network</t>
+        </is>
+      </c>
+      <c r="AD422" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE1JaGRkaHpGODN4bGpQdFl6S3VyUjZKYzRvWUxjUjhyQ0lVXzZMZEltdGkwMEo2d0lhVWVmMDVUYUJfRXF4emdyX0ZTd0N6SVgwN3kxMFVXTkt5WXZJbE8ybVNRLUJYTVZy?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-09-30T14:43:03+00:00</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>CL=F</t>
+        </is>
+      </c>
+      <c r="E423" t="n">
+        <v>90.58</v>
+      </c>
+      <c r="F423" t="n">
+        <v>91.73999999999999</v>
+      </c>
+      <c r="G423" t="n">
+        <v>90.06</v>
+      </c>
+      <c r="H423" t="n">
+        <v>91.26000000000001</v>
+      </c>
+      <c r="I423" t="n">
+        <v>71871</v>
+      </c>
+      <c r="J423" t="n">
+        <v>4</v>
+      </c>
+      <c r="K423" t="n">
+        <v>40</v>
+      </c>
+      <c r="L423" t="n">
+        <v>-0.019</v>
+      </c>
+      <c r="M423" t="n">
+        <v>-0.264</v>
+      </c>
+      <c r="N423" t="n">
+        <v>40</v>
+      </c>
+      <c r="O423" t="n">
+        <v>0.212</v>
+      </c>
+      <c r="P423" t="n">
+        <v>-0.104</v>
+      </c>
+      <c r="Q423" t="n">
+        <v>3.862</v>
+      </c>
+      <c r="R423" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S423" t="inlineStr">
+        <is>
+          <t>Iran War Raises Demand for US Fuel, Boosting Gulf Coast Refining Margins - EnergyNow.com</t>
+        </is>
+      </c>
+      <c r="T423" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOaFBFeE9aMXltVV9yS0xqMEFpaVJGaG10NkVOa09mNTEwM1JyT1p6eEdKYkxvYnJQTWtaaUItS1hZbC1xandMZHpaV3N3Yzh4MmwzUVZPZnZyOGtjcVNlcFAxSFZSanVRcXhwOXpxR1R5M0U3NjRkV2NKODRmaUM2R05jY2RfTk15bkpKMFdTMVlQSFo3b3l5MVFIVUtPTFdZSFJtcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="U423" t="inlineStr">
+        <is>
+          <t>Oil prices surge 15% as Strait of Hormuz disruptions tighten supply - Offshore Technology</t>
+        </is>
+      </c>
+      <c r="V423" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPdndjemtyTkduUUpSVnR6aXJUNXBBR0JNd1FaaURNWmtvWm9WTkZUME50Qk1NVDUtdEtqcWE2R0xvUGRKNHBWZDMtblpaY1h1TE5zcmgycU5kS29mYU02N1BOdThBMUhUMDM0T1FScDZRY0JzYlRXTTJVajFYbkh3Rmp0MDFDeVZQcFhKSjhpaklySjZrVWJCZVoyWkw?oc=5</t>
+        </is>
+      </c>
+      <c r="W423" t="inlineStr">
+        <is>
+          <t>Crude Oil &amp; Gold Forecast: Key Levels to Watch - FOREX.com</t>
+        </is>
+      </c>
+      <c r="X423" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPWTB1cHRpdk5MalktTnBqZV91SUZjNDZDRV9Fc0tLZ2ZCUFVqSmk0d21BYTk3SnBHVVJsQ0tyVGwyQnVhd1lrNFEzV2M3Vk5jbC15aVlVM1Zyd0QtVWlCR2ktZ19UNDdRSDFwQlNtdV9PTk5sa1pfTzFhSTJQZ1pXVVFud3VrcVhGR2JWLURfZ19VS3NFQ1RVTlFR?oc=5</t>
+        </is>
+      </c>
+      <c r="Y423" t="inlineStr">
+        <is>
+          <t>Current price of oil as of Sept. 28, 2026 - Fortune</t>
+        </is>
+      </c>
+      <c r="Z423" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9rRk9pZkN0bERaRFVvU0wyVmU3SVQwWEpsYm1EMkR1eWg5dnJjNDBzNGlpZHpyVmFiRUlJYUF1MnhYMnFSalRMWXRSWWZfWHpNX0hJNXJyaTg2T2ZKckNOSFVn?oc=5</t>
+        </is>
+      </c>
+      <c r="AA423" t="inlineStr">
+        <is>
+          <t>OPEC+ approves further oil output increase as Hormuz exports start to recover - cnbc.com</t>
+        </is>
+      </c>
+      <c r="AB423" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNS2hIVlN3T2xXekl4NzRBN0xWcE8yVnZoMkJEUWRFc2lDLWhSUjVaLXFLbTJhWWc1dzY0YlJaUXVtQ2FmRXdPZGJtSzJ3SnJWM1REVWhvVGNjRHF2T1FEaG1fNHJGR2VuWktvVHNZNFpkbHhRODVBSllaaGNCV1Y4cUdOaFVDcFZqTWNXVtIBkgFBVV95cUxNaV9JVVVaUGRVTXFFSFVBdWZDLUwxcjl4dTJIb21CZFRCX2prVndxLVV6RVphUzFhSlRFRzNJQlRXb0h2WW9reUtsaS1iVDNMMG9LUWZsdEhYN2gzLUwtM1JYaVVScnk0STlyMHl1emRJU0k4dE1SZnB5VXVkM3pyYXNBZGtzaVdSOGpMejBjRTlKQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="AC423" t="inlineStr">
+        <is>
+          <t>Brent Oil breaks $101.50 neckline, eyes $97.49 support: Live - Investing.com</t>
+        </is>
+      </c>
+      <c r="AD423" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNNkJzUzhFV0FCT1pubGlZY2hZREFHb000NnRGNzROamFXNXd6Wk1oMjdqQlVKRW5iS3ZOZkh0SmNkeXAxbHVHV19OY3hERG0wNVZaZzhGWWx3c3FWWGpQXzhCQVl4VkJpcWJxbmtVMXVjdncxdFpHTjc5ZGJQWG9DTmJ1amlnV0gyS3I1c2NfWGtGb3NhWW9CUkd1OVotVk12OTRVNS0wWGpGV0VoSFN0XzcyQ2h0dw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-09-30T14:43:03+00:00</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>US Dollar</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>DX-Y.NYB</t>
+        </is>
+      </c>
+      <c r="E424" t="n">
+        <v>101.192</v>
+      </c>
+      <c r="F424" t="n">
+        <v>101.28</v>
+      </c>
+      <c r="G424" t="n">
+        <v>101.026</v>
+      </c>
+      <c r="H424" t="n">
+        <v>101.254</v>
+      </c>
+      <c r="I424" t="n">
+        <v>0</v>
+      </c>
+      <c r="J424" t="n">
+        <v>4</v>
+      </c>
+      <c r="K424" t="n">
+        <v>39</v>
+      </c>
+      <c r="L424" t="n">
+        <v>-0.005</v>
+      </c>
+      <c r="M424" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="N424" t="n">
+        <v>40</v>
+      </c>
+      <c r="O424" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="P424" t="n">
+        <v>-0.043</v>
+      </c>
+      <c r="Q424" t="n">
+        <v>2.217</v>
+      </c>
+      <c r="R424" t="inlineStr">
+        <is>
+          <t>finbert</t>
+        </is>
+      </c>
+      <c r="S424" t="inlineStr">
+        <is>
+          <t>U.S. Dollar Gains From a New Wave of Safe Haven Demand - stonex.com</t>
+        </is>
+      </c>
+      <c r="T424" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxObnI1LWEyU0VuTFRTVlN3dFZ5UEp1M08weUxGaHFjVFVYeFFtbkdVTUtWUUpWU2d3cU5XWWVWMjc5SkNrMmtEZTNrYUZBUHo0SmpRNDctQm5oZkQtOEpZcUNHRTVpQVFUNmJIeUowLTJRbjNxeWJlY2kwOHc1RVRrMXA1SmRjM1FaZFdBVGgzMFdlbXc?oc=5</t>
+        </is>
+      </c>
+      <c r="U424" t="inlineStr">
+        <is>
+          <t>United States Dollar Index approaches yearly peak on hawkish Fed outlook - FXStreet</t>
+        </is>
+      </c>
+      <c r="V424" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQdUVDWVdBQ1FGa1UtNFpxLXFPQ2h6R3REb2gyWm5ZcWhoLUNEbmJVZGl1V1VGdlNmNW9XdHZleXNRV1lMQVF4NnRTWlpEamJMTTk1U1ptU0pNY005RFh3dUhncjVvRFFWRWR3akIyeVVuWlI1TWZtdGZydm0wblpodDVZNzJ2MkdWM0RhdFJWZExfYV8tckwwYXFVZkdrb21zRm9jRlJyenlkV0FDRlBLMXcyTHFZZw?oc=5</t>
+        </is>
+      </c>
+      <c r="W424" t="inlineStr">
+        <is>
+          <t>Dollar rides safe-haven demand, set for best month since July - Virginia Business</t>
+        </is>
+      </c>
+      <c r="X424" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOcXlFekFKUkpNd0ZrQjd4Xzl6ZS00UjltYUx1Ri12N3F4NDdmMTZSRlV0eFFKeXVwNEJ2aXd6cUM5cFpaQ0hfNDlLZVpSWUxUOVVNUEhkTHJqUmhCZ1ItaTJhd2QxZUhQQXJrX0MwVnZpMHdLYkh4NEFsY1FuZDRvZQ?oc=5</t>
+        </is>
+      </c>
+      <c r="Y424" t="inlineStr">
+        <is>
+          <t>A Hawkish Fed And A Dovish SNB Are Driving Gains In USD/CHF - Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="Z424" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMWJTSjNwNUl1WXQwODN3UXVUc1lZcWJxSXNreFdCZ3d5a2p4Q2ZpUjkzZXlIcDFWczlpN1RDRUxXU0FIVk5VTE90dXA3NTc3SkN5Z3RFNUc0QUpua2hicUoweHZPdXlfTk5kOF92dldyQTh3bno2YU1HVXJNTkxscDhKQThuSTd4SjVNWkpBU21FWXBRbG80?oc=5</t>
+        </is>
+      </c>
+      <c r="AA424" t="inlineStr">
+        <is>
+          <t>FX Daily: Bond sell-off helps USD consolidate gains - ING Think</t>
+        </is>
+      </c>
+      <c r="AB424" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNbzMtME9DWnA3YzBIa1FYM2VjQ1Zzcnp2T1RVcGljSEVuUVdFdHQxYW1TNl9nbXRJb0FObTRUekNya1VQa3FrVUpLekFqNzF0NXVpaVk4RXV2WVZFdzJTbXV1MFczYmY1cndYQXQ3Mlc2UFZ2bGdDRmxTNGxTVDFQTWd4TVlCa0VF?oc=5</t>
+        </is>
+      </c>
+      <c r="AC424" t="inlineStr">
+        <is>
+          <t>British Pound gains as US Dollar weakens despite hawkish Fed, geopolitical tensions - FXStreet</t>
+        </is>
+      </c>
+      <c r